<commit_message>
Fix DCF Gordon vs exit-multiple sanity check to use spread column
The reconciliation PASS/REVIEW flag was incorrectly testing the Gordon
implied multiple (~7.0x) instead of the variance vs the 8.0x exit
assumption. Update formulas to reference column D (spread) so ~1.0 turn
difference correctly shows PASS within the ±1.5 turn tolerance.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0x"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -192,6 +192,18 @@
       <b val="1"/>
       <color rgb="00006100"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="00C8102E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Garamond"/>
@@ -269,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -389,26 +401,45 @@
     <xf numFmtId="164" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="168" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="168" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -417,6 +448,9 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1607,7 +1641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2123,365 +2157,495 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="inlineStr">
-        <is>
-          <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
-        </is>
-      </c>
-      <c r="C25" s="37">
-        <f>H17*(1+Scenarios!$D$9)/(Scenarios!$D$8-Scenarios!$D$9)</f>
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
+        </is>
+      </c>
+      <c r="C25" s="28">
+        <f>H8+H12</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Implied terminal EV/EBITDA (sanity check)</t>
-        </is>
-      </c>
-      <c r="C26" s="45">
-        <f>C25/(H8+H12)</f>
+          <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
+        </is>
+      </c>
+      <c r="C26" s="37">
+        <f>H17*(1+Scenarios!$D$9)/(Scenarios!$D$8-Scenarios!$D$9)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>PV of terminal value</t>
-        </is>
-      </c>
-      <c r="C27" s="44">
-        <f>C25/(1+Scenarios!$D$8)^H18</f>
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Implied exit EV/EBITDA (Gordon Growth)</t>
+        </is>
+      </c>
+      <c r="C27" s="45">
+        <f>C26/C25</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
         <is>
+          <t>PV of terminal value</t>
+        </is>
+      </c>
+      <c r="C28" s="44">
+        <f>C26/(1+Scenarios!$D$8)^H18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
+        <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="C28" s="28">
-        <f>C23+C27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="14" t="inlineStr">
-        <is>
-          <t>Plus: cash &amp; equivalents (FY2025)</t>
-        </is>
-      </c>
-      <c r="C29" s="36" t="n">
-        <v>1807202</v>
+      <c r="C29" s="28">
+        <f>C23+C28</f>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
+          <t>Plus: cash &amp; equivalents (FY2025)</t>
+        </is>
+      </c>
+      <c r="C30" s="36" t="n">
+        <v>1807202</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
           <t>Less: total debt</t>
         </is>
       </c>
-      <c r="C30" s="36" t="n">
+      <c r="C31" s="36" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="18" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
       </c>
-      <c r="C31" s="28">
-        <f>C28+C29+C30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="14" t="inlineStr">
+      <c r="C32" s="28">
+        <f>C29+C30+C31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>Diluted shares outstanding (000)</t>
         </is>
       </c>
-      <c r="C32" s="36" t="n">
+      <c r="C33" s="36" t="n">
         <v>111380</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="18" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>Implied value per share</t>
         </is>
       </c>
-      <c r="C33" s="46">
-        <f>C31/C32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="14" t="inlineStr">
+      <c r="C34" s="46">
+        <f>C32/C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
         <is>
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C34" s="47" t="n">
+      <c r="C35" s="47" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="18" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>Implied upside / (downside)</t>
         </is>
       </c>
-      <c r="C35" s="48">
-        <f>C33/C34-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="14" t="inlineStr">
+      <c r="C36" s="48">
+        <f>C34/C35-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: % of EV from terminal value</t>
         </is>
       </c>
-      <c r="C36" s="38">
-        <f>C27/C28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="43" t="inlineStr">
+      <c r="C37" s="38">
+        <f>C28/C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="43" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
       </c>
-      <c r="B38" s="12" t="n"/>
-      <c r="C38" s="12" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="18" t="inlineStr">
-        <is>
-          <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
-        </is>
-      </c>
-      <c r="C39" s="44">
-        <f>H8+H12</f>
-        <v/>
-      </c>
+      <c r="B39" s="12" t="n"/>
+      <c r="C39" s="12" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="14" t="inlineStr">
-        <is>
-          <t>Exit EV/EBITDA multiple</t>
-        </is>
-      </c>
-      <c r="C40" s="49" t="n">
-        <v>8</v>
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>Exit multiple selection (see Comps tab for peer build)</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>Terminal value (exit multiple)</t>
-        </is>
-      </c>
-      <c r="C41" s="37">
-        <f>C39*C40</f>
-        <v/>
+          <t>Selected exit EV/EBITDA multiple (FY2030E)</t>
+        </is>
+      </c>
+      <c r="C41" s="50" t="n">
+        <v>8</v>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>Base-case terminal multiple; see Comps → Exit Multiple Build</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
+          <t>Terminal value = Terminal EBITDA × exit multiple</t>
+        </is>
+      </c>
+      <c r="C42" s="37">
+        <f>C25*C41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="C42" s="37">
-        <f>C41/(1+Scenarios!$D$8)^H18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="18" t="inlineStr">
-        <is>
-          <t>Enterprise value (exit method)</t>
-        </is>
-      </c>
-      <c r="C43" s="28">
-        <f>C23+C42</f>
+      <c r="C43" s="37">
+        <f>C42/(1+Scenarios!$D$8)^H18</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="18" t="inlineStr">
         <is>
+          <t>Enterprise value (exit method)</t>
+        </is>
+      </c>
+      <c r="C44" s="28">
+        <f>C23+C43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="18" t="inlineStr">
+        <is>
           <t>Implied value per share (exit method)</t>
         </is>
       </c>
-      <c r="C44" s="50">
-        <f>(C43+C29+C30)/C32</f>
+      <c r="C45" s="51">
+        <f>(C44+C30+C31)/C33</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="43" t="inlineStr">
         <is>
-          <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
+          <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
         </is>
       </c>
       <c r="B47" s="12" t="n"/>
       <c r="C47" s="12" t="n"/>
       <c r="D47" s="12" t="n"/>
-      <c r="E47" s="12" t="n"/>
-      <c r="F47" s="12" t="n"/>
-      <c r="G47" s="12" t="n"/>
-      <c r="H47" s="12" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="51" t="inlineStr">
+      <c r="A48" s="52" t="inlineStr"/>
+      <c r="B48" s="53" t="inlineStr">
+        <is>
+          <t>Gordon Growth</t>
+        </is>
+      </c>
+      <c r="C48" s="53" t="inlineStr">
+        <is>
+          <t>Exit Multiple</t>
+        </is>
+      </c>
+      <c r="D48" s="53" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="18" t="inlineStr">
+        <is>
+          <t>Terminal value ($)</t>
+        </is>
+      </c>
+      <c r="B49" s="44">
+        <f>C26</f>
+        <v/>
+      </c>
+      <c r="C49" s="44">
+        <f>C42</f>
+        <v/>
+      </c>
+      <c r="D49" s="44">
+        <f>B49-C49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="inlineStr">
+        <is>
+          <t>Exit EV/EBITDA (implied vs selected)</t>
+        </is>
+      </c>
+      <c r="B50" s="54">
+        <f>C27</f>
+        <v/>
+      </c>
+      <c r="C50" s="54">
+        <f>C41</f>
+        <v/>
+      </c>
+      <c r="D50" s="54">
+        <f>B50-C50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>Terminal value variance (%)</t>
+        </is>
+      </c>
+      <c r="B51" s="38" t="inlineStr"/>
+      <c r="C51" s="38" t="inlineStr"/>
+      <c r="D51" s="38">
+        <f>(B49-C49)/B49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="18" t="inlineStr">
+        <is>
+          <t>Implied share price</t>
+        </is>
+      </c>
+      <c r="B52" s="55">
+        <f>C34</f>
+        <v/>
+      </c>
+      <c r="C52" s="55">
+        <f>C45</f>
+        <v/>
+      </c>
+      <c r="D52" s="55">
+        <f>B52-C52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="56" t="inlineStr">
+        <is>
+          <t>Sanity check: multiples within ±1.5 turns?</t>
+        </is>
+      </c>
+      <c r="B53" s="57">
+        <f>IF(ABS(D50)&lt;=1.5,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="C53" s="58">
+        <f>TEXT(D50,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
+        <v/>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>Gordon implied should bracket exit assumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="43" t="inlineStr">
+        <is>
+          <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
+        </is>
+      </c>
+      <c r="B56" s="12" t="n"/>
+      <c r="C56" s="12" t="n"/>
+      <c r="D56" s="12" t="n"/>
+      <c r="E56" s="12" t="n"/>
+      <c r="F56" s="12" t="n"/>
+      <c r="G56" s="12" t="n"/>
+      <c r="H56" s="12" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="59" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
       </c>
-      <c r="D48" s="52" t="n">
+      <c r="D57" s="60" t="n">
         <v>0.015</v>
       </c>
-      <c r="E48" s="52" t="n">
+      <c r="E57" s="60" t="n">
         <v>0.02</v>
       </c>
-      <c r="F48" s="52" t="n">
+      <c r="F57" s="60" t="n">
         <v>0.0225</v>
       </c>
-      <c r="G48" s="52" t="n">
+      <c r="G57" s="60" t="n">
         <v>0.025</v>
       </c>
-      <c r="H48" s="52" t="n">
+      <c r="H57" s="60" t="n">
         <v>0.03</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="52" t="n">
+    <row r="58">
+      <c r="A58" s="60" t="n">
         <v>0.09</v>
       </c>
-      <c r="D49" s="53">
-        <f>(NPV(0.09,D17:H17)+(H17*(1+0.015)/(0.09-0.015))/(1+0.09)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="E49" s="53">
-        <f>(NPV(0.09,D17:H17)+(H17*(1+0.02)/(0.09-0.02))/(1+0.09)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="F49" s="53">
-        <f>(NPV(0.09,D17:H17)+(H17*(1+0.0225)/(0.09-0.0225))/(1+0.09)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="G49" s="53">
-        <f>(NPV(0.09,D17:H17)+(H17*(1+0.025)/(0.09-0.025))/(1+0.09)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="H49" s="53">
-        <f>(NPV(0.09,D17:H17)+(H17*(1+0.03)/(0.09-0.03))/(1+0.09)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="52" t="n">
+      <c r="D58" s="61">
+        <f>(NPV(0.09,D17:H17)+(H17*(1+0.015)/(0.09-0.015))/(1+0.09)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="E58" s="61">
+        <f>(NPV(0.09,D17:H17)+(H17*(1+0.02)/(0.09-0.02))/(1+0.09)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="F58" s="61">
+        <f>(NPV(0.09,D17:H17)+(H17*(1+0.0225)/(0.09-0.0225))/(1+0.09)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="G58" s="61">
+        <f>(NPV(0.09,D17:H17)+(H17*(1+0.025)/(0.09-0.025))/(1+0.09)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="H58" s="61">
+        <f>(NPV(0.09,D17:H17)+(H17*(1+0.03)/(0.09-0.03))/(1+0.09)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="60" t="n">
         <v>0.095</v>
       </c>
-      <c r="D50" s="53">
-        <f>(NPV(0.095,D17:H17)+(H17*(1+0.015)/(0.095-0.015))/(1+0.095)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="E50" s="53">
-        <f>(NPV(0.095,D17:H17)+(H17*(1+0.02)/(0.095-0.02))/(1+0.095)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="F50" s="53">
-        <f>(NPV(0.095,D17:H17)+(H17*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="G50" s="53">
-        <f>(NPV(0.095,D17:H17)+(H17*(1+0.025)/(0.095-0.025))/(1+0.095)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="H50" s="53">
-        <f>(NPV(0.095,D17:H17)+(H17*(1+0.03)/(0.095-0.03))/(1+0.095)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="52" t="n">
+      <c r="D59" s="61">
+        <f>(NPV(0.095,D17:H17)+(H17*(1+0.015)/(0.095-0.015))/(1+0.095)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="E59" s="61">
+        <f>(NPV(0.095,D17:H17)+(H17*(1+0.02)/(0.095-0.02))/(1+0.095)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="F59" s="61">
+        <f>(NPV(0.095,D17:H17)+(H17*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="G59" s="61">
+        <f>(NPV(0.095,D17:H17)+(H17*(1+0.025)/(0.095-0.025))/(1+0.095)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="H59" s="61">
+        <f>(NPV(0.095,D17:H17)+(H17*(1+0.03)/(0.095-0.03))/(1+0.095)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="60" t="n">
         <v>0.1</v>
       </c>
-      <c r="D51" s="53">
-        <f>(NPV(0.1,D17:H17)+(H17*(1+0.015)/(0.1-0.015))/(1+0.1)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="E51" s="53">
-        <f>(NPV(0.1,D17:H17)+(H17*(1+0.02)/(0.1-0.02))/(1+0.1)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="F51" s="54">
-        <f>(NPV(0.1,D17:H17)+(H17*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="G51" s="53">
-        <f>(NPV(0.1,D17:H17)+(H17*(1+0.025)/(0.1-0.025))/(1+0.1)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="H51" s="53">
-        <f>(NPV(0.1,D17:H17)+(H17*(1+0.03)/(0.1-0.03))/(1+0.1)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="52" t="n">
+      <c r="D60" s="61">
+        <f>(NPV(0.1,D17:H17)+(H17*(1+0.015)/(0.1-0.015))/(1+0.1)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="E60" s="61">
+        <f>(NPV(0.1,D17:H17)+(H17*(1+0.02)/(0.1-0.02))/(1+0.1)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="F60" s="62">
+        <f>(NPV(0.1,D17:H17)+(H17*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="G60" s="61">
+        <f>(NPV(0.1,D17:H17)+(H17*(1+0.025)/(0.1-0.025))/(1+0.1)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="H60" s="61">
+        <f>(NPV(0.1,D17:H17)+(H17*(1+0.03)/(0.1-0.03))/(1+0.1)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="60" t="n">
         <v>0.105</v>
       </c>
-      <c r="D52" s="53">
-        <f>(NPV(0.105,D17:H17)+(H17*(1+0.015)/(0.105-0.015))/(1+0.105)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="E52" s="53">
-        <f>(NPV(0.105,D17:H17)+(H17*(1+0.02)/(0.105-0.02))/(1+0.105)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="F52" s="53">
-        <f>(NPV(0.105,D17:H17)+(H17*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="G52" s="53">
-        <f>(NPV(0.105,D17:H17)+(H17*(1+0.025)/(0.105-0.025))/(1+0.105)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="H52" s="53">
-        <f>(NPV(0.105,D17:H17)+(H17*(1+0.03)/(0.105-0.03))/(1+0.105)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="52" t="n">
+      <c r="D61" s="61">
+        <f>(NPV(0.105,D17:H17)+(H17*(1+0.015)/(0.105-0.015))/(1+0.105)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="E61" s="61">
+        <f>(NPV(0.105,D17:H17)+(H17*(1+0.02)/(0.105-0.02))/(1+0.105)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="F61" s="61">
+        <f>(NPV(0.105,D17:H17)+(H17*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="G61" s="61">
+        <f>(NPV(0.105,D17:H17)+(H17*(1+0.025)/(0.105-0.025))/(1+0.105)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="H61" s="61">
+        <f>(NPV(0.105,D17:H17)+(H17*(1+0.03)/(0.105-0.03))/(1+0.105)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="60" t="n">
         <v>0.11</v>
       </c>
-      <c r="D53" s="53">
-        <f>(NPV(0.11,D17:H17)+(H17*(1+0.015)/(0.11-0.015))/(1+0.11)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="E53" s="53">
-        <f>(NPV(0.11,D17:H17)+(H17*(1+0.02)/(0.11-0.02))/(1+0.11)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="F53" s="53">
-        <f>(NPV(0.11,D17:H17)+(H17*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="G53" s="53">
-        <f>(NPV(0.11,D17:H17)+(H17*(1+0.025)/(0.11-0.025))/(1+0.11)^5+C29+C30)/C32</f>
-        <v/>
-      </c>
-      <c r="H53" s="53">
-        <f>(NPV(0.11,D17:H17)+(H17*(1+0.03)/(0.11-0.03))/(1+0.11)^5+C29+C30)/C32</f>
+      <c r="D62" s="61">
+        <f>(NPV(0.11,D17:H17)+(H17*(1+0.015)/(0.11-0.015))/(1+0.11)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="E62" s="61">
+        <f>(NPV(0.11,D17:H17)+(H17*(1+0.02)/(0.11-0.02))/(1+0.11)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="F62" s="61">
+        <f>(NPV(0.11,D17:H17)+(H17*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="G62" s="61">
+        <f>(NPV(0.11,D17:H17)+(H17*(1+0.025)/(0.11-0.025))/(1+0.11)^5+C30+C31)/C33</f>
+        <v/>
+      </c>
+      <c r="H62" s="61">
+        <f>(NPV(0.11,D17:H17)+(H17*(1+0.03)/(0.11-0.03))/(1+0.11)^5+C30+C31)/C33</f>
         <v/>
       </c>
     </row>
@@ -2496,7 +2660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2588,23 +2752,23 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="55" t="inlineStr">
+      <c r="A10" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current EV / EBITDA</t>
         </is>
       </c>
-      <c r="C10" s="56">
+      <c r="C10" s="63">
         <f>(C9*C8-C7)/C5</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="55" t="inlineStr">
+      <c r="A11" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current P / E (FY2026E)</t>
         </is>
       </c>
-      <c r="C11" s="56">
+      <c r="C11" s="63">
         <f>C9/C6</f>
         <v/>
       </c>
@@ -2612,116 +2776,320 @@
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Methodology / multiple ranges</t>
+          <t>EXIT MULTIPLE BUILD — FY2030E TERMINAL YEAR</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="57" t="inlineStr">
-        <is>
-          <t>Method</t>
-        </is>
-      </c>
-      <c r="C14" s="58" t="inlineStr">
-        <is>
-          <t>Low mult.</t>
-        </is>
-      </c>
-      <c r="D14" s="58" t="inlineStr">
-        <is>
-          <t>High mult.</t>
-        </is>
-      </c>
-      <c r="E14" s="58" t="inlineStr">
-        <is>
-          <t>Implied px (low)</t>
-        </is>
-      </c>
-      <c r="F14" s="58" t="inlineStr">
-        <is>
-          <t>Implied px (high)</t>
+      <c r="A14" s="58" t="inlineStr">
+        <is>
+          <t>Peer / reference EV/EBITDA (forward / illustrative)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
-        <is>
-          <t>EV / EBITDA (FY2025A)</t>
-        </is>
-      </c>
-      <c r="C15" s="59" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="D15" s="59" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="E15" s="60">
-        <f>(C5*C15+C7)/C8</f>
-        <v/>
-      </c>
-      <c r="F15" s="60">
-        <f>(C5*D15+C7)/C8</f>
-        <v/>
+      <c r="A15" s="64" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C15" s="65" t="inlineStr">
+        <is>
+          <t>EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="D15" s="64" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>P / E (FY2026E EPS)</t>
-        </is>
-      </c>
-      <c r="C16" s="59" t="n">
-        <v>10</v>
-      </c>
-      <c r="D16" s="59" t="n">
-        <v>18</v>
-      </c>
-      <c r="E16" s="60">
-        <f>C6*C16</f>
-        <v/>
-      </c>
-      <c r="F16" s="60">
-        <f>C6*D16</f>
-        <v/>
+          <t>lululemon (LULU) — current</t>
+        </is>
+      </c>
+      <c r="C16" s="66">
+        <f>(C9*C8-C7)/C5</f>
+        <v/>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Distressed trough; FY2025A EBITDA</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
+          <t>Nike (NKE)</t>
+        </is>
+      </c>
+      <c r="C17" s="67" t="n">
+        <v>18</v>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Mature global brand; lower growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Deckers (DECK)</t>
+        </is>
+      </c>
+      <c r="C18" s="67" t="n">
+        <v>15</v>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>Premium footwear peer; HOKA/UGG</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>On Holding (ONON)</t>
+        </is>
+      </c>
+      <c r="C19" s="67" t="n">
+        <v>25</v>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>High-growth athletic peer</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>adidas (ADS)</t>
+        </is>
+      </c>
+      <c r="C20" s="67" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Global incumbent; restructuring</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>V.F. Corp (VFC)</t>
+        </is>
+      </c>
+      <c r="C21" s="67" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Multi-brand apparel; challenged</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Terminal multiple selection (DCF exit method)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>Gordon Growth implied exit EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="C24" s="45">
+        <f>DCF!C27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="56" t="inlineStr">
+        <is>
+          <t>Selected exit multiple (base case)</t>
+        </is>
+      </c>
+      <c r="C25" s="54">
+        <f>DCF!C41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Spread (selected − Gordon implied)</t>
+        </is>
+      </c>
+      <c r="C26" s="45">
+        <f>C25-C24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="56" t="inlineStr">
+        <is>
+          <t>Rationale for 8.0x</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="25" t="inlineStr">
+        <is>
+          <t>•  Above current LULU (~3.5x) — assumes partial recovery from trough, not full re-rating</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="25" t="inlineStr">
+        <is>
+          <t>•  Above comps football-field high (7.5x on FY2025A) — terminal year has higher EBITDA &amp; normalized margins</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="25" t="inlineStr">
+        <is>
+          <t>•  Below premium-growth peers (ONON ~25x, DECK ~15x) — reflects Americas maturity</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="25" t="inlineStr">
+        <is>
+          <t>•  ~1 turn above Gordon-implied exit multiple — conservative buffer vs perpetuity math</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="25" t="inlineStr">
+        <is>
+          <t>•  Well below historical LULU peak multiples (20–30x) — avoids heroic assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>Methodology / multiple ranges (FY2025A — football field)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="64" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="C35" s="65" t="inlineStr">
+        <is>
+          <t>Low mult.</t>
+        </is>
+      </c>
+      <c r="D35" s="65" t="inlineStr">
+        <is>
+          <t>High mult.</t>
+        </is>
+      </c>
+      <c r="E35" s="65" t="inlineStr">
+        <is>
+          <t>Implied px (low)</t>
+        </is>
+      </c>
+      <c r="F35" s="65" t="inlineStr">
+        <is>
+          <t>Implied px (high)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>EV / EBITDA (FY2025A)</t>
+        </is>
+      </c>
+      <c r="C36" s="67" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D36" s="67" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E36" s="68">
+        <f>(C5*C36+C7)/C8</f>
+        <v/>
+      </c>
+      <c r="F36" s="68">
+        <f>(C5*D36+C7)/C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>P / E (FY2026E EPS)</t>
+        </is>
+      </c>
+      <c r="C37" s="67" t="n">
+        <v>10</v>
+      </c>
+      <c r="D37" s="67" t="n">
+        <v>18</v>
+      </c>
+      <c r="E37" s="68">
+        <f>C6*C37</f>
+        <v/>
+      </c>
+      <c r="F37" s="68">
+        <f>C6*D37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="C17" s="61" t="inlineStr">
+      <c r="C38" s="69" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D17" s="61" t="inlineStr">
+      <c r="D38" s="69" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E17" s="60">
+      <c r="E38" s="68">
         <f>Scenarios!C29</f>
         <v/>
       </c>
-      <c r="F17" s="60">
+      <c r="F38" s="68">
         <f>Scenarios!E29</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="62" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="70" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C19" s="63" t="n">
+      <c r="C40" s="71" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t>Note: peer set includes NKE, DECK, ONON, adidas, VFC; multiples are analyst ranges (red).</t>
         </is>

</xml_diff>

<commit_message>
Add clickable source links for blue-font reported figures
- SEC 10-K links per fiscal year under historical column headers
- Blue reported values hyperlink to filing (underlined, click to open)
- Cover page SOURCES section uses live links (EDGAR, 10-K, release, NASDAQ)
- DCF/Comps: source label in column D next to reported inputs

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0x"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="38">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,6 +90,17 @@
     </font>
     <font>
       <name val="Garamond"/>
+      <color rgb="000000CC"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <color rgb="000000CC"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
       <i val="1"/>
       <color rgb="00000000"/>
       <sz val="9"/>
@@ -166,6 +177,19 @@
     </font>
     <font>
       <name val="Garamond"/>
+      <i val="1"/>
+      <color rgb="000000CC"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <i val="1"/>
+      <color rgb="000000CC"/>
+      <sz val="8"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
@@ -178,8 +202,10 @@
     </font>
     <font>
       <name val="Garamond"/>
+      <b val="1"/>
       <color rgb="000000CC"/>
       <sz val="10"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Garamond"/>
@@ -221,6 +247,13 @@
       <name val="Garamond"/>
       <color rgb="00006100"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="000000CC"/>
+      <sz val="11"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="7">
@@ -281,7 +314,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -294,77 +327,81 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="2" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="19" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="21" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="23" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="17" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="19" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -373,10 +410,10 @@
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="29" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -385,75 +422,78 @@
     <xf numFmtId="167" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="30" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="168" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="34" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="35" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -465,8 +505,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="166" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -833,7 +873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B21"/>
+  <dimension ref="B2:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -878,7 +918,7 @@
     <row r="10">
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Blue font  =  figures reported by the company (release, filing, or call)</t>
+          <t>Blue font  =  figures reported by the company (click value or source link)</t>
         </is>
       </c>
     </row>
@@ -918,27 +958,47 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>SEC EDGAR XBRL company facts, CIK 0001397187 (Form 10-K, FY2025 ended Feb 1, 2026).</t>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>SEC EDGAR XBRL company facts, CIK 0001397187 (Form 10-K, FY2025)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>Market data &amp; Q2 FY2026 results per company release dated Sep 3, 2026.</t>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>FY2025 Form 10-K (ended Feb 1, 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Market data &amp; Q2 FY2026 results (Sep 3, 2026 earnings release)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="10" t="inlineStr">
         <is>
+          <t>Current share price (NASDAQ: LULU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="11" t="inlineStr">
+        <is>
           <t>Built from scratch for the GIS IR selection assignment.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId4"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -959,165 +1019,165 @@
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>WEIGHTED AVERAGE COST OF CAPITAL</t>
         </is>
       </c>
-      <c r="B1" s="12" t="n"/>
-      <c r="C1" s="12" t="n"/>
-      <c r="D1" s="12" t="n"/>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Cost of equity (CAPM)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Risk-free rate (10-yr UST)</t>
         </is>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" s="16" t="n">
         <v>0.043</v>
       </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>analyst input</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Equity risk premium</t>
         </is>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C4" s="16" t="n">
         <v>0.06</v>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>analyst input</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Levered beta</t>
         </is>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="18" t="n">
         <v>0.95</v>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>~0.86 market beta; 0.95 used for near-term uncertainty</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Cost of equity = rf + β × ERP</t>
         </is>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="20">
         <f>C3+C5*C4</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Cost of debt</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Pre-tax cost of debt</t>
         </is>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="16" t="n">
         <v>0.05</v>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>illustrative; LULU has no funded debt</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="16" t="n">
         <v>0.27</v>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>normalized marginal rate</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="C11" s="20">
+      <c r="C11" s="21">
         <f>C9*(1-C10)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Capital structure (market values)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Equity weight</t>
         </is>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>net-cash balance sheet → ~100% equity</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Debt weight</t>
         </is>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="22">
         <f>C14*C6+C15*C11</f>
         <v/>
       </c>
@@ -1144,487 +1204,487 @@
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>SCENARIO ANALYSIS</t>
         </is>
       </c>
-      <c r="B1" s="12" t="n"/>
-      <c r="C1" s="12" t="n"/>
-      <c r="D1" s="12" t="n"/>
-      <c r="E1" s="12" t="n"/>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="C2" s="22" t="inlineStr">
+      <c r="C2" s="23" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="D2" s="23" t="inlineStr">
+      <c r="D2" s="24" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="E2" s="24" t="inlineStr">
+      <c r="E2" s="25" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Key assumptions (5-yr forecast)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>FY2026E revenue growth</t>
         </is>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C4" s="16" t="n">
         <v>-0.09</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="16" t="n">
         <v>-0.061</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="16" t="n">
         <v>-0.04</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>FY2027–FY2030E revenue growth (avg)</t>
         </is>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="16" t="n">
         <v>-0.01</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="16" t="n">
         <v>0.028</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="16" t="n">
         <v>0.06</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>FY2026E EBIT margin</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="16" t="n">
         <v>0.125</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="16" t="n">
         <v>0.139</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="16" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Terminal (FY2030E) EBIT margin</t>
         </is>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="16" t="n">
         <v>0.12</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="16" t="n">
         <v>0.155</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="16" t="n">
         <v>0.19</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="16" t="n">
         <v>0.11</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="16" t="n">
         <v>0.09</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Terminal growth</t>
         </is>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="16" t="n">
         <v>0.015</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="16" t="n">
         <v>0.0225</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="16" t="n">
         <v>0.03</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>5-year forecast paths (by scenario)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 1</t>
         </is>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="27">
         <f>11102600*(1+C4)</f>
         <v/>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="27">
         <f>11102600*(1+D4)</f>
         <v/>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="27">
         <f>11102600*(1+E4)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="inlineStr">
+      <c r="A13" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 2</t>
         </is>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="27">
         <f>C12*(1+C5)</f>
         <v/>
       </c>
-      <c r="D13" s="26">
+      <c r="D13" s="27">
         <f>D12*(1+D5)</f>
         <v/>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="27">
         <f>E12*(1+E5)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 3</t>
         </is>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="27">
         <f>C13*(1+C5)</f>
         <v/>
       </c>
-      <c r="D14" s="26">
+      <c r="D14" s="27">
         <f>D13*(1+D5)</f>
         <v/>
       </c>
-      <c r="E14" s="26">
+      <c r="E14" s="27">
         <f>E13*(1+E5)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 4</t>
         </is>
       </c>
-      <c r="C15" s="26">
+      <c r="C15" s="27">
         <f>C14*(1+C5)</f>
         <v/>
       </c>
-      <c r="D15" s="26">
+      <c r="D15" s="27">
         <f>D14*(1+D5)</f>
         <v/>
       </c>
-      <c r="E15" s="26">
+      <c r="E15" s="27">
         <f>E14*(1+E5)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 5</t>
         </is>
       </c>
-      <c r="C16" s="26">
+      <c r="C16" s="27">
         <f>C15*(1+C5)</f>
         <v/>
       </c>
-      <c r="D16" s="26">
+      <c r="D16" s="27">
         <f>D15*(1+D5)</f>
         <v/>
       </c>
-      <c r="E16" s="26">
+      <c r="E16" s="27">
         <f>E15*(1+E5)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="inlineStr">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT margin – year 1</t>
         </is>
       </c>
-      <c r="C17" s="27">
+      <c r="C17" s="28">
         <f>C6+(C7-C6)*0/4</f>
         <v/>
       </c>
-      <c r="D17" s="27">
+      <c r="D17" s="28">
         <f>D6+(D7-D6)*0/4</f>
         <v/>
       </c>
-      <c r="E17" s="27">
+      <c r="E17" s="28">
         <f>E6+(E7-E6)*0/4</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="inlineStr">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT margin – year 2</t>
         </is>
       </c>
-      <c r="C18" s="27">
+      <c r="C18" s="28">
         <f>C6+(C7-C6)*1/4</f>
         <v/>
       </c>
-      <c r="D18" s="27">
+      <c r="D18" s="28">
         <f>D6+(D7-D6)*1/4</f>
         <v/>
       </c>
-      <c r="E18" s="27">
+      <c r="E18" s="28">
         <f>E6+(E7-E6)*1/4</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT margin – year 3</t>
         </is>
       </c>
-      <c r="C19" s="27">
+      <c r="C19" s="28">
         <f>C6+(C7-C6)*2/4</f>
         <v/>
       </c>
-      <c r="D19" s="27">
+      <c r="D19" s="28">
         <f>D6+(D7-D6)*2/4</f>
         <v/>
       </c>
-      <c r="E19" s="27">
+      <c r="E19" s="28">
         <f>E6+(E7-E6)*2/4</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="inlineStr">
+      <c r="A20" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT margin – year 4</t>
         </is>
       </c>
-      <c r="C20" s="27">
+      <c r="C20" s="28">
         <f>C6+(C7-C6)*3/4</f>
         <v/>
       </c>
-      <c r="D20" s="27">
+      <c r="D20" s="28">
         <f>D6+(D7-D6)*3/4</f>
         <v/>
       </c>
-      <c r="E20" s="27">
+      <c r="E20" s="28">
         <f>E6+(E7-E6)*3/4</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT margin – year 5</t>
         </is>
       </c>
-      <c r="C21" s="27">
+      <c r="C21" s="28">
         <f>C6+(C7-C6)*4/4</f>
         <v/>
       </c>
-      <c r="D21" s="27">
+      <c r="D21" s="28">
         <f>D6+(D7-D6)*4/4</f>
         <v/>
       </c>
-      <c r="E21" s="27">
+      <c r="E21" s="28">
         <f>E6+(E7-E6)*4/4</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 1</t>
         </is>
       </c>
-      <c r="C22" s="26">
+      <c r="C22" s="27">
         <f>(C12*C17)*(1-0.27)+C12*0.045-C12*0.05-0.075*(C12-11102600)</f>
         <v/>
       </c>
-      <c r="D22" s="26">
+      <c r="D22" s="27">
         <f>(D12*D17)*(1-0.27)+D12*0.045-D12*0.05-0.075*(D12-11102600)</f>
         <v/>
       </c>
-      <c r="E22" s="26">
+      <c r="E22" s="27">
         <f>(E12*E17)*(1-0.27)+E12*0.045-E12*0.05-0.075*(E12-11102600)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 2</t>
         </is>
       </c>
-      <c r="C23" s="26">
+      <c r="C23" s="27">
         <f>(C13*C18)*(1-0.27)+C13*0.045-C13*0.05-0.075*(C13-C12)</f>
         <v/>
       </c>
-      <c r="D23" s="26">
+      <c r="D23" s="27">
         <f>(D13*D18)*(1-0.27)+D13*0.045-D13*0.05-0.075*(D13-D12)</f>
         <v/>
       </c>
-      <c r="E23" s="26">
+      <c r="E23" s="27">
         <f>(E13*E18)*(1-0.27)+E13*0.045-E13*0.05-0.075*(E13-E12)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="25" t="inlineStr">
+      <c r="A24" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 3</t>
         </is>
       </c>
-      <c r="C24" s="26">
+      <c r="C24" s="27">
         <f>(C14*C19)*(1-0.27)+C14*0.045-C14*0.05-0.075*(C14-C13)</f>
         <v/>
       </c>
-      <c r="D24" s="26">
+      <c r="D24" s="27">
         <f>(D14*D19)*(1-0.27)+D14*0.045-D14*0.05-0.075*(D14-D13)</f>
         <v/>
       </c>
-      <c r="E24" s="26">
+      <c r="E24" s="27">
         <f>(E14*E19)*(1-0.27)+E14*0.045-E14*0.05-0.075*(E14-E13)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="25" t="inlineStr">
+      <c r="A25" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 4</t>
         </is>
       </c>
-      <c r="C25" s="26">
+      <c r="C25" s="27">
         <f>(C15*C20)*(1-0.27)+C15*0.045-C15*0.05-0.075*(C15-C14)</f>
         <v/>
       </c>
-      <c r="D25" s="26">
+      <c r="D25" s="27">
         <f>(D15*D20)*(1-0.27)+D15*0.045-D15*0.05-0.075*(D15-D14)</f>
         <v/>
       </c>
-      <c r="E25" s="26">
+      <c r="E25" s="27">
         <f>(E15*E20)*(1-0.27)+E15*0.045-E15*0.05-0.075*(E15-E14)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="25" t="inlineStr">
+      <c r="A26" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 5</t>
         </is>
       </c>
-      <c r="C26" s="26">
+      <c r="C26" s="27">
         <f>(C16*C21)*(1-0.27)+C16*0.045-C16*0.05-0.075*(C16-C15)</f>
         <v/>
       </c>
-      <c r="D26" s="26">
+      <c r="D26" s="27">
         <f>(D16*D21)*(1-0.27)+D16*0.045-D16*0.05-0.075*(D16-D15)</f>
         <v/>
       </c>
-      <c r="E26" s="26">
+      <c r="E26" s="27">
         <f>(E16*E21)*(1-0.27)+E16*0.045-E16*0.05-0.075*(E16-E15)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="inlineStr">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>Enterprise value (DCF)</t>
         </is>
       </c>
-      <c r="C28" s="28">
+      <c r="C28" s="29">
         <f>NPV(C8,C22,C23,C24,C25,C26)+(C26*(1+C9)/(C8-C9))/(1+C8)^5</f>
         <v/>
       </c>
-      <c r="D28" s="28">
+      <c r="D28" s="29">
         <f>NPV(D8,D22,D23,D24,D25,D26)+(D26*(1+D9)/(D8-D9))/(1+D8)^5</f>
         <v/>
       </c>
-      <c r="E28" s="28">
+      <c r="E28" s="29">
         <f>NPV(E8,E22,E23,E24,E25,E26)+(E26*(1+E9)/(E8-E9))/(1+E8)^5</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="29" t="inlineStr">
+      <c r="A29" s="30" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="C29" s="30">
+      <c r="C29" s="31">
         <f>(C28+1807202-0)/111380</f>
         <v/>
       </c>
-      <c r="D29" s="31">
+      <c r="D29" s="32">
         <f>(D28+1807202-0)/111380</f>
         <v/>
       </c>
-      <c r="E29" s="30">
+      <c r="E29" s="31">
         <f>(E28+1807202-0)/111380</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="inlineStr">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>Upside / (downside) vs current</t>
         </is>
       </c>
-      <c r="C30" s="32">
+      <c r="C30" s="33">
         <f>C29/100.0-1</f>
         <v/>
       </c>
-      <c r="D30" s="32">
+      <c r="D30" s="33">
         <f>D29/100.0-1</f>
         <v/>
       </c>
-      <c r="E30" s="32">
+      <c r="E30" s="33">
         <f>E29/100.0-1</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Current price $100.00; cash $1,807,202 k; net debt $0 (net-cash balance sheet).</t>
         </is>
@@ -1647,7 +1707,7 @@
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="2" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
@@ -1655,1001 +1715,1039 @@
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>DISCOUNTED CASH FLOW — BASE CASE  (US$ thousands)</t>
         </is>
       </c>
-      <c r="B1" s="12" t="n"/>
-      <c r="C1" s="12" t="n"/>
-      <c r="D1" s="12" t="n"/>
-      <c r="E1" s="12" t="n"/>
-      <c r="F1" s="12" t="n"/>
-      <c r="G1" s="12" t="n"/>
-      <c r="H1" s="12" t="n"/>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="13" t="n"/>
+      <c r="H1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="C2" s="33" t="inlineStr">
+      <c r="C2" s="34" t="inlineStr">
         <is>
           <t>FY2025A</t>
         </is>
       </c>
-      <c r="D2" s="34" t="inlineStr">
+      <c r="D2" s="35" t="inlineStr">
         <is>
           <t>FY2026E</t>
         </is>
       </c>
-      <c r="E2" s="34" t="inlineStr">
+      <c r="E2" s="35" t="inlineStr">
         <is>
           <t>FY2027E</t>
         </is>
       </c>
-      <c r="F2" s="34" t="inlineStr">
+      <c r="F2" s="35" t="inlineStr">
         <is>
           <t>FY2028E</t>
         </is>
       </c>
-      <c r="G2" s="34" t="inlineStr">
+      <c r="G2" s="35" t="inlineStr">
         <is>
           <t>FY2029E</t>
         </is>
       </c>
-      <c r="H2" s="34" t="inlineStr">
+      <c r="H2" s="35" t="inlineStr">
         <is>
           <t>FY2030E</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="35" t="inlineStr">
+      <c r="A3" s="36" t="inlineStr">
         <is>
           <t>Forecast drivers linked to Scenarios tab → Base case (column D)</t>
         </is>
       </c>
+      <c r="C3" s="37" t="inlineStr">
+        <is>
+          <t>10-K source</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Net revenue</t>
         </is>
       </c>
-      <c r="C5" s="36" t="n">
+      <c r="C5" s="38" t="n">
         <v>11102600</v>
       </c>
-      <c r="D5" s="37">
+      <c r="D5" s="39">
         <f>Scenarios!D12</f>
         <v/>
       </c>
-      <c r="E5" s="37">
+      <c r="E5" s="39">
         <f>Scenarios!D13</f>
         <v/>
       </c>
-      <c r="F5" s="37">
+      <c r="F5" s="39">
         <f>Scenarios!D14</f>
         <v/>
       </c>
-      <c r="G5" s="37">
+      <c r="G5" s="39">
         <f>Scenarios!D15</f>
         <v/>
       </c>
-      <c r="H5" s="37">
+      <c r="H5" s="39">
         <f>Scenarios!D16</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Revenue growth %</t>
         </is>
       </c>
-      <c r="D6" s="38">
+      <c r="D6" s="40">
         <f>D5/C5-1</f>
         <v/>
       </c>
-      <c r="E6" s="38">
+      <c r="E6" s="40">
         <f>E5/D5-1</f>
         <v/>
       </c>
-      <c r="F6" s="38">
+      <c r="F6" s="40">
         <f>F5/E5-1</f>
         <v/>
       </c>
-      <c r="G6" s="38">
+      <c r="G6" s="40">
         <f>G5/F5-1</f>
         <v/>
       </c>
-      <c r="H6" s="38">
+      <c r="H6" s="40">
         <f>H5/G5-1</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>EBIT (operating) margin %</t>
         </is>
       </c>
-      <c r="D7" s="38">
+      <c r="D7" s="40">
         <f>Scenarios!D17</f>
         <v/>
       </c>
-      <c r="E7" s="38">
+      <c r="E7" s="40">
         <f>Scenarios!D18</f>
         <v/>
       </c>
-      <c r="F7" s="38">
+      <c r="F7" s="40">
         <f>Scenarios!D19</f>
         <v/>
       </c>
-      <c r="G7" s="38">
+      <c r="G7" s="40">
         <f>Scenarios!D20</f>
         <v/>
       </c>
-      <c r="H7" s="38">
+      <c r="H7" s="40">
         <f>Scenarios!D21</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>EBIT</t>
         </is>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="C8" s="41" t="n">
         <v>2210615</v>
       </c>
-      <c r="D8" s="28">
+      <c r="D8" s="29">
         <f>D5*D7</f>
         <v/>
       </c>
-      <c r="E8" s="28">
+      <c r="E8" s="29">
         <f>E5*E7</f>
         <v/>
       </c>
-      <c r="F8" s="28">
+      <c r="F8" s="29">
         <f>F5*F7</f>
         <v/>
       </c>
-      <c r="G8" s="28">
+      <c r="G8" s="29">
         <f>G5*G7</f>
         <v/>
       </c>
-      <c r="H8" s="28">
+      <c r="H8" s="29">
         <f>H5*H7</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Less: cash taxes on EBIT</t>
         </is>
       </c>
-      <c r="D9" s="37">
+      <c r="D9" s="39">
         <f>-D8*WACC!C10</f>
         <v/>
       </c>
-      <c r="E9" s="37">
+      <c r="E9" s="39">
         <f>-E8*WACC!C10</f>
         <v/>
       </c>
-      <c r="F9" s="37">
+      <c r="F9" s="39">
         <f>-F8*WACC!C10</f>
         <v/>
       </c>
-      <c r="G9" s="37">
+      <c r="G9" s="39">
         <f>-G8*WACC!C10</f>
         <v/>
       </c>
-      <c r="H9" s="37">
+      <c r="H9" s="39">
         <f>-H8*WACC!C10</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>NOPAT</t>
         </is>
       </c>
-      <c r="D10" s="28">
+      <c r="D10" s="29">
         <f>D8+D9</f>
         <v/>
       </c>
-      <c r="E10" s="28">
+      <c r="E10" s="29">
         <f>E8+E9</f>
         <v/>
       </c>
-      <c r="F10" s="28">
+      <c r="F10" s="29">
         <f>F8+F9</f>
         <v/>
       </c>
-      <c r="G10" s="28">
+      <c r="G10" s="29">
         <f>G8+G9</f>
         <v/>
       </c>
-      <c r="H10" s="28">
+      <c r="H10" s="29">
         <f>H8+H9</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A % of revenue</t>
         </is>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="16" t="n">
         <v>0.045</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="16" t="n">
         <v>0.045</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="F11" s="16" t="n">
         <v>0.045</v>
       </c>
-      <c r="G11" s="15" t="n">
+      <c r="G11" s="16" t="n">
         <v>0.045</v>
       </c>
-      <c r="H11" s="15" t="n">
+      <c r="H11" s="16" t="n">
         <v>0.045</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Plus: depreciation &amp; amortization</t>
         </is>
       </c>
-      <c r="D12" s="37">
+      <c r="D12" s="39">
         <f>D5*D11</f>
         <v/>
       </c>
-      <c r="E12" s="37">
+      <c r="E12" s="39">
         <f>E5*E11</f>
         <v/>
       </c>
-      <c r="F12" s="37">
+      <c r="F12" s="39">
         <f>F5*F11</f>
         <v/>
       </c>
-      <c r="G12" s="37">
+      <c r="G12" s="39">
         <f>G5*G11</f>
         <v/>
       </c>
-      <c r="H12" s="37">
+      <c r="H12" s="39">
         <f>H5*H11</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex % of revenue</t>
         </is>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="16" t="n">
         <v>0.05</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="16" t="n">
         <v>0.05</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="F13" s="16" t="n">
         <v>0.05</v>
       </c>
-      <c r="G13" s="15" t="n">
+      <c r="G13" s="16" t="n">
         <v>0.05</v>
       </c>
-      <c r="H13" s="15" t="n">
+      <c r="H13" s="16" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Less: capital expenditures</t>
         </is>
       </c>
-      <c r="D14" s="37">
+      <c r="D14" s="39">
         <f>-D5*D13</f>
         <v/>
       </c>
-      <c r="E14" s="37">
+      <c r="E14" s="39">
         <f>-E5*E13</f>
         <v/>
       </c>
-      <c r="F14" s="37">
+      <c r="F14" s="39">
         <f>-F5*F13</f>
         <v/>
       </c>
-      <c r="G14" s="37">
+      <c r="G14" s="39">
         <f>-G5*G13</f>
         <v/>
       </c>
-      <c r="H14" s="37">
+      <c r="H14" s="39">
         <f>-H5*H13</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC % of revenue</t>
         </is>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="D15" s="16" t="n">
         <v>0.075</v>
       </c>
-      <c r="E15" s="15" t="n">
+      <c r="E15" s="16" t="n">
         <v>0.075</v>
       </c>
-      <c r="F15" s="15" t="n">
+      <c r="F15" s="16" t="n">
         <v>0.075</v>
       </c>
-      <c r="G15" s="15" t="n">
+      <c r="G15" s="16" t="n">
         <v>0.075</v>
       </c>
-      <c r="H15" s="15" t="n">
+      <c r="H15" s="16" t="n">
         <v>0.075</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Less: increase in net working capital</t>
         </is>
       </c>
-      <c r="D16" s="37">
+      <c r="D16" s="39">
         <f>-D15*(D5-C5)</f>
         <v/>
       </c>
-      <c r="E16" s="37">
+      <c r="E16" s="39">
         <f>-E15*(E5-D5)</f>
         <v/>
       </c>
-      <c r="F16" s="37">
+      <c r="F16" s="39">
         <f>-F15*(F5-E5)</f>
         <v/>
       </c>
-      <c r="G16" s="37">
+      <c r="G16" s="39">
         <f>-G15*(G5-F5)</f>
         <v/>
       </c>
-      <c r="H16" s="37">
+      <c r="H16" s="39">
         <f>-H15*(H5-G5)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Unlevered free cash flow</t>
         </is>
       </c>
-      <c r="D17" s="40">
+      <c r="D17" s="42">
         <f>D10+D12+D14+D16</f>
         <v/>
       </c>
-      <c r="E17" s="40">
+      <c r="E17" s="42">
         <f>E10+E12+E14+E16</f>
         <v/>
       </c>
-      <c r="F17" s="40">
+      <c r="F17" s="42">
         <f>F10+F12+F14+F16</f>
         <v/>
       </c>
-      <c r="G17" s="40">
+      <c r="G17" s="42">
         <f>G10+G12+G14+G16</f>
         <v/>
       </c>
-      <c r="H17" s="40">
+      <c r="H17" s="42">
         <f>H10+H12+H14+H16</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>Discount period (years)</t>
         </is>
       </c>
-      <c r="D18" s="41" t="n">
+      <c r="D18" s="43" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="41" t="n">
+      <c r="E18" s="43" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="41" t="n">
+      <c r="F18" s="43" t="n">
         <v>3</v>
       </c>
-      <c r="G18" s="41" t="n">
+      <c r="G18" s="43" t="n">
         <v>4</v>
       </c>
-      <c r="H18" s="41" t="n">
+      <c r="H18" s="43" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Discount factor @ WACC</t>
         </is>
       </c>
-      <c r="D19" s="42">
+      <c r="D19" s="44">
         <f>1/(1+Scenarios!$D$8)^D18</f>
         <v/>
       </c>
-      <c r="E19" s="42">
+      <c r="E19" s="44">
         <f>1/(1+Scenarios!$D$8)^E18</f>
         <v/>
       </c>
-      <c r="F19" s="42">
+      <c r="F19" s="44">
         <f>1/(1+Scenarios!$D$8)^F18</f>
         <v/>
       </c>
-      <c r="G19" s="42">
+      <c r="G19" s="44">
         <f>1/(1+Scenarios!$D$8)^G18</f>
         <v/>
       </c>
-      <c r="H19" s="42">
+      <c r="H19" s="44">
         <f>1/(1+Scenarios!$D$8)^H18</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>PV of unlevered FCF</t>
         </is>
       </c>
-      <c r="D20" s="28">
+      <c r="D20" s="29">
         <f>D17*D19</f>
         <v/>
       </c>
-      <c r="E20" s="28">
+      <c r="E20" s="29">
         <f>E17*E19</f>
         <v/>
       </c>
-      <c r="F20" s="28">
+      <c r="F20" s="29">
         <f>F17*F19</f>
         <v/>
       </c>
-      <c r="G20" s="28">
+      <c r="G20" s="29">
         <f>G17*G19</f>
         <v/>
       </c>
-      <c r="H20" s="28">
+      <c r="H20" s="29">
         <f>H17*H19</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="43" t="inlineStr">
+      <c r="A22" s="45" t="inlineStr">
         <is>
           <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
         </is>
       </c>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Sum of PV of explicit FCF (FY26–FY30)</t>
         </is>
       </c>
-      <c r="C23" s="44">
+      <c r="C23" s="46">
         <f>SUM(D20:H20)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Terminal growth rate (g)</t>
         </is>
       </c>
-      <c r="C24" s="38">
+      <c r="C24" s="40">
         <f>Scenarios!$D$9</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="18" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="C25" s="28">
+      <c r="C25" s="29">
         <f>H8+H12</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
         </is>
       </c>
-      <c r="C26" s="37">
+      <c r="C26" s="39">
         <f>H17*(1+Scenarios!$D$9)/(Scenarios!$D$8-Scenarios!$D$9)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Implied exit EV/EBITDA (Gordon Growth)</t>
         </is>
       </c>
-      <c r="C27" s="45">
+      <c r="C27" s="47">
         <f>C26/C25</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="inlineStr">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="C28" s="44">
+      <c r="C28" s="46">
         <f>C26/(1+Scenarios!$D$8)^H18</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="18" t="inlineStr">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="C29" s="28">
+      <c r="C29" s="29">
         <f>C23+C28</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>Plus: cash &amp; equivalents (FY2025)</t>
         </is>
       </c>
-      <c r="C30" s="36" t="n">
+      <c r="C30" s="38" t="n">
         <v>1807202</v>
       </c>
+      <c r="D30" s="48" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Less: total debt</t>
         </is>
       </c>
-      <c r="C31" s="36" t="n">
+      <c r="C31" s="38" t="n">
         <v>0</v>
       </c>
+      <c r="D31" s="48" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="18" t="inlineStr">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
       </c>
-      <c r="C32" s="28">
+      <c r="C32" s="29">
         <f>C29+C30+C31</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>Diluted shares outstanding (000)</t>
         </is>
       </c>
-      <c r="C33" s="36" t="n">
+      <c r="C33" s="38" t="n">
         <v>111380</v>
       </c>
+      <c r="D33" s="48" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>Implied value per share</t>
         </is>
       </c>
-      <c r="C34" s="46">
+      <c r="C34" s="49">
         <f>C32/C33</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="inlineStr">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C35" s="47" t="n">
+      <c r="C35" s="50" t="n">
         <v>100</v>
       </c>
+      <c r="D35" s="48" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>Implied upside / (downside)</t>
         </is>
       </c>
-      <c r="C36" s="48">
+      <c r="C36" s="51">
         <f>C34/C35-1</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="14" t="inlineStr">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: % of EV from terminal value</t>
         </is>
       </c>
-      <c r="C37" s="38">
+      <c r="C37" s="40">
         <f>C28/C29</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="43" t="inlineStr">
+      <c r="A39" s="45" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
       </c>
-      <c r="B39" s="12" t="n"/>
-      <c r="C39" s="12" t="n"/>
+      <c r="B39" s="13" t="n"/>
+      <c r="C39" s="13" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="49" t="inlineStr">
+      <c r="A40" s="52" t="inlineStr">
         <is>
           <t>Exit multiple selection (see Comps tab for peer build)</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="14" t="inlineStr">
+      <c r="A41" s="15" t="inlineStr">
         <is>
           <t>Selected exit EV/EBITDA multiple (FY2030E)</t>
         </is>
       </c>
-      <c r="C41" s="50" t="n">
+      <c r="C41" s="53" t="n">
         <v>8</v>
       </c>
-      <c r="D41" s="16" t="inlineStr">
+      <c r="D41" s="17" t="inlineStr">
         <is>
           <t>Base-case terminal multiple; see Comps → Exit Multiple Build</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="14" t="inlineStr">
+      <c r="A42" s="15" t="inlineStr">
         <is>
           <t>Terminal value = Terminal EBITDA × exit multiple</t>
         </is>
       </c>
-      <c r="C42" s="37">
+      <c r="C42" s="39">
         <f>C25*C41</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="14" t="inlineStr">
+      <c r="A43" s="15" t="inlineStr">
         <is>
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="C43" s="37">
+      <c r="C43" s="39">
         <f>C42/(1+Scenarios!$D$8)^H18</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="18" t="inlineStr">
+      <c r="A44" s="19" t="inlineStr">
         <is>
           <t>Enterprise value (exit method)</t>
         </is>
       </c>
-      <c r="C44" s="28">
+      <c r="C44" s="29">
         <f>C23+C43</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="18" t="inlineStr">
+      <c r="A45" s="19" t="inlineStr">
         <is>
           <t>Implied value per share (exit method)</t>
         </is>
       </c>
-      <c r="C45" s="51">
+      <c r="C45" s="54">
         <f>(C44+C30+C31)/C33</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="43" t="inlineStr">
+      <c r="A47" s="45" t="inlineStr">
         <is>
           <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
         </is>
       </c>
-      <c r="B47" s="12" t="n"/>
-      <c r="C47" s="12" t="n"/>
-      <c r="D47" s="12" t="n"/>
+      <c r="B47" s="13" t="n"/>
+      <c r="C47" s="13" t="n"/>
+      <c r="D47" s="13" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="52" t="inlineStr"/>
-      <c r="B48" s="53" t="inlineStr">
+      <c r="A48" s="55" t="inlineStr"/>
+      <c r="B48" s="56" t="inlineStr">
         <is>
           <t>Gordon Growth</t>
         </is>
       </c>
-      <c r="C48" s="53" t="inlineStr">
+      <c r="C48" s="56" t="inlineStr">
         <is>
           <t>Exit Multiple</t>
         </is>
       </c>
-      <c r="D48" s="53" t="inlineStr">
+      <c r="D48" s="56" t="inlineStr">
         <is>
           <t>Variance</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="18" t="inlineStr">
+      <c r="A49" s="19" t="inlineStr">
         <is>
           <t>Terminal value ($)</t>
         </is>
       </c>
-      <c r="B49" s="44">
+      <c r="B49" s="46">
         <f>C26</f>
         <v/>
       </c>
-      <c r="C49" s="44">
+      <c r="C49" s="46">
         <f>C42</f>
         <v/>
       </c>
-      <c r="D49" s="44">
+      <c r="D49" s="46">
         <f>B49-C49</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="18" t="inlineStr">
+      <c r="A50" s="19" t="inlineStr">
         <is>
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
       </c>
-      <c r="B50" s="54">
+      <c r="B50" s="57">
         <f>C27</f>
         <v/>
       </c>
-      <c r="C50" s="54">
+      <c r="C50" s="57">
         <f>C41</f>
         <v/>
       </c>
-      <c r="D50" s="54">
+      <c r="D50" s="57">
         <f>B50-C50</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="14" t="inlineStr">
+      <c r="A51" s="15" t="inlineStr">
         <is>
           <t>Terminal value variance (%)</t>
         </is>
       </c>
-      <c r="B51" s="38" t="inlineStr"/>
-      <c r="C51" s="38" t="inlineStr"/>
-      <c r="D51" s="38">
+      <c r="B51" s="40" t="inlineStr"/>
+      <c r="C51" s="40" t="inlineStr"/>
+      <c r="D51" s="40">
         <f>(B49-C49)/B49</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="18" t="inlineStr">
+      <c r="A52" s="19" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="B52" s="55">
+      <c r="B52" s="58">
         <f>C34</f>
         <v/>
       </c>
-      <c r="C52" s="55">
+      <c r="C52" s="58">
         <f>C45</f>
         <v/>
       </c>
-      <c r="D52" s="55">
+      <c r="D52" s="58">
         <f>B52-C52</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="56" t="inlineStr">
+      <c r="A53" s="59" t="inlineStr">
         <is>
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B53" s="57">
+      <c r="B53" s="60">
         <f>IF(ABS(D50)&lt;=1.5,"PASS","REVIEW")</f>
         <v/>
       </c>
-      <c r="C53" s="58">
+      <c r="C53" s="61">
         <f>TEXT(D50,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
         <v/>
       </c>
-      <c r="D53" s="16" t="inlineStr">
+      <c r="D53" s="17" t="inlineStr">
         <is>
           <t>Gordon implied should bracket exit assumption</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="43" t="inlineStr">
+      <c r="A56" s="45" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
       </c>
-      <c r="B56" s="12" t="n"/>
-      <c r="C56" s="12" t="n"/>
-      <c r="D56" s="12" t="n"/>
-      <c r="E56" s="12" t="n"/>
-      <c r="F56" s="12" t="n"/>
-      <c r="G56" s="12" t="n"/>
-      <c r="H56" s="12" t="n"/>
+      <c r="B56" s="13" t="n"/>
+      <c r="C56" s="13" t="n"/>
+      <c r="D56" s="13" t="n"/>
+      <c r="E56" s="13" t="n"/>
+      <c r="F56" s="13" t="n"/>
+      <c r="G56" s="13" t="n"/>
+      <c r="H56" s="13" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="59" t="inlineStr">
+      <c r="A57" s="62" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
       </c>
-      <c r="D57" s="60" t="n">
+      <c r="D57" s="63" t="n">
         <v>0.015</v>
       </c>
-      <c r="E57" s="60" t="n">
+      <c r="E57" s="63" t="n">
         <v>0.02</v>
       </c>
-      <c r="F57" s="60" t="n">
+      <c r="F57" s="63" t="n">
         <v>0.0225</v>
       </c>
-      <c r="G57" s="60" t="n">
+      <c r="G57" s="63" t="n">
         <v>0.025</v>
       </c>
-      <c r="H57" s="60" t="n">
+      <c r="H57" s="63" t="n">
         <v>0.03</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="60" t="n">
+      <c r="A58" s="63" t="n">
         <v>0.09</v>
       </c>
-      <c r="D58" s="61">
+      <c r="D58" s="64">
         <f>(NPV(0.09,D17:H17)+(H17*(1+0.015)/(0.09-0.015))/(1+0.09)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="E58" s="61">
+      <c r="E58" s="64">
         <f>(NPV(0.09,D17:H17)+(H17*(1+0.02)/(0.09-0.02))/(1+0.09)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="F58" s="61">
+      <c r="F58" s="64">
         <f>(NPV(0.09,D17:H17)+(H17*(1+0.0225)/(0.09-0.0225))/(1+0.09)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="G58" s="61">
+      <c r="G58" s="64">
         <f>(NPV(0.09,D17:H17)+(H17*(1+0.025)/(0.09-0.025))/(1+0.09)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="H58" s="61">
+      <c r="H58" s="64">
         <f>(NPV(0.09,D17:H17)+(H17*(1+0.03)/(0.09-0.03))/(1+0.09)^5+C30+C31)/C33</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="60" t="n">
+      <c r="A59" s="63" t="n">
         <v>0.095</v>
       </c>
-      <c r="D59" s="61">
+      <c r="D59" s="64">
         <f>(NPV(0.095,D17:H17)+(H17*(1+0.015)/(0.095-0.015))/(1+0.095)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="E59" s="61">
+      <c r="E59" s="64">
         <f>(NPV(0.095,D17:H17)+(H17*(1+0.02)/(0.095-0.02))/(1+0.095)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="F59" s="61">
+      <c r="F59" s="64">
         <f>(NPV(0.095,D17:H17)+(H17*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="G59" s="61">
+      <c r="G59" s="64">
         <f>(NPV(0.095,D17:H17)+(H17*(1+0.025)/(0.095-0.025))/(1+0.095)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="H59" s="61">
+      <c r="H59" s="64">
         <f>(NPV(0.095,D17:H17)+(H17*(1+0.03)/(0.095-0.03))/(1+0.095)^5+C30+C31)/C33</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="60" t="n">
+      <c r="A60" s="63" t="n">
         <v>0.1</v>
       </c>
-      <c r="D60" s="61">
+      <c r="D60" s="64">
         <f>(NPV(0.1,D17:H17)+(H17*(1+0.015)/(0.1-0.015))/(1+0.1)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="E60" s="61">
+      <c r="E60" s="64">
         <f>(NPV(0.1,D17:H17)+(H17*(1+0.02)/(0.1-0.02))/(1+0.1)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="F60" s="62">
+      <c r="F60" s="65">
         <f>(NPV(0.1,D17:H17)+(H17*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="G60" s="61">
+      <c r="G60" s="64">
         <f>(NPV(0.1,D17:H17)+(H17*(1+0.025)/(0.1-0.025))/(1+0.1)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="H60" s="61">
+      <c r="H60" s="64">
         <f>(NPV(0.1,D17:H17)+(H17*(1+0.03)/(0.1-0.03))/(1+0.1)^5+C30+C31)/C33</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="60" t="n">
+      <c r="A61" s="63" t="n">
         <v>0.105</v>
       </c>
-      <c r="D61" s="61">
+      <c r="D61" s="64">
         <f>(NPV(0.105,D17:H17)+(H17*(1+0.015)/(0.105-0.015))/(1+0.105)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="E61" s="61">
+      <c r="E61" s="64">
         <f>(NPV(0.105,D17:H17)+(H17*(1+0.02)/(0.105-0.02))/(1+0.105)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="F61" s="61">
+      <c r="F61" s="64">
         <f>(NPV(0.105,D17:H17)+(H17*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="G61" s="61">
+      <c r="G61" s="64">
         <f>(NPV(0.105,D17:H17)+(H17*(1+0.025)/(0.105-0.025))/(1+0.105)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="H61" s="61">
+      <c r="H61" s="64">
         <f>(NPV(0.105,D17:H17)+(H17*(1+0.03)/(0.105-0.03))/(1+0.105)^5+C30+C31)/C33</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="60" t="n">
+      <c r="A62" s="63" t="n">
         <v>0.11</v>
       </c>
-      <c r="D62" s="61">
+      <c r="D62" s="64">
         <f>(NPV(0.11,D17:H17)+(H17*(1+0.015)/(0.11-0.015))/(1+0.11)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="E62" s="61">
+      <c r="E62" s="64">
         <f>(NPV(0.11,D17:H17)+(H17*(1+0.02)/(0.11-0.02))/(1+0.11)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="F62" s="61">
+      <c r="F62" s="64">
         <f>(NPV(0.11,D17:H17)+(H17*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="G62" s="61">
+      <c r="G62" s="64">
         <f>(NPV(0.11,D17:H17)+(H17*(1+0.025)/(0.11-0.025))/(1+0.11)^5+C30+C31)/C33</f>
         <v/>
       </c>
-      <c r="H62" s="61">
+      <c r="H62" s="64">
         <f>(NPV(0.11,D17:H17)+(H17*(1+0.03)/(0.11-0.03))/(1+0.11)^5+C30+C31)/C33</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId11"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2672,430 +2770,474 @@
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>RELATIVE VALUATION — IMPLIED PRICE RANGES (FOOTBALL FIELD)</t>
         </is>
       </c>
-      <c r="B1" s="12" t="n"/>
-      <c r="C1" s="12" t="n"/>
-      <c r="D1" s="12" t="n"/>
-      <c r="E1" s="12" t="n"/>
-      <c r="F1" s="12" t="n"/>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>LULU operating metrics (FY2025A / FY2026E)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>FY2025A revenue</t>
         </is>
       </c>
-      <c r="C4" s="36" t="n">
+      <c r="C4" s="38" t="n">
         <v>11102600</v>
       </c>
+      <c r="D4" s="48" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>FY2025A EBITDA (EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="C5" s="37">
+      <c r="C5" s="39">
         <f>2210615+496228</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>FY2026E diluted EPS (guidance midpoint)</t>
         </is>
       </c>
-      <c r="C6" s="47" t="n">
+      <c r="C6" s="50" t="n">
         <v>9.609999999999999</v>
       </c>
+      <c r="D6" s="48" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Cash &amp; equivalents</t>
         </is>
       </c>
-      <c r="C7" s="36" t="n">
+      <c r="C7" s="38" t="n">
         <v>1807202</v>
       </c>
+      <c r="D7" s="48" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Diluted shares (000)</t>
         </is>
       </c>
-      <c r="C8" s="36" t="n">
+      <c r="C8" s="38" t="n">
         <v>111380</v>
       </c>
+      <c r="D8" s="48" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C9" s="47" t="n">
+      <c r="C9" s="50" t="n">
         <v>100</v>
       </c>
+      <c r="D9" s="48" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="58" t="inlineStr">
+      <c r="A10" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current EV / EBITDA</t>
         </is>
       </c>
-      <c r="C10" s="63">
+      <c r="C10" s="66">
         <f>(C9*C8-C7)/C5</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="58" t="inlineStr">
+      <c r="A11" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current P / E (FY2026E)</t>
         </is>
       </c>
-      <c r="C11" s="63">
+      <c r="C11" s="66">
         <f>C9/C6</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>EXIT MULTIPLE BUILD — FY2030E TERMINAL YEAR</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="58" t="inlineStr">
+      <c r="A14" s="61" t="inlineStr">
         <is>
           <t>Peer / reference EV/EBITDA (forward / illustrative)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="64" t="inlineStr">
+      <c r="A15" s="67" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C15" s="65" t="inlineStr">
+      <c r="C15" s="68" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="D15" s="64" t="inlineStr">
+      <c r="D15" s="67" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>lululemon (LULU) — current</t>
         </is>
       </c>
-      <c r="C16" s="66">
+      <c r="C16" s="69">
         <f>(C9*C8-C7)/C5</f>
         <v/>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D16" s="17" t="inlineStr">
         <is>
           <t>Distressed trough; FY2025A EBITDA</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Nike (NKE)</t>
         </is>
       </c>
-      <c r="C17" s="67" t="n">
+      <c r="C17" s="70" t="n">
         <v>18</v>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>Mature global brand; lower growth</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>Deckers (DECK)</t>
         </is>
       </c>
-      <c r="C18" s="67" t="n">
+      <c r="C18" s="70" t="n">
         <v>15</v>
       </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>Premium footwear peer; HOKA/UGG</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>On Holding (ONON)</t>
         </is>
       </c>
-      <c r="C19" s="67" t="n">
+      <c r="C19" s="70" t="n">
         <v>25</v>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>High-growth athletic peer</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>adidas (ADS)</t>
         </is>
       </c>
-      <c r="C20" s="67" t="n">
+      <c r="C20" s="70" t="n">
         <v>12</v>
       </c>
-      <c r="D20" s="16" t="inlineStr">
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>Global incumbent; restructuring</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>V.F. Corp (VFC)</t>
         </is>
       </c>
-      <c r="C21" s="67" t="n">
+      <c r="C21" s="70" t="n">
         <v>10</v>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>Multi-brand apparel; challenged</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>Terminal multiple selection (DCF exit method)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Gordon Growth implied exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="C24" s="45">
+      <c r="C24" s="47">
         <f>DCF!C27</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="56" t="inlineStr">
+      <c r="A25" s="59" t="inlineStr">
         <is>
           <t>Selected exit multiple (base case)</t>
         </is>
       </c>
-      <c r="C25" s="54">
+      <c r="C25" s="57">
         <f>DCF!C41</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>Spread (selected − Gordon implied)</t>
         </is>
       </c>
-      <c r="C26" s="45">
+      <c r="C26" s="47">
         <f>C25-C24</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="56" t="inlineStr">
+      <c r="A27" s="59" t="inlineStr">
         <is>
           <t>Rationale for 8.0x</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="25" t="inlineStr">
+      <c r="A28" s="26" t="inlineStr">
         <is>
           <t>•  Above current LULU (~3.5x) — assumes partial recovery from trough, not full re-rating</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="25" t="inlineStr">
+      <c r="A29" s="26" t="inlineStr">
         <is>
           <t>•  Above comps football-field high (7.5x on FY2025A) — terminal year has higher EBITDA &amp; normalized margins</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="25" t="inlineStr">
+      <c r="A30" s="26" t="inlineStr">
         <is>
           <t>•  Below premium-growth peers (ONON ~25x, DECK ~15x) — reflects Americas maturity</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="25" t="inlineStr">
+      <c r="A31" s="26" t="inlineStr">
         <is>
           <t>•  ~1 turn above Gordon-implied exit multiple — conservative buffer vs perpetuity math</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="25" t="inlineStr">
+      <c r="A32" s="26" t="inlineStr">
         <is>
           <t>•  Well below historical LULU peak multiples (20–30x) — avoids heroic assumptions</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="14" t="inlineStr">
         <is>
           <t>Methodology / multiple ranges (FY2025A — football field)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="64" t="inlineStr">
+      <c r="A35" s="67" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="C35" s="65" t="inlineStr">
+      <c r="C35" s="68" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="D35" s="65" t="inlineStr">
+      <c r="D35" s="68" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="E35" s="65" t="inlineStr">
+      <c r="E35" s="68" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="F35" s="65" t="inlineStr">
+      <c r="F35" s="68" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="inlineStr">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>EV / EBITDA (FY2025A)</t>
         </is>
       </c>
-      <c r="C36" s="67" t="n">
+      <c r="C36" s="70" t="n">
         <v>4.5</v>
       </c>
-      <c r="D36" s="67" t="n">
+      <c r="D36" s="70" t="n">
         <v>7.5</v>
       </c>
-      <c r="E36" s="68">
+      <c r="E36" s="71">
         <f>(C5*C36+C7)/C8</f>
         <v/>
       </c>
-      <c r="F36" s="68">
+      <c r="F36" s="71">
         <f>(C5*D36+C7)/C8</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="14" t="inlineStr">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>P / E (FY2026E EPS)</t>
         </is>
       </c>
-      <c r="C37" s="67" t="n">
+      <c r="C37" s="70" t="n">
         <v>10</v>
       </c>
-      <c r="D37" s="67" t="n">
+      <c r="D37" s="70" t="n">
         <v>18</v>
       </c>
-      <c r="E37" s="68">
+      <c r="E37" s="71">
         <f>C6*C37</f>
         <v/>
       </c>
-      <c r="F37" s="68">
+      <c r="F37" s="71">
         <f>C6*D37</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="14" t="inlineStr">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="C38" s="69" t="inlineStr">
+      <c r="C38" s="72" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D38" s="69" t="inlineStr">
+      <c r="D38" s="72" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E38" s="68">
+      <c r="E38" s="71">
         <f>Scenarios!C29</f>
         <v/>
       </c>
-      <c r="F38" s="68">
+      <c r="F38" s="71">
         <f>Scenarios!E29</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="70" t="inlineStr">
+      <c r="A40" s="73" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C40" s="71" t="n">
+      <c r="C40" s="74" t="n">
         <v>100</v>
       </c>
+      <c r="D40" s="48" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>Note: peer set includes NKE, DECK, ONON, adidas, VFC; multiples are analyst ranges (red).</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId12"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Link all DCF forecast lines to Scenarios base case with reconciliation checks
- Expand Scenarios tab with full FCF build (EBIT, NOPAT, D&A, capex, ΔNWC)
- Add shared assumptions (tax, D&A%, capex%, NWC%) to Scenarios
- DCF forecast columns now reference Scenarios column D line-by-line
- Column I shows OK/CHECK variance vs Scenarios for each line item
- Summary row and implied price cross-check vs Scenarios base PT

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0x"/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="43">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -203,6 +203,23 @@
     <font>
       <name val="Garamond"/>
       <b val="1"/>
+      <color rgb="00C8102E"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <i val="1"/>
+      <color rgb="00F2F2F2"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <color rgb="00000000"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <b val="1"/>
       <color rgb="000000CC"/>
       <sz val="10"/>
       <u val="single"/>
@@ -210,6 +227,24 @@
     <font>
       <name val="Garamond"/>
       <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="00C8102E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <b val="1"/>
       <color rgb="00006100"/>
       <sz val="13"/>
     </font>
@@ -218,12 +253,6 @@
       <b val="1"/>
       <color rgb="00006100"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Garamond"/>
-      <b val="1"/>
-      <color rgb="00C8102E"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Garamond"/>
@@ -314,7 +343,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -395,23 +424,35 @@
     <xf numFmtId="0" fontId="27" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="29" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="32" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -421,6 +462,12 @@
     </xf>
     <xf numFmtId="167" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -432,26 +479,23 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="30" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="36" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="168" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -463,22 +507,22 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="39" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="35" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="40" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -505,7 +549,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1193,7 +1237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1334,357 +1378,896 @@
         <v>0.03</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Cash tax rate</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>D&amp;A % of revenue</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>Capex % of revenue</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>NWC build % of Δrevenue</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="E13" s="16" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>5-year forecast paths (by scenario)</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Revenue – year 1</t>
-        </is>
-      </c>
-      <c r="C12" s="27">
-        <f>11102600*(1+C4)</f>
-        <v/>
-      </c>
-      <c r="D12" s="27">
-        <f>11102600*(1+D4)</f>
-        <v/>
-      </c>
-      <c r="E12" s="27">
-        <f>11102600*(1+E4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Revenue – year 2</t>
-        </is>
-      </c>
-      <c r="C13" s="27">
-        <f>C12*(1+C5)</f>
-        <v/>
-      </c>
-      <c r="D13" s="27">
-        <f>D12*(1+D5)</f>
-        <v/>
-      </c>
-      <c r="E13" s="27">
-        <f>E12*(1+E5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Revenue – year 3</t>
-        </is>
-      </c>
-      <c r="C14" s="27">
-        <f>C13*(1+C5)</f>
-        <v/>
-      </c>
-      <c r="D14" s="27">
-        <f>D13*(1+D5)</f>
-        <v/>
-      </c>
-      <c r="E14" s="27">
-        <f>E13*(1+E5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Revenue – year 4</t>
-        </is>
-      </c>
-      <c r="C15" s="27">
-        <f>C14*(1+C5)</f>
-        <v/>
-      </c>
-      <c r="D15" s="27">
-        <f>D14*(1+D5)</f>
-        <v/>
-      </c>
-      <c r="E15" s="27">
-        <f>E14*(1+E5)</f>
-        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Revenue – year 5</t>
+          <t xml:space="preserve">  Revenue – year 1</t>
         </is>
       </c>
       <c r="C16" s="27">
-        <f>C15*(1+C5)</f>
+        <f>11102600*(1+C4)</f>
         <v/>
       </c>
       <c r="D16" s="27">
-        <f>D15*(1+D5)</f>
+        <f>11102600*(1+D4)</f>
         <v/>
       </c>
       <c r="E16" s="27">
-        <f>E15*(1+E5)</f>
+        <f>11102600*(1+E4)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT margin – year 1</t>
-        </is>
-      </c>
-      <c r="C17" s="28">
-        <f>C6+(C7-C6)*0/4</f>
-        <v/>
-      </c>
-      <c r="D17" s="28">
-        <f>D6+(D7-D6)*0/4</f>
-        <v/>
-      </c>
-      <c r="E17" s="28">
-        <f>E6+(E7-E6)*0/4</f>
+          <t xml:space="preserve">  Revenue – year 2</t>
+        </is>
+      </c>
+      <c r="C17" s="27">
+        <f>C16*(1+C5)</f>
+        <v/>
+      </c>
+      <c r="D17" s="27">
+        <f>D16*(1+D5)</f>
+        <v/>
+      </c>
+      <c r="E17" s="27">
+        <f>E16*(1+E5)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT margin – year 2</t>
-        </is>
-      </c>
-      <c r="C18" s="28">
-        <f>C6+(C7-C6)*1/4</f>
-        <v/>
-      </c>
-      <c r="D18" s="28">
-        <f>D6+(D7-D6)*1/4</f>
-        <v/>
-      </c>
-      <c r="E18" s="28">
-        <f>E6+(E7-E6)*1/4</f>
+          <t xml:space="preserve">  Revenue – year 3</t>
+        </is>
+      </c>
+      <c r="C18" s="27">
+        <f>C17*(1+C5)</f>
+        <v/>
+      </c>
+      <c r="D18" s="27">
+        <f>D17*(1+D5)</f>
+        <v/>
+      </c>
+      <c r="E18" s="27">
+        <f>E17*(1+E5)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT margin – year 3</t>
-        </is>
-      </c>
-      <c r="C19" s="28">
-        <f>C6+(C7-C6)*2/4</f>
-        <v/>
-      </c>
-      <c r="D19" s="28">
-        <f>D6+(D7-D6)*2/4</f>
-        <v/>
-      </c>
-      <c r="E19" s="28">
-        <f>E6+(E7-E6)*2/4</f>
+          <t xml:space="preserve">  Revenue – year 4</t>
+        </is>
+      </c>
+      <c r="C19" s="27">
+        <f>C18*(1+C5)</f>
+        <v/>
+      </c>
+      <c r="D19" s="27">
+        <f>D18*(1+D5)</f>
+        <v/>
+      </c>
+      <c r="E19" s="27">
+        <f>E18*(1+E5)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT margin – year 4</t>
-        </is>
-      </c>
-      <c r="C20" s="28">
-        <f>C6+(C7-C6)*3/4</f>
-        <v/>
-      </c>
-      <c r="D20" s="28">
-        <f>D6+(D7-D6)*3/4</f>
-        <v/>
-      </c>
-      <c r="E20" s="28">
-        <f>E6+(E7-E6)*3/4</f>
+          <t xml:space="preserve">  Revenue – year 5</t>
+        </is>
+      </c>
+      <c r="C20" s="27">
+        <f>C19*(1+C5)</f>
+        <v/>
+      </c>
+      <c r="D20" s="27">
+        <f>D19*(1+D5)</f>
+        <v/>
+      </c>
+      <c r="E20" s="27">
+        <f>E19*(1+E5)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT margin – year 5</t>
+          <t xml:space="preserve">  EBIT margin – year 1</t>
         </is>
       </c>
       <c r="C21" s="28">
-        <f>C6+(C7-C6)*4/4</f>
+        <f>C6+(C7-C6)*0/4</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>D6+(D7-D6)*4/4</f>
+        <f>D6+(D7-D6)*0/4</f>
         <v/>
       </c>
       <c r="E21" s="28">
-        <f>E6+(E7-E6)*4/4</f>
+        <f>E6+(E7-E6)*0/4</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 1</t>
-        </is>
-      </c>
-      <c r="C22" s="27">
-        <f>(C12*C17)*(1-0.27)+C12*0.045-C12*0.05-0.075*(C12-11102600)</f>
-        <v/>
-      </c>
-      <c r="D22" s="27">
-        <f>(D12*D17)*(1-0.27)+D12*0.045-D12*0.05-0.075*(D12-11102600)</f>
-        <v/>
-      </c>
-      <c r="E22" s="27">
-        <f>(E12*E17)*(1-0.27)+E12*0.045-E12*0.05-0.075*(E12-11102600)</f>
+          <t xml:space="preserve">  EBIT margin – year 2</t>
+        </is>
+      </c>
+      <c r="C22" s="28">
+        <f>C6+(C7-C6)*1/4</f>
+        <v/>
+      </c>
+      <c r="D22" s="28">
+        <f>D6+(D7-D6)*1/4</f>
+        <v/>
+      </c>
+      <c r="E22" s="28">
+        <f>E6+(E7-E6)*1/4</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 2</t>
-        </is>
-      </c>
-      <c r="C23" s="27">
-        <f>(C13*C18)*(1-0.27)+C13*0.045-C13*0.05-0.075*(C13-C12)</f>
-        <v/>
-      </c>
-      <c r="D23" s="27">
-        <f>(D13*D18)*(1-0.27)+D13*0.045-D13*0.05-0.075*(D13-D12)</f>
-        <v/>
-      </c>
-      <c r="E23" s="27">
-        <f>(E13*E18)*(1-0.27)+E13*0.045-E13*0.05-0.075*(E13-E12)</f>
+          <t xml:space="preserve">  EBIT margin – year 3</t>
+        </is>
+      </c>
+      <c r="C23" s="28">
+        <f>C6+(C7-C6)*2/4</f>
+        <v/>
+      </c>
+      <c r="D23" s="28">
+        <f>D6+(D7-D6)*2/4</f>
+        <v/>
+      </c>
+      <c r="E23" s="28">
+        <f>E6+(E7-E6)*2/4</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 3</t>
-        </is>
-      </c>
-      <c r="C24" s="27">
-        <f>(C14*C19)*(1-0.27)+C14*0.045-C14*0.05-0.075*(C14-C13)</f>
-        <v/>
-      </c>
-      <c r="D24" s="27">
-        <f>(D14*D19)*(1-0.27)+D14*0.045-D14*0.05-0.075*(D14-D13)</f>
-        <v/>
-      </c>
-      <c r="E24" s="27">
-        <f>(E14*E19)*(1-0.27)+E14*0.045-E14*0.05-0.075*(E14-E13)</f>
+          <t xml:space="preserve">  EBIT margin – year 4</t>
+        </is>
+      </c>
+      <c r="C24" s="28">
+        <f>C6+(C7-C6)*3/4</f>
+        <v/>
+      </c>
+      <c r="D24" s="28">
+        <f>D6+(D7-D6)*3/4</f>
+        <v/>
+      </c>
+      <c r="E24" s="28">
+        <f>E6+(E7-E6)*3/4</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 4</t>
-        </is>
-      </c>
-      <c r="C25" s="27">
-        <f>(C15*C20)*(1-0.27)+C15*0.045-C15*0.05-0.075*(C15-C14)</f>
-        <v/>
-      </c>
-      <c r="D25" s="27">
-        <f>(D15*D20)*(1-0.27)+D15*0.045-D15*0.05-0.075*(D15-D14)</f>
-        <v/>
-      </c>
-      <c r="E25" s="27">
-        <f>(E15*E20)*(1-0.27)+E15*0.045-E15*0.05-0.075*(E15-E14)</f>
+          <t xml:space="preserve">  EBIT margin – year 5</t>
+        </is>
+      </c>
+      <c r="C25" s="28">
+        <f>C6+(C7-C6)*4/4</f>
+        <v/>
+      </c>
+      <c r="D25" s="28">
+        <f>D6+(D7-D6)*4/4</f>
+        <v/>
+      </c>
+      <c r="E25" s="28">
+        <f>E6+(E7-E6)*4/4</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="26" t="inlineStr">
         <is>
+          <t xml:space="preserve">  EBIT – year 1</t>
+        </is>
+      </c>
+      <c r="C26" s="27">
+        <f>C16*C21</f>
+        <v/>
+      </c>
+      <c r="D26" s="27">
+        <f>D16*D21</f>
+        <v/>
+      </c>
+      <c r="E26" s="27">
+        <f>E16*E21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EBIT – year 2</t>
+        </is>
+      </c>
+      <c r="C27" s="27">
+        <f>C17*C22</f>
+        <v/>
+      </c>
+      <c r="D27" s="27">
+        <f>D17*D22</f>
+        <v/>
+      </c>
+      <c r="E27" s="27">
+        <f>E17*E22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EBIT – year 3</t>
+        </is>
+      </c>
+      <c r="C28" s="27">
+        <f>C18*C23</f>
+        <v/>
+      </c>
+      <c r="D28" s="27">
+        <f>D18*D23</f>
+        <v/>
+      </c>
+      <c r="E28" s="27">
+        <f>E18*E23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EBIT – year 4</t>
+        </is>
+      </c>
+      <c r="C29" s="27">
+        <f>C19*C24</f>
+        <v/>
+      </c>
+      <c r="D29" s="27">
+        <f>D19*D24</f>
+        <v/>
+      </c>
+      <c r="E29" s="27">
+        <f>E19*E24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EBIT – year 5</t>
+        </is>
+      </c>
+      <c r="C30" s="27">
+        <f>C20*C25</f>
+        <v/>
+      </c>
+      <c r="D30" s="27">
+        <f>D20*D25</f>
+        <v/>
+      </c>
+      <c r="E30" s="27">
+        <f>E20*E25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOPAT – year 1</t>
+        </is>
+      </c>
+      <c r="C31" s="27">
+        <f>C26*(1-C10)</f>
+        <v/>
+      </c>
+      <c r="D31" s="27">
+        <f>D26*(1-D10)</f>
+        <v/>
+      </c>
+      <c r="E31" s="27">
+        <f>E26*(1-E10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOPAT – year 2</t>
+        </is>
+      </c>
+      <c r="C32" s="27">
+        <f>C27*(1-C10)</f>
+        <v/>
+      </c>
+      <c r="D32" s="27">
+        <f>D27*(1-D10)</f>
+        <v/>
+      </c>
+      <c r="E32" s="27">
+        <f>E27*(1-E10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOPAT – year 3</t>
+        </is>
+      </c>
+      <c r="C33" s="27">
+        <f>C28*(1-C10)</f>
+        <v/>
+      </c>
+      <c r="D33" s="27">
+        <f>D28*(1-D10)</f>
+        <v/>
+      </c>
+      <c r="E33" s="27">
+        <f>E28*(1-E10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOPAT – year 4</t>
+        </is>
+      </c>
+      <c r="C34" s="27">
+        <f>C29*(1-C10)</f>
+        <v/>
+      </c>
+      <c r="D34" s="27">
+        <f>D29*(1-D10)</f>
+        <v/>
+      </c>
+      <c r="E34" s="27">
+        <f>E29*(1-E10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOPAT – year 5</t>
+        </is>
+      </c>
+      <c r="C35" s="27">
+        <f>C30*(1-C10)</f>
+        <v/>
+      </c>
+      <c r="D35" s="27">
+        <f>D30*(1-D10)</f>
+        <v/>
+      </c>
+      <c r="E35" s="27">
+        <f>E30*(1-E10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D&amp;A – year 1</t>
+        </is>
+      </c>
+      <c r="C36" s="27">
+        <f>C16*C11</f>
+        <v/>
+      </c>
+      <c r="D36" s="27">
+        <f>D16*D11</f>
+        <v/>
+      </c>
+      <c r="E36" s="27">
+        <f>E16*E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D&amp;A – year 2</t>
+        </is>
+      </c>
+      <c r="C37" s="27">
+        <f>C17*C11</f>
+        <v/>
+      </c>
+      <c r="D37" s="27">
+        <f>D17*D11</f>
+        <v/>
+      </c>
+      <c r="E37" s="27">
+        <f>E17*E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D&amp;A – year 3</t>
+        </is>
+      </c>
+      <c r="C38" s="27">
+        <f>C18*C11</f>
+        <v/>
+      </c>
+      <c r="D38" s="27">
+        <f>D18*D11</f>
+        <v/>
+      </c>
+      <c r="E38" s="27">
+        <f>E18*E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D&amp;A – year 4</t>
+        </is>
+      </c>
+      <c r="C39" s="27">
+        <f>C19*C11</f>
+        <v/>
+      </c>
+      <c r="D39" s="27">
+        <f>D19*D11</f>
+        <v/>
+      </c>
+      <c r="E39" s="27">
+        <f>E19*E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D&amp;A – year 5</t>
+        </is>
+      </c>
+      <c r="C40" s="27">
+        <f>C20*C11</f>
+        <v/>
+      </c>
+      <c r="D40" s="27">
+        <f>D20*D11</f>
+        <v/>
+      </c>
+      <c r="E40" s="27">
+        <f>E20*E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Capex – year 1</t>
+        </is>
+      </c>
+      <c r="C41" s="27">
+        <f>C16*C12</f>
+        <v/>
+      </c>
+      <c r="D41" s="27">
+        <f>D16*D12</f>
+        <v/>
+      </c>
+      <c r="E41" s="27">
+        <f>E16*E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Capex – year 2</t>
+        </is>
+      </c>
+      <c r="C42" s="27">
+        <f>C17*C12</f>
+        <v/>
+      </c>
+      <c r="D42" s="27">
+        <f>D17*D12</f>
+        <v/>
+      </c>
+      <c r="E42" s="27">
+        <f>E17*E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Capex – year 3</t>
+        </is>
+      </c>
+      <c r="C43" s="27">
+        <f>C18*C12</f>
+        <v/>
+      </c>
+      <c r="D43" s="27">
+        <f>D18*D12</f>
+        <v/>
+      </c>
+      <c r="E43" s="27">
+        <f>E18*E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Capex – year 4</t>
+        </is>
+      </c>
+      <c r="C44" s="27">
+        <f>C19*C12</f>
+        <v/>
+      </c>
+      <c r="D44" s="27">
+        <f>D19*D12</f>
+        <v/>
+      </c>
+      <c r="E44" s="27">
+        <f>E19*E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Capex – year 5</t>
+        </is>
+      </c>
+      <c r="C45" s="27">
+        <f>C20*C12</f>
+        <v/>
+      </c>
+      <c r="D45" s="27">
+        <f>D20*D12</f>
+        <v/>
+      </c>
+      <c r="E45" s="27">
+        <f>E20*E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ΔNWC – year 1</t>
+        </is>
+      </c>
+      <c r="C46" s="27">
+        <f>C13*(C16-11102600)</f>
+        <v/>
+      </c>
+      <c r="D46" s="27">
+        <f>D13*(D16-11102600)</f>
+        <v/>
+      </c>
+      <c r="E46" s="27">
+        <f>E13*(E16-11102600)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ΔNWC – year 2</t>
+        </is>
+      </c>
+      <c r="C47" s="27">
+        <f>C13*(C17-C16)</f>
+        <v/>
+      </c>
+      <c r="D47" s="27">
+        <f>D13*(D17-D16)</f>
+        <v/>
+      </c>
+      <c r="E47" s="27">
+        <f>E13*(E17-E16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ΔNWC – year 3</t>
+        </is>
+      </c>
+      <c r="C48" s="27">
+        <f>C13*(C18-C17)</f>
+        <v/>
+      </c>
+      <c r="D48" s="27">
+        <f>D13*(D18-D17)</f>
+        <v/>
+      </c>
+      <c r="E48" s="27">
+        <f>E13*(E18-E17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ΔNWC – year 4</t>
+        </is>
+      </c>
+      <c r="C49" s="27">
+        <f>C13*(C19-C18)</f>
+        <v/>
+      </c>
+      <c r="D49" s="27">
+        <f>D13*(D19-D18)</f>
+        <v/>
+      </c>
+      <c r="E49" s="27">
+        <f>E13*(E19-E18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ΔNWC – year 5</t>
+        </is>
+      </c>
+      <c r="C50" s="27">
+        <f>C13*(C20-C19)</f>
+        <v/>
+      </c>
+      <c r="D50" s="27">
+        <f>D13*(D20-D19)</f>
+        <v/>
+      </c>
+      <c r="E50" s="27">
+        <f>E13*(E20-E19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Unlevered FCF – year 1</t>
+        </is>
+      </c>
+      <c r="C51" s="27">
+        <f>C31+C36-C41-C46</f>
+        <v/>
+      </c>
+      <c r="D51" s="27">
+        <f>D31+D36-D41-D46</f>
+        <v/>
+      </c>
+      <c r="E51" s="27">
+        <f>E31+E36-E41-E46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Unlevered FCF – year 2</t>
+        </is>
+      </c>
+      <c r="C52" s="27">
+        <f>C32+C37-C42-C47</f>
+        <v/>
+      </c>
+      <c r="D52" s="27">
+        <f>D32+D37-D42-D47</f>
+        <v/>
+      </c>
+      <c r="E52" s="27">
+        <f>E32+E37-E42-E47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Unlevered FCF – year 3</t>
+        </is>
+      </c>
+      <c r="C53" s="27">
+        <f>C33+C38-C43-C48</f>
+        <v/>
+      </c>
+      <c r="D53" s="27">
+        <f>D33+D38-D43-D48</f>
+        <v/>
+      </c>
+      <c r="E53" s="27">
+        <f>E33+E38-E43-E48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Unlevered FCF – year 4</t>
+        </is>
+      </c>
+      <c r="C54" s="27">
+        <f>C34+C39-C44-C49</f>
+        <v/>
+      </c>
+      <c r="D54" s="27">
+        <f>D34+D39-D44-D49</f>
+        <v/>
+      </c>
+      <c r="E54" s="27">
+        <f>E34+E39-E44-E49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="26" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Unlevered FCF – year 5</t>
         </is>
       </c>
-      <c r="C26" s="27">
-        <f>(C16*C21)*(1-0.27)+C16*0.045-C16*0.05-0.075*(C16-C15)</f>
-        <v/>
-      </c>
-      <c r="D26" s="27">
-        <f>(D16*D21)*(1-0.27)+D16*0.045-D16*0.05-0.075*(D16-D15)</f>
-        <v/>
-      </c>
-      <c r="E26" s="27">
-        <f>(E16*E21)*(1-0.27)+E16*0.045-E16*0.05-0.075*(E16-E15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="19" t="inlineStr">
+      <c r="C55" s="27">
+        <f>C35+C40-C45-C50</f>
+        <v/>
+      </c>
+      <c r="D55" s="27">
+        <f>D35+D40-D45-D50</f>
+        <v/>
+      </c>
+      <c r="E55" s="27">
+        <f>E35+E40-E45-E50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="19" t="inlineStr">
         <is>
           <t>Enterprise value (DCF)</t>
         </is>
       </c>
-      <c r="C28" s="29">
-        <f>NPV(C8,C22,C23,C24,C25,C26)+(C26*(1+C9)/(C8-C9))/(1+C8)^5</f>
-        <v/>
-      </c>
-      <c r="D28" s="29">
-        <f>NPV(D8,D22,D23,D24,D25,D26)+(D26*(1+D9)/(D8-D9))/(1+D8)^5</f>
-        <v/>
-      </c>
-      <c r="E28" s="29">
-        <f>NPV(E8,E22,E23,E24,E25,E26)+(E26*(1+E9)/(E8-E9))/(1+E8)^5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="30" t="inlineStr">
+      <c r="C57" s="29">
+        <f>NPV(C8,C51,C52,C53,C54,C55)+(C55*(1+C9)/(C8-C9))/(1+C8)^5</f>
+        <v/>
+      </c>
+      <c r="D57" s="29">
+        <f>NPV(D8,D51,D52,D53,D54,D55)+(D55*(1+D9)/(D8-D9))/(1+D8)^5</f>
+        <v/>
+      </c>
+      <c r="E57" s="29">
+        <f>NPV(E8,E51,E52,E53,E54,E55)+(E55*(1+E9)/(E8-E9))/(1+E8)^5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="30" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="C29" s="31">
-        <f>(C28+1807202-0)/111380</f>
-        <v/>
-      </c>
-      <c r="D29" s="32">
-        <f>(D28+1807202-0)/111380</f>
-        <v/>
-      </c>
-      <c r="E29" s="31">
-        <f>(E28+1807202-0)/111380</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="19" t="inlineStr">
+      <c r="C58" s="31">
+        <f>(C57+1807202-0)/111380</f>
+        <v/>
+      </c>
+      <c r="D58" s="32">
+        <f>(D57+1807202-0)/111380</f>
+        <v/>
+      </c>
+      <c r="E58" s="31">
+        <f>(E57+1807202-0)/111380</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="19" t="inlineStr">
         <is>
           <t>Upside / (downside) vs current</t>
         </is>
       </c>
-      <c r="C30" s="33">
-        <f>C29/100.0-1</f>
-        <v/>
-      </c>
-      <c r="D30" s="33">
-        <f>D29/100.0-1</f>
-        <v/>
-      </c>
-      <c r="E30" s="33">
-        <f>E29/100.0-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr">
+      <c r="C59" s="33">
+        <f>C58/100.0-1</f>
+        <v/>
+      </c>
+      <c r="D59" s="33">
+        <f>D58/100.0-1</f>
+        <v/>
+      </c>
+      <c r="E59" s="33">
+        <f>E58/100.0-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
         <is>
           <t>Current price $100.00; cash $1,807,202 k; net debt $0 (net-cash balance sheet).</t>
         </is>
@@ -1701,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1712,6 +2295,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -1759,16 +2343,26 @@
           <t>FY2030E</t>
         </is>
       </c>
+      <c r="I2" s="36" t="inlineStr">
+        <is>
+          <t>Δ vs Scenarios</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="36" t="inlineStr">
+      <c r="A3" s="37" t="inlineStr">
         <is>
           <t>Forecast drivers linked to Scenarios tab → Base case (column D)</t>
         </is>
       </c>
-      <c r="C3" s="37" t="inlineStr">
+      <c r="C3" s="38" t="inlineStr">
         <is>
           <t>10-K source</t>
+        </is>
+      </c>
+      <c r="I3" s="39" t="inlineStr">
+        <is>
+          <t>(should be 0)</t>
         </is>
       </c>
     </row>
@@ -1778,27 +2372,31 @@
           <t>Net revenue</t>
         </is>
       </c>
-      <c r="C5" s="38" t="n">
+      <c r="C5" s="40" t="n">
         <v>11102600</v>
       </c>
-      <c r="D5" s="39">
-        <f>Scenarios!D12</f>
-        <v/>
-      </c>
-      <c r="E5" s="39">
-        <f>Scenarios!D13</f>
-        <v/>
-      </c>
-      <c r="F5" s="39">
-        <f>Scenarios!D14</f>
-        <v/>
-      </c>
-      <c r="G5" s="39">
-        <f>Scenarios!D15</f>
-        <v/>
-      </c>
-      <c r="H5" s="39">
+      <c r="D5" s="41">
         <f>Scenarios!D16</f>
+        <v/>
+      </c>
+      <c r="E5" s="41">
+        <f>Scenarios!D17</f>
+        <v/>
+      </c>
+      <c r="F5" s="41">
+        <f>Scenarios!D18</f>
+        <v/>
+      </c>
+      <c r="G5" s="41">
+        <f>Scenarios!D19</f>
+        <v/>
+      </c>
+      <c r="H5" s="41">
+        <f>Scenarios!D20</f>
+        <v/>
+      </c>
+      <c r="I5" s="42">
+        <f>IF(MAX(ABS(D5-Scenarios!$D$16),ABS(E5-Scenarios!$D$17),ABS(F5-Scenarios!$D$18),ABS(G5-Scenarios!$D$19),ABS(H5-Scenarios!$D$20))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -1808,23 +2406,23 @@
           <t>Revenue growth %</t>
         </is>
       </c>
-      <c r="D6" s="40">
+      <c r="D6" s="43">
         <f>D5/C5-1</f>
         <v/>
       </c>
-      <c r="E6" s="40">
+      <c r="E6" s="43">
         <f>E5/D5-1</f>
         <v/>
       </c>
-      <c r="F6" s="40">
+      <c r="F6" s="43">
         <f>F5/E5-1</f>
         <v/>
       </c>
-      <c r="G6" s="40">
+      <c r="G6" s="43">
         <f>G5/F5-1</f>
         <v/>
       </c>
-      <c r="H6" s="40">
+      <c r="H6" s="43">
         <f>H5/G5-1</f>
         <v/>
       </c>
@@ -1835,24 +2433,28 @@
           <t>EBIT (operating) margin %</t>
         </is>
       </c>
-      <c r="D7" s="40">
-        <f>Scenarios!D17</f>
-        <v/>
-      </c>
-      <c r="E7" s="40">
-        <f>Scenarios!D18</f>
-        <v/>
-      </c>
-      <c r="F7" s="40">
-        <f>Scenarios!D19</f>
-        <v/>
-      </c>
-      <c r="G7" s="40">
-        <f>Scenarios!D20</f>
-        <v/>
-      </c>
-      <c r="H7" s="40">
+      <c r="D7" s="43">
         <f>Scenarios!D21</f>
+        <v/>
+      </c>
+      <c r="E7" s="43">
+        <f>Scenarios!D22</f>
+        <v/>
+      </c>
+      <c r="F7" s="43">
+        <f>Scenarios!D23</f>
+        <v/>
+      </c>
+      <c r="G7" s="43">
+        <f>Scenarios!D24</f>
+        <v/>
+      </c>
+      <c r="H7" s="43">
+        <f>Scenarios!D25</f>
+        <v/>
+      </c>
+      <c r="I7" s="42">
+        <f>IF(MAX(ABS(D7-Scenarios!$D$21),ABS(E7-Scenarios!$D$22),ABS(F7-Scenarios!$D$23),ABS(G7-Scenarios!$D$24),ABS(H7-Scenarios!$D$25))&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -1862,27 +2464,31 @@
           <t>EBIT</t>
         </is>
       </c>
-      <c r="C8" s="41" t="n">
+      <c r="C8" s="44" t="n">
         <v>2210615</v>
       </c>
       <c r="D8" s="29">
-        <f>D5*D7</f>
+        <f>Scenarios!D26</f>
         <v/>
       </c>
       <c r="E8" s="29">
-        <f>E5*E7</f>
+        <f>Scenarios!D27</f>
         <v/>
       </c>
       <c r="F8" s="29">
-        <f>F5*F7</f>
+        <f>Scenarios!D28</f>
         <v/>
       </c>
       <c r="G8" s="29">
-        <f>G5*G7</f>
+        <f>Scenarios!D29</f>
         <v/>
       </c>
       <c r="H8" s="29">
-        <f>H5*H7</f>
+        <f>Scenarios!D30</f>
+        <v/>
+      </c>
+      <c r="I8" s="45">
+        <f>IF(MAX(ABS(D8-Scenarios!$D$26),ABS(E8-Scenarios!$D$27),ABS(F8-Scenarios!$D$28),ABS(G8-Scenarios!$D$29),ABS(H8-Scenarios!$D$30))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -1892,24 +2498,24 @@
           <t>Less: cash taxes on EBIT</t>
         </is>
       </c>
-      <c r="D9" s="39">
-        <f>-D8*WACC!C10</f>
-        <v/>
-      </c>
-      <c r="E9" s="39">
-        <f>-E8*WACC!C10</f>
-        <v/>
-      </c>
-      <c r="F9" s="39">
-        <f>-F8*WACC!C10</f>
-        <v/>
-      </c>
-      <c r="G9" s="39">
-        <f>-G8*WACC!C10</f>
-        <v/>
-      </c>
-      <c r="H9" s="39">
-        <f>-H8*WACC!C10</f>
+      <c r="D9" s="41">
+        <f>-Scenarios!D26*Scenarios!$D$10</f>
+        <v/>
+      </c>
+      <c r="E9" s="41">
+        <f>-Scenarios!D27*Scenarios!$D$10</f>
+        <v/>
+      </c>
+      <c r="F9" s="41">
+        <f>-Scenarios!D28*Scenarios!$D$10</f>
+        <v/>
+      </c>
+      <c r="G9" s="41">
+        <f>-Scenarios!D29*Scenarios!$D$10</f>
+        <v/>
+      </c>
+      <c r="H9" s="41">
+        <f>-Scenarios!D30*Scenarios!$D$10</f>
         <v/>
       </c>
     </row>
@@ -1920,23 +2526,27 @@
         </is>
       </c>
       <c r="D10" s="29">
-        <f>D8+D9</f>
+        <f>Scenarios!D31</f>
         <v/>
       </c>
       <c r="E10" s="29">
-        <f>E8+E9</f>
+        <f>Scenarios!D32</f>
         <v/>
       </c>
       <c r="F10" s="29">
-        <f>F8+F9</f>
+        <f>Scenarios!D33</f>
         <v/>
       </c>
       <c r="G10" s="29">
-        <f>G8+G9</f>
+        <f>Scenarios!D34</f>
         <v/>
       </c>
       <c r="H10" s="29">
-        <f>H8+H9</f>
+        <f>Scenarios!D35</f>
+        <v/>
+      </c>
+      <c r="I10" s="45">
+        <f>IF(MAX(ABS(D10-Scenarios!$D$31),ABS(E10-Scenarios!$D$32),ABS(F10-Scenarios!$D$33),ABS(G10-Scenarios!$D$34),ABS(H10-Scenarios!$D$35))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -1946,20 +2556,25 @@
           <t xml:space="preserve">  D&amp;A % of revenue</t>
         </is>
       </c>
-      <c r="D11" s="16" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="E11" s="16" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="F11" s="16" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="G11" s="16" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="H11" s="16" t="n">
-        <v>0.045</v>
+      <c r="D11" s="16">
+        <f>Scenarios!$D$11</f>
+        <v/>
+      </c>
+      <c r="E11" s="16">
+        <f>Scenarios!$D$11</f>
+        <v/>
+      </c>
+      <c r="F11" s="16">
+        <f>Scenarios!$D$11</f>
+        <v/>
+      </c>
+      <c r="G11" s="16">
+        <f>Scenarios!$D$11</f>
+        <v/>
+      </c>
+      <c r="H11" s="16">
+        <f>Scenarios!$D$11</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -1968,24 +2583,28 @@
           <t>Plus: depreciation &amp; amortization</t>
         </is>
       </c>
-      <c r="D12" s="39">
-        <f>D5*D11</f>
-        <v/>
-      </c>
-      <c r="E12" s="39">
-        <f>E5*E11</f>
-        <v/>
-      </c>
-      <c r="F12" s="39">
-        <f>F5*F11</f>
-        <v/>
-      </c>
-      <c r="G12" s="39">
-        <f>G5*G11</f>
-        <v/>
-      </c>
-      <c r="H12" s="39">
-        <f>H5*H11</f>
+      <c r="D12" s="41">
+        <f>Scenarios!D36</f>
+        <v/>
+      </c>
+      <c r="E12" s="41">
+        <f>Scenarios!D37</f>
+        <v/>
+      </c>
+      <c r="F12" s="41">
+        <f>Scenarios!D38</f>
+        <v/>
+      </c>
+      <c r="G12" s="41">
+        <f>Scenarios!D39</f>
+        <v/>
+      </c>
+      <c r="H12" s="41">
+        <f>Scenarios!D40</f>
+        <v/>
+      </c>
+      <c r="I12" s="42">
+        <f>IF(MAX(ABS(D12-Scenarios!$D$36),ABS(E12-Scenarios!$D$37),ABS(F12-Scenarios!$D$38),ABS(G12-Scenarios!$D$39),ABS(H12-Scenarios!$D$40))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -1995,20 +2614,25 @@
           <t xml:space="preserve">  Capex % of revenue</t>
         </is>
       </c>
-      <c r="D13" s="16" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E13" s="16" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="F13" s="16" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G13" s="16" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H13" s="16" t="n">
-        <v>0.05</v>
+      <c r="D13" s="16">
+        <f>Scenarios!$D$12</f>
+        <v/>
+      </c>
+      <c r="E13" s="16">
+        <f>Scenarios!$D$12</f>
+        <v/>
+      </c>
+      <c r="F13" s="16">
+        <f>Scenarios!$D$12</f>
+        <v/>
+      </c>
+      <c r="G13" s="16">
+        <f>Scenarios!$D$12</f>
+        <v/>
+      </c>
+      <c r="H13" s="16">
+        <f>Scenarios!$D$12</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -2017,47 +2641,56 @@
           <t>Less: capital expenditures</t>
         </is>
       </c>
-      <c r="D14" s="39">
-        <f>-D5*D13</f>
-        <v/>
-      </c>
-      <c r="E14" s="39">
-        <f>-E5*E13</f>
-        <v/>
-      </c>
-      <c r="F14" s="39">
-        <f>-F5*F13</f>
-        <v/>
-      </c>
-      <c r="G14" s="39">
-        <f>-G5*G13</f>
-        <v/>
-      </c>
-      <c r="H14" s="39">
-        <f>-H5*H13</f>
+      <c r="D14" s="41">
+        <f>-Scenarios!D41</f>
+        <v/>
+      </c>
+      <c r="E14" s="41">
+        <f>-Scenarios!D42</f>
+        <v/>
+      </c>
+      <c r="F14" s="41">
+        <f>-Scenarios!D43</f>
+        <v/>
+      </c>
+      <c r="G14" s="41">
+        <f>-Scenarios!D44</f>
+        <v/>
+      </c>
+      <c r="H14" s="41">
+        <f>-Scenarios!D45</f>
+        <v/>
+      </c>
+      <c r="I14" s="42">
+        <f>IF(MAX(ABS(D14+Scenarios!$D$41),ABS(E14+Scenarios!$D$42),ABS(F14+Scenarios!$D$43),ABS(G14+Scenarios!$D$44),ABS(H14+Scenarios!$D$45))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NWC % of revenue</t>
-        </is>
-      </c>
-      <c r="D15" s="16" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="E15" s="16" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="F15" s="16" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="G15" s="16" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="H15" s="16" t="n">
-        <v>0.075</v>
+          <t xml:space="preserve">  NWC build % of Δrevenue</t>
+        </is>
+      </c>
+      <c r="D15" s="16">
+        <f>Scenarios!$D$13</f>
+        <v/>
+      </c>
+      <c r="E15" s="16">
+        <f>Scenarios!$D$13</f>
+        <v/>
+      </c>
+      <c r="F15" s="16">
+        <f>Scenarios!$D$13</f>
+        <v/>
+      </c>
+      <c r="G15" s="16">
+        <f>Scenarios!$D$13</f>
+        <v/>
+      </c>
+      <c r="H15" s="16">
+        <f>Scenarios!$D$13</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -2066,24 +2699,28 @@
           <t>Less: increase in net working capital</t>
         </is>
       </c>
-      <c r="D16" s="39">
-        <f>-D15*(D5-C5)</f>
-        <v/>
-      </c>
-      <c r="E16" s="39">
-        <f>-E15*(E5-D5)</f>
-        <v/>
-      </c>
-      <c r="F16" s="39">
-        <f>-F15*(F5-E5)</f>
-        <v/>
-      </c>
-      <c r="G16" s="39">
-        <f>-G15*(G5-F5)</f>
-        <v/>
-      </c>
-      <c r="H16" s="39">
-        <f>-H15*(H5-G5)</f>
+      <c r="D16" s="41">
+        <f>-Scenarios!D46</f>
+        <v/>
+      </c>
+      <c r="E16" s="41">
+        <f>-Scenarios!D47</f>
+        <v/>
+      </c>
+      <c r="F16" s="41">
+        <f>-Scenarios!D48</f>
+        <v/>
+      </c>
+      <c r="G16" s="41">
+        <f>-Scenarios!D49</f>
+        <v/>
+      </c>
+      <c r="H16" s="41">
+        <f>-Scenarios!D50</f>
+        <v/>
+      </c>
+      <c r="I16" s="42">
+        <f>IF(MAX(ABS(D16+Scenarios!$D$46),ABS(E16+Scenarios!$D$47),ABS(F16+Scenarios!$D$48),ABS(G16+Scenarios!$D$49),ABS(H16+Scenarios!$D$50))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2093,24 +2730,28 @@
           <t>Unlevered free cash flow</t>
         </is>
       </c>
-      <c r="D17" s="42">
-        <f>D10+D12+D14+D16</f>
-        <v/>
-      </c>
-      <c r="E17" s="42">
-        <f>E10+E12+E14+E16</f>
-        <v/>
-      </c>
-      <c r="F17" s="42">
-        <f>F10+F12+F14+F16</f>
-        <v/>
-      </c>
-      <c r="G17" s="42">
-        <f>G10+G12+G14+G16</f>
-        <v/>
-      </c>
-      <c r="H17" s="42">
-        <f>H10+H12+H14+H16</f>
+      <c r="D17" s="46">
+        <f>Scenarios!D51</f>
+        <v/>
+      </c>
+      <c r="E17" s="46">
+        <f>Scenarios!D52</f>
+        <v/>
+      </c>
+      <c r="F17" s="46">
+        <f>Scenarios!D53</f>
+        <v/>
+      </c>
+      <c r="G17" s="46">
+        <f>Scenarios!D54</f>
+        <v/>
+      </c>
+      <c r="H17" s="46">
+        <f>Scenarios!D55</f>
+        <v/>
+      </c>
+      <c r="I17" s="45">
+        <f>IF(MAX(ABS(D17-Scenarios!$D$51),ABS(E17-Scenarios!$D$52),ABS(F17-Scenarios!$D$53),ABS(G17-Scenarios!$D$54),ABS(H17-Scenarios!$D$55))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2120,19 +2761,19 @@
           <t>Discount period (years)</t>
         </is>
       </c>
-      <c r="D18" s="43" t="n">
+      <c r="D18" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="43" t="n">
+      <c r="E18" s="47" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="43" t="n">
+      <c r="F18" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="G18" s="43" t="n">
+      <c r="G18" s="47" t="n">
         <v>4</v>
       </c>
-      <c r="H18" s="43" t="n">
+      <c r="H18" s="47" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2142,23 +2783,23 @@
           <t>Discount factor @ WACC</t>
         </is>
       </c>
-      <c r="D19" s="44">
+      <c r="D19" s="48">
         <f>1/(1+Scenarios!$D$8)^D18</f>
         <v/>
       </c>
-      <c r="E19" s="44">
+      <c r="E19" s="48">
         <f>1/(1+Scenarios!$D$8)^E18</f>
         <v/>
       </c>
-      <c r="F19" s="44">
+      <c r="F19" s="48">
         <f>1/(1+Scenarios!$D$8)^F18</f>
         <v/>
       </c>
-      <c r="G19" s="44">
+      <c r="G19" s="48">
         <f>1/(1+Scenarios!$D$8)^G18</f>
         <v/>
       </c>
-      <c r="H19" s="44">
+      <c r="H19" s="48">
         <f>1/(1+Scenarios!$D$8)^H18</f>
         <v/>
       </c>
@@ -2191,546 +2832,561 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="45" t="inlineStr">
+      <c r="A22" s="49" t="inlineStr">
+        <is>
+          <t>Scenarios linkage summary (column I should all read OK)</t>
+        </is>
+      </c>
+      <c r="I22" s="50">
+        <f>IF(COUNTIF(I5:I17,"CHECK")=0,"ALL OK","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="51" t="inlineStr">
         <is>
           <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
         </is>
       </c>
-      <c r="B22" s="13" t="n"/>
-      <c r="C22" s="13" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="19" t="inlineStr">
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Sum of PV of explicit FCF (FY26–FY30)</t>
         </is>
       </c>
-      <c r="C23" s="46">
+      <c r="C24" s="52">
         <f>SUM(D20:H20)</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Terminal growth rate (g)</t>
         </is>
       </c>
-      <c r="C24" s="40">
+      <c r="C25" s="43">
         <f>Scenarios!$D$9</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="19" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="C25" s="29">
+      <c r="C26" s="29">
         <f>H8+H12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
-        </is>
-      </c>
-      <c r="C26" s="39">
-        <f>H17*(1+Scenarios!$D$9)/(Scenarios!$D$8-Scenarios!$D$9)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
+          <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
+        </is>
+      </c>
+      <c r="C27" s="41">
+        <f>H17*(1+Scenarios!$D$9)/(Scenarios!$D$8-Scenarios!$D$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Implied exit EV/EBITDA (Gordon Growth)</t>
         </is>
       </c>
-      <c r="C27" s="47">
-        <f>C26/C25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="19" t="inlineStr">
-        <is>
-          <t>PV of terminal value</t>
-        </is>
-      </c>
-      <c r="C28" s="46">
-        <f>C26/(1+Scenarios!$D$8)^H18</f>
+      <c r="C28" s="53">
+        <f>C27/C26</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="19" t="inlineStr">
         <is>
+          <t>PV of terminal value</t>
+        </is>
+      </c>
+      <c r="C29" s="52">
+        <f>C27/(1+Scenarios!$D$8)^H18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="C29" s="29">
-        <f>C23+C28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>Plus: cash &amp; equivalents (FY2025)</t>
-        </is>
-      </c>
-      <c r="C30" s="38" t="n">
-        <v>1807202</v>
-      </c>
-      <c r="D30" s="48" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
+      <c r="C30" s="29">
+        <f>C24+C29</f>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
         <is>
+          <t>Plus: cash &amp; equivalents (FY2025)</t>
+        </is>
+      </c>
+      <c r="C31" s="40" t="n">
+        <v>1807202</v>
+      </c>
+      <c r="D31" s="54" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
           <t>Less: total debt</t>
         </is>
       </c>
-      <c r="C31" s="38" t="n">
+      <c r="C32" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="D31" s="48" t="inlineStr">
+      <c r="D32" s="54" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="19" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
       </c>
-      <c r="C32" s="29">
-        <f>C29+C30+C31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+      <c r="C33" s="29">
+        <f>C30+C31+C32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>Diluted shares outstanding (000)</t>
         </is>
       </c>
-      <c r="C33" s="38" t="n">
+      <c r="C34" s="40" t="n">
         <v>111380</v>
       </c>
-      <c r="D33" s="48" t="inlineStr">
+      <c r="D34" s="54" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="19" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>Implied value per share</t>
         </is>
       </c>
-      <c r="C34" s="49">
-        <f>C32/C33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="15" t="inlineStr">
+      <c r="C35" s="55">
+        <f>C33/C34</f>
+        <v/>
+      </c>
+      <c r="I35" s="45">
+        <f>IF(ABS(C35-Scenarios!$D$58)&lt;0.05,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C35" s="50" t="n">
+      <c r="C36" s="56" t="n">
         <v>100</v>
       </c>
-      <c r="D35" s="48" t="inlineStr">
+      <c r="D36" s="54" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="19" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="19" t="inlineStr">
         <is>
           <t>Implied upside / (downside)</t>
         </is>
       </c>
-      <c r="C36" s="51">
-        <f>C34/C35-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="15" t="inlineStr">
+      <c r="C37" s="57">
+        <f>C35/C36-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: % of EV from terminal value</t>
         </is>
       </c>
-      <c r="C37" s="40">
-        <f>C28/C29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="45" t="inlineStr">
+      <c r="C38" s="43">
+        <f>C29/C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="51" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
       </c>
-      <c r="B39" s="13" t="n"/>
-      <c r="C39" s="13" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="52" t="inlineStr">
+      <c r="B40" s="13" t="n"/>
+      <c r="C40" s="13" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="49" t="inlineStr">
         <is>
           <t>Exit multiple selection (see Comps tab for peer build)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="15" t="inlineStr">
-        <is>
-          <t>Selected exit EV/EBITDA multiple (FY2030E)</t>
-        </is>
-      </c>
-      <c r="C41" s="53" t="n">
-        <v>8</v>
-      </c>
-      <c r="D41" s="17" t="inlineStr">
-        <is>
-          <t>Base-case terminal multiple; see Comps → Exit Multiple Build</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>Terminal value = Terminal EBITDA × exit multiple</t>
-        </is>
-      </c>
-      <c r="C42" s="39">
-        <f>C25*C41</f>
-        <v/>
+          <t>Selected exit EV/EBITDA multiple (FY2030E)</t>
+        </is>
+      </c>
+      <c r="C42" s="58" t="n">
+        <v>8</v>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
+        <is>
+          <t>Base-case terminal multiple; see Comps → Exit Multiple Build</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="15" t="inlineStr">
         <is>
+          <t>Terminal value = Terminal EBITDA × exit multiple</t>
+        </is>
+      </c>
+      <c r="C43" s="41">
+        <f>C26*C42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="C43" s="39">
-        <f>C42/(1+Scenarios!$D$8)^H18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="19" t="inlineStr">
-        <is>
-          <t>Enterprise value (exit method)</t>
-        </is>
-      </c>
-      <c r="C44" s="29">
-        <f>C23+C43</f>
+      <c r="C44" s="41">
+        <f>C43/(1+Scenarios!$D$8)^H18</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="19" t="inlineStr">
         <is>
+          <t>Enterprise value (exit method)</t>
+        </is>
+      </c>
+      <c r="C45" s="29">
+        <f>C24+C44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="19" t="inlineStr">
+        <is>
           <t>Implied value per share (exit method)</t>
         </is>
       </c>
-      <c r="C45" s="54">
-        <f>(C44+C30+C31)/C33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="45" t="inlineStr">
+      <c r="C46" s="59">
+        <f>(C45+C31+C32)/C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="51" t="inlineStr">
         <is>
           <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
         </is>
       </c>
-      <c r="B47" s="13" t="n"/>
-      <c r="C47" s="13" t="n"/>
-      <c r="D47" s="13" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="55" t="inlineStr"/>
-      <c r="B48" s="56" t="inlineStr">
+      <c r="B48" s="13" t="n"/>
+      <c r="C48" s="13" t="n"/>
+      <c r="D48" s="13" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="60" t="inlineStr"/>
+      <c r="B49" s="61" t="inlineStr">
         <is>
           <t>Gordon Growth</t>
         </is>
       </c>
-      <c r="C48" s="56" t="inlineStr">
+      <c r="C49" s="61" t="inlineStr">
         <is>
           <t>Exit Multiple</t>
         </is>
       </c>
-      <c r="D48" s="56" t="inlineStr">
+      <c r="D49" s="61" t="inlineStr">
         <is>
           <t>Variance</t>
         </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="19" t="inlineStr">
-        <is>
-          <t>Terminal value ($)</t>
-        </is>
-      </c>
-      <c r="B49" s="46">
-        <f>C26</f>
-        <v/>
-      </c>
-      <c r="C49" s="46">
-        <f>C42</f>
-        <v/>
-      </c>
-      <c r="D49" s="46">
-        <f>B49-C49</f>
-        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="19" t="inlineStr">
         <is>
+          <t>Terminal value ($)</t>
+        </is>
+      </c>
+      <c r="B50" s="52">
+        <f>C27</f>
+        <v/>
+      </c>
+      <c r="C50" s="52">
+        <f>C43</f>
+        <v/>
+      </c>
+      <c r="D50" s="52">
+        <f>B50-C50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="19" t="inlineStr">
+        <is>
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
       </c>
-      <c r="B50" s="57">
-        <f>C27</f>
-        <v/>
-      </c>
-      <c r="C50" s="57">
-        <f>C41</f>
-        <v/>
-      </c>
-      <c r="D50" s="57">
-        <f>B50-C50</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="15" t="inlineStr">
+      <c r="B51" s="62">
+        <f>C28</f>
+        <v/>
+      </c>
+      <c r="C51" s="62">
+        <f>C42</f>
+        <v/>
+      </c>
+      <c r="D51" s="62">
+        <f>B51-C51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="15" t="inlineStr">
         <is>
           <t>Terminal value variance (%)</t>
         </is>
       </c>
-      <c r="B51" s="40" t="inlineStr"/>
-      <c r="C51" s="40" t="inlineStr"/>
-      <c r="D51" s="40">
-        <f>(B49-C49)/B49</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="19" t="inlineStr">
+      <c r="B52" s="43" t="inlineStr"/>
+      <c r="C52" s="43" t="inlineStr"/>
+      <c r="D52" s="43">
+        <f>(B50-C50)/B50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="19" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="B52" s="58">
-        <f>C34</f>
-        <v/>
-      </c>
-      <c r="C52" s="58">
-        <f>C45</f>
-        <v/>
-      </c>
-      <c r="D52" s="58">
-        <f>B52-C52</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="59" t="inlineStr">
+      <c r="B53" s="63">
+        <f>C35</f>
+        <v/>
+      </c>
+      <c r="C53" s="63">
+        <f>C46</f>
+        <v/>
+      </c>
+      <c r="D53" s="63">
+        <f>B53-C53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="64" t="inlineStr">
         <is>
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B53" s="60">
-        <f>IF(ABS(D50)&lt;=1.5,"PASS","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="C53" s="61">
-        <f>TEXT(D50,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
-        <v/>
-      </c>
-      <c r="D53" s="17" t="inlineStr">
+      <c r="B54" s="65">
+        <f>IF(ABS(D51)&lt;=1.5,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="C54" s="66">
+        <f>TEXT(D51,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
+        <v/>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
         <is>
           <t>Gordon implied should bracket exit assumption</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="45" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="51" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
       </c>
-      <c r="B56" s="13" t="n"/>
-      <c r="C56" s="13" t="n"/>
-      <c r="D56" s="13" t="n"/>
-      <c r="E56" s="13" t="n"/>
-      <c r="F56" s="13" t="n"/>
-      <c r="G56" s="13" t="n"/>
-      <c r="H56" s="13" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="62" t="inlineStr">
+      <c r="B57" s="13" t="n"/>
+      <c r="C57" s="13" t="n"/>
+      <c r="D57" s="13" t="n"/>
+      <c r="E57" s="13" t="n"/>
+      <c r="F57" s="13" t="n"/>
+      <c r="G57" s="13" t="n"/>
+      <c r="H57" s="13" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="67" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
       </c>
-      <c r="D57" s="63" t="n">
+      <c r="D58" s="68" t="n">
         <v>0.015</v>
       </c>
-      <c r="E57" s="63" t="n">
+      <c r="E58" s="68" t="n">
         <v>0.02</v>
       </c>
-      <c r="F57" s="63" t="n">
+      <c r="F58" s="68" t="n">
         <v>0.0225</v>
       </c>
-      <c r="G57" s="63" t="n">
+      <c r="G58" s="68" t="n">
         <v>0.025</v>
       </c>
-      <c r="H57" s="63" t="n">
+      <c r="H58" s="68" t="n">
         <v>0.03</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="63" t="n">
+    <row r="59">
+      <c r="A59" s="68" t="n">
         <v>0.09</v>
       </c>
-      <c r="D58" s="64">
-        <f>(NPV(0.09,D17:H17)+(H17*(1+0.015)/(0.09-0.015))/(1+0.09)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="E58" s="64">
-        <f>(NPV(0.09,D17:H17)+(H17*(1+0.02)/(0.09-0.02))/(1+0.09)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="F58" s="64">
-        <f>(NPV(0.09,D17:H17)+(H17*(1+0.0225)/(0.09-0.0225))/(1+0.09)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="G58" s="64">
-        <f>(NPV(0.09,D17:H17)+(H17*(1+0.025)/(0.09-0.025))/(1+0.09)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="H58" s="64">
-        <f>(NPV(0.09,D17:H17)+(H17*(1+0.03)/(0.09-0.03))/(1+0.09)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="63" t="n">
+      <c r="D59" s="69">
+        <f>(NPV(0.09,D17:H17)+(H17*(1+0.015)/(0.09-0.015))/(1+0.09)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="E59" s="69">
+        <f>(NPV(0.09,D17:H17)+(H17*(1+0.02)/(0.09-0.02))/(1+0.09)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="F59" s="69">
+        <f>(NPV(0.09,D17:H17)+(H17*(1+0.0225)/(0.09-0.0225))/(1+0.09)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="G59" s="69">
+        <f>(NPV(0.09,D17:H17)+(H17*(1+0.025)/(0.09-0.025))/(1+0.09)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="H59" s="69">
+        <f>(NPV(0.09,D17:H17)+(H17*(1+0.03)/(0.09-0.03))/(1+0.09)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="68" t="n">
         <v>0.095</v>
       </c>
-      <c r="D59" s="64">
-        <f>(NPV(0.095,D17:H17)+(H17*(1+0.015)/(0.095-0.015))/(1+0.095)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="E59" s="64">
-        <f>(NPV(0.095,D17:H17)+(H17*(1+0.02)/(0.095-0.02))/(1+0.095)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="F59" s="64">
-        <f>(NPV(0.095,D17:H17)+(H17*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="G59" s="64">
-        <f>(NPV(0.095,D17:H17)+(H17*(1+0.025)/(0.095-0.025))/(1+0.095)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="H59" s="64">
-        <f>(NPV(0.095,D17:H17)+(H17*(1+0.03)/(0.095-0.03))/(1+0.095)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="63" t="n">
+      <c r="D60" s="69">
+        <f>(NPV(0.095,D17:H17)+(H17*(1+0.015)/(0.095-0.015))/(1+0.095)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="E60" s="69">
+        <f>(NPV(0.095,D17:H17)+(H17*(1+0.02)/(0.095-0.02))/(1+0.095)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="F60" s="69">
+        <f>(NPV(0.095,D17:H17)+(H17*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="G60" s="69">
+        <f>(NPV(0.095,D17:H17)+(H17*(1+0.025)/(0.095-0.025))/(1+0.095)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="H60" s="69">
+        <f>(NPV(0.095,D17:H17)+(H17*(1+0.03)/(0.095-0.03))/(1+0.095)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="68" t="n">
         <v>0.1</v>
       </c>
-      <c r="D60" s="64">
-        <f>(NPV(0.1,D17:H17)+(H17*(1+0.015)/(0.1-0.015))/(1+0.1)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="E60" s="64">
-        <f>(NPV(0.1,D17:H17)+(H17*(1+0.02)/(0.1-0.02))/(1+0.1)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="F60" s="65">
-        <f>(NPV(0.1,D17:H17)+(H17*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="G60" s="64">
-        <f>(NPV(0.1,D17:H17)+(H17*(1+0.025)/(0.1-0.025))/(1+0.1)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="H60" s="64">
-        <f>(NPV(0.1,D17:H17)+(H17*(1+0.03)/(0.1-0.03))/(1+0.1)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="63" t="n">
+      <c r="D61" s="69">
+        <f>(NPV(0.1,D17:H17)+(H17*(1+0.015)/(0.1-0.015))/(1+0.1)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="E61" s="69">
+        <f>(NPV(0.1,D17:H17)+(H17*(1+0.02)/(0.1-0.02))/(1+0.1)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="F61" s="70">
+        <f>(NPV(0.1,D17:H17)+(H17*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="G61" s="69">
+        <f>(NPV(0.1,D17:H17)+(H17*(1+0.025)/(0.1-0.025))/(1+0.1)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="H61" s="69">
+        <f>(NPV(0.1,D17:H17)+(H17*(1+0.03)/(0.1-0.03))/(1+0.1)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="68" t="n">
         <v>0.105</v>
       </c>
-      <c r="D61" s="64">
-        <f>(NPV(0.105,D17:H17)+(H17*(1+0.015)/(0.105-0.015))/(1+0.105)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="E61" s="64">
-        <f>(NPV(0.105,D17:H17)+(H17*(1+0.02)/(0.105-0.02))/(1+0.105)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="F61" s="64">
-        <f>(NPV(0.105,D17:H17)+(H17*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="G61" s="64">
-        <f>(NPV(0.105,D17:H17)+(H17*(1+0.025)/(0.105-0.025))/(1+0.105)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="H61" s="64">
-        <f>(NPV(0.105,D17:H17)+(H17*(1+0.03)/(0.105-0.03))/(1+0.105)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="63" t="n">
+      <c r="D62" s="69">
+        <f>(NPV(0.105,D17:H17)+(H17*(1+0.015)/(0.105-0.015))/(1+0.105)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="E62" s="69">
+        <f>(NPV(0.105,D17:H17)+(H17*(1+0.02)/(0.105-0.02))/(1+0.105)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="F62" s="69">
+        <f>(NPV(0.105,D17:H17)+(H17*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="G62" s="69">
+        <f>(NPV(0.105,D17:H17)+(H17*(1+0.025)/(0.105-0.025))/(1+0.105)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="H62" s="69">
+        <f>(NPV(0.105,D17:H17)+(H17*(1+0.03)/(0.105-0.03))/(1+0.105)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="68" t="n">
         <v>0.11</v>
       </c>
-      <c r="D62" s="64">
-        <f>(NPV(0.11,D17:H17)+(H17*(1+0.015)/(0.11-0.015))/(1+0.11)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="E62" s="64">
-        <f>(NPV(0.11,D17:H17)+(H17*(1+0.02)/(0.11-0.02))/(1+0.11)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="F62" s="64">
-        <f>(NPV(0.11,D17:H17)+(H17*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="G62" s="64">
-        <f>(NPV(0.11,D17:H17)+(H17*(1+0.025)/(0.11-0.025))/(1+0.11)^5+C30+C31)/C33</f>
-        <v/>
-      </c>
-      <c r="H62" s="64">
-        <f>(NPV(0.11,D17:H17)+(H17*(1+0.03)/(0.11-0.03))/(1+0.11)^5+C30+C31)/C33</f>
+      <c r="D63" s="69">
+        <f>(NPV(0.11,D17:H17)+(H17*(1+0.015)/(0.11-0.015))/(1+0.11)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="E63" s="69">
+        <f>(NPV(0.11,D17:H17)+(H17*(1+0.02)/(0.11-0.02))/(1+0.11)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="F63" s="69">
+        <f>(NPV(0.11,D17:H17)+(H17*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="G63" s="69">
+        <f>(NPV(0.11,D17:H17)+(H17*(1+0.025)/(0.11-0.025))/(1+0.11)^5+C31+C32)/C34</f>
+        <v/>
+      </c>
+      <c r="H63" s="69">
+        <f>(NPV(0.11,D17:H17)+(H17*(1+0.03)/(0.11-0.03))/(1+0.11)^5+C31+C32)/C34</f>
         <v/>
       </c>
     </row>
@@ -2739,14 +3395,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2794,10 +3450,10 @@
           <t>FY2025A revenue</t>
         </is>
       </c>
-      <c r="C4" s="38" t="n">
+      <c r="C4" s="40" t="n">
         <v>11102600</v>
       </c>
-      <c r="D4" s="48" t="inlineStr">
+      <c r="D4" s="54" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -2809,7 +3465,7 @@
           <t>FY2025A EBITDA (EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="C5" s="39">
+      <c r="C5" s="41">
         <f>2210615+496228</f>
         <v/>
       </c>
@@ -2820,10 +3476,10 @@
           <t>FY2026E diluted EPS (guidance midpoint)</t>
         </is>
       </c>
-      <c r="C6" s="50" t="n">
+      <c r="C6" s="56" t="n">
         <v>9.609999999999999</v>
       </c>
-      <c r="D6" s="48" t="inlineStr">
+      <c r="D6" s="54" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
@@ -2835,10 +3491,10 @@
           <t>Cash &amp; equivalents</t>
         </is>
       </c>
-      <c r="C7" s="38" t="n">
+      <c r="C7" s="40" t="n">
         <v>1807202</v>
       </c>
-      <c r="D7" s="48" t="inlineStr">
+      <c r="D7" s="54" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -2850,10 +3506,10 @@
           <t>Diluted shares (000)</t>
         </is>
       </c>
-      <c r="C8" s="38" t="n">
+      <c r="C8" s="40" t="n">
         <v>111380</v>
       </c>
-      <c r="D8" s="48" t="inlineStr">
+      <c r="D8" s="54" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -2865,33 +3521,33 @@
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C9" s="50" t="n">
+      <c r="C9" s="56" t="n">
         <v>100</v>
       </c>
-      <c r="D9" s="48" t="inlineStr">
+      <c r="D9" s="54" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="61" t="inlineStr">
+      <c r="A10" s="66" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current EV / EBITDA</t>
         </is>
       </c>
-      <c r="C10" s="66">
+      <c r="C10" s="71">
         <f>(C9*C8-C7)/C5</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="61" t="inlineStr">
+      <c r="A11" s="66" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current P / E (FY2026E)</t>
         </is>
       </c>
-      <c r="C11" s="66">
+      <c r="C11" s="71">
         <f>C9/C6</f>
         <v/>
       </c>
@@ -2904,24 +3560,24 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="61" t="inlineStr">
+      <c r="A14" s="66" t="inlineStr">
         <is>
           <t>Peer / reference EV/EBITDA (forward / illustrative)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="67" t="inlineStr">
+      <c r="A15" s="72" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C15" s="68" t="inlineStr">
+      <c r="C15" s="73" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="D15" s="67" t="inlineStr">
+      <c r="D15" s="72" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2933,7 +3589,7 @@
           <t>lululemon (LULU) — current</t>
         </is>
       </c>
-      <c r="C16" s="69">
+      <c r="C16" s="74">
         <f>(C9*C8-C7)/C5</f>
         <v/>
       </c>
@@ -2949,7 +3605,7 @@
           <t>Nike (NKE)</t>
         </is>
       </c>
-      <c r="C17" s="70" t="n">
+      <c r="C17" s="75" t="n">
         <v>18</v>
       </c>
       <c r="D17" s="17" t="inlineStr">
@@ -2964,7 +3620,7 @@
           <t>Deckers (DECK)</t>
         </is>
       </c>
-      <c r="C18" s="70" t="n">
+      <c r="C18" s="75" t="n">
         <v>15</v>
       </c>
       <c r="D18" s="17" t="inlineStr">
@@ -2979,7 +3635,7 @@
           <t>On Holding (ONON)</t>
         </is>
       </c>
-      <c r="C19" s="70" t="n">
+      <c r="C19" s="75" t="n">
         <v>25</v>
       </c>
       <c r="D19" s="17" t="inlineStr">
@@ -2994,7 +3650,7 @@
           <t>adidas (ADS)</t>
         </is>
       </c>
-      <c r="C20" s="70" t="n">
+      <c r="C20" s="75" t="n">
         <v>12</v>
       </c>
       <c r="D20" s="17" t="inlineStr">
@@ -3009,7 +3665,7 @@
           <t>V.F. Corp (VFC)</t>
         </is>
       </c>
-      <c r="C21" s="70" t="n">
+      <c r="C21" s="75" t="n">
         <v>10</v>
       </c>
       <c r="D21" s="17" t="inlineStr">
@@ -3031,19 +3687,19 @@
           <t>Gordon Growth implied exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="C24" s="47">
-        <f>DCF!C27</f>
+      <c r="C24" s="53">
+        <f>DCF!C28</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="59" t="inlineStr">
+      <c r="A25" s="64" t="inlineStr">
         <is>
           <t>Selected exit multiple (base case)</t>
         </is>
       </c>
-      <c r="C25" s="57">
-        <f>DCF!C41</f>
+      <c r="C25" s="62">
+        <f>DCF!C42</f>
         <v/>
       </c>
     </row>
@@ -3053,13 +3709,13 @@
           <t>Spread (selected − Gordon implied)</t>
         </is>
       </c>
-      <c r="C26" s="47">
+      <c r="C26" s="53">
         <f>C25-C24</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="59" t="inlineStr">
+      <c r="A27" s="64" t="inlineStr">
         <is>
           <t>Rationale for 8.0x</t>
         </is>
@@ -3108,27 +3764,27 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="67" t="inlineStr">
+      <c r="A35" s="72" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="C35" s="68" t="inlineStr">
+      <c r="C35" s="73" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="D35" s="68" t="inlineStr">
+      <c r="D35" s="73" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="E35" s="68" t="inlineStr">
+      <c r="E35" s="73" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="F35" s="68" t="inlineStr">
+      <c r="F35" s="73" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
@@ -3140,17 +3796,17 @@
           <t>EV / EBITDA (FY2025A)</t>
         </is>
       </c>
-      <c r="C36" s="70" t="n">
+      <c r="C36" s="75" t="n">
         <v>4.5</v>
       </c>
-      <c r="D36" s="70" t="n">
+      <c r="D36" s="75" t="n">
         <v>7.5</v>
       </c>
-      <c r="E36" s="71">
+      <c r="E36" s="76">
         <f>(C5*C36+C7)/C8</f>
         <v/>
       </c>
-      <c r="F36" s="71">
+      <c r="F36" s="76">
         <f>(C5*D36+C7)/C8</f>
         <v/>
       </c>
@@ -3161,17 +3817,17 @@
           <t>P / E (FY2026E EPS)</t>
         </is>
       </c>
-      <c r="C37" s="70" t="n">
+      <c r="C37" s="75" t="n">
         <v>10</v>
       </c>
-      <c r="D37" s="70" t="n">
+      <c r="D37" s="75" t="n">
         <v>18</v>
       </c>
-      <c r="E37" s="71">
+      <c r="E37" s="76">
         <f>C6*C37</f>
         <v/>
       </c>
-      <c r="F37" s="71">
+      <c r="F37" s="76">
         <f>C6*D37</f>
         <v/>
       </c>
@@ -3182,35 +3838,35 @@
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="C38" s="72" t="inlineStr">
+      <c r="C38" s="77" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D38" s="72" t="inlineStr">
+      <c r="D38" s="77" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E38" s="71">
-        <f>Scenarios!C29</f>
-        <v/>
-      </c>
-      <c r="F38" s="71">
-        <f>Scenarios!E29</f>
+      <c r="E38" s="76">
+        <f>Scenarios!C58</f>
+        <v/>
+      </c>
+      <c r="F38" s="76">
+        <f>Scenarios!E58</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="73" t="inlineStr">
+      <c r="A40" s="78" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C40" s="74" t="n">
+      <c r="C40" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="D40" s="48" t="inlineStr">
+      <c r="D40" s="54" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>

</xml_diff>

<commit_message>
Link every red assumption to its external or model source
Complete ASSUMPTION_SRC coverage across WACC, Scenarios, DCF, Comps, and
3-statement tabs. Add internal workbook links for cross-tab derivations
(WACC build, Comps exit multiple, sensitivity axes). Fill former placeholder
sources with FRED, Damodaran, Macrotrends, Yahoo Finance, and SEC 10-K URLs.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0x"/>
   </numFmts>
-  <fonts count="44">
+  <fonts count="46">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -282,6 +282,19 @@
       <i val="1"/>
       <color rgb="00000000"/>
       <sz val="7"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <i val="1"/>
+      <color rgb="000000CC"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <i val="1"/>
+      <color rgb="000000CC"/>
+      <sz val="7"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Garamond"/>
@@ -349,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -404,7 +417,7 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -562,13 +575,14 @@
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="45" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1489,7 +1503,7 @@
       </c>
       <c r="G8" s="28" t="inlineStr">
         <is>
-          <t>WACC tab CAPM build (this model)</t>
+          <t>WACC tab: CAPM build</t>
         </is>
       </c>
     </row>
@@ -2460,6 +2474,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId4"/>
+    <hyperlink ref="G8" location="'WACC'!C16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId7"/>
@@ -2476,7 +2491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2490,6 +2505,7 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -2552,6 +2568,11 @@
           <t>Source</t>
         </is>
       </c>
+      <c r="L2" s="41" t="inlineStr">
+        <is>
+          <t>Alt. source</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="42" t="inlineStr">
@@ -2630,6 +2651,21 @@
         <f>H5/G5-1</f>
         <v/>
       </c>
+      <c r="J6" s="17" t="inlineStr">
+        <is>
+          <t>−6.1% FY2026 revenue growth matches company guidance midpoint of −5% to −7% after Q2 FY2026 print.</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
+        <is>
+          <t>LULU Q2 FY2026 earnings release</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>LULU historical revenue (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -2661,6 +2697,21 @@
         <f>IF(MAX(ABS(D7-Scenarios!$D$21),ABS(E7-Scenarios!$D$22),ABS(F7-Scenarios!$D$23),ABS(G7-Scenarios!$D$24),ABS(H7-Scenarios!$D$25))&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
+      <c r="J7" s="17" t="inlineStr">
+        <is>
+          <t>13.9% FY2026 EBIT margin reflects Americas weakness and guided compression; above bear, below historical peak.</t>
+        </is>
+      </c>
+      <c r="K7" s="18" t="inlineStr">
+        <is>
+          <t>LULU Q2 FY2026 guidance / 10-K margins</t>
+        </is>
+      </c>
+      <c r="L7" s="18" t="inlineStr">
+        <is>
+          <t>LULU historical EBIT margins (10-K)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
@@ -3113,6 +3164,16 @@
         <f>Scenarios!$D$9</f>
         <v/>
       </c>
+      <c r="J26" s="17" t="inlineStr">
+        <is>
+          <t>2.25% terminal growth approximates long-run GDP plus inflation; conservative perpetuity rate for mature apparel.</t>
+        </is>
+      </c>
+      <c r="K26" s="18" t="inlineStr">
+        <is>
+          <t>BEA: Real GDP (FRED GDPC1)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="20" t="inlineStr">
@@ -3302,14 +3363,19 @@
       <c r="C43" s="62" t="n">
         <v>8</v>
       </c>
-      <c r="D43" s="17" t="inlineStr">
+      <c r="J43" s="17" t="inlineStr">
         <is>
           <t>8.0x FY2030E exit EV/EBITDA; above trough, below premium peers, roughly one turn above Gordon-implied multiple.</t>
         </is>
       </c>
-      <c r="E43" s="28" t="inlineStr">
-        <is>
-          <t>DCF Comps tab: Exit Multiple Build</t>
+      <c r="K43" s="18" t="inlineStr">
+        <is>
+          <t>Macrotrends: LULU EV/EBITDA history</t>
+        </is>
+      </c>
+      <c r="L43" s="28" t="inlineStr">
+        <is>
+          <t>Comps: Exit Multiple Build</t>
         </is>
       </c>
     </row>
@@ -3510,6 +3576,21 @@
       <c r="H59" s="72" t="n">
         <v>0.03</v>
       </c>
+      <c r="I59" s="28" t="inlineStr">
+        <is>
+          <t>Scenarios: terminal g</t>
+        </is>
+      </c>
+      <c r="J59" s="17" t="inlineStr">
+        <is>
+          <t>Terminal-g axis 1.5–3.0% brackets 2.25% base; bounded by long-run real GDP and inflation benchmarks.</t>
+        </is>
+      </c>
+      <c r="K59" s="18" t="inlineStr">
+        <is>
+          <t>FRED: Real GDP (GDPC1)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="72" t="n">
@@ -3535,6 +3616,16 @@
         <f>(NPV(0.09,D18:H18)+(H18*(1+0.03)/(0.09-0.03))/(1+0.09)^5+C32+C33)/C35</f>
         <v/>
       </c>
+      <c r="I60" s="28" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
+      <c r="J60" s="18" t="inlineStr">
+        <is>
+          <t>Damodaran: Historical Implied ERP</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="72" t="n">
@@ -3560,6 +3651,11 @@
         <f>(NPV(0.095,D18:H18)+(H18*(1+0.03)/(0.095-0.03))/(1+0.095)^5+C32+C33)/C35</f>
         <v/>
       </c>
+      <c r="I61" s="28" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="72" t="n">
@@ -3585,6 +3681,11 @@
         <f>(NPV(0.1,D18:H18)+(H18*(1+0.03)/(0.1-0.03))/(1+0.1)^5+C32+C33)/C35</f>
         <v/>
       </c>
+      <c r="I62" s="28" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="72" t="n">
@@ -3610,6 +3711,11 @@
         <f>(NPV(0.105,D18:H18)+(H18*(1+0.03)/(0.105-0.03))/(1+0.105)^5+C32+C33)/C35</f>
         <v/>
       </c>
+      <c r="I63" s="28" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="72" t="n">
@@ -3635,6 +3741,11 @@
         <f>(NPV(0.11,D18:H18)+(H18*(1+0.03)/(0.11-0.03))/(1+0.11)^5+C32+C33)/C35</f>
         <v/>
       </c>
+      <c r="I64" s="28" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="J65" s="17" t="inlineStr">
@@ -3644,7 +3755,12 @@
       </c>
       <c r="K65" s="28" t="inlineStr">
         <is>
-          <t>Base WACC/g from Scenarios tab</t>
+          <t>Scenarios: WACC &amp; terminal g</t>
+        </is>
+      </c>
+      <c r="L65" s="18" t="inlineStr">
+        <is>
+          <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
     </row>
@@ -3652,18 +3768,35 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId20"/>
+    <hyperlink ref="L43" location="'Comps'!A25"/>
+    <hyperlink ref="I59" location="'Scenarios'!D9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId21"/>
+    <hyperlink ref="I60" location="'WACC'!C16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId22"/>
+    <hyperlink ref="I61" location="'WACC'!C16"/>
+    <hyperlink ref="I62" location="'WACC'!C16"/>
+    <hyperlink ref="I63" location="'WACC'!C16"/>
+    <hyperlink ref="I64" location="'WACC'!C16"/>
+    <hyperlink ref="K65" location="'Scenarios'!D8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3687,6 +3820,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -4119,14 +4253,14 @@
           <t>7.5x EV/EBITDA high case on FY2025A; partial recovery before terminal year, below historical peaks.</t>
         </is>
       </c>
-      <c r="I36" s="28" t="inlineStr">
-        <is>
-          <t>LULU current EV/EBITDA (model)</t>
-        </is>
-      </c>
-      <c r="J36" s="81" t="inlineStr">
-        <is>
-          <t>Peer comp set (Comps tab)</t>
+      <c r="I36" s="18" t="inlineStr">
+        <is>
+          <t>Yahoo Finance: LULU EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="J36" s="82" t="inlineStr">
+        <is>
+          <t>Macrotrends: LULU EV/EBITDA history</t>
         </is>
       </c>
     </row>
@@ -4160,14 +4294,14 @@
           <t>18x P/E high on FY2026E EPS; modest recovery case still below historical premium LULU multiples.</t>
         </is>
       </c>
-      <c r="I37" s="28" t="inlineStr">
-        <is>
-          <t>LULU current P/E vs FY26E EPS</t>
-        </is>
-      </c>
-      <c r="J37" s="81" t="inlineStr">
-        <is>
-          <t>Peer P/E ranges (illustrative)</t>
+      <c r="I37" s="18" t="inlineStr">
+        <is>
+          <t>Yahoo Finance: LULU P/E (FY26E)</t>
+        </is>
+      </c>
+      <c r="J37" s="82" t="inlineStr">
+        <is>
+          <t>Yahoo Finance: NKE P/E (peer benchmark)</t>
         </is>
       </c>
     </row>
@@ -4177,12 +4311,12 @@
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="C38" s="82" t="inlineStr">
+      <c r="C38" s="83" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D38" s="82" t="inlineStr">
+      <c r="D38" s="83" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4197,12 +4331,12 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="83" t="inlineStr">
+      <c r="A40" s="84" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C40" s="84" t="n">
+      <c r="C40" s="85" t="n">
         <v>100</v>
       </c>
       <c r="D40" s="58" t="inlineStr">
@@ -4236,8 +4370,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix WACC source links visibility and terminal football field
Move WACC source hyperlinks to column B (visible next to inputs) using
Excel HYPERLINK formulas. Rebuild EV/EBITDA football field on FY2030E
terminal EBITDA (6.5–9.5x range) with 8.0x DCF exit as midpoint row.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -115,6 +115,12 @@
       <name val="Garamond"/>
       <b val="1"/>
       <color rgb="00C8102E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="00C8102E"/>
       <sz val="10"/>
     </font>
     <font>
@@ -126,12 +132,6 @@
       <name val="Garamond"/>
       <i val="1"/>
       <color rgb="00000000"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Garamond"/>
-      <i val="1"/>
-      <color rgb="000000CC"/>
       <sz val="8"/>
     </font>
     <font>
@@ -167,9 +167,9 @@
     </font>
     <font>
       <name val="Garamond"/>
-      <b val="1"/>
-      <color rgb="00C8102E"/>
-      <sz val="9"/>
+      <i val="1"/>
+      <color rgb="000000CC"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Garamond"/>
@@ -288,13 +288,13 @@
       <i val="1"/>
       <color rgb="000000CC"/>
       <sz val="7"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Garamond"/>
       <i val="1"/>
       <color rgb="000000CC"/>
       <sz val="7"/>
-      <u val="single"/>
     </font>
     <font>
       <name val="Garamond"/>
@@ -362,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -379,18 +379,23 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -414,9 +419,6 @@
     <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -444,7 +446,7 @@
     <xf numFmtId="164" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -480,6 +482,7 @@
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="33" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -517,7 +520,7 @@
     <xf numFmtId="164" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -566,8 +569,11 @@
     <xf numFmtId="168" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -575,7 +581,13 @@
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1086,14 +1098,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="2" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -1112,74 +1123,81 @@
           <t>Cost of equity (CAPM)</t>
         </is>
       </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Source (click link)</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>Justification (~20 words)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Risk-free rate (10-yr UST)</t>
         </is>
       </c>
-      <c r="C3" s="16" t="n">
+      <c r="B3" s="17">
+        <f>HYPERLINK("https://fred.stlouisfed.org/series/DGS10","↳ FRED: 10Y Treasury (DGS10)")</f>
+        <v/>
+      </c>
+      <c r="C3" s="18" t="n">
         <v>0.043</v>
       </c>
-      <c r="D3" s="17" t="inlineStr">
+      <c r="D3" s="19" t="inlineStr">
         <is>
           <t>4.3% risk-free anchored to FRED 10Y Treasury (DGS10); rounded early-Sep-2026 level for DCF stability.</t>
         </is>
       </c>
-      <c r="E3" s="18" t="inlineStr">
-        <is>
-          <t>FRED: 10Y Treasury (DGS10)</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Equity risk premium</t>
         </is>
       </c>
-      <c r="C4" s="16" t="n">
+      <c r="B4" s="17">
+        <f>HYPERLINK("https://pages.stern.nyu.edu/~adamodar/New_Home_Page/datafile/histimpl.html","↳ Damodaran: Historical Implied ERP")</f>
+        <v/>
+      </c>
+      <c r="C4" s="18" t="n">
         <v>0.06</v>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>6.0% additive ERP; conservative vs Damodaran implied ~4.2% (Jan-26); within long-run historical US range.</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
-        <is>
-          <t>Damodaran: Historical Implied ERP</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Levered beta</t>
         </is>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="B5" s="17">
+        <f>HYPERLINK("https://finance.yahoo.com/quote/LULU/key-statistics/","↳ Yahoo Finance: LULU Beta")</f>
+        <v/>
+      </c>
+      <c r="C5" s="20" t="n">
         <v>0.95</v>
       </c>
-      <c r="D5" s="17" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>0.95 levered beta vs ~0.86 market; modest uplift for near-term earnings volatility and post-guidance de-rating.</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Yahoo Finance: LULU Beta</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Cost of equity = rf + β × ERP</t>
         </is>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="22">
         <f>C3+C5*C4</f>
         <v/>
       </c>
@@ -1192,52 +1210,50 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Pre-tax cost of debt</t>
         </is>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="B9" s="17">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU FY2025 10-K (no funded debt)")</f>
+        <v/>
+      </c>
+      <c r="C9" s="18" t="n">
         <v>0.05</v>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>5.0% illustrative pre-tax debt cost; LULU has no funded term debt, only an undrawn revolving credit facility.</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K (no funded debt)</t>
-        </is>
-      </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="B10" s="17">
+        <f>HYPERLINK("https://pages.stern.nyu.edu/~adamodar/New_Home_Page/datafile/taxrate.html","↳ Damodaran: US tax rate dataset")</f>
+        <v/>
+      </c>
+      <c r="C10" s="18" t="n">
         <v>0.27</v>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>27% normalized marginal cash tax rate; mid-point between recent effective rates and US federal-plus-state blend.</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>Damodaran: US tax rate dataset</t>
-        </is>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="23">
         <f>C9*(1-C10)</f>
         <v/>
       </c>
@@ -1250,66 +1266,55 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Equity weight</t>
         </is>
       </c>
-      <c r="C14" s="16" t="n">
+      <c r="B14" s="17">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU FY2025 10-K balance sheet")</f>
+        <v/>
+      </c>
+      <c r="C14" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>100% equity weight; net-cash balance sheet with no material funded debt at market values per FY2025 10-K.</t>
         </is>
       </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K balance sheet</t>
-        </is>
-      </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Debt weight</t>
         </is>
       </c>
-      <c r="C15" s="16" t="n">
+      <c r="B15" s="17">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU FY2025 10-K balance sheet")</f>
+        <v/>
+      </c>
+      <c r="C15" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>0% debt weight; no outstanding term loans or bonds, so WACC effectively equals levered cost of equity here.</t>
         </is>
       </c>
-      <c r="E15" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K balance sheet</t>
-        </is>
-      </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="C16" s="23">
+      <c r="C16" s="24">
         <f>C14*C6+C15*C11</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId7"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1344,17 +1349,17 @@
       <c r="E1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="C2" s="24" t="inlineStr">
+      <c r="C2" s="25" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="D2" s="25" t="inlineStr">
+      <c r="D2" s="26" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="E2" s="26" t="inlineStr">
+      <c r="E2" s="27" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
@@ -1366,275 +1371,266 @@
           <t>Key assumptions (5-yr forecast)</t>
         </is>
       </c>
-      <c r="F3" s="27" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>Justification (~20 words)</t>
         </is>
       </c>
-      <c r="G3" s="27" t="inlineStr">
-        <is>
-          <t>Source</t>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>Source (click link)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>FY2026E revenue growth</t>
         </is>
       </c>
-      <c r="C4" s="16" t="n">
+      <c r="C4" s="18" t="n">
         <v>-0.09</v>
       </c>
-      <c r="D4" s="16" t="n">
+      <c r="D4" s="18" t="n">
         <v>-0.061</v>
       </c>
-      <c r="E4" s="16" t="n">
+      <c r="E4" s="18" t="n">
         <v>-0.04</v>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="F4" s="19" t="inlineStr">
         <is>
           <t>−6.1% FY2026 revenue growth matches company guidance midpoint of −5% to −7% after Q2 FY2026 print.</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
-        <is>
-          <t>LULU Q2 FY2026 earnings release</t>
-        </is>
+      <c r="G4" s="17">
+        <f>HYPERLINK("https://investor.lululemon.com/news-releases","↳ LULU Q2 FY2026 earnings release")</f>
+        <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>FY2027–FY2030E revenue growth (avg)</t>
         </is>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="18" t="n">
         <v>-0.01</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="18" t="n">
         <v>0.028</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="18" t="n">
         <v>0.06</v>
       </c>
-      <c r="F5" s="17" t="inlineStr">
+      <c r="F5" s="19" t="inlineStr">
         <is>
           <t>2.8% avg FY27–30 growth assumes gradual recovery; well below historical double-digit LULU revenue expansion.</t>
         </is>
       </c>
-      <c r="G5" s="18" t="inlineStr">
-        <is>
-          <t>LULU historical revenue (10-K)</t>
-        </is>
+      <c r="G5" s="17">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU historical revenue (10-K)")</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>FY2026E EBIT margin</t>
         </is>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="18" t="n">
         <v>0.125</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="18" t="n">
         <v>0.139</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="18" t="n">
         <v>0.15</v>
       </c>
-      <c r="F6" s="17" t="inlineStr">
+      <c r="F6" s="19" t="inlineStr">
         <is>
           <t>13.9% FY2026 EBIT margin reflects Americas weakness and guided compression; above bear, below historical peak.</t>
         </is>
       </c>
-      <c r="G6" s="18" t="inlineStr">
-        <is>
-          <t>LULU Q2 FY2026 guidance / 10-K margins</t>
-        </is>
+      <c r="G6" s="17">
+        <f>HYPERLINK("https://investor.lululemon.com/news-releases","↳ LULU Q2 FY2026 guidance / 10-K margins")</f>
+        <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Terminal (FY2030E) EBIT margin</t>
         </is>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="18" t="n">
         <v>0.12</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="18" t="n">
         <v>0.155</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="18" t="n">
         <v>0.19</v>
       </c>
-      <c r="F7" s="17" t="inlineStr">
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>15.5% FY2030 EBIT margin assumes partial recovery; still materially below ~20–24% peak operating margins.</t>
         </is>
       </c>
-      <c r="G7" s="18" t="inlineStr">
-        <is>
-          <t>LULU historical EBIT margins (10-K)</t>
-        </is>
+      <c r="G7" s="17">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU historical EBIT margins (10-K)")</f>
+        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="18" t="n">
         <v>0.11</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="18" t="n">
         <v>0.1</v>
       </c>
-      <c r="E8" s="16" t="n">
+      <c r="E8" s="18" t="n">
         <v>0.09</v>
       </c>
-      <c r="F8" s="17" t="inlineStr">
+      <c r="F8" s="19" t="inlineStr">
         <is>
           <t>10.0% base WACC ties to CAPM build on WACC tab; drives scenario DCFs and base-case valuation.</t>
         </is>
       </c>
       <c r="G8" s="28" t="inlineStr">
         <is>
-          <t>WACC tab: CAPM build</t>
+          <t>↳ WACC tab: CAPM build</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Terminal growth</t>
         </is>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C9" s="18" t="n">
         <v>0.015</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="18" t="n">
         <v>0.0225</v>
       </c>
-      <c r="E9" s="16" t="n">
+      <c r="E9" s="18" t="n">
         <v>0.03</v>
       </c>
-      <c r="F9" s="17" t="inlineStr">
+      <c r="F9" s="19" t="inlineStr">
         <is>
           <t>2.25% terminal growth approximates long-run GDP plus inflation; conservative perpetuity rate for mature apparel.</t>
         </is>
       </c>
-      <c r="G9" s="18" t="inlineStr">
-        <is>
-          <t>BEA: Real GDP (FRED GDPC1)</t>
-        </is>
+      <c r="G9" s="17">
+        <f>HYPERLINK("https://fred.stlouisfed.org/series/GDPC1","↳ BEA: Real GDP (FRED GDPC1)")</f>
+        <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Cash tax rate</t>
         </is>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10" s="18" t="n">
         <v>0.3</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="18" t="n">
         <v>0.27</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="18" t="n">
         <v>0.25</v>
       </c>
-      <c r="F10" s="17" t="inlineStr">
+      <c r="F10" s="19" t="inlineStr">
         <is>
           <t>27% cash tax rate for scenario FCF; consistent with WACC normalized rate and DCF unlevered cash conversion.</t>
         </is>
       </c>
-      <c r="G10" s="18" t="inlineStr">
-        <is>
-          <t>Damodaran: US tax rate dataset</t>
-        </is>
+      <c r="G10" s="17">
+        <f>HYPERLINK("https://pages.stern.nyu.edu/~adamodar/New_Home_Page/datafile/taxrate.html","↳ Damodaran: US tax rate dataset")</f>
+        <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>D&amp;A % of revenue</t>
         </is>
       </c>
-      <c r="C11" s="16" t="n">
+      <c r="C11" s="18" t="n">
         <v>0.045</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="18" t="n">
         <v>0.045</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E11" s="18" t="n">
         <v>0.045</v>
       </c>
-      <c r="F11" s="17" t="inlineStr">
+      <c r="F11" s="19" t="inlineStr">
         <is>
           <t>4.5% D&amp;A to revenue near FY22–25 average; reflects store fleet, distribution, and technology amortization load.</t>
         </is>
       </c>
-      <c r="G11" s="18" t="inlineStr">
-        <is>
-          <t>LULU CF statement (10-K)</t>
-        </is>
+      <c r="G11" s="17">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU CF statement (10-K)")</f>
+        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Capex % of revenue</t>
         </is>
       </c>
-      <c r="C12" s="16" t="n">
+      <c r="C12" s="18" t="n">
         <v>0.055</v>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="18" t="n">
         <v>0.05</v>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="E12" s="18" t="n">
         <v>0.045</v>
       </c>
-      <c r="F12" s="17" t="inlineStr">
+      <c r="F12" s="19" t="inlineStr">
         <is>
           <t>5.0% capex to revenue aligned with recent investment intensity and continued global store expansion plans.</t>
         </is>
       </c>
-      <c r="G12" s="18" t="inlineStr">
-        <is>
-          <t>LULU CF statement (10-K)</t>
-        </is>
+      <c r="G12" s="17">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU CF statement (10-K)")</f>
+        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>NWC build % of Δrevenue</t>
         </is>
       </c>
-      <c r="C13" s="16" t="n">
+      <c r="C13" s="18" t="n">
         <v>0.08</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="18" t="n">
         <v>0.075</v>
       </c>
-      <c r="E13" s="16" t="n">
+      <c r="E13" s="18" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="F13" s="17" t="inlineStr">
+      <c r="F13" s="19" t="inlineStr">
         <is>
           <t>7.5% of revenue change for ΔNWC; ties working-capital swings to sales trajectory per historical sensitivity.</t>
         </is>
       </c>
-      <c r="G13" s="18" t="inlineStr">
-        <is>
-          <t>LULU BS/IS historical (10-K)</t>
-        </is>
+      <c r="G13" s="17">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU BS/IS historical (10-K)")</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -2405,7 +2401,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="20" t="inlineStr">
+      <c r="A57" s="21" t="inlineStr">
         <is>
           <t>Enterprise value (DCF)</t>
         </is>
@@ -2443,7 +2439,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="20" t="inlineStr">
+      <c r="A59" s="21" t="inlineStr">
         <is>
           <t>Upside / (downside) vs current</t>
         </is>
@@ -2470,16 +2466,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId4"/>
     <hyperlink ref="G8" location="'WACC'!C16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2592,7 +2579,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Net revenue</t>
         </is>
@@ -2626,7 +2613,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Revenue growth %</t>
         </is>
@@ -2651,24 +2638,23 @@
         <f>H5/G5-1</f>
         <v/>
       </c>
-      <c r="J6" s="17" t="inlineStr">
+      <c r="J6" s="19" t="inlineStr">
         <is>
           <t>−6.1% FY2026 revenue growth matches company guidance midpoint of −5% to −7% after Q2 FY2026 print.</t>
         </is>
       </c>
-      <c r="K6" s="18" t="inlineStr">
-        <is>
-          <t>LULU Q2 FY2026 earnings release</t>
-        </is>
-      </c>
-      <c r="L6" s="18" t="inlineStr">
+      <c r="K6" s="17">
+        <f>HYPERLINK("https://investor.lululemon.com/news-releases","↳ LULU Q2 FY2026 earnings release")</f>
+        <v/>
+      </c>
+      <c r="L6" s="49" t="inlineStr">
         <is>
           <t>LULU historical revenue (10-K)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>EBIT (operating) margin %</t>
         </is>
@@ -2697,29 +2683,28 @@
         <f>IF(MAX(ABS(D7-Scenarios!$D$21),ABS(E7-Scenarios!$D$22),ABS(F7-Scenarios!$D$23),ABS(G7-Scenarios!$D$24),ABS(H7-Scenarios!$D$25))&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
-      <c r="J7" s="17" t="inlineStr">
+      <c r="J7" s="19" t="inlineStr">
         <is>
           <t>13.9% FY2026 EBIT margin reflects Americas weakness and guided compression; above bear, below historical peak.</t>
         </is>
       </c>
-      <c r="K7" s="18" t="inlineStr">
-        <is>
-          <t>LULU Q2 FY2026 guidance / 10-K margins</t>
-        </is>
-      </c>
-      <c r="L7" s="18" t="inlineStr">
+      <c r="K7" s="17">
+        <f>HYPERLINK("https://investor.lululemon.com/news-releases","↳ LULU Q2 FY2026 guidance / 10-K margins")</f>
+        <v/>
+      </c>
+      <c r="L7" s="49" t="inlineStr">
         <is>
           <t>LULU historical EBIT margins (10-K)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>EBIT</t>
         </is>
       </c>
-      <c r="C8" s="49" t="n">
+      <c r="C8" s="50" t="n">
         <v>2210615</v>
       </c>
       <c r="D8" s="32">
@@ -2742,13 +2727,13 @@
         <f>Scenarios!D30</f>
         <v/>
       </c>
-      <c r="I8" s="50">
+      <c r="I8" s="51">
         <f>IF(MAX(ABS(D8-Scenarios!$D$26),ABS(E8-Scenarios!$D$27),ABS(F8-Scenarios!$D$28),ABS(G8-Scenarios!$D$29),ABS(H8-Scenarios!$D$30))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Less: cash taxes on EBIT</t>
         </is>
@@ -2775,7 +2760,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>NOPAT</t>
         </is>
@@ -2800,50 +2785,49 @@
         <f>Scenarios!D35</f>
         <v/>
       </c>
-      <c r="I10" s="50">
+      <c r="I10" s="51">
         <f>IF(MAX(ABS(D10-Scenarios!$D$31),ABS(E10-Scenarios!$D$32),ABS(F10-Scenarios!$D$33),ABS(G10-Scenarios!$D$34),ABS(H10-Scenarios!$D$35))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A % of revenue</t>
         </is>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="18">
         <f>Scenarios!$D$11</f>
         <v/>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="18">
         <f>Scenarios!$D$11</f>
         <v/>
       </c>
-      <c r="F11" s="16">
+      <c r="F11" s="18">
         <f>Scenarios!$D$11</f>
         <v/>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="18">
         <f>Scenarios!$D$11</f>
         <v/>
       </c>
-      <c r="H11" s="16">
+      <c r="H11" s="18">
         <f>Scenarios!$D$11</f>
         <v/>
       </c>
-      <c r="J11" s="17" t="inlineStr">
+      <c r="J11" s="19" t="inlineStr">
         <is>
           <t>4.5% D&amp;A to revenue near FY22–25 average; reflects store fleet, distribution, and technology amortization load.</t>
         </is>
       </c>
-      <c r="K11" s="18" t="inlineStr">
-        <is>
-          <t>LULU CF statement (10-K)</t>
-        </is>
+      <c r="K11" s="17">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU CF statement (10-K)")</f>
+        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Plus: depreciation &amp; amortization</t>
         </is>
@@ -2874,44 +2858,43 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex % of revenue</t>
         </is>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="18">
         <f>Scenarios!$D$12</f>
         <v/>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="18">
         <f>Scenarios!$D$12</f>
         <v/>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="18">
         <f>Scenarios!$D$12</f>
         <v/>
       </c>
-      <c r="G13" s="16">
+      <c r="G13" s="18">
         <f>Scenarios!$D$12</f>
         <v/>
       </c>
-      <c r="H13" s="16">
+      <c r="H13" s="18">
         <f>Scenarios!$D$12</f>
         <v/>
       </c>
-      <c r="J13" s="17" t="inlineStr">
+      <c r="J13" s="19" t="inlineStr">
         <is>
           <t>5.0% capex to revenue aligned with recent investment intensity and continued global store expansion plans.</t>
         </is>
       </c>
-      <c r="K13" s="18" t="inlineStr">
-        <is>
-          <t>LULU CF statement (10-K)</t>
-        </is>
+      <c r="K13" s="17">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU CF statement (10-K)")</f>
+        <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Less: capital expenditures</t>
         </is>
@@ -2942,44 +2925,43 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC build % of Δrevenue</t>
         </is>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="18">
         <f>Scenarios!$D$13</f>
         <v/>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="18">
         <f>Scenarios!$D$13</f>
         <v/>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="18">
         <f>Scenarios!$D$13</f>
         <v/>
       </c>
-      <c r="G15" s="16">
+      <c r="G15" s="18">
         <f>Scenarios!$D$13</f>
         <v/>
       </c>
-      <c r="H15" s="16">
+      <c r="H15" s="18">
         <f>Scenarios!$D$13</f>
         <v/>
       </c>
-      <c r="J15" s="17" t="inlineStr">
+      <c r="J15" s="19" t="inlineStr">
         <is>
           <t>7.5% of revenue change for ΔNWC; ties working-capital swings to sales trajectory per historical sensitivity.</t>
         </is>
       </c>
-      <c r="K15" s="18" t="inlineStr">
-        <is>
-          <t>LULU BS/IS historical (10-K)</t>
-        </is>
+      <c r="K15" s="17">
+        <f>HYPERLINK("https://www.sec.gov/Archives/edgar/data/1397187/000139718726000020/lulu-20260201.htm","↳ LULU BS/IS historical (10-K)")</f>
+        <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>(Increase)/decrease in net working capital</t>
         </is>
@@ -3017,87 +2999,87 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>Unlevered free cash flow</t>
         </is>
       </c>
-      <c r="D18" s="51">
+      <c r="D18" s="52">
         <f>Scenarios!D51</f>
         <v/>
       </c>
-      <c r="E18" s="51">
+      <c r="E18" s="52">
         <f>Scenarios!D52</f>
         <v/>
       </c>
-      <c r="F18" s="51">
+      <c r="F18" s="52">
         <f>Scenarios!D53</f>
         <v/>
       </c>
-      <c r="G18" s="51">
+      <c r="G18" s="52">
         <f>Scenarios!D54</f>
         <v/>
       </c>
-      <c r="H18" s="51">
+      <c r="H18" s="52">
         <f>Scenarios!D55</f>
         <v/>
       </c>
-      <c r="I18" s="50">
+      <c r="I18" s="51">
         <f>IF(MAX(ABS(D18-Scenarios!$D$51),ABS(E18-Scenarios!$D$52),ABS(F18-Scenarios!$D$53),ABS(G18-Scenarios!$D$54),ABS(H18-Scenarios!$D$55))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Discount period (years)</t>
         </is>
       </c>
-      <c r="D19" s="52" t="n">
+      <c r="D19" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="52" t="n">
+      <c r="E19" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="F19" s="52" t="n">
+      <c r="F19" s="53" t="n">
         <v>3</v>
       </c>
-      <c r="G19" s="52" t="n">
+      <c r="G19" s="53" t="n">
         <v>4</v>
       </c>
-      <c r="H19" s="52" t="n">
+      <c r="H19" s="53" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Discount factor @ WACC</t>
         </is>
       </c>
-      <c r="D20" s="53">
+      <c r="D20" s="54">
         <f>1/(1+Scenarios!$D$8)^D19</f>
         <v/>
       </c>
-      <c r="E20" s="53">
+      <c r="E20" s="54">
         <f>1/(1+Scenarios!$D$8)^E19</f>
         <v/>
       </c>
-      <c r="F20" s="53">
+      <c r="F20" s="54">
         <f>1/(1+Scenarios!$D$8)^F19</f>
         <v/>
       </c>
-      <c r="G20" s="53">
+      <c r="G20" s="54">
         <f>1/(1+Scenarios!$D$8)^G19</f>
         <v/>
       </c>
-      <c r="H20" s="53">
+      <c r="H20" s="54">
         <f>1/(1+Scenarios!$D$8)^H19</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>PV of unlevered FCF</t>
         </is>
@@ -3124,18 +3106,18 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>Scenarios linkage summary (column I should all read OK)</t>
         </is>
       </c>
-      <c r="I23" s="54">
+      <c r="I23" s="55">
         <f>IF(COUNTIF(I5:I18,"CHECK")=0,"ALL OK","REVIEW")</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="55" t="inlineStr">
+      <c r="A24" s="56" t="inlineStr">
         <is>
           <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
         </is>
@@ -3144,18 +3126,18 @@
       <c r="C24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="20" t="inlineStr">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>Sum of PV of explicit FCF (FY26–FY30)</t>
         </is>
       </c>
-      <c r="C25" s="56">
+      <c r="C25" s="57">
         <f>SUM(D21:H21)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>Terminal growth rate (g)</t>
         </is>
@@ -3164,19 +3146,18 @@
         <f>Scenarios!$D$9</f>
         <v/>
       </c>
-      <c r="J26" s="17" t="inlineStr">
+      <c r="J26" s="19" t="inlineStr">
         <is>
           <t>2.25% terminal growth approximates long-run GDP plus inflation; conservative perpetuity rate for mature apparel.</t>
         </is>
       </c>
-      <c r="K26" s="18" t="inlineStr">
-        <is>
-          <t>BEA: Real GDP (FRED GDPC1)</t>
-        </is>
+      <c r="K26" s="17">
+        <f>HYPERLINK("https://fred.stlouisfed.org/series/GDPC1","↳ BEA: Real GDP (FRED GDPC1)")</f>
+        <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="20" t="inlineStr">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
         </is>
@@ -3187,7 +3168,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
         </is>
@@ -3198,29 +3179,29 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Implied exit EV/EBITDA (Gordon Growth)</t>
         </is>
       </c>
-      <c r="C29" s="57">
+      <c r="C29" s="58">
         <f>C28/C27</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="20" t="inlineStr">
+      <c r="A30" s="21" t="inlineStr">
         <is>
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="C30" s="56">
+      <c r="C30" s="57">
         <f>C28/(1+Scenarios!$D$8)^H19</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="20" t="inlineStr">
+      <c r="A31" s="21" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
@@ -3231,7 +3212,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="15" t="inlineStr">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>Plus: cash &amp; equivalents (FY2025)</t>
         </is>
@@ -3239,14 +3220,14 @@
       <c r="C32" s="45" t="n">
         <v>1807202</v>
       </c>
-      <c r="D32" s="58" t="inlineStr">
+      <c r="D32" s="59" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>Less: total debt</t>
         </is>
@@ -3254,14 +3235,14 @@
       <c r="C33" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="D33" s="58" t="inlineStr">
+      <c r="D33" s="59" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="20" t="inlineStr">
+      <c r="A34" s="21" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
@@ -3272,7 +3253,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="15" t="inlineStr">
+      <c r="A35" s="16" t="inlineStr">
         <is>
           <t>Diluted shares outstanding (000)</t>
         </is>
@@ -3280,55 +3261,55 @@
       <c r="C35" s="45" t="n">
         <v>111380</v>
       </c>
-      <c r="D35" s="58" t="inlineStr">
+      <c r="D35" s="59" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="20" t="inlineStr">
+      <c r="A36" s="21" t="inlineStr">
         <is>
           <t>Implied value per share</t>
         </is>
       </c>
-      <c r="C36" s="59">
+      <c r="C36" s="60">
         <f>C34/C35</f>
         <v/>
       </c>
-      <c r="I36" s="50">
+      <c r="I36" s="51">
         <f>IF(ABS(C36-Scenarios!$D$58)&lt;0.05,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="15" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C37" s="60" t="n">
+      <c r="C37" s="61" t="n">
         <v>100</v>
       </c>
-      <c r="D37" s="58" t="inlineStr">
+      <c r="D37" s="59" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="20" t="inlineStr">
+      <c r="A38" s="21" t="inlineStr">
         <is>
           <t>Implied upside / (downside)</t>
         </is>
       </c>
-      <c r="C38" s="61">
+      <c r="C38" s="62">
         <f>C36/C37-1</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="15" t="inlineStr">
+      <c r="A39" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: % of EV from terminal value</t>
         </is>
@@ -3339,7 +3320,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="55" t="inlineStr">
+      <c r="A41" s="56" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
@@ -3348,30 +3329,29 @@
       <c r="C41" s="13" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="27" t="inlineStr">
+      <c r="A42" s="15" t="inlineStr">
         <is>
           <t>Exit multiple selection (see Comps tab for peer build)</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="15" t="inlineStr">
+      <c r="A43" s="16" t="inlineStr">
         <is>
           <t>Selected exit EV/EBITDA multiple (FY2030E)</t>
         </is>
       </c>
-      <c r="C43" s="62" t="n">
+      <c r="C43" s="63" t="n">
         <v>8</v>
       </c>
-      <c r="J43" s="17" t="inlineStr">
-        <is>
-          <t>8.0x FY2030E exit EV/EBITDA; above trough, below premium peers, roughly one turn above Gordon-implied multiple.</t>
-        </is>
-      </c>
-      <c r="K43" s="18" t="inlineStr">
-        <is>
-          <t>Macrotrends: LULU EV/EBITDA history</t>
-        </is>
+      <c r="J43" s="19" t="inlineStr">
+        <is>
+          <t>8.0x FY2030E exit EV/EBITDA; mid-point of terminal football field (6.5–9.5x); ~1 turn above Gordon-implied ~7x.</t>
+        </is>
+      </c>
+      <c r="K43" s="17">
+        <f>HYPERLINK("https://www.macrotrends.net/stocks/charts/LULU/lululemon-athletica/enterprise-value-ebitda","↳ Macrotrends: LULU EV/EBITDA history")</f>
+        <v/>
       </c>
       <c r="L43" s="28" t="inlineStr">
         <is>
@@ -3380,7 +3360,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="15" t="inlineStr">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t>Terminal value = Terminal EBITDA × exit multiple</t>
         </is>
@@ -3391,7 +3371,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="15" t="inlineStr">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>PV of terminal value</t>
         </is>
@@ -3402,7 +3382,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="20" t="inlineStr">
+      <c r="A46" s="21" t="inlineStr">
         <is>
           <t>Enterprise value (exit method)</t>
         </is>
@@ -3413,18 +3393,18 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="20" t="inlineStr">
+      <c r="A47" s="21" t="inlineStr">
         <is>
           <t>Implied value per share (exit method)</t>
         </is>
       </c>
-      <c r="C47" s="63">
+      <c r="C47" s="64">
         <f>(C46+C32+C33)/C35</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="55" t="inlineStr">
+      <c r="A49" s="56" t="inlineStr">
         <is>
           <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
         </is>
@@ -3434,63 +3414,63 @@
       <c r="D49" s="13" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="64" t="inlineStr"/>
-      <c r="B50" s="65" t="inlineStr">
+      <c r="A50" s="65" t="inlineStr"/>
+      <c r="B50" s="66" t="inlineStr">
         <is>
           <t>Gordon Growth</t>
         </is>
       </c>
-      <c r="C50" s="65" t="inlineStr">
+      <c r="C50" s="66" t="inlineStr">
         <is>
           <t>Exit Multiple</t>
         </is>
       </c>
-      <c r="D50" s="65" t="inlineStr">
+      <c r="D50" s="66" t="inlineStr">
         <is>
           <t>Variance</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="20" t="inlineStr">
+      <c r="A51" s="21" t="inlineStr">
         <is>
           <t>Terminal value ($)</t>
         </is>
       </c>
-      <c r="B51" s="56">
+      <c r="B51" s="57">
         <f>C28</f>
         <v/>
       </c>
-      <c r="C51" s="56">
+      <c r="C51" s="57">
         <f>C44</f>
         <v/>
       </c>
-      <c r="D51" s="56">
+      <c r="D51" s="57">
         <f>B51-C51</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="20" t="inlineStr">
+      <c r="A52" s="21" t="inlineStr">
         <is>
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
       </c>
-      <c r="B52" s="66">
+      <c r="B52" s="67">
         <f>C29</f>
         <v/>
       </c>
-      <c r="C52" s="66">
+      <c r="C52" s="67">
         <f>C43</f>
         <v/>
       </c>
-      <c r="D52" s="66">
+      <c r="D52" s="67">
         <f>B52-C52</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="15" t="inlineStr">
+      <c r="A53" s="16" t="inlineStr">
         <is>
           <t>Terminal value variance (%)</t>
         </is>
@@ -3503,35 +3483,35 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="20" t="inlineStr">
+      <c r="A54" s="21" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="B54" s="67">
+      <c r="B54" s="68">
         <f>C36</f>
         <v/>
       </c>
-      <c r="C54" s="67">
+      <c r="C54" s="68">
         <f>C47</f>
         <v/>
       </c>
-      <c r="D54" s="67">
+      <c r="D54" s="68">
         <f>B54-C54</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="68" t="inlineStr">
+      <c r="A55" s="69" t="inlineStr">
         <is>
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B55" s="69">
+      <c r="B55" s="70">
         <f>IF(ABS(D52)&lt;=1.5,"PASS","REVIEW")</f>
         <v/>
       </c>
-      <c r="C55" s="70">
+      <c r="C55" s="71">
         <f>TEXT(D52,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
         <v/>
       </c>
@@ -3542,7 +3522,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="55" t="inlineStr">
+      <c r="A58" s="56" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
@@ -3556,24 +3536,24 @@
       <c r="H58" s="13" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="71" t="inlineStr">
+      <c r="A59" s="72" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
       </c>
-      <c r="D59" s="72" t="n">
+      <c r="D59" s="73" t="n">
         <v>0.015</v>
       </c>
-      <c r="E59" s="72" t="n">
+      <c r="E59" s="73" t="n">
         <v>0.02</v>
       </c>
-      <c r="F59" s="72" t="n">
+      <c r="F59" s="73" t="n">
         <v>0.0225</v>
       </c>
-      <c r="G59" s="72" t="n">
+      <c r="G59" s="73" t="n">
         <v>0.025</v>
       </c>
-      <c r="H59" s="72" t="n">
+      <c r="H59" s="73" t="n">
         <v>0.03</v>
       </c>
       <c r="I59" s="28" t="inlineStr">
@@ -3581,38 +3561,37 @@
           <t>Scenarios: terminal g</t>
         </is>
       </c>
-      <c r="J59" s="17" t="inlineStr">
+      <c r="J59" s="19" t="inlineStr">
         <is>
           <t>Terminal-g axis 1.5–3.0% brackets 2.25% base; bounded by long-run real GDP and inflation benchmarks.</t>
         </is>
       </c>
-      <c r="K59" s="18" t="inlineStr">
-        <is>
-          <t>FRED: Real GDP (GDPC1)</t>
-        </is>
+      <c r="K59" s="17">
+        <f>HYPERLINK("https://fred.stlouisfed.org/series/GDPC1","↳ FRED: Real GDP (GDPC1)")</f>
+        <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="72" t="n">
+      <c r="A60" s="73" t="n">
         <v>0.09</v>
       </c>
-      <c r="D60" s="73">
+      <c r="D60" s="74">
         <f>(NPV(0.09,D18:H18)+(H18*(1+0.015)/(0.09-0.015))/(1+0.09)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="E60" s="73">
+      <c r="E60" s="74">
         <f>(NPV(0.09,D18:H18)+(H18*(1+0.02)/(0.09-0.02))/(1+0.09)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="F60" s="73">
+      <c r="F60" s="74">
         <f>(NPV(0.09,D18:H18)+(H18*(1+0.0225)/(0.09-0.0225))/(1+0.09)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="G60" s="73">
+      <c r="G60" s="74">
         <f>(NPV(0.09,D18:H18)+(H18*(1+0.025)/(0.09-0.025))/(1+0.09)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="H60" s="73">
+      <c r="H60" s="74">
         <f>(NPV(0.09,D18:H18)+(H18*(1+0.03)/(0.09-0.03))/(1+0.09)^5+C32+C33)/C35</f>
         <v/>
       </c>
@@ -3621,33 +3600,33 @@
           <t>WACC tab</t>
         </is>
       </c>
-      <c r="J60" s="18" t="inlineStr">
+      <c r="J60" s="49" t="inlineStr">
         <is>
           <t>Damodaran: Historical Implied ERP</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="72" t="n">
+      <c r="A61" s="73" t="n">
         <v>0.095</v>
       </c>
-      <c r="D61" s="73">
+      <c r="D61" s="74">
         <f>(NPV(0.095,D18:H18)+(H18*(1+0.015)/(0.095-0.015))/(1+0.095)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="E61" s="73">
+      <c r="E61" s="74">
         <f>(NPV(0.095,D18:H18)+(H18*(1+0.02)/(0.095-0.02))/(1+0.095)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="F61" s="73">
+      <c r="F61" s="74">
         <f>(NPV(0.095,D18:H18)+(H18*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="G61" s="73">
+      <c r="G61" s="74">
         <f>(NPV(0.095,D18:H18)+(H18*(1+0.025)/(0.095-0.025))/(1+0.095)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="H61" s="73">
+      <c r="H61" s="74">
         <f>(NPV(0.095,D18:H18)+(H18*(1+0.03)/(0.095-0.03))/(1+0.095)^5+C32+C33)/C35</f>
         <v/>
       </c>
@@ -3658,26 +3637,26 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="72" t="n">
+      <c r="A62" s="73" t="n">
         <v>0.1</v>
       </c>
-      <c r="D62" s="73">
+      <c r="D62" s="74">
         <f>(NPV(0.1,D18:H18)+(H18*(1+0.015)/(0.1-0.015))/(1+0.1)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="E62" s="73">
+      <c r="E62" s="74">
         <f>(NPV(0.1,D18:H18)+(H18*(1+0.02)/(0.1-0.02))/(1+0.1)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="F62" s="74">
+      <c r="F62" s="75">
         <f>(NPV(0.1,D18:H18)+(H18*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="G62" s="73">
+      <c r="G62" s="74">
         <f>(NPV(0.1,D18:H18)+(H18*(1+0.025)/(0.1-0.025))/(1+0.1)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="H62" s="73">
+      <c r="H62" s="74">
         <f>(NPV(0.1,D18:H18)+(H18*(1+0.03)/(0.1-0.03))/(1+0.1)^5+C32+C33)/C35</f>
         <v/>
       </c>
@@ -3688,26 +3667,26 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="72" t="n">
+      <c r="A63" s="73" t="n">
         <v>0.105</v>
       </c>
-      <c r="D63" s="73">
+      <c r="D63" s="74">
         <f>(NPV(0.105,D18:H18)+(H18*(1+0.015)/(0.105-0.015))/(1+0.105)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="E63" s="73">
+      <c r="E63" s="74">
         <f>(NPV(0.105,D18:H18)+(H18*(1+0.02)/(0.105-0.02))/(1+0.105)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="F63" s="73">
+      <c r="F63" s="74">
         <f>(NPV(0.105,D18:H18)+(H18*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="G63" s="73">
+      <c r="G63" s="74">
         <f>(NPV(0.105,D18:H18)+(H18*(1+0.025)/(0.105-0.025))/(1+0.105)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="H63" s="73">
+      <c r="H63" s="74">
         <f>(NPV(0.105,D18:H18)+(H18*(1+0.03)/(0.105-0.03))/(1+0.105)^5+C32+C33)/C35</f>
         <v/>
       </c>
@@ -3718,26 +3697,26 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="72" t="n">
+      <c r="A64" s="73" t="n">
         <v>0.11</v>
       </c>
-      <c r="D64" s="73">
+      <c r="D64" s="74">
         <f>(NPV(0.11,D18:H18)+(H18*(1+0.015)/(0.11-0.015))/(1+0.11)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="E64" s="73">
+      <c r="E64" s="74">
         <f>(NPV(0.11,D18:H18)+(H18*(1+0.02)/(0.11-0.02))/(1+0.11)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="F64" s="73">
+      <c r="F64" s="74">
         <f>(NPV(0.11,D18:H18)+(H18*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="G64" s="73">
+      <c r="G64" s="74">
         <f>(NPV(0.11,D18:H18)+(H18*(1+0.025)/(0.11-0.025))/(1+0.11)^5+C32+C33)/C35</f>
         <v/>
       </c>
-      <c r="H64" s="73">
+      <c r="H64" s="74">
         <f>(NPV(0.11,D18:H18)+(H18*(1+0.03)/(0.11-0.03))/(1+0.11)^5+C32+C33)/C35</f>
         <v/>
       </c>
@@ -3748,55 +3727,45 @@
       </c>
     </row>
     <row r="65">
-      <c r="J65" s="17" t="inlineStr">
+      <c r="J65" s="19" t="inlineStr">
         <is>
           <t>Red WACC and g grid values bracket base case ±100bps discount rate and ±75bps terminal growth for sensitivity.</t>
         </is>
       </c>
       <c r="K65" s="28" t="inlineStr">
         <is>
-          <t>Scenarios: WACC &amp; terminal g</t>
-        </is>
-      </c>
-      <c r="L65" s="18" t="inlineStr">
-        <is>
-          <t>FRED: Real GDP (GDPC1)</t>
-        </is>
+          <t>↳ Scenarios: WACC &amp; terminal g</t>
+        </is>
+      </c>
+      <c r="L65" s="49">
+        <f>HYPERLINK("https://fred.stlouisfed.org/series/GDPC1","↳ FRED: Real GDP (GDPC1)")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId20"/>
-    <hyperlink ref="L43" location="'Comps'!A25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId13"/>
+    <hyperlink ref="L43" location="'Comps'!A26"/>
     <hyperlink ref="I59" location="'Scenarios'!D9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId21"/>
     <hyperlink ref="I60" location="'WACC'!C16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId14"/>
     <hyperlink ref="I61" location="'WACC'!C16"/>
     <hyperlink ref="I62" location="'WACC'!C16"/>
     <hyperlink ref="I63" location="'WACC'!C16"/>
     <hyperlink ref="I64" location="'WACC'!C16"/>
     <hyperlink ref="K65" location="'Scenarios'!D8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3808,7 +3777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3843,7 +3812,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>FY2025A revenue</t>
         </is>
@@ -3851,14 +3820,14 @@
       <c r="C4" s="45" t="n">
         <v>11102600</v>
       </c>
-      <c r="D4" s="58" t="inlineStr">
+      <c r="D4" s="59" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>FY2025A EBITDA (EBIT + D&amp;A)</t>
         </is>
@@ -3869,484 +3838,532 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>FY2030E terminal EBITDA (DCF EBIT + D&amp;A)</t>
+        </is>
+      </c>
+      <c r="C6" s="46">
+        <f>DCF!C27</f>
+        <v/>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>↳ DCF base case</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>FY2026E diluted EPS (guidance midpoint)</t>
         </is>
       </c>
-      <c r="C6" s="60" t="n">
+      <c r="C7" s="61" t="n">
         <v>9.609999999999999</v>
       </c>
-      <c r="D6" s="58" t="inlineStr">
+      <c r="D7" s="59" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Cash &amp; equivalents</t>
         </is>
       </c>
-      <c r="C7" s="45" t="n">
+      <c r="C8" s="45" t="n">
         <v>1807202</v>
       </c>
-      <c r="D7" s="58" t="inlineStr">
+      <c r="D8" s="59" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Diluted shares (000)</t>
         </is>
       </c>
-      <c r="C8" s="45" t="n">
+      <c r="C9" s="45" t="n">
         <v>111380</v>
       </c>
-      <c r="D8" s="58" t="inlineStr">
+      <c r="D9" s="59" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C9" s="60" t="n">
+      <c r="C10" s="61" t="n">
         <v>100</v>
       </c>
-      <c r="D9" s="58" t="inlineStr">
+      <c r="D10" s="59" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="70" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="71" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current EV / EBITDA</t>
         </is>
       </c>
-      <c r="C10" s="75">
-        <f>(C9*C8-C7)/C5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="70" t="inlineStr">
+      <c r="C11" s="76">
+        <f>(C10*C9-C8)/C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="71" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current P / E (FY2026E)</t>
         </is>
       </c>
-      <c r="C11" s="75">
-        <f>C9/C6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="C12" s="76">
+        <f>C10/C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>EXIT MULTIPLE BUILD — FY2030E TERMINAL YEAR</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="70" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="71" t="inlineStr">
         <is>
           <t>Peer / reference EV/EBITDA (forward / illustrative)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="76" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="77" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C15" s="77" t="inlineStr">
+      <c r="C16" s="78" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="D15" s="76" t="inlineStr">
+      <c r="D16" s="77" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="E15" s="76" t="inlineStr">
+      <c r="E16" s="77" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>lululemon (LULU) — current</t>
         </is>
       </c>
-      <c r="C16" s="78">
-        <f>(C9*C8-C7)/C5</f>
-        <v/>
-      </c>
-      <c r="D16" s="37" t="inlineStr">
+      <c r="C17" s="79">
+        <f>(C10*C9-C8)/C5</f>
+        <v/>
+      </c>
+      <c r="D17" s="37" t="inlineStr">
         <is>
           <t>Distressed trough multiple on FY2025A EBITDA</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E17" s="49" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>Nike (NKE)</t>
         </is>
       </c>
-      <c r="C17" s="79" t="n">
+      <c r="C18" s="80" t="n">
         <v>18</v>
       </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>Nike ~18x forward EV/EBITDA illustrative; mature global athletic benchmark with slower growth than LULU peak.</t>
         </is>
       </c>
-      <c r="E17" s="18" t="inlineStr">
-        <is>
-          <t>Yahoo Finance: NKE statistics</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="E18" s="17">
+        <f>HYPERLINK("https://finance.yahoo.com/quote/NKE/key-statistics/","↳ Yahoo Finance: NKE statistics")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Deckers (DECK)</t>
         </is>
       </c>
-      <c r="C18" s="79" t="n">
+      <c r="C19" s="80" t="n">
         <v>15</v>
       </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>Deckers ~15x reference; premium footwear peer with HOKA/UGG momentum and strong brand heat.</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>Yahoo Finance: DECK statistics</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="E19" s="17">
+        <f>HYPERLINK("https://finance.yahoo.com/quote/DECK/key-statistics/","↳ Yahoo Finance: DECK statistics")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>On Holding (ONON)</t>
         </is>
       </c>
-      <c r="C19" s="79" t="n">
+      <c r="C20" s="80" t="n">
         <v>25</v>
       </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>On Holding ~25x; high-growth athletic peer setting upper bound for premium positioning and white space.</t>
         </is>
       </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>Yahoo Finance: ONON statistics</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="E20" s="17">
+        <f>HYPERLINK("https://finance.yahoo.com/quote/ONON/key-statistics/","↳ Yahoo Finance: ONON statistics")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>adidas (ADS)</t>
         </is>
       </c>
-      <c r="C20" s="79" t="n">
+      <c r="C21" s="80" t="n">
         <v>12</v>
       </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>adidas ~12x; global incumbent in restructuring with moderate growth and complex brand portfolio.</t>
         </is>
       </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>Yahoo Finance: ADS.DE statistics</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="E21" s="17">
+        <f>HYPERLINK("https://finance.yahoo.com/quote/ADS.DE/key-statistics/","↳ Yahoo Finance: ADS.DE statistics")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>V.F. Corp (VFC)</t>
         </is>
       </c>
-      <c r="C21" s="79" t="n">
+      <c r="C22" s="80" t="n">
         <v>10</v>
       </c>
-      <c r="D21" s="17" t="inlineStr">
+      <c r="D22" s="19" t="inlineStr">
         <is>
           <t>VFC ~10x; challenged multi-brand apparel operator representing lower bound for scaled apparel peers.</t>
         </is>
       </c>
-      <c r="E21" s="18" t="inlineStr">
-        <is>
-          <t>Yahoo Finance: VFC statistics</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="E22" s="17">
+        <f>HYPERLINK("https://finance.yahoo.com/quote/VFC/key-statistics/","↳ Yahoo Finance: VFC statistics")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>Terminal multiple selection (DCF exit method)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Gordon Growth implied exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="C24" s="57">
+      <c r="C25" s="58">
         <f>DCF!C29</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="68" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="69" t="inlineStr">
         <is>
           <t>Selected exit multiple (base case)</t>
         </is>
       </c>
-      <c r="C25" s="66">
+      <c r="C26" s="67">
         <f>DCF!C43</f>
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="15" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>Spread (selected − Gordon implied)</t>
         </is>
       </c>
-      <c r="C26" s="57">
-        <f>C25-C24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="68" t="inlineStr">
+      <c r="C27" s="58">
+        <f>C26-C25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="69" t="inlineStr">
         <is>
           <t>Rationale for 8.0x</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="29" t="inlineStr">
-        <is>
-          <t>•  Above current LULU (~3.5x) — assumes partial recovery from trough, not full re-rating</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="29" t="inlineStr">
         <is>
-          <t>•  Above comps football-field high (7.5x on FY2025A) — terminal year has higher EBITDA &amp; normalized margins</t>
+          <t>•  Mid-point of terminal football field (6.5–9.5x on FY2030E EBITDA) — 8.0x sits between bear and bull exit</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="29" t="inlineStr">
         <is>
-          <t>•  Below premium-growth peers (ONON ~25x, DECK ~15x) — reflects Americas maturity</t>
+          <t>•  Above Gordon-implied exit (~7x) — ~1 turn buffer vs perpetuity math on terminal FCF</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="29" t="inlineStr">
         <is>
-          <t>•  ~1 turn above Gordon-implied exit multiple — conservative buffer vs perpetuity math</t>
+          <t>•  Below premium-growth peers (ONON ~25x, DECK ~15x) — reflects Americas maturity at terminal</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="29" t="inlineStr">
         <is>
-          <t>•  Well below historical LULU peak multiples (20–30x) — avoids heroic assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="14" t="inlineStr">
-        <is>
-          <t>Methodology / multiple ranges (FY2025A — football field)</t>
+          <t>•  Above current LULU (~3.5x on FY2025A) — assumes partial recovery, not full re-rating to historical peaks</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="29" t="inlineStr">
+        <is>
+          <t>•  Peer simple avg ~16x not used — terminal multiple discounted for lower terminal growth vs ONON/NKE</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="76" t="inlineStr">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>Methodology / multiple ranges (FY2030E terminal EBITDA — football field)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="77" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="C35" s="77" t="inlineStr">
+      <c r="C36" s="78" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="D35" s="77" t="inlineStr">
+      <c r="D36" s="78" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="E35" s="77" t="inlineStr">
+      <c r="E36" s="78" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="F35" s="77" t="inlineStr">
+      <c r="F36" s="78" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
       </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="15" t="inlineStr">
-        <is>
-          <t>EV / EBITDA (FY2025A)</t>
-        </is>
-      </c>
-      <c r="C36" s="79" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="D36" s="79" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="E36" s="80">
-        <f>(C5*C36+C7)/C8</f>
-        <v/>
-      </c>
-      <c r="F36" s="80">
-        <f>(C5*D36+C7)/C8</f>
-        <v/>
-      </c>
-      <c r="G36" s="17" t="inlineStr">
-        <is>
-          <t>4.5x EV/EBITDA low case on FY2025A; distressed trough pricing near current market de-rating.</t>
+      <c r="G36" s="81" t="inlineStr">
+        <is>
+          <t>Lo justification</t>
         </is>
       </c>
       <c r="H36" s="81" t="inlineStr">
         <is>
-          <t>7.5x EV/EBITDA high case on FY2025A; partial recovery before terminal year, below historical peaks.</t>
-        </is>
-      </c>
-      <c r="I36" s="18" t="inlineStr">
-        <is>
-          <t>Yahoo Finance: LULU EV/EBITDA</t>
-        </is>
-      </c>
-      <c r="J36" s="82" t="inlineStr">
-        <is>
-          <t>Macrotrends: LULU EV/EBITDA history</t>
+          <t>Hi justification</t>
+        </is>
+      </c>
+      <c r="I36" s="81" t="inlineStr">
+        <is>
+          <t>Lo source</t>
+        </is>
+      </c>
+      <c r="J36" s="81" t="inlineStr">
+        <is>
+          <t>Hi source</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="15" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>EV / EBITDA (FY2030E terminal)</t>
+        </is>
+      </c>
+      <c r="C37" s="80" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D37" s="80" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E37" s="82">
+        <f>(C6*C37+C8)/C9</f>
+        <v/>
+      </c>
+      <c r="F37" s="82">
+        <f>(C6*D37+C8)/C9</f>
+        <v/>
+      </c>
+      <c r="G37" s="19" t="inlineStr">
+        <is>
+          <t>6.5x on FY2030E terminal EBITDA; bear exit below Gordon-implied ~7x; brackets DCF downside.</t>
+        </is>
+      </c>
+      <c r="H37" s="83" t="inlineStr">
+        <is>
+          <t>9.5x on FY2030E terminal EBITDA; bull exit above 8.0x DCF base; still below peer median ~15x.</t>
+        </is>
+      </c>
+      <c r="I37" s="17">
+        <f>HYPERLINK("https://finance.yahoo.com/quote/LULU/key-statistics/","↳ Yahoo Finance: LULU EV/EBITDA")</f>
+        <v/>
+      </c>
+      <c r="J37" s="84">
+        <f>HYPERLINK("https://www.macrotrends.net/stocks/charts/LULU/lululemon-athletica/enterprise-value-ebitda","↳ Macrotrends: LULU EV/EBITDA history")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="69" t="inlineStr">
+        <is>
+          <t>DCF exit method (8.0x on FY2030E EBITDA)</t>
+        </is>
+      </c>
+      <c r="C38" s="85">
+        <f>DCF!C43</f>
+        <v/>
+      </c>
+      <c r="E38" s="86">
+        <f>(C6*C38+C8)/C9</f>
+        <v/>
+      </c>
+      <c r="I38" s="28" t="inlineStr">
+        <is>
+          <t>↳ DCF exit multiple</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
         <is>
           <t>P / E (FY2026E EPS)</t>
         </is>
       </c>
-      <c r="C37" s="79" t="n">
+      <c r="C39" s="80" t="n">
         <v>10</v>
       </c>
-      <c r="D37" s="79" t="n">
+      <c r="D39" s="80" t="n">
         <v>18</v>
       </c>
-      <c r="E37" s="80">
-        <f>C6*C37</f>
-        <v/>
-      </c>
-      <c r="F37" s="80">
-        <f>C6*D37</f>
-        <v/>
-      </c>
-      <c r="G37" s="17" t="inlineStr">
+      <c r="E39" s="82">
+        <f>C7*C39</f>
+        <v/>
+      </c>
+      <c r="F39" s="82">
+        <f>C7*D39</f>
+        <v/>
+      </c>
+      <c r="G39" s="19" t="inlineStr">
         <is>
           <t>10x P/E low on FY2026E EPS; trough earnings multiple after guidance reset and sentiment de-rating.</t>
         </is>
       </c>
-      <c r="H37" s="81" t="inlineStr">
+      <c r="H39" s="83" t="inlineStr">
         <is>
           <t>18x P/E high on FY2026E EPS; modest recovery case still below historical premium LULU multiples.</t>
         </is>
       </c>
-      <c r="I37" s="18" t="inlineStr">
-        <is>
-          <t>Yahoo Finance: LULU P/E (FY26E)</t>
-        </is>
-      </c>
-      <c r="J37" s="82" t="inlineStr">
+      <c r="I39" s="17">
+        <f>HYPERLINK("https://finance.yahoo.com/quote/LULU/key-statistics/","↳ Yahoo Finance: LULU P/E (FY26E)")</f>
+        <v/>
+      </c>
+      <c r="J39" s="84" t="inlineStr">
         <is>
           <t>Yahoo Finance: NKE P/E (peer benchmark)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="15" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="C38" s="83" t="inlineStr">
+      <c r="C40" s="87" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D38" s="83" t="inlineStr">
+      <c r="D40" s="87" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E38" s="80">
+      <c r="E40" s="82">
         <f>Scenarios!C58</f>
         <v/>
       </c>
-      <c r="F38" s="80">
+      <c r="F40" s="82">
         <f>Scenarios!E58</f>
         <v/>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="84" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="88" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C40" s="85" t="n">
+      <c r="C42" s="89" t="n">
         <v>100</v>
       </c>
-      <c r="D40" s="58" t="inlineStr">
+      <c r="D42" s="59" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="37" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="37" t="inlineStr">
         <is>
           <t>Note: peer set includes NKE, DECK, ONON, adidas, VFC; multiples are analyst ranges (red).</t>
         </is>
@@ -4356,26 +4373,20 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId22"/>
+    <hyperlink ref="D6" location="'DCF'!C27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId11"/>
+    <hyperlink ref="I38" location="'DCF'!C43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix broken source hyperlinks in LULU Excel models
Replace dead investor.lululemon.com and macrotrends URLs with working
corporate press release, StockAnalysis, and SEC EDGAR viewer links.
Rebuild DCF and 3-statement workbooks with corrected assumption sources.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1487,7 +1487,7 @@
       </c>
       <c r="G6" s="19" t="inlineStr">
         <is>
-          <t>LULU Q2 FY2026 guidance / 10-K margins</t>
+          <t>LULU Q2 FY2026 earnings release</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>BEA: Real GDP (FRED GDPC1)</t>
+          <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="K7" s="19" t="inlineStr">
         <is>
-          <t>LULU Q2 FY2026 guidance / 10-K margins</t>
+          <t>LULU Q2 FY2026 earnings release</t>
         </is>
       </c>
       <c r="L7" s="49" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="K26" s="19" t="inlineStr">
         <is>
-          <t>BEA: Real GDP (FRED GDPC1)</t>
+          <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="K43" s="19" t="inlineStr">
         <is>
-          <t>Macrotrends: LULU EV/EBITDA history</t>
+          <t>StockAnalysis: LULU EV/EBITDA</t>
         </is>
       </c>
       <c r="L43" s="64" t="inlineStr">
@@ -4136,7 +4136,7 @@
       </c>
       <c r="F21" s="19" t="inlineStr">
         <is>
-          <t>Yahoo Finance: ADS.DE statistics</t>
+          <t>Yahoo Finance: adidas (ADDYY)</t>
         </is>
       </c>
     </row>
@@ -4323,7 +4323,7 @@
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>Yahoo Finance: LULU EV/EBITDA</t>
+          <t>StockAnalysis: LULU EV/EBITDA</t>
         </is>
       </c>
       <c r="I37" s="84" t="inlineStr">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="J37" s="85" t="inlineStr">
         <is>
-          <t>Macrotrends: LULU EV/EBITDA history</t>
+          <t>StockAnalysis: LULU valuation</t>
         </is>
       </c>
     </row>
@@ -4384,7 +4384,7 @@
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>Yahoo Finance: LULU P/E (FY26E)</t>
+          <t>Yahoo Finance: LULU P/E</t>
         </is>
       </c>
       <c r="I39" s="84" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="J39" s="85" t="inlineStr">
         <is>
-          <t>Yahoo Finance: NKE P/E (peer benchmark)</t>
+          <t>Yahoo Finance: NKE P/E (peer)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document Scenarios operating-margin source as 18.8% minus 560bps tariffs
FY26 13.9% is derived from the Q2 print (clean OM 13.2%), not from the 13% YoY dollar decline.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1513,17 +1513,17 @@
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>13.9% is a FY2026E model assumption — not the 13% YoY drop in Q2 operating income. Q2 OM was 18.8% (incl. 560bps tariffs); ex-tariff ~13.2%.</t>
+          <t>FY26 13.9% is derived: Q2 OM 18.8% minus 560bps tariff refunds = 13.2% clean; we set base slightly above that run-rate.</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>LULU Q2 FY2026 earnings release</t>
+          <t>Q2 FY2026 release: OM 18.8% less 560bps tariffs</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "decreased 190 basis points to 18.8%" — that is Q2 operating margin. "decreased 13%" is YoY $ decline in income from operations, NOT the margin. Model FY26 EBIT margin 13.9% (assumption; Q2 ex-tariff OM ≈ 18.8% − 560bps = 13.2%)</t>
+          <t>1) Ctrl+F "18.8%" = Q2 operating margin. 2) Ctrl+F "560 basis points" = tariff add. 3) Clean Q2 = 18.8% − 5.6% = 13.2%. Model FY26 base 13.9% sits just above that. Do not use "decreased 13%" — that is the YoY $ decline in income from operations.</t>
         </is>
       </c>
       <c r="F6" s="20" t="n">
@@ -1544,17 +1544,17 @@
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>15.5% FY2030 EBIT margin assumes partial recovery; still materially below ~20–24% peak operating margins.</t>
+          <t>FY30 15.5% is a recovery assumption vs FY25 10-K OM 19.9% (2,210,615 / 11,102,600); still well below FY24 peak ~23.7%.</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>LULU historical EBIT margins (10-K)</t>
+          <t>FY2025 10-K: Income from operations / revenue</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Income from operations" → 2,210,615 ÷ "Net revenue" 11,102,600 = 19.9% FY25</t>
+          <t>Ctrl+F "Income from operations" → 2,210,615 and "Net revenue" → 11,102,600. FY25 OM = 19.9%. Model FY30 15.5% is a partial-recovery assumption, not a reported figure.</t>
         </is>
       </c>
       <c r="F7" s="20" t="n">
@@ -2812,20 +2812,20 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>13.9% is a FY2026E model assumption — not the 13% YoY drop in Q2 operating income. Q2 OM was 18.8% (incl. 560bps tariffs); ex-tariff ~13.2%.
-Also: 15.5% FY2030 EBIT margin assumes partial recovery; still materially below ~20–24% peak operating margins.</t>
+          <t>FY26 13.9% is derived: Q2 OM 18.8% minus 560bps tariff refunds = 13.2% clean; we set base slightly above that run-rate.
+Also: FY30 15.5% is a recovery assumption vs FY25 10-K OM 19.9% (2,210,615 / 11,102,600); still well below FY24 peak ~23.7%.</t>
         </is>
       </c>
       <c r="C7" s="47" t="inlineStr">
         <is>
-          <t>LULU Q2 FY2026 earnings release
-Also: LULU historical EBIT margins (10-K)</t>
+          <t>Q2 FY2026 release: OM 18.8% less 560bps tariffs
+Also: FY2025 10-K: Income from operations / revenue</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "decreased 190 basis points to 18.8%" — that is Q2 operating margin. "decreased 13%" is YoY $ decline in income from operations, NOT the margin. Model FY26 EBIT margin 13.9% (assumption; Q2 ex-tariff OM ≈ 18.8% − 560bps = 13.2%)
-Also: Ctrl+F "Income from operations" → 2,210,615 ÷ "Net revenue" 11,102,600 = 19.9% FY25</t>
+          <t>1) Ctrl+F "18.8%" = Q2 operating margin. 2) Ctrl+F "560 basis points" = tariff add. 3) Clean Q2 = 18.8% − 5.6% = 13.2%. Model FY26 base 13.9% sits just above that. Do not use "decreased 13%" — that is the YoY $ decline in income from operations.
+Also: Ctrl+F "Income from operations" → 2,210,615 and "Net revenue" → 11,102,600. FY25 OM = 19.9%. Model FY30 15.5% is a partial-recovery assumption, not a reported figure.</t>
         </is>
       </c>
       <c r="F7" s="48">

</xml_diff>

<commit_message>
Split AR out as its own DCF NWC line
Accounts receivable is now 1.7% of sales on the DCF NWC build, with other NWC at 5.8% of Δrevenue so the two still add to 7.5%.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1387,7 +1387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1778,83 +1778,95 @@
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>NWC build % of Δrevenue</t>
+          <t>AR % of revenue (NWC)</t>
         </is>
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>7.5% of Δsales is operating NWC: AR + inventory + other CA − AP − accrued. AR is on the 10-K ($190,657); not omitted.</t>
+          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Own DCF NWC line; wholesale / marketplace mix.</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
+          <t>LULU FY2025 10-K: Accounts receivable, net</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. This is the DCF AR / NWC line.</t>
+        </is>
+      </c>
+      <c r="F14" s="20" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="G14" s="20" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="H14" s="20" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Other NWC (ex-AR) % of Δrevenue</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>5.8% of Δsales is other NWC (Inv + OCA − AP − accrued). AR is the 1.7% line above, not inside this residual. 1.7+5.8=7.5%.</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
           <t>LULU BS/IS historical (10-K)</t>
         </is>
       </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Accounts receivable, net" → 190,657. Ctrl+F "Inventories" → 1,700,753. Ctrl+F "Accounts payable" → 331,421. Ctrl+F "Accrued liabilities and other" → 662,982. NWC = AR + Inv + other CA − AP − accrued; 7.5% of Δsales.</t>
-        </is>
-      </c>
-      <c r="F14" s="20" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="G14" s="20" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="H14" s="20" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Other NWC ex-AR. Ctrl+F "Inventories" → 1,700,753 | "Accounts payable" → 331,421 | "Accrued liabilities and other" → 662,982. 5.8% of Δsales; AR is the 1.7% line, not in this residual.</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="G15" s="20" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>5-year forecast paths (by scenario)</t>
         </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Revenue – year 1</t>
-        </is>
-      </c>
-      <c r="F17" s="32">
-        <f>11102600*(1+F4)</f>
-        <v/>
-      </c>
-      <c r="G17" s="32">
-        <f>11102600*(1+G4)</f>
-        <v/>
-      </c>
-      <c r="H17" s="32">
-        <f>11102600*(1+H4)</f>
-        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Revenue – year 2</t>
+          <t xml:space="preserve">  Revenue – year 1</t>
         </is>
       </c>
       <c r="F18" s="32">
-        <f>F17*(1+F5)</f>
+        <f>11102600*(1+F4)</f>
         <v/>
       </c>
       <c r="G18" s="32">
-        <f>G17*(1+G5)</f>
+        <f>11102600*(1+G4)</f>
         <v/>
       </c>
       <c r="H18" s="32">
-        <f>H17*(1+H5)</f>
+        <f>11102600*(1+H4)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Revenue – year 3</t>
+          <t xml:space="preserve">  Revenue – year 2</t>
         </is>
       </c>
       <c r="F19" s="32">
@@ -1873,7 +1885,7 @@
     <row r="20">
       <c r="A20" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Revenue – year 4</t>
+          <t xml:space="preserve">  Revenue – year 3</t>
         </is>
       </c>
       <c r="F20" s="32">
@@ -1892,7 +1904,7 @@
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Revenue – year 5</t>
+          <t xml:space="preserve">  Revenue – year 4</t>
         </is>
       </c>
       <c r="F21" s="32">
@@ -1911,140 +1923,140 @@
     <row r="22">
       <c r="A22" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Clean EBIT margin – year 1</t>
-        </is>
-      </c>
-      <c r="F22" s="33">
-        <f>F6+(F8-F6)*0/4</f>
-        <v/>
-      </c>
-      <c r="G22" s="33">
-        <f>G6+(G8-G6)*0/4</f>
-        <v/>
-      </c>
-      <c r="H22" s="33">
-        <f>H6+(H8-H6)*0/4</f>
+          <t xml:space="preserve">  Revenue – year 5</t>
+        </is>
+      </c>
+      <c r="F22" s="32">
+        <f>F21*(1+F5)</f>
+        <v/>
+      </c>
+      <c r="G22" s="32">
+        <f>G21*(1+G5)</f>
+        <v/>
+      </c>
+      <c r="H22" s="32">
+        <f>H21*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Clean EBIT margin – year 2</t>
+          <t xml:space="preserve">  Clean EBIT margin – year 1</t>
         </is>
       </c>
       <c r="F23" s="33">
-        <f>F6+(F8-F6)*1/4</f>
+        <f>F6+(F8-F6)*0/4</f>
         <v/>
       </c>
       <c r="G23" s="33">
-        <f>G6+(G8-G6)*1/4</f>
+        <f>G6+(G8-G6)*0/4</f>
         <v/>
       </c>
       <c r="H23" s="33">
-        <f>H6+(H8-H6)*1/4</f>
+        <f>H6+(H8-H6)*0/4</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Clean EBIT margin – year 3</t>
+          <t xml:space="preserve">  Clean EBIT margin – year 2</t>
         </is>
       </c>
       <c r="F24" s="33">
-        <f>F6+(F8-F6)*2/4</f>
+        <f>F6+(F8-F6)*1/4</f>
         <v/>
       </c>
       <c r="G24" s="33">
-        <f>G6+(G8-G6)*2/4</f>
+        <f>G6+(G8-G6)*1/4</f>
         <v/>
       </c>
       <c r="H24" s="33">
-        <f>H6+(H8-H6)*2/4</f>
+        <f>H6+(H8-H6)*1/4</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Clean EBIT margin – year 4</t>
+          <t xml:space="preserve">  Clean EBIT margin – year 3</t>
         </is>
       </c>
       <c r="F25" s="33">
-        <f>F6+(F8-F6)*3/4</f>
+        <f>F6+(F8-F6)*2/4</f>
         <v/>
       </c>
       <c r="G25" s="33">
-        <f>G6+(G8-G6)*3/4</f>
+        <f>G6+(G8-G6)*2/4</f>
         <v/>
       </c>
       <c r="H25" s="33">
-        <f>H6+(H8-H6)*3/4</f>
+        <f>H6+(H8-H6)*2/4</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Clean EBIT margin – year 5</t>
+          <t xml:space="preserve">  Clean EBIT margin – year 4</t>
         </is>
       </c>
       <c r="F26" s="33">
-        <f>F6+(F8-F6)*4/4</f>
+        <f>F6+(F8-F6)*3/4</f>
         <v/>
       </c>
       <c r="G26" s="33">
-        <f>G6+(G8-G6)*4/4</f>
+        <f>G6+(G8-G6)*3/4</f>
         <v/>
       </c>
       <c r="H26" s="33">
-        <f>H6+(H8-H6)*4/4</f>
+        <f>H6+(H8-H6)*3/4</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT – year 1</t>
-        </is>
-      </c>
-      <c r="F27" s="32">
-        <f>F17*F22+F7</f>
-        <v/>
-      </c>
-      <c r="G27" s="32">
-        <f>G17*G22+G7</f>
-        <v/>
-      </c>
-      <c r="H27" s="32">
-        <f>H17*H22+H7</f>
+          <t xml:space="preserve">  Clean EBIT margin – year 5</t>
+        </is>
+      </c>
+      <c r="F27" s="33">
+        <f>F6+(F8-F6)*4/4</f>
+        <v/>
+      </c>
+      <c r="G27" s="33">
+        <f>G6+(G8-G6)*4/4</f>
+        <v/>
+      </c>
+      <c r="H27" s="33">
+        <f>H6+(H8-H6)*4/4</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT – year 2</t>
+          <t xml:space="preserve">  EBIT – year 1</t>
         </is>
       </c>
       <c r="F28" s="32">
-        <f>F18*F23</f>
+        <f>F18*F23+F7</f>
         <v/>
       </c>
       <c r="G28" s="32">
-        <f>G18*G23</f>
+        <f>G18*G23+G7</f>
         <v/>
       </c>
       <c r="H28" s="32">
-        <f>H18*H23</f>
+        <f>H18*H23+H7</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT – year 3</t>
+          <t xml:space="preserve">  EBIT – year 2</t>
         </is>
       </c>
       <c r="F29" s="32">
@@ -2063,7 +2075,7 @@
     <row r="30">
       <c r="A30" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT – year 4</t>
+          <t xml:space="preserve">  EBIT – year 3</t>
         </is>
       </c>
       <c r="F30" s="32">
@@ -2082,7 +2094,7 @@
     <row r="31">
       <c r="A31" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EBIT – year 5</t>
+          <t xml:space="preserve">  EBIT – year 4</t>
         </is>
       </c>
       <c r="F31" s="32">
@@ -2101,26 +2113,26 @@
     <row r="32">
       <c r="A32" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOPAT – year 1</t>
+          <t xml:space="preserve">  EBIT – year 5</t>
         </is>
       </c>
       <c r="F32" s="32">
-        <f>F27*(1-F11)</f>
+        <f>F22*F27</f>
         <v/>
       </c>
       <c r="G32" s="32">
-        <f>G27*(1-G11)</f>
+        <f>G22*G27</f>
         <v/>
       </c>
       <c r="H32" s="32">
-        <f>H27*(1-H11)</f>
+        <f>H22*H27</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOPAT – year 2</t>
+          <t xml:space="preserve">  NOPAT – year 1</t>
         </is>
       </c>
       <c r="F33" s="32">
@@ -2139,7 +2151,7 @@
     <row r="34">
       <c r="A34" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOPAT – year 3</t>
+          <t xml:space="preserve">  NOPAT – year 2</t>
         </is>
       </c>
       <c r="F34" s="32">
@@ -2158,7 +2170,7 @@
     <row r="35">
       <c r="A35" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOPAT – year 4</t>
+          <t xml:space="preserve">  NOPAT – year 3</t>
         </is>
       </c>
       <c r="F35" s="32">
@@ -2177,7 +2189,7 @@
     <row r="36">
       <c r="A36" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOPAT – year 5</t>
+          <t xml:space="preserve">  NOPAT – year 4</t>
         </is>
       </c>
       <c r="F36" s="32">
@@ -2196,26 +2208,26 @@
     <row r="37">
       <c r="A37" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A – year 1</t>
+          <t xml:space="preserve">  NOPAT – year 5</t>
         </is>
       </c>
       <c r="F37" s="32">
-        <f>F17*F12</f>
+        <f>F32*(1-F11)</f>
         <v/>
       </c>
       <c r="G37" s="32">
-        <f>G17*G12</f>
+        <f>G32*(1-G11)</f>
         <v/>
       </c>
       <c r="H37" s="32">
-        <f>H17*H12</f>
+        <f>H32*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A – year 2</t>
+          <t xml:space="preserve">  D&amp;A – year 1</t>
         </is>
       </c>
       <c r="F38" s="32">
@@ -2234,7 +2246,7 @@
     <row r="39">
       <c r="A39" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A – year 3</t>
+          <t xml:space="preserve">  D&amp;A – year 2</t>
         </is>
       </c>
       <c r="F39" s="32">
@@ -2253,7 +2265,7 @@
     <row r="40">
       <c r="A40" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A – year 4</t>
+          <t xml:space="preserve">  D&amp;A – year 3</t>
         </is>
       </c>
       <c r="F40" s="32">
@@ -2272,7 +2284,7 @@
     <row r="41">
       <c r="A41" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A – year 5</t>
+          <t xml:space="preserve">  D&amp;A – year 4</t>
         </is>
       </c>
       <c r="F41" s="32">
@@ -2291,26 +2303,26 @@
     <row r="42">
       <c r="A42" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex – year 1</t>
+          <t xml:space="preserve">  D&amp;A – year 5</t>
         </is>
       </c>
       <c r="F42" s="32">
-        <f>F17*F13</f>
+        <f>F22*F12</f>
         <v/>
       </c>
       <c r="G42" s="32">
-        <f>G17*G13</f>
+        <f>G22*G12</f>
         <v/>
       </c>
       <c r="H42" s="32">
-        <f>H17*H13</f>
+        <f>H22*H12</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex – year 2</t>
+          <t xml:space="preserve">  Capex – year 1</t>
         </is>
       </c>
       <c r="F43" s="32">
@@ -2329,7 +2341,7 @@
     <row r="44">
       <c r="A44" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex – year 3</t>
+          <t xml:space="preserve">  Capex – year 2</t>
         </is>
       </c>
       <c r="F44" s="32">
@@ -2348,7 +2360,7 @@
     <row r="45">
       <c r="A45" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex – year 4</t>
+          <t xml:space="preserve">  Capex – year 3</t>
         </is>
       </c>
       <c r="F45" s="32">
@@ -2367,7 +2379,7 @@
     <row r="46">
       <c r="A46" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex – year 5</t>
+          <t xml:space="preserve">  Capex – year 4</t>
         </is>
       </c>
       <c r="F46" s="32">
@@ -2386,252 +2398,556 @@
     <row r="47">
       <c r="A47" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔNWC – year 1</t>
+          <t xml:space="preserve">  Capex – year 5</t>
         </is>
       </c>
       <c r="F47" s="32">
-        <f>F14*(F17-11102600)</f>
+        <f>F22*F13</f>
         <v/>
       </c>
       <c r="G47" s="32">
-        <f>G14*(G17-11102600)</f>
+        <f>G22*G13</f>
         <v/>
       </c>
       <c r="H47" s="32">
-        <f>H14*(H17-11102600)</f>
+        <f>H22*H13</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔNWC – year 2</t>
+          <t xml:space="preserve">  Accounts receivable – year 1</t>
         </is>
       </c>
       <c r="F48" s="32">
-        <f>F14*(F18-F17)</f>
+        <f>F18*F14</f>
         <v/>
       </c>
       <c r="G48" s="32">
-        <f>G14*(G18-G17)</f>
+        <f>G18*G14</f>
         <v/>
       </c>
       <c r="H48" s="32">
-        <f>H14*(H18-H17)</f>
+        <f>H18*H14</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔNWC – year 3</t>
+          <t xml:space="preserve">  Accounts receivable – year 2</t>
         </is>
       </c>
       <c r="F49" s="32">
-        <f>F14*(F19-F18)</f>
+        <f>F19*F14</f>
         <v/>
       </c>
       <c r="G49" s="32">
-        <f>G14*(G19-G18)</f>
+        <f>G19*G14</f>
         <v/>
       </c>
       <c r="H49" s="32">
-        <f>H14*(H19-H18)</f>
+        <f>H19*H14</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔNWC – year 4</t>
+          <t xml:space="preserve">  Accounts receivable – year 3</t>
         </is>
       </c>
       <c r="F50" s="32">
-        <f>F14*(F20-F19)</f>
+        <f>F20*F14</f>
         <v/>
       </c>
       <c r="G50" s="32">
-        <f>G14*(G20-G19)</f>
+        <f>G20*G14</f>
         <v/>
       </c>
       <c r="H50" s="32">
-        <f>H14*(H20-H19)</f>
+        <f>H20*H14</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔNWC – year 5</t>
+          <t xml:space="preserve">  Accounts receivable – year 4</t>
         </is>
       </c>
       <c r="F51" s="32">
-        <f>F14*(F21-F20)</f>
+        <f>F21*F14</f>
         <v/>
       </c>
       <c r="G51" s="32">
-        <f>G14*(G21-G20)</f>
+        <f>G21*G14</f>
         <v/>
       </c>
       <c r="H51" s="32">
-        <f>H14*(H21-H20)</f>
+        <f>H21*H14</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 1</t>
+          <t xml:space="preserve">  Accounts receivable – year 5</t>
         </is>
       </c>
       <c r="F52" s="32">
-        <f>F32+F37-F42-F47</f>
+        <f>F22*F14</f>
         <v/>
       </c>
       <c r="G52" s="32">
-        <f>G32+G37-G42-G47</f>
+        <f>G22*G14</f>
         <v/>
       </c>
       <c r="H52" s="32">
-        <f>H32+H37-H42-H47</f>
+        <f>H22*H14</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 2</t>
+          <t xml:space="preserve">  ΔAR – year 1</t>
         </is>
       </c>
       <c r="F53" s="32">
-        <f>F33+F38-F43-F48</f>
+        <f>F48-190657</f>
         <v/>
       </c>
       <c r="G53" s="32">
-        <f>G33+G38-G43-G48</f>
+        <f>G48-190657</f>
         <v/>
       </c>
       <c r="H53" s="32">
-        <f>H33+H38-H43-H48</f>
+        <f>H48-190657</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 3</t>
+          <t xml:space="preserve">  ΔAR – year 2</t>
         </is>
       </c>
       <c r="F54" s="32">
-        <f>F34+F39-F44-F49</f>
+        <f>F49-F48</f>
         <v/>
       </c>
       <c r="G54" s="32">
-        <f>G34+G39-G44-G49</f>
+        <f>G49-G48</f>
         <v/>
       </c>
       <c r="H54" s="32">
-        <f>H34+H39-H44-H49</f>
+        <f>H49-H48</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unlevered FCF – year 4</t>
+          <t xml:space="preserve">  ΔAR – year 3</t>
         </is>
       </c>
       <c r="F55" s="32">
-        <f>F35+F40-F45-F50</f>
+        <f>F50-F49</f>
         <v/>
       </c>
       <c r="G55" s="32">
-        <f>G35+G40-G45-G50</f>
+        <f>G50-G49</f>
         <v/>
       </c>
       <c r="H55" s="32">
-        <f>H35+H40-H45-H50</f>
+        <f>H50-H49</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="31" t="inlineStr">
         <is>
+          <t xml:space="preserve">  ΔAR – year 4</t>
+        </is>
+      </c>
+      <c r="F56" s="32">
+        <f>F51-F50</f>
+        <v/>
+      </c>
+      <c r="G56" s="32">
+        <f>G51-G50</f>
+        <v/>
+      </c>
+      <c r="H56" s="32">
+        <f>H51-H50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ΔAR – year 5</t>
+        </is>
+      </c>
+      <c r="F57" s="32">
+        <f>F52-F51</f>
+        <v/>
+      </c>
+      <c r="G57" s="32">
+        <f>G52-G51</f>
+        <v/>
+      </c>
+      <c r="H57" s="32">
+        <f>H52-H51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Other ΔNWC (ex-AR) – year 1</t>
+        </is>
+      </c>
+      <c r="F58" s="32">
+        <f>F15*(F18-11102600)</f>
+        <v/>
+      </c>
+      <c r="G58" s="32">
+        <f>G15*(G18-11102600)</f>
+        <v/>
+      </c>
+      <c r="H58" s="32">
+        <f>H15*(H18-11102600)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Other ΔNWC (ex-AR) – year 2</t>
+        </is>
+      </c>
+      <c r="F59" s="32">
+        <f>F15*(F19-F18)</f>
+        <v/>
+      </c>
+      <c r="G59" s="32">
+        <f>G15*(G19-G18)</f>
+        <v/>
+      </c>
+      <c r="H59" s="32">
+        <f>H15*(H19-H18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Other ΔNWC (ex-AR) – year 3</t>
+        </is>
+      </c>
+      <c r="F60" s="32">
+        <f>F15*(F20-F19)</f>
+        <v/>
+      </c>
+      <c r="G60" s="32">
+        <f>G15*(G20-G19)</f>
+        <v/>
+      </c>
+      <c r="H60" s="32">
+        <f>H15*(H20-H19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Other ΔNWC (ex-AR) – year 4</t>
+        </is>
+      </c>
+      <c r="F61" s="32">
+        <f>F15*(F21-F20)</f>
+        <v/>
+      </c>
+      <c r="G61" s="32">
+        <f>G15*(G21-G20)</f>
+        <v/>
+      </c>
+      <c r="H61" s="32">
+        <f>H15*(H21-H20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Other ΔNWC (ex-AR) – year 5</t>
+        </is>
+      </c>
+      <c r="F62" s="32">
+        <f>F15*(F22-F21)</f>
+        <v/>
+      </c>
+      <c r="G62" s="32">
+        <f>G15*(G22-G21)</f>
+        <v/>
+      </c>
+      <c r="H62" s="32">
+        <f>H15*(H22-H21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ΔNWC – year 1</t>
+        </is>
+      </c>
+      <c r="F63" s="32">
+        <f>F53+F58</f>
+        <v/>
+      </c>
+      <c r="G63" s="32">
+        <f>G53+G58</f>
+        <v/>
+      </c>
+      <c r="H63" s="32">
+        <f>H53+H58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ΔNWC – year 2</t>
+        </is>
+      </c>
+      <c r="F64" s="32">
+        <f>F54+F59</f>
+        <v/>
+      </c>
+      <c r="G64" s="32">
+        <f>G54+G59</f>
+        <v/>
+      </c>
+      <c r="H64" s="32">
+        <f>H54+H59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ΔNWC – year 3</t>
+        </is>
+      </c>
+      <c r="F65" s="32">
+        <f>F55+F60</f>
+        <v/>
+      </c>
+      <c r="G65" s="32">
+        <f>G55+G60</f>
+        <v/>
+      </c>
+      <c r="H65" s="32">
+        <f>H55+H60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ΔNWC – year 4</t>
+        </is>
+      </c>
+      <c r="F66" s="32">
+        <f>F56+F61</f>
+        <v/>
+      </c>
+      <c r="G66" s="32">
+        <f>G56+G61</f>
+        <v/>
+      </c>
+      <c r="H66" s="32">
+        <f>H56+H61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ΔNWC – year 5</t>
+        </is>
+      </c>
+      <c r="F67" s="32">
+        <f>F57+F62</f>
+        <v/>
+      </c>
+      <c r="G67" s="32">
+        <f>G57+G62</f>
+        <v/>
+      </c>
+      <c r="H67" s="32">
+        <f>H57+H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Unlevered FCF – year 1</t>
+        </is>
+      </c>
+      <c r="F68" s="32">
+        <f>F33+F38-F43-F63</f>
+        <v/>
+      </c>
+      <c r="G68" s="32">
+        <f>G33+G38-G43-G63</f>
+        <v/>
+      </c>
+      <c r="H68" s="32">
+        <f>H33+H38-H43-H63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Unlevered FCF – year 2</t>
+        </is>
+      </c>
+      <c r="F69" s="32">
+        <f>F34+F39-F44-F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="32">
+        <f>G34+G39-G44-G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="32">
+        <f>H34+H39-H44-H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Unlevered FCF – year 3</t>
+        </is>
+      </c>
+      <c r="F70" s="32">
+        <f>F35+F40-F45-F65</f>
+        <v/>
+      </c>
+      <c r="G70" s="32">
+        <f>G35+G40-G45-G65</f>
+        <v/>
+      </c>
+      <c r="H70" s="32">
+        <f>H35+H40-H45-H65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Unlevered FCF – year 4</t>
+        </is>
+      </c>
+      <c r="F71" s="32">
+        <f>F36+F41-F46-F66</f>
+        <v/>
+      </c>
+      <c r="G71" s="32">
+        <f>G36+G41-G46-G66</f>
+        <v/>
+      </c>
+      <c r="H71" s="32">
+        <f>H36+H41-H46-H66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="31" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Unlevered FCF – year 5</t>
         </is>
       </c>
-      <c r="F56" s="32">
-        <f>F36+F41-F46-F51</f>
-        <v/>
-      </c>
-      <c r="G56" s="32">
-        <f>G36+G41-G46-G51</f>
-        <v/>
-      </c>
-      <c r="H56" s="32">
-        <f>H36+H41-H46-H51</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="22" t="inlineStr">
+      <c r="F72" s="32">
+        <f>F37+F42-F47-F67</f>
+        <v/>
+      </c>
+      <c r="G72" s="32">
+        <f>G37+G42-G47-G67</f>
+        <v/>
+      </c>
+      <c r="H72" s="32">
+        <f>H37+H42-H47-H67</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="22" t="inlineStr">
         <is>
           <t>Enterprise value (DCF)</t>
         </is>
       </c>
-      <c r="F58" s="34">
-        <f>NPV(F9,F52,F53,F54,F55,F56)+(F56*(1+F10)/(F9-F10))/(1+F9)^5</f>
-        <v/>
-      </c>
-      <c r="G58" s="34">
-        <f>NPV(G9,G52,G53,G54,G55,G56)+(G56*(1+G10)/(G9-G10))/(1+G9)^5</f>
-        <v/>
-      </c>
-      <c r="H58" s="34">
-        <f>NPV(H9,H52,H53,H54,H55,H56)+(H56*(1+H10)/(H9-H10))/(1+H9)^5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="35" t="inlineStr">
+      <c r="F74" s="34">
+        <f>NPV(F9,F68,F69,F70,F71,F72)+(F72*(1+F10)/(F9-F10))/(1+F9)^5</f>
+        <v/>
+      </c>
+      <c r="G74" s="34">
+        <f>NPV(G9,G68,G69,G70,G71,G72)+(G72*(1+G10)/(G9-G10))/(1+G9)^5</f>
+        <v/>
+      </c>
+      <c r="H74" s="34">
+        <f>NPV(H9,H68,H69,H70,H71,H72)+(H72*(1+H10)/(H9-H10))/(1+H9)^5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="35" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="F59" s="36">
-        <f>(F58+1807202-0)/111380</f>
-        <v/>
-      </c>
-      <c r="G59" s="37">
-        <f>(G58+1807202-0)/111380</f>
-        <v/>
-      </c>
-      <c r="H59" s="36">
-        <f>(H58+1807202-0)/111380</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="22" t="inlineStr">
+      <c r="F75" s="36">
+        <f>(F74+1807202-0)/111380</f>
+        <v/>
+      </c>
+      <c r="G75" s="37">
+        <f>(G74+1807202-0)/111380</f>
+        <v/>
+      </c>
+      <c r="H75" s="36">
+        <f>(H74+1807202-0)/111380</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="22" t="inlineStr">
         <is>
           <t>Upside / (downside) vs current</t>
         </is>
       </c>
-      <c r="F60" s="38">
-        <f>F59/100.0-1</f>
-        <v/>
-      </c>
-      <c r="G60" s="38">
-        <f>G59/100.0-1</f>
-        <v/>
-      </c>
-      <c r="H60" s="38">
-        <f>H59/100.0-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="39" t="inlineStr">
+      <c r="F76" s="38">
+        <f>F75/100.0-1</f>
+        <v/>
+      </c>
+      <c r="G76" s="38">
+        <f>G75/100.0-1</f>
+        <v/>
+      </c>
+      <c r="H76" s="38">
+        <f>H75/100.0-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="39" t="inlineStr">
         <is>
           <t>Current price $100.00; cash $1,807,202 k; net debt $0 (net-cash balance sheet).</t>
         </is>
@@ -2650,6 +2966,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2661,7 +2978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M67"/>
+  <dimension ref="A1:M71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2789,27 +3106,27 @@
         <v>11102600</v>
       </c>
       <c r="F5" s="48">
-        <f>Scenarios!G17</f>
+        <f>Scenarios!G18</f>
         <v/>
       </c>
       <c r="G5" s="48">
-        <f>Scenarios!G18</f>
+        <f>Scenarios!G19</f>
         <v/>
       </c>
       <c r="H5" s="48">
-        <f>Scenarios!G19</f>
+        <f>Scenarios!G20</f>
         <v/>
       </c>
       <c r="I5" s="48">
-        <f>Scenarios!G20</f>
+        <f>Scenarios!G21</f>
         <v/>
       </c>
       <c r="J5" s="48">
-        <f>Scenarios!G21</f>
+        <f>Scenarios!G22</f>
         <v/>
       </c>
       <c r="K5" s="49">
-        <f>IF(MAX(ABS(F5-Scenarios!$G$17),ABS(G5-Scenarios!$G$18),ABS(H5-Scenarios!$G$19),ABS(I5-Scenarios!$G$20),ABS(J5-Scenarios!$G$21))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F5-Scenarios!$G$18),ABS(G5-Scenarios!$G$19),ABS(H5-Scenarios!$G$20),ABS(I5-Scenarios!$G$21),ABS(J5-Scenarios!$G$22))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2883,27 +3200,27 @@
         </is>
       </c>
       <c r="F7" s="50">
-        <f>Scenarios!G22</f>
+        <f>Scenarios!G23</f>
         <v/>
       </c>
       <c r="G7" s="50">
-        <f>Scenarios!G23</f>
+        <f>Scenarios!G24</f>
         <v/>
       </c>
       <c r="H7" s="50">
-        <f>Scenarios!G24</f>
+        <f>Scenarios!G25</f>
         <v/>
       </c>
       <c r="I7" s="50">
-        <f>Scenarios!G25</f>
+        <f>Scenarios!G26</f>
         <v/>
       </c>
       <c r="J7" s="50">
-        <f>Scenarios!G26</f>
+        <f>Scenarios!G27</f>
         <v/>
       </c>
       <c r="K7" s="49">
-        <f>IF(MAX(ABS(F7-Scenarios!$G$22),ABS(G7-Scenarios!$G$23),ABS(H7-Scenarios!$G$24),ABS(I7-Scenarios!$G$25),ABS(J7-Scenarios!$G$26))&lt;0.0001,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F7-Scenarios!$G$23),ABS(G7-Scenarios!$G$24),ABS(H7-Scenarios!$G$25),ABS(I7-Scenarios!$G$26),ABS(J7-Scenarios!$G$27))&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -2958,27 +3275,27 @@
         <v>2210615</v>
       </c>
       <c r="F9" s="34">
-        <f>Scenarios!G27</f>
+        <f>Scenarios!G28</f>
         <v/>
       </c>
       <c r="G9" s="34">
-        <f>Scenarios!G28</f>
+        <f>Scenarios!G29</f>
         <v/>
       </c>
       <c r="H9" s="34">
-        <f>Scenarios!G29</f>
+        <f>Scenarios!G30</f>
         <v/>
       </c>
       <c r="I9" s="34">
-        <f>Scenarios!G30</f>
+        <f>Scenarios!G31</f>
         <v/>
       </c>
       <c r="J9" s="34">
-        <f>Scenarios!G31</f>
+        <f>Scenarios!G32</f>
         <v/>
       </c>
       <c r="K9" s="52">
-        <f>IF(MAX(ABS(F9-Scenarios!$G$27),ABS(G9-Scenarios!$G$28),ABS(H9-Scenarios!$G$29),ABS(I9-Scenarios!$G$30),ABS(J9-Scenarios!$G$31))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F9-Scenarios!$G$28),ABS(G9-Scenarios!$G$29),ABS(H9-Scenarios!$G$30),ABS(I9-Scenarios!$G$31),ABS(J9-Scenarios!$G$32))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -3019,23 +3336,23 @@
         </is>
       </c>
       <c r="F11" s="48">
-        <f>-Scenarios!G27*Scenarios!$G$11</f>
+        <f>-Scenarios!G28*Scenarios!$G$11</f>
         <v/>
       </c>
       <c r="G11" s="48">
-        <f>-Scenarios!G28*Scenarios!$G$11</f>
+        <f>-Scenarios!G29*Scenarios!$G$11</f>
         <v/>
       </c>
       <c r="H11" s="48">
-        <f>-Scenarios!G29*Scenarios!$G$11</f>
+        <f>-Scenarios!G30*Scenarios!$G$11</f>
         <v/>
       </c>
       <c r="I11" s="48">
-        <f>-Scenarios!G30*Scenarios!$G$11</f>
+        <f>-Scenarios!G31*Scenarios!$G$11</f>
         <v/>
       </c>
       <c r="J11" s="48">
-        <f>-Scenarios!G31*Scenarios!$G$11</f>
+        <f>-Scenarios!G32*Scenarios!$G$11</f>
         <v/>
       </c>
     </row>
@@ -3046,27 +3363,27 @@
         </is>
       </c>
       <c r="F12" s="34">
-        <f>Scenarios!G32</f>
+        <f>Scenarios!G33</f>
         <v/>
       </c>
       <c r="G12" s="34">
-        <f>Scenarios!G33</f>
+        <f>Scenarios!G34</f>
         <v/>
       </c>
       <c r="H12" s="34">
-        <f>Scenarios!G34</f>
+        <f>Scenarios!G35</f>
         <v/>
       </c>
       <c r="I12" s="34">
-        <f>Scenarios!G35</f>
+        <f>Scenarios!G36</f>
         <v/>
       </c>
       <c r="J12" s="34">
-        <f>Scenarios!G36</f>
+        <f>Scenarios!G37</f>
         <v/>
       </c>
       <c r="K12" s="52">
-        <f>IF(MAX(ABS(F12-Scenarios!$G$32),ABS(G12-Scenarios!$G$33),ABS(H12-Scenarios!$G$34),ABS(I12-Scenarios!$G$35),ABS(J12-Scenarios!$G$36))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F12-Scenarios!$G$33),ABS(G12-Scenarios!$G$34),ABS(H12-Scenarios!$G$35),ABS(I12-Scenarios!$G$36),ABS(J12-Scenarios!$G$37))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -3119,27 +3436,27 @@
         </is>
       </c>
       <c r="F14" s="48">
-        <f>Scenarios!G37</f>
+        <f>Scenarios!G38</f>
         <v/>
       </c>
       <c r="G14" s="48">
-        <f>Scenarios!G38</f>
+        <f>Scenarios!G39</f>
         <v/>
       </c>
       <c r="H14" s="48">
-        <f>Scenarios!G39</f>
+        <f>Scenarios!G40</f>
         <v/>
       </c>
       <c r="I14" s="48">
-        <f>Scenarios!G40</f>
+        <f>Scenarios!G41</f>
         <v/>
       </c>
       <c r="J14" s="48">
-        <f>Scenarios!G41</f>
+        <f>Scenarios!G42</f>
         <v/>
       </c>
       <c r="K14" s="49">
-        <f>IF(MAX(ABS(F14-Scenarios!$G$37),ABS(G14-Scenarios!$G$38),ABS(H14-Scenarios!$G$39),ABS(I14-Scenarios!$G$40),ABS(J14-Scenarios!$G$41))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F14-Scenarios!$G$38),ABS(G14-Scenarios!$G$39),ABS(H14-Scenarios!$G$40),ABS(I14-Scenarios!$G$41),ABS(J14-Scenarios!$G$42))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
@@ -3205,49 +3522,49 @@
         </is>
       </c>
       <c r="F16" s="48">
-        <f>-Scenarios!G42</f>
+        <f>-Scenarios!G43</f>
         <v/>
       </c>
       <c r="G16" s="48">
-        <f>-Scenarios!G43</f>
+        <f>-Scenarios!G44</f>
         <v/>
       </c>
       <c r="H16" s="48">
-        <f>-Scenarios!G44</f>
+        <f>-Scenarios!G45</f>
         <v/>
       </c>
       <c r="I16" s="48">
-        <f>-Scenarios!G45</f>
+        <f>-Scenarios!G46</f>
         <v/>
       </c>
       <c r="J16" s="48">
-        <f>-Scenarios!G46</f>
+        <f>-Scenarios!G47</f>
         <v/>
       </c>
       <c r="K16" s="49">
-        <f>IF(MAX(ABS(F16+Scenarios!$G$42),ABS(G16+Scenarios!$G$43),ABS(H16+Scenarios!$G$44),ABS(I16+Scenarios!$G$45),ABS(J16+Scenarios!$G$46))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F16+Scenarios!$G$43),ABS(G16+Scenarios!$G$44),ABS(H16+Scenarios!$G$45),ABS(I16+Scenarios!$G$46),ABS(J16+Scenarios!$G$47))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NWC build % of Δrevenue</t>
+          <t xml:space="preserve">  AR % of revenue</t>
         </is>
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>7.5% of Δsales is operating NWC: AR + inventory + other CA − AP − accrued. AR is on the 10-K ($190,657); not omitted.</t>
+          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Own DCF NWC line; wholesale / marketplace mix.</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>LULU BS/IS historical (10-K)</t>
+          <t>LULU FY2025 10-K: Accounts receivable, net</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts receivable, net" → 190,657. Ctrl+F "Inventories" → 1,700,753. Ctrl+F "Accounts payable" → 331,421. Ctrl+F "Accrued liabilities and other" → 662,982. NWC = AR + Inv + other CA − AP − accrued; 7.5% of Δsales.</t>
+          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. This is the DCF AR / NWC line.</t>
         </is>
       </c>
       <c r="F17" s="20">
@@ -3271,857 +3588,1010 @@
         <v/>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="28" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>(Increase)/decrease in net working capital</t>
-        </is>
+          <t>Accounts receivable, net</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Own DCF NWC line; wholesale / marketplace mix.</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: Accounts receivable, net</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. This is the DCF AR / NWC line.</t>
+        </is>
+      </c>
+      <c r="E18" s="47" t="n">
+        <v>190657</v>
       </c>
       <c r="F18" s="48">
-        <f>-Scenarios!G47</f>
+        <f>Scenarios!G48</f>
         <v/>
       </c>
       <c r="G18" s="48">
-        <f>-Scenarios!G48</f>
+        <f>Scenarios!G49</f>
         <v/>
       </c>
       <c r="H18" s="48">
-        <f>-Scenarios!G49</f>
+        <f>Scenarios!G50</f>
         <v/>
       </c>
       <c r="I18" s="48">
-        <f>-Scenarios!G50</f>
+        <f>Scenarios!G51</f>
         <v/>
       </c>
       <c r="J18" s="48">
-        <f>-Scenarios!G51</f>
+        <f>Scenarios!G52</f>
         <v/>
       </c>
       <c r="K18" s="49">
-        <f>IF(MAX(ABS(F18+Scenarios!$G$47),ABS(G18+Scenarios!$G$48),ABS(H18+Scenarios!$G$49),ABS(I18+Scenarios!$G$50),ABS(J18+Scenarios!$G$51))&lt;0.5,"OK","CHECK")</f>
+        <f>IF(MAX(ABS(F18-Scenarios!$G$48),ABS(G18-Scenarios!$G$49),ABS(H18-Scenarios!$G$50),ABS(I18-Scenarios!$G$51),ABS(J18-Scenarios!$G$52))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  memo: FY26 revenue falls −6.1%; negative ΔNWC releases ~$51M cash (adds to FCF, not a use).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="22" t="inlineStr">
-        <is>
-          <t>Unlevered free cash flow</t>
-        </is>
-      </c>
-      <c r="F20" s="54">
-        <f>Scenarios!G52</f>
-        <v/>
-      </c>
-      <c r="G20" s="54">
-        <f>Scenarios!G53</f>
-        <v/>
-      </c>
-      <c r="H20" s="54">
-        <f>Scenarios!G54</f>
-        <v/>
-      </c>
-      <c r="I20" s="54">
-        <f>Scenarios!G55</f>
-        <v/>
-      </c>
-      <c r="J20" s="54">
-        <f>Scenarios!G56</f>
-        <v/>
-      </c>
-      <c r="K20" s="52">
-        <f>IF(MAX(ABS(F20-Scenarios!$G$52),ABS(G20-Scenarios!$G$53),ABS(H20-Scenarios!$G$54),ABS(I20-Scenarios!$G$55),ABS(J20-Scenarios!$G$56))&lt;0.5,"OK","CHECK")</f>
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ΔAR (increase)/decrease — part of NWC</t>
+        </is>
+      </c>
+      <c r="F19" s="48">
+        <f>-Scenarios!G53</f>
+        <v/>
+      </c>
+      <c r="G19" s="48">
+        <f>-Scenarios!G54</f>
+        <v/>
+      </c>
+      <c r="H19" s="48">
+        <f>-Scenarios!G55</f>
+        <v/>
+      </c>
+      <c r="I19" s="48">
+        <f>-Scenarios!G56</f>
+        <v/>
+      </c>
+      <c r="J19" s="48">
+        <f>-Scenarios!G57</f>
+        <v/>
+      </c>
+      <c r="K19" s="49">
+        <f>IF(MAX(ABS(F19+Scenarios!$G$53),ABS(G19+Scenarios!$G$54),ABS(H19+Scenarios!$G$55),ABS(I19+Scenarios!$G$56),ABS(J19+Scenarios!$G$57))&lt;0.5,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Other NWC (ex-AR) % of Δrevenue</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>5.8% of Δsales is other NWC (Inv + OCA − AP − accrued). AR is the 1.7% line above, not inside this residual. 1.7+5.8=7.5%.</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>LULU BS/IS historical (10-K)</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Other NWC ex-AR. Ctrl+F "Inventories" → 1,700,753 | "Accounts payable" → 331,421 | "Accrued liabilities and other" → 662,982. 5.8% of Δsales; AR is the 1.7% line, not in this residual.</t>
+        </is>
+      </c>
+      <c r="F20" s="20">
+        <f>Scenarios!$G$15</f>
+        <v/>
+      </c>
+      <c r="G20" s="20">
+        <f>Scenarios!$G$15</f>
+        <v/>
+      </c>
+      <c r="H20" s="20">
+        <f>Scenarios!$G$15</f>
+        <v/>
+      </c>
+      <c r="I20" s="20">
+        <f>Scenarios!$G$15</f>
+        <v/>
+      </c>
+      <c r="J20" s="20">
+        <f>Scenarios!$G$15</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>Discount period (years)</t>
-        </is>
-      </c>
-      <c r="F21" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="55" t="n">
-        <v>2</v>
-      </c>
-      <c r="H21" s="55" t="n">
-        <v>3</v>
-      </c>
-      <c r="I21" s="55" t="n">
-        <v>4</v>
-      </c>
-      <c r="J21" s="55" t="n">
-        <v>5</v>
+          <t xml:space="preserve">  Other ΔNWC (ex-AR) (increase)/decrease</t>
+        </is>
+      </c>
+      <c r="F21" s="48">
+        <f>-Scenarios!G58</f>
+        <v/>
+      </c>
+      <c r="G21" s="48">
+        <f>-Scenarios!G59</f>
+        <v/>
+      </c>
+      <c r="H21" s="48">
+        <f>-Scenarios!G60</f>
+        <v/>
+      </c>
+      <c r="I21" s="48">
+        <f>-Scenarios!G61</f>
+        <v/>
+      </c>
+      <c r="J21" s="48">
+        <f>-Scenarios!G62</f>
+        <v/>
+      </c>
+      <c r="K21" s="49">
+        <f>IF(MAX(ABS(F21+Scenarios!$G$58),ABS(G21+Scenarios!$G$59),ABS(H21+Scenarios!$G$60),ABS(I21+Scenarios!$G$61),ABS(J21+Scenarios!$G$62))&lt;0.5,"OK","CHECK")</f>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
+          <t>Total (increase)/decrease in net working capital</t>
+        </is>
+      </c>
+      <c r="F22" s="48">
+        <f>-Scenarios!G63</f>
+        <v/>
+      </c>
+      <c r="G22" s="48">
+        <f>-Scenarios!G64</f>
+        <v/>
+      </c>
+      <c r="H22" s="48">
+        <f>-Scenarios!G65</f>
+        <v/>
+      </c>
+      <c r="I22" s="48">
+        <f>-Scenarios!G66</f>
+        <v/>
+      </c>
+      <c r="J22" s="48">
+        <f>-Scenarios!G67</f>
+        <v/>
+      </c>
+      <c r="K22" s="49">
+        <f>IF(MAX(ABS(F22+Scenarios!$G$63),ABS(G22+Scenarios!$G$64),ABS(H22+Scenarios!$G$65),ABS(I22+Scenarios!$G$66),ABS(J22+Scenarios!$G$67))&lt;0.5,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  memo: ΔNWC = ΔAR + other ΔNWC. AR is 1.7% of sales (own line); other is 5.8% of Δsales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>Unlevered free cash flow</t>
+        </is>
+      </c>
+      <c r="F24" s="54">
+        <f>Scenarios!G68</f>
+        <v/>
+      </c>
+      <c r="G24" s="54">
+        <f>Scenarios!G69</f>
+        <v/>
+      </c>
+      <c r="H24" s="54">
+        <f>Scenarios!G70</f>
+        <v/>
+      </c>
+      <c r="I24" s="54">
+        <f>Scenarios!G71</f>
+        <v/>
+      </c>
+      <c r="J24" s="54">
+        <f>Scenarios!G72</f>
+        <v/>
+      </c>
+      <c r="K24" s="52">
+        <f>IF(MAX(ABS(F24-Scenarios!$G$68),ABS(G24-Scenarios!$G$69),ABS(H24-Scenarios!$G$70),ABS(I24-Scenarios!$G$71),ABS(J24-Scenarios!$G$72))&lt;0.5,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>Discount period (years)</t>
+        </is>
+      </c>
+      <c r="F25" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="H25" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="I25" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="J25" s="55" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
           <t>Discount factor @ WACC</t>
         </is>
       </c>
-      <c r="F22" s="56">
-        <f>1/(1+Scenarios!$G$9)^F21</f>
-        <v/>
-      </c>
-      <c r="G22" s="56">
-        <f>1/(1+Scenarios!$G$9)^G21</f>
-        <v/>
-      </c>
-      <c r="H22" s="56">
-        <f>1/(1+Scenarios!$G$9)^H21</f>
-        <v/>
-      </c>
-      <c r="I22" s="56">
-        <f>1/(1+Scenarios!$G$9)^I21</f>
-        <v/>
-      </c>
-      <c r="J22" s="56">
-        <f>1/(1+Scenarios!$G$9)^J21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="22" t="inlineStr">
-        <is>
-          <t>PV of unlevered FCF</t>
-        </is>
-      </c>
-      <c r="F23" s="34">
-        <f>F20*F22</f>
-        <v/>
-      </c>
-      <c r="G23" s="34">
-        <f>G20*G22</f>
-        <v/>
-      </c>
-      <c r="H23" s="34">
-        <f>H20*H22</f>
-        <v/>
-      </c>
-      <c r="I23" s="34">
-        <f>I20*I22</f>
-        <v/>
-      </c>
-      <c r="J23" s="34">
-        <f>J20*J22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>Scenarios linkage summary (column K should all read OK)</t>
-        </is>
-      </c>
-      <c r="K25" s="57">
-        <f>IF(COUNTIF(K5:K20,"CHECK")=0,"ALL OK","REVIEW")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="58" t="inlineStr">
-        <is>
-          <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
-        </is>
-      </c>
-      <c r="B26" s="13" t="n"/>
-      <c r="C26" s="13" t="n"/>
+      <c r="F26" s="56">
+        <f>1/(1+Scenarios!$G$9)^F25</f>
+        <v/>
+      </c>
+      <c r="G26" s="56">
+        <f>1/(1+Scenarios!$G$9)^G25</f>
+        <v/>
+      </c>
+      <c r="H26" s="56">
+        <f>1/(1+Scenarios!$G$9)^H25</f>
+        <v/>
+      </c>
+      <c r="I26" s="56">
+        <f>1/(1+Scenarios!$G$9)^I25</f>
+        <v/>
+      </c>
+      <c r="J26" s="56">
+        <f>1/(1+Scenarios!$G$9)^J25</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="22" t="inlineStr">
         <is>
+          <t>PV of unlevered FCF</t>
+        </is>
+      </c>
+      <c r="F27" s="34">
+        <f>F24*F26</f>
+        <v/>
+      </c>
+      <c r="G27" s="34">
+        <f>G24*G26</f>
+        <v/>
+      </c>
+      <c r="H27" s="34">
+        <f>H24*H26</f>
+        <v/>
+      </c>
+      <c r="I27" s="34">
+        <f>I24*I26</f>
+        <v/>
+      </c>
+      <c r="J27" s="34">
+        <f>J24*J26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>Scenarios linkage summary (column K should all read OK)</t>
+        </is>
+      </c>
+      <c r="K29" s="57">
+        <f>IF(COUNTIF(K5:K24,"CHECK")=0,"ALL OK","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="58" t="inlineStr">
+        <is>
+          <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="n"/>
+      <c r="C30" s="13" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
           <t>Sum of PV of explicit FCF (FY26–FY30)</t>
         </is>
       </c>
-      <c r="E27" s="59">
-        <f>SUM(F23:J23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="E31" s="59">
+        <f>SUM(F27:J27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>Terminal growth rate (g)</t>
         </is>
       </c>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>2.25% terminal g sits next to FRED GDPC1 Q2/Q2 real GDP ≈ 2.1% (24,269.613 / 23,770.976 − 1).</t>
         </is>
       </c>
-      <c r="C28" s="18" t="inlineStr">
+      <c r="C32" s="18" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="D28" s="19" t="inlineStr">
+      <c r="D32" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Q2 2026" → 24,269.613 and "Q2 2025" → 23,770.976. YoY = 2.1%. Model terminal g 2.25%.</t>
         </is>
       </c>
-      <c r="E28" s="50">
+      <c r="E32" s="50">
         <f>Scenarios!$G$10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="22" t="inlineStr">
-        <is>
-          <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
-        </is>
-      </c>
-      <c r="E29" s="34">
-        <f>J9+J14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
-        </is>
-      </c>
-      <c r="E30" s="48">
-        <f>J20*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Implied exit EV/EBITDA (Gordon Growth)</t>
-        </is>
-      </c>
-      <c r="E31" s="60">
-        <f>E30/E29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="22" t="inlineStr">
-        <is>
-          <t>PV of terminal value</t>
-        </is>
-      </c>
-      <c r="E32" s="59">
-        <f>E30/(1+Scenarios!$G$9)^J21</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="22" t="inlineStr">
         <is>
-          <t>Enterprise value</t>
+          <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
         </is>
       </c>
       <c r="E33" s="34">
-        <f>E27+E32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="28" customHeight="1">
+        <f>J9+J14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
       <c r="A34" s="16" t="inlineStr">
         <is>
-          <t>Plus: cash &amp; equivalents (FY2025)</t>
-        </is>
-      </c>
-      <c r="C34" s="61" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="D34" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
-        </is>
-      </c>
-      <c r="E34" s="47" t="n">
-        <v>1807202</v>
-      </c>
-    </row>
-    <row r="35" ht="28" customHeight="1">
+          <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
+        </is>
+      </c>
+      <c r="E34" s="48">
+        <f>J24*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
       <c r="A35" s="16" t="inlineStr">
         <is>
-          <t>Less: total debt</t>
-        </is>
-      </c>
-      <c r="C35" s="61" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="D35" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "no borrowings were outstanding under this facility" → no funded term debt</t>
-        </is>
-      </c>
-      <c r="E35" s="47" t="n">
-        <v>0</v>
+          <t xml:space="preserve">  Implied exit EV/EBITDA (Gordon Growth)</t>
+        </is>
+      </c>
+      <c r="E35" s="60">
+        <f>E34/E33</f>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="22" t="inlineStr">
         <is>
-          <t>Equity value</t>
-        </is>
-      </c>
-      <c r="E36" s="34">
-        <f>E33+E34+E35</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="28" customHeight="1">
-      <c r="A37" s="16" t="inlineStr">
-        <is>
-          <t>Diluted shares outstanding (000)</t>
-        </is>
-      </c>
-      <c r="C37" s="61" t="inlineStr">
+          <t>PV of terminal value</t>
+        </is>
+      </c>
+      <c r="E36" s="59">
+        <f>E34/(1+Scenarios!$G$9)^J25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>Enterprise value</t>
+        </is>
+      </c>
+      <c r="E37" s="34">
+        <f>E31+E36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>Plus: cash &amp; equivalents (FY2025)</t>
+        </is>
+      </c>
+      <c r="C38" s="61" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="D37" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Diluted weighted-average number of shares outstanding" → 119,068 (000)</t>
-        </is>
-      </c>
-      <c r="E37" s="47" t="n">
-        <v>111380</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="22" t="inlineStr">
-        <is>
-          <t>Implied value per share</t>
-        </is>
-      </c>
-      <c r="E38" s="62">
-        <f>E36/E37</f>
-        <v/>
-      </c>
-      <c r="K38" s="52">
-        <f>IF(ABS(E38-Scenarios!$G$59)&lt;0.05,"OK","CHECK")</f>
-        <v/>
+      <c r="D38" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
+        </is>
+      </c>
+      <c r="E38" s="47" t="n">
+        <v>1807202</v>
       </c>
     </row>
     <row r="39" ht="28" customHeight="1">
       <c r="A39" s="16" t="inlineStr">
         <is>
-          <t>Current share price</t>
+          <t>Less: total debt</t>
         </is>
       </c>
       <c r="C39" s="61" t="inlineStr">
         <is>
-          <t>NASDAQ</t>
+          <t>10-K</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
-        </is>
-      </c>
-      <c r="E39" s="63" t="n">
-        <v>100</v>
+          <t>Ctrl+F "no borrowings were outstanding under this facility" → no funded term debt</t>
+        </is>
+      </c>
+      <c r="E39" s="47" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="22" t="inlineStr">
         <is>
+          <t>Equity value</t>
+        </is>
+      </c>
+      <c r="E40" s="34">
+        <f>E37+E38+E39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>Diluted shares outstanding (000)</t>
+        </is>
+      </c>
+      <c r="C41" s="61" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="D41" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Diluted weighted-average number of shares outstanding" → 119,068 (000)</t>
+        </is>
+      </c>
+      <c r="E41" s="47" t="n">
+        <v>111380</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="22" t="inlineStr">
+        <is>
+          <t>Implied value per share</t>
+        </is>
+      </c>
+      <c r="E42" s="62">
+        <f>E40/E41</f>
+        <v/>
+      </c>
+      <c r="K42" s="52">
+        <f>IF(ABS(E42-Scenarios!$G$75)&lt;0.05,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>Current share price</t>
+        </is>
+      </c>
+      <c r="C43" s="61" t="inlineStr">
+        <is>
+          <t>NASDAQ</t>
+        </is>
+      </c>
+      <c r="D43" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
+        </is>
+      </c>
+      <c r="E43" s="63" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
           <t>Implied upside / (downside)</t>
         </is>
       </c>
-      <c r="E40" s="64">
-        <f>E38/E39-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="E44" s="64">
+        <f>E42/E43-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: % of EV from terminal value</t>
         </is>
       </c>
-      <c r="E41" s="50">
-        <f>E32/E33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="58" t="inlineStr">
+      <c r="E45" s="50">
+        <f>E36/E37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="58" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
       </c>
-      <c r="B43" s="13" t="n"/>
-      <c r="C43" s="13" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="15" t="inlineStr">
+      <c r="B47" s="13" t="n"/>
+      <c r="C47" s="13" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>Exit multiple selection (see Comps tab for peer build)</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="28" customHeight="1">
-      <c r="A45" s="16" t="inlineStr">
+    <row r="49" ht="28" customHeight="1">
+      <c r="A49" s="16" t="inlineStr">
         <is>
           <t>Selected exit EV/EBITDA multiple (FY2030E)</t>
         </is>
       </c>
-      <c r="B45" s="17" t="inlineStr">
+      <c r="B49" s="17" t="inlineStr">
         <is>
           <t>8.0x FY2030E exit EV/EBITDA; mid-point of terminal football field (6.5–9.5x); ~1 turn above Gordon-implied ~7x.</t>
         </is>
       </c>
-      <c r="C45" s="18" t="inlineStr">
+      <c r="C49" s="18" t="inlineStr">
         <is>
           <t>StockAnalysis: LULU EV/EBITDA</t>
         </is>
       </c>
-      <c r="D45" s="19" t="inlineStr">
+      <c r="D49" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x (assumption)</t>
         </is>
       </c>
-      <c r="E45" s="65" t="n">
+      <c r="E49" s="65" t="n">
         <v>8</v>
       </c>
-      <c r="M45" s="61" t="inlineStr">
+      <c r="M49" s="61" t="inlineStr">
         <is>
           <t>Comps: Exit Multiple Build</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="16" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
         <is>
           <t>Terminal value = Terminal EBITDA × exit multiple</t>
         </is>
       </c>
-      <c r="E46" s="48">
-        <f>E29*E45</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="16" t="inlineStr">
+      <c r="E50" s="48">
+        <f>E33*E49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
         <is>
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="E47" s="48">
-        <f>E46/(1+Scenarios!$G$9)^J21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="22" t="inlineStr">
+      <c r="E51" s="48">
+        <f>E50/(1+Scenarios!$G$9)^J25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="22" t="inlineStr">
         <is>
           <t>Enterprise value (exit method)</t>
         </is>
       </c>
-      <c r="E48" s="34">
-        <f>E27+E47</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="22" t="inlineStr">
-        <is>
-          <t>Implied value per share (exit method)</t>
-        </is>
-      </c>
-      <c r="E49" s="66">
-        <f>(E48+E34+E35)/E37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="58" t="inlineStr">
-        <is>
-          <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
-        </is>
-      </c>
-      <c r="B51" s="13" t="n"/>
-      <c r="C51" s="13" t="n"/>
-      <c r="D51" s="13" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="67" t="inlineStr"/>
-      <c r="B52" s="68" t="inlineStr">
-        <is>
-          <t>Gordon Growth</t>
-        </is>
-      </c>
-      <c r="C52" s="68" t="inlineStr">
-        <is>
-          <t>Exit Multiple</t>
-        </is>
-      </c>
-      <c r="D52" s="68" t="inlineStr">
-        <is>
-          <t>Variance</t>
-        </is>
+      <c r="E52" s="34">
+        <f>E31+E51</f>
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="22" t="inlineStr">
         <is>
+          <t>Implied value per share (exit method)</t>
+        </is>
+      </c>
+      <c r="E53" s="66">
+        <f>(E52+E38+E39)/E41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="58" t="inlineStr">
+        <is>
+          <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="n"/>
+      <c r="C55" s="13" t="n"/>
+      <c r="D55" s="13" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="67" t="inlineStr"/>
+      <c r="B56" s="68" t="inlineStr">
+        <is>
+          <t>Gordon Growth</t>
+        </is>
+      </c>
+      <c r="C56" s="68" t="inlineStr">
+        <is>
+          <t>Exit Multiple</t>
+        </is>
+      </c>
+      <c r="D56" s="68" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="22" t="inlineStr">
+        <is>
           <t>Terminal value ($)</t>
         </is>
       </c>
-      <c r="B53" s="59">
-        <f>E30</f>
-        <v/>
-      </c>
-      <c r="C53" s="59">
-        <f>E46</f>
-        <v/>
-      </c>
-      <c r="D53" s="59">
-        <f>B53-C53</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="22" t="inlineStr">
+      <c r="B57" s="59">
+        <f>E34</f>
+        <v/>
+      </c>
+      <c r="C57" s="59">
+        <f>E50</f>
+        <v/>
+      </c>
+      <c r="D57" s="59">
+        <f>B57-C57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
       </c>
-      <c r="B54" s="69">
-        <f>E31</f>
-        <v/>
-      </c>
-      <c r="C54" s="69">
-        <f>E45</f>
-        <v/>
-      </c>
-      <c r="D54" s="69">
-        <f>B54-C54</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="16" t="inlineStr">
+      <c r="B58" s="69">
+        <f>E35</f>
+        <v/>
+      </c>
+      <c r="C58" s="69">
+        <f>E49</f>
+        <v/>
+      </c>
+      <c r="D58" s="69">
+        <f>B58-C58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="inlineStr">
         <is>
           <t>Terminal value variance (%)</t>
         </is>
       </c>
-      <c r="B55" s="50" t="inlineStr"/>
-      <c r="C55" s="50" t="inlineStr"/>
-      <c r="D55" s="50">
-        <f>(B53-C53)/B53</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="22" t="inlineStr">
+      <c r="B59" s="50" t="inlineStr"/>
+      <c r="C59" s="50" t="inlineStr"/>
+      <c r="D59" s="50">
+        <f>(B57-C57)/B57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="22" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="B56" s="70">
-        <f>E38</f>
-        <v/>
-      </c>
-      <c r="C56" s="70">
-        <f>E49</f>
-        <v/>
-      </c>
-      <c r="D56" s="70">
-        <f>B56-C56</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="71" t="inlineStr">
+      <c r="B60" s="70">
+        <f>E42</f>
+        <v/>
+      </c>
+      <c r="C60" s="70">
+        <f>E53</f>
+        <v/>
+      </c>
+      <c r="D60" s="70">
+        <f>B60-C60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="71" t="inlineStr">
         <is>
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B57" s="72">
-        <f>IF(ABS(D54)&lt;=1.5,"PASS","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="C57" s="73">
-        <f>TEXT(D54,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
-        <v/>
-      </c>
-      <c r="D57" s="39" t="inlineStr">
+      <c r="B61" s="72">
+        <f>IF(ABS(D58)&lt;=1.5,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="C61" s="73">
+        <f>TEXT(D58,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
+        <v/>
+      </c>
+      <c r="D61" s="39" t="inlineStr">
         <is>
           <t>Gordon implied should bracket exit assumption</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="58" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="58" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
       </c>
-      <c r="B60" s="13" t="n"/>
-      <c r="C60" s="13" t="n"/>
-      <c r="D60" s="13" t="n"/>
-      <c r="E60" s="13" t="n"/>
-      <c r="F60" s="13" t="n"/>
-      <c r="G60" s="13" t="n"/>
-      <c r="H60" s="13" t="n"/>
-    </row>
-    <row r="61" ht="28" customHeight="1">
-      <c r="A61" s="74" t="inlineStr">
+      <c r="B64" s="13" t="n"/>
+      <c r="C64" s="13" t="n"/>
+      <c r="D64" s="13" t="n"/>
+      <c r="E64" s="13" t="n"/>
+      <c r="F64" s="13" t="n"/>
+      <c r="G64" s="13" t="n"/>
+      <c r="H64" s="13" t="n"/>
+    </row>
+    <row r="65" ht="28" customHeight="1">
+      <c r="A65" s="74" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
       </c>
-      <c r="B61" s="17" t="inlineStr">
+      <c r="B65" s="17" t="inlineStr">
         <is>
           <t>Terminal-g axis 1.5–3.0% brackets 2.25% base; bounded by long-run real GDP and inflation benchmarks.</t>
         </is>
       </c>
-      <c r="C61" s="18" t="inlineStr">
+      <c r="C65" s="18" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="D61" s="19" t="inlineStr">
+      <c r="D65" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
       </c>
-      <c r="F61" s="75" t="n">
+      <c r="F65" s="75" t="n">
         <v>0.015</v>
       </c>
-      <c r="G61" s="75" t="n">
+      <c r="G65" s="75" t="n">
         <v>0.02</v>
       </c>
-      <c r="H61" s="75" t="n">
+      <c r="H65" s="75" t="n">
         <v>0.0225</v>
       </c>
-      <c r="I61" s="75" t="n">
+      <c r="I65" s="75" t="n">
         <v>0.025</v>
       </c>
-      <c r="J61" s="75" t="n">
+      <c r="J65" s="75" t="n">
         <v>0.03</v>
       </c>
-      <c r="L61" s="61" t="inlineStr">
+      <c r="L65" s="61" t="inlineStr">
         <is>
           <t>Scenarios: terminal g</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="28" customHeight="1">
-      <c r="A62" s="75" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="C62" s="61" t="inlineStr">
-        <is>
-          <t>Damodaran: Historical Implied ERP</t>
-        </is>
-      </c>
-      <c r="D62" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
-        </is>
-      </c>
-      <c r="F62" s="76">
-        <f>(NPV(0.095,F20:J20)+(J20*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="G62" s="76">
-        <f>(NPV(0.095,F20:J20)+(J20*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="H62" s="76">
-        <f>(NPV(0.095,F20:J20)+(J20*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="I62" s="76">
-        <f>(NPV(0.095,F20:J20)+(J20*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="J62" s="76">
-        <f>(NPV(0.095,F20:J20)+(J20*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="L62" s="61" t="inlineStr">
-        <is>
-          <t>WACC tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="28" customHeight="1">
-      <c r="A63" s="75" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
-        </is>
-      </c>
-      <c r="F63" s="76">
-        <f>(NPV(0.1,F20:J20)+(J20*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="G63" s="76">
-        <f>(NPV(0.1,F20:J20)+(J20*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="H63" s="76">
-        <f>(NPV(0.1,F20:J20)+(J20*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="I63" s="76">
-        <f>(NPV(0.1,F20:J20)+(J20*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="J63" s="76">
-        <f>(NPV(0.1,F20:J20)+(J20*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="L63" s="61" t="inlineStr">
-        <is>
-          <t>WACC tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="28" customHeight="1">
-      <c r="A64" s="75" t="n">
-        <v>0.105</v>
-      </c>
-      <c r="D64" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
-        </is>
-      </c>
-      <c r="F64" s="76">
-        <f>(NPV(0.105,F20:J20)+(J20*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="G64" s="76">
-        <f>(NPV(0.105,F20:J20)+(J20*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="H64" s="77">
-        <f>(NPV(0.105,F20:J20)+(J20*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="I64" s="76">
-        <f>(NPV(0.105,F20:J20)+(J20*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="J64" s="76">
-        <f>(NPV(0.105,F20:J20)+(J20*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="L64" s="61" t="inlineStr">
-        <is>
-          <t>WACC tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="28" customHeight="1">
-      <c r="A65" s="75" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="D65" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
-        </is>
-      </c>
-      <c r="F65" s="76">
-        <f>(NPV(0.11,F20:J20)+(J20*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="G65" s="76">
-        <f>(NPV(0.11,F20:J20)+(J20*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="H65" s="76">
-        <f>(NPV(0.11,F20:J20)+(J20*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="I65" s="76">
-        <f>(NPV(0.11,F20:J20)+(J20*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="J65" s="76">
-        <f>(NPV(0.11,F20:J20)+(J20*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="L65" s="61" t="inlineStr">
-        <is>
-          <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="75" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="C66" s="61" t="inlineStr">
+        <is>
+          <t>Damodaran: Historical Implied ERP</t>
+        </is>
+      </c>
+      <c r="D66" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
+        </is>
+      </c>
+      <c r="F66" s="76">
+        <f>(NPV(0.095,F24:J24)+(J24*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="G66" s="76">
+        <f>(NPV(0.095,F24:J24)+(J24*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="H66" s="76">
+        <f>(NPV(0.095,F24:J24)+(J24*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="I66" s="76">
+        <f>(NPV(0.095,F24:J24)+(J24*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="J66" s="76">
+        <f>(NPV(0.095,F24:J24)+(J24*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="L66" s="61" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="28" customHeight="1">
+      <c r="A67" s="75" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D67" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
+        </is>
+      </c>
+      <c r="F67" s="76">
+        <f>(NPV(0.1,F24:J24)+(J24*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="G67" s="76">
+        <f>(NPV(0.1,F24:J24)+(J24*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="H67" s="76">
+        <f>(NPV(0.1,F24:J24)+(J24*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="I67" s="76">
+        <f>(NPV(0.1,F24:J24)+(J24*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="J67" s="76">
+        <f>(NPV(0.1,F24:J24)+(J24*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="L67" s="61" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="28" customHeight="1">
+      <c r="A68" s="75" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="D68" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
+        </is>
+      </c>
+      <c r="F68" s="76">
+        <f>(NPV(0.105,F24:J24)+(J24*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="G68" s="76">
+        <f>(NPV(0.105,F24:J24)+(J24*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="H68" s="77">
+        <f>(NPV(0.105,F24:J24)+(J24*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="I68" s="76">
+        <f>(NPV(0.105,F24:J24)+(J24*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="J68" s="76">
+        <f>(NPV(0.105,F24:J24)+(J24*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="L68" s="61" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="28" customHeight="1">
+      <c r="A69" s="75" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="D69" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
+        </is>
+      </c>
+      <c r="F69" s="76">
+        <f>(NPV(0.11,F24:J24)+(J24*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="G69" s="76">
+        <f>(NPV(0.11,F24:J24)+(J24*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="H69" s="76">
+        <f>(NPV(0.11,F24:J24)+(J24*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="I69" s="76">
+        <f>(NPV(0.11,F24:J24)+(J24*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="J69" s="76">
+        <f>(NPV(0.11,F24:J24)+(J24*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="L69" s="61" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="28" customHeight="1">
+      <c r="A70" s="75" t="n">
         <v>0.115</v>
       </c>
-      <c r="D66" s="19" t="inlineStr">
+      <c r="D70" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F66" s="76">
-        <f>(NPV(0.115,F20:J20)+(J20*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="G66" s="76">
-        <f>(NPV(0.115,F20:J20)+(J20*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="H66" s="76">
-        <f>(NPV(0.115,F20:J20)+(J20*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="I66" s="76">
-        <f>(NPV(0.115,F20:J20)+(J20*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="J66" s="76">
-        <f>(NPV(0.115,F20:J20)+(J20*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E34+E35)/E37</f>
-        <v/>
-      </c>
-      <c r="L66" s="61" t="inlineStr">
+      <c r="F70" s="76">
+        <f>(NPV(0.115,F24:J24)+(J24*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="G70" s="76">
+        <f>(NPV(0.115,F24:J24)+(J24*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="H70" s="76">
+        <f>(NPV(0.115,F24:J24)+(J24*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="I70" s="76">
+        <f>(NPV(0.115,F24:J24)+(J24*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="J70" s="76">
+        <f>(NPV(0.115,F24:J24)+(J24*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E38+E39)/E41</f>
+        <v/>
+      </c>
+      <c r="L70" s="61" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="28" customHeight="1">
-      <c r="B67" s="17" t="inlineStr">
+    <row r="71" ht="28" customHeight="1">
+      <c r="B71" s="17" t="inlineStr">
         <is>
           <t>Red WACC and g grid values bracket base case ±100bps discount rate and ±75bps terminal growth for sensitivity.</t>
         </is>
       </c>
-      <c r="C67" s="18" t="inlineStr">
+      <c r="C71" s="18" t="inlineStr">
         <is>
           <t>Scenarios: WACC &amp; terminal g</t>
         </is>
       </c>
-      <c r="D67" s="19" t="inlineStr">
+      <c r="D71" s="19" t="inlineStr">
         <is>
           <t>Scenarios tab → Ctrl+F "WACC" and "Terminal growth" rows (base-case inputs)</t>
         </is>
       </c>
-      <c r="L67" s="61" t="inlineStr">
+      <c r="L71" s="61" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="M67" s="19" t="inlineStr">
+      <c r="M71" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
@@ -4140,27 +4610,30 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId21"/>
-    <hyperlink ref="M45" location="'Comps'!A26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId22"/>
-    <hyperlink ref="L61" location="'Scenarios'!G10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId23"/>
-    <hyperlink ref="L62" location="'WACC'!E16"/>
-    <hyperlink ref="L63" location="'WACC'!E16"/>
-    <hyperlink ref="L64" location="'WACC'!E16"/>
-    <hyperlink ref="L65" location="'WACC'!E16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId24"/>
+    <hyperlink ref="M49" location="'Comps'!A26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId25"/>
+    <hyperlink ref="L65" location="'Scenarios'!G10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId26"/>
     <hyperlink ref="L66" location="'WACC'!E16"/>
-    <hyperlink ref="C67" location="'Scenarios'!G9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId24"/>
+    <hyperlink ref="L67" location="'WACC'!E16"/>
+    <hyperlink ref="L68" location="'WACC'!E16"/>
+    <hyperlink ref="L69" location="'WACC'!E16"/>
+    <hyperlink ref="L70" location="'WACC'!E16"/>
+    <hyperlink ref="C71" location="'Scenarios'!G9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4266,7 +4739,7 @@
         </is>
       </c>
       <c r="E6" s="48">
-        <f>DCF!E29</f>
+        <f>DCF!E33</f>
         <v/>
       </c>
     </row>
@@ -4578,7 +5051,7 @@
         </is>
       </c>
       <c r="E25" s="60">
-        <f>DCF!E31</f>
+        <f>DCF!E35</f>
         <v/>
       </c>
     </row>
@@ -4589,7 +5062,7 @@
         </is>
       </c>
       <c r="E26" s="69">
-        <f>DCF!E45</f>
+        <f>DCF!E49</f>
         <v/>
       </c>
     </row>
@@ -4756,7 +5229,7 @@
         </is>
       </c>
       <c r="E38" s="85">
-        <f>DCF!E45</f>
+        <f>DCF!E49</f>
         <v/>
       </c>
       <c r="G38" s="86">
@@ -4820,11 +5293,11 @@
         </is>
       </c>
       <c r="G40" s="84">
-        <f>Scenarios!F59</f>
+        <f>Scenarios!F75</f>
         <v/>
       </c>
       <c r="H40" s="84">
-        <f>Scenarios!H59</f>
+        <f>Scenarios!H75</f>
         <v/>
       </c>
     </row>
@@ -4859,7 +5332,7 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId2"/>
-    <hyperlink ref="C6" location="'DCF'!E29"/>
+    <hyperlink ref="C6" location="'DCF'!E33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
@@ -4875,7 +5348,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId17"/>
-    <hyperlink ref="C38" location="'DCF'!E45"/>
+    <hyperlink ref="C38" location="'DCF'!E49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId20"/>

</xml_diff>

<commit_message>
Widen DCF labels so the AR NWC lines are readable
Column A was 30 characters and was clipping Accounts receivable and total ΔNWC.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1390,7 +1390,7 @@
   <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
@@ -2981,7 +2981,7 @@
   <dimension ref="A1:M71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>

</xml_diff>

<commit_message>
Include AR inside the 7.5% DCF NWC
AR stays its own line, but the NWC % is 7.5% of Δsales including AR so it is not counted twice.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1778,12 +1778,12 @@
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>AR % of revenue (NWC)</t>
+          <t>AR % of revenue (inside NWC)</t>
         </is>
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Own DCF NWC line; wholesale / marketplace mix.</t>
+          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Included in the 7.5% NWC, not added on top.</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. This is the DCF AR / NWC line.</t>
+          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. This AR is inside the 7.5% NWC, not extra.</t>
         </is>
       </c>
       <c r="F14" s="20" t="n">
@@ -1809,12 +1809,12 @@
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>Other NWC (ex-AR) % of Δrevenue</t>
+          <t>NWC % of Δrevenue (includes AR)</t>
         </is>
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>5.8% of Δsales is other NWC (Inv + OCA − AP − accrued). AR is the 1.7% line above, not inside this residual. 1.7+5.8=7.5%.</t>
+          <t>7.5% of Δsales is total NWC and includes AR (1.7% of sales) plus inv, OCA, AP, accrued. AR is inside this 7.5%.</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
@@ -1824,17 +1824,17 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Other NWC ex-AR. Ctrl+F "Inventories" → 1,700,753 | "Accounts payable" → 331,421 | "Accrued liabilities and other" → 662,982. 5.8% of Δsales; AR is the 1.7% line, not in this residual.</t>
+          <t>Ctrl+F "Accounts receivable, net" → 190,657 | "Inventories" → 1,700,753 | "Accounts payable" → 331,421 | "Accrued liabilities and other" → 662,982. 7.5% of Δsales includes AR.</t>
         </is>
       </c>
       <c r="F15" s="20" t="n">
-        <v>0.065</v>
+        <v>0.08</v>
       </c>
       <c r="G15" s="20" t="n">
-        <v>0.058</v>
+        <v>0.075</v>
       </c>
       <c r="H15" s="20" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -2607,95 +2607,95 @@
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other ΔNWC (ex-AR) – year 1</t>
+          <t xml:space="preserve">  Other ΔNWC (NWC − ΔAR) – year 1</t>
         </is>
       </c>
       <c r="F58" s="32">
-        <f>F15*(F18-11102600)</f>
+        <f>F15*(F18-11102600)-F53</f>
         <v/>
       </c>
       <c r="G58" s="32">
-        <f>G15*(G18-11102600)</f>
+        <f>G15*(G18-11102600)-G53</f>
         <v/>
       </c>
       <c r="H58" s="32">
-        <f>H15*(H18-11102600)</f>
+        <f>H15*(H18-11102600)-H53</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other ΔNWC (ex-AR) – year 2</t>
+          <t xml:space="preserve">  Other ΔNWC (NWC − ΔAR) – year 2</t>
         </is>
       </c>
       <c r="F59" s="32">
-        <f>F15*(F19-F18)</f>
+        <f>F15*(F19-F18)-F54</f>
         <v/>
       </c>
       <c r="G59" s="32">
-        <f>G15*(G19-G18)</f>
+        <f>G15*(G19-G18)-G54</f>
         <v/>
       </c>
       <c r="H59" s="32">
-        <f>H15*(H19-H18)</f>
+        <f>H15*(H19-H18)-H54</f>
         <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other ΔNWC (ex-AR) – year 3</t>
+          <t xml:space="preserve">  Other ΔNWC (NWC − ΔAR) – year 3</t>
         </is>
       </c>
       <c r="F60" s="32">
-        <f>F15*(F20-F19)</f>
+        <f>F15*(F20-F19)-F55</f>
         <v/>
       </c>
       <c r="G60" s="32">
-        <f>G15*(G20-G19)</f>
+        <f>G15*(G20-G19)-G55</f>
         <v/>
       </c>
       <c r="H60" s="32">
-        <f>H15*(H20-H19)</f>
+        <f>H15*(H20-H19)-H55</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other ΔNWC (ex-AR) – year 4</t>
+          <t xml:space="preserve">  Other ΔNWC (NWC − ΔAR) – year 4</t>
         </is>
       </c>
       <c r="F61" s="32">
-        <f>F15*(F21-F20)</f>
+        <f>F15*(F21-F20)-F56</f>
         <v/>
       </c>
       <c r="G61" s="32">
-        <f>G15*(G21-G20)</f>
+        <f>G15*(G21-G20)-G56</f>
         <v/>
       </c>
       <c r="H61" s="32">
-        <f>H15*(H21-H20)</f>
+        <f>H15*(H21-H20)-H56</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other ΔNWC (ex-AR) – year 5</t>
+          <t xml:space="preserve">  Other ΔNWC (NWC − ΔAR) – year 5</t>
         </is>
       </c>
       <c r="F62" s="32">
-        <f>F15*(F22-F21)</f>
+        <f>F15*(F22-F21)-F57</f>
         <v/>
       </c>
       <c r="G62" s="32">
-        <f>G15*(G22-G21)</f>
+        <f>G15*(G22-G21)-G57</f>
         <v/>
       </c>
       <c r="H62" s="32">
-        <f>H15*(H22-H21)</f>
+        <f>H15*(H22-H21)-H57</f>
         <v/>
       </c>
     </row>
@@ -3549,12 +3549,12 @@
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AR % of revenue</t>
+          <t xml:space="preserve">  AR % of revenue (included in NWC)</t>
         </is>
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Own DCF NWC line; wholesale / marketplace mix.</t>
+          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Included in the 7.5% NWC, not added on top.</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. This is the DCF AR / NWC line.</t>
+          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. This AR is inside the 7.5% NWC, not extra.</t>
         </is>
       </c>
       <c r="F17" s="20">
@@ -3596,7 +3596,7 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Own DCF NWC line; wholesale / marketplace mix.</t>
+          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Included in the 7.5% NWC, not added on top.</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. This is the DCF AR / NWC line.</t>
+          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. This AR is inside the 7.5% NWC, not extra.</t>
         </is>
       </c>
       <c r="E18" s="47" t="n">
@@ -3640,7 +3640,7 @@
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔAR (increase)/decrease — part of NWC</t>
+          <t xml:space="preserve">  ΔAR (increase)/decrease — included in NWC</t>
         </is>
       </c>
       <c r="F19" s="48">
@@ -3671,12 +3671,12 @@
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other NWC (ex-AR) % of Δrevenue</t>
+          <t xml:space="preserve">  NWC % of Δrevenue (includes AR)</t>
         </is>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>5.8% of Δsales is other NWC (Inv + OCA − AP − accrued). AR is the 1.7% line above, not inside this residual. 1.7+5.8=7.5%.</t>
+          <t>7.5% of Δsales is total NWC and includes AR (1.7% of sales) plus inv, OCA, AP, accrued. AR is inside this 7.5%.</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Other NWC ex-AR. Ctrl+F "Inventories" → 1,700,753 | "Accounts payable" → 331,421 | "Accrued liabilities and other" → 662,982. 5.8% of Δsales; AR is the 1.7% line, not in this residual.</t>
+          <t>Ctrl+F "Accounts receivable, net" → 190,657 | "Inventories" → 1,700,753 | "Accounts payable" → 331,421 | "Accrued liabilities and other" → 662,982. 7.5% of Δsales includes AR.</t>
         </is>
       </c>
       <c r="F20" s="20">
@@ -3713,7 +3713,7 @@
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other ΔNWC (ex-AR) (increase)/decrease</t>
+          <t xml:space="preserve">  Other ΔNWC (NWC − ΔAR)</t>
         </is>
       </c>
       <c r="F21" s="48">
@@ -3775,7 +3775,7 @@
     <row r="23">
       <c r="A23" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: ΔNWC = ΔAR + other ΔNWC. AR is 1.7% of sales (own line); other is 5.8% of Δsales.</t>
+          <t xml:space="preserve">  memo: 7.5% ΔNWC includes AR. ΔAR is shown above and is inside the 7.5%, not added on top.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Put AR inside one DCF NWC line
NWC is a single 7.5% of Δsales that already includes AR. AR is an of-which line, not a separate FCF item.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1387,7 +1387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1778,63 +1778,63 @@
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>AR % of revenue (inside NWC)</t>
+          <t>NWC % of Δrevenue (AR + inv + OCA − AP − accrued)</t>
         </is>
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Included in the 7.5% NWC, not added on top.</t>
+          <t>One NWC line: 7.5% of Δsales = AR + inv + OCA − AP − accrued. AR is not a separate FCF item.</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K: Accounts receivable, net</t>
+          <t>LULU BS/IS historical (10-K)</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. This AR is inside the 7.5% NWC, not extra.</t>
+          <t>One NWC. Ctrl+F "Accounts receivable, net" → 190,657 | "Inventories" → 1,700,753 | "Accounts payable" → 331,421 | "Accrued liabilities and other" → 662,982.</t>
         </is>
       </c>
       <c r="F14" s="20" t="n">
-        <v>0.015</v>
+        <v>0.08</v>
       </c>
       <c r="G14" s="20" t="n">
-        <v>0.017</v>
+        <v>0.075</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>0.02</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>NWC % of Δrevenue (includes AR)</t>
+          <t xml:space="preserve">  of which: AR % of revenue</t>
         </is>
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>7.5% of Δsales is total NWC and includes AR (1.7% of sales) plus inv, OCA, AP, accrued. AR is inside this 7.5%.</t>
+          <t>AR sits inside NWC: 190,657 / 11,102,600 = 1.7% of sales. Same NWC block as inv, OCA, AP, accrued.</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>LULU BS/IS historical (10-K)</t>
+          <t>LULU FY2025 10-K: Accounts receivable, net</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts receivable, net" → 190,657 | "Inventories" → 1,700,753 | "Accounts payable" → 331,421 | "Accrued liabilities and other" → 662,982. 7.5% of Δsales includes AR.</t>
+          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. Lives inside the NWC line below.</t>
         </is>
       </c>
       <c r="F15" s="20" t="n">
-        <v>0.08</v>
+        <v>0.015</v>
       </c>
       <c r="G15" s="20" t="n">
-        <v>0.075</v>
+        <v>0.017</v>
       </c>
       <c r="H15" s="20" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="17">
@@ -2417,537 +2417,347 @@
     <row r="48">
       <c r="A48" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts receivable – year 1</t>
+          <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 1</t>
         </is>
       </c>
       <c r="F48" s="32">
-        <f>F18*F14</f>
+        <f>F18*F15</f>
         <v/>
       </c>
       <c r="G48" s="32">
-        <f>G18*G14</f>
+        <f>G18*G15</f>
         <v/>
       </c>
       <c r="H48" s="32">
-        <f>H18*H14</f>
+        <f>H18*H15</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts receivable – year 2</t>
+          <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 2</t>
         </is>
       </c>
       <c r="F49" s="32">
-        <f>F19*F14</f>
+        <f>F19*F15</f>
         <v/>
       </c>
       <c r="G49" s="32">
-        <f>G19*G14</f>
+        <f>G19*G15</f>
         <v/>
       </c>
       <c r="H49" s="32">
-        <f>H19*H14</f>
+        <f>H19*H15</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts receivable – year 3</t>
+          <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 3</t>
         </is>
       </c>
       <c r="F50" s="32">
-        <f>F20*F14</f>
+        <f>F20*F15</f>
         <v/>
       </c>
       <c r="G50" s="32">
-        <f>G20*G14</f>
+        <f>G20*G15</f>
         <v/>
       </c>
       <c r="H50" s="32">
-        <f>H20*H14</f>
+        <f>H20*H15</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts receivable – year 4</t>
+          <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 4</t>
         </is>
       </c>
       <c r="F51" s="32">
-        <f>F21*F14</f>
+        <f>F21*F15</f>
         <v/>
       </c>
       <c r="G51" s="32">
-        <f>G21*G14</f>
+        <f>G21*G15</f>
         <v/>
       </c>
       <c r="H51" s="32">
-        <f>H21*H14</f>
+        <f>H21*H15</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts receivable – year 5</t>
+          <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 5</t>
         </is>
       </c>
       <c r="F52" s="32">
-        <f>F22*F14</f>
+        <f>F22*F15</f>
         <v/>
       </c>
       <c r="G52" s="32">
-        <f>G22*G14</f>
+        <f>G22*G15</f>
         <v/>
       </c>
       <c r="H52" s="32">
-        <f>H22*H14</f>
+        <f>H22*H15</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔAR – year 1</t>
+          <t xml:space="preserve">  ΔNWC (includes AR) – year 1</t>
         </is>
       </c>
       <c r="F53" s="32">
-        <f>F48-190657</f>
+        <f>F14*(F18-11102600)</f>
         <v/>
       </c>
       <c r="G53" s="32">
-        <f>G48-190657</f>
+        <f>G14*(G18-11102600)</f>
         <v/>
       </c>
       <c r="H53" s="32">
-        <f>H48-190657</f>
+        <f>H14*(H18-11102600)</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔAR – year 2</t>
+          <t xml:space="preserve">  ΔNWC (includes AR) – year 2</t>
         </is>
       </c>
       <c r="F54" s="32">
-        <f>F49-F48</f>
+        <f>F14*(F19-F18)</f>
         <v/>
       </c>
       <c r="G54" s="32">
-        <f>G49-G48</f>
+        <f>G14*(G19-G18)</f>
         <v/>
       </c>
       <c r="H54" s="32">
-        <f>H49-H48</f>
+        <f>H14*(H19-H18)</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔAR – year 3</t>
+          <t xml:space="preserve">  ΔNWC (includes AR) – year 3</t>
         </is>
       </c>
       <c r="F55" s="32">
-        <f>F50-F49</f>
+        <f>F14*(F20-F19)</f>
         <v/>
       </c>
       <c r="G55" s="32">
-        <f>G50-G49</f>
+        <f>G14*(G20-G19)</f>
         <v/>
       </c>
       <c r="H55" s="32">
-        <f>H50-H49</f>
+        <f>H14*(H20-H19)</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔAR – year 4</t>
+          <t xml:space="preserve">  ΔNWC (includes AR) – year 4</t>
         </is>
       </c>
       <c r="F56" s="32">
-        <f>F51-F50</f>
+        <f>F14*(F21-F20)</f>
         <v/>
       </c>
       <c r="G56" s="32">
-        <f>G51-G50</f>
+        <f>G14*(G21-G20)</f>
         <v/>
       </c>
       <c r="H56" s="32">
-        <f>H51-H50</f>
+        <f>H14*(H21-H20)</f>
         <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ΔAR – year 5</t>
+          <t xml:space="preserve">  ΔNWC (includes AR) – year 5</t>
         </is>
       </c>
       <c r="F57" s="32">
-        <f>F52-F51</f>
+        <f>F14*(F22-F21)</f>
         <v/>
       </c>
       <c r="G57" s="32">
-        <f>G52-G51</f>
+        <f>G14*(G22-G21)</f>
         <v/>
       </c>
       <c r="H57" s="32">
-        <f>H52-H51</f>
+        <f>H14*(H22-H21)</f>
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other ΔNWC (NWC − ΔAR) – year 1</t>
+          <t xml:space="preserve">  Unlevered FCF – year 1</t>
         </is>
       </c>
       <c r="F58" s="32">
-        <f>F15*(F18-11102600)-F53</f>
+        <f>F33+F38-F43-F53</f>
         <v/>
       </c>
       <c r="G58" s="32">
-        <f>G15*(G18-11102600)-G53</f>
+        <f>G33+G38-G43-G53</f>
         <v/>
       </c>
       <c r="H58" s="32">
-        <f>H15*(H18-11102600)-H53</f>
+        <f>H33+H38-H43-H53</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other ΔNWC (NWC − ΔAR) – year 2</t>
+          <t xml:space="preserve">  Unlevered FCF – year 2</t>
         </is>
       </c>
       <c r="F59" s="32">
-        <f>F15*(F19-F18)-F54</f>
+        <f>F34+F39-F44-F54</f>
         <v/>
       </c>
       <c r="G59" s="32">
-        <f>G15*(G19-G18)-G54</f>
+        <f>G34+G39-G44-G54</f>
         <v/>
       </c>
       <c r="H59" s="32">
-        <f>H15*(H19-H18)-H54</f>
+        <f>H34+H39-H44-H54</f>
         <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other ΔNWC (NWC − ΔAR) – year 3</t>
+          <t xml:space="preserve">  Unlevered FCF – year 3</t>
         </is>
       </c>
       <c r="F60" s="32">
-        <f>F15*(F20-F19)-F55</f>
+        <f>F35+F40-F45-F55</f>
         <v/>
       </c>
       <c r="G60" s="32">
-        <f>G15*(G20-G19)-G55</f>
+        <f>G35+G40-G45-G55</f>
         <v/>
       </c>
       <c r="H60" s="32">
-        <f>H15*(H20-H19)-H55</f>
+        <f>H35+H40-H45-H55</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other ΔNWC (NWC − ΔAR) – year 4</t>
+          <t xml:space="preserve">  Unlevered FCF – year 4</t>
         </is>
       </c>
       <c r="F61" s="32">
-        <f>F15*(F21-F20)-F56</f>
+        <f>F36+F41-F46-F56</f>
         <v/>
       </c>
       <c r="G61" s="32">
-        <f>G15*(G21-G20)-G56</f>
+        <f>G36+G41-G46-G56</f>
         <v/>
       </c>
       <c r="H61" s="32">
-        <f>H15*(H21-H20)-H56</f>
+        <f>H36+H41-H46-H56</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Other ΔNWC (NWC − ΔAR) – year 5</t>
+          <t xml:space="preserve">  Unlevered FCF – year 5</t>
         </is>
       </c>
       <c r="F62" s="32">
-        <f>F15*(F22-F21)-F57</f>
+        <f>F37+F42-F47-F57</f>
         <v/>
       </c>
       <c r="G62" s="32">
-        <f>G15*(G22-G21)-G57</f>
+        <f>G37+G42-G47-G57</f>
         <v/>
       </c>
       <c r="H62" s="32">
-        <f>H15*(H22-H21)-H57</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ΔNWC – year 1</t>
-        </is>
-      </c>
-      <c r="F63" s="32">
-        <f>F53+F58</f>
-        <v/>
-      </c>
-      <c r="G63" s="32">
-        <f>G53+G58</f>
-        <v/>
-      </c>
-      <c r="H63" s="32">
-        <f>H53+H58</f>
+        <f>H37+H42-H47-H57</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ΔNWC – year 2</t>
-        </is>
-      </c>
-      <c r="F64" s="32">
-        <f>F54+F59</f>
-        <v/>
-      </c>
-      <c r="G64" s="32">
-        <f>G54+G59</f>
-        <v/>
-      </c>
-      <c r="H64" s="32">
-        <f>H54+H59</f>
+      <c r="A64" s="22" t="inlineStr">
+        <is>
+          <t>Enterprise value (DCF)</t>
+        </is>
+      </c>
+      <c r="F64" s="34">
+        <f>NPV(F9,F58,F59,F60,F61,F62)+(F62*(1+F10)/(F9-F10))/(1+F9)^5</f>
+        <v/>
+      </c>
+      <c r="G64" s="34">
+        <f>NPV(G9,G58,G59,G60,G61,G62)+(G62*(1+G10)/(G9-G10))/(1+G9)^5</f>
+        <v/>
+      </c>
+      <c r="H64" s="34">
+        <f>NPV(H9,H58,H59,H60,H61,H62)+(H62*(1+H10)/(H9-H10))/(1+H9)^5</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ΔNWC – year 3</t>
-        </is>
-      </c>
-      <c r="F65" s="32">
-        <f>F55+F60</f>
-        <v/>
-      </c>
-      <c r="G65" s="32">
-        <f>G55+G60</f>
-        <v/>
-      </c>
-      <c r="H65" s="32">
-        <f>H55+H60</f>
+      <c r="A65" s="35" t="inlineStr">
+        <is>
+          <t>Implied share price</t>
+        </is>
+      </c>
+      <c r="F65" s="36">
+        <f>(F64+1807202-0)/111380</f>
+        <v/>
+      </c>
+      <c r="G65" s="37">
+        <f>(G64+1807202-0)/111380</f>
+        <v/>
+      </c>
+      <c r="H65" s="36">
+        <f>(H64+1807202-0)/111380</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ΔNWC – year 4</t>
-        </is>
-      </c>
-      <c r="F66" s="32">
-        <f>F56+F61</f>
-        <v/>
-      </c>
-      <c r="G66" s="32">
-        <f>G56+G61</f>
-        <v/>
-      </c>
-      <c r="H66" s="32">
-        <f>H56+H61</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ΔNWC – year 5</t>
-        </is>
-      </c>
-      <c r="F67" s="32">
-        <f>F57+F62</f>
-        <v/>
-      </c>
-      <c r="G67" s="32">
-        <f>G57+G62</f>
-        <v/>
-      </c>
-      <c r="H67" s="32">
-        <f>H57+H62</f>
+      <c r="A66" s="22" t="inlineStr">
+        <is>
+          <t>Upside / (downside) vs current</t>
+        </is>
+      </c>
+      <c r="F66" s="38">
+        <f>F65/100.0-1</f>
+        <v/>
+      </c>
+      <c r="G66" s="38">
+        <f>G65/100.0-1</f>
+        <v/>
+      </c>
+      <c r="H66" s="38">
+        <f>H65/100.0-1</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Unlevered FCF – year 1</t>
-        </is>
-      </c>
-      <c r="F68" s="32">
-        <f>F33+F38-F43-F63</f>
-        <v/>
-      </c>
-      <c r="G68" s="32">
-        <f>G33+G38-G43-G63</f>
-        <v/>
-      </c>
-      <c r="H68" s="32">
-        <f>H33+H38-H43-H63</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Unlevered FCF – year 2</t>
-        </is>
-      </c>
-      <c r="F69" s="32">
-        <f>F34+F39-F44-F64</f>
-        <v/>
-      </c>
-      <c r="G69" s="32">
-        <f>G34+G39-G44-G64</f>
-        <v/>
-      </c>
-      <c r="H69" s="32">
-        <f>H34+H39-H44-H64</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Unlevered FCF – year 3</t>
-        </is>
-      </c>
-      <c r="F70" s="32">
-        <f>F35+F40-F45-F65</f>
-        <v/>
-      </c>
-      <c r="G70" s="32">
-        <f>G35+G40-G45-G65</f>
-        <v/>
-      </c>
-      <c r="H70" s="32">
-        <f>H35+H40-H45-H65</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Unlevered FCF – year 4</t>
-        </is>
-      </c>
-      <c r="F71" s="32">
-        <f>F36+F41-F46-F66</f>
-        <v/>
-      </c>
-      <c r="G71" s="32">
-        <f>G36+G41-G46-G66</f>
-        <v/>
-      </c>
-      <c r="H71" s="32">
-        <f>H36+H41-H46-H66</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Unlevered FCF – year 5</t>
-        </is>
-      </c>
-      <c r="F72" s="32">
-        <f>F37+F42-F47-F67</f>
-        <v/>
-      </c>
-      <c r="G72" s="32">
-        <f>G37+G42-G47-G67</f>
-        <v/>
-      </c>
-      <c r="H72" s="32">
-        <f>H37+H42-H47-H67</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="22" t="inlineStr">
-        <is>
-          <t>Enterprise value (DCF)</t>
-        </is>
-      </c>
-      <c r="F74" s="34">
-        <f>NPV(F9,F68,F69,F70,F71,F72)+(F72*(1+F10)/(F9-F10))/(1+F9)^5</f>
-        <v/>
-      </c>
-      <c r="G74" s="34">
-        <f>NPV(G9,G68,G69,G70,G71,G72)+(G72*(1+G10)/(G9-G10))/(1+G9)^5</f>
-        <v/>
-      </c>
-      <c r="H74" s="34">
-        <f>NPV(H9,H68,H69,H70,H71,H72)+(H72*(1+H10)/(H9-H10))/(1+H9)^5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="35" t="inlineStr">
-        <is>
-          <t>Implied share price</t>
-        </is>
-      </c>
-      <c r="F75" s="36">
-        <f>(F74+1807202-0)/111380</f>
-        <v/>
-      </c>
-      <c r="G75" s="37">
-        <f>(G74+1807202-0)/111380</f>
-        <v/>
-      </c>
-      <c r="H75" s="36">
-        <f>(H74+1807202-0)/111380</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="22" t="inlineStr">
-        <is>
-          <t>Upside / (downside) vs current</t>
-        </is>
-      </c>
-      <c r="F76" s="38">
-        <f>F75/100.0-1</f>
-        <v/>
-      </c>
-      <c r="G76" s="38">
-        <f>G75/100.0-1</f>
-        <v/>
-      </c>
-      <c r="H76" s="38">
-        <f>H75/100.0-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="39" t="inlineStr">
+      <c r="A68" s="39" t="inlineStr">
         <is>
           <t>Current price $100.00; cash $1,807,202 k; net debt $0 (net-cash balance sheet).</t>
         </is>
@@ -2978,7 +2788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M71"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -3549,22 +3359,22 @@
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AR % of revenue (included in NWC)</t>
+          <t>NWC % of Δrevenue (AR + inv + OCA − AP − accrued)</t>
         </is>
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Included in the 7.5% NWC, not added on top.</t>
+          <t>One NWC line: 7.5% of Δsales = AR + inv + OCA − AP − accrued. AR is not a separate FCF item.</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K: Accounts receivable, net</t>
+          <t>LULU BS/IS historical (10-K)</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. This AR is inside the 7.5% NWC, not extra.</t>
+          <t>One NWC. Ctrl+F "Accounts receivable, net" → 190,657 | "Inventories" → 1,700,753 | "Accounts payable" → 331,421 | "Accrued liabilities and other" → 662,982.</t>
         </is>
       </c>
       <c r="F17" s="20">
@@ -3591,12 +3401,12 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>Accounts receivable, net</t>
+          <t xml:space="preserve">  of which: AR % of revenue</t>
         </is>
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>AR 1.7% of sales = FY25 Accounts receivable, net 190,657 / 11,102,600. Included in the 7.5% NWC, not added on top.</t>
+          <t>AR sits inside NWC: 190,657 / 11,102,600 = 1.7% of sales. Same NWC block as inv, OCA, AP, accrued.</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
@@ -3606,422 +3416,391 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. This AR is inside the 7.5% NWC, not extra.</t>
-        </is>
-      </c>
-      <c r="E18" s="47" t="n">
+          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. Lives inside the NWC line below.</t>
+        </is>
+      </c>
+      <c r="F18" s="20">
+        <f>Scenarios!$G$15</f>
+        <v/>
+      </c>
+      <c r="G18" s="20">
+        <f>Scenarios!$G$15</f>
+        <v/>
+      </c>
+      <c r="H18" s="20">
+        <f>Scenarios!$G$15</f>
+        <v/>
+      </c>
+      <c r="I18" s="20">
+        <f>Scenarios!$G$15</f>
+        <v/>
+      </c>
+      <c r="J18" s="20">
+        <f>Scenarios!$G$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which: Accounts receivable, net</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>AR sits inside NWC: 190,657 / 11,102,600 = 1.7% of sales. Same NWC block as inv, OCA, AP, accrued.</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: Accounts receivable, net</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. Lives inside the NWC line below.</t>
+        </is>
+      </c>
+      <c r="E19" s="47" t="n">
         <v>190657</v>
       </c>
-      <c r="F18" s="48">
+      <c r="F19" s="48">
         <f>Scenarios!G48</f>
         <v/>
       </c>
-      <c r="G18" s="48">
+      <c r="G19" s="48">
         <f>Scenarios!G49</f>
         <v/>
       </c>
-      <c r="H18" s="48">
+      <c r="H19" s="48">
         <f>Scenarios!G50</f>
         <v/>
       </c>
-      <c r="I18" s="48">
+      <c r="I19" s="48">
         <f>Scenarios!G51</f>
         <v/>
       </c>
-      <c r="J18" s="48">
+      <c r="J19" s="48">
         <f>Scenarios!G52</f>
         <v/>
       </c>
-      <c r="K18" s="49">
-        <f>IF(MAX(ABS(F18-Scenarios!$G$48),ABS(G18-Scenarios!$G$49),ABS(H18-Scenarios!$G$50),ABS(I18-Scenarios!$G$51),ABS(J18-Scenarios!$G$52))&lt;0.5,"OK","CHECK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ΔAR (increase)/decrease — included in NWC</t>
-        </is>
-      </c>
-      <c r="F19" s="48">
+      <c r="K19" s="49">
+        <f>IF(MAX(ABS(F19-Scenarios!$G$48),ABS(G19-Scenarios!$G$49),ABS(H19-Scenarios!$G$50),ABS(I19-Scenarios!$G$51),ABS(J19-Scenarios!$G$52))&lt;0.5,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>(Increase)/decrease in NWC (includes AR)</t>
+        </is>
+      </c>
+      <c r="F20" s="48">
         <f>-Scenarios!G53</f>
         <v/>
       </c>
-      <c r="G19" s="48">
+      <c r="G20" s="48">
         <f>-Scenarios!G54</f>
         <v/>
       </c>
-      <c r="H19" s="48">
+      <c r="H20" s="48">
         <f>-Scenarios!G55</f>
         <v/>
       </c>
-      <c r="I19" s="48">
+      <c r="I20" s="48">
         <f>-Scenarios!G56</f>
         <v/>
       </c>
-      <c r="J19" s="48">
+      <c r="J20" s="48">
         <f>-Scenarios!G57</f>
         <v/>
       </c>
-      <c r="K19" s="49">
-        <f>IF(MAX(ABS(F19+Scenarios!$G$53),ABS(G19+Scenarios!$G$54),ABS(H19+Scenarios!$G$55),ABS(I19+Scenarios!$G$56),ABS(J19+Scenarios!$G$57))&lt;0.5,"OK","CHECK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NWC % of Δrevenue (includes AR)</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>7.5% of Δsales is total NWC and includes AR (1.7% of sales) plus inv, OCA, AP, accrued. AR is inside this 7.5%.</t>
-        </is>
-      </c>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>LULU BS/IS historical (10-K)</t>
-        </is>
-      </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Accounts receivable, net" → 190,657 | "Inventories" → 1,700,753 | "Accounts payable" → 331,421 | "Accrued liabilities and other" → 662,982. 7.5% of Δsales includes AR.</t>
-        </is>
-      </c>
-      <c r="F20" s="20">
-        <f>Scenarios!$G$15</f>
-        <v/>
-      </c>
-      <c r="G20" s="20">
-        <f>Scenarios!$G$15</f>
-        <v/>
-      </c>
-      <c r="H20" s="20">
-        <f>Scenarios!$G$15</f>
-        <v/>
-      </c>
-      <c r="I20" s="20">
-        <f>Scenarios!$G$15</f>
-        <v/>
-      </c>
-      <c r="J20" s="20">
-        <f>Scenarios!$G$15</f>
+      <c r="K20" s="49">
+        <f>IF(MAX(ABS(F20+Scenarios!$G$53),ABS(G20+Scenarios!$G$54),ABS(H20+Scenarios!$G$55),ABS(I20+Scenarios!$G$56),ABS(J20+Scenarios!$G$57))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Other ΔNWC (NWC − ΔAR)</t>
-        </is>
-      </c>
-      <c r="F21" s="48">
-        <f>-Scenarios!G58</f>
-        <v/>
-      </c>
-      <c r="G21" s="48">
-        <f>-Scenarios!G59</f>
-        <v/>
-      </c>
-      <c r="H21" s="48">
-        <f>-Scenarios!G60</f>
-        <v/>
-      </c>
-      <c r="I21" s="48">
-        <f>-Scenarios!G61</f>
-        <v/>
-      </c>
-      <c r="J21" s="48">
-        <f>-Scenarios!G62</f>
-        <v/>
-      </c>
-      <c r="K21" s="49">
-        <f>IF(MAX(ABS(F21+Scenarios!$G$58),ABS(G21+Scenarios!$G$59),ABS(H21+Scenarios!$G$60),ABS(I21+Scenarios!$G$61),ABS(J21+Scenarios!$G$62))&lt;0.5,"OK","CHECK")</f>
-        <v/>
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  memo: NWC and AR are one line. 7.5% of Δsales already includes AR; UFCF does not take ΔAR separately.</t>
+        </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>Total (increase)/decrease in net working capital</t>
-        </is>
-      </c>
-      <c r="F22" s="48">
-        <f>-Scenarios!G63</f>
-        <v/>
-      </c>
-      <c r="G22" s="48">
-        <f>-Scenarios!G64</f>
-        <v/>
-      </c>
-      <c r="H22" s="48">
-        <f>-Scenarios!G65</f>
-        <v/>
-      </c>
-      <c r="I22" s="48">
-        <f>-Scenarios!G66</f>
-        <v/>
-      </c>
-      <c r="J22" s="48">
-        <f>-Scenarios!G67</f>
-        <v/>
-      </c>
-      <c r="K22" s="49">
-        <f>IF(MAX(ABS(F22+Scenarios!$G$63),ABS(G22+Scenarios!$G$64),ABS(H22+Scenarios!$G$65),ABS(I22+Scenarios!$G$66),ABS(J22+Scenarios!$G$67))&lt;0.5,"OK","CHECK")</f>
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>Unlevered free cash flow</t>
+        </is>
+      </c>
+      <c r="F22" s="54">
+        <f>Scenarios!G58</f>
+        <v/>
+      </c>
+      <c r="G22" s="54">
+        <f>Scenarios!G59</f>
+        <v/>
+      </c>
+      <c r="H22" s="54">
+        <f>Scenarios!G60</f>
+        <v/>
+      </c>
+      <c r="I22" s="54">
+        <f>Scenarios!G61</f>
+        <v/>
+      </c>
+      <c r="J22" s="54">
+        <f>Scenarios!G62</f>
+        <v/>
+      </c>
+      <c r="K22" s="52">
+        <f>IF(MAX(ABS(F22-Scenarios!$G$58),ABS(G22-Scenarios!$G$59),ABS(H22-Scenarios!$G$60),ABS(I22-Scenarios!$G$61),ABS(J22-Scenarios!$G$62))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  memo: 7.5% ΔNWC includes AR. ΔAR is shown above and is inside the 7.5%, not added on top.</t>
-        </is>
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Discount period (years)</t>
+        </is>
+      </c>
+      <c r="F23" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="I23" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="J23" s="55" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="22" t="inlineStr">
-        <is>
-          <t>Unlevered free cash flow</t>
-        </is>
-      </c>
-      <c r="F24" s="54">
-        <f>Scenarios!G68</f>
-        <v/>
-      </c>
-      <c r="G24" s="54">
-        <f>Scenarios!G69</f>
-        <v/>
-      </c>
-      <c r="H24" s="54">
-        <f>Scenarios!G70</f>
-        <v/>
-      </c>
-      <c r="I24" s="54">
-        <f>Scenarios!G71</f>
-        <v/>
-      </c>
-      <c r="J24" s="54">
-        <f>Scenarios!G72</f>
-        <v/>
-      </c>
-      <c r="K24" s="52">
-        <f>IF(MAX(ABS(F24-Scenarios!$G$68),ABS(G24-Scenarios!$G$69),ABS(H24-Scenarios!$G$70),ABS(I24-Scenarios!$G$71),ABS(J24-Scenarios!$G$72))&lt;0.5,"OK","CHECK")</f>
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>Discount factor @ WACC</t>
+        </is>
+      </c>
+      <c r="F24" s="56">
+        <f>1/(1+Scenarios!$G$9)^F23</f>
+        <v/>
+      </c>
+      <c r="G24" s="56">
+        <f>1/(1+Scenarios!$G$9)^G23</f>
+        <v/>
+      </c>
+      <c r="H24" s="56">
+        <f>1/(1+Scenarios!$G$9)^H23</f>
+        <v/>
+      </c>
+      <c r="I24" s="56">
+        <f>1/(1+Scenarios!$G$9)^I23</f>
+        <v/>
+      </c>
+      <c r="J24" s="56">
+        <f>1/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>Discount period (years)</t>
-        </is>
-      </c>
-      <c r="F25" s="55" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" s="55" t="n">
-        <v>2</v>
-      </c>
-      <c r="H25" s="55" t="n">
-        <v>3</v>
-      </c>
-      <c r="I25" s="55" t="n">
-        <v>4</v>
-      </c>
-      <c r="J25" s="55" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t>Discount factor @ WACC</t>
-        </is>
-      </c>
-      <c r="F26" s="56">
-        <f>1/(1+Scenarios!$G$9)^F25</f>
-        <v/>
-      </c>
-      <c r="G26" s="56">
-        <f>1/(1+Scenarios!$G$9)^G25</f>
-        <v/>
-      </c>
-      <c r="H26" s="56">
-        <f>1/(1+Scenarios!$G$9)^H25</f>
-        <v/>
-      </c>
-      <c r="I26" s="56">
-        <f>1/(1+Scenarios!$G$9)^I25</f>
-        <v/>
-      </c>
-      <c r="J26" s="56">
-        <f>1/(1+Scenarios!$G$9)^J25</f>
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>PV of unlevered FCF</t>
+        </is>
+      </c>
+      <c r="F25" s="34">
+        <f>F22*F24</f>
+        <v/>
+      </c>
+      <c r="G25" s="34">
+        <f>G22*G24</f>
+        <v/>
+      </c>
+      <c r="H25" s="34">
+        <f>H22*H24</f>
+        <v/>
+      </c>
+      <c r="I25" s="34">
+        <f>I22*I24</f>
+        <v/>
+      </c>
+      <c r="J25" s="34">
+        <f>J22*J24</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="22" t="inlineStr">
-        <is>
-          <t>PV of unlevered FCF</t>
-        </is>
-      </c>
-      <c r="F27" s="34">
-        <f>F24*F26</f>
-        <v/>
-      </c>
-      <c r="G27" s="34">
-        <f>G24*G26</f>
-        <v/>
-      </c>
-      <c r="H27" s="34">
-        <f>H24*H26</f>
-        <v/>
-      </c>
-      <c r="I27" s="34">
-        <f>I24*I26</f>
-        <v/>
-      </c>
-      <c r="J27" s="34">
-        <f>J24*J26</f>
-        <v/>
-      </c>
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>Scenarios linkage summary (column K should all read OK)</t>
+        </is>
+      </c>
+      <c r="K27" s="57">
+        <f>IF(COUNTIF(K5:K22,"CHECK")=0,"ALL OK","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="58" t="inlineStr">
+        <is>
+          <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="n"/>
+      <c r="C28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t>Scenarios linkage summary (column K should all read OK)</t>
-        </is>
-      </c>
-      <c r="K29" s="57">
-        <f>IF(COUNTIF(K5:K24,"CHECK")=0,"ALL OK","REVIEW")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="58" t="inlineStr">
-        <is>
-          <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="n"/>
-      <c r="C30" s="13" t="n"/>
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>Sum of PV of explicit FCF (FY26–FY30)</t>
+        </is>
+      </c>
+      <c r="E29" s="59">
+        <f>SUM(F25:J25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>Terminal growth rate (g)</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>2.25% terminal g sits next to FRED GDPC1 Q2/Q2 real GDP ≈ 2.1% (24,269.613 / 23,770.976 − 1).</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>FRED: Real GDP (GDPC1)</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Q2 2026" → 24,269.613 and "Q2 2025" → 23,770.976. YoY = 2.1%. Model terminal g 2.25%.</t>
+        </is>
+      </c>
+      <c r="E30" s="50">
+        <f>Scenarios!$G$10</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="22" t="inlineStr">
         <is>
-          <t>Sum of PV of explicit FCF (FY26–FY30)</t>
-        </is>
-      </c>
-      <c r="E31" s="59">
-        <f>SUM(F27:J27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1">
+          <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
+        </is>
+      </c>
+      <c r="E31" s="34">
+        <f>J9+J14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t>Terminal growth rate (g)</t>
-        </is>
-      </c>
-      <c r="B32" s="17" t="inlineStr">
-        <is>
-          <t>2.25% terminal g sits next to FRED GDPC1 Q2/Q2 real GDP ≈ 2.1% (24,269.613 / 23,770.976 − 1).</t>
-        </is>
-      </c>
-      <c r="C32" s="18" t="inlineStr">
-        <is>
-          <t>FRED: Real GDP (GDPC1)</t>
-        </is>
-      </c>
-      <c r="D32" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Q2 2026" → 24,269.613 and "Q2 2025" → 23,770.976. YoY = 2.1%. Model terminal g 2.25%.</t>
-        </is>
-      </c>
-      <c r="E32" s="50">
-        <f>Scenarios!$G$10</f>
+          <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
+        </is>
+      </c>
+      <c r="E32" s="48">
+        <f>J22*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="22" t="inlineStr">
-        <is>
-          <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
-        </is>
-      </c>
-      <c r="E33" s="34">
-        <f>J9+J14</f>
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Implied exit EV/EBITDA (Gordon Growth)</t>
+        </is>
+      </c>
+      <c r="E33" s="60">
+        <f>E32/E31</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
-        </is>
-      </c>
-      <c r="E34" s="48">
-        <f>J24*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
+      <c r="A34" s="22" t="inlineStr">
+        <is>
+          <t>PV of terminal value</t>
+        </is>
+      </c>
+      <c r="E34" s="59">
+        <f>E32/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Implied exit EV/EBITDA (Gordon Growth)</t>
-        </is>
-      </c>
-      <c r="E35" s="60">
-        <f>E34/E33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="22" t="inlineStr">
-        <is>
-          <t>PV of terminal value</t>
-        </is>
-      </c>
-      <c r="E36" s="59">
-        <f>E34/(1+Scenarios!$G$9)^J25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="22" t="inlineStr">
+      <c r="A35" s="22" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="E37" s="34">
-        <f>E31+E36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="16" t="inlineStr">
+      <c r="E35" s="34">
+        <f>E29+E34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>Plus: cash &amp; equivalents (FY2025)</t>
         </is>
       </c>
-      <c r="C38" s="61" t="inlineStr">
+      <c r="C36" s="61" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="D38" s="19" t="inlineStr">
+      <c r="D36" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
         </is>
       </c>
-      <c r="E38" s="47" t="n">
+      <c r="E36" s="47" t="n">
         <v>1807202</v>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>Less: total debt</t>
+        </is>
+      </c>
+      <c r="C37" s="61" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "no borrowings were outstanding under this facility" → no funded term debt</t>
+        </is>
+      </c>
+      <c r="E37" s="47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>Equity value</t>
+        </is>
+      </c>
+      <c r="E38" s="34">
+        <f>E35+E36+E37</f>
+        <v/>
       </c>
     </row>
     <row r="39" ht="28" customHeight="1">
       <c r="A39" s="16" t="inlineStr">
         <is>
-          <t>Less: total debt</t>
+          <t>Diluted shares outstanding (000)</t>
         </is>
       </c>
       <c r="C39" s="61" t="inlineStr">
@@ -4031,373 +3810,412 @@
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "no borrowings were outstanding under this facility" → no funded term debt</t>
+          <t>Ctrl+F "Diluted weighted-average number of shares outstanding" → 119,068 (000)</t>
         </is>
       </c>
       <c r="E39" s="47" t="n">
-        <v>0</v>
+        <v>111380</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="22" t="inlineStr">
         <is>
-          <t>Equity value</t>
-        </is>
-      </c>
-      <c r="E40" s="34">
-        <f>E37+E38+E39</f>
+          <t>Implied value per share</t>
+        </is>
+      </c>
+      <c r="E40" s="62">
+        <f>E38/E39</f>
+        <v/>
+      </c>
+      <c r="K40" s="52">
+        <f>IF(ABS(E40-Scenarios!$G$65)&lt;0.05,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="16" t="inlineStr">
         <is>
-          <t>Diluted shares outstanding (000)</t>
+          <t>Current share price</t>
         </is>
       </c>
       <c r="C41" s="61" t="inlineStr">
         <is>
-          <t>10-K</t>
+          <t>NASDAQ</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Diluted weighted-average number of shares outstanding" → 119,068 (000)</t>
-        </is>
-      </c>
-      <c r="E41" s="47" t="n">
-        <v>111380</v>
+          <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
+        </is>
+      </c>
+      <c r="E41" s="63" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="22" t="inlineStr">
         <is>
-          <t>Implied value per share</t>
-        </is>
-      </c>
-      <c r="E42" s="62">
-        <f>E40/E41</f>
-        <v/>
-      </c>
-      <c r="K42" s="52">
-        <f>IF(ABS(E42-Scenarios!$G$75)&lt;0.05,"OK","CHECK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" ht="28" customHeight="1">
+          <t>Implied upside / (downside)</t>
+        </is>
+      </c>
+      <c r="E42" s="64">
+        <f>E40/E41-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
       <c r="A43" s="16" t="inlineStr">
         <is>
-          <t>Current share price</t>
-        </is>
-      </c>
-      <c r="C43" s="61" t="inlineStr">
-        <is>
-          <t>NASDAQ</t>
-        </is>
-      </c>
-      <c r="D43" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
-        </is>
-      </c>
-      <c r="E43" s="63" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="22" t="inlineStr">
-        <is>
-          <t>Implied upside / (downside)</t>
-        </is>
-      </c>
-      <c r="E44" s="64">
-        <f>E42/E43-1</f>
+          <t xml:space="preserve">  memo: % of EV from terminal value</t>
+        </is>
+      </c>
+      <c r="E43" s="50">
+        <f>E34/E35</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  memo: % of EV from terminal value</t>
-        </is>
-      </c>
-      <c r="E45" s="50">
-        <f>E36/E37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="58" t="inlineStr">
+      <c r="A45" s="58" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
       </c>
-      <c r="B47" s="13" t="n"/>
-      <c r="C47" s="13" t="n"/>
+      <c r="B45" s="13" t="n"/>
+      <c r="C45" s="13" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>Exit multiple selection (see Comps tab for peer build)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="28" customHeight="1">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>Selected exit EV/EBITDA multiple (FY2030E)</t>
+        </is>
+      </c>
+      <c r="B47" s="17" t="inlineStr">
+        <is>
+          <t>8.0x FY2030E exit EV/EBITDA; mid-point of terminal football field (6.5–9.5x); ~1 turn above Gordon-implied ~7x.</t>
+        </is>
+      </c>
+      <c r="C47" s="18" t="inlineStr">
+        <is>
+          <t>StockAnalysis: LULU EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="D47" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x (assumption)</t>
+        </is>
+      </c>
+      <c r="E47" s="65" t="n">
+        <v>8</v>
+      </c>
+      <c r="M47" s="61" t="inlineStr">
+        <is>
+          <t>Comps: Exit Multiple Build</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="15" t="inlineStr">
-        <is>
-          <t>Exit multiple selection (see Comps tab for peer build)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="28" customHeight="1">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>Terminal value = Terminal EBITDA × exit multiple</t>
+        </is>
+      </c>
+      <c r="E48" s="48">
+        <f>E31*E47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>Selected exit EV/EBITDA multiple (FY2030E)</t>
-        </is>
-      </c>
-      <c r="B49" s="17" t="inlineStr">
-        <is>
-          <t>8.0x FY2030E exit EV/EBITDA; mid-point of terminal football field (6.5–9.5x); ~1 turn above Gordon-implied ~7x.</t>
-        </is>
-      </c>
-      <c r="C49" s="18" t="inlineStr">
-        <is>
-          <t>StockAnalysis: LULU EV/EBITDA</t>
-        </is>
-      </c>
-      <c r="D49" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x (assumption)</t>
-        </is>
-      </c>
-      <c r="E49" s="65" t="n">
-        <v>8</v>
-      </c>
-      <c r="M49" s="61" t="inlineStr">
-        <is>
-          <t>Comps: Exit Multiple Build</t>
-        </is>
+          <t>PV of terminal value</t>
+        </is>
+      </c>
+      <c r="E49" s="48">
+        <f>E48/(1+Scenarios!$G$9)^J23</f>
+        <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="16" t="inlineStr">
-        <is>
-          <t>Terminal value = Terminal EBITDA × exit multiple</t>
-        </is>
-      </c>
-      <c r="E50" s="48">
-        <f>E33*E49</f>
+      <c r="A50" s="22" t="inlineStr">
+        <is>
+          <t>Enterprise value (exit method)</t>
+        </is>
+      </c>
+      <c r="E50" s="34">
+        <f>E29+E49</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="16" t="inlineStr">
-        <is>
-          <t>PV of terminal value</t>
-        </is>
-      </c>
-      <c r="E51" s="48">
-        <f>E50/(1+Scenarios!$G$9)^J25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="22" t="inlineStr">
-        <is>
-          <t>Enterprise value (exit method)</t>
-        </is>
-      </c>
-      <c r="E52" s="34">
-        <f>E31+E51</f>
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>Implied value per share (exit method)</t>
+        </is>
+      </c>
+      <c r="E51" s="66">
+        <f>(E50+E36+E37)/E39</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="22" t="inlineStr">
-        <is>
-          <t>Implied value per share (exit method)</t>
-        </is>
-      </c>
-      <c r="E53" s="66">
-        <f>(E52+E38+E39)/E41</f>
-        <v/>
+      <c r="A53" s="58" t="inlineStr">
+        <is>
+          <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
+        </is>
+      </c>
+      <c r="B53" s="13" t="n"/>
+      <c r="C53" s="13" t="n"/>
+      <c r="D53" s="13" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="67" t="inlineStr"/>
+      <c r="B54" s="68" t="inlineStr">
+        <is>
+          <t>Gordon Growth</t>
+        </is>
+      </c>
+      <c r="C54" s="68" t="inlineStr">
+        <is>
+          <t>Exit Multiple</t>
+        </is>
+      </c>
+      <c r="D54" s="68" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="58" t="inlineStr">
-        <is>
-          <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
-        </is>
-      </c>
-      <c r="B55" s="13" t="n"/>
-      <c r="C55" s="13" t="n"/>
-      <c r="D55" s="13" t="n"/>
+      <c r="A55" s="22" t="inlineStr">
+        <is>
+          <t>Terminal value ($)</t>
+        </is>
+      </c>
+      <c r="B55" s="59">
+        <f>E32</f>
+        <v/>
+      </c>
+      <c r="C55" s="59">
+        <f>E48</f>
+        <v/>
+      </c>
+      <c r="D55" s="59">
+        <f>B55-C55</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="67" t="inlineStr"/>
-      <c r="B56" s="68" t="inlineStr">
-        <is>
-          <t>Gordon Growth</t>
-        </is>
-      </c>
-      <c r="C56" s="68" t="inlineStr">
-        <is>
-          <t>Exit Multiple</t>
-        </is>
-      </c>
-      <c r="D56" s="68" t="inlineStr">
-        <is>
-          <t>Variance</t>
-        </is>
+      <c r="A56" s="22" t="inlineStr">
+        <is>
+          <t>Exit EV/EBITDA (implied vs selected)</t>
+        </is>
+      </c>
+      <c r="B56" s="69">
+        <f>E33</f>
+        <v/>
+      </c>
+      <c r="C56" s="69">
+        <f>E47</f>
+        <v/>
+      </c>
+      <c r="D56" s="69">
+        <f>B56-C56</f>
+        <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="22" t="inlineStr">
-        <is>
-          <t>Terminal value ($)</t>
-        </is>
-      </c>
-      <c r="B57" s="59">
-        <f>E34</f>
-        <v/>
-      </c>
-      <c r="C57" s="59">
-        <f>E50</f>
-        <v/>
-      </c>
-      <c r="D57" s="59">
-        <f>B57-C57</f>
+      <c r="A57" s="16" t="inlineStr">
+        <is>
+          <t>Terminal value variance (%)</t>
+        </is>
+      </c>
+      <c r="B57" s="50" t="inlineStr"/>
+      <c r="C57" s="50" t="inlineStr"/>
+      <c r="D57" s="50">
+        <f>(B55-C55)/B55</f>
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="22" t="inlineStr">
         <is>
-          <t>Exit EV/EBITDA (implied vs selected)</t>
-        </is>
-      </c>
-      <c r="B58" s="69">
-        <f>E35</f>
-        <v/>
-      </c>
-      <c r="C58" s="69">
-        <f>E49</f>
-        <v/>
-      </c>
-      <c r="D58" s="69">
+          <t>Implied share price</t>
+        </is>
+      </c>
+      <c r="B58" s="70">
+        <f>E40</f>
+        <v/>
+      </c>
+      <c r="C58" s="70">
+        <f>E51</f>
+        <v/>
+      </c>
+      <c r="D58" s="70">
         <f>B58-C58</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="16" t="inlineStr">
-        <is>
-          <t>Terminal value variance (%)</t>
-        </is>
-      </c>
-      <c r="B59" s="50" t="inlineStr"/>
-      <c r="C59" s="50" t="inlineStr"/>
-      <c r="D59" s="50">
-        <f>(B57-C57)/B57</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="22" t="inlineStr">
-        <is>
-          <t>Implied share price</t>
-        </is>
-      </c>
-      <c r="B60" s="70">
-        <f>E42</f>
-        <v/>
-      </c>
-      <c r="C60" s="70">
-        <f>E53</f>
-        <v/>
-      </c>
-      <c r="D60" s="70">
-        <f>B60-C60</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="71" t="inlineStr">
+      <c r="A59" s="71" t="inlineStr">
         <is>
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B61" s="72">
-        <f>IF(ABS(D58)&lt;=1.5,"PASS","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="C61" s="73">
-        <f>TEXT(D58,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
-        <v/>
-      </c>
-      <c r="D61" s="39" t="inlineStr">
+      <c r="B59" s="72">
+        <f>IF(ABS(D56)&lt;=1.5,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="C59" s="73">
+        <f>TEXT(D56,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
+        <v/>
+      </c>
+      <c r="D59" s="39" t="inlineStr">
         <is>
           <t>Gordon implied should bracket exit assumption</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="58" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="58" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
       </c>
-      <c r="B64" s="13" t="n"/>
-      <c r="C64" s="13" t="n"/>
-      <c r="D64" s="13" t="n"/>
-      <c r="E64" s="13" t="n"/>
-      <c r="F64" s="13" t="n"/>
-      <c r="G64" s="13" t="n"/>
-      <c r="H64" s="13" t="n"/>
+      <c r="B62" s="13" t="n"/>
+      <c r="C62" s="13" t="n"/>
+      <c r="D62" s="13" t="n"/>
+      <c r="E62" s="13" t="n"/>
+      <c r="F62" s="13" t="n"/>
+      <c r="G62" s="13" t="n"/>
+      <c r="H62" s="13" t="n"/>
+    </row>
+    <row r="63" ht="28" customHeight="1">
+      <c r="A63" s="74" t="inlineStr">
+        <is>
+          <t>WACC \ g</t>
+        </is>
+      </c>
+      <c r="B63" s="17" t="inlineStr">
+        <is>
+          <t>Terminal-g axis 1.5–3.0% brackets 2.25% base; bounded by long-run real GDP and inflation benchmarks.</t>
+        </is>
+      </c>
+      <c r="C63" s="18" t="inlineStr">
+        <is>
+          <t>FRED: Real GDP (GDPC1)</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
+        </is>
+      </c>
+      <c r="F63" s="75" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="G63" s="75" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H63" s="75" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="I63" s="75" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="J63" s="75" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L63" s="61" t="inlineStr">
+        <is>
+          <t>Scenarios: terminal g</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="28" customHeight="1">
+      <c r="A64" s="75" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="C64" s="61" t="inlineStr">
+        <is>
+          <t>Damodaran: Historical Implied ERP</t>
+        </is>
+      </c>
+      <c r="D64" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
+        </is>
+      </c>
+      <c r="F64" s="76">
+        <f>(NPV(0.095,F22:J22)+(J22*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E36+E37)/E39</f>
+        <v/>
+      </c>
+      <c r="G64" s="76">
+        <f>(NPV(0.095,F22:J22)+(J22*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E36+E37)/E39</f>
+        <v/>
+      </c>
+      <c r="H64" s="76">
+        <f>(NPV(0.095,F22:J22)+(J22*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E36+E37)/E39</f>
+        <v/>
+      </c>
+      <c r="I64" s="76">
+        <f>(NPV(0.095,F22:J22)+(J22*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E36+E37)/E39</f>
+        <v/>
+      </c>
+      <c r="J64" s="76">
+        <f>(NPV(0.095,F22:J22)+(J22*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E36+E37)/E39</f>
+        <v/>
+      </c>
+      <c r="L64" s="61" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="28" customHeight="1">
-      <c r="A65" s="74" t="inlineStr">
-        <is>
-          <t>WACC \ g</t>
-        </is>
-      </c>
-      <c r="B65" s="17" t="inlineStr">
-        <is>
-          <t>Terminal-g axis 1.5–3.0% brackets 2.25% base; bounded by long-run real GDP and inflation benchmarks.</t>
-        </is>
-      </c>
-      <c r="C65" s="18" t="inlineStr">
-        <is>
-          <t>FRED: Real GDP (GDPC1)</t>
-        </is>
+      <c r="A65" s="75" t="n">
+        <v>0.1</v>
       </c>
       <c r="D65" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
-        </is>
-      </c>
-      <c r="F65" s="75" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="G65" s="75" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="H65" s="75" t="n">
-        <v>0.0225</v>
-      </c>
-      <c r="I65" s="75" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="J65" s="75" t="n">
-        <v>0.03</v>
+          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
+        </is>
+      </c>
+      <c r="F65" s="76">
+        <f>(NPV(0.1,F22:J22)+(J22*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E36+E37)/E39</f>
+        <v/>
+      </c>
+      <c r="G65" s="76">
+        <f>(NPV(0.1,F22:J22)+(J22*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E36+E37)/E39</f>
+        <v/>
+      </c>
+      <c r="H65" s="76">
+        <f>(NPV(0.1,F22:J22)+(J22*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E36+E37)/E39</f>
+        <v/>
+      </c>
+      <c r="I65" s="76">
+        <f>(NPV(0.1,F22:J22)+(J22*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E36+E37)/E39</f>
+        <v/>
+      </c>
+      <c r="J65" s="76">
+        <f>(NPV(0.1,F22:J22)+(J22*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E36+E37)/E39</f>
+        <v/>
       </c>
       <c r="L65" s="61" t="inlineStr">
         <is>
-          <t>Scenarios: terminal g</t>
+          <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="75" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="C66" s="61" t="inlineStr">
-        <is>
-          <t>Damodaran: Historical Implied ERP</t>
-        </is>
+        <v>0.105</v>
       </c>
       <c r="D66" s="19" t="inlineStr">
         <is>
@@ -4405,23 +4223,23 @@
         </is>
       </c>
       <c r="F66" s="76">
-        <f>(NPV(0.095,F24:J24)+(J24*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E38+E39)/E41</f>
+        <f>(NPV(0.105,F22:J22)+(J22*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="G66" s="76">
-        <f>(NPV(0.095,F24:J24)+(J24*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E38+E39)/E41</f>
-        <v/>
-      </c>
-      <c r="H66" s="76">
-        <f>(NPV(0.095,F24:J24)+(J24*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E38+E39)/E41</f>
+        <f>(NPV(0.105,F22:J22)+(J22*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E36+E37)/E39</f>
+        <v/>
+      </c>
+      <c r="H66" s="77">
+        <f>(NPV(0.105,F22:J22)+(J22*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="I66" s="76">
-        <f>(NPV(0.095,F24:J24)+(J24*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E38+E39)/E41</f>
+        <f>(NPV(0.105,F22:J22)+(J22*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="J66" s="76">
-        <f>(NPV(0.095,F24:J24)+(J24*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E38+E39)/E41</f>
+        <f>(NPV(0.105,F22:J22)+(J22*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="L66" s="61" t="inlineStr">
@@ -4432,7 +4250,7 @@
     </row>
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="75" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="D67" s="19" t="inlineStr">
         <is>
@@ -4440,23 +4258,23 @@
         </is>
       </c>
       <c r="F67" s="76">
-        <f>(NPV(0.1,F24:J24)+(J24*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E38+E39)/E41</f>
+        <f>(NPV(0.11,F22:J22)+(J22*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="G67" s="76">
-        <f>(NPV(0.1,F24:J24)+(J24*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E38+E39)/E41</f>
+        <f>(NPV(0.11,F22:J22)+(J22*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="H67" s="76">
-        <f>(NPV(0.1,F24:J24)+(J24*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E38+E39)/E41</f>
+        <f>(NPV(0.11,F22:J22)+(J22*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="I67" s="76">
-        <f>(NPV(0.1,F24:J24)+(J24*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E38+E39)/E41</f>
+        <f>(NPV(0.11,F22:J22)+(J22*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="J67" s="76">
-        <f>(NPV(0.1,F24:J24)+(J24*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E38+E39)/E41</f>
+        <f>(NPV(0.11,F22:J22)+(J22*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="L67" s="61" t="inlineStr">
@@ -4467,7 +4285,7 @@
     </row>
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="75" t="n">
-        <v>0.105</v>
+        <v>0.115</v>
       </c>
       <c r="D68" s="19" t="inlineStr">
         <is>
@@ -4475,23 +4293,23 @@
         </is>
       </c>
       <c r="F68" s="76">
-        <f>(NPV(0.105,F24:J24)+(J24*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E38+E39)/E41</f>
+        <f>(NPV(0.115,F22:J22)+(J22*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="G68" s="76">
-        <f>(NPV(0.105,F24:J24)+(J24*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E38+E39)/E41</f>
-        <v/>
-      </c>
-      <c r="H68" s="77">
-        <f>(NPV(0.105,F24:J24)+(J24*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E38+E39)/E41</f>
+        <f>(NPV(0.115,F22:J22)+(J22*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E36+E37)/E39</f>
+        <v/>
+      </c>
+      <c r="H68" s="76">
+        <f>(NPV(0.115,F22:J22)+(J22*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="I68" s="76">
-        <f>(NPV(0.105,F24:J24)+(J24*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E38+E39)/E41</f>
+        <f>(NPV(0.115,F22:J22)+(J22*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="J68" s="76">
-        <f>(NPV(0.105,F24:J24)+(J24*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E38+E39)/E41</f>
+        <f>(NPV(0.115,F22:J22)+(J22*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
       <c r="L68" s="61" t="inlineStr">
@@ -4501,97 +4319,27 @@
       </c>
     </row>
     <row r="69" ht="28" customHeight="1">
-      <c r="A69" s="75" t="n">
-        <v>0.11</v>
+      <c r="B69" s="17" t="inlineStr">
+        <is>
+          <t>Red WACC and g grid values bracket base case ±100bps discount rate and ±75bps terminal growth for sensitivity.</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>Scenarios: WACC &amp; terminal g</t>
+        </is>
       </c>
       <c r="D69" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
-        </is>
-      </c>
-      <c r="F69" s="76">
-        <f>(NPV(0.11,F24:J24)+(J24*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E38+E39)/E41</f>
-        <v/>
-      </c>
-      <c r="G69" s="76">
-        <f>(NPV(0.11,F24:J24)+(J24*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E38+E39)/E41</f>
-        <v/>
-      </c>
-      <c r="H69" s="76">
-        <f>(NPV(0.11,F24:J24)+(J24*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E38+E39)/E41</f>
-        <v/>
-      </c>
-      <c r="I69" s="76">
-        <f>(NPV(0.11,F24:J24)+(J24*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E38+E39)/E41</f>
-        <v/>
-      </c>
-      <c r="J69" s="76">
-        <f>(NPV(0.11,F24:J24)+(J24*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E38+E39)/E41</f>
-        <v/>
+          <t>Scenarios tab → Ctrl+F "WACC" and "Terminal growth" rows (base-case inputs)</t>
+        </is>
       </c>
       <c r="L69" s="61" t="inlineStr">
         <is>
-          <t>WACC tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="28" customHeight="1">
-      <c r="A70" s="75" t="n">
-        <v>0.115</v>
-      </c>
-      <c r="D70" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
-        </is>
-      </c>
-      <c r="F70" s="76">
-        <f>(NPV(0.115,F24:J24)+(J24*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E38+E39)/E41</f>
-        <v/>
-      </c>
-      <c r="G70" s="76">
-        <f>(NPV(0.115,F24:J24)+(J24*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E38+E39)/E41</f>
-        <v/>
-      </c>
-      <c r="H70" s="76">
-        <f>(NPV(0.115,F24:J24)+(J24*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E38+E39)/E41</f>
-        <v/>
-      </c>
-      <c r="I70" s="76">
-        <f>(NPV(0.115,F24:J24)+(J24*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E38+E39)/E41</f>
-        <v/>
-      </c>
-      <c r="J70" s="76">
-        <f>(NPV(0.115,F24:J24)+(J24*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E38+E39)/E41</f>
-        <v/>
-      </c>
-      <c r="L70" s="61" t="inlineStr">
-        <is>
-          <t>WACC tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="28" customHeight="1">
-      <c r="B71" s="17" t="inlineStr">
-        <is>
-          <t>Red WACC and g grid values bracket base case ±100bps discount rate and ±75bps terminal growth for sensitivity.</t>
-        </is>
-      </c>
-      <c r="C71" s="18" t="inlineStr">
-        <is>
-          <t>Scenarios: WACC &amp; terminal g</t>
-        </is>
-      </c>
-      <c r="D71" s="19" t="inlineStr">
-        <is>
-          <t>Scenarios tab → Ctrl+F "WACC" and "Terminal growth" rows (base-case inputs)</t>
-        </is>
-      </c>
-      <c r="L71" s="61" t="inlineStr">
-        <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="M71" s="19" t="inlineStr">
+      <c r="M69" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
@@ -4611,29 +4359,29 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId24"/>
-    <hyperlink ref="M49" location="'Comps'!A26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId25"/>
-    <hyperlink ref="L65" location="'Scenarios'!G10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId24"/>
+    <hyperlink ref="M47" location="'Comps'!A26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId25"/>
+    <hyperlink ref="L63" location="'Scenarios'!G10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId26"/>
+    <hyperlink ref="L64" location="'WACC'!E16"/>
+    <hyperlink ref="L65" location="'WACC'!E16"/>
     <hyperlink ref="L66" location="'WACC'!E16"/>
     <hyperlink ref="L67" location="'WACC'!E16"/>
     <hyperlink ref="L68" location="'WACC'!E16"/>
-    <hyperlink ref="L69" location="'WACC'!E16"/>
-    <hyperlink ref="L70" location="'WACC'!E16"/>
-    <hyperlink ref="C71" location="'Scenarios'!G9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId27"/>
+    <hyperlink ref="C69" location="'Scenarios'!G9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4739,7 +4487,7 @@
         </is>
       </c>
       <c r="E6" s="48">
-        <f>DCF!E33</f>
+        <f>DCF!E31</f>
         <v/>
       </c>
     </row>
@@ -5051,7 +4799,7 @@
         </is>
       </c>
       <c r="E25" s="60">
-        <f>DCF!E35</f>
+        <f>DCF!E33</f>
         <v/>
       </c>
     </row>
@@ -5062,7 +4810,7 @@
         </is>
       </c>
       <c r="E26" s="69">
-        <f>DCF!E49</f>
+        <f>DCF!E47</f>
         <v/>
       </c>
     </row>
@@ -5229,7 +4977,7 @@
         </is>
       </c>
       <c r="E38" s="85">
-        <f>DCF!E49</f>
+        <f>DCF!E47</f>
         <v/>
       </c>
       <c r="G38" s="86">
@@ -5293,11 +5041,11 @@
         </is>
       </c>
       <c r="G40" s="84">
-        <f>Scenarios!F75</f>
+        <f>Scenarios!F65</f>
         <v/>
       </c>
       <c r="H40" s="84">
-        <f>Scenarios!H75</f>
+        <f>Scenarios!H65</f>
         <v/>
       </c>
     </row>
@@ -5332,7 +5080,7 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId2"/>
-    <hyperlink ref="C6" location="'DCF'!E33"/>
+    <hyperlink ref="C6" location="'DCF'!E31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
@@ -5348,7 +5096,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId17"/>
-    <hyperlink ref="C38" location="'DCF'!E49"/>
+    <hyperlink ref="C38" location="'DCF'!E47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId20"/>

</xml_diff>

<commit_message>
Show the 0.86 × 1.10 math behind levered beta 0.95
WACC now builds 0.95 from StockAnalysis Beta (5Y) 0.86 plus a 10% overlay after the Sep-4 print, instead of a free-typed 0.95.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -356,7 +356,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -394,11 +394,14 @@
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -1102,10 +1105,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
@@ -1198,12 +1201,12 @@
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>Levered beta</t>
+          <t>Observed Beta (5Y)</t>
         </is>
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>0.95 levered beta vs StockAnalysis Beta (5Y) 0.86; modest uplift for post-guidance volatility.</t>
+          <t>StockAnalysis Beta (5Y) is 0.86. Raw 5-year equity beta; no funded debt so levered ≈ unlevered.</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
@@ -1213,157 +1216,216 @@
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Beta (5Y)" → 0.86. Model uses 0.95.</t>
+          <t>Ctrl+F "Beta (5Y)" → 0.86. This is the raw 5-year beta, not the 0.95 the model uses.</t>
         </is>
       </c>
       <c r="E5" s="21" t="n">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Post-guide vol uplift</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>10% because that 5Y beta is too calm after the Sep-4 −17% print and FY26 guide cut.</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>StockAnalysis: LULU Sep-4 print</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "-17.38%" → Sep 4 close after Sep 3 earnings. Also Ctrl+F "52-Week Price Change" → -49.32%. +10% is the analyst overlay.</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Levered beta = ROUND(5Y × (1+uplift), 2)</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>0.95 = ROUND(0.86 × 1.10, 2). 0.86 × 1.10 = 0.946, which rounds to 0.95. Formula, not a free 0.95.</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>StockAnalysis: LULU Beta (5Y)</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Observed 5Y beta (StockAnalysis)
+  Ctrl+F "Beta (5Y)"  →  0.86
+Why not use 0.86 as-is
+  Ctrl+F "-17.38%"  →  Sep 4 close after Sep 3 earnings
+  Ctrl+F "52-Week Price Change"  →  -49.32%
+  5Y beta is too calm for a name that just printed a guide cut
+Model levered beta
+  0.86 × 1.10 = 0.946
+  0.95 = ROUND(0.86 × 1.10, 2)</t>
+        </is>
+      </c>
+      <c r="E7" s="23">
+        <f>ROUND(E5*(1+E6),2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>Cost of equity = rf + β × ERP</t>
         </is>
       </c>
-      <c r="E6" s="23">
-        <f>E3+E5*E4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="E8" s="24">
+        <f>E3+E7*E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Cost of debt</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Pre-tax cost of debt</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>5.0% illustrative pre-tax debt cost; 10-K: no borrowings outstanding on the revolver.</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K (no funded debt)</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "no borrowings were outstanding under this facility" on this 10-K HTML page (search the document, do not use the EDGAR viewer TOC).</t>
         </is>
       </c>
-      <c r="E9" s="20" t="n">
+      <c r="E11" s="20" t="n">
         <v>0.05</v>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>30% cash tax matches FY2026 guidance (“approximately 30%”); FY25 effective was 29.5%.</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Q2 FY2026 outlook: tax rate ≈ 30%</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "a tax rate of approximately 30%" on the FY2026 outlook paragraph.</t>
         </is>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E12" s="20" t="n">
         <v>0.3</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="E11" s="24">
-        <f>E9*(1-E10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="E13" s="25">
+        <f>E11*(1-E12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Capital structure (market values)</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Equity weight</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>100% equity weight; net-cash balance sheet with no material funded debt at market values per FY2025 10-K.</t>
         </is>
       </c>
-      <c r="C14" s="18" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K balance sheet</t>
         </is>
       </c>
-      <c r="D14" s="19" t="inlineStr">
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) | no funded term debt</t>
         </is>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E16" s="20" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Debt weight</t>
         </is>
       </c>
-      <c r="B15" s="17" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>0% debt weight; no outstanding term loans or bonds, so WACC effectively equals levered cost of equity here.</t>
         </is>
       </c>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K balance sheet</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "no borrowings were outstanding under this facility" → debt weight 0%</t>
         </is>
       </c>
-      <c r="E15" s="20" t="n">
+      <c r="E17" s="20" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="22" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="E16" s="25">
-        <f>E14*E6+E15*E11</f>
+      <c r="E18" s="26">
+        <f>E16*E8+E17*E13</f>
         <v/>
       </c>
     </row>
@@ -1372,10 +1434,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1414,17 +1478,17 @@
       <c r="H1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="F2" s="26" t="inlineStr">
+      <c r="F2" s="27" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="G2" s="27" t="inlineStr">
+      <c r="G2" s="28" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="H2" s="28" t="inlineStr">
+      <c r="H2" s="29" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
@@ -1566,13 +1630,13 @@
           <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
         </is>
       </c>
-      <c r="F7" s="29" t="n">
+      <c r="F7" s="30" t="n">
         <v>134500</v>
       </c>
-      <c r="G7" s="29" t="n">
+      <c r="G7" s="30" t="n">
         <v>134500</v>
       </c>
-      <c r="H7" s="29" t="n">
+      <c r="H7" s="30" t="n">
         <v>134500</v>
       </c>
     </row>
@@ -1743,7 +1807,7 @@
 Also: FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
         </is>
       </c>
-      <c r="C13" s="30" t="inlineStr">
+      <c r="C13" s="31" t="inlineStr">
         <is>
           <t>LULU 10-K: 2026 capex guide $725–745M
 Also: Q2 FY2026 outlook: $10.350B–$10.500B sales</t>
@@ -1845,856 +1909,856 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="31" t="inlineStr">
+      <c r="A18" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 1</t>
         </is>
       </c>
-      <c r="F18" s="32">
+      <c r="F18" s="33">
         <f>11102600*(1+F4)</f>
         <v/>
       </c>
-      <c r="G18" s="32">
+      <c r="G18" s="33">
         <f>11102600*(1+G4)</f>
         <v/>
       </c>
-      <c r="H18" s="32">
+      <c r="H18" s="33">
         <f>11102600*(1+H4)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 2</t>
         </is>
       </c>
-      <c r="F19" s="32">
+      <c r="F19" s="33">
         <f>F18*(1+F5)</f>
         <v/>
       </c>
-      <c r="G19" s="32">
+      <c r="G19" s="33">
         <f>G18*(1+G5)</f>
         <v/>
       </c>
-      <c r="H19" s="32">
+      <c r="H19" s="33">
         <f>H18*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="31" t="inlineStr">
+      <c r="A20" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 3</t>
         </is>
       </c>
-      <c r="F20" s="32">
+      <c r="F20" s="33">
         <f>F19*(1+F5)</f>
         <v/>
       </c>
-      <c r="G20" s="32">
+      <c r="G20" s="33">
         <f>G19*(1+G5)</f>
         <v/>
       </c>
-      <c r="H20" s="32">
+      <c r="H20" s="33">
         <f>H19*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="31" t="inlineStr">
+      <c r="A21" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 4</t>
         </is>
       </c>
-      <c r="F21" s="32">
+      <c r="F21" s="33">
         <f>F20*(1+F5)</f>
         <v/>
       </c>
-      <c r="G21" s="32">
+      <c r="G21" s="33">
         <f>G20*(1+G5)</f>
         <v/>
       </c>
-      <c r="H21" s="32">
+      <c r="H21" s="33">
         <f>H20*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="31" t="inlineStr">
+      <c r="A22" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 5</t>
         </is>
       </c>
-      <c r="F22" s="32">
+      <c r="F22" s="33">
         <f>F21*(1+F5)</f>
         <v/>
       </c>
-      <c r="G22" s="32">
+      <c r="G22" s="33">
         <f>G21*(1+G5)</f>
         <v/>
       </c>
-      <c r="H22" s="32">
+      <c r="H22" s="33">
         <f>H21*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="A23" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 1</t>
         </is>
       </c>
-      <c r="F23" s="33">
+      <c r="F23" s="34">
         <f>F6+(F8-F6)*0/4</f>
         <v/>
       </c>
-      <c r="G23" s="33">
+      <c r="G23" s="34">
         <f>G6+(G8-G6)*0/4</f>
         <v/>
       </c>
-      <c r="H23" s="33">
+      <c r="H23" s="34">
         <f>H6+(H8-H6)*0/4</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 2</t>
         </is>
       </c>
-      <c r="F24" s="33">
+      <c r="F24" s="34">
         <f>F6+(F8-F6)*1/4</f>
         <v/>
       </c>
-      <c r="G24" s="33">
+      <c r="G24" s="34">
         <f>G6+(G8-G6)*1/4</f>
         <v/>
       </c>
-      <c r="H24" s="33">
+      <c r="H24" s="34">
         <f>H6+(H8-H6)*1/4</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="31" t="inlineStr">
+      <c r="A25" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 3</t>
         </is>
       </c>
-      <c r="F25" s="33">
+      <c r="F25" s="34">
         <f>F6+(F8-F6)*2/4</f>
         <v/>
       </c>
-      <c r="G25" s="33">
+      <c r="G25" s="34">
         <f>G6+(G8-G6)*2/4</f>
         <v/>
       </c>
-      <c r="H25" s="33">
+      <c r="H25" s="34">
         <f>H6+(H8-H6)*2/4</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="31" t="inlineStr">
+      <c r="A26" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 4</t>
         </is>
       </c>
-      <c r="F26" s="33">
+      <c r="F26" s="34">
         <f>F6+(F8-F6)*3/4</f>
         <v/>
       </c>
-      <c r="G26" s="33">
+      <c r="G26" s="34">
         <f>G6+(G8-G6)*3/4</f>
         <v/>
       </c>
-      <c r="H26" s="33">
+      <c r="H26" s="34">
         <f>H6+(H8-H6)*3/4</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="31" t="inlineStr">
+      <c r="A27" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 5</t>
         </is>
       </c>
-      <c r="F27" s="33">
+      <c r="F27" s="34">
         <f>F6+(F8-F6)*4/4</f>
         <v/>
       </c>
-      <c r="G27" s="33">
+      <c r="G27" s="34">
         <f>G6+(G8-G6)*4/4</f>
         <v/>
       </c>
-      <c r="H27" s="33">
+      <c r="H27" s="34">
         <f>H6+(H8-H6)*4/4</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="31" t="inlineStr">
+      <c r="A28" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 1</t>
         </is>
       </c>
-      <c r="F28" s="32">
+      <c r="F28" s="33">
         <f>F18*F23+F7</f>
         <v/>
       </c>
-      <c r="G28" s="32">
+      <c r="G28" s="33">
         <f>G18*G23+G7</f>
         <v/>
       </c>
-      <c r="H28" s="32">
+      <c r="H28" s="33">
         <f>H18*H23+H7</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="31" t="inlineStr">
+      <c r="A29" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 2</t>
         </is>
       </c>
-      <c r="F29" s="32">
+      <c r="F29" s="33">
         <f>F19*F24</f>
         <v/>
       </c>
-      <c r="G29" s="32">
+      <c r="G29" s="33">
         <f>G19*G24</f>
         <v/>
       </c>
-      <c r="H29" s="32">
+      <c r="H29" s="33">
         <f>H19*H24</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="31" t="inlineStr">
+      <c r="A30" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 3</t>
         </is>
       </c>
-      <c r="F30" s="32">
+      <c r="F30" s="33">
         <f>F20*F25</f>
         <v/>
       </c>
-      <c r="G30" s="32">
+      <c r="G30" s="33">
         <f>G20*G25</f>
         <v/>
       </c>
-      <c r="H30" s="32">
+      <c r="H30" s="33">
         <f>H20*H25</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="31" t="inlineStr">
+      <c r="A31" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 4</t>
         </is>
       </c>
-      <c r="F31" s="32">
+      <c r="F31" s="33">
         <f>F21*F26</f>
         <v/>
       </c>
-      <c r="G31" s="32">
+      <c r="G31" s="33">
         <f>G21*G26</f>
         <v/>
       </c>
-      <c r="H31" s="32">
+      <c r="H31" s="33">
         <f>H21*H26</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="31" t="inlineStr">
+      <c r="A32" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 5</t>
         </is>
       </c>
-      <c r="F32" s="32">
+      <c r="F32" s="33">
         <f>F22*F27</f>
         <v/>
       </c>
-      <c r="G32" s="32">
+      <c r="G32" s="33">
         <f>G22*G27</f>
         <v/>
       </c>
-      <c r="H32" s="32">
+      <c r="H32" s="33">
         <f>H22*H27</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="31" t="inlineStr">
+      <c r="A33" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 1</t>
         </is>
       </c>
-      <c r="F33" s="32">
+      <c r="F33" s="33">
         <f>F28*(1-F11)</f>
         <v/>
       </c>
-      <c r="G33" s="32">
+      <c r="G33" s="33">
         <f>G28*(1-G11)</f>
         <v/>
       </c>
-      <c r="H33" s="32">
+      <c r="H33" s="33">
         <f>H28*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="31" t="inlineStr">
+      <c r="A34" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 2</t>
         </is>
       </c>
-      <c r="F34" s="32">
+      <c r="F34" s="33">
         <f>F29*(1-F11)</f>
         <v/>
       </c>
-      <c r="G34" s="32">
+      <c r="G34" s="33">
         <f>G29*(1-G11)</f>
         <v/>
       </c>
-      <c r="H34" s="32">
+      <c r="H34" s="33">
         <f>H29*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="31" t="inlineStr">
+      <c r="A35" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 3</t>
         </is>
       </c>
-      <c r="F35" s="32">
+      <c r="F35" s="33">
         <f>F30*(1-F11)</f>
         <v/>
       </c>
-      <c r="G35" s="32">
+      <c r="G35" s="33">
         <f>G30*(1-G11)</f>
         <v/>
       </c>
-      <c r="H35" s="32">
+      <c r="H35" s="33">
         <f>H30*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="31" t="inlineStr">
+      <c r="A36" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 4</t>
         </is>
       </c>
-      <c r="F36" s="32">
+      <c r="F36" s="33">
         <f>F31*(1-F11)</f>
         <v/>
       </c>
-      <c r="G36" s="32">
+      <c r="G36" s="33">
         <f>G31*(1-G11)</f>
         <v/>
       </c>
-      <c r="H36" s="32">
+      <c r="H36" s="33">
         <f>H31*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="31" t="inlineStr">
+      <c r="A37" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 5</t>
         </is>
       </c>
-      <c r="F37" s="32">
+      <c r="F37" s="33">
         <f>F32*(1-F11)</f>
         <v/>
       </c>
-      <c r="G37" s="32">
+      <c r="G37" s="33">
         <f>G32*(1-G11)</f>
         <v/>
       </c>
-      <c r="H37" s="32">
+      <c r="H37" s="33">
         <f>H32*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="31" t="inlineStr">
+      <c r="A38" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 1</t>
         </is>
       </c>
-      <c r="F38" s="32">
+      <c r="F38" s="33">
         <f>F18*F12</f>
         <v/>
       </c>
-      <c r="G38" s="32">
+      <c r="G38" s="33">
         <f>G18*G12</f>
         <v/>
       </c>
-      <c r="H38" s="32">
+      <c r="H38" s="33">
         <f>H18*H12</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="31" t="inlineStr">
+      <c r="A39" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 2</t>
         </is>
       </c>
-      <c r="F39" s="32">
+      <c r="F39" s="33">
         <f>F19*F12</f>
         <v/>
       </c>
-      <c r="G39" s="32">
+      <c r="G39" s="33">
         <f>G19*G12</f>
         <v/>
       </c>
-      <c r="H39" s="32">
+      <c r="H39" s="33">
         <f>H19*H12</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="31" t="inlineStr">
+      <c r="A40" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 3</t>
         </is>
       </c>
-      <c r="F40" s="32">
+      <c r="F40" s="33">
         <f>F20*F12</f>
         <v/>
       </c>
-      <c r="G40" s="32">
+      <c r="G40" s="33">
         <f>G20*G12</f>
         <v/>
       </c>
-      <c r="H40" s="32">
+      <c r="H40" s="33">
         <f>H20*H12</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="31" t="inlineStr">
+      <c r="A41" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 4</t>
         </is>
       </c>
-      <c r="F41" s="32">
+      <c r="F41" s="33">
         <f>F21*F12</f>
         <v/>
       </c>
-      <c r="G41" s="32">
+      <c r="G41" s="33">
         <f>G21*G12</f>
         <v/>
       </c>
-      <c r="H41" s="32">
+      <c r="H41" s="33">
         <f>H21*H12</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="31" t="inlineStr">
+      <c r="A42" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 5</t>
         </is>
       </c>
-      <c r="F42" s="32">
+      <c r="F42" s="33">
         <f>F22*F12</f>
         <v/>
       </c>
-      <c r="G42" s="32">
+      <c r="G42" s="33">
         <f>G22*G12</f>
         <v/>
       </c>
-      <c r="H42" s="32">
+      <c r="H42" s="33">
         <f>H22*H12</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="31" t="inlineStr">
+      <c r="A43" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 1</t>
         </is>
       </c>
-      <c r="F43" s="32">
+      <c r="F43" s="33">
         <f>F18*F13</f>
         <v/>
       </c>
-      <c r="G43" s="32">
+      <c r="G43" s="33">
         <f>G18*G13</f>
         <v/>
       </c>
-      <c r="H43" s="32">
+      <c r="H43" s="33">
         <f>H18*H13</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="31" t="inlineStr">
+      <c r="A44" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 2</t>
         </is>
       </c>
-      <c r="F44" s="32">
+      <c r="F44" s="33">
         <f>F19*F13</f>
         <v/>
       </c>
-      <c r="G44" s="32">
+      <c r="G44" s="33">
         <f>G19*G13</f>
         <v/>
       </c>
-      <c r="H44" s="32">
+      <c r="H44" s="33">
         <f>H19*H13</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="31" t="inlineStr">
+      <c r="A45" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 3</t>
         </is>
       </c>
-      <c r="F45" s="32">
+      <c r="F45" s="33">
         <f>F20*F13</f>
         <v/>
       </c>
-      <c r="G45" s="32">
+      <c r="G45" s="33">
         <f>G20*G13</f>
         <v/>
       </c>
-      <c r="H45" s="32">
+      <c r="H45" s="33">
         <f>H20*H13</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="31" t="inlineStr">
+      <c r="A46" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 4</t>
         </is>
       </c>
-      <c r="F46" s="32">
+      <c r="F46" s="33">
         <f>F21*F13</f>
         <v/>
       </c>
-      <c r="G46" s="32">
+      <c r="G46" s="33">
         <f>G21*G13</f>
         <v/>
       </c>
-      <c r="H46" s="32">
+      <c r="H46" s="33">
         <f>H21*H13</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="31" t="inlineStr">
+      <c r="A47" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 5</t>
         </is>
       </c>
-      <c r="F47" s="32">
+      <c r="F47" s="33">
         <f>F22*F13</f>
         <v/>
       </c>
-      <c r="G47" s="32">
+      <c r="G47" s="33">
         <f>G22*G13</f>
         <v/>
       </c>
-      <c r="H47" s="32">
+      <c r="H47" s="33">
         <f>H22*H13</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="31" t="inlineStr">
+      <c r="A48" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 1</t>
         </is>
       </c>
-      <c r="F48" s="32">
+      <c r="F48" s="33">
         <f>F18*F15</f>
         <v/>
       </c>
-      <c r="G48" s="32">
+      <c r="G48" s="33">
         <f>G18*G15</f>
         <v/>
       </c>
-      <c r="H48" s="32">
+      <c r="H48" s="33">
         <f>H18*H15</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="31" t="inlineStr">
+      <c r="A49" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 2</t>
         </is>
       </c>
-      <c r="F49" s="32">
+      <c r="F49" s="33">
         <f>F19*F15</f>
         <v/>
       </c>
-      <c r="G49" s="32">
+      <c r="G49" s="33">
         <f>G19*G15</f>
         <v/>
       </c>
-      <c r="H49" s="32">
+      <c r="H49" s="33">
         <f>H19*H15</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="31" t="inlineStr">
+      <c r="A50" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 3</t>
         </is>
       </c>
-      <c r="F50" s="32">
+      <c r="F50" s="33">
         <f>F20*F15</f>
         <v/>
       </c>
-      <c r="G50" s="32">
+      <c r="G50" s="33">
         <f>G20*G15</f>
         <v/>
       </c>
-      <c r="H50" s="32">
+      <c r="H50" s="33">
         <f>H20*H15</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="31" t="inlineStr">
+      <c r="A51" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 4</t>
         </is>
       </c>
-      <c r="F51" s="32">
+      <c r="F51" s="33">
         <f>F21*F15</f>
         <v/>
       </c>
-      <c r="G51" s="32">
+      <c r="G51" s="33">
         <f>G21*G15</f>
         <v/>
       </c>
-      <c r="H51" s="32">
+      <c r="H51" s="33">
         <f>H21*H15</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="31" t="inlineStr">
+      <c r="A52" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 5</t>
         </is>
       </c>
-      <c r="F52" s="32">
+      <c r="F52" s="33">
         <f>F22*F15</f>
         <v/>
       </c>
-      <c r="G52" s="32">
+      <c r="G52" s="33">
         <f>G22*G15</f>
         <v/>
       </c>
-      <c r="H52" s="32">
+      <c r="H52" s="33">
         <f>H22*H15</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="31" t="inlineStr">
+      <c r="A53" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 1</t>
         </is>
       </c>
-      <c r="F53" s="32">
+      <c r="F53" s="33">
         <f>F14*(F18-11102600)</f>
         <v/>
       </c>
-      <c r="G53" s="32">
+      <c r="G53" s="33">
         <f>G14*(G18-11102600)</f>
         <v/>
       </c>
-      <c r="H53" s="32">
+      <c r="H53" s="33">
         <f>H14*(H18-11102600)</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="31" t="inlineStr">
+      <c r="A54" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 2</t>
         </is>
       </c>
-      <c r="F54" s="32">
+      <c r="F54" s="33">
         <f>F14*(F19-F18)</f>
         <v/>
       </c>
-      <c r="G54" s="32">
+      <c r="G54" s="33">
         <f>G14*(G19-G18)</f>
         <v/>
       </c>
-      <c r="H54" s="32">
+      <c r="H54" s="33">
         <f>H14*(H19-H18)</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="31" t="inlineStr">
+      <c r="A55" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 3</t>
         </is>
       </c>
-      <c r="F55" s="32">
+      <c r="F55" s="33">
         <f>F14*(F20-F19)</f>
         <v/>
       </c>
-      <c r="G55" s="32">
+      <c r="G55" s="33">
         <f>G14*(G20-G19)</f>
         <v/>
       </c>
-      <c r="H55" s="32">
+      <c r="H55" s="33">
         <f>H14*(H20-H19)</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="31" t="inlineStr">
+      <c r="A56" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 4</t>
         </is>
       </c>
-      <c r="F56" s="32">
+      <c r="F56" s="33">
         <f>F14*(F21-F20)</f>
         <v/>
       </c>
-      <c r="G56" s="32">
+      <c r="G56" s="33">
         <f>G14*(G21-G20)</f>
         <v/>
       </c>
-      <c r="H56" s="32">
+      <c r="H56" s="33">
         <f>H14*(H21-H20)</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="31" t="inlineStr">
+      <c r="A57" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 5</t>
         </is>
       </c>
-      <c r="F57" s="32">
+      <c r="F57" s="33">
         <f>F14*(F22-F21)</f>
         <v/>
       </c>
-      <c r="G57" s="32">
+      <c r="G57" s="33">
         <f>G14*(G22-G21)</f>
         <v/>
       </c>
-      <c r="H57" s="32">
+      <c r="H57" s="33">
         <f>H14*(H22-H21)</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="31" t="inlineStr">
+      <c r="A58" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 1</t>
         </is>
       </c>
-      <c r="F58" s="32">
+      <c r="F58" s="33">
         <f>F33+F38-F43-F53</f>
         <v/>
       </c>
-      <c r="G58" s="32">
+      <c r="G58" s="33">
         <f>G33+G38-G43-G53</f>
         <v/>
       </c>
-      <c r="H58" s="32">
+      <c r="H58" s="33">
         <f>H33+H38-H43-H53</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="31" t="inlineStr">
+      <c r="A59" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 2</t>
         </is>
       </c>
-      <c r="F59" s="32">
+      <c r="F59" s="33">
         <f>F34+F39-F44-F54</f>
         <v/>
       </c>
-      <c r="G59" s="32">
+      <c r="G59" s="33">
         <f>G34+G39-G44-G54</f>
         <v/>
       </c>
-      <c r="H59" s="32">
+      <c r="H59" s="33">
         <f>H34+H39-H44-H54</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="31" t="inlineStr">
+      <c r="A60" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 3</t>
         </is>
       </c>
-      <c r="F60" s="32">
+      <c r="F60" s="33">
         <f>F35+F40-F45-F55</f>
         <v/>
       </c>
-      <c r="G60" s="32">
+      <c r="G60" s="33">
         <f>G35+G40-G45-G55</f>
         <v/>
       </c>
-      <c r="H60" s="32">
+      <c r="H60" s="33">
         <f>H35+H40-H45-H55</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="31" t="inlineStr">
+      <c r="A61" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 4</t>
         </is>
       </c>
-      <c r="F61" s="32">
+      <c r="F61" s="33">
         <f>F36+F41-F46-F56</f>
         <v/>
       </c>
-      <c r="G61" s="32">
+      <c r="G61" s="33">
         <f>G36+G41-G46-G56</f>
         <v/>
       </c>
-      <c r="H61" s="32">
+      <c r="H61" s="33">
         <f>H36+H41-H46-H56</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="31" t="inlineStr">
+      <c r="A62" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 5</t>
         </is>
       </c>
-      <c r="F62" s="32">
+      <c r="F62" s="33">
         <f>F37+F42-F47-F57</f>
         <v/>
       </c>
-      <c r="G62" s="32">
+      <c r="G62" s="33">
         <f>G37+G42-G47-G57</f>
         <v/>
       </c>
-      <c r="H62" s="32">
+      <c r="H62" s="33">
         <f>H37+H42-H47-H57</f>
         <v/>
       </c>
@@ -2705,34 +2769,34 @@
           <t>Enterprise value (DCF)</t>
         </is>
       </c>
-      <c r="F64" s="34">
+      <c r="F64" s="35">
         <f>NPV(F9,F58,F59,F60,F61,F62)+(F62*(1+F10)/(F9-F10))/(1+F9)^5</f>
         <v/>
       </c>
-      <c r="G64" s="34">
+      <c r="G64" s="35">
         <f>NPV(G9,G58,G59,G60,G61,G62)+(G62*(1+G10)/(G9-G10))/(1+G9)^5</f>
         <v/>
       </c>
-      <c r="H64" s="34">
+      <c r="H64" s="35">
         <f>NPV(H9,H58,H59,H60,H61,H62)+(H62*(1+H10)/(H9-H10))/(1+H9)^5</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="35" t="inlineStr">
+      <c r="A65" s="36" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="F65" s="36">
+      <c r="F65" s="37">
         <f>(F64+1807202-0)/111380</f>
         <v/>
       </c>
-      <c r="G65" s="37">
+      <c r="G65" s="38">
         <f>(G64+1807202-0)/111380</f>
         <v/>
       </c>
-      <c r="H65" s="36">
+      <c r="H65" s="37">
         <f>(H64+1807202-0)/111380</f>
         <v/>
       </c>
@@ -2743,21 +2807,21 @@
           <t>Upside / (downside) vs current</t>
         </is>
       </c>
-      <c r="F66" s="38">
+      <c r="F66" s="39">
         <f>F65/100.0-1</f>
         <v/>
       </c>
-      <c r="G66" s="38">
+      <c r="G66" s="39">
         <f>G65/100.0-1</f>
         <v/>
       </c>
-      <c r="H66" s="38">
+      <c r="H66" s="39">
         <f>H65/100.0-1</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="39" t="inlineStr">
+      <c r="A68" s="40" t="inlineStr">
         <is>
           <t>Current price $100.00; cash $1,807,202 k; net debt $0 (net-cash balance sheet).</t>
         </is>
@@ -2770,7 +2834,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
-    <hyperlink ref="C9" location="'WACC'!E16"/>
+    <hyperlink ref="C9" location="'WACC'!E18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
@@ -2823,69 +2887,69 @@
       <c r="J1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="B2" s="40" t="inlineStr">
+      <c r="B2" s="41" t="inlineStr">
         <is>
           <t>Justification (~20 words)</t>
         </is>
       </c>
-      <c r="C2" s="40" t="inlineStr">
+      <c r="C2" s="41" t="inlineStr">
         <is>
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D2" s="40" t="inlineStr">
+      <c r="D2" s="41" t="inlineStr">
         <is>
           <t>Ctrl+F (prove number)</t>
         </is>
       </c>
-      <c r="E2" s="41" t="inlineStr">
+      <c r="E2" s="42" t="inlineStr">
         <is>
           <t>FY2025A</t>
         </is>
       </c>
-      <c r="F2" s="42" t="inlineStr">
+      <c r="F2" s="43" t="inlineStr">
         <is>
           <t>FY2026E</t>
         </is>
       </c>
-      <c r="G2" s="42" t="inlineStr">
+      <c r="G2" s="43" t="inlineStr">
         <is>
           <t>FY2027E</t>
         </is>
       </c>
-      <c r="H2" s="42" t="inlineStr">
+      <c r="H2" s="43" t="inlineStr">
         <is>
           <t>FY2028E</t>
         </is>
       </c>
-      <c r="I2" s="42" t="inlineStr">
+      <c r="I2" s="43" t="inlineStr">
         <is>
           <t>FY2029E</t>
         </is>
       </c>
-      <c r="J2" s="42" t="inlineStr">
+      <c r="J2" s="43" t="inlineStr">
         <is>
           <t>FY2030E</t>
         </is>
       </c>
-      <c r="K2" s="43" t="inlineStr">
+      <c r="K2" s="44" t="inlineStr">
         <is>
           <t>Δ vs Scenarios</t>
         </is>
       </c>
-      <c r="L2" s="40" t="inlineStr">
+      <c r="L2" s="41" t="inlineStr">
         <is>
           <t>Alt. source</t>
         </is>
       </c>
-      <c r="M2" s="40" t="inlineStr">
+      <c r="M2" s="41" t="inlineStr">
         <is>
           <t>Alt. Ctrl+F</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="44" t="inlineStr">
+      <c r="A3" s="45" t="inlineStr">
         <is>
           <t>Forecast drivers linked to Scenarios tab → Base case (column G)</t>
         </is>
@@ -2895,12 +2959,12 @@
           <t>Ctrl+F "Net revenue" → 11,102,600 or "Depreciation and amortization" → 496,228 on this 10-K HTML file</t>
         </is>
       </c>
-      <c r="E3" s="45" t="inlineStr">
+      <c r="E3" s="46" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="K3" s="46" t="inlineStr">
+      <c r="K3" s="47" t="inlineStr">
         <is>
           <t>(should be 0)</t>
         </is>
@@ -2912,30 +2976,30 @@
           <t>Net revenue</t>
         </is>
       </c>
-      <c r="E5" s="47" t="n">
+      <c r="E5" s="48" t="n">
         <v>11102600</v>
       </c>
-      <c r="F5" s="48">
+      <c r="F5" s="49">
         <f>Scenarios!G18</f>
         <v/>
       </c>
-      <c r="G5" s="48">
+      <c r="G5" s="49">
         <f>Scenarios!G19</f>
         <v/>
       </c>
-      <c r="H5" s="48">
+      <c r="H5" s="49">
         <f>Scenarios!G20</f>
         <v/>
       </c>
-      <c r="I5" s="48">
+      <c r="I5" s="49">
         <f>Scenarios!G21</f>
         <v/>
       </c>
-      <c r="J5" s="48">
+      <c r="J5" s="49">
         <f>Scenarios!G22</f>
         <v/>
       </c>
-      <c r="K5" s="49">
+      <c r="K5" s="50">
         <f>IF(MAX(ABS(F5-Scenarios!$G$18),ABS(G5-Scenarios!$G$19),ABS(H5-Scenarios!$G$20),ABS(I5-Scenarios!$G$21),ABS(J5-Scenarios!$G$22))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -2952,7 +3016,7 @@
 Also: 2.3% FY27–30 growth matches StockAnalysis Revenue Growth Forecast (3Y) of 2.26%; next-year consensus is +2.64%.</t>
         </is>
       </c>
-      <c r="C6" s="30" t="inlineStr">
+      <c r="C6" s="31" t="inlineStr">
         <is>
           <t>LULU Q2 FY2026 earnings release
 Also: StockAnalysis: LULU 3Y revenue forecast</t>
@@ -2964,23 +3028,23 @@
 Also: Ctrl+F "Revenue Growth Forecast (3Y)" → 2.26%. That is the unique line (do not search "Net revenue"). Model FY27–30 uses 2.3%.</t>
         </is>
       </c>
-      <c r="F6" s="50">
+      <c r="F6" s="51">
         <f>F5/E5-1</f>
         <v/>
       </c>
-      <c r="G6" s="50">
+      <c r="G6" s="51">
         <f>G5/F5-1</f>
         <v/>
       </c>
-      <c r="H6" s="50">
+      <c r="H6" s="51">
         <f>H5/G5-1</f>
         <v/>
       </c>
-      <c r="I6" s="50">
+      <c r="I6" s="51">
         <f>I5/H5-1</f>
         <v/>
       </c>
-      <c r="J6" s="50">
+      <c r="J6" s="51">
         <f>J5/I5-1</f>
         <v/>
       </c>
@@ -2997,7 +3061,7 @@
 Also: FY30 15.5% is a partial recovery vs the FY25 10-K OM of 19.9% (unique Ctrl+F). Still well below the FY24 23.7% peak.</t>
         </is>
       </c>
-      <c r="C7" s="30" t="inlineStr">
+      <c r="C7" s="31" t="inlineStr">
         <is>
           <t>Q2 FY2026 release: 18.8% OM minus 560bps tariffs
 Also: FY2025 10-K: Operating margin 19.9% (one hit)</t>
@@ -3009,27 +3073,27 @@
 Also: Ctrl+F "19.9%" (one hit) → Operating margin decreased 380 basis points to 19.9%. That is FY25 OM. Do not search the words Income from operations (17 hits). Model FY30 15.5% is a partial-recovery assumption.</t>
         </is>
       </c>
-      <c r="F7" s="50">
+      <c r="F7" s="51">
         <f>Scenarios!G23</f>
         <v/>
       </c>
-      <c r="G7" s="50">
+      <c r="G7" s="51">
         <f>Scenarios!G24</f>
         <v/>
       </c>
-      <c r="H7" s="50">
+      <c r="H7" s="51">
         <f>Scenarios!G25</f>
         <v/>
       </c>
-      <c r="I7" s="50">
+      <c r="I7" s="51">
         <f>Scenarios!G26</f>
         <v/>
       </c>
-      <c r="J7" s="50">
+      <c r="J7" s="51">
         <f>Scenarios!G27</f>
         <v/>
       </c>
-      <c r="K7" s="49">
+      <c r="K7" s="50">
         <f>IF(MAX(ABS(F7-Scenarios!$G$23),ABS(G7-Scenarios!$G$24),ABS(H7-Scenarios!$G$25),ABS(I7-Scenarios!$G$26),ABS(J7-Scenarios!$G$27))&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3055,23 +3119,23 @@
           <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
         </is>
       </c>
-      <c r="E8" s="47" t="n">
+      <c r="E8" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="29">
+      <c r="F8" s="30">
         <f>Scenarios!$G$7</f>
         <v/>
       </c>
-      <c r="G8" s="29" t="n">
+      <c r="G8" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="29" t="n">
+      <c r="H8" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="29" t="n">
+      <c r="I8" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="29" t="n">
+      <c r="J8" s="30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3081,30 +3145,30 @@
           <t>EBIT (incl. FY26 refund)</t>
         </is>
       </c>
-      <c r="E9" s="51" t="n">
+      <c r="E9" s="52" t="n">
         <v>2210615</v>
       </c>
-      <c r="F9" s="34">
+      <c r="F9" s="35">
         <f>Scenarios!G28</f>
         <v/>
       </c>
-      <c r="G9" s="34">
+      <c r="G9" s="35">
         <f>Scenarios!G29</f>
         <v/>
       </c>
-      <c r="H9" s="34">
+      <c r="H9" s="35">
         <f>Scenarios!G30</f>
         <v/>
       </c>
-      <c r="I9" s="34">
+      <c r="I9" s="35">
         <f>Scenarios!G31</f>
         <v/>
       </c>
-      <c r="J9" s="34">
+      <c r="J9" s="35">
         <f>Scenarios!G32</f>
         <v/>
       </c>
-      <c r="K9" s="52">
+      <c r="K9" s="53">
         <f>IF(MAX(ABS(F9-Scenarios!$G$28),ABS(G9-Scenarios!$G$29),ABS(H9-Scenarios!$G$30),ABS(I9-Scenarios!$G$31),ABS(J9-Scenarios!$G$32))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3115,26 +3179,26 @@
           <t>Reported EBIT margin % (incl. FY26 refund)</t>
         </is>
       </c>
-      <c r="E10" s="53" t="n">
+      <c r="E10" s="54" t="n">
         <v>0.1991078666258354</v>
       </c>
-      <c r="F10" s="50">
+      <c r="F10" s="51">
         <f>F9/F5</f>
         <v/>
       </c>
-      <c r="G10" s="50">
+      <c r="G10" s="51">
         <f>G9/G5</f>
         <v/>
       </c>
-      <c r="H10" s="50">
+      <c r="H10" s="51">
         <f>H9/H5</f>
         <v/>
       </c>
-      <c r="I10" s="50">
+      <c r="I10" s="51">
         <f>I9/I5</f>
         <v/>
       </c>
-      <c r="J10" s="50">
+      <c r="J10" s="51">
         <f>J9/J5</f>
         <v/>
       </c>
@@ -3145,23 +3209,23 @@
           <t>Less: cash taxes on EBIT</t>
         </is>
       </c>
-      <c r="F11" s="48">
+      <c r="F11" s="49">
         <f>-Scenarios!G28*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="G11" s="48">
+      <c r="G11" s="49">
         <f>-Scenarios!G29*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="H11" s="48">
+      <c r="H11" s="49">
         <f>-Scenarios!G30*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="I11" s="48">
+      <c r="I11" s="49">
         <f>-Scenarios!G31*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="J11" s="48">
+      <c r="J11" s="49">
         <f>-Scenarios!G32*Scenarios!$G$11</f>
         <v/>
       </c>
@@ -3172,27 +3236,27 @@
           <t>NOPAT</t>
         </is>
       </c>
-      <c r="F12" s="34">
+      <c r="F12" s="35">
         <f>Scenarios!G33</f>
         <v/>
       </c>
-      <c r="G12" s="34">
+      <c r="G12" s="35">
         <f>Scenarios!G34</f>
         <v/>
       </c>
-      <c r="H12" s="34">
+      <c r="H12" s="35">
         <f>Scenarios!G35</f>
         <v/>
       </c>
-      <c r="I12" s="34">
+      <c r="I12" s="35">
         <f>Scenarios!G36</f>
         <v/>
       </c>
-      <c r="J12" s="34">
+      <c r="J12" s="35">
         <f>Scenarios!G37</f>
         <v/>
       </c>
-      <c r="K12" s="52">
+      <c r="K12" s="53">
         <f>IF(MAX(ABS(F12-Scenarios!$G$33),ABS(G12-Scenarios!$G$34),ABS(H12-Scenarios!$G$35),ABS(I12-Scenarios!$G$36),ABS(J12-Scenarios!$G$37))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3245,27 +3309,27 @@
           <t>Plus: depreciation &amp; amortization</t>
         </is>
       </c>
-      <c r="F14" s="48">
+      <c r="F14" s="49">
         <f>Scenarios!G38</f>
         <v/>
       </c>
-      <c r="G14" s="48">
+      <c r="G14" s="49">
         <f>Scenarios!G39</f>
         <v/>
       </c>
-      <c r="H14" s="48">
+      <c r="H14" s="49">
         <f>Scenarios!G40</f>
         <v/>
       </c>
-      <c r="I14" s="48">
+      <c r="I14" s="49">
         <f>Scenarios!G41</f>
         <v/>
       </c>
-      <c r="J14" s="48">
+      <c r="J14" s="49">
         <f>Scenarios!G42</f>
         <v/>
       </c>
-      <c r="K14" s="49">
+      <c r="K14" s="50">
         <f>IF(MAX(ABS(F14-Scenarios!$G$38),ABS(G14-Scenarios!$G$39),ABS(H14-Scenarios!$G$40),ABS(I14-Scenarios!$G$41),ABS(J14-Scenarios!$G$42))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3282,7 +3346,7 @@
 Also: FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
         </is>
       </c>
-      <c r="C15" s="30" t="inlineStr">
+      <c r="C15" s="31" t="inlineStr">
         <is>
           <t>LULU 10-K: 2026 capex guide $725–745M
 Also: Q2 FY2026 outlook: $10.350B–$10.500B sales</t>
@@ -3331,27 +3395,27 @@
           <t>Less: capital expenditures</t>
         </is>
       </c>
-      <c r="F16" s="48">
+      <c r="F16" s="49">
         <f>-Scenarios!G43</f>
         <v/>
       </c>
-      <c r="G16" s="48">
+      <c r="G16" s="49">
         <f>-Scenarios!G44</f>
         <v/>
       </c>
-      <c r="H16" s="48">
+      <c r="H16" s="49">
         <f>-Scenarios!G45</f>
         <v/>
       </c>
-      <c r="I16" s="48">
+      <c r="I16" s="49">
         <f>-Scenarios!G46</f>
         <v/>
       </c>
-      <c r="J16" s="48">
+      <c r="J16" s="49">
         <f>-Scenarios!G47</f>
         <v/>
       </c>
-      <c r="K16" s="49">
+      <c r="K16" s="50">
         <f>IF(MAX(ABS(F16+Scenarios!$G$43),ABS(G16+Scenarios!$G$44),ABS(H16+Scenarios!$G$45),ABS(I16+Scenarios!$G$46),ABS(J16+Scenarios!$G$47))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3461,30 +3525,30 @@
           <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. Lives inside the NWC line below.</t>
         </is>
       </c>
-      <c r="E19" s="47" t="n">
+      <c r="E19" s="48" t="n">
         <v>190657</v>
       </c>
-      <c r="F19" s="48">
+      <c r="F19" s="49">
         <f>Scenarios!G48</f>
         <v/>
       </c>
-      <c r="G19" s="48">
+      <c r="G19" s="49">
         <f>Scenarios!G49</f>
         <v/>
       </c>
-      <c r="H19" s="48">
+      <c r="H19" s="49">
         <f>Scenarios!G50</f>
         <v/>
       </c>
-      <c r="I19" s="48">
+      <c r="I19" s="49">
         <f>Scenarios!G51</f>
         <v/>
       </c>
-      <c r="J19" s="48">
+      <c r="J19" s="49">
         <f>Scenarios!G52</f>
         <v/>
       </c>
-      <c r="K19" s="49">
+      <c r="K19" s="50">
         <f>IF(MAX(ABS(F19-Scenarios!$G$48),ABS(G19-Scenarios!$G$49),ABS(H19-Scenarios!$G$50),ABS(I19-Scenarios!$G$51),ABS(J19-Scenarios!$G$52))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3495,33 +3559,33 @@
           <t>(Increase)/decrease in NWC (includes AR)</t>
         </is>
       </c>
-      <c r="F20" s="48">
+      <c r="F20" s="49">
         <f>-Scenarios!G53</f>
         <v/>
       </c>
-      <c r="G20" s="48">
+      <c r="G20" s="49">
         <f>-Scenarios!G54</f>
         <v/>
       </c>
-      <c r="H20" s="48">
+      <c r="H20" s="49">
         <f>-Scenarios!G55</f>
         <v/>
       </c>
-      <c r="I20" s="48">
+      <c r="I20" s="49">
         <f>-Scenarios!G56</f>
         <v/>
       </c>
-      <c r="J20" s="48">
+      <c r="J20" s="49">
         <f>-Scenarios!G57</f>
         <v/>
       </c>
-      <c r="K20" s="49">
+      <c r="K20" s="50">
         <f>IF(MAX(ABS(F20+Scenarios!$G$53),ABS(G20+Scenarios!$G$54),ABS(H20+Scenarios!$G$55),ABS(I20+Scenarios!$G$56),ABS(J20+Scenarios!$G$57))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="39" t="inlineStr">
+      <c r="A21" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: NWC and AR are one line. 7.5% of Δsales already includes AR; UFCF does not take ΔAR separately.</t>
         </is>
@@ -3533,27 +3597,27 @@
           <t>Unlevered free cash flow</t>
         </is>
       </c>
-      <c r="F22" s="54">
+      <c r="F22" s="55">
         <f>Scenarios!G58</f>
         <v/>
       </c>
-      <c r="G22" s="54">
+      <c r="G22" s="55">
         <f>Scenarios!G59</f>
         <v/>
       </c>
-      <c r="H22" s="54">
+      <c r="H22" s="55">
         <f>Scenarios!G60</f>
         <v/>
       </c>
-      <c r="I22" s="54">
+      <c r="I22" s="55">
         <f>Scenarios!G61</f>
         <v/>
       </c>
-      <c r="J22" s="54">
+      <c r="J22" s="55">
         <f>Scenarios!G62</f>
         <v/>
       </c>
-      <c r="K22" s="52">
+      <c r="K22" s="53">
         <f>IF(MAX(ABS(F22-Scenarios!$G$58),ABS(G22-Scenarios!$G$59),ABS(H22-Scenarios!$G$60),ABS(I22-Scenarios!$G$61),ABS(J22-Scenarios!$G$62))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3564,19 +3628,19 @@
           <t>Discount period (years)</t>
         </is>
       </c>
-      <c r="F23" s="55" t="n">
+      <c r="F23" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="55" t="n">
+      <c r="G23" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="55" t="n">
+      <c r="H23" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="I23" s="55" t="n">
+      <c r="I23" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="J23" s="55" t="n">
+      <c r="J23" s="56" t="n">
         <v>5</v>
       </c>
     </row>
@@ -3586,23 +3650,23 @@
           <t>Discount factor @ WACC</t>
         </is>
       </c>
-      <c r="F24" s="56">
+      <c r="F24" s="57">
         <f>1/(1+Scenarios!$G$9)^F23</f>
         <v/>
       </c>
-      <c r="G24" s="56">
+      <c r="G24" s="57">
         <f>1/(1+Scenarios!$G$9)^G23</f>
         <v/>
       </c>
-      <c r="H24" s="56">
+      <c r="H24" s="57">
         <f>1/(1+Scenarios!$G$9)^H23</f>
         <v/>
       </c>
-      <c r="I24" s="56">
+      <c r="I24" s="57">
         <f>1/(1+Scenarios!$G$9)^I23</f>
         <v/>
       </c>
-      <c r="J24" s="56">
+      <c r="J24" s="57">
         <f>1/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
@@ -3613,23 +3677,23 @@
           <t>PV of unlevered FCF</t>
         </is>
       </c>
-      <c r="F25" s="34">
+      <c r="F25" s="35">
         <f>F22*F24</f>
         <v/>
       </c>
-      <c r="G25" s="34">
+      <c r="G25" s="35">
         <f>G22*G24</f>
         <v/>
       </c>
-      <c r="H25" s="34">
+      <c r="H25" s="35">
         <f>H22*H24</f>
         <v/>
       </c>
-      <c r="I25" s="34">
+      <c r="I25" s="35">
         <f>I22*I24</f>
         <v/>
       </c>
-      <c r="J25" s="34">
+      <c r="J25" s="35">
         <f>J22*J24</f>
         <v/>
       </c>
@@ -3640,13 +3704,13 @@
           <t>Scenarios linkage summary (column K should all read OK)</t>
         </is>
       </c>
-      <c r="K27" s="57">
+      <c r="K27" s="58">
         <f>IF(COUNTIF(K5:K22,"CHECK")=0,"ALL OK","REVIEW")</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="58" t="inlineStr">
+      <c r="A28" s="59" t="inlineStr">
         <is>
           <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
         </is>
@@ -3660,7 +3724,7 @@
           <t>Sum of PV of explicit FCF (FY26–FY30)</t>
         </is>
       </c>
-      <c r="E29" s="59">
+      <c r="E29" s="60">
         <f>SUM(F25:J25)</f>
         <v/>
       </c>
@@ -3686,7 +3750,7 @@
           <t>Ctrl+F "Q2 2026" → 24,269.613 and "Q2 2025" → 23,770.976. YoY = 2.1%. Model terminal g 2.25%.</t>
         </is>
       </c>
-      <c r="E30" s="50">
+      <c r="E30" s="51">
         <f>Scenarios!$G$10</f>
         <v/>
       </c>
@@ -3697,7 +3761,7 @@
           <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="E31" s="34">
+      <c r="E31" s="35">
         <f>J9+J14</f>
         <v/>
       </c>
@@ -3708,7 +3772,7 @@
           <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
         </is>
       </c>
-      <c r="E32" s="48">
+      <c r="E32" s="49">
         <f>J22*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
         <v/>
       </c>
@@ -3719,7 +3783,7 @@
           <t xml:space="preserve">  Implied exit EV/EBITDA (Gordon Growth)</t>
         </is>
       </c>
-      <c r="E33" s="60">
+      <c r="E33" s="61">
         <f>E32/E31</f>
         <v/>
       </c>
@@ -3730,7 +3794,7 @@
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="E34" s="59">
+      <c r="E34" s="60">
         <f>E32/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
@@ -3741,7 +3805,7 @@
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="E35" s="34">
+      <c r="E35" s="35">
         <f>E29+E34</f>
         <v/>
       </c>
@@ -3752,7 +3816,7 @@
           <t>Plus: cash &amp; equivalents (FY2025)</t>
         </is>
       </c>
-      <c r="C36" s="61" t="inlineStr">
+      <c r="C36" s="62" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -3762,7 +3826,7 @@
           <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
         </is>
       </c>
-      <c r="E36" s="47" t="n">
+      <c r="E36" s="48" t="n">
         <v>1807202</v>
       </c>
     </row>
@@ -3772,7 +3836,7 @@
           <t>Less: total debt</t>
         </is>
       </c>
-      <c r="C37" s="61" t="inlineStr">
+      <c r="C37" s="62" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -3782,7 +3846,7 @@
           <t>Ctrl+F "no borrowings were outstanding under this facility" → no funded term debt</t>
         </is>
       </c>
-      <c r="E37" s="47" t="n">
+      <c r="E37" s="48" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3792,7 +3856,7 @@
           <t>Equity value</t>
         </is>
       </c>
-      <c r="E38" s="34">
+      <c r="E38" s="35">
         <f>E35+E36+E37</f>
         <v/>
       </c>
@@ -3803,7 +3867,7 @@
           <t>Diluted shares outstanding (000)</t>
         </is>
       </c>
-      <c r="C39" s="61" t="inlineStr">
+      <c r="C39" s="62" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -3813,7 +3877,7 @@
           <t>Ctrl+F "Diluted weighted-average number of shares outstanding" → 119,068 (000)</t>
         </is>
       </c>
-      <c r="E39" s="47" t="n">
+      <c r="E39" s="48" t="n">
         <v>111380</v>
       </c>
     </row>
@@ -3823,11 +3887,11 @@
           <t>Implied value per share</t>
         </is>
       </c>
-      <c r="E40" s="62">
+      <c r="E40" s="63">
         <f>E38/E39</f>
         <v/>
       </c>
-      <c r="K40" s="52">
+      <c r="K40" s="53">
         <f>IF(ABS(E40-Scenarios!$G$65)&lt;0.05,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3838,7 +3902,7 @@
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C41" s="61" t="inlineStr">
+      <c r="C41" s="62" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -3848,7 +3912,7 @@
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E41" s="63" t="n">
+      <c r="E41" s="64" t="n">
         <v>100</v>
       </c>
     </row>
@@ -3858,7 +3922,7 @@
           <t>Implied upside / (downside)</t>
         </is>
       </c>
-      <c r="E42" s="64">
+      <c r="E42" s="65">
         <f>E40/E41-1</f>
         <v/>
       </c>
@@ -3869,13 +3933,13 @@
           <t xml:space="preserve">  memo: % of EV from terminal value</t>
         </is>
       </c>
-      <c r="E43" s="50">
+      <c r="E43" s="51">
         <f>E34/E35</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="58" t="inlineStr">
+      <c r="A45" s="59" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
@@ -3911,10 +3975,10 @@
           <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x (assumption)</t>
         </is>
       </c>
-      <c r="E47" s="65" t="n">
+      <c r="E47" s="66" t="n">
         <v>8</v>
       </c>
-      <c r="M47" s="61" t="inlineStr">
+      <c r="M47" s="62" t="inlineStr">
         <is>
           <t>Comps: Exit Multiple Build</t>
         </is>
@@ -3926,7 +3990,7 @@
           <t>Terminal value = Terminal EBITDA × exit multiple</t>
         </is>
       </c>
-      <c r="E48" s="48">
+      <c r="E48" s="49">
         <f>E31*E47</f>
         <v/>
       </c>
@@ -3937,7 +4001,7 @@
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="E49" s="48">
+      <c r="E49" s="49">
         <f>E48/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
@@ -3948,7 +4012,7 @@
           <t>Enterprise value (exit method)</t>
         </is>
       </c>
-      <c r="E50" s="34">
+      <c r="E50" s="35">
         <f>E29+E49</f>
         <v/>
       </c>
@@ -3959,13 +4023,13 @@
           <t>Implied value per share (exit method)</t>
         </is>
       </c>
-      <c r="E51" s="66">
+      <c r="E51" s="67">
         <f>(E50+E36+E37)/E39</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="58" t="inlineStr">
+      <c r="A53" s="59" t="inlineStr">
         <is>
           <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
         </is>
@@ -3975,18 +4039,18 @@
       <c r="D53" s="13" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="67" t="inlineStr"/>
-      <c r="B54" s="68" t="inlineStr">
+      <c r="A54" s="68" t="inlineStr"/>
+      <c r="B54" s="69" t="inlineStr">
         <is>
           <t>Gordon Growth</t>
         </is>
       </c>
-      <c r="C54" s="68" t="inlineStr">
+      <c r="C54" s="69" t="inlineStr">
         <is>
           <t>Exit Multiple</t>
         </is>
       </c>
-      <c r="D54" s="68" t="inlineStr">
+      <c r="D54" s="69" t="inlineStr">
         <is>
           <t>Variance</t>
         </is>
@@ -3998,15 +4062,15 @@
           <t>Terminal value ($)</t>
         </is>
       </c>
-      <c r="B55" s="59">
+      <c r="B55" s="60">
         <f>E32</f>
         <v/>
       </c>
-      <c r="C55" s="59">
+      <c r="C55" s="60">
         <f>E48</f>
         <v/>
       </c>
-      <c r="D55" s="59">
+      <c r="D55" s="60">
         <f>B55-C55</f>
         <v/>
       </c>
@@ -4017,15 +4081,15 @@
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
       </c>
-      <c r="B56" s="69">
+      <c r="B56" s="70">
         <f>E33</f>
         <v/>
       </c>
-      <c r="C56" s="69">
+      <c r="C56" s="70">
         <f>E47</f>
         <v/>
       </c>
-      <c r="D56" s="69">
+      <c r="D56" s="70">
         <f>B56-C56</f>
         <v/>
       </c>
@@ -4036,9 +4100,9 @@
           <t>Terminal value variance (%)</t>
         </is>
       </c>
-      <c r="B57" s="50" t="inlineStr"/>
-      <c r="C57" s="50" t="inlineStr"/>
-      <c r="D57" s="50">
+      <c r="B57" s="51" t="inlineStr"/>
+      <c r="C57" s="51" t="inlineStr"/>
+      <c r="D57" s="51">
         <f>(B55-C55)/B55</f>
         <v/>
       </c>
@@ -4049,41 +4113,41 @@
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="B58" s="70">
+      <c r="B58" s="71">
         <f>E40</f>
         <v/>
       </c>
-      <c r="C58" s="70">
+      <c r="C58" s="71">
         <f>E51</f>
         <v/>
       </c>
-      <c r="D58" s="70">
+      <c r="D58" s="71">
         <f>B58-C58</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="71" t="inlineStr">
+      <c r="A59" s="72" t="inlineStr">
         <is>
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B59" s="72">
+      <c r="B59" s="73">
         <f>IF(ABS(D56)&lt;=1.5,"PASS","REVIEW")</f>
         <v/>
       </c>
-      <c r="C59" s="73">
+      <c r="C59" s="74">
         <f>TEXT(D56,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
         <v/>
       </c>
-      <c r="D59" s="39" t="inlineStr">
+      <c r="D59" s="40" t="inlineStr">
         <is>
           <t>Gordon implied should bracket exit assumption</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="58" t="inlineStr">
+      <c r="A62" s="59" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
@@ -4097,7 +4161,7 @@
       <c r="H62" s="13" t="n"/>
     </row>
     <row r="63" ht="28" customHeight="1">
-      <c r="A63" s="74" t="inlineStr">
+      <c r="A63" s="75" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
@@ -4117,32 +4181,32 @@
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
       </c>
-      <c r="F63" s="75" t="n">
+      <c r="F63" s="76" t="n">
         <v>0.015</v>
       </c>
-      <c r="G63" s="75" t="n">
+      <c r="G63" s="76" t="n">
         <v>0.02</v>
       </c>
-      <c r="H63" s="75" t="n">
+      <c r="H63" s="76" t="n">
         <v>0.0225</v>
       </c>
-      <c r="I63" s="75" t="n">
+      <c r="I63" s="76" t="n">
         <v>0.025</v>
       </c>
-      <c r="J63" s="75" t="n">
+      <c r="J63" s="76" t="n">
         <v>0.03</v>
       </c>
-      <c r="L63" s="61" t="inlineStr">
+      <c r="L63" s="62" t="inlineStr">
         <is>
           <t>Scenarios: terminal g</t>
         </is>
       </c>
     </row>
     <row r="64" ht="28" customHeight="1">
-      <c r="A64" s="75" t="n">
+      <c r="A64" s="76" t="n">
         <v>0.095</v>
       </c>
-      <c r="C64" s="61" t="inlineStr">
+      <c r="C64" s="62" t="inlineStr">
         <is>
           <t>Damodaran: Historical Implied ERP</t>
         </is>
@@ -4152,34 +4216,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F64" s="76">
+      <c r="F64" s="77">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="G64" s="76">
+      <c r="G64" s="77">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="H64" s="76">
+      <c r="H64" s="77">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="I64" s="76">
+      <c r="I64" s="77">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="J64" s="76">
+      <c r="J64" s="77">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="L64" s="61" t="inlineStr">
+      <c r="L64" s="62" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="65" ht="28" customHeight="1">
-      <c r="A65" s="75" t="n">
+      <c r="A65" s="76" t="n">
         <v>0.1</v>
       </c>
       <c r="D65" s="19" t="inlineStr">
@@ -4187,34 +4251,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F65" s="76">
+      <c r="F65" s="77">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="G65" s="76">
+      <c r="G65" s="77">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="H65" s="76">
+      <c r="H65" s="77">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="I65" s="76">
+      <c r="I65" s="77">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="J65" s="76">
+      <c r="J65" s="77">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="L65" s="61" t="inlineStr">
+      <c r="L65" s="62" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="66" ht="28" customHeight="1">
-      <c r="A66" s="75" t="n">
+      <c r="A66" s="76" t="n">
         <v>0.105</v>
       </c>
       <c r="D66" s="19" t="inlineStr">
@@ -4222,34 +4286,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F66" s="76">
+      <c r="F66" s="77">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="G66" s="76">
+      <c r="G66" s="77">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="H66" s="77">
+      <c r="H66" s="78">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="I66" s="76">
+      <c r="I66" s="77">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="J66" s="76">
+      <c r="J66" s="77">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="L66" s="61" t="inlineStr">
+      <c r="L66" s="62" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="67" ht="28" customHeight="1">
-      <c r="A67" s="75" t="n">
+      <c r="A67" s="76" t="n">
         <v>0.11</v>
       </c>
       <c r="D67" s="19" t="inlineStr">
@@ -4257,34 +4321,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F67" s="76">
+      <c r="F67" s="77">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="G67" s="76">
+      <c r="G67" s="77">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="H67" s="76">
+      <c r="H67" s="77">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="I67" s="76">
+      <c r="I67" s="77">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="J67" s="76">
+      <c r="J67" s="77">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="L67" s="61" t="inlineStr">
+      <c r="L67" s="62" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="68" ht="28" customHeight="1">
-      <c r="A68" s="75" t="n">
+      <c r="A68" s="76" t="n">
         <v>0.115</v>
       </c>
       <c r="D68" s="19" t="inlineStr">
@@ -4292,27 +4356,27 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F68" s="76">
+      <c r="F68" s="77">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="G68" s="76">
+      <c r="G68" s="77">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="H68" s="76">
+      <c r="H68" s="77">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="I68" s="76">
+      <c r="I68" s="77">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="J68" s="76">
+      <c r="J68" s="77">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="L68" s="61" t="inlineStr">
+      <c r="L68" s="62" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
@@ -4334,7 +4398,7 @@
           <t>Scenarios tab → Ctrl+F "WACC" and "Terminal growth" rows (base-case inputs)</t>
         </is>
       </c>
-      <c r="L69" s="61" t="inlineStr">
+      <c r="L69" s="62" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
@@ -4375,11 +4439,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId25"/>
     <hyperlink ref="L63" location="'Scenarios'!G10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId26"/>
-    <hyperlink ref="L64" location="'WACC'!E16"/>
-    <hyperlink ref="L65" location="'WACC'!E16"/>
-    <hyperlink ref="L66" location="'WACC'!E16"/>
-    <hyperlink ref="L67" location="'WACC'!E16"/>
-    <hyperlink ref="L68" location="'WACC'!E16"/>
+    <hyperlink ref="L64" location="'WACC'!E18"/>
+    <hyperlink ref="L65" location="'WACC'!E18"/>
+    <hyperlink ref="L66" location="'WACC'!E18"/>
+    <hyperlink ref="L67" location="'WACC'!E18"/>
+    <hyperlink ref="L68" location="'WACC'!E18"/>
     <hyperlink ref="C69" location="'Scenarios'!G9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId27"/>
   </hyperlinks>
@@ -4450,7 +4514,7 @@
           <t>FY2025A revenue</t>
         </is>
       </c>
-      <c r="C4" s="61" t="inlineStr">
+      <c r="C4" s="62" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -4460,7 +4524,7 @@
           <t>Ctrl+F "Net revenue" → 11,102,600 ($000) in FY2025 column</t>
         </is>
       </c>
-      <c r="E4" s="47" t="n">
+      <c r="E4" s="48" t="n">
         <v>11102600</v>
       </c>
     </row>
@@ -4470,7 +4534,7 @@
           <t>FY2025A EBITDA (EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="E5" s="48">
+      <c r="E5" s="49">
         <f>2210615+496228</f>
         <v/>
       </c>
@@ -4481,12 +4545,12 @@
           <t>FY2030E terminal EBITDA (DCF EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="C6" s="61" t="inlineStr">
+      <c r="C6" s="62" t="inlineStr">
         <is>
           <t>↳ DCF base case</t>
         </is>
       </c>
-      <c r="E6" s="48">
+      <c r="E6" s="49">
         <f>DCF!E31</f>
         <v/>
       </c>
@@ -4497,7 +4561,7 @@
           <t>FY2026E diluted EPS (guidance midpoint)</t>
         </is>
       </c>
-      <c r="C7" s="61" t="inlineStr">
+      <c r="C7" s="62" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
@@ -4507,7 +4571,7 @@
           <t>Ctrl+F "$9.48 to $9.73" → FY2026 diluted EPS guidance; model midpoint $9.61</t>
         </is>
       </c>
-      <c r="E7" s="63" t="n">
+      <c r="E7" s="64" t="n">
         <v>9.609999999999999</v>
       </c>
     </row>
@@ -4517,7 +4581,7 @@
           <t>Cash &amp; equivalents</t>
         </is>
       </c>
-      <c r="C8" s="61" t="inlineStr">
+      <c r="C8" s="62" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -4527,7 +4591,7 @@
           <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
         </is>
       </c>
-      <c r="E8" s="47" t="n">
+      <c r="E8" s="48" t="n">
         <v>1807202</v>
       </c>
     </row>
@@ -4537,7 +4601,7 @@
           <t>Diluted shares (000)</t>
         </is>
       </c>
-      <c r="C9" s="61" t="inlineStr">
+      <c r="C9" s="62" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -4547,7 +4611,7 @@
           <t>Ctrl+F "Diluted weighted-average number of shares outstanding" → 119,068 (000)</t>
         </is>
       </c>
-      <c r="E9" s="47" t="n">
+      <c r="E9" s="48" t="n">
         <v>111380</v>
       </c>
     </row>
@@ -4557,7 +4621,7 @@
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C10" s="61" t="inlineStr">
+      <c r="C10" s="62" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -4567,28 +4631,28 @@
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E10" s="63" t="n">
+      <c r="E10" s="64" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="73" t="inlineStr">
+      <c r="A11" s="74" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current EV / EBITDA</t>
         </is>
       </c>
-      <c r="E11" s="78">
+      <c r="E11" s="79">
         <f>(E10*E9-E8)/E5</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="73" t="inlineStr">
+      <c r="A12" s="74" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current P / E (FY2026E)</t>
         </is>
       </c>
-      <c r="E12" s="78">
+      <c r="E12" s="79">
         <f>E10/E7</f>
         <v/>
       </c>
@@ -4601,34 +4665,34 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="73" t="inlineStr">
+      <c r="A15" s="74" t="inlineStr">
         <is>
           <t>Peer / reference EV/EBITDA (forward / illustrative)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="79" t="inlineStr">
+      <c r="A16" s="80" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B16" s="79" t="inlineStr">
+      <c r="B16" s="80" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C16" s="79" t="inlineStr">
+      <c r="C16" s="80" t="inlineStr">
         <is>
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D16" s="79" t="inlineStr">
+      <c r="D16" s="80" t="inlineStr">
         <is>
           <t>Ctrl+F (prove number)</t>
         </is>
       </c>
-      <c r="E16" s="80" t="inlineStr">
+      <c r="E16" s="81" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
@@ -4640,12 +4704,12 @@
           <t>lululemon (LULU) — current</t>
         </is>
       </c>
-      <c r="B17" s="39" t="inlineStr">
+      <c r="B17" s="40" t="inlineStr">
         <is>
           <t>Distressed trough multiple on FY2025A EBITDA</t>
         </is>
       </c>
-      <c r="C17" s="61" t="inlineStr">
+      <c r="C17" s="62" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K</t>
         </is>
@@ -4655,7 +4719,7 @@
           <t>Ctrl+F "19.9%" → FY25 OM (EBIT $2,210,615). Ctrl+F "496,228" → Depreciation and amortization. Do not search the words Income from operations (17 hits).</t>
         </is>
       </c>
-      <c r="E17" s="81">
+      <c r="E17" s="82">
         <f>(E10*E9-E8)/E5</f>
         <v/>
       </c>
@@ -4681,7 +4745,7 @@
           <t>Ctrl+F "EV / EBITDA" → 11.97. Model uses 12.0x.</t>
         </is>
       </c>
-      <c r="E18" s="82" t="n">
+      <c r="E18" s="83" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4706,7 +4770,7 @@
           <t>Ctrl+F "EV / EBITDA" → 7.95. Model uses 8.0x.</t>
         </is>
       </c>
-      <c r="E19" s="82" t="n">
+      <c r="E19" s="83" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4731,7 +4795,7 @@
           <t>Ctrl+F "EV / EBITDA" → 14.03. Model uses 14.0x.</t>
         </is>
       </c>
-      <c r="E20" s="82" t="n">
+      <c r="E20" s="83" t="n">
         <v>14</v>
       </c>
     </row>
@@ -4756,7 +4820,7 @@
           <t>Ctrl+F "EV / EBITDA" → 9.31. Model uses 9.3x.</t>
         </is>
       </c>
-      <c r="E21" s="82" t="n">
+      <c r="E21" s="83" t="n">
         <v>9.300000000000001</v>
       </c>
     </row>
@@ -4781,7 +4845,7 @@
           <t>Ctrl+F "EV / EBITDA" → 10.71. Model uses 10.7x.</t>
         </is>
       </c>
-      <c r="E22" s="82" t="n">
+      <c r="E22" s="83" t="n">
         <v>10.7</v>
       </c>
     </row>
@@ -4798,18 +4862,18 @@
           <t>Gordon Growth implied exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="E25" s="60">
+      <c r="E25" s="61">
         <f>DCF!E33</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="71" t="inlineStr">
+      <c r="A26" s="72" t="inlineStr">
         <is>
           <t>Selected exit multiple (base case)</t>
         </is>
       </c>
-      <c r="E26" s="69">
+      <c r="E26" s="70">
         <f>DCF!E47</f>
         <v/>
       </c>
@@ -4820,48 +4884,48 @@
           <t>Spread (selected − Gordon implied)</t>
         </is>
       </c>
-      <c r="E27" s="60">
+      <c r="E27" s="61">
         <f>E26-E25</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="71" t="inlineStr">
+      <c r="A28" s="72" t="inlineStr">
         <is>
           <t>Rationale for 8.0x</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="31" t="inlineStr">
+      <c r="A29" s="32" t="inlineStr">
         <is>
           <t>•  Mid-point of terminal football field (6.5–9.5x on FY2030E EBITDA) — 8.0x sits between bear and bull exit</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="31" t="inlineStr">
+      <c r="A30" s="32" t="inlineStr">
         <is>
           <t>•  Above Gordon-implied exit (~7x) — ~1 turn buffer vs perpetuity math on terminal FCF</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="31" t="inlineStr">
+      <c r="A31" s="32" t="inlineStr">
         <is>
           <t>•  Below premium-growth peers (ONON ~25x, DECK ~15x) — reflects Americas maturity at terminal</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="31" t="inlineStr">
+      <c r="A32" s="32" t="inlineStr">
         <is>
           <t>•  Above current LULU (~3.5x on FY2025A) — assumes partial recovery, not full re-rating to historical peaks</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="31" t="inlineStr">
+      <c r="A33" s="32" t="inlineStr">
         <is>
           <t>•  Peer simple avg ~16x not used — terminal multiple discounted for lower terminal growth vs ONON/NKE</t>
         </is>
@@ -4875,42 +4939,42 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="79" t="inlineStr">
+      <c r="A36" s="80" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B36" s="79" t="inlineStr">
+      <c r="B36" s="80" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C36" s="79" t="inlineStr">
+      <c r="C36" s="80" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D36" s="79" t="inlineStr">
+      <c r="D36" s="80" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
-      <c r="E36" s="80" t="inlineStr">
+      <c r="E36" s="81" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="F36" s="80" t="inlineStr">
+      <c r="F36" s="81" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="G36" s="80" t="inlineStr">
+      <c r="G36" s="81" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="H36" s="80" t="inlineStr">
+      <c r="H36" s="81" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
@@ -4928,7 +4992,7 @@
 Hi: 9.5x on FY2030E terminal EBITDA; bull exit above 8.0x DCF base; still below peer median ~15x.</t>
         </is>
       </c>
-      <c r="C37" s="83" t="inlineStr">
+      <c r="C37" s="84" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU EV/EBITDA
 Hi: StockAnalysis: LULU valuation</t>
@@ -4940,23 +5004,23 @@
 Hi: Ctrl+F "EV / EBITDA" → bull terminal exit assumption 9.5x on FY2030E EBITDA</t>
         </is>
       </c>
-      <c r="E37" s="82" t="n">
+      <c r="E37" s="83" t="n">
         <v>6.5</v>
       </c>
-      <c r="F37" s="82" t="n">
+      <c r="F37" s="83" t="n">
         <v>9.5</v>
       </c>
-      <c r="G37" s="84">
+      <c r="G37" s="85">
         <f>(E6*E37+E8)/E9</f>
         <v/>
       </c>
-      <c r="H37" s="84">
+      <c r="H37" s="85">
         <f>(E6*F37+E8)/E9</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="71" t="inlineStr">
+      <c r="A38" s="72" t="inlineStr">
         <is>
           <t>DCF exit method (8.0x on FY2030E EBITDA)</t>
         </is>
@@ -4976,11 +5040,11 @@
           <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x (assumption)</t>
         </is>
       </c>
-      <c r="E38" s="85">
+      <c r="E38" s="86">
         <f>DCF!E47</f>
         <v/>
       </c>
-      <c r="G38" s="86">
+      <c r="G38" s="87">
         <f>(E6*E38+E8)/E9</f>
         <v/>
       </c>
@@ -4997,7 +5061,7 @@
 Hi: 18x P/E high on FY2026E EPS; modest recovery case still below historical premium LULU multiples.</t>
         </is>
       </c>
-      <c r="C39" s="83" t="inlineStr">
+      <c r="C39" s="84" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU Forward P/E
 Hi: StockAnalysis: NKE Forward P/E</t>
@@ -5009,17 +5073,17 @@
 Hi: Ctrl+F "Forward PE" → NKE peer benchmark; high-case assumption 18.0x</t>
         </is>
       </c>
-      <c r="E39" s="82" t="n">
+      <c r="E39" s="83" t="n">
         <v>10</v>
       </c>
-      <c r="F39" s="82" t="n">
+      <c r="F39" s="83" t="n">
         <v>18</v>
       </c>
-      <c r="G39" s="84">
+      <c r="G39" s="85">
         <f>E7*E39</f>
         <v/>
       </c>
-      <c r="H39" s="84">
+      <c r="H39" s="85">
         <f>E7*F39</f>
         <v/>
       </c>
@@ -5030,32 +5094,32 @@
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="E40" s="87" t="inlineStr">
+      <c r="E40" s="88" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F40" s="87" t="inlineStr">
+      <c r="F40" s="88" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G40" s="84">
+      <c r="G40" s="85">
         <f>Scenarios!F65</f>
         <v/>
       </c>
-      <c r="H40" s="84">
+      <c r="H40" s="85">
         <f>Scenarios!H65</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="88" t="inlineStr">
+      <c r="A42" s="89" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C42" s="61" t="inlineStr">
+      <c r="C42" s="62" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -5065,12 +5129,12 @@
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E42" s="89" t="n">
+      <c r="E42" s="90" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="39" t="inlineStr">
+      <c r="A43" s="40" t="inlineStr">
         <is>
           <t>Note: peer set includes NKE, DECK, ONON, adidas, VFC; multiples are analyst ranges (red).</t>
         </is>

</xml_diff>

<commit_message>
Source levered beta 0.95 from Damodaran, not a 10% overlay
The +10% markup had no source. 0.95 is now Damodaran Jan-2026 Retail (Special Lines) unlevered beta; company 5Y 0.86 is shown and not used.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -356,7 +356,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -395,6 +395,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1201,12 +1204,12 @@
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>Observed Beta (5Y)</t>
+          <t>Observed Beta (5Y) — not used in WACC</t>
         </is>
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>StockAnalysis Beta (5Y) is 0.86. Raw 5-year equity beta; no funded debt so levered ≈ unlevered.</t>
+          <t>StockAnalysis Beta (5Y) is 0.86. Company 5Y print; too calm after the guide cut, so not the WACC input.</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
@@ -1216,7 +1219,7 @@
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Beta (5Y)" → 0.86. This is the raw 5-year beta, not the 0.95 the model uses.</t>
+          <t>Ctrl+F "Beta (5Y)" → 0.86. Company 5Y beta. Not the WACC input.</t>
         </is>
       </c>
       <c r="E5" s="21" t="n">
@@ -1226,69 +1229,66 @@
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Post-guide vol uplift</t>
+          <t>Damodaran Retail (Special Lines) βu</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>10% because that 5Y beta is too calm after the Sep-4 −17% print and FY26 guide cut.</t>
+          <t>Damodaran Jan-2026 Retail (Special Lines) unlevered beta is 0.95. No funded debt, so that is our levered beta.</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>StockAnalysis: LULU Sep-4 print</t>
+          <t>Damodaran: US betas by sector (Jan 2026)</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "-17.38%" → Sep 4 close after Sep 3 earnings. Also Ctrl+F "52-Week Price Change" → -49.32%. +10% is the analyst overlay.</t>
-        </is>
-      </c>
-      <c r="E6" s="20" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="7" ht="150" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
-        <is>
-          <t>Levered beta = ROUND(5Y × (1+uplift), 2)</t>
+          <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95 (column after Effective Tax rate). Do not take the levered Beta column (1.09). Date of Analysis is January 2026.</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="7" ht="112" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>Levered beta (industry βu; no funded debt)</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>0.95 = ROUND(0.86 × 1.10, 2). 0.86 × 1.10 = 0.946, which rounds to 0.95. Formula, not a free 0.95.</t>
+          <t>0.95 is Damodaran’s industry unlevered beta, not 0.86 times a 10% overlay. Links to the industry row above.</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>StockAnalysis: LULU Beta (5Y)</t>
+          <t>Damodaran: Retail (Special Lines) βu</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Observed 5Y beta (StockAnalysis)
+          <t>Company 5Y (StockAnalysis) — not the WACC input
   Ctrl+F "Beta (5Y)"  →  0.86
-Why not use 0.86 as-is
-  Ctrl+F "-17.38%"  →  Sep 4 close after Sep 3 earnings
-  Ctrl+F "52-Week Price Change"  →  -49.32%
-  5Y beta is too calm for a name that just printed a guide cut
-Model levered beta
-  0.86 × 1.10 = 0.946
-  0.95 = ROUND(0.86 × 1.10, 2)</t>
-        </is>
-      </c>
-      <c r="E7" s="23">
-        <f>ROUND(E5*(1+E6),2)</f>
+Industry bottom-up (Damodaran, Jan 2026) — this is the 0.95
+  Ctrl+F "Retail (Special Lines)"  →  Unlevered beta 0.95
+  Do not take the levered Beta column (1.09)
+  LULU has no funded debt, so unlevered = levered</t>
+        </is>
+      </c>
+      <c r="E7" s="24">
+        <f>E6</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>Cost of equity = rf + β × ERP</t>
         </is>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="25">
         <f>E3+E7*E4</f>
         <v/>
       </c>
@@ -1356,7 +1356,7 @@
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="26">
         <f>E11*(1-E12)</f>
         <v/>
       </c>
@@ -1419,12 +1419,12 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="E18" s="26">
+      <c r="E18" s="27">
         <f>E16*E8+E17*E13</f>
         <v/>
       </c>
@@ -1478,17 +1478,17 @@
       <c r="H1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="F2" s="27" t="inlineStr">
+      <c r="F2" s="28" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="G2" s="28" t="inlineStr">
+      <c r="G2" s="29" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="H2" s="29" t="inlineStr">
+      <c r="H2" s="30" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
@@ -1630,13 +1630,13 @@
           <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
         </is>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="F7" s="31" t="n">
         <v>134500</v>
       </c>
-      <c r="G7" s="30" t="n">
+      <c r="G7" s="31" t="n">
         <v>134500</v>
       </c>
-      <c r="H7" s="30" t="n">
+      <c r="H7" s="31" t="n">
         <v>134500</v>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
 Also: FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
         </is>
       </c>
-      <c r="C13" s="31" t="inlineStr">
+      <c r="C13" s="32" t="inlineStr">
         <is>
           <t>LULU 10-K: 2026 capex guide $725–745M
 Also: Q2 FY2026 outlook: $10.350B–$10.500B sales</t>
@@ -1909,919 +1909,919 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 1</t>
         </is>
       </c>
-      <c r="F18" s="33">
+      <c r="F18" s="34">
         <f>11102600*(1+F4)</f>
         <v/>
       </c>
-      <c r="G18" s="33">
+      <c r="G18" s="34">
         <f>11102600*(1+G4)</f>
         <v/>
       </c>
-      <c r="H18" s="33">
+      <c r="H18" s="34">
         <f>11102600*(1+H4)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="32" t="inlineStr">
+      <c r="A19" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 2</t>
         </is>
       </c>
-      <c r="F19" s="33">
+      <c r="F19" s="34">
         <f>F18*(1+F5)</f>
         <v/>
       </c>
-      <c r="G19" s="33">
+      <c r="G19" s="34">
         <f>G18*(1+G5)</f>
         <v/>
       </c>
-      <c r="H19" s="33">
+      <c r="H19" s="34">
         <f>H18*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 3</t>
         </is>
       </c>
-      <c r="F20" s="33">
+      <c r="F20" s="34">
         <f>F19*(1+F5)</f>
         <v/>
       </c>
-      <c r="G20" s="33">
+      <c r="G20" s="34">
         <f>G19*(1+G5)</f>
         <v/>
       </c>
-      <c r="H20" s="33">
+      <c r="H20" s="34">
         <f>H19*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 4</t>
         </is>
       </c>
-      <c r="F21" s="33">
+      <c r="F21" s="34">
         <f>F20*(1+F5)</f>
         <v/>
       </c>
-      <c r="G21" s="33">
+      <c r="G21" s="34">
         <f>G20*(1+G5)</f>
         <v/>
       </c>
-      <c r="H21" s="33">
+      <c r="H21" s="34">
         <f>H20*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="32" t="inlineStr">
+      <c r="A22" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 5</t>
         </is>
       </c>
-      <c r="F22" s="33">
+      <c r="F22" s="34">
         <f>F21*(1+F5)</f>
         <v/>
       </c>
-      <c r="G22" s="33">
+      <c r="G22" s="34">
         <f>G21*(1+G5)</f>
         <v/>
       </c>
-      <c r="H22" s="33">
+      <c r="H22" s="34">
         <f>H21*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="32" t="inlineStr">
+      <c r="A23" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 1</t>
         </is>
       </c>
-      <c r="F23" s="34">
+      <c r="F23" s="35">
         <f>F6+(F8-F6)*0/4</f>
         <v/>
       </c>
-      <c r="G23" s="34">
+      <c r="G23" s="35">
         <f>G6+(G8-G6)*0/4</f>
         <v/>
       </c>
-      <c r="H23" s="34">
+      <c r="H23" s="35">
         <f>H6+(H8-H6)*0/4</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="32" t="inlineStr">
+      <c r="A24" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 2</t>
         </is>
       </c>
-      <c r="F24" s="34">
+      <c r="F24" s="35">
         <f>F6+(F8-F6)*1/4</f>
         <v/>
       </c>
-      <c r="G24" s="34">
+      <c r="G24" s="35">
         <f>G6+(G8-G6)*1/4</f>
         <v/>
       </c>
-      <c r="H24" s="34">
+      <c r="H24" s="35">
         <f>H6+(H8-H6)*1/4</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="32" t="inlineStr">
+      <c r="A25" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 3</t>
         </is>
       </c>
-      <c r="F25" s="34">
+      <c r="F25" s="35">
         <f>F6+(F8-F6)*2/4</f>
         <v/>
       </c>
-      <c r="G25" s="34">
+      <c r="G25" s="35">
         <f>G6+(G8-G6)*2/4</f>
         <v/>
       </c>
-      <c r="H25" s="34">
+      <c r="H25" s="35">
         <f>H6+(H8-H6)*2/4</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="32" t="inlineStr">
+      <c r="A26" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 4</t>
         </is>
       </c>
-      <c r="F26" s="34">
+      <c r="F26" s="35">
         <f>F6+(F8-F6)*3/4</f>
         <v/>
       </c>
-      <c r="G26" s="34">
+      <c r="G26" s="35">
         <f>G6+(G8-G6)*3/4</f>
         <v/>
       </c>
-      <c r="H26" s="34">
+      <c r="H26" s="35">
         <f>H6+(H8-H6)*3/4</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="32" t="inlineStr">
+      <c r="A27" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 5</t>
         </is>
       </c>
-      <c r="F27" s="34">
+      <c r="F27" s="35">
         <f>F6+(F8-F6)*4/4</f>
         <v/>
       </c>
-      <c r="G27" s="34">
+      <c r="G27" s="35">
         <f>G6+(G8-G6)*4/4</f>
         <v/>
       </c>
-      <c r="H27" s="34">
+      <c r="H27" s="35">
         <f>H6+(H8-H6)*4/4</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="32" t="inlineStr">
+      <c r="A28" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 1</t>
         </is>
       </c>
-      <c r="F28" s="33">
+      <c r="F28" s="34">
         <f>F18*F23+F7</f>
         <v/>
       </c>
-      <c r="G28" s="33">
+      <c r="G28" s="34">
         <f>G18*G23+G7</f>
         <v/>
       </c>
-      <c r="H28" s="33">
+      <c r="H28" s="34">
         <f>H18*H23+H7</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="32" t="inlineStr">
+      <c r="A29" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 2</t>
         </is>
       </c>
-      <c r="F29" s="33">
+      <c r="F29" s="34">
         <f>F19*F24</f>
         <v/>
       </c>
-      <c r="G29" s="33">
+      <c r="G29" s="34">
         <f>G19*G24</f>
         <v/>
       </c>
-      <c r="H29" s="33">
+      <c r="H29" s="34">
         <f>H19*H24</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="32" t="inlineStr">
+      <c r="A30" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 3</t>
         </is>
       </c>
-      <c r="F30" s="33">
+      <c r="F30" s="34">
         <f>F20*F25</f>
         <v/>
       </c>
-      <c r="G30" s="33">
+      <c r="G30" s="34">
         <f>G20*G25</f>
         <v/>
       </c>
-      <c r="H30" s="33">
+      <c r="H30" s="34">
         <f>H20*H25</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="32" t="inlineStr">
+      <c r="A31" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 4</t>
         </is>
       </c>
-      <c r="F31" s="33">
+      <c r="F31" s="34">
         <f>F21*F26</f>
         <v/>
       </c>
-      <c r="G31" s="33">
+      <c r="G31" s="34">
         <f>G21*G26</f>
         <v/>
       </c>
-      <c r="H31" s="33">
+      <c r="H31" s="34">
         <f>H21*H26</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="32" t="inlineStr">
+      <c r="A32" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 5</t>
         </is>
       </c>
-      <c r="F32" s="33">
+      <c r="F32" s="34">
         <f>F22*F27</f>
         <v/>
       </c>
-      <c r="G32" s="33">
+      <c r="G32" s="34">
         <f>G22*G27</f>
         <v/>
       </c>
-      <c r="H32" s="33">
+      <c r="H32" s="34">
         <f>H22*H27</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="32" t="inlineStr">
+      <c r="A33" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 1</t>
         </is>
       </c>
-      <c r="F33" s="33">
+      <c r="F33" s="34">
         <f>F28*(1-F11)</f>
         <v/>
       </c>
-      <c r="G33" s="33">
+      <c r="G33" s="34">
         <f>G28*(1-G11)</f>
         <v/>
       </c>
-      <c r="H33" s="33">
+      <c r="H33" s="34">
         <f>H28*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="32" t="inlineStr">
+      <c r="A34" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 2</t>
         </is>
       </c>
-      <c r="F34" s="33">
+      <c r="F34" s="34">
         <f>F29*(1-F11)</f>
         <v/>
       </c>
-      <c r="G34" s="33">
+      <c r="G34" s="34">
         <f>G29*(1-G11)</f>
         <v/>
       </c>
-      <c r="H34" s="33">
+      <c r="H34" s="34">
         <f>H29*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="32" t="inlineStr">
+      <c r="A35" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 3</t>
         </is>
       </c>
-      <c r="F35" s="33">
+      <c r="F35" s="34">
         <f>F30*(1-F11)</f>
         <v/>
       </c>
-      <c r="G35" s="33">
+      <c r="G35" s="34">
         <f>G30*(1-G11)</f>
         <v/>
       </c>
-      <c r="H35" s="33">
+      <c r="H35" s="34">
         <f>H30*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="32" t="inlineStr">
+      <c r="A36" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 4</t>
         </is>
       </c>
-      <c r="F36" s="33">
+      <c r="F36" s="34">
         <f>F31*(1-F11)</f>
         <v/>
       </c>
-      <c r="G36" s="33">
+      <c r="G36" s="34">
         <f>G31*(1-G11)</f>
         <v/>
       </c>
-      <c r="H36" s="33">
+      <c r="H36" s="34">
         <f>H31*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="32" t="inlineStr">
+      <c r="A37" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 5</t>
         </is>
       </c>
-      <c r="F37" s="33">
+      <c r="F37" s="34">
         <f>F32*(1-F11)</f>
         <v/>
       </c>
-      <c r="G37" s="33">
+      <c r="G37" s="34">
         <f>G32*(1-G11)</f>
         <v/>
       </c>
-      <c r="H37" s="33">
+      <c r="H37" s="34">
         <f>H32*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="32" t="inlineStr">
+      <c r="A38" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 1</t>
         </is>
       </c>
-      <c r="F38" s="33">
+      <c r="F38" s="34">
         <f>F18*F12</f>
         <v/>
       </c>
-      <c r="G38" s="33">
+      <c r="G38" s="34">
         <f>G18*G12</f>
         <v/>
       </c>
-      <c r="H38" s="33">
+      <c r="H38" s="34">
         <f>H18*H12</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="32" t="inlineStr">
+      <c r="A39" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 2</t>
         </is>
       </c>
-      <c r="F39" s="33">
+      <c r="F39" s="34">
         <f>F19*F12</f>
         <v/>
       </c>
-      <c r="G39" s="33">
+      <c r="G39" s="34">
         <f>G19*G12</f>
         <v/>
       </c>
-      <c r="H39" s="33">
+      <c r="H39" s="34">
         <f>H19*H12</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="32" t="inlineStr">
+      <c r="A40" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 3</t>
         </is>
       </c>
-      <c r="F40" s="33">
+      <c r="F40" s="34">
         <f>F20*F12</f>
         <v/>
       </c>
-      <c r="G40" s="33">
+      <c r="G40" s="34">
         <f>G20*G12</f>
         <v/>
       </c>
-      <c r="H40" s="33">
+      <c r="H40" s="34">
         <f>H20*H12</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="32" t="inlineStr">
+      <c r="A41" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 4</t>
         </is>
       </c>
-      <c r="F41" s="33">
+      <c r="F41" s="34">
         <f>F21*F12</f>
         <v/>
       </c>
-      <c r="G41" s="33">
+      <c r="G41" s="34">
         <f>G21*G12</f>
         <v/>
       </c>
-      <c r="H41" s="33">
+      <c r="H41" s="34">
         <f>H21*H12</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="32" t="inlineStr">
+      <c r="A42" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 5</t>
         </is>
       </c>
-      <c r="F42" s="33">
+      <c r="F42" s="34">
         <f>F22*F12</f>
         <v/>
       </c>
-      <c r="G42" s="33">
+      <c r="G42" s="34">
         <f>G22*G12</f>
         <v/>
       </c>
-      <c r="H42" s="33">
+      <c r="H42" s="34">
         <f>H22*H12</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="32" t="inlineStr">
+      <c r="A43" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 1</t>
         </is>
       </c>
-      <c r="F43" s="33">
+      <c r="F43" s="34">
         <f>F18*F13</f>
         <v/>
       </c>
-      <c r="G43" s="33">
+      <c r="G43" s="34">
         <f>G18*G13</f>
         <v/>
       </c>
-      <c r="H43" s="33">
+      <c r="H43" s="34">
         <f>H18*H13</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="32" t="inlineStr">
+      <c r="A44" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 2</t>
         </is>
       </c>
-      <c r="F44" s="33">
+      <c r="F44" s="34">
         <f>F19*F13</f>
         <v/>
       </c>
-      <c r="G44" s="33">
+      <c r="G44" s="34">
         <f>G19*G13</f>
         <v/>
       </c>
-      <c r="H44" s="33">
+      <c r="H44" s="34">
         <f>H19*H13</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="32" t="inlineStr">
+      <c r="A45" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 3</t>
         </is>
       </c>
-      <c r="F45" s="33">
+      <c r="F45" s="34">
         <f>F20*F13</f>
         <v/>
       </c>
-      <c r="G45" s="33">
+      <c r="G45" s="34">
         <f>G20*G13</f>
         <v/>
       </c>
-      <c r="H45" s="33">
+      <c r="H45" s="34">
         <f>H20*H13</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="32" t="inlineStr">
+      <c r="A46" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 4</t>
         </is>
       </c>
-      <c r="F46" s="33">
+      <c r="F46" s="34">
         <f>F21*F13</f>
         <v/>
       </c>
-      <c r="G46" s="33">
+      <c r="G46" s="34">
         <f>G21*G13</f>
         <v/>
       </c>
-      <c r="H46" s="33">
+      <c r="H46" s="34">
         <f>H21*H13</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="32" t="inlineStr">
+      <c r="A47" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 5</t>
         </is>
       </c>
-      <c r="F47" s="33">
+      <c r="F47" s="34">
         <f>F22*F13</f>
         <v/>
       </c>
-      <c r="G47" s="33">
+      <c r="G47" s="34">
         <f>G22*G13</f>
         <v/>
       </c>
-      <c r="H47" s="33">
+      <c r="H47" s="34">
         <f>H22*H13</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="32" t="inlineStr">
+      <c r="A48" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 1</t>
         </is>
       </c>
-      <c r="F48" s="33">
+      <c r="F48" s="34">
         <f>F18*F15</f>
         <v/>
       </c>
-      <c r="G48" s="33">
+      <c r="G48" s="34">
         <f>G18*G15</f>
         <v/>
       </c>
-      <c r="H48" s="33">
+      <c r="H48" s="34">
         <f>H18*H15</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="32" t="inlineStr">
+      <c r="A49" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 2</t>
         </is>
       </c>
-      <c r="F49" s="33">
+      <c r="F49" s="34">
         <f>F19*F15</f>
         <v/>
       </c>
-      <c r="G49" s="33">
+      <c r="G49" s="34">
         <f>G19*G15</f>
         <v/>
       </c>
-      <c r="H49" s="33">
+      <c r="H49" s="34">
         <f>H19*H15</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="32" t="inlineStr">
+      <c r="A50" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 3</t>
         </is>
       </c>
-      <c r="F50" s="33">
+      <c r="F50" s="34">
         <f>F20*F15</f>
         <v/>
       </c>
-      <c r="G50" s="33">
+      <c r="G50" s="34">
         <f>G20*G15</f>
         <v/>
       </c>
-      <c r="H50" s="33">
+      <c r="H50" s="34">
         <f>H20*H15</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="32" t="inlineStr">
+      <c r="A51" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 4</t>
         </is>
       </c>
-      <c r="F51" s="33">
+      <c r="F51" s="34">
         <f>F21*F15</f>
         <v/>
       </c>
-      <c r="G51" s="33">
+      <c r="G51" s="34">
         <f>G21*G15</f>
         <v/>
       </c>
-      <c r="H51" s="33">
+      <c r="H51" s="34">
         <f>H21*H15</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="32" t="inlineStr">
+      <c r="A52" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 5</t>
         </is>
       </c>
-      <c r="F52" s="33">
+      <c r="F52" s="34">
         <f>F22*F15</f>
         <v/>
       </c>
-      <c r="G52" s="33">
+      <c r="G52" s="34">
         <f>G22*G15</f>
         <v/>
       </c>
-      <c r="H52" s="33">
+      <c r="H52" s="34">
         <f>H22*H15</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="32" t="inlineStr">
+      <c r="A53" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 1</t>
         </is>
       </c>
-      <c r="F53" s="33">
+      <c r="F53" s="34">
         <f>F14*(F18-11102600)</f>
         <v/>
       </c>
-      <c r="G53" s="33">
+      <c r="G53" s="34">
         <f>G14*(G18-11102600)</f>
         <v/>
       </c>
-      <c r="H53" s="33">
+      <c r="H53" s="34">
         <f>H14*(H18-11102600)</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="32" t="inlineStr">
+      <c r="A54" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 2</t>
         </is>
       </c>
-      <c r="F54" s="33">
+      <c r="F54" s="34">
         <f>F14*(F19-F18)</f>
         <v/>
       </c>
-      <c r="G54" s="33">
+      <c r="G54" s="34">
         <f>G14*(G19-G18)</f>
         <v/>
       </c>
-      <c r="H54" s="33">
+      <c r="H54" s="34">
         <f>H14*(H19-H18)</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="32" t="inlineStr">
+      <c r="A55" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 3</t>
         </is>
       </c>
-      <c r="F55" s="33">
+      <c r="F55" s="34">
         <f>F14*(F20-F19)</f>
         <v/>
       </c>
-      <c r="G55" s="33">
+      <c r="G55" s="34">
         <f>G14*(G20-G19)</f>
         <v/>
       </c>
-      <c r="H55" s="33">
+      <c r="H55" s="34">
         <f>H14*(H20-H19)</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="32" t="inlineStr">
+      <c r="A56" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 4</t>
         </is>
       </c>
-      <c r="F56" s="33">
+      <c r="F56" s="34">
         <f>F14*(F21-F20)</f>
         <v/>
       </c>
-      <c r="G56" s="33">
+      <c r="G56" s="34">
         <f>G14*(G21-G20)</f>
         <v/>
       </c>
-      <c r="H56" s="33">
+      <c r="H56" s="34">
         <f>H14*(H21-H20)</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="32" t="inlineStr">
+      <c r="A57" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 5</t>
         </is>
       </c>
-      <c r="F57" s="33">
+      <c r="F57" s="34">
         <f>F14*(F22-F21)</f>
         <v/>
       </c>
-      <c r="G57" s="33">
+      <c r="G57" s="34">
         <f>G14*(G22-G21)</f>
         <v/>
       </c>
-      <c r="H57" s="33">
+      <c r="H57" s="34">
         <f>H14*(H22-H21)</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="32" t="inlineStr">
+      <c r="A58" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 1</t>
         </is>
       </c>
-      <c r="F58" s="33">
+      <c r="F58" s="34">
         <f>F33+F38-F43-F53</f>
         <v/>
       </c>
-      <c r="G58" s="33">
+      <c r="G58" s="34">
         <f>G33+G38-G43-G53</f>
         <v/>
       </c>
-      <c r="H58" s="33">
+      <c r="H58" s="34">
         <f>H33+H38-H43-H53</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="32" t="inlineStr">
+      <c r="A59" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 2</t>
         </is>
       </c>
-      <c r="F59" s="33">
+      <c r="F59" s="34">
         <f>F34+F39-F44-F54</f>
         <v/>
       </c>
-      <c r="G59" s="33">
+      <c r="G59" s="34">
         <f>G34+G39-G44-G54</f>
         <v/>
       </c>
-      <c r="H59" s="33">
+      <c r="H59" s="34">
         <f>H34+H39-H44-H54</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="32" t="inlineStr">
+      <c r="A60" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 3</t>
         </is>
       </c>
-      <c r="F60" s="33">
+      <c r="F60" s="34">
         <f>F35+F40-F45-F55</f>
         <v/>
       </c>
-      <c r="G60" s="33">
+      <c r="G60" s="34">
         <f>G35+G40-G45-G55</f>
         <v/>
       </c>
-      <c r="H60" s="33">
+      <c r="H60" s="34">
         <f>H35+H40-H45-H55</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="32" t="inlineStr">
+      <c r="A61" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 4</t>
         </is>
       </c>
-      <c r="F61" s="33">
+      <c r="F61" s="34">
         <f>F36+F41-F46-F56</f>
         <v/>
       </c>
-      <c r="G61" s="33">
+      <c r="G61" s="34">
         <f>G36+G41-G46-G56</f>
         <v/>
       </c>
-      <c r="H61" s="33">
+      <c r="H61" s="34">
         <f>H36+H41-H46-H56</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="32" t="inlineStr">
+      <c r="A62" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 5</t>
         </is>
       </c>
-      <c r="F62" s="33">
+      <c r="F62" s="34">
         <f>F37+F42-F47-F57</f>
         <v/>
       </c>
-      <c r="G62" s="33">
+      <c r="G62" s="34">
         <f>G37+G42-G47-G57</f>
         <v/>
       </c>
-      <c r="H62" s="33">
+      <c r="H62" s="34">
         <f>H37+H42-H47-H57</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="22" t="inlineStr">
+      <c r="A64" s="23" t="inlineStr">
         <is>
           <t>Enterprise value (DCF)</t>
         </is>
       </c>
-      <c r="F64" s="35">
+      <c r="F64" s="36">
         <f>NPV(F9,F58,F59,F60,F61,F62)+(F62*(1+F10)/(F9-F10))/(1+F9)^5</f>
         <v/>
       </c>
-      <c r="G64" s="35">
+      <c r="G64" s="36">
         <f>NPV(G9,G58,G59,G60,G61,G62)+(G62*(1+G10)/(G9-G10))/(1+G9)^5</f>
         <v/>
       </c>
-      <c r="H64" s="35">
+      <c r="H64" s="36">
         <f>NPV(H9,H58,H59,H60,H61,H62)+(H62*(1+H10)/(H9-H10))/(1+H9)^5</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="36" t="inlineStr">
+      <c r="A65" s="37" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="F65" s="37">
+      <c r="F65" s="38">
         <f>(F64+1807202-0)/111380</f>
         <v/>
       </c>
-      <c r="G65" s="38">
+      <c r="G65" s="39">
         <f>(G64+1807202-0)/111380</f>
         <v/>
       </c>
-      <c r="H65" s="37">
+      <c r="H65" s="38">
         <f>(H64+1807202-0)/111380</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="22" t="inlineStr">
+      <c r="A66" s="23" t="inlineStr">
         <is>
           <t>Upside / (downside) vs current</t>
         </is>
       </c>
-      <c r="F66" s="39">
+      <c r="F66" s="40">
         <f>F65/100.0-1</f>
         <v/>
       </c>
-      <c r="G66" s="39">
+      <c r="G66" s="40">
         <f>G65/100.0-1</f>
         <v/>
       </c>
-      <c r="H66" s="39">
+      <c r="H66" s="40">
         <f>H65/100.0-1</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="40" t="inlineStr">
+      <c r="A68" s="41" t="inlineStr">
         <is>
           <t>Current price $100.00; cash $1,807,202 k; net debt $0 (net-cash balance sheet).</t>
         </is>
@@ -2887,69 +2887,69 @@
       <c r="J1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="B2" s="41" t="inlineStr">
+      <c r="B2" s="42" t="inlineStr">
         <is>
           <t>Justification (~20 words)</t>
         </is>
       </c>
-      <c r="C2" s="41" t="inlineStr">
+      <c r="C2" s="42" t="inlineStr">
         <is>
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D2" s="41" t="inlineStr">
+      <c r="D2" s="42" t="inlineStr">
         <is>
           <t>Ctrl+F (prove number)</t>
         </is>
       </c>
-      <c r="E2" s="42" t="inlineStr">
+      <c r="E2" s="43" t="inlineStr">
         <is>
           <t>FY2025A</t>
         </is>
       </c>
-      <c r="F2" s="43" t="inlineStr">
+      <c r="F2" s="44" t="inlineStr">
         <is>
           <t>FY2026E</t>
         </is>
       </c>
-      <c r="G2" s="43" t="inlineStr">
+      <c r="G2" s="44" t="inlineStr">
         <is>
           <t>FY2027E</t>
         </is>
       </c>
-      <c r="H2" s="43" t="inlineStr">
+      <c r="H2" s="44" t="inlineStr">
         <is>
           <t>FY2028E</t>
         </is>
       </c>
-      <c r="I2" s="43" t="inlineStr">
+      <c r="I2" s="44" t="inlineStr">
         <is>
           <t>FY2029E</t>
         </is>
       </c>
-      <c r="J2" s="43" t="inlineStr">
+      <c r="J2" s="44" t="inlineStr">
         <is>
           <t>FY2030E</t>
         </is>
       </c>
-      <c r="K2" s="44" t="inlineStr">
+      <c r="K2" s="45" t="inlineStr">
         <is>
           <t>Δ vs Scenarios</t>
         </is>
       </c>
-      <c r="L2" s="41" t="inlineStr">
+      <c r="L2" s="42" t="inlineStr">
         <is>
           <t>Alt. source</t>
         </is>
       </c>
-      <c r="M2" s="41" t="inlineStr">
+      <c r="M2" s="42" t="inlineStr">
         <is>
           <t>Alt. Ctrl+F</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="45" t="inlineStr">
+      <c r="A3" s="46" t="inlineStr">
         <is>
           <t>Forecast drivers linked to Scenarios tab → Base case (column G)</t>
         </is>
@@ -2959,12 +2959,12 @@
           <t>Ctrl+F "Net revenue" → 11,102,600 or "Depreciation and amortization" → 496,228 on this 10-K HTML file</t>
         </is>
       </c>
-      <c r="E3" s="46" t="inlineStr">
+      <c r="E3" s="47" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="K3" s="47" t="inlineStr">
+      <c r="K3" s="48" t="inlineStr">
         <is>
           <t>(should be 0)</t>
         </is>
@@ -2976,30 +2976,30 @@
           <t>Net revenue</t>
         </is>
       </c>
-      <c r="E5" s="48" t="n">
+      <c r="E5" s="49" t="n">
         <v>11102600</v>
       </c>
-      <c r="F5" s="49">
+      <c r="F5" s="50">
         <f>Scenarios!G18</f>
         <v/>
       </c>
-      <c r="G5" s="49">
+      <c r="G5" s="50">
         <f>Scenarios!G19</f>
         <v/>
       </c>
-      <c r="H5" s="49">
+      <c r="H5" s="50">
         <f>Scenarios!G20</f>
         <v/>
       </c>
-      <c r="I5" s="49">
+      <c r="I5" s="50">
         <f>Scenarios!G21</f>
         <v/>
       </c>
-      <c r="J5" s="49">
+      <c r="J5" s="50">
         <f>Scenarios!G22</f>
         <v/>
       </c>
-      <c r="K5" s="50">
+      <c r="K5" s="51">
         <f>IF(MAX(ABS(F5-Scenarios!$G$18),ABS(G5-Scenarios!$G$19),ABS(H5-Scenarios!$G$20),ABS(I5-Scenarios!$G$21),ABS(J5-Scenarios!$G$22))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3016,7 +3016,7 @@
 Also: 2.3% FY27–30 growth matches StockAnalysis Revenue Growth Forecast (3Y) of 2.26%; next-year consensus is +2.64%.</t>
         </is>
       </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C6" s="32" t="inlineStr">
         <is>
           <t>LULU Q2 FY2026 earnings release
 Also: StockAnalysis: LULU 3Y revenue forecast</t>
@@ -3028,23 +3028,23 @@
 Also: Ctrl+F "Revenue Growth Forecast (3Y)" → 2.26%. That is the unique line (do not search "Net revenue"). Model FY27–30 uses 2.3%.</t>
         </is>
       </c>
-      <c r="F6" s="51">
+      <c r="F6" s="52">
         <f>F5/E5-1</f>
         <v/>
       </c>
-      <c r="G6" s="51">
+      <c r="G6" s="52">
         <f>G5/F5-1</f>
         <v/>
       </c>
-      <c r="H6" s="51">
+      <c r="H6" s="52">
         <f>H5/G5-1</f>
         <v/>
       </c>
-      <c r="I6" s="51">
+      <c r="I6" s="52">
         <f>I5/H5-1</f>
         <v/>
       </c>
-      <c r="J6" s="51">
+      <c r="J6" s="52">
         <f>J5/I5-1</f>
         <v/>
       </c>
@@ -3061,7 +3061,7 @@
 Also: FY30 15.5% is a partial recovery vs the FY25 10-K OM of 19.9% (unique Ctrl+F). Still well below the FY24 23.7% peak.</t>
         </is>
       </c>
-      <c r="C7" s="31" t="inlineStr">
+      <c r="C7" s="32" t="inlineStr">
         <is>
           <t>Q2 FY2026 release: 18.8% OM minus 560bps tariffs
 Also: FY2025 10-K: Operating margin 19.9% (one hit)</t>
@@ -3073,27 +3073,27 @@
 Also: Ctrl+F "19.9%" (one hit) → Operating margin decreased 380 basis points to 19.9%. That is FY25 OM. Do not search the words Income from operations (17 hits). Model FY30 15.5% is a partial-recovery assumption.</t>
         </is>
       </c>
-      <c r="F7" s="51">
+      <c r="F7" s="52">
         <f>Scenarios!G23</f>
         <v/>
       </c>
-      <c r="G7" s="51">
+      <c r="G7" s="52">
         <f>Scenarios!G24</f>
         <v/>
       </c>
-      <c r="H7" s="51">
+      <c r="H7" s="52">
         <f>Scenarios!G25</f>
         <v/>
       </c>
-      <c r="I7" s="51">
+      <c r="I7" s="52">
         <f>Scenarios!G26</f>
         <v/>
       </c>
-      <c r="J7" s="51">
+      <c r="J7" s="52">
         <f>Scenarios!G27</f>
         <v/>
       </c>
-      <c r="K7" s="50">
+      <c r="K7" s="51">
         <f>IF(MAX(ABS(F7-Scenarios!$G$23),ABS(G7-Scenarios!$G$24),ABS(H7-Scenarios!$G$25),ABS(I7-Scenarios!$G$26),ABS(J7-Scenarios!$G$27))&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3119,56 +3119,56 @@
           <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
         </is>
       </c>
-      <c r="E8" s="48" t="n">
+      <c r="E8" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="30">
+      <c r="F8" s="31">
         <f>Scenarios!$G$7</f>
         <v/>
       </c>
-      <c r="G8" s="30" t="n">
+      <c r="G8" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="30" t="n">
+      <c r="H8" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="30" t="n">
+      <c r="I8" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="30" t="n">
+      <c r="J8" s="31" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>EBIT (incl. FY26 refund)</t>
         </is>
       </c>
-      <c r="E9" s="52" t="n">
+      <c r="E9" s="53" t="n">
         <v>2210615</v>
       </c>
-      <c r="F9" s="35">
+      <c r="F9" s="36">
         <f>Scenarios!G28</f>
         <v/>
       </c>
-      <c r="G9" s="35">
+      <c r="G9" s="36">
         <f>Scenarios!G29</f>
         <v/>
       </c>
-      <c r="H9" s="35">
+      <c r="H9" s="36">
         <f>Scenarios!G30</f>
         <v/>
       </c>
-      <c r="I9" s="35">
+      <c r="I9" s="36">
         <f>Scenarios!G31</f>
         <v/>
       </c>
-      <c r="J9" s="35">
+      <c r="J9" s="36">
         <f>Scenarios!G32</f>
         <v/>
       </c>
-      <c r="K9" s="53">
+      <c r="K9" s="54">
         <f>IF(MAX(ABS(F9-Scenarios!$G$28),ABS(G9-Scenarios!$G$29),ABS(H9-Scenarios!$G$30),ABS(I9-Scenarios!$G$31),ABS(J9-Scenarios!$G$32))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3179,26 +3179,26 @@
           <t>Reported EBIT margin % (incl. FY26 refund)</t>
         </is>
       </c>
-      <c r="E10" s="54" t="n">
+      <c r="E10" s="55" t="n">
         <v>0.1991078666258354</v>
       </c>
-      <c r="F10" s="51">
+      <c r="F10" s="52">
         <f>F9/F5</f>
         <v/>
       </c>
-      <c r="G10" s="51">
+      <c r="G10" s="52">
         <f>G9/G5</f>
         <v/>
       </c>
-      <c r="H10" s="51">
+      <c r="H10" s="52">
         <f>H9/H5</f>
         <v/>
       </c>
-      <c r="I10" s="51">
+      <c r="I10" s="52">
         <f>I9/I5</f>
         <v/>
       </c>
-      <c r="J10" s="51">
+      <c r="J10" s="52">
         <f>J9/J5</f>
         <v/>
       </c>
@@ -3209,54 +3209,54 @@
           <t>Less: cash taxes on EBIT</t>
         </is>
       </c>
-      <c r="F11" s="49">
+      <c r="F11" s="50">
         <f>-Scenarios!G28*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="G11" s="49">
+      <c r="G11" s="50">
         <f>-Scenarios!G29*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="H11" s="49">
+      <c r="H11" s="50">
         <f>-Scenarios!G30*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="I11" s="49">
+      <c r="I11" s="50">
         <f>-Scenarios!G31*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="J11" s="49">
+      <c r="J11" s="50">
         <f>-Scenarios!G32*Scenarios!$G$11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>NOPAT</t>
         </is>
       </c>
-      <c r="F12" s="35">
+      <c r="F12" s="36">
         <f>Scenarios!G33</f>
         <v/>
       </c>
-      <c r="G12" s="35">
+      <c r="G12" s="36">
         <f>Scenarios!G34</f>
         <v/>
       </c>
-      <c r="H12" s="35">
+      <c r="H12" s="36">
         <f>Scenarios!G35</f>
         <v/>
       </c>
-      <c r="I12" s="35">
+      <c r="I12" s="36">
         <f>Scenarios!G36</f>
         <v/>
       </c>
-      <c r="J12" s="35">
+      <c r="J12" s="36">
         <f>Scenarios!G37</f>
         <v/>
       </c>
-      <c r="K12" s="53">
+      <c r="K12" s="54">
         <f>IF(MAX(ABS(F12-Scenarios!$G$33),ABS(G12-Scenarios!$G$34),ABS(H12-Scenarios!$G$35),ABS(I12-Scenarios!$G$36),ABS(J12-Scenarios!$G$37))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3309,27 +3309,27 @@
           <t>Plus: depreciation &amp; amortization</t>
         </is>
       </c>
-      <c r="F14" s="49">
+      <c r="F14" s="50">
         <f>Scenarios!G38</f>
         <v/>
       </c>
-      <c r="G14" s="49">
+      <c r="G14" s="50">
         <f>Scenarios!G39</f>
         <v/>
       </c>
-      <c r="H14" s="49">
+      <c r="H14" s="50">
         <f>Scenarios!G40</f>
         <v/>
       </c>
-      <c r="I14" s="49">
+      <c r="I14" s="50">
         <f>Scenarios!G41</f>
         <v/>
       </c>
-      <c r="J14" s="49">
+      <c r="J14" s="50">
         <f>Scenarios!G42</f>
         <v/>
       </c>
-      <c r="K14" s="50">
+      <c r="K14" s="51">
         <f>IF(MAX(ABS(F14-Scenarios!$G$38),ABS(G14-Scenarios!$G$39),ABS(H14-Scenarios!$G$40),ABS(I14-Scenarios!$G$41),ABS(J14-Scenarios!$G$42))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3346,7 +3346,7 @@
 Also: FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
         </is>
       </c>
-      <c r="C15" s="31" t="inlineStr">
+      <c r="C15" s="32" t="inlineStr">
         <is>
           <t>LULU 10-K: 2026 capex guide $725–745M
 Also: Q2 FY2026 outlook: $10.350B–$10.500B sales</t>
@@ -3395,27 +3395,27 @@
           <t>Less: capital expenditures</t>
         </is>
       </c>
-      <c r="F16" s="49">
+      <c r="F16" s="50">
         <f>-Scenarios!G43</f>
         <v/>
       </c>
-      <c r="G16" s="49">
+      <c r="G16" s="50">
         <f>-Scenarios!G44</f>
         <v/>
       </c>
-      <c r="H16" s="49">
+      <c r="H16" s="50">
         <f>-Scenarios!G45</f>
         <v/>
       </c>
-      <c r="I16" s="49">
+      <c r="I16" s="50">
         <f>-Scenarios!G46</f>
         <v/>
       </c>
-      <c r="J16" s="49">
+      <c r="J16" s="50">
         <f>-Scenarios!G47</f>
         <v/>
       </c>
-      <c r="K16" s="50">
+      <c r="K16" s="51">
         <f>IF(MAX(ABS(F16+Scenarios!$G$43),ABS(G16+Scenarios!$G$44),ABS(H16+Scenarios!$G$45),ABS(I16+Scenarios!$G$46),ABS(J16+Scenarios!$G$47))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3525,30 +3525,30 @@
           <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. Lives inside the NWC line below.</t>
         </is>
       </c>
-      <c r="E19" s="48" t="n">
+      <c r="E19" s="49" t="n">
         <v>190657</v>
       </c>
-      <c r="F19" s="49">
+      <c r="F19" s="50">
         <f>Scenarios!G48</f>
         <v/>
       </c>
-      <c r="G19" s="49">
+      <c r="G19" s="50">
         <f>Scenarios!G49</f>
         <v/>
       </c>
-      <c r="H19" s="49">
+      <c r="H19" s="50">
         <f>Scenarios!G50</f>
         <v/>
       </c>
-      <c r="I19" s="49">
+      <c r="I19" s="50">
         <f>Scenarios!G51</f>
         <v/>
       </c>
-      <c r="J19" s="49">
+      <c r="J19" s="50">
         <f>Scenarios!G52</f>
         <v/>
       </c>
-      <c r="K19" s="50">
+      <c r="K19" s="51">
         <f>IF(MAX(ABS(F19-Scenarios!$G$48),ABS(G19-Scenarios!$G$49),ABS(H19-Scenarios!$G$50),ABS(I19-Scenarios!$G$51),ABS(J19-Scenarios!$G$52))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3559,65 +3559,65 @@
           <t>(Increase)/decrease in NWC (includes AR)</t>
         </is>
       </c>
-      <c r="F20" s="49">
+      <c r="F20" s="50">
         <f>-Scenarios!G53</f>
         <v/>
       </c>
-      <c r="G20" s="49">
+      <c r="G20" s="50">
         <f>-Scenarios!G54</f>
         <v/>
       </c>
-      <c r="H20" s="49">
+      <c r="H20" s="50">
         <f>-Scenarios!G55</f>
         <v/>
       </c>
-      <c r="I20" s="49">
+      <c r="I20" s="50">
         <f>-Scenarios!G56</f>
         <v/>
       </c>
-      <c r="J20" s="49">
+      <c r="J20" s="50">
         <f>-Scenarios!G57</f>
         <v/>
       </c>
-      <c r="K20" s="50">
+      <c r="K20" s="51">
         <f>IF(MAX(ABS(F20+Scenarios!$G$53),ABS(G20+Scenarios!$G$54),ABS(H20+Scenarios!$G$55),ABS(I20+Scenarios!$G$56),ABS(J20+Scenarios!$G$57))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="40" t="inlineStr">
+      <c r="A21" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: NWC and AR are one line. 7.5% of Δsales already includes AR; UFCF does not take ΔAR separately.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t>Unlevered free cash flow</t>
         </is>
       </c>
-      <c r="F22" s="55">
+      <c r="F22" s="56">
         <f>Scenarios!G58</f>
         <v/>
       </c>
-      <c r="G22" s="55">
+      <c r="G22" s="56">
         <f>Scenarios!G59</f>
         <v/>
       </c>
-      <c r="H22" s="55">
+      <c r="H22" s="56">
         <f>Scenarios!G60</f>
         <v/>
       </c>
-      <c r="I22" s="55">
+      <c r="I22" s="56">
         <f>Scenarios!G61</f>
         <v/>
       </c>
-      <c r="J22" s="55">
+      <c r="J22" s="56">
         <f>Scenarios!G62</f>
         <v/>
       </c>
-      <c r="K22" s="53">
+      <c r="K22" s="54">
         <f>IF(MAX(ABS(F22-Scenarios!$G$58),ABS(G22-Scenarios!$G$59),ABS(H22-Scenarios!$G$60),ABS(I22-Scenarios!$G$61),ABS(J22-Scenarios!$G$62))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3628,19 +3628,19 @@
           <t>Discount period (years)</t>
         </is>
       </c>
-      <c r="F23" s="56" t="n">
+      <c r="F23" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="56" t="n">
+      <c r="G23" s="57" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="56" t="n">
+      <c r="H23" s="57" t="n">
         <v>3</v>
       </c>
-      <c r="I23" s="56" t="n">
+      <c r="I23" s="57" t="n">
         <v>4</v>
       </c>
-      <c r="J23" s="56" t="n">
+      <c r="J23" s="57" t="n">
         <v>5</v>
       </c>
     </row>
@@ -3650,50 +3650,50 @@
           <t>Discount factor @ WACC</t>
         </is>
       </c>
-      <c r="F24" s="57">
+      <c r="F24" s="58">
         <f>1/(1+Scenarios!$G$9)^F23</f>
         <v/>
       </c>
-      <c r="G24" s="57">
+      <c r="G24" s="58">
         <f>1/(1+Scenarios!$G$9)^G23</f>
         <v/>
       </c>
-      <c r="H24" s="57">
+      <c r="H24" s="58">
         <f>1/(1+Scenarios!$G$9)^H23</f>
         <v/>
       </c>
-      <c r="I24" s="57">
+      <c r="I24" s="58">
         <f>1/(1+Scenarios!$G$9)^I23</f>
         <v/>
       </c>
-      <c r="J24" s="57">
+      <c r="J24" s="58">
         <f>1/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="22" t="inlineStr">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>PV of unlevered FCF</t>
         </is>
       </c>
-      <c r="F25" s="35">
+      <c r="F25" s="36">
         <f>F22*F24</f>
         <v/>
       </c>
-      <c r="G25" s="35">
+      <c r="G25" s="36">
         <f>G22*G24</f>
         <v/>
       </c>
-      <c r="H25" s="35">
+      <c r="H25" s="36">
         <f>H22*H24</f>
         <v/>
       </c>
-      <c r="I25" s="35">
+      <c r="I25" s="36">
         <f>I22*I24</f>
         <v/>
       </c>
-      <c r="J25" s="35">
+      <c r="J25" s="36">
         <f>J22*J24</f>
         <v/>
       </c>
@@ -3704,13 +3704,13 @@
           <t>Scenarios linkage summary (column K should all read OK)</t>
         </is>
       </c>
-      <c r="K27" s="58">
+      <c r="K27" s="59">
         <f>IF(COUNTIF(K5:K22,"CHECK")=0,"ALL OK","REVIEW")</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="59" t="inlineStr">
+      <c r="A28" s="60" t="inlineStr">
         <is>
           <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
         </is>
@@ -3719,12 +3719,12 @@
       <c r="C28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="22" t="inlineStr">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>Sum of PV of explicit FCF (FY26–FY30)</t>
         </is>
       </c>
-      <c r="E29" s="60">
+      <c r="E29" s="61">
         <f>SUM(F25:J25)</f>
         <v/>
       </c>
@@ -3750,18 +3750,18 @@
           <t>Ctrl+F "Q2 2026" → 24,269.613 and "Q2 2025" → 23,770.976. YoY = 2.1%. Model terminal g 2.25%.</t>
         </is>
       </c>
-      <c r="E30" s="51">
+      <c r="E30" s="52">
         <f>Scenarios!$G$10</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="22" t="inlineStr">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="E31" s="35">
+      <c r="E31" s="36">
         <f>J9+J14</f>
         <v/>
       </c>
@@ -3772,7 +3772,7 @@
           <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
         </is>
       </c>
-      <c r="E32" s="49">
+      <c r="E32" s="50">
         <f>J22*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
         <v/>
       </c>
@@ -3783,29 +3783,29 @@
           <t xml:space="preserve">  Implied exit EV/EBITDA (Gordon Growth)</t>
         </is>
       </c>
-      <c r="E33" s="61">
+      <c r="E33" s="62">
         <f>E32/E31</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="22" t="inlineStr">
+      <c r="A34" s="23" t="inlineStr">
         <is>
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="E34" s="60">
+      <c r="E34" s="61">
         <f>E32/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="22" t="inlineStr">
+      <c r="A35" s="23" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="E35" s="35">
+      <c r="E35" s="36">
         <f>E29+E34</f>
         <v/>
       </c>
@@ -3816,7 +3816,7 @@
           <t>Plus: cash &amp; equivalents (FY2025)</t>
         </is>
       </c>
-      <c r="C36" s="62" t="inlineStr">
+      <c r="C36" s="63" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -3826,7 +3826,7 @@
           <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
         </is>
       </c>
-      <c r="E36" s="48" t="n">
+      <c r="E36" s="49" t="n">
         <v>1807202</v>
       </c>
     </row>
@@ -3836,7 +3836,7 @@
           <t>Less: total debt</t>
         </is>
       </c>
-      <c r="C37" s="62" t="inlineStr">
+      <c r="C37" s="63" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -3846,17 +3846,17 @@
           <t>Ctrl+F "no borrowings were outstanding under this facility" → no funded term debt</t>
         </is>
       </c>
-      <c r="E37" s="48" t="n">
+      <c r="E37" s="49" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="22" t="inlineStr">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
       </c>
-      <c r="E38" s="35">
+      <c r="E38" s="36">
         <f>E35+E36+E37</f>
         <v/>
       </c>
@@ -3867,7 +3867,7 @@
           <t>Diluted shares outstanding (000)</t>
         </is>
       </c>
-      <c r="C39" s="62" t="inlineStr">
+      <c r="C39" s="63" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -3877,21 +3877,21 @@
           <t>Ctrl+F "Diluted weighted-average number of shares outstanding" → 119,068 (000)</t>
         </is>
       </c>
-      <c r="E39" s="48" t="n">
+      <c r="E39" s="49" t="n">
         <v>111380</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="22" t="inlineStr">
+      <c r="A40" s="23" t="inlineStr">
         <is>
           <t>Implied value per share</t>
         </is>
       </c>
-      <c r="E40" s="63">
+      <c r="E40" s="64">
         <f>E38/E39</f>
         <v/>
       </c>
-      <c r="K40" s="53">
+      <c r="K40" s="54">
         <f>IF(ABS(E40-Scenarios!$G$65)&lt;0.05,"OK","CHECK")</f>
         <v/>
       </c>
@@ -3902,7 +3902,7 @@
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C41" s="62" t="inlineStr">
+      <c r="C41" s="63" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -3912,17 +3912,17 @@
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E41" s="64" t="n">
+      <c r="E41" s="65" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="22" t="inlineStr">
+      <c r="A42" s="23" t="inlineStr">
         <is>
           <t>Implied upside / (downside)</t>
         </is>
       </c>
-      <c r="E42" s="65">
+      <c r="E42" s="66">
         <f>E40/E41-1</f>
         <v/>
       </c>
@@ -3933,13 +3933,13 @@
           <t xml:space="preserve">  memo: % of EV from terminal value</t>
         </is>
       </c>
-      <c r="E43" s="51">
+      <c r="E43" s="52">
         <f>E34/E35</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="59" t="inlineStr">
+      <c r="A45" s="60" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
@@ -3975,10 +3975,10 @@
           <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x (assumption)</t>
         </is>
       </c>
-      <c r="E47" s="66" t="n">
+      <c r="E47" s="67" t="n">
         <v>8</v>
       </c>
-      <c r="M47" s="62" t="inlineStr">
+      <c r="M47" s="63" t="inlineStr">
         <is>
           <t>Comps: Exit Multiple Build</t>
         </is>
@@ -3990,7 +3990,7 @@
           <t>Terminal value = Terminal EBITDA × exit multiple</t>
         </is>
       </c>
-      <c r="E48" s="49">
+      <c r="E48" s="50">
         <f>E31*E47</f>
         <v/>
       </c>
@@ -4001,35 +4001,35 @@
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="E49" s="49">
+      <c r="E49" s="50">
         <f>E48/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="22" t="inlineStr">
+      <c r="A50" s="23" t="inlineStr">
         <is>
           <t>Enterprise value (exit method)</t>
         </is>
       </c>
-      <c r="E50" s="35">
+      <c r="E50" s="36">
         <f>E29+E49</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="22" t="inlineStr">
+      <c r="A51" s="23" t="inlineStr">
         <is>
           <t>Implied value per share (exit method)</t>
         </is>
       </c>
-      <c r="E51" s="67">
+      <c r="E51" s="68">
         <f>(E50+E36+E37)/E39</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="59" t="inlineStr">
+      <c r="A53" s="60" t="inlineStr">
         <is>
           <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
         </is>
@@ -4039,57 +4039,57 @@
       <c r="D53" s="13" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="68" t="inlineStr"/>
-      <c r="B54" s="69" t="inlineStr">
+      <c r="A54" s="69" t="inlineStr"/>
+      <c r="B54" s="70" t="inlineStr">
         <is>
           <t>Gordon Growth</t>
         </is>
       </c>
-      <c r="C54" s="69" t="inlineStr">
+      <c r="C54" s="70" t="inlineStr">
         <is>
           <t>Exit Multiple</t>
         </is>
       </c>
-      <c r="D54" s="69" t="inlineStr">
+      <c r="D54" s="70" t="inlineStr">
         <is>
           <t>Variance</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="22" t="inlineStr">
+      <c r="A55" s="23" t="inlineStr">
         <is>
           <t>Terminal value ($)</t>
         </is>
       </c>
-      <c r="B55" s="60">
+      <c r="B55" s="61">
         <f>E32</f>
         <v/>
       </c>
-      <c r="C55" s="60">
+      <c r="C55" s="61">
         <f>E48</f>
         <v/>
       </c>
-      <c r="D55" s="60">
+      <c r="D55" s="61">
         <f>B55-C55</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="22" t="inlineStr">
+      <c r="A56" s="23" t="inlineStr">
         <is>
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
       </c>
-      <c r="B56" s="70">
+      <c r="B56" s="71">
         <f>E33</f>
         <v/>
       </c>
-      <c r="C56" s="70">
+      <c r="C56" s="71">
         <f>E47</f>
         <v/>
       </c>
-      <c r="D56" s="70">
+      <c r="D56" s="71">
         <f>B56-C56</f>
         <v/>
       </c>
@@ -4100,54 +4100,54 @@
           <t>Terminal value variance (%)</t>
         </is>
       </c>
-      <c r="B57" s="51" t="inlineStr"/>
-      <c r="C57" s="51" t="inlineStr"/>
-      <c r="D57" s="51">
+      <c r="B57" s="52" t="inlineStr"/>
+      <c r="C57" s="52" t="inlineStr"/>
+      <c r="D57" s="52">
         <f>(B55-C55)/B55</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="22" t="inlineStr">
+      <c r="A58" s="23" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="B58" s="71">
+      <c r="B58" s="72">
         <f>E40</f>
         <v/>
       </c>
-      <c r="C58" s="71">
+      <c r="C58" s="72">
         <f>E51</f>
         <v/>
       </c>
-      <c r="D58" s="71">
+      <c r="D58" s="72">
         <f>B58-C58</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="72" t="inlineStr">
+      <c r="A59" s="73" t="inlineStr">
         <is>
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B59" s="73">
+      <c r="B59" s="74">
         <f>IF(ABS(D56)&lt;=1.5,"PASS","REVIEW")</f>
         <v/>
       </c>
-      <c r="C59" s="74">
+      <c r="C59" s="75">
         <f>TEXT(D56,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
         <v/>
       </c>
-      <c r="D59" s="40" t="inlineStr">
+      <c r="D59" s="41" t="inlineStr">
         <is>
           <t>Gordon implied should bracket exit assumption</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="59" t="inlineStr">
+      <c r="A62" s="60" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
@@ -4161,7 +4161,7 @@
       <c r="H62" s="13" t="n"/>
     </row>
     <row r="63" ht="28" customHeight="1">
-      <c r="A63" s="75" t="inlineStr">
+      <c r="A63" s="76" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
@@ -4181,32 +4181,32 @@
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
       </c>
-      <c r="F63" s="76" t="n">
+      <c r="F63" s="77" t="n">
         <v>0.015</v>
       </c>
-      <c r="G63" s="76" t="n">
+      <c r="G63" s="77" t="n">
         <v>0.02</v>
       </c>
-      <c r="H63" s="76" t="n">
+      <c r="H63" s="77" t="n">
         <v>0.0225</v>
       </c>
-      <c r="I63" s="76" t="n">
+      <c r="I63" s="77" t="n">
         <v>0.025</v>
       </c>
-      <c r="J63" s="76" t="n">
+      <c r="J63" s="77" t="n">
         <v>0.03</v>
       </c>
-      <c r="L63" s="62" t="inlineStr">
+      <c r="L63" s="63" t="inlineStr">
         <is>
           <t>Scenarios: terminal g</t>
         </is>
       </c>
     </row>
     <row r="64" ht="28" customHeight="1">
-      <c r="A64" s="76" t="n">
+      <c r="A64" s="77" t="n">
         <v>0.095</v>
       </c>
-      <c r="C64" s="62" t="inlineStr">
+      <c r="C64" s="63" t="inlineStr">
         <is>
           <t>Damodaran: Historical Implied ERP</t>
         </is>
@@ -4216,34 +4216,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F64" s="77">
+      <c r="F64" s="78">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="G64" s="77">
+      <c r="G64" s="78">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="H64" s="77">
+      <c r="H64" s="78">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="I64" s="77">
+      <c r="I64" s="78">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="J64" s="77">
+      <c r="J64" s="78">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="L64" s="62" t="inlineStr">
+      <c r="L64" s="63" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="65" ht="28" customHeight="1">
-      <c r="A65" s="76" t="n">
+      <c r="A65" s="77" t="n">
         <v>0.1</v>
       </c>
       <c r="D65" s="19" t="inlineStr">
@@ -4251,34 +4251,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F65" s="77">
+      <c r="F65" s="78">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="G65" s="77">
+      <c r="G65" s="78">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="H65" s="77">
+      <c r="H65" s="78">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="I65" s="77">
+      <c r="I65" s="78">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="J65" s="77">
+      <c r="J65" s="78">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="L65" s="62" t="inlineStr">
+      <c r="L65" s="63" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="66" ht="28" customHeight="1">
-      <c r="A66" s="76" t="n">
+      <c r="A66" s="77" t="n">
         <v>0.105</v>
       </c>
       <c r="D66" s="19" t="inlineStr">
@@ -4286,34 +4286,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F66" s="77">
+      <c r="F66" s="78">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="G66" s="77">
+      <c r="G66" s="78">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="H66" s="78">
+      <c r="H66" s="79">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="I66" s="77">
+      <c r="I66" s="78">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="J66" s="77">
+      <c r="J66" s="78">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="L66" s="62" t="inlineStr">
+      <c r="L66" s="63" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="67" ht="28" customHeight="1">
-      <c r="A67" s="76" t="n">
+      <c r="A67" s="77" t="n">
         <v>0.11</v>
       </c>
       <c r="D67" s="19" t="inlineStr">
@@ -4321,34 +4321,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F67" s="77">
+      <c r="F67" s="78">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="G67" s="77">
+      <c r="G67" s="78">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="H67" s="77">
+      <c r="H67" s="78">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="I67" s="77">
+      <c r="I67" s="78">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="J67" s="77">
+      <c r="J67" s="78">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="L67" s="62" t="inlineStr">
+      <c r="L67" s="63" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="68" ht="28" customHeight="1">
-      <c r="A68" s="76" t="n">
+      <c r="A68" s="77" t="n">
         <v>0.115</v>
       </c>
       <c r="D68" s="19" t="inlineStr">
@@ -4356,27 +4356,27 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F68" s="77">
+      <c r="F68" s="78">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="G68" s="77">
+      <c r="G68" s="78">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="H68" s="77">
+      <c r="H68" s="78">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="I68" s="77">
+      <c r="I68" s="78">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="J68" s="77">
+      <c r="J68" s="78">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E36+E37)/E39</f>
         <v/>
       </c>
-      <c r="L68" s="62" t="inlineStr">
+      <c r="L68" s="63" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
@@ -4398,7 +4398,7 @@
           <t>Scenarios tab → Ctrl+F "WACC" and "Terminal growth" rows (base-case inputs)</t>
         </is>
       </c>
-      <c r="L69" s="62" t="inlineStr">
+      <c r="L69" s="63" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
@@ -4514,7 +4514,7 @@
           <t>FY2025A revenue</t>
         </is>
       </c>
-      <c r="C4" s="62" t="inlineStr">
+      <c r="C4" s="63" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -4524,7 +4524,7 @@
           <t>Ctrl+F "Net revenue" → 11,102,600 ($000) in FY2025 column</t>
         </is>
       </c>
-      <c r="E4" s="48" t="n">
+      <c r="E4" s="49" t="n">
         <v>11102600</v>
       </c>
     </row>
@@ -4534,7 +4534,7 @@
           <t>FY2025A EBITDA (EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="E5" s="49">
+      <c r="E5" s="50">
         <f>2210615+496228</f>
         <v/>
       </c>
@@ -4545,12 +4545,12 @@
           <t>FY2030E terminal EBITDA (DCF EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="C6" s="62" t="inlineStr">
+      <c r="C6" s="63" t="inlineStr">
         <is>
           <t>↳ DCF base case</t>
         </is>
       </c>
-      <c r="E6" s="49">
+      <c r="E6" s="50">
         <f>DCF!E31</f>
         <v/>
       </c>
@@ -4561,7 +4561,7 @@
           <t>FY2026E diluted EPS (guidance midpoint)</t>
         </is>
       </c>
-      <c r="C7" s="62" t="inlineStr">
+      <c r="C7" s="63" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
@@ -4571,7 +4571,7 @@
           <t>Ctrl+F "$9.48 to $9.73" → FY2026 diluted EPS guidance; model midpoint $9.61</t>
         </is>
       </c>
-      <c r="E7" s="64" t="n">
+      <c r="E7" s="65" t="n">
         <v>9.609999999999999</v>
       </c>
     </row>
@@ -4581,7 +4581,7 @@
           <t>Cash &amp; equivalents</t>
         </is>
       </c>
-      <c r="C8" s="62" t="inlineStr">
+      <c r="C8" s="63" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -4591,7 +4591,7 @@
           <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
         </is>
       </c>
-      <c r="E8" s="48" t="n">
+      <c r="E8" s="49" t="n">
         <v>1807202</v>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
           <t>Diluted shares (000)</t>
         </is>
       </c>
-      <c r="C9" s="62" t="inlineStr">
+      <c r="C9" s="63" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -4611,7 +4611,7 @@
           <t>Ctrl+F "Diluted weighted-average number of shares outstanding" → 119,068 (000)</t>
         </is>
       </c>
-      <c r="E9" s="48" t="n">
+      <c r="E9" s="49" t="n">
         <v>111380</v>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C10" s="62" t="inlineStr">
+      <c r="C10" s="63" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -4631,28 +4631,28 @@
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E10" s="64" t="n">
+      <c r="E10" s="65" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="74" t="inlineStr">
+      <c r="A11" s="75" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current EV / EBITDA</t>
         </is>
       </c>
-      <c r="E11" s="79">
+      <c r="E11" s="80">
         <f>(E10*E9-E8)/E5</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="74" t="inlineStr">
+      <c r="A12" s="75" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current P / E (FY2026E)</t>
         </is>
       </c>
-      <c r="E12" s="79">
+      <c r="E12" s="80">
         <f>E10/E7</f>
         <v/>
       </c>
@@ -4665,34 +4665,34 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="74" t="inlineStr">
+      <c r="A15" s="75" t="inlineStr">
         <is>
           <t>Peer / reference EV/EBITDA (forward / illustrative)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="80" t="inlineStr">
+      <c r="A16" s="81" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B16" s="80" t="inlineStr">
+      <c r="B16" s="81" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C16" s="80" t="inlineStr">
+      <c r="C16" s="81" t="inlineStr">
         <is>
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D16" s="80" t="inlineStr">
+      <c r="D16" s="81" t="inlineStr">
         <is>
           <t>Ctrl+F (prove number)</t>
         </is>
       </c>
-      <c r="E16" s="81" t="inlineStr">
+      <c r="E16" s="82" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
@@ -4704,12 +4704,12 @@
           <t>lululemon (LULU) — current</t>
         </is>
       </c>
-      <c r="B17" s="40" t="inlineStr">
+      <c r="B17" s="41" t="inlineStr">
         <is>
           <t>Distressed trough multiple on FY2025A EBITDA</t>
         </is>
       </c>
-      <c r="C17" s="62" t="inlineStr">
+      <c r="C17" s="63" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K</t>
         </is>
@@ -4719,7 +4719,7 @@
           <t>Ctrl+F "19.9%" → FY25 OM (EBIT $2,210,615). Ctrl+F "496,228" → Depreciation and amortization. Do not search the words Income from operations (17 hits).</t>
         </is>
       </c>
-      <c r="E17" s="82">
+      <c r="E17" s="83">
         <f>(E10*E9-E8)/E5</f>
         <v/>
       </c>
@@ -4745,7 +4745,7 @@
           <t>Ctrl+F "EV / EBITDA" → 11.97. Model uses 12.0x.</t>
         </is>
       </c>
-      <c r="E18" s="83" t="n">
+      <c r="E18" s="84" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4770,7 +4770,7 @@
           <t>Ctrl+F "EV / EBITDA" → 7.95. Model uses 8.0x.</t>
         </is>
       </c>
-      <c r="E19" s="83" t="n">
+      <c r="E19" s="84" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4795,7 +4795,7 @@
           <t>Ctrl+F "EV / EBITDA" → 14.03. Model uses 14.0x.</t>
         </is>
       </c>
-      <c r="E20" s="83" t="n">
+      <c r="E20" s="84" t="n">
         <v>14</v>
       </c>
     </row>
@@ -4820,7 +4820,7 @@
           <t>Ctrl+F "EV / EBITDA" → 9.31. Model uses 9.3x.</t>
         </is>
       </c>
-      <c r="E21" s="83" t="n">
+      <c r="E21" s="84" t="n">
         <v>9.300000000000001</v>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
           <t>Ctrl+F "EV / EBITDA" → 10.71. Model uses 10.7x.</t>
         </is>
       </c>
-      <c r="E22" s="83" t="n">
+      <c r="E22" s="84" t="n">
         <v>10.7</v>
       </c>
     </row>
@@ -4862,18 +4862,18 @@
           <t>Gordon Growth implied exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="E25" s="61">
+      <c r="E25" s="62">
         <f>DCF!E33</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="72" t="inlineStr">
+      <c r="A26" s="73" t="inlineStr">
         <is>
           <t>Selected exit multiple (base case)</t>
         </is>
       </c>
-      <c r="E26" s="70">
+      <c r="E26" s="71">
         <f>DCF!E47</f>
         <v/>
       </c>
@@ -4884,48 +4884,48 @@
           <t>Spread (selected − Gordon implied)</t>
         </is>
       </c>
-      <c r="E27" s="61">
+      <c r="E27" s="62">
         <f>E26-E25</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="72" t="inlineStr">
+      <c r="A28" s="73" t="inlineStr">
         <is>
           <t>Rationale for 8.0x</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="32" t="inlineStr">
+      <c r="A29" s="33" t="inlineStr">
         <is>
           <t>•  Mid-point of terminal football field (6.5–9.5x on FY2030E EBITDA) — 8.0x sits between bear and bull exit</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="32" t="inlineStr">
+      <c r="A30" s="33" t="inlineStr">
         <is>
           <t>•  Above Gordon-implied exit (~7x) — ~1 turn buffer vs perpetuity math on terminal FCF</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="32" t="inlineStr">
+      <c r="A31" s="33" t="inlineStr">
         <is>
           <t>•  Below premium-growth peers (ONON ~25x, DECK ~15x) — reflects Americas maturity at terminal</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="32" t="inlineStr">
+      <c r="A32" s="33" t="inlineStr">
         <is>
           <t>•  Above current LULU (~3.5x on FY2025A) — assumes partial recovery, not full re-rating to historical peaks</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="32" t="inlineStr">
+      <c r="A33" s="33" t="inlineStr">
         <is>
           <t>•  Peer simple avg ~16x not used — terminal multiple discounted for lower terminal growth vs ONON/NKE</t>
         </is>
@@ -4939,42 +4939,42 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="80" t="inlineStr">
+      <c r="A36" s="81" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B36" s="80" t="inlineStr">
+      <c r="B36" s="81" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C36" s="80" t="inlineStr">
+      <c r="C36" s="81" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D36" s="80" t="inlineStr">
+      <c r="D36" s="81" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
-      <c r="E36" s="81" t="inlineStr">
+      <c r="E36" s="82" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="F36" s="81" t="inlineStr">
+      <c r="F36" s="82" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="G36" s="81" t="inlineStr">
+      <c r="G36" s="82" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="H36" s="81" t="inlineStr">
+      <c r="H36" s="82" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
@@ -4992,7 +4992,7 @@
 Hi: 9.5x on FY2030E terminal EBITDA; bull exit above 8.0x DCF base; still below peer median ~15x.</t>
         </is>
       </c>
-      <c r="C37" s="84" t="inlineStr">
+      <c r="C37" s="85" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU EV/EBITDA
 Hi: StockAnalysis: LULU valuation</t>
@@ -5004,23 +5004,23 @@
 Hi: Ctrl+F "EV / EBITDA" → bull terminal exit assumption 9.5x on FY2030E EBITDA</t>
         </is>
       </c>
-      <c r="E37" s="83" t="n">
+      <c r="E37" s="84" t="n">
         <v>6.5</v>
       </c>
-      <c r="F37" s="83" t="n">
+      <c r="F37" s="84" t="n">
         <v>9.5</v>
       </c>
-      <c r="G37" s="85">
+      <c r="G37" s="86">
         <f>(E6*E37+E8)/E9</f>
         <v/>
       </c>
-      <c r="H37" s="85">
+      <c r="H37" s="86">
         <f>(E6*F37+E8)/E9</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="72" t="inlineStr">
+      <c r="A38" s="73" t="inlineStr">
         <is>
           <t>DCF exit method (8.0x on FY2030E EBITDA)</t>
         </is>
@@ -5040,11 +5040,11 @@
           <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x (assumption)</t>
         </is>
       </c>
-      <c r="E38" s="86">
+      <c r="E38" s="87">
         <f>DCF!E47</f>
         <v/>
       </c>
-      <c r="G38" s="87">
+      <c r="G38" s="88">
         <f>(E6*E38+E8)/E9</f>
         <v/>
       </c>
@@ -5061,7 +5061,7 @@
 Hi: 18x P/E high on FY2026E EPS; modest recovery case still below historical premium LULU multiples.</t>
         </is>
       </c>
-      <c r="C39" s="84" t="inlineStr">
+      <c r="C39" s="85" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU Forward P/E
 Hi: StockAnalysis: NKE Forward P/E</t>
@@ -5073,17 +5073,17 @@
 Hi: Ctrl+F "Forward PE" → NKE peer benchmark; high-case assumption 18.0x</t>
         </is>
       </c>
-      <c r="E39" s="83" t="n">
+      <c r="E39" s="84" t="n">
         <v>10</v>
       </c>
-      <c r="F39" s="83" t="n">
+      <c r="F39" s="84" t="n">
         <v>18</v>
       </c>
-      <c r="G39" s="85">
+      <c r="G39" s="86">
         <f>E7*E39</f>
         <v/>
       </c>
-      <c r="H39" s="85">
+      <c r="H39" s="86">
         <f>E7*F39</f>
         <v/>
       </c>
@@ -5094,32 +5094,32 @@
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="E40" s="88" t="inlineStr">
+      <c r="E40" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F40" s="88" t="inlineStr">
+      <c r="F40" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G40" s="85">
+      <c r="G40" s="86">
         <f>Scenarios!F65</f>
         <v/>
       </c>
-      <c r="H40" s="85">
+      <c r="H40" s="86">
         <f>Scenarios!H65</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="89" t="inlineStr">
+      <c r="A42" s="90" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C42" s="62" t="inlineStr">
+      <c r="C42" s="63" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -5129,12 +5129,12 @@
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E42" s="90" t="n">
+      <c r="E42" s="91" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="40" t="inlineStr">
+      <c r="A43" s="41" t="inlineStr">
         <is>
           <t>Note: peer set includes NKE, DECK, ONON, adidas, VFC; multiples are analyst ranges (red).</t>
         </is>

</xml_diff>

<commit_message>
State that we use unlevered retail beta because LULU has no debt
WACC labels, memo, justification, and the pitch now say βu = βe and not Damodaran's levered 1.09.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -397,6 +397,9 @@
     <xf numFmtId="2" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="2" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -406,6 +409,9 @@
     <xf numFmtId="2" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -427,9 +433,6 @@
     <xf numFmtId="165" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -453,9 +456,6 @@
     </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1108,7 +1108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1226,40 +1226,43 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Damodaran Retail (Special Lines) βu</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Damodaran Jan-2026 Retail (Special Lines) unlevered beta is 0.95. No funded debt, so that is our levered beta.</t>
-        </is>
-      </c>
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>Damodaran: US betas by sector (Jan 2026)</t>
+          <t>Unlevered retail beta (Damodaran Special Lines)</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>We use Damodaran’s unlevered Retail (Special Lines) beta of 0.95 because LULU has no debt.
+No debt: 0% debt weight; no outstanding term loans or bonds, so WACC effectively equals levered cost of equity here.</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>Damodaran: US betas by sector (Jan 2026)
+No debt: LULU FY2025 10-K balance sheet</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95 (column after Effective Tax rate). Do not take the levered Beta column (1.09). Date of Analysis is January 2026.</t>
-        </is>
-      </c>
-      <c r="E6" s="22" t="n">
+          <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95 (not the levered Beta 1.09). We take unlevered because LULU has no debt.
+No debt: Ctrl+F "no borrowings were outstanding under this facility" → debt weight 0%</t>
+        </is>
+      </c>
+      <c r="E6" s="23" t="n">
         <v>0.95</v>
       </c>
     </row>
-    <row r="7" ht="112" customHeight="1">
-      <c r="A7" s="23" t="inlineStr">
-        <is>
-          <t>Levered beta (industry βu; no funded debt)</t>
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Beta used = unlevered retail β — LULU has no debt</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>0.95 is Damodaran’s industry unlevered beta, not 0.86 times a 10% overlay. Links to the industry row above.</t>
+          <t>Beta used is that unlevered retail β. No funded debt → βu = βe. Do not use the levered industry 1.09.</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
@@ -1269,163 +1272,172 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Company 5Y (StockAnalysis) — not the WACC input
-  Ctrl+F "Beta (5Y)"  →  0.86
-Industry bottom-up (Damodaran, Jan 2026) — this is the 0.95
+          <t>We use the unlevered retail beta because LULU has no debt (βu = βe).
+Damodaran Jan 2026 — this is the 0.95
   Ctrl+F "Retail (Special Lines)"  →  Unlevered beta 0.95
   Do not take the levered Beta column (1.09)
-  LULU has no funded debt, so unlevered = levered</t>
-        </is>
-      </c>
-      <c r="E7" s="24">
+Why unlevered, not levered 1.09
+  Ctrl+F "no borrowings were outstanding under this facility" on the FY25 10-K
+Company 5Y (StockAnalysis) — shown, not used
+  Ctrl+F "Beta (5Y)"  →  0.86</t>
+        </is>
+      </c>
+      <c r="E7" s="25">
         <f>E6</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  memo: we use the unlevered retail beta because LULU has no debt (βu = βe). Not the levered industry 1.09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>Cost of equity = rf + β × ERP</t>
         </is>
       </c>
-      <c r="E8" s="25">
+      <c r="E9" s="27">
         <f>E3+E7*E4</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Cost of debt</t>
         </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>Pre-tax cost of debt</t>
-        </is>
-      </c>
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>5.0% illustrative pre-tax debt cost; 10-K: no borrowings outstanding on the revolver.</t>
-        </is>
-      </c>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K (no funded debt)</t>
-        </is>
-      </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "no borrowings were outstanding under this facility" on this 10-K HTML page (search the document, do not use the EDGAR viewer TOC).</t>
-        </is>
-      </c>
-      <c r="E11" s="20" t="n">
-        <v>0.05</v>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
+          <t>Pre-tax cost of debt</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>5.0% illustrative pre-tax debt cost; 10-K: no borrowings outstanding on the revolver.</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K (no funded debt)</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "no borrowings were outstanding under this facility" on this 10-K HTML page (search the document, do not use the EDGAR viewer TOC).</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>30% cash tax matches FY2026 guidance (“approximately 30%”); FY25 effective was 29.5%.</t>
         </is>
       </c>
-      <c r="C12" s="18" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>Q2 FY2026 outlook: tax rate ≈ 30%</t>
         </is>
       </c>
-      <c r="D12" s="19" t="inlineStr">
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "a tax rate of approximately 30%" on the FY2026 outlook paragraph.</t>
         </is>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E13" s="20" t="n">
         <v>0.3</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="E13" s="26">
-        <f>E11*(1-E12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="E14" s="28">
+        <f>E12*(1-E13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Capital structure (market values)</t>
         </is>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>Equity weight</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>100% equity weight; net-cash balance sheet with no material funded debt at market values per FY2025 10-K.</t>
-        </is>
-      </c>
-      <c r="C16" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K balance sheet</t>
-        </is>
-      </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) | no funded term debt</t>
-        </is>
-      </c>
-      <c r="E16" s="20" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
+          <t>Equity weight</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>100% equity weight; net-cash balance sheet with no material funded debt at market values per FY2025 10-K.</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K balance sheet</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) | no funded term debt</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
           <t>Debt weight</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>0% debt weight; no outstanding term loans or bonds, so WACC effectively equals levered cost of equity here.</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K balance sheet</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "no borrowings were outstanding under this facility" → debt weight 0%</t>
         </is>
       </c>
-      <c r="E17" s="20" t="n">
+      <c r="E18" s="20" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="23" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="E18" s="27">
-        <f>E16*E8+E17*E13</f>
+      <c r="E19" s="29">
+        <f>E17*E9+E18*E14</f>
         <v/>
       </c>
     </row>
@@ -1436,10 +1448,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1478,17 +1490,17 @@
       <c r="H1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="F2" s="28" t="inlineStr">
+      <c r="F2" s="30" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="G2" s="29" t="inlineStr">
+      <c r="G2" s="31" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="H2" s="30" t="inlineStr">
+      <c r="H2" s="32" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
@@ -1630,13 +1642,13 @@
           <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
         </is>
       </c>
-      <c r="F7" s="31" t="n">
+      <c r="F7" s="33" t="n">
         <v>134500</v>
       </c>
-      <c r="G7" s="31" t="n">
+      <c r="G7" s="33" t="n">
         <v>134500</v>
       </c>
-      <c r="H7" s="31" t="n">
+      <c r="H7" s="33" t="n">
         <v>134500</v>
       </c>
     </row>
@@ -1807,7 +1819,7 @@
 Also: FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
         </is>
       </c>
-      <c r="C13" s="32" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>LULU 10-K: 2026 capex guide $725–745M
 Also: Q2 FY2026 outlook: $10.350B–$10.500B sales</t>
@@ -1909,919 +1921,919 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="33" t="inlineStr">
+      <c r="A18" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 1</t>
         </is>
       </c>
-      <c r="F18" s="34">
+      <c r="F18" s="35">
         <f>11102600*(1+F4)</f>
         <v/>
       </c>
-      <c r="G18" s="34">
+      <c r="G18" s="35">
         <f>11102600*(1+G4)</f>
         <v/>
       </c>
-      <c r="H18" s="34">
+      <c r="H18" s="35">
         <f>11102600*(1+H4)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="33" t="inlineStr">
+      <c r="A19" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 2</t>
         </is>
       </c>
-      <c r="F19" s="34">
+      <c r="F19" s="35">
         <f>F18*(1+F5)</f>
         <v/>
       </c>
-      <c r="G19" s="34">
+      <c r="G19" s="35">
         <f>G18*(1+G5)</f>
         <v/>
       </c>
-      <c r="H19" s="34">
+      <c r="H19" s="35">
         <f>H18*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="33" t="inlineStr">
+      <c r="A20" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 3</t>
         </is>
       </c>
-      <c r="F20" s="34">
+      <c r="F20" s="35">
         <f>F19*(1+F5)</f>
         <v/>
       </c>
-      <c r="G20" s="34">
+      <c r="G20" s="35">
         <f>G19*(1+G5)</f>
         <v/>
       </c>
-      <c r="H20" s="34">
+      <c r="H20" s="35">
         <f>H19*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="33" t="inlineStr">
+      <c r="A21" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 4</t>
         </is>
       </c>
-      <c r="F21" s="34">
+      <c r="F21" s="35">
         <f>F20*(1+F5)</f>
         <v/>
       </c>
-      <c r="G21" s="34">
+      <c r="G21" s="35">
         <f>G20*(1+G5)</f>
         <v/>
       </c>
-      <c r="H21" s="34">
+      <c r="H21" s="35">
         <f>H20*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="33" t="inlineStr">
+      <c r="A22" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue – year 5</t>
         </is>
       </c>
-      <c r="F22" s="34">
+      <c r="F22" s="35">
         <f>F21*(1+F5)</f>
         <v/>
       </c>
-      <c r="G22" s="34">
+      <c r="G22" s="35">
         <f>G21*(1+G5)</f>
         <v/>
       </c>
-      <c r="H22" s="34">
+      <c r="H22" s="35">
         <f>H21*(1+H5)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="33" t="inlineStr">
+      <c r="A23" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 1</t>
         </is>
       </c>
-      <c r="F23" s="35">
+      <c r="F23" s="36">
         <f>F6+(F8-F6)*0/4</f>
         <v/>
       </c>
-      <c r="G23" s="35">
+      <c r="G23" s="36">
         <f>G6+(G8-G6)*0/4</f>
         <v/>
       </c>
-      <c r="H23" s="35">
+      <c r="H23" s="36">
         <f>H6+(H8-H6)*0/4</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="33" t="inlineStr">
+      <c r="A24" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 2</t>
         </is>
       </c>
-      <c r="F24" s="35">
+      <c r="F24" s="36">
         <f>F6+(F8-F6)*1/4</f>
         <v/>
       </c>
-      <c r="G24" s="35">
+      <c r="G24" s="36">
         <f>G6+(G8-G6)*1/4</f>
         <v/>
       </c>
-      <c r="H24" s="35">
+      <c r="H24" s="36">
         <f>H6+(H8-H6)*1/4</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="33" t="inlineStr">
+      <c r="A25" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 3</t>
         </is>
       </c>
-      <c r="F25" s="35">
+      <c r="F25" s="36">
         <f>F6+(F8-F6)*2/4</f>
         <v/>
       </c>
-      <c r="G25" s="35">
+      <c r="G25" s="36">
         <f>G6+(G8-G6)*2/4</f>
         <v/>
       </c>
-      <c r="H25" s="35">
+      <c r="H25" s="36">
         <f>H6+(H8-H6)*2/4</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="33" t="inlineStr">
+      <c r="A26" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 4</t>
         </is>
       </c>
-      <c r="F26" s="35">
+      <c r="F26" s="36">
         <f>F6+(F8-F6)*3/4</f>
         <v/>
       </c>
-      <c r="G26" s="35">
+      <c r="G26" s="36">
         <f>G6+(G8-G6)*3/4</f>
         <v/>
       </c>
-      <c r="H26" s="35">
+      <c r="H26" s="36">
         <f>H6+(H8-H6)*3/4</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="33" t="inlineStr">
+      <c r="A27" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Clean EBIT margin – year 5</t>
         </is>
       </c>
-      <c r="F27" s="35">
+      <c r="F27" s="36">
         <f>F6+(F8-F6)*4/4</f>
         <v/>
       </c>
-      <c r="G27" s="35">
+      <c r="G27" s="36">
         <f>G6+(G8-G6)*4/4</f>
         <v/>
       </c>
-      <c r="H27" s="35">
+      <c r="H27" s="36">
         <f>H6+(H8-H6)*4/4</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="33" t="inlineStr">
+      <c r="A28" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 1</t>
         </is>
       </c>
-      <c r="F28" s="34">
+      <c r="F28" s="35">
         <f>F18*F23+F7</f>
         <v/>
       </c>
-      <c r="G28" s="34">
+      <c r="G28" s="35">
         <f>G18*G23+G7</f>
         <v/>
       </c>
-      <c r="H28" s="34">
+      <c r="H28" s="35">
         <f>H18*H23+H7</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="33" t="inlineStr">
+      <c r="A29" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 2</t>
         </is>
       </c>
-      <c r="F29" s="34">
+      <c r="F29" s="35">
         <f>F19*F24</f>
         <v/>
       </c>
-      <c r="G29" s="34">
+      <c r="G29" s="35">
         <f>G19*G24</f>
         <v/>
       </c>
-      <c r="H29" s="34">
+      <c r="H29" s="35">
         <f>H19*H24</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="33" t="inlineStr">
+      <c r="A30" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 3</t>
         </is>
       </c>
-      <c r="F30" s="34">
+      <c r="F30" s="35">
         <f>F20*F25</f>
         <v/>
       </c>
-      <c r="G30" s="34">
+      <c r="G30" s="35">
         <f>G20*G25</f>
         <v/>
       </c>
-      <c r="H30" s="34">
+      <c r="H30" s="35">
         <f>H20*H25</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="33" t="inlineStr">
+      <c r="A31" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 4</t>
         </is>
       </c>
-      <c r="F31" s="34">
+      <c r="F31" s="35">
         <f>F21*F26</f>
         <v/>
       </c>
-      <c r="G31" s="34">
+      <c r="G31" s="35">
         <f>G21*G26</f>
         <v/>
       </c>
-      <c r="H31" s="34">
+      <c r="H31" s="35">
         <f>H21*H26</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="33" t="inlineStr">
+      <c r="A32" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT – year 5</t>
         </is>
       </c>
-      <c r="F32" s="34">
+      <c r="F32" s="35">
         <f>F22*F27</f>
         <v/>
       </c>
-      <c r="G32" s="34">
+      <c r="G32" s="35">
         <f>G22*G27</f>
         <v/>
       </c>
-      <c r="H32" s="34">
+      <c r="H32" s="35">
         <f>H22*H27</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="33" t="inlineStr">
+      <c r="A33" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 1</t>
         </is>
       </c>
-      <c r="F33" s="34">
+      <c r="F33" s="35">
         <f>F28*(1-F11)</f>
         <v/>
       </c>
-      <c r="G33" s="34">
+      <c r="G33" s="35">
         <f>G28*(1-G11)</f>
         <v/>
       </c>
-      <c r="H33" s="34">
+      <c r="H33" s="35">
         <f>H28*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="33" t="inlineStr">
+      <c r="A34" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 2</t>
         </is>
       </c>
-      <c r="F34" s="34">
+      <c r="F34" s="35">
         <f>F29*(1-F11)</f>
         <v/>
       </c>
-      <c r="G34" s="34">
+      <c r="G34" s="35">
         <f>G29*(1-G11)</f>
         <v/>
       </c>
-      <c r="H34" s="34">
+      <c r="H34" s="35">
         <f>H29*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="33" t="inlineStr">
+      <c r="A35" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 3</t>
         </is>
       </c>
-      <c r="F35" s="34">
+      <c r="F35" s="35">
         <f>F30*(1-F11)</f>
         <v/>
       </c>
-      <c r="G35" s="34">
+      <c r="G35" s="35">
         <f>G30*(1-G11)</f>
         <v/>
       </c>
-      <c r="H35" s="34">
+      <c r="H35" s="35">
         <f>H30*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="33" t="inlineStr">
+      <c r="A36" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 4</t>
         </is>
       </c>
-      <c r="F36" s="34">
+      <c r="F36" s="35">
         <f>F31*(1-F11)</f>
         <v/>
       </c>
-      <c r="G36" s="34">
+      <c r="G36" s="35">
         <f>G31*(1-G11)</f>
         <v/>
       </c>
-      <c r="H36" s="34">
+      <c r="H36" s="35">
         <f>H31*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="33" t="inlineStr">
+      <c r="A37" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  NOPAT – year 5</t>
         </is>
       </c>
-      <c r="F37" s="34">
+      <c r="F37" s="35">
         <f>F32*(1-F11)</f>
         <v/>
       </c>
-      <c r="G37" s="34">
+      <c r="G37" s="35">
         <f>G32*(1-G11)</f>
         <v/>
       </c>
-      <c r="H37" s="34">
+      <c r="H37" s="35">
         <f>H32*(1-H11)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="33" t="inlineStr">
+      <c r="A38" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 1</t>
         </is>
       </c>
-      <c r="F38" s="34">
+      <c r="F38" s="35">
         <f>F18*F12</f>
         <v/>
       </c>
-      <c r="G38" s="34">
+      <c r="G38" s="35">
         <f>G18*G12</f>
         <v/>
       </c>
-      <c r="H38" s="34">
+      <c r="H38" s="35">
         <f>H18*H12</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="33" t="inlineStr">
+      <c r="A39" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 2</t>
         </is>
       </c>
-      <c r="F39" s="34">
+      <c r="F39" s="35">
         <f>F19*F12</f>
         <v/>
       </c>
-      <c r="G39" s="34">
+      <c r="G39" s="35">
         <f>G19*G12</f>
         <v/>
       </c>
-      <c r="H39" s="34">
+      <c r="H39" s="35">
         <f>H19*H12</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="33" t="inlineStr">
+      <c r="A40" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 3</t>
         </is>
       </c>
-      <c r="F40" s="34">
+      <c r="F40" s="35">
         <f>F20*F12</f>
         <v/>
       </c>
-      <c r="G40" s="34">
+      <c r="G40" s="35">
         <f>G20*G12</f>
         <v/>
       </c>
-      <c r="H40" s="34">
+      <c r="H40" s="35">
         <f>H20*H12</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="33" t="inlineStr">
+      <c r="A41" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 4</t>
         </is>
       </c>
-      <c r="F41" s="34">
+      <c r="F41" s="35">
         <f>F21*F12</f>
         <v/>
       </c>
-      <c r="G41" s="34">
+      <c r="G41" s="35">
         <f>G21*G12</f>
         <v/>
       </c>
-      <c r="H41" s="34">
+      <c r="H41" s="35">
         <f>H21*H12</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="33" t="inlineStr">
+      <c r="A42" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  D&amp;A – year 5</t>
         </is>
       </c>
-      <c r="F42" s="34">
+      <c r="F42" s="35">
         <f>F22*F12</f>
         <v/>
       </c>
-      <c r="G42" s="34">
+      <c r="G42" s="35">
         <f>G22*G12</f>
         <v/>
       </c>
-      <c r="H42" s="34">
+      <c r="H42" s="35">
         <f>H22*H12</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="33" t="inlineStr">
+      <c r="A43" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 1</t>
         </is>
       </c>
-      <c r="F43" s="34">
+      <c r="F43" s="35">
         <f>F18*F13</f>
         <v/>
       </c>
-      <c r="G43" s="34">
+      <c r="G43" s="35">
         <f>G18*G13</f>
         <v/>
       </c>
-      <c r="H43" s="34">
+      <c r="H43" s="35">
         <f>H18*H13</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="33" t="inlineStr">
+      <c r="A44" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 2</t>
         </is>
       </c>
-      <c r="F44" s="34">
+      <c r="F44" s="35">
         <f>F19*F13</f>
         <v/>
       </c>
-      <c r="G44" s="34">
+      <c r="G44" s="35">
         <f>G19*G13</f>
         <v/>
       </c>
-      <c r="H44" s="34">
+      <c r="H44" s="35">
         <f>H19*H13</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="33" t="inlineStr">
+      <c r="A45" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 3</t>
         </is>
       </c>
-      <c r="F45" s="34">
+      <c r="F45" s="35">
         <f>F20*F13</f>
         <v/>
       </c>
-      <c r="G45" s="34">
+      <c r="G45" s="35">
         <f>G20*G13</f>
         <v/>
       </c>
-      <c r="H45" s="34">
+      <c r="H45" s="35">
         <f>H20*H13</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="33" t="inlineStr">
+      <c r="A46" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 4</t>
         </is>
       </c>
-      <c r="F46" s="34">
+      <c r="F46" s="35">
         <f>F21*F13</f>
         <v/>
       </c>
-      <c r="G46" s="34">
+      <c r="G46" s="35">
         <f>G21*G13</f>
         <v/>
       </c>
-      <c r="H46" s="34">
+      <c r="H46" s="35">
         <f>H21*H13</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="33" t="inlineStr">
+      <c r="A47" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Capex – year 5</t>
         </is>
       </c>
-      <c r="F47" s="34">
+      <c r="F47" s="35">
         <f>F22*F13</f>
         <v/>
       </c>
-      <c r="G47" s="34">
+      <c r="G47" s="35">
         <f>G22*G13</f>
         <v/>
       </c>
-      <c r="H47" s="34">
+      <c r="H47" s="35">
         <f>H22*H13</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="33" t="inlineStr">
+      <c r="A48" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 1</t>
         </is>
       </c>
-      <c r="F48" s="34">
+      <c r="F48" s="35">
         <f>F18*F15</f>
         <v/>
       </c>
-      <c r="G48" s="34">
+      <c r="G48" s="35">
         <f>G18*G15</f>
         <v/>
       </c>
-      <c r="H48" s="34">
+      <c r="H48" s="35">
         <f>H18*H15</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="33" t="inlineStr">
+      <c r="A49" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 2</t>
         </is>
       </c>
-      <c r="F49" s="34">
+      <c r="F49" s="35">
         <f>F19*F15</f>
         <v/>
       </c>
-      <c r="G49" s="34">
+      <c r="G49" s="35">
         <f>G19*G15</f>
         <v/>
       </c>
-      <c r="H49" s="34">
+      <c r="H49" s="35">
         <f>H19*H15</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="33" t="inlineStr">
+      <c r="A50" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 3</t>
         </is>
       </c>
-      <c r="F50" s="34">
+      <c r="F50" s="35">
         <f>F20*F15</f>
         <v/>
       </c>
-      <c r="G50" s="34">
+      <c r="G50" s="35">
         <f>G20*G15</f>
         <v/>
       </c>
-      <c r="H50" s="34">
+      <c r="H50" s="35">
         <f>H20*H15</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="33" t="inlineStr">
+      <c r="A51" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 4</t>
         </is>
       </c>
-      <c r="F51" s="34">
+      <c r="F51" s="35">
         <f>F21*F15</f>
         <v/>
       </c>
-      <c r="G51" s="34">
+      <c r="G51" s="35">
         <f>G21*G15</f>
         <v/>
       </c>
-      <c r="H51" s="34">
+      <c r="H51" s="35">
         <f>H21*H15</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="33" t="inlineStr">
+      <c r="A52" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  NWC – AR balance (inside NWC) – year 5</t>
         </is>
       </c>
-      <c r="F52" s="34">
+      <c r="F52" s="35">
         <f>F22*F15</f>
         <v/>
       </c>
-      <c r="G52" s="34">
+      <c r="G52" s="35">
         <f>G22*G15</f>
         <v/>
       </c>
-      <c r="H52" s="34">
+      <c r="H52" s="35">
         <f>H22*H15</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="33" t="inlineStr">
+      <c r="A53" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 1</t>
         </is>
       </c>
-      <c r="F53" s="34">
+      <c r="F53" s="35">
         <f>F14*(F18-11102600)</f>
         <v/>
       </c>
-      <c r="G53" s="34">
+      <c r="G53" s="35">
         <f>G14*(G18-11102600)</f>
         <v/>
       </c>
-      <c r="H53" s="34">
+      <c r="H53" s="35">
         <f>H14*(H18-11102600)</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="33" t="inlineStr">
+      <c r="A54" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 2</t>
         </is>
       </c>
-      <c r="F54" s="34">
+      <c r="F54" s="35">
         <f>F14*(F19-F18)</f>
         <v/>
       </c>
-      <c r="G54" s="34">
+      <c r="G54" s="35">
         <f>G14*(G19-G18)</f>
         <v/>
       </c>
-      <c r="H54" s="34">
+      <c r="H54" s="35">
         <f>H14*(H19-H18)</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="33" t="inlineStr">
+      <c r="A55" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 3</t>
         </is>
       </c>
-      <c r="F55" s="34">
+      <c r="F55" s="35">
         <f>F14*(F20-F19)</f>
         <v/>
       </c>
-      <c r="G55" s="34">
+      <c r="G55" s="35">
         <f>G14*(G20-G19)</f>
         <v/>
       </c>
-      <c r="H55" s="34">
+      <c r="H55" s="35">
         <f>H14*(H20-H19)</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="33" t="inlineStr">
+      <c r="A56" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 4</t>
         </is>
       </c>
-      <c r="F56" s="34">
+      <c r="F56" s="35">
         <f>F14*(F21-F20)</f>
         <v/>
       </c>
-      <c r="G56" s="34">
+      <c r="G56" s="35">
         <f>G14*(G21-G20)</f>
         <v/>
       </c>
-      <c r="H56" s="34">
+      <c r="H56" s="35">
         <f>H14*(H21-H20)</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="33" t="inlineStr">
+      <c r="A57" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  ΔNWC (includes AR) – year 5</t>
         </is>
       </c>
-      <c r="F57" s="34">
+      <c r="F57" s="35">
         <f>F14*(F22-F21)</f>
         <v/>
       </c>
-      <c r="G57" s="34">
+      <c r="G57" s="35">
         <f>G14*(G22-G21)</f>
         <v/>
       </c>
-      <c r="H57" s="34">
+      <c r="H57" s="35">
         <f>H14*(H22-H21)</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="33" t="inlineStr">
+      <c r="A58" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 1</t>
         </is>
       </c>
-      <c r="F58" s="34">
+      <c r="F58" s="35">
         <f>F33+F38-F43-F53</f>
         <v/>
       </c>
-      <c r="G58" s="34">
+      <c r="G58" s="35">
         <f>G33+G38-G43-G53</f>
         <v/>
       </c>
-      <c r="H58" s="34">
+      <c r="H58" s="35">
         <f>H33+H38-H43-H53</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="33" t="inlineStr">
+      <c r="A59" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 2</t>
         </is>
       </c>
-      <c r="F59" s="34">
+      <c r="F59" s="35">
         <f>F34+F39-F44-F54</f>
         <v/>
       </c>
-      <c r="G59" s="34">
+      <c r="G59" s="35">
         <f>G34+G39-G44-G54</f>
         <v/>
       </c>
-      <c r="H59" s="34">
+      <c r="H59" s="35">
         <f>H34+H39-H44-H54</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="33" t="inlineStr">
+      <c r="A60" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 3</t>
         </is>
       </c>
-      <c r="F60" s="34">
+      <c r="F60" s="35">
         <f>F35+F40-F45-F55</f>
         <v/>
       </c>
-      <c r="G60" s="34">
+      <c r="G60" s="35">
         <f>G35+G40-G45-G55</f>
         <v/>
       </c>
-      <c r="H60" s="34">
+      <c r="H60" s="35">
         <f>H35+H40-H45-H55</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="33" t="inlineStr">
+      <c r="A61" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 4</t>
         </is>
       </c>
-      <c r="F61" s="34">
+      <c r="F61" s="35">
         <f>F36+F41-F46-F56</f>
         <v/>
       </c>
-      <c r="G61" s="34">
+      <c r="G61" s="35">
         <f>G36+G41-G46-G56</f>
         <v/>
       </c>
-      <c r="H61" s="34">
+      <c r="H61" s="35">
         <f>H36+H41-H46-H56</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="33" t="inlineStr">
+      <c r="A62" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Unlevered FCF – year 5</t>
         </is>
       </c>
-      <c r="F62" s="34">
+      <c r="F62" s="35">
         <f>F37+F42-F47-F57</f>
         <v/>
       </c>
-      <c r="G62" s="34">
+      <c r="G62" s="35">
         <f>G37+G42-G47-G57</f>
         <v/>
       </c>
-      <c r="H62" s="34">
+      <c r="H62" s="35">
         <f>H37+H42-H47-H57</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="23" t="inlineStr">
+      <c r="A64" s="24" t="inlineStr">
         <is>
           <t>Enterprise value (DCF)</t>
         </is>
       </c>
-      <c r="F64" s="36">
+      <c r="F64" s="37">
         <f>NPV(F9,F58,F59,F60,F61,F62)+(F62*(1+F10)/(F9-F10))/(1+F9)^5</f>
         <v/>
       </c>
-      <c r="G64" s="36">
+      <c r="G64" s="37">
         <f>NPV(G9,G58,G59,G60,G61,G62)+(G62*(1+G10)/(G9-G10))/(1+G9)^5</f>
         <v/>
       </c>
-      <c r="H64" s="36">
+      <c r="H64" s="37">
         <f>NPV(H9,H58,H59,H60,H61,H62)+(H62*(1+H10)/(H9-H10))/(1+H9)^5</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="37" t="inlineStr">
+      <c r="A65" s="38" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="F65" s="38">
+      <c r="F65" s="39">
         <f>(F64+1807202-0)/111380</f>
         <v/>
       </c>
-      <c r="G65" s="39">
+      <c r="G65" s="40">
         <f>(G64+1807202-0)/111380</f>
         <v/>
       </c>
-      <c r="H65" s="38">
+      <c r="H65" s="39">
         <f>(H64+1807202-0)/111380</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="23" t="inlineStr">
+      <c r="A66" s="24" t="inlineStr">
         <is>
           <t>Upside / (downside) vs current</t>
         </is>
       </c>
-      <c r="F66" s="40">
+      <c r="F66" s="41">
         <f>F65/100.0-1</f>
         <v/>
       </c>
-      <c r="G66" s="40">
+      <c r="G66" s="41">
         <f>G65/100.0-1</f>
         <v/>
       </c>
-      <c r="H66" s="40">
+      <c r="H66" s="41">
         <f>H65/100.0-1</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="41" t="inlineStr">
+      <c r="A68" s="26" t="inlineStr">
         <is>
           <t>Current price $100.00; cash $1,807,202 k; net debt $0 (net-cash balance sheet).</t>
         </is>
@@ -2834,7 +2846,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
-    <hyperlink ref="C9" location="'WACC'!E18"/>
+    <hyperlink ref="C9" location="'WACC'!E19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
@@ -3016,7 +3028,7 @@
 Also: 2.3% FY27–30 growth matches StockAnalysis Revenue Growth Forecast (3Y) of 2.26%; next-year consensus is +2.64%.</t>
         </is>
       </c>
-      <c r="C6" s="32" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>LULU Q2 FY2026 earnings release
 Also: StockAnalysis: LULU 3Y revenue forecast</t>
@@ -3061,7 +3073,7 @@
 Also: FY30 15.5% is a partial recovery vs the FY25 10-K OM of 19.9% (unique Ctrl+F). Still well below the FY24 23.7% peak.</t>
         </is>
       </c>
-      <c r="C7" s="32" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>Q2 FY2026 release: 18.8% OM minus 560bps tariffs
 Also: FY2025 10-K: Operating margin 19.9% (one hit)</t>
@@ -3122,25 +3134,25 @@
       <c r="E8" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="31">
+      <c r="F8" s="33">
         <f>Scenarios!$G$7</f>
         <v/>
       </c>
-      <c r="G8" s="31" t="n">
+      <c r="G8" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="31" t="n">
+      <c r="H8" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="31" t="n">
+      <c r="I8" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="31" t="n">
+      <c r="J8" s="33" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>EBIT (incl. FY26 refund)</t>
         </is>
@@ -3148,23 +3160,23 @@
       <c r="E9" s="53" t="n">
         <v>2210615</v>
       </c>
-      <c r="F9" s="36">
+      <c r="F9" s="37">
         <f>Scenarios!G28</f>
         <v/>
       </c>
-      <c r="G9" s="36">
+      <c r="G9" s="37">
         <f>Scenarios!G29</f>
         <v/>
       </c>
-      <c r="H9" s="36">
+      <c r="H9" s="37">
         <f>Scenarios!G30</f>
         <v/>
       </c>
-      <c r="I9" s="36">
+      <c r="I9" s="37">
         <f>Scenarios!G31</f>
         <v/>
       </c>
-      <c r="J9" s="36">
+      <c r="J9" s="37">
         <f>Scenarios!G32</f>
         <v/>
       </c>
@@ -3231,28 +3243,28 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>NOPAT</t>
         </is>
       </c>
-      <c r="F12" s="36">
+      <c r="F12" s="37">
         <f>Scenarios!G33</f>
         <v/>
       </c>
-      <c r="G12" s="36">
+      <c r="G12" s="37">
         <f>Scenarios!G34</f>
         <v/>
       </c>
-      <c r="H12" s="36">
+      <c r="H12" s="37">
         <f>Scenarios!G35</f>
         <v/>
       </c>
-      <c r="I12" s="36">
+      <c r="I12" s="37">
         <f>Scenarios!G36</f>
         <v/>
       </c>
-      <c r="J12" s="36">
+      <c r="J12" s="37">
         <f>Scenarios!G37</f>
         <v/>
       </c>
@@ -3346,7 +3358,7 @@
 Also: FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
         </is>
       </c>
-      <c r="C15" s="32" t="inlineStr">
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>LULU 10-K: 2026 capex guide $725–745M
 Also: Q2 FY2026 outlook: $10.350B–$10.500B sales</t>
@@ -3585,14 +3597,14 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="41" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: NWC and AR are one line. 7.5% of Δsales already includes AR; UFCF does not take ΔAR separately.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="inlineStr">
+      <c r="A22" s="24" t="inlineStr">
         <is>
           <t>Unlevered free cash flow</t>
         </is>
@@ -3672,28 +3684,28 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="inlineStr">
+      <c r="A25" s="24" t="inlineStr">
         <is>
           <t>PV of unlevered FCF</t>
         </is>
       </c>
-      <c r="F25" s="36">
+      <c r="F25" s="37">
         <f>F22*F24</f>
         <v/>
       </c>
-      <c r="G25" s="36">
+      <c r="G25" s="37">
         <f>G22*G24</f>
         <v/>
       </c>
-      <c r="H25" s="36">
+      <c r="H25" s="37">
         <f>H22*H24</f>
         <v/>
       </c>
-      <c r="I25" s="36">
+      <c r="I25" s="37">
         <f>I22*I24</f>
         <v/>
       </c>
-      <c r="J25" s="36">
+      <c r="J25" s="37">
         <f>J22*J24</f>
         <v/>
       </c>
@@ -3719,7 +3731,7 @@
       <c r="C28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="inlineStr">
+      <c r="A29" s="24" t="inlineStr">
         <is>
           <t>Sum of PV of explicit FCF (FY26–FY30)</t>
         </is>
@@ -3756,12 +3768,12 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="inlineStr">
+      <c r="A31" s="24" t="inlineStr">
         <is>
           <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="E31" s="36">
+      <c r="E31" s="37">
         <f>J9+J14</f>
         <v/>
       </c>
@@ -3789,7 +3801,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="23" t="inlineStr">
+      <c r="A34" s="24" t="inlineStr">
         <is>
           <t>PV of terminal value</t>
         </is>
@@ -3800,12 +3812,12 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="23" t="inlineStr">
+      <c r="A35" s="24" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="E35" s="36">
+      <c r="E35" s="37">
         <f>E29+E34</f>
         <v/>
       </c>
@@ -3851,12 +3863,12 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="23" t="inlineStr">
+      <c r="A38" s="24" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
       </c>
-      <c r="E38" s="36">
+      <c r="E38" s="37">
         <f>E35+E36+E37</f>
         <v/>
       </c>
@@ -3882,7 +3894,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="23" t="inlineStr">
+      <c r="A40" s="24" t="inlineStr">
         <is>
           <t>Implied value per share</t>
         </is>
@@ -3917,7 +3929,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="23" t="inlineStr">
+      <c r="A42" s="24" t="inlineStr">
         <is>
           <t>Implied upside / (downside)</t>
         </is>
@@ -4007,18 +4019,18 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="23" t="inlineStr">
+      <c r="A50" s="24" t="inlineStr">
         <is>
           <t>Enterprise value (exit method)</t>
         </is>
       </c>
-      <c r="E50" s="36">
+      <c r="E50" s="37">
         <f>E29+E49</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="23" t="inlineStr">
+      <c r="A51" s="24" t="inlineStr">
         <is>
           <t>Implied value per share (exit method)</t>
         </is>
@@ -4057,7 +4069,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="23" t="inlineStr">
+      <c r="A55" s="24" t="inlineStr">
         <is>
           <t>Terminal value ($)</t>
         </is>
@@ -4076,7 +4088,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="23" t="inlineStr">
+      <c r="A56" s="24" t="inlineStr">
         <is>
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
@@ -4108,7 +4120,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="23" t="inlineStr">
+      <c r="A58" s="24" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
@@ -4140,7 +4152,7 @@
         <f>TEXT(D56,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
         <v/>
       </c>
-      <c r="D59" s="41" t="inlineStr">
+      <c r="D59" s="26" t="inlineStr">
         <is>
           <t>Gordon implied should bracket exit assumption</t>
         </is>
@@ -4439,11 +4451,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId25"/>
     <hyperlink ref="L63" location="'Scenarios'!G10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId26"/>
-    <hyperlink ref="L64" location="'WACC'!E18"/>
-    <hyperlink ref="L65" location="'WACC'!E18"/>
-    <hyperlink ref="L66" location="'WACC'!E18"/>
-    <hyperlink ref="L67" location="'WACC'!E18"/>
-    <hyperlink ref="L68" location="'WACC'!E18"/>
+    <hyperlink ref="L64" location="'WACC'!E19"/>
+    <hyperlink ref="L65" location="'WACC'!E19"/>
+    <hyperlink ref="L66" location="'WACC'!E19"/>
+    <hyperlink ref="L67" location="'WACC'!E19"/>
+    <hyperlink ref="L68" location="'WACC'!E19"/>
     <hyperlink ref="C69" location="'Scenarios'!G9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId27"/>
   </hyperlinks>
@@ -4704,7 +4716,7 @@
           <t>lululemon (LULU) — current</t>
         </is>
       </c>
-      <c r="B17" s="41" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <t>Distressed trough multiple on FY2025A EBITDA</t>
         </is>
@@ -4897,35 +4909,35 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="33" t="inlineStr">
+      <c r="A29" s="34" t="inlineStr">
         <is>
           <t>•  Mid-point of terminal football field (6.5–9.5x on FY2030E EBITDA) — 8.0x sits between bear and bull exit</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="33" t="inlineStr">
+      <c r="A30" s="34" t="inlineStr">
         <is>
           <t>•  Above Gordon-implied exit (~7x) — ~1 turn buffer vs perpetuity math on terminal FCF</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="33" t="inlineStr">
+      <c r="A31" s="34" t="inlineStr">
         <is>
           <t>•  Below premium-growth peers (ONON ~25x, DECK ~15x) — reflects Americas maturity at terminal</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="33" t="inlineStr">
+      <c r="A32" s="34" t="inlineStr">
         <is>
           <t>•  Above current LULU (~3.5x on FY2025A) — assumes partial recovery, not full re-rating to historical peaks</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="33" t="inlineStr">
+      <c r="A33" s="34" t="inlineStr">
         <is>
           <t>•  Peer simple avg ~16x not used — terminal multiple discounted for lower terminal growth vs ONON/NKE</t>
         </is>
@@ -5134,7 +5146,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="41" t="inlineStr">
+      <c r="A43" s="26" t="inlineStr">
         <is>
           <t>Note: peer set includes NKE, DECK, ONON, adidas, VFC; multiples are analyst ranges (red).</t>
         </is>

</xml_diff>

<commit_message>
Add Gymshark to comps TV build; keep 8.0x exit, not the average
Gymshark 23.5x = 2020 GA £1.25bn / FY25 EBITDA £53.3m is a private
growth print. Live AVERAGE rows show public 10.8x, mature 9.3x, and
12.9x with Gymshark so the selected 8.0x (Deckers / ~1 turn above
Gordon) is explicit rather than a blended tape.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1111,7 +1111,7 @@
   <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="B47" s="17" t="inlineStr">
         <is>
-          <t>8.0x FY2030E exit EV/EBITDA; mid-point of terminal football field (6.5–9.5x); ~1 turn above Gordon-implied ~7x.</t>
+          <t>8.0x equals Deckers; ~1 turn above Gordon ~7x. Public mean 10.8x and Gymshark 23.5x are growth prints, not FY30 exit.</t>
         </is>
       </c>
       <c r="C47" s="18" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x (assumption)</t>
+          <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x equals Deckers, not the public mean</t>
         </is>
       </c>
       <c r="E47" s="67" t="n">
@@ -4447,7 +4447,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId24"/>
-    <hyperlink ref="M47" location="'Comps'!A26"/>
+    <hyperlink ref="M47" location="'Comps'!A33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId25"/>
     <hyperlink ref="L63" location="'Scenarios'!G10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId26"/>
@@ -4469,13 +4469,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -4861,294 +4861,429 @@
         <v>10.7</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>Terminal multiple selection (DCF exit method)</t>
-        </is>
+    <row r="23" ht="150" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Gymshark (private)</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>23.5x = 1,250 / 53.3. 2020 GA EV on FY25 EBITDA; private growth print, not an FY30 exit.
+Also: FY25 EBITDA £53.3m (SGB). 62.3% is gross margin, not EBITDA. Margin ≈ 53.3 / 646 = 8.3%.</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>Guardian: Gymshark 2020 GA £1.25bn
+Also: SGB: Gymshark FY25 EBITDA £53.3m</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>Private print — do not use as FY30 exit
+  23.5x = 1,250 / 53.3
+2020 GA EV (Guardian)
+  Ctrl+F "£1.25bn valuation"
+  Ctrl+F "sold a 21% stake"
+FY25 EBITDA (SGB)
+  Ctrl+F "our EBITDA, which reached £53.3 million"
+  Do not take "62.3 percent" — that is gross margin
+  EBITDA margin ≈ 53.3 / 646 = 8.3%</t>
+        </is>
+      </c>
+      <c r="E23" s="84">
+        <f>1250/53.3</f>
+        <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>Gordon Growth implied exit EV/EBITDA</t>
-        </is>
-      </c>
-      <c r="E25" s="62">
-        <f>DCF!E33</f>
-        <v/>
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Averages (live Excel AVERAGE — shown so TV is not a blended print)</t>
+        </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="73" t="inlineStr">
-        <is>
-          <t>Selected exit multiple (base case)</t>
-        </is>
-      </c>
-      <c r="E26" s="71">
-        <f>DCF!E47</f>
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>Public 5-name mean (NKE / DECK / ONON / ADS / VFC)</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>10.8x simple mean. Too high for a 2.25% g / 15.5% OM terminal year — not the TV.</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>Derived: Excel AVERAGE of the five public prints</t>
+        </is>
+      </c>
+      <c r="D26" s="26" t="inlineStr">
+        <is>
+          <t>Math: (12.0+8.0+14.0+9.3+10.7)/5 = 10.8x. Do not use as FY30 exit.</t>
+        </is>
+      </c>
+      <c r="E26" s="83">
+        <f>AVERAGE(E18,E19,E20,E21,E22)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
+          <t>Mature public mean (DECK / ADS / VFC)</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>~9.3x closest mature set. Still haircut ~1 turn to 8.0x for 2.25% terminal g.</t>
+        </is>
+      </c>
+      <c r="C27" s="26" t="inlineStr">
+        <is>
+          <t>Derived: Excel AVERAGE of Deckers, adidas, VFC</t>
+        </is>
+      </c>
+      <c r="D27" s="26" t="inlineStr">
+        <is>
+          <t>Math: (8.0+9.3+10.7)/3 = 9.3x. Haircut to selected 8.0x.</t>
+        </is>
+      </c>
+      <c r="E27" s="83">
+        <f>AVERAGE(E19,E21,E22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>Mean incl. Gymshark (do not use for TV)</t>
+        </is>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>~12.9x. Gymshark 23.5x is a 2020 growth print; averaging it overstates FY30 exit.</t>
+        </is>
+      </c>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>Derived: Excel AVERAGE of five publics + Gymshark</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr">
+        <is>
+          <t>Math: (12.0+8.0+14.0+9.3+10.7+1,250/53.3)/6 ≈ 12.9x. Not the TV.</t>
+        </is>
+      </c>
+      <c r="E28" s="83">
+        <f>AVERAGE(E18,E19,E20,E21,E22,E23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="75" t="inlineStr">
+        <is>
+          <t>We do not average EV/EBITDA for terminal value. A 2.25% g year is not a growth-comp tape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Terminal multiple selection (DCF exit method)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>Gordon Growth implied exit EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="E32" s="62">
+        <f>DCF!E33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="73" t="inlineStr">
+        <is>
+          <t>Selected exit multiple (base case)</t>
+        </is>
+      </c>
+      <c r="E33" s="71">
+        <f>DCF!E47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
           <t>Spread (selected − Gordon implied)</t>
         </is>
       </c>
-      <c r="E27" s="62">
-        <f>E26-E25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="73" t="inlineStr">
-        <is>
-          <t>Rationale for 8.0x</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="34" t="inlineStr">
-        <is>
-          <t>•  Mid-point of terminal football field (6.5–9.5x on FY2030E EBITDA) — 8.0x sits between bear and bull exit</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="34" t="inlineStr">
-        <is>
-          <t>•  Above Gordon-implied exit (~7x) — ~1 turn buffer vs perpetuity math on terminal FCF</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="34" t="inlineStr">
-        <is>
-          <t>•  Below premium-growth peers (ONON ~25x, DECK ~15x) — reflects Americas maturity at terminal</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="34" t="inlineStr">
-        <is>
-          <t>•  Above current LULU (~3.5x on FY2025A) — assumes partial recovery, not full re-rating to historical peaks</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="34" t="inlineStr">
-        <is>
-          <t>•  Peer simple avg ~16x not used — terminal multiple discounted for lower terminal growth vs ONON/NKE</t>
-        </is>
+      <c r="E34" s="62">
+        <f>E33-E32</f>
+        <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="inlineStr">
+      <c r="A35" s="73" t="inlineStr">
+        <is>
+          <t>Rationale for 8.0x (not the average)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="34" t="inlineStr">
+        <is>
+          <t>•  8.0x equals Deckers (7.95x rounded) — closest mature premium analog on the tape</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="34" t="inlineStr">
+        <is>
+          <t>•  ~1 turn above Gordon-implied ~7x — buffer vs perpetuity math on 2.25% terminal g</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="34" t="inlineStr">
+        <is>
+          <t>•  Mid-point of the 6.5–9.5x football field — not the 10.8x public 5-name mean</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="34" t="inlineStr">
+        <is>
+          <t>•  Mature public mean (DECK / ADS / VFC) is ~9.3x; we haircut ~1 turn for 2.25% terminal g</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="34" t="inlineStr">
+        <is>
+          <t>•  Gymshark 23.5x = 1,250 / 53.3 is a 2020 private growth print; averaging it (~12.9x) is not an FY30 exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="34" t="inlineStr">
+        <is>
+          <t>•  Current LULU ~3.5x on FY2025A is a trough — 8.0x assumes partial recovery, not a re-rate to ONON 14x</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>Methodology / multiple ranges (FY2030E terminal EBITDA — football field)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="81" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="81" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B36" s="81" t="inlineStr">
+      <c r="B44" s="81" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C36" s="81" t="inlineStr">
+      <c r="C44" s="81" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D36" s="81" t="inlineStr">
+      <c r="D44" s="81" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
-      <c r="E36" s="82" t="inlineStr">
+      <c r="E44" s="82" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="F36" s="82" t="inlineStr">
+      <c r="F44" s="82" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="G36" s="82" t="inlineStr">
+      <c r="G44" s="82" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="H36" s="82" t="inlineStr">
+      <c r="H44" s="82" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="42" customHeight="1">
-      <c r="A37" s="16" t="inlineStr">
+    <row r="45" ht="42" customHeight="1">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>EV / EBITDA (FY2030E terminal)</t>
         </is>
       </c>
-      <c r="B37" s="19" t="inlineStr">
+      <c r="B45" s="19" t="inlineStr">
         <is>
           <t>Lo: 6.5x on FY2030E terminal EBITDA; bear exit below Gordon-implied ~7x; brackets DCF downside.
-Hi: 9.5x on FY2030E terminal EBITDA; bull exit above 8.0x DCF base; still below peer median ~15x.</t>
-        </is>
-      </c>
-      <c r="C37" s="85" t="inlineStr">
+Hi: 9.5x on FY2030E terminal EBITDA; bull exit above 8.0x DCF base; still below public mean ~10.8x.</t>
+        </is>
+      </c>
+      <c r="C45" s="85" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU EV/EBITDA
 Hi: StockAnalysis: LULU valuation</t>
         </is>
       </c>
-      <c r="D37" s="19" t="inlineStr">
+      <c r="D45" s="19" t="inlineStr">
         <is>
           <t>Lo: Ctrl+F "EV / EBITDA" → LULU trough ~5x; bear terminal exit assumption 6.5x
 Hi: Ctrl+F "EV / EBITDA" → bull terminal exit assumption 9.5x on FY2030E EBITDA</t>
         </is>
       </c>
-      <c r="E37" s="84" t="n">
+      <c r="E45" s="84" t="n">
         <v>6.5</v>
       </c>
-      <c r="F37" s="84" t="n">
+      <c r="F45" s="84" t="n">
         <v>9.5</v>
       </c>
-      <c r="G37" s="86">
-        <f>(E6*E37+E8)/E9</f>
-        <v/>
-      </c>
-      <c r="H37" s="86">
-        <f>(E6*F37+E8)/E9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="73" t="inlineStr">
+      <c r="G45" s="86">
+        <f>(E6*E45+E8)/E9</f>
+        <v/>
+      </c>
+      <c r="H45" s="86">
+        <f>(E6*F45+E8)/E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="28" customHeight="1">
+      <c r="A46" s="73" t="inlineStr">
         <is>
           <t>DCF exit method (8.0x on FY2030E EBITDA)</t>
         </is>
       </c>
-      <c r="B38" s="17" t="inlineStr">
-        <is>
-          <t>8.0x FY2030E exit EV/EBITDA; mid-point of terminal football field (6.5–9.5x); ~1 turn above Gordon-implied ~7x.</t>
-        </is>
-      </c>
-      <c r="C38" s="18" t="inlineStr">
+      <c r="B46" s="17" t="inlineStr">
+        <is>
+          <t>8.0x equals Deckers; ~1 turn above Gordon ~7x. Public mean 10.8x and Gymshark 23.5x are growth prints, not FY30 exit.</t>
+        </is>
+      </c>
+      <c r="C46" s="18" t="inlineStr">
         <is>
           <t>StockAnalysis: LULU EV/EBITDA</t>
         </is>
       </c>
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x (assumption)</t>
-        </is>
-      </c>
-      <c r="E38" s="87">
+      <c r="D46" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x equals Deckers, not the public mean</t>
+        </is>
+      </c>
+      <c r="E46" s="87">
         <f>DCF!E47</f>
         <v/>
       </c>
-      <c r="G38" s="88">
-        <f>(E6*E38+E8)/E9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="42" customHeight="1">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="G46" s="88">
+        <f>(E6*E46+E8)/E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="42" customHeight="1">
+      <c r="A47" s="16" t="inlineStr">
         <is>
           <t>P / E (FY2026E EPS)</t>
         </is>
       </c>
-      <c r="B39" s="19" t="inlineStr">
+      <c r="B47" s="19" t="inlineStr">
         <is>
           <t>Lo: 10x P/E low on FY2026E EPS; trough earnings multiple after guidance reset and sentiment de-rating.
 Hi: 18x P/E high on FY2026E EPS; modest recovery case still below historical premium LULU multiples.</t>
         </is>
       </c>
-      <c r="C39" s="85" t="inlineStr">
+      <c r="C47" s="85" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU Forward P/E
 Hi: StockAnalysis: NKE Forward P/E</t>
         </is>
       </c>
-      <c r="D39" s="19" t="inlineStr">
+      <c r="D47" s="19" t="inlineStr">
         <is>
           <t>Lo: Ctrl+F "Forward PE" → LULU ~12.3x; low-case multiple assumption 10.0x
 Hi: Ctrl+F "Forward PE" → NKE peer benchmark; high-case assumption 18.0x</t>
         </is>
       </c>
-      <c r="E39" s="84" t="n">
+      <c r="E47" s="84" t="n">
         <v>10</v>
       </c>
-      <c r="F39" s="84" t="n">
+      <c r="F47" s="84" t="n">
         <v>18</v>
       </c>
-      <c r="G39" s="86">
-        <f>E7*E39</f>
-        <v/>
-      </c>
-      <c r="H39" s="86">
-        <f>E7*F39</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="16" t="inlineStr">
+      <c r="G47" s="86">
+        <f>E7*E47</f>
+        <v/>
+      </c>
+      <c r="H47" s="86">
+        <f>E7*F47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
         <is>
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="E40" s="89" t="inlineStr">
+      <c r="E48" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F40" s="89" t="inlineStr">
+      <c r="F48" s="89" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G40" s="86">
+      <c r="G48" s="86">
         <f>Scenarios!F65</f>
         <v/>
       </c>
-      <c r="H40" s="86">
+      <c r="H48" s="86">
         <f>Scenarios!H65</f>
         <v/>
       </c>
     </row>
-    <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="90" t="inlineStr">
+    <row r="50" ht="28" customHeight="1">
+      <c r="A50" s="90" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C42" s="63" t="inlineStr">
+      <c r="C50" s="63" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="D42" s="19" t="inlineStr">
+      <c r="D50" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E42" s="91" t="n">
+      <c r="E50" s="91" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="26" t="inlineStr">
-        <is>
-          <t>Note: peer set includes NKE, DECK, ONON, adidas, VFC; multiples are analyst ranges (red).</t>
+    <row r="51">
+      <c r="A51" s="26" t="inlineStr">
+        <is>
+          <t>Note: public set is NKE, DECK, ONON, adidas, VFC (red). Gymshark is a private reference (23.5x = 1,250/53.3). Selected TV is 8.0x, not the average.</t>
         </is>
       </c>
     </row>
@@ -5171,11 +5306,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId17"/>
-    <hyperlink ref="C38" location="'DCF'!E47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId18"/>
+    <hyperlink ref="C46" location="'DCF'!E47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Prove Gymshark inputs, not a published EV/EBITDA
Split the private print into sourced £1.25bn valuation and £53.3m
EBITDA rows. 23.5x is now a black valuation/EBITDA formula with no
Ctrl+F claim, because neither page prints that multiple.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -20,12 +20,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0;(#,##0)"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
     <numFmt numFmtId="168" formatCode="0.0x"/>
+    <numFmt numFmtId="169" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="45">
     <font>
@@ -356,7 +357,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -582,13 +583,19 @@
     <xf numFmtId="168" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3974,7 +3981,7 @@
       </c>
       <c r="B47" s="17" t="inlineStr">
         <is>
-          <t>8.0x equals Deckers; ~1 turn above Gordon ~7x. Public mean 10.8x and Gymshark 23.5x are growth prints, not FY30 exit.</t>
+          <t>8.0x equals Deckers; ~1 turn above Gordon ~7x. Public mean 10.8x and Gymshark implied 23.5x are not FY30 exit.</t>
         </is>
       </c>
       <c r="C47" s="18" t="inlineStr">
@@ -4447,7 +4454,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId24"/>
-    <hyperlink ref="M47" location="'Comps'!A33"/>
+    <hyperlink ref="M47" location="'Comps'!A38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId25"/>
     <hyperlink ref="L63" location="'Scenarios'!G10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId26"/>
@@ -4469,7 +4476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -4861,429 +4868,483 @@
         <v>10.7</v>
       </c>
     </row>
-    <row r="23" ht="150" customHeight="1">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>Gymshark (private)</t>
-        </is>
-      </c>
-      <c r="B23" s="19" t="inlineStr">
-        <is>
-          <t>23.5x = 1,250 / 53.3. 2020 GA EV on FY25 EBITDA; private growth print, not an FY30 exit.
-Also: FY25 EBITDA £53.3m (SGB). 62.3% is gross margin, not EBITDA. Margin ≈ 53.3 / 646 = 8.3%.</t>
-        </is>
-      </c>
-      <c r="C23" s="22" t="inlineStr">
-        <is>
-          <t>Guardian: Gymshark 2020 GA £1.25bn
-Also: SGB: Gymshark FY25 EBITDA £53.3m</t>
-        </is>
-      </c>
-      <c r="D23" s="19" t="inlineStr">
-        <is>
-          <t>Private print — do not use as FY30 exit
-  23.5x = 1,250 / 53.3
-2020 GA EV (Guardian)
-  Ctrl+F "£1.25bn valuation"
-  Ctrl+F "sold a 21% stake"
-FY25 EBITDA (SGB)
-  Ctrl+F "our EBITDA, which reached £53.3 million"
-  Do not take "62.3 percent" — that is gross margin
-  EBITDA margin ≈ 53.3 / 646 = 8.3%</t>
-        </is>
-      </c>
-      <c r="E23" s="84">
-        <f>1250/53.3</f>
-        <v/>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>GYMSHARK BUILD — implied multiple (no source prints EV/EBITDA)</t>
+        </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="inlineStr">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>Column E on the next two rows is £m, not a multiple. Implied EV/EBITDA is the black formula below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>Gymshark 2020 GA valuation (£m)</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>£1.25bn = 1,250 in £m. 2020 GA headline valuation (Guardian). Not a published EV or EV/EBITDA.</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>Guardian: Gymshark 2020 GA £1.25bn</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "£1.25bn valuation" and "sold a 21% stake". That proves the 2020 valuation (£m = 1,250), not EV/EBITDA.</t>
+        </is>
+      </c>
+      <c r="E26" s="85" t="n">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>Gymshark FY25 EBITDA (£m)</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>FY25 EBITDA is £53.3m (SGB). 62.3% is gross margin. This cell is EBITDA £m, not a multiple.</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>SGB: Gymshark FY25 EBITDA £53.3m</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "our EBITDA, which reached £53.3 million". That proves FY25 EBITDA £m. Do not take "62.3 percent" (gross margin).</t>
+        </is>
+      </c>
+      <c r="E27" s="86" t="n">
+        <v>53.3</v>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="73" t="inlineStr">
+        <is>
+          <t>Gymshark implied EV/EBITDA (model math)</t>
+        </is>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>No page prints Gymshark EV/EBITDA. Black formula = 2020 valuation / FY25 EBITDA. Cross-year; not the TV.</t>
+        </is>
+      </c>
+      <c r="C28" s="63" t="inlineStr">
+        <is>
+          <t>Comps: Gymshark valuation / EBITDA</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>No Ctrl+F. Neither Guardian nor SGB prints EV/EBITDA. This cell is E26 / E27 (2020 valuation ÷ FY25 EBITDA).</t>
+        </is>
+      </c>
+      <c r="E28" s="87">
+        <f>E26/E27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>Averages (live Excel AVERAGE — shown so TV is not a blended print)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>Public 5-name mean (NKE / DECK / ONON / ADS / VFC)</t>
         </is>
       </c>
-      <c r="B26" s="26" t="inlineStr">
+      <c r="B31" s="26" t="inlineStr">
         <is>
           <t>10.8x simple mean. Too high for a 2.25% g / 15.5% OM terminal year — not the TV.</t>
         </is>
       </c>
-      <c r="C26" s="26" t="inlineStr">
+      <c r="C31" s="26" t="inlineStr">
         <is>
           <t>Derived: Excel AVERAGE of the five public prints</t>
         </is>
       </c>
-      <c r="D26" s="26" t="inlineStr">
+      <c r="D31" s="26" t="inlineStr">
         <is>
           <t>Math: (12.0+8.0+14.0+9.3+10.7)/5 = 10.8x. Do not use as FY30 exit.</t>
         </is>
       </c>
-      <c r="E26" s="83">
+      <c r="E31" s="83">
         <f>AVERAGE(E18,E19,E20,E21,E22)</f>
         <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t>Mature public mean (DECK / ADS / VFC)</t>
-        </is>
-      </c>
-      <c r="B27" s="26" t="inlineStr">
-        <is>
-          <t>~9.3x closest mature set. Still haircut ~1 turn to 8.0x for 2.25% terminal g.</t>
-        </is>
-      </c>
-      <c r="C27" s="26" t="inlineStr">
-        <is>
-          <t>Derived: Excel AVERAGE of Deckers, adidas, VFC</t>
-        </is>
-      </c>
-      <c r="D27" s="26" t="inlineStr">
-        <is>
-          <t>Math: (8.0+9.3+10.7)/3 = 9.3x. Haircut to selected 8.0x.</t>
-        </is>
-      </c>
-      <c r="E27" s="83">
-        <f>AVERAGE(E19,E21,E22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>Mean incl. Gymshark (do not use for TV)</t>
-        </is>
-      </c>
-      <c r="B28" s="26" t="inlineStr">
-        <is>
-          <t>~12.9x. Gymshark 23.5x is a 2020 growth print; averaging it overstates FY30 exit.</t>
-        </is>
-      </c>
-      <c r="C28" s="26" t="inlineStr">
-        <is>
-          <t>Derived: Excel AVERAGE of five publics + Gymshark</t>
-        </is>
-      </c>
-      <c r="D28" s="26" t="inlineStr">
-        <is>
-          <t>Math: (12.0+8.0+14.0+9.3+10.7+1,250/53.3)/6 ≈ 12.9x. Not the TV.</t>
-        </is>
-      </c>
-      <c r="E28" s="83">
-        <f>AVERAGE(E18,E19,E20,E21,E22,E23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="75" t="inlineStr">
-        <is>
-          <t>We do not average EV/EBITDA for terminal value. A 2.25% g year is not a growth-comp tape.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="14" t="inlineStr">
-        <is>
-          <t>Terminal multiple selection (DCF exit method)</t>
-        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
         <is>
+          <t>Mature public mean (DECK / ADS / VFC)</t>
+        </is>
+      </c>
+      <c r="B32" s="26" t="inlineStr">
+        <is>
+          <t>~9.3x closest mature set. Still haircut ~1 turn to 8.0x for 2.25% terminal g.</t>
+        </is>
+      </c>
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>Derived: Excel AVERAGE of Deckers, adidas, VFC</t>
+        </is>
+      </c>
+      <c r="D32" s="26" t="inlineStr">
+        <is>
+          <t>Math: (8.0+9.3+10.7)/3 = 9.3x. Haircut to selected 8.0x.</t>
+        </is>
+      </c>
+      <c r="E32" s="83">
+        <f>AVERAGE(E19,E21,E22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>Mean incl. Gymshark (do not use for TV)</t>
+        </is>
+      </c>
+      <c r="B33" s="26" t="inlineStr">
+        <is>
+          <t>~12.9x. Gymshark implied 23.5x is model math (2020 val / FY25 EBITDA); averaging it overstates FY30 exit.</t>
+        </is>
+      </c>
+      <c r="C33" s="26" t="inlineStr">
+        <is>
+          <t>Derived: Excel AVERAGE of five publics + Gymshark</t>
+        </is>
+      </c>
+      <c r="D33" s="26" t="inlineStr">
+        <is>
+          <t>Math: (12.0+8.0+14.0+9.3+10.7+1,250/53.3)/6 ≈ 12.9x. Not the TV.</t>
+        </is>
+      </c>
+      <c r="E33" s="83">
+        <f>AVERAGE(E18,E19,E20,E21,E22,E28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="75" t="inlineStr">
+        <is>
+          <t>We do not average EV/EBITDA for terminal value. A 2.25% g year is not a growth-comp tape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>Terminal multiple selection (DCF exit method)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
           <t>Gordon Growth implied exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="E32" s="62">
+      <c r="E37" s="62">
         <f>DCF!E33</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="73" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="73" t="inlineStr">
         <is>
           <t>Selected exit multiple (base case)</t>
         </is>
       </c>
-      <c r="E33" s="71">
+      <c r="E38" s="71">
         <f>DCF!E47</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
         <is>
           <t>Spread (selected − Gordon implied)</t>
         </is>
       </c>
-      <c r="E34" s="62">
-        <f>E33-E32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="73" t="inlineStr">
+      <c r="E39" s="62">
+        <f>E38-E37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="73" t="inlineStr">
         <is>
           <t>Rationale for 8.0x (not the average)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="34" t="inlineStr">
-        <is>
-          <t>•  8.0x equals Deckers (7.95x rounded) — closest mature premium analog on the tape</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="34" t="inlineStr">
-        <is>
-          <t>•  ~1 turn above Gordon-implied ~7x — buffer vs perpetuity math on 2.25% terminal g</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="34" t="inlineStr">
-        <is>
-          <t>•  Mid-point of the 6.5–9.5x football field — not the 10.8x public 5-name mean</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="34" t="inlineStr">
-        <is>
-          <t>•  Mature public mean (DECK / ADS / VFC) is ~9.3x; we haircut ~1 turn for 2.25% terminal g</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="34" t="inlineStr">
-        <is>
-          <t>•  Gymshark 23.5x = 1,250 / 53.3 is a 2020 private growth print; averaging it (~12.9x) is not an FY30 exit</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="34" t="inlineStr">
         <is>
+          <t>•  8.0x equals Deckers (7.95x rounded) — closest mature premium analog on the tape</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="34" t="inlineStr">
+        <is>
+          <t>•  ~1 turn above Gordon-implied ~7x — buffer vs perpetuity math on 2.25% terminal g</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="34" t="inlineStr">
+        <is>
+          <t>•  Mid-point of the 6.5–9.5x football field — not the 10.8x public 5-name mean</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="34" t="inlineStr">
+        <is>
+          <t>•  Mature public mean (DECK / ADS / VFC) is ~9.3x; we haircut ~1 turn for 2.25% terminal g</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="34" t="inlineStr">
+        <is>
+          <t>•  Gymshark implied 23.5x is 2020 valuation / FY25 EBITDA — no page prints that multiple; averaging it (~12.9x) is not an FY30 exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="34" t="inlineStr">
+        <is>
           <t>•  Current LULU ~3.5x on FY2025A is a trough — 8.0x assumes partial recovery, not a re-rate to ONON 14x</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="14" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="14" t="inlineStr">
         <is>
           <t>Methodology / multiple ranges (FY2030E terminal EBITDA — football field)</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="81" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="81" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B44" s="81" t="inlineStr">
+      <c r="B49" s="81" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C44" s="81" t="inlineStr">
+      <c r="C49" s="81" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D44" s="81" t="inlineStr">
+      <c r="D49" s="81" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
-      <c r="E44" s="82" t="inlineStr">
+      <c r="E49" s="82" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="F44" s="82" t="inlineStr">
+      <c r="F49" s="82" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="G44" s="82" t="inlineStr">
+      <c r="G49" s="82" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="H44" s="82" t="inlineStr">
+      <c r="H49" s="82" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="42" customHeight="1">
-      <c r="A45" s="16" t="inlineStr">
+    <row r="50" ht="42" customHeight="1">
+      <c r="A50" s="16" t="inlineStr">
         <is>
           <t>EV / EBITDA (FY2030E terminal)</t>
         </is>
       </c>
-      <c r="B45" s="19" t="inlineStr">
+      <c r="B50" s="19" t="inlineStr">
         <is>
           <t>Lo: 6.5x on FY2030E terminal EBITDA; bear exit below Gordon-implied ~7x; brackets DCF downside.
 Hi: 9.5x on FY2030E terminal EBITDA; bull exit above 8.0x DCF base; still below public mean ~10.8x.</t>
         </is>
       </c>
-      <c r="C45" s="85" t="inlineStr">
+      <c r="C50" s="88" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU EV/EBITDA
 Hi: StockAnalysis: LULU valuation</t>
         </is>
       </c>
-      <c r="D45" s="19" t="inlineStr">
+      <c r="D50" s="19" t="inlineStr">
         <is>
           <t>Lo: Ctrl+F "EV / EBITDA" → LULU trough ~5x; bear terminal exit assumption 6.5x
 Hi: Ctrl+F "EV / EBITDA" → bull terminal exit assumption 9.5x on FY2030E EBITDA</t>
         </is>
       </c>
-      <c r="E45" s="84" t="n">
+      <c r="E50" s="84" t="n">
         <v>6.5</v>
       </c>
-      <c r="F45" s="84" t="n">
+      <c r="F50" s="84" t="n">
         <v>9.5</v>
       </c>
-      <c r="G45" s="86">
-        <f>(E6*E45+E8)/E9</f>
-        <v/>
-      </c>
-      <c r="H45" s="86">
-        <f>(E6*F45+E8)/E9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" ht="28" customHeight="1">
-      <c r="A46" s="73" t="inlineStr">
+      <c r="G50" s="89">
+        <f>(E6*E50+E8)/E9</f>
+        <v/>
+      </c>
+      <c r="H50" s="89">
+        <f>(E6*F50+E8)/E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="73" t="inlineStr">
         <is>
           <t>DCF exit method (8.0x on FY2030E EBITDA)</t>
         </is>
       </c>
-      <c r="B46" s="17" t="inlineStr">
-        <is>
-          <t>8.0x equals Deckers; ~1 turn above Gordon ~7x. Public mean 10.8x and Gymshark 23.5x are growth prints, not FY30 exit.</t>
-        </is>
-      </c>
-      <c r="C46" s="18" t="inlineStr">
+      <c r="B51" s="17" t="inlineStr">
+        <is>
+          <t>8.0x equals Deckers; ~1 turn above Gordon ~7x. Public mean 10.8x and Gymshark implied 23.5x are not FY30 exit.</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
         <is>
           <t>StockAnalysis: LULU EV/EBITDA</t>
         </is>
       </c>
-      <c r="D46" s="19" t="inlineStr">
+      <c r="D51" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x equals Deckers, not the public mean</t>
         </is>
       </c>
-      <c r="E46" s="87">
+      <c r="E51" s="87">
         <f>DCF!E47</f>
         <v/>
       </c>
-      <c r="G46" s="88">
-        <f>(E6*E46+E8)/E9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" ht="42" customHeight="1">
-      <c r="A47" s="16" t="inlineStr">
+      <c r="G51" s="90">
+        <f>(E6*E51+E8)/E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="42" customHeight="1">
+      <c r="A52" s="16" t="inlineStr">
         <is>
           <t>P / E (FY2026E EPS)</t>
         </is>
       </c>
-      <c r="B47" s="19" t="inlineStr">
+      <c r="B52" s="19" t="inlineStr">
         <is>
           <t>Lo: 10x P/E low on FY2026E EPS; trough earnings multiple after guidance reset and sentiment de-rating.
 Hi: 18x P/E high on FY2026E EPS; modest recovery case still below historical premium LULU multiples.</t>
         </is>
       </c>
-      <c r="C47" s="85" t="inlineStr">
+      <c r="C52" s="88" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU Forward P/E
 Hi: StockAnalysis: NKE Forward P/E</t>
         </is>
       </c>
-      <c r="D47" s="19" t="inlineStr">
+      <c r="D52" s="19" t="inlineStr">
         <is>
           <t>Lo: Ctrl+F "Forward PE" → LULU ~12.3x; low-case multiple assumption 10.0x
 Hi: Ctrl+F "Forward PE" → NKE peer benchmark; high-case assumption 18.0x</t>
         </is>
       </c>
-      <c r="E47" s="84" t="n">
+      <c r="E52" s="84" t="n">
         <v>10</v>
       </c>
-      <c r="F47" s="84" t="n">
+      <c r="F52" s="84" t="n">
         <v>18</v>
       </c>
-      <c r="G47" s="86">
-        <f>E7*E47</f>
-        <v/>
-      </c>
-      <c r="H47" s="86">
-        <f>E7*F47</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="16" t="inlineStr">
+      <c r="G52" s="89">
+        <f>E7*E52</f>
+        <v/>
+      </c>
+      <c r="H52" s="89">
+        <f>E7*F52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
         <is>
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="E48" s="89" t="inlineStr">
+      <c r="E53" s="91" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F48" s="89" t="inlineStr">
+      <c r="F53" s="91" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G48" s="86">
+      <c r="G53" s="89">
         <f>Scenarios!F65</f>
         <v/>
       </c>
-      <c r="H48" s="86">
+      <c r="H53" s="89">
         <f>Scenarios!H65</f>
         <v/>
       </c>
     </row>
-    <row r="50" ht="28" customHeight="1">
-      <c r="A50" s="90" t="inlineStr">
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="92" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C50" s="63" t="inlineStr">
+      <c r="C55" s="63" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="D50" s="19" t="inlineStr">
+      <c r="D55" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E50" s="91" t="n">
+      <c r="E55" s="93" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="26" t="inlineStr">
-        <is>
-          <t>Note: public set is NKE, DECK, ONON, adidas, VFC (red). Gymshark is a private reference (23.5x = 1,250/53.3). Selected TV is 8.0x, not the average.</t>
+    <row r="56">
+      <c r="A56" s="26" t="inlineStr">
+        <is>
+          <t>Note: public set is NKE, DECK, ONON, adidas, VFC (red). Gymshark 23.5x is implied (2020 £1.25bn / FY25 £53.3m) — no source prints EV/EBITDA. Selected TV is 8.0x, not the average.</t>
         </is>
       </c>
     </row>
@@ -5306,12 +5367,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId18"/>
-    <hyperlink ref="C46" location="'DCF'!E47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId20"/>
+    <hyperlink ref="C28" location="'Comps'!E26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId21"/>
+    <hyperlink ref="C51" location="'DCF'!E47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Derive the FY30 exit from the Gordon identity, not Deckers
8.0x was a typed judgment that happened to match Deckers. Selected
exit is now the live formula TV / FY30 EBITDA, which equals
(UFCF/EBITDA)×(1+g)/(WACC−g) (~6.0x at base). Comps stay a check,
not the derivation.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -357,7 +357,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -529,9 +529,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2871,7 +2868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M69"/>
+  <dimension ref="A1:M70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -3799,7 +3796,7 @@
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Implied exit EV/EBITDA (Gordon Growth)</t>
+          <t xml:space="preserve">  Implied exit EV/EBITDA = Gordon TV / FY30 EBITDA</t>
         </is>
       </c>
       <c r="E33" s="62">
@@ -3808,621 +3805,633 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="24" t="inlineStr">
-        <is>
-          <t>PV of terminal value</t>
-        </is>
-      </c>
-      <c r="E34" s="61">
-        <f>E32/(1+Scenarios!$G$9)^J23</f>
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  memo: (UFCF₃₀ / EBITDA₃₀) × (1+g) / (WACC−g)</t>
+        </is>
+      </c>
+      <c r="E34" s="62">
+        <f>J22/E31*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
+          <t>PV of terminal value</t>
+        </is>
+      </c>
+      <c r="E35" s="61">
+        <f>E32/(1+Scenarios!$G$9)^J23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="E35" s="37">
-        <f>E29+E34</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="16" t="inlineStr">
-        <is>
-          <t>Plus: cash &amp; equivalents (FY2025)</t>
-        </is>
-      </c>
-      <c r="C36" s="63" t="inlineStr">
-        <is>
-          <t>10-K</t>
-        </is>
-      </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
-        </is>
-      </c>
-      <c r="E36" s="49" t="n">
-        <v>1807202</v>
+      <c r="E36" s="37">
+        <f>E29+E35</f>
+        <v/>
       </c>
     </row>
     <row r="37" ht="28" customHeight="1">
       <c r="A37" s="16" t="inlineStr">
         <is>
+          <t>Plus: cash &amp; equivalents (FY2025)</t>
+        </is>
+      </c>
+      <c r="C37" s="63" t="inlineStr">
+        <is>
+          <t>10-K</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
+        </is>
+      </c>
+      <c r="E37" s="49" t="n">
+        <v>1807202</v>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
           <t>Less: total debt</t>
         </is>
       </c>
-      <c r="C37" s="63" t="inlineStr">
+      <c r="C38" s="63" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="D37" s="19" t="inlineStr">
+      <c r="D38" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "no borrowings were outstanding under this facility" → no funded term debt</t>
         </is>
       </c>
-      <c r="E37" s="49" t="n">
+      <c r="E38" s="49" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="24" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="24" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
       </c>
-      <c r="E38" s="37">
-        <f>E35+E36+E37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="28" customHeight="1">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="E39" s="37">
+        <f>E36+E37+E38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>Diluted shares outstanding (000)</t>
         </is>
       </c>
-      <c r="C39" s="63" t="inlineStr">
+      <c r="C40" s="63" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="D39" s="19" t="inlineStr">
+      <c r="D40" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Diluted weighted-average number of shares outstanding" → 119,068 (000)</t>
         </is>
       </c>
-      <c r="E39" s="49" t="n">
+      <c r="E40" s="49" t="n">
         <v>111380</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="24" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="24" t="inlineStr">
         <is>
           <t>Implied value per share</t>
         </is>
       </c>
-      <c r="E40" s="64">
-        <f>E38/E39</f>
-        <v/>
-      </c>
-      <c r="K40" s="54">
-        <f>IF(ABS(E40-Scenarios!$G$65)&lt;0.05,"OK","CHECK")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="E41" s="64">
+        <f>E39/E40</f>
+        <v/>
+      </c>
+      <c r="K41" s="54">
+        <f>IF(ABS(E41-Scenarios!$G$65)&lt;0.05,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="16" t="inlineStr">
         <is>
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C41" s="63" t="inlineStr">
+      <c r="C42" s="63" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="D41" s="19" t="inlineStr">
+      <c r="D42" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E41" s="65" t="n">
+      <c r="E42" s="65" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="24" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="24" t="inlineStr">
         <is>
           <t>Implied upside / (downside)</t>
         </is>
       </c>
-      <c r="E42" s="66">
-        <f>E40/E41-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="16" t="inlineStr">
+      <c r="E43" s="66">
+        <f>E41/E42-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: % of EV from terminal value</t>
         </is>
       </c>
-      <c r="E43" s="52">
-        <f>E34/E35</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="60" t="inlineStr">
+      <c r="E44" s="52">
+        <f>E35/E36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="60" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
       </c>
-      <c r="B45" s="13" t="n"/>
-      <c r="C45" s="13" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="15" t="inlineStr">
-        <is>
-          <t>Exit multiple selection (see Comps tab for peer build)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="28" customHeight="1">
-      <c r="A47" s="16" t="inlineStr">
-        <is>
-          <t>Selected exit EV/EBITDA multiple (FY2030E)</t>
-        </is>
-      </c>
-      <c r="B47" s="17" t="inlineStr">
-        <is>
-          <t>8.0x equals Deckers; ~1 turn above Gordon ~7x. Public mean 10.8x and Gymshark implied 23.5x are not FY30 exit.</t>
-        </is>
-      </c>
-      <c r="C47" s="18" t="inlineStr">
-        <is>
-          <t>StockAnalysis: LULU EV/EBITDA</t>
-        </is>
-      </c>
-      <c r="D47" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x equals Deckers, not the public mean</t>
-        </is>
-      </c>
-      <c r="E47" s="67" t="n">
-        <v>8</v>
-      </c>
-      <c r="M47" s="63" t="inlineStr">
+      <c r="B46" s="13" t="n"/>
+      <c r="C46" s="13" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>Exit multiple is the Gordon identity — not a peer pick or an average</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>Selected exit EV/EBITDA (Gordon implied)</t>
+        </is>
+      </c>
+      <c r="B48" s="17" t="inlineStr">
+        <is>
+          <t>Selected exit is Gordon TV / FY30 EBITDA. Identity: (UFCF/EBITDA)×(1+g)/(WACC−g). Not Deckers and not a peer average.</t>
+        </is>
+      </c>
+      <c r="C48" s="18" t="inlineStr">
+        <is>
+          <t>DCF: Gordon implied exit (TV / FY30 EBITDA)</t>
+        </is>
+      </c>
+      <c r="D48" s="19" t="inlineStr">
+        <is>
+          <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
+        </is>
+      </c>
+      <c r="E48" s="62">
+        <f>E33</f>
+        <v/>
+      </c>
+      <c r="M48" s="63" t="inlineStr">
         <is>
           <t>Comps: Exit Multiple Build</t>
         </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="16" t="inlineStr">
-        <is>
-          <t>Terminal value = Terminal EBITDA × exit multiple</t>
-        </is>
-      </c>
-      <c r="E48" s="50">
-        <f>E31*E47</f>
-        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
         <is>
+          <t>Terminal value = Terminal EBITDA × exit multiple</t>
+        </is>
+      </c>
+      <c r="E49" s="50">
+        <f>E31*E48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="E49" s="50">
-        <f>E48/(1+Scenarios!$G$9)^J23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="24" t="inlineStr">
-        <is>
-          <t>Enterprise value (exit method)</t>
-        </is>
-      </c>
-      <c r="E50" s="37">
-        <f>E29+E49</f>
+      <c r="E50" s="50">
+        <f>E49/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="24" t="inlineStr">
         <is>
+          <t>Enterprise value (exit method)</t>
+        </is>
+      </c>
+      <c r="E51" s="37">
+        <f>E29+E50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="24" t="inlineStr">
+        <is>
           <t>Implied value per share (exit method)</t>
         </is>
       </c>
-      <c r="E51" s="68">
-        <f>(E50+E36+E37)/E39</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="60" t="inlineStr">
+      <c r="E52" s="67">
+        <f>(E51+E37+E38)/E40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="60" t="inlineStr">
         <is>
           <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
         </is>
       </c>
-      <c r="B53" s="13" t="n"/>
-      <c r="C53" s="13" t="n"/>
-      <c r="D53" s="13" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="69" t="inlineStr"/>
-      <c r="B54" s="70" t="inlineStr">
+      <c r="B54" s="13" t="n"/>
+      <c r="C54" s="13" t="n"/>
+      <c r="D54" s="13" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="68" t="inlineStr"/>
+      <c r="B55" s="69" t="inlineStr">
         <is>
           <t>Gordon Growth</t>
         </is>
       </c>
-      <c r="C54" s="70" t="inlineStr">
+      <c r="C55" s="69" t="inlineStr">
         <is>
           <t>Exit Multiple</t>
         </is>
       </c>
-      <c r="D54" s="70" t="inlineStr">
+      <c r="D55" s="69" t="inlineStr">
         <is>
           <t>Variance</t>
         </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="24" t="inlineStr">
-        <is>
-          <t>Terminal value ($)</t>
-        </is>
-      </c>
-      <c r="B55" s="61">
-        <f>E32</f>
-        <v/>
-      </c>
-      <c r="C55" s="61">
-        <f>E48</f>
-        <v/>
-      </c>
-      <c r="D55" s="61">
-        <f>B55-C55</f>
-        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="24" t="inlineStr">
         <is>
+          <t>Terminal value ($)</t>
+        </is>
+      </c>
+      <c r="B56" s="61">
+        <f>E32</f>
+        <v/>
+      </c>
+      <c r="C56" s="61">
+        <f>E49</f>
+        <v/>
+      </c>
+      <c r="D56" s="61">
+        <f>B56-C56</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="24" t="inlineStr">
+        <is>
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
       </c>
-      <c r="B56" s="71">
+      <c r="B57" s="70">
         <f>E33</f>
         <v/>
       </c>
-      <c r="C56" s="71">
-        <f>E47</f>
-        <v/>
-      </c>
-      <c r="D56" s="71">
-        <f>B56-C56</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="16" t="inlineStr">
+      <c r="C57" s="70">
+        <f>E48</f>
+        <v/>
+      </c>
+      <c r="D57" s="70">
+        <f>B57-C57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="inlineStr">
         <is>
           <t>Terminal value variance (%)</t>
         </is>
       </c>
-      <c r="B57" s="52" t="inlineStr"/>
-      <c r="C57" s="52" t="inlineStr"/>
-      <c r="D57" s="52">
-        <f>(B55-C55)/B55</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="24" t="inlineStr">
+      <c r="B58" s="52" t="inlineStr"/>
+      <c r="C58" s="52" t="inlineStr"/>
+      <c r="D58" s="52">
+        <f>(B56-C56)/B56</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="24" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="B58" s="72">
-        <f>E40</f>
-        <v/>
-      </c>
-      <c r="C58" s="72">
-        <f>E51</f>
-        <v/>
-      </c>
-      <c r="D58" s="72">
-        <f>B58-C58</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="73" t="inlineStr">
+      <c r="B59" s="71">
+        <f>E41</f>
+        <v/>
+      </c>
+      <c r="C59" s="71">
+        <f>E52</f>
+        <v/>
+      </c>
+      <c r="D59" s="71">
+        <f>B59-C59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="72" t="inlineStr">
         <is>
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B59" s="74">
-        <f>IF(ABS(D56)&lt;=1.5,"PASS","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="C59" s="75">
-        <f>TEXT(D56,"0.0")&amp;"x spread vs 8.0x exit multiple"</f>
-        <v/>
-      </c>
-      <c r="D59" s="26" t="inlineStr">
-        <is>
-          <t>Gordon implied should bracket exit assumption</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="60" t="inlineStr">
+      <c r="B60" s="73">
+        <f>IF(ABS(D57)&lt;=1.5,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="C60" s="74">
+        <f>TEXT(D57,"0.0")&amp;"x spread vs Gordon-implied exit"</f>
+        <v/>
+      </c>
+      <c r="D60" s="26" t="inlineStr">
+        <is>
+          <t>Selected exit is the Gordon identity, so spread should be 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="60" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
       </c>
-      <c r="B62" s="13" t="n"/>
-      <c r="C62" s="13" t="n"/>
-      <c r="D62" s="13" t="n"/>
-      <c r="E62" s="13" t="n"/>
-      <c r="F62" s="13" t="n"/>
-      <c r="G62" s="13" t="n"/>
-      <c r="H62" s="13" t="n"/>
-    </row>
-    <row r="63" ht="28" customHeight="1">
-      <c r="A63" s="76" t="inlineStr">
+      <c r="B63" s="13" t="n"/>
+      <c r="C63" s="13" t="n"/>
+      <c r="D63" s="13" t="n"/>
+      <c r="E63" s="13" t="n"/>
+      <c r="F63" s="13" t="n"/>
+      <c r="G63" s="13" t="n"/>
+      <c r="H63" s="13" t="n"/>
+    </row>
+    <row r="64" ht="28" customHeight="1">
+      <c r="A64" s="75" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
       </c>
-      <c r="B63" s="17" t="inlineStr">
+      <c r="B64" s="17" t="inlineStr">
         <is>
           <t>Terminal-g axis 1.5–3.0% brackets 2.25% base; bounded by long-run real GDP and inflation benchmarks.</t>
         </is>
       </c>
-      <c r="C63" s="18" t="inlineStr">
+      <c r="C64" s="18" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="D63" s="19" t="inlineStr">
+      <c r="D64" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
       </c>
-      <c r="F63" s="77" t="n">
+      <c r="F64" s="76" t="n">
         <v>0.015</v>
       </c>
-      <c r="G63" s="77" t="n">
+      <c r="G64" s="76" t="n">
         <v>0.02</v>
       </c>
-      <c r="H63" s="77" t="n">
+      <c r="H64" s="76" t="n">
         <v>0.0225</v>
       </c>
-      <c r="I63" s="77" t="n">
+      <c r="I64" s="76" t="n">
         <v>0.025</v>
       </c>
-      <c r="J63" s="77" t="n">
+      <c r="J64" s="76" t="n">
         <v>0.03</v>
       </c>
-      <c r="L63" s="63" t="inlineStr">
+      <c r="L64" s="63" t="inlineStr">
         <is>
           <t>Scenarios: terminal g</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="28" customHeight="1">
-      <c r="A64" s="77" t="n">
+    <row r="65" ht="28" customHeight="1">
+      <c r="A65" s="76" t="n">
         <v>0.095</v>
       </c>
-      <c r="C64" s="63" t="inlineStr">
+      <c r="C65" s="63" t="inlineStr">
         <is>
           <t>Damodaran: Historical Implied ERP</t>
         </is>
       </c>
-      <c r="D64" s="19" t="inlineStr">
+      <c r="D65" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F64" s="78">
-        <f>(NPV(0.095,F22:J22)+(J22*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="G64" s="78">
-        <f>(NPV(0.095,F22:J22)+(J22*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="H64" s="78">
-        <f>(NPV(0.095,F22:J22)+(J22*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="I64" s="78">
-        <f>(NPV(0.095,F22:J22)+(J22*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="J64" s="78">
-        <f>(NPV(0.095,F22:J22)+(J22*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="L64" s="63" t="inlineStr">
+      <c r="F65" s="77">
+        <f>(NPV(0.095,F22:J22)+(J22*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="G65" s="77">
+        <f>(NPV(0.095,F22:J22)+(J22*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="H65" s="77">
+        <f>(NPV(0.095,F22:J22)+(J22*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="I65" s="77">
+        <f>(NPV(0.095,F22:J22)+(J22*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="J65" s="77">
+        <f>(NPV(0.095,F22:J22)+(J22*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="L65" s="63" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="28" customHeight="1">
-      <c r="A65" s="77" t="n">
+    <row r="66" ht="28" customHeight="1">
+      <c r="A66" s="76" t="n">
         <v>0.1</v>
       </c>
-      <c r="D65" s="19" t="inlineStr">
+      <c r="D66" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F65" s="78">
-        <f>(NPV(0.1,F22:J22)+(J22*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="G65" s="78">
-        <f>(NPV(0.1,F22:J22)+(J22*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="H65" s="78">
-        <f>(NPV(0.1,F22:J22)+(J22*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="I65" s="78">
-        <f>(NPV(0.1,F22:J22)+(J22*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="J65" s="78">
-        <f>(NPV(0.1,F22:J22)+(J22*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="L65" s="63" t="inlineStr">
+      <c r="F66" s="77">
+        <f>(NPV(0.1,F22:J22)+(J22*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="G66" s="77">
+        <f>(NPV(0.1,F22:J22)+(J22*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="H66" s="77">
+        <f>(NPV(0.1,F22:J22)+(J22*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="I66" s="77">
+        <f>(NPV(0.1,F22:J22)+(J22*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="J66" s="77">
+        <f>(NPV(0.1,F22:J22)+(J22*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="L66" s="63" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="28" customHeight="1">
-      <c r="A66" s="77" t="n">
+    <row r="67" ht="28" customHeight="1">
+      <c r="A67" s="76" t="n">
         <v>0.105</v>
       </c>
-      <c r="D66" s="19" t="inlineStr">
+      <c r="D67" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F66" s="78">
-        <f>(NPV(0.105,F22:J22)+(J22*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="G66" s="78">
-        <f>(NPV(0.105,F22:J22)+(J22*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="H66" s="79">
-        <f>(NPV(0.105,F22:J22)+(J22*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="I66" s="78">
-        <f>(NPV(0.105,F22:J22)+(J22*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="J66" s="78">
-        <f>(NPV(0.105,F22:J22)+(J22*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="L66" s="63" t="inlineStr">
+      <c r="F67" s="77">
+        <f>(NPV(0.105,F22:J22)+(J22*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="G67" s="77">
+        <f>(NPV(0.105,F22:J22)+(J22*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="H67" s="78">
+        <f>(NPV(0.105,F22:J22)+(J22*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="I67" s="77">
+        <f>(NPV(0.105,F22:J22)+(J22*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="J67" s="77">
+        <f>(NPV(0.105,F22:J22)+(J22*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="L67" s="63" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="28" customHeight="1">
-      <c r="A67" s="77" t="n">
+    <row r="68" ht="28" customHeight="1">
+      <c r="A68" s="76" t="n">
         <v>0.11</v>
       </c>
-      <c r="D67" s="19" t="inlineStr">
+      <c r="D68" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F67" s="78">
-        <f>(NPV(0.11,F22:J22)+(J22*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="G67" s="78">
-        <f>(NPV(0.11,F22:J22)+(J22*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="H67" s="78">
-        <f>(NPV(0.11,F22:J22)+(J22*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="I67" s="78">
-        <f>(NPV(0.11,F22:J22)+(J22*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="J67" s="78">
-        <f>(NPV(0.11,F22:J22)+(J22*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="L67" s="63" t="inlineStr">
+      <c r="F68" s="77">
+        <f>(NPV(0.11,F22:J22)+(J22*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="G68" s="77">
+        <f>(NPV(0.11,F22:J22)+(J22*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="H68" s="77">
+        <f>(NPV(0.11,F22:J22)+(J22*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="I68" s="77">
+        <f>(NPV(0.11,F22:J22)+(J22*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="J68" s="77">
+        <f>(NPV(0.11,F22:J22)+(J22*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="L68" s="63" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="28" customHeight="1">
-      <c r="A68" s="77" t="n">
+    <row r="69" ht="28" customHeight="1">
+      <c r="A69" s="76" t="n">
         <v>0.115</v>
       </c>
-      <c r="D68" s="19" t="inlineStr">
+      <c r="D69" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F68" s="78">
-        <f>(NPV(0.115,F22:J22)+(J22*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="G68" s="78">
-        <f>(NPV(0.115,F22:J22)+(J22*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="H68" s="78">
-        <f>(NPV(0.115,F22:J22)+(J22*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="I68" s="78">
-        <f>(NPV(0.115,F22:J22)+(J22*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="J68" s="78">
-        <f>(NPV(0.115,F22:J22)+(J22*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E36+E37)/E39</f>
-        <v/>
-      </c>
-      <c r="L68" s="63" t="inlineStr">
+      <c r="F69" s="77">
+        <f>(NPV(0.115,F22:J22)+(J22*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>(NPV(0.115,F22:J22)+(J22*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="H69" s="77">
+        <f>(NPV(0.115,F22:J22)+(J22*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="I69" s="77">
+        <f>(NPV(0.115,F22:J22)+(J22*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="J69" s="77">
+        <f>(NPV(0.115,F22:J22)+(J22*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E37+E38)/E40</f>
+        <v/>
+      </c>
+      <c r="L69" s="63" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="28" customHeight="1">
-      <c r="B69" s="17" t="inlineStr">
+    <row r="70" ht="28" customHeight="1">
+      <c r="B70" s="17" t="inlineStr">
         <is>
           <t>Red WACC and g grid values bracket base case ±100bps discount rate and ±75bps terminal growth for sensitivity.</t>
         </is>
       </c>
-      <c r="C69" s="18" t="inlineStr">
+      <c r="C70" s="18" t="inlineStr">
         <is>
           <t>Scenarios: WACC &amp; terminal g</t>
         </is>
       </c>
-      <c r="D69" s="19" t="inlineStr">
+      <c r="D70" s="19" t="inlineStr">
         <is>
           <t>Scenarios tab → Ctrl+F "WACC" and "Terminal growth" rows (base-case inputs)</t>
         </is>
       </c>
-      <c r="L69" s="63" t="inlineStr">
+      <c r="L70" s="63" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="M69" s="19" t="inlineStr">
+      <c r="M70" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
@@ -4445,26 +4454,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId24"/>
-    <hyperlink ref="M47" location="'Comps'!A38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId25"/>
-    <hyperlink ref="L63" location="'Scenarios'!G10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId26"/>
-    <hyperlink ref="L64" location="'WACC'!E19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId23"/>
+    <hyperlink ref="C48" location="'DCF'!E33"/>
+    <hyperlink ref="M48" location="'Comps'!A38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId24"/>
+    <hyperlink ref="L64" location="'Scenarios'!G10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId25"/>
     <hyperlink ref="L65" location="'WACC'!E19"/>
     <hyperlink ref="L66" location="'WACC'!E19"/>
     <hyperlink ref="L67" location="'WACC'!E19"/>
     <hyperlink ref="L68" location="'WACC'!E19"/>
-    <hyperlink ref="C69" location="'Scenarios'!G9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId27"/>
+    <hyperlink ref="L69" location="'WACC'!E19"/>
+    <hyperlink ref="C70" location="'Scenarios'!G9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4655,23 +4664,23 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="75" t="inlineStr">
+      <c r="A11" s="74" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current EV / EBITDA</t>
         </is>
       </c>
-      <c r="E11" s="80">
+      <c r="E11" s="79">
         <f>(E10*E9-E8)/E5</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="75" t="inlineStr">
+      <c r="A12" s="74" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current P / E (FY2026E)</t>
         </is>
       </c>
-      <c r="E12" s="80">
+      <c r="E12" s="79">
         <f>E10/E7</f>
         <v/>
       </c>
@@ -4684,34 +4693,34 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="75" t="inlineStr">
+      <c r="A15" s="74" t="inlineStr">
         <is>
           <t>Peer / reference EV/EBITDA (forward / illustrative)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="81" t="inlineStr">
+      <c r="A16" s="80" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B16" s="81" t="inlineStr">
+      <c r="B16" s="80" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C16" s="81" t="inlineStr">
+      <c r="C16" s="80" t="inlineStr">
         <is>
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D16" s="81" t="inlineStr">
+      <c r="D16" s="80" t="inlineStr">
         <is>
           <t>Ctrl+F (prove number)</t>
         </is>
       </c>
-      <c r="E16" s="82" t="inlineStr">
+      <c r="E16" s="81" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
@@ -4738,7 +4747,7 @@
           <t>Ctrl+F "19.9%" → FY25 OM (EBIT $2,210,615). Ctrl+F "496,228" → Depreciation and amortization. Do not search the words Income from operations (17 hits).</t>
         </is>
       </c>
-      <c r="E17" s="83">
+      <c r="E17" s="82">
         <f>(E10*E9-E8)/E5</f>
         <v/>
       </c>
@@ -4764,7 +4773,7 @@
           <t>Ctrl+F "EV / EBITDA" → 11.97. Model uses 12.0x.</t>
         </is>
       </c>
-      <c r="E18" s="84" t="n">
+      <c r="E18" s="83" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4789,7 +4798,7 @@
           <t>Ctrl+F "EV / EBITDA" → 7.95. Model uses 8.0x.</t>
         </is>
       </c>
-      <c r="E19" s="84" t="n">
+      <c r="E19" s="83" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4814,7 +4823,7 @@
           <t>Ctrl+F "EV / EBITDA" → 14.03. Model uses 14.0x.</t>
         </is>
       </c>
-      <c r="E20" s="84" t="n">
+      <c r="E20" s="83" t="n">
         <v>14</v>
       </c>
     </row>
@@ -4839,7 +4848,7 @@
           <t>Ctrl+F "EV / EBITDA" → 9.31. Model uses 9.3x.</t>
         </is>
       </c>
-      <c r="E21" s="84" t="n">
+      <c r="E21" s="83" t="n">
         <v>9.300000000000001</v>
       </c>
     </row>
@@ -4864,7 +4873,7 @@
           <t>Ctrl+F "EV / EBITDA" → 10.71. Model uses 10.7x.</t>
         </is>
       </c>
-      <c r="E22" s="84" t="n">
+      <c r="E22" s="83" t="n">
         <v>10.7</v>
       </c>
     </row>
@@ -4903,7 +4912,7 @@
           <t>Ctrl+F "£1.25bn valuation" and "sold a 21% stake". That proves the 2020 valuation (£m = 1,250), not EV/EBITDA.</t>
         </is>
       </c>
-      <c r="E26" s="85" t="n">
+      <c r="E26" s="84" t="n">
         <v>1250</v>
       </c>
     </row>
@@ -4928,12 +4937,12 @@
           <t>Ctrl+F "our EBITDA, which reached £53.3 million". That proves FY25 EBITDA £m. Do not take "62.3 percent" (gross margin).</t>
         </is>
       </c>
-      <c r="E27" s="86" t="n">
+      <c r="E27" s="85" t="n">
         <v>53.3</v>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="73" t="inlineStr">
+      <c r="A28" s="72" t="inlineStr">
         <is>
           <t>Gymshark implied EV/EBITDA (model math)</t>
         </is>
@@ -4953,7 +4962,7 @@
           <t>No Ctrl+F. Neither Guardian nor SGB prints EV/EBITDA. This cell is E26 / E27 (2020 valuation ÷ FY25 EBITDA).</t>
         </is>
       </c>
-      <c r="E28" s="87">
+      <c r="E28" s="86">
         <f>E26/E27</f>
         <v/>
       </c>
@@ -4986,7 +4995,7 @@
           <t>Math: (12.0+8.0+14.0+9.3+10.7)/5 = 10.8x. Do not use as FY30 exit.</t>
         </is>
       </c>
-      <c r="E31" s="83">
+      <c r="E31" s="82">
         <f>AVERAGE(E18,E19,E20,E21,E22)</f>
         <v/>
       </c>
@@ -4999,7 +5008,7 @@
       </c>
       <c r="B32" s="26" t="inlineStr">
         <is>
-          <t>~9.3x closest mature set. Still haircut ~1 turn to 8.0x for 2.25% terminal g.</t>
+          <t>~9.3x closest mature set. Comps check only — selected exit is Gordon implied, below this tape.</t>
         </is>
       </c>
       <c r="C32" s="26" t="inlineStr">
@@ -5009,10 +5018,10 @@
       </c>
       <c r="D32" s="26" t="inlineStr">
         <is>
-          <t>Math: (8.0+9.3+10.7)/3 = 9.3x. Haircut to selected 8.0x.</t>
-        </is>
-      </c>
-      <c r="E32" s="83">
+          <t>Math: (8.0+9.3+10.7)/3 = 9.3x. Not the selected FY30 exit.</t>
+        </is>
+      </c>
+      <c r="E32" s="82">
         <f>AVERAGE(E19,E21,E22)</f>
         <v/>
       </c>
@@ -5038,13 +5047,13 @@
           <t>Math: (12.0+8.0+14.0+9.3+10.7+1,250/53.3)/6 ≈ 12.9x. Not the TV.</t>
         </is>
       </c>
-      <c r="E33" s="83">
+      <c r="E33" s="82">
         <f>AVERAGE(E18,E19,E20,E21,E22,E28)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="75" t="inlineStr">
+      <c r="A34" s="74" t="inlineStr">
         <is>
           <t>We do not average EV/EBITDA for terminal value. A 2.25% g year is not a growth-comp tape.</t>
         </is>
@@ -5069,13 +5078,13 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="73" t="inlineStr">
+      <c r="A38" s="72" t="inlineStr">
         <is>
           <t>Selected exit multiple (base case)</t>
         </is>
       </c>
-      <c r="E38" s="71">
-        <f>DCF!E47</f>
+      <c r="E38" s="70">
+        <f>DCF!E48</f>
         <v/>
       </c>
     </row>
@@ -5091,51 +5100,51 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="73" t="inlineStr">
-        <is>
-          <t>Rationale for 8.0x (not the average)</t>
+      <c r="A40" s="72" t="inlineStr">
+        <is>
+          <t>Rationale for selected exit (Gordon identity, not a peer pick)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="34" t="inlineStr">
         <is>
-          <t>•  8.0x equals Deckers (7.95x rounded) — closest mature premium analog on the tape</t>
+          <t>•  Selected exit = Gordon TV / FY30 EBITDA. Identity: (UFCF/EBITDA)×(1+g)/(WACC−g). Live formula, not a typed 8.0x</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="34" t="inlineStr">
         <is>
-          <t>•  ~1 turn above Gordon-implied ~7x — buffer vs perpetuity math on 2.25% terminal g</t>
+          <t>•  At base WACC 10.5% and g 2.25% that identity is ~6.0x — the stale “Gordon ~7x / pick Deckers 8.0x” overlay is gone</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="34" t="inlineStr">
         <is>
-          <t>•  Mid-point of the 6.5–9.5x football field — not the 10.8x public 5-name mean</t>
+          <t>•  Deckers 8.0x is a public print, not a derivation of our exit. It is only the football-field cap</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="34" t="inlineStr">
         <is>
-          <t>•  Mature public mean (DECK / ADS / VFC) is ~9.3x; we haircut ~1 turn for 2.25% terminal g</t>
+          <t>•  Public 5-name mean 10.8x and mature mean 9.3x are current trading tapes, not a 2.25% g terminal year</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="34" t="inlineStr">
         <is>
-          <t>•  Gymshark implied 23.5x is 2020 valuation / FY25 EBITDA — no page prints that multiple; averaging it (~12.9x) is not an FY30 exit</t>
+          <t>•  Gymshark implied 23.5x is 2020 valuation / FY25 EBITDA — no page prints that multiple; averaging it is not an FY30 exit</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="34" t="inlineStr">
         <is>
-          <t>•  Current LULU ~3.5x on FY2025A is a trough — 8.0x assumes partial recovery, not a re-rate to ONON 14x</t>
+          <t>•  Current LULU ~3.5–5x is a trough. Gordon 6.0x is a partial recovery, not a re-rate to ONON 14x</t>
         </is>
       </c>
     </row>
@@ -5147,42 +5156,42 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="81" t="inlineStr">
+      <c r="A49" s="80" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B49" s="81" t="inlineStr">
+      <c r="B49" s="80" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C49" s="81" t="inlineStr">
+      <c r="C49" s="80" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D49" s="81" t="inlineStr">
+      <c r="D49" s="80" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
-      <c r="E49" s="82" t="inlineStr">
+      <c r="E49" s="81" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="F49" s="82" t="inlineStr">
+      <c r="F49" s="81" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="G49" s="82" t="inlineStr">
+      <c r="G49" s="81" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="H49" s="82" t="inlineStr">
+      <c r="H49" s="81" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
@@ -5196,63 +5205,63 @@
       </c>
       <c r="B50" s="19" t="inlineStr">
         <is>
-          <t>Lo: 6.5x on FY2030E terminal EBITDA; bear exit below Gordon-implied ~7x; brackets DCF downside.
-Hi: 9.5x on FY2030E terminal EBITDA; bull exit above 8.0x DCF base; still below public mean ~10.8x.</t>
-        </is>
-      </c>
-      <c r="C50" s="88" t="inlineStr">
+          <t>Lo: 5.0x on FY2030E EBITDA ≈ LULU current trough print. Floor of the range, not the selected exit.
+Hi: 8.0x = Deckers print as the high end of the range only. Selected exit is Gordon implied, not this cap.</t>
+        </is>
+      </c>
+      <c r="C50" s="87" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU EV/EBITDA
-Hi: StockAnalysis: LULU valuation</t>
+Hi: StockAnalysis: DECK EV/EBITDA</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
         <is>
-          <t>Lo: Ctrl+F "EV / EBITDA" → LULU trough ~5x; bear terminal exit assumption 6.5x
-Hi: Ctrl+F "EV / EBITDA" → bull terminal exit assumption 9.5x on FY2030E EBITDA</t>
-        </is>
-      </c>
-      <c r="E50" s="84" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="F50" s="84" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="G50" s="89">
+          <t>Lo: Ctrl+F "EV / EBITDA" → LULU trough ~5x; football-field floor 5.0x
+Hi: Ctrl+F "EV / EBITDA" → 7.95. Football-field cap 8.0x (Deckers). Not the selected exit.</t>
+        </is>
+      </c>
+      <c r="E50" s="83" t="n">
+        <v>5</v>
+      </c>
+      <c r="F50" s="83" t="n">
+        <v>8</v>
+      </c>
+      <c r="G50" s="88">
         <f>(E6*E50+E8)/E9</f>
         <v/>
       </c>
-      <c r="H50" s="89">
+      <c r="H50" s="88">
         <f>(E6*F50+E8)/E9</f>
         <v/>
       </c>
     </row>
     <row r="51" ht="28" customHeight="1">
-      <c r="A51" s="73" t="inlineStr">
-        <is>
-          <t>DCF exit method (8.0x on FY2030E EBITDA)</t>
+      <c r="A51" s="72" t="inlineStr">
+        <is>
+          <t>DCF exit method (Gordon-implied on FY2030E EBITDA)</t>
         </is>
       </c>
       <c r="B51" s="17" t="inlineStr">
         <is>
-          <t>8.0x equals Deckers; ~1 turn above Gordon ~7x. Public mean 10.8x and Gymshark implied 23.5x are not FY30 exit.</t>
+          <t>Selected exit is Gordon TV / FY30 EBITDA. Identity: (UFCF/EBITDA)×(1+g)/(WACC−g). Not Deckers and not a peer average.</t>
         </is>
       </c>
       <c r="C51" s="18" t="inlineStr">
         <is>
-          <t>StockAnalysis: LULU EV/EBITDA</t>
+          <t>DCF: Gordon implied exit (TV / FY30 EBITDA)</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "EV / EBITDA" → LULU ~4.99x on page; model terminal exit 8.0x equals Deckers, not the public mean</t>
-        </is>
-      </c>
-      <c r="E51" s="87">
-        <f>DCF!E47</f>
-        <v/>
-      </c>
-      <c r="G51" s="90">
+          <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
+        </is>
+      </c>
+      <c r="E51" s="86">
+        <f>DCF!E48</f>
+        <v/>
+      </c>
+      <c r="G51" s="89">
         <f>(E6*E51+E8)/E9</f>
         <v/>
       </c>
@@ -5269,7 +5278,7 @@
 Hi: 18x P/E high on FY2026E EPS; modest recovery case still below historical premium LULU multiples.</t>
         </is>
       </c>
-      <c r="C52" s="88" t="inlineStr">
+      <c r="C52" s="87" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU Forward P/E
 Hi: StockAnalysis: NKE Forward P/E</t>
@@ -5281,17 +5290,17 @@
 Hi: Ctrl+F "Forward PE" → NKE peer benchmark; high-case assumption 18.0x</t>
         </is>
       </c>
-      <c r="E52" s="84" t="n">
+      <c r="E52" s="83" t="n">
         <v>10</v>
       </c>
-      <c r="F52" s="84" t="n">
+      <c r="F52" s="83" t="n">
         <v>18</v>
       </c>
-      <c r="G52" s="89">
+      <c r="G52" s="88">
         <f>E7*E52</f>
         <v/>
       </c>
-      <c r="H52" s="89">
+      <c r="H52" s="88">
         <f>E7*F52</f>
         <v/>
       </c>
@@ -5302,27 +5311,27 @@
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="E53" s="91" t="inlineStr">
+      <c r="E53" s="90" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F53" s="91" t="inlineStr">
+      <c r="F53" s="90" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G53" s="89">
+      <c r="G53" s="88">
         <f>Scenarios!F65</f>
         <v/>
       </c>
-      <c r="H53" s="89">
+      <c r="H53" s="88">
         <f>Scenarios!H65</f>
         <v/>
       </c>
     </row>
     <row r="55" ht="28" customHeight="1">
-      <c r="A55" s="92" t="inlineStr">
+      <c r="A55" s="91" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
@@ -5337,14 +5346,14 @@
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E55" s="93" t="n">
+      <c r="E55" s="92" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="26" t="inlineStr">
         <is>
-          <t>Note: public set is NKE, DECK, ONON, adidas, VFC (red). Gymshark 23.5x is implied (2020 £1.25bn / FY25 £53.3m) — no source prints EV/EBITDA. Selected TV is 8.0x, not the average.</t>
+          <t>Note: public set is NKE, DECK, ONON, adidas, VFC (red). Selected TV is Gordon implied (TV/EBITDA), not Deckers and not an average. Gymshark 23.5x is implied only.</t>
         </is>
       </c>
     </row>
@@ -5373,7 +5382,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId20"/>
     <hyperlink ref="C28" location="'Comps'!E26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId21"/>
-    <hyperlink ref="C51" location="'DCF'!E47"/>
+    <hyperlink ref="C51" location="'DCF'!E48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId24"/>

</xml_diff>

<commit_message>
Replace Gymshark with Alo; no EV/EBITDA print exists
Firecrawl of Reuters and Forbes finds a $10bn unclosed Moelis ask and
Forbes ~$2bn parent sales. Implied 5.0x is EV/Sales, not EV/EBITDA.
Alo EV/EBITDA is n.a. Selected TV stays the Gordon identity.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="168" formatCode="0.0x"/>
     <numFmt numFmtId="169" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="45">
+  <fonts count="46">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -293,6 +293,12 @@
     </font>
     <font>
       <name val="Garamond"/>
+      <i val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
       <b val="1"/>
       <color rgb="000000CC"/>
       <sz val="11"/>
@@ -580,15 +586,15 @@
     <xf numFmtId="168" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="169" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -604,7 +610,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="45" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4880,182 +4886,186 @@
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>GYMSHARK BUILD — implied multiple (no source prints EV/EBITDA)</t>
+          <t>ALO YOGA BUILD — no source prints EV/EBITDA (Firecrawl: Reuters + Forbes)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>Column E on the next two rows is £m, not a multiple. Implied EV/EBITDA is the black formula below.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="28" customHeight="1">
+          <t>Column E on the next two rows is $bn, not EV/EBITDA. The black formula is implied EV/Sales on an unclosed ask.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="42" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t>Gymshark 2020 GA valuation (£m)</t>
-        </is>
-      </c>
-      <c r="B26" s="17" t="inlineStr">
-        <is>
-          <t>£1.25bn = 1,250 in £m. 2020 GA headline valuation (Guardian). Not a published EV or EV/EBITDA.</t>
-        </is>
-      </c>
-      <c r="C26" s="18" t="inlineStr">
-        <is>
-          <t>Guardian: Gymshark 2020 GA £1.25bn</t>
+          <t>Alo / Color Image 2023 Moelis ask ($bn)</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Reuters: about $10 billion Moelis ask for Color Image. 2026 follow-up: no deal announced. Ask, not a print.
+Also: Reuters June 2026: no deal was announced on the 2023 process. The $10bn is still an ask.</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="inlineStr">
+        <is>
+          <t>Reuters: Alo parent $10bn Moelis ask
+Also: Reuters: Alo 2023 process — no deal</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "£1.25bn valuation" and "sold a 21% stake". That proves the 2020 valuation (£m = 1,250), not EV/EBITDA.</t>
+          <t>Ctrl+F "at about $10 billion" and "hired investment bank Moelis". That is the 2023 ask, not a closed EV.
+Also: Ctrl+F "roughly $10 billion" and "No deal was announced". Still an ask.</t>
         </is>
       </c>
       <c r="E26" s="84" t="n">
-        <v>1250</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>Gymshark FY25 EBITDA (£m)</t>
+          <t>Color Image parent sales, Forbes est. ($bn)</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>FY25 EBITDA is £53.3m (SGB). 62.3% is gross margin. This cell is EBITDA £m, not a multiple.</t>
+          <t>Forbes estimates Color Image parent sales nearly $2 billion. Mixed Alo + Bella+Canvas. Not Alo-only, not audited.</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>SGB: Gymshark FY25 EBITDA £53.3m</t>
+          <t>Forbes: Color Image nearly $2bn sales</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "our EBITDA, which reached £53.3 million". That proves FY25 EBITDA £m. Do not take "62.3 percent" (gross margin).</t>
-        </is>
-      </c>
-      <c r="E27" s="85" t="n">
-        <v>53.3</v>
+          <t>Ctrl+F "nearly $2 billion". Forbes estimate for Color Image parent (Alo + Bella+Canvas), not Alo-only EBITDA.</t>
+        </is>
+      </c>
+      <c r="E27" s="84" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="72" t="inlineStr">
         <is>
-          <t>Gymshark implied EV/EBITDA (model math)</t>
+          <t>Alo implied EV/Sales (ask / parent sales)</t>
         </is>
       </c>
       <c r="B28" s="26" t="inlineStr">
         <is>
-          <t>No page prints Gymshark EV/EBITDA. Black formula = 2020 valuation / FY25 EBITDA. Cross-year; not the TV.</t>
+          <t>5.0x = 10 / 2. Implied EV/Sales on an unclosed ask and parent sales. Not EV/EBITDA. Not the TV.</t>
         </is>
       </c>
       <c r="C28" s="63" t="inlineStr">
         <is>
-          <t>Comps: Gymshark valuation / EBITDA</t>
+          <t>Comps: Alo ask / parent sales</t>
         </is>
       </c>
       <c r="D28" s="19" t="inlineStr">
         <is>
-          <t>No Ctrl+F. Neither Guardian nor SGB prints EV/EBITDA. This cell is E26 / E27 (2020 valuation ÷ FY25 EBITDA).</t>
-        </is>
-      </c>
-      <c r="E28" s="86">
+          <t>No Ctrl+F for EV/EBITDA — Firecrawl found none on Reuters or Forbes. This cell is E26 / E27 (ask ÷ parent sales). Not the TV.</t>
+        </is>
+      </c>
+      <c r="E28" s="85">
         <f>E26/E27</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="14" t="inlineStr">
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>Alo EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="B29" s="26" t="inlineStr">
+        <is>
+          <t>No page prints Alo or Color Image EBITDA. PitchBook Alo column is blank. Cannot imply EV/EBITDA.</t>
+        </is>
+      </c>
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>None — no EBITDA source</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>No Ctrl+F. Reuters, Forbes, and PitchBook do not print Alo EV/EBITDA.</t>
+        </is>
+      </c>
+      <c r="E29" s="86" t="inlineStr">
+        <is>
+          <t>n.a.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>Averages (live Excel AVERAGE — shown so TV is not a blended print)</t>
         </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>Public 5-name mean (NKE / DECK / ONON / ADS / VFC)</t>
-        </is>
-      </c>
-      <c r="B31" s="26" t="inlineStr">
-        <is>
-          <t>10.8x simple mean. Too high for a 2.25% g / 15.5% OM terminal year — not the TV.</t>
-        </is>
-      </c>
-      <c r="C31" s="26" t="inlineStr">
-        <is>
-          <t>Derived: Excel AVERAGE of the five public prints</t>
-        </is>
-      </c>
-      <c r="D31" s="26" t="inlineStr">
-        <is>
-          <t>Math: (12.0+8.0+14.0+9.3+10.7)/5 = 10.8x. Do not use as FY30 exit.</t>
-        </is>
-      </c>
-      <c r="E31" s="82">
-        <f>AVERAGE(E18,E19,E20,E21,E22)</f>
-        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t>Mature public mean (DECK / ADS / VFC)</t>
+          <t>Public 5-name mean (NKE / DECK / ONON / ADS / VFC)</t>
         </is>
       </c>
       <c r="B32" s="26" t="inlineStr">
         <is>
-          <t>~9.3x closest mature set. Comps check only — selected exit is Gordon implied, below this tape.</t>
+          <t>10.8x simple mean. Too high for a 2.25% g / 15.5% OM terminal year — not the TV.</t>
         </is>
       </c>
       <c r="C32" s="26" t="inlineStr">
         <is>
-          <t>Derived: Excel AVERAGE of Deckers, adidas, VFC</t>
+          <t>Derived: Excel AVERAGE of the five public prints</t>
         </is>
       </c>
       <c r="D32" s="26" t="inlineStr">
         <is>
-          <t>Math: (8.0+9.3+10.7)/3 = 9.3x. Not the selected FY30 exit.</t>
+          <t>Math: (12.0+8.0+14.0+9.3+10.7)/5 = 10.8x. Do not use as FY30 exit.</t>
         </is>
       </c>
       <c r="E32" s="82">
-        <f>AVERAGE(E19,E21,E22)</f>
+        <f>AVERAGE(E18,E19,E20,E21,E22)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t>Mean incl. Gymshark (do not use for TV)</t>
+          <t>Mature public mean (DECK / ADS / VFC)</t>
         </is>
       </c>
       <c r="B33" s="26" t="inlineStr">
         <is>
-          <t>~12.9x. Gymshark implied 23.5x is model math (2020 val / FY25 EBITDA); averaging it overstates FY30 exit.</t>
+          <t>~9.3x closest mature set. Comps check only — selected exit is Gordon implied, below this tape.</t>
         </is>
       </c>
       <c r="C33" s="26" t="inlineStr">
         <is>
-          <t>Derived: Excel AVERAGE of five publics + Gymshark</t>
+          <t>Derived: Excel AVERAGE of Deckers, adidas, VFC</t>
         </is>
       </c>
       <c r="D33" s="26" t="inlineStr">
         <is>
-          <t>Math: (12.0+8.0+14.0+9.3+10.7+1,250/53.3)/6 ≈ 12.9x. Not the TV.</t>
+          <t>Math: (8.0+9.3+10.7)/3 = 9.3x. Not the selected FY30 exit.</t>
         </is>
       </c>
       <c r="E33" s="82">
-        <f>AVERAGE(E18,E19,E20,E21,E22,E28)</f>
+        <f>AVERAGE(E19,E21,E22)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="74" t="inlineStr">
         <is>
-          <t>We do not average EV/EBITDA for terminal value. A 2.25% g year is not a growth-comp tape.</t>
+          <t>We do not average peers for terminal value, and we do not use Alo 5.0x EV/Sales as EV/EBITDA.</t>
         </is>
       </c>
     </row>
@@ -5137,7 +5147,7 @@
     <row r="45">
       <c r="A45" s="34" t="inlineStr">
         <is>
-          <t>•  Gymshark implied 23.5x is 2020 valuation / FY25 EBITDA — no page prints that multiple; averaging it is not an FY30 exit</t>
+          <t>•  Alo has no EV/EBITDA print. Implied 5.0x is EV/Sales (unclosed $10bn ask / ~$2bn parent sales) — not the FY30 exit</t>
         </is>
       </c>
     </row>
@@ -5257,7 +5267,7 @@
           <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
         </is>
       </c>
-      <c r="E51" s="86">
+      <c r="E51" s="85">
         <f>DCF!E48</f>
         <v/>
       </c>
@@ -5353,7 +5363,7 @@
     <row r="56">
       <c r="A56" s="26" t="inlineStr">
         <is>
-          <t>Note: public set is NKE, DECK, ONON, adidas, VFC (red). Selected TV is Gordon implied (TV/EBITDA), not Deckers and not an average. Gymshark 23.5x is implied only.</t>
+          <t>Note: public set is NKE, DECK, ONON, adidas, VFC (red). Alo is a private reference (implied 5.0x EV/Sales; EV/EBITDA n.a.). Selected TV is Gordon implied, not Alo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use the PitchBook 04-Sep-2026 set as public comps
Each EV/EBITDA is a live daily-EV / TTM-EBITDA formula from the
extract. UAA is shown but excluded from averages (negative EBITDA).
Selected FY30 exit stays the Gordon identity, not the PitchBook mean.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -363,7 +363,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -580,23 +580,29 @@
     <xf numFmtId="0" fontId="30" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="168" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="168" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4469,7 +4475,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId23"/>
     <hyperlink ref="C48" location="'DCF'!E33"/>
-    <hyperlink ref="M48" location="'Comps'!A38"/>
+    <hyperlink ref="M48" location="'Comps'!A45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId24"/>
     <hyperlink ref="L64" location="'Scenarios'!G10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId25"/>
@@ -4491,7 +4497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:J63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -4502,6 +4508,8 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -4706,131 +4714,118 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="80" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>PITCHBOOK PUBCOMPS — daily EV / TTM EBITDA as of 04-Sep-2026 ($000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>EV/EBITDA is a black formula (I/J). UAA is shown but excluded from averages (negative TTM EBITDA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="80" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B16" s="80" t="inlineStr">
+      <c r="B18" s="80" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C16" s="80" t="inlineStr">
-        <is>
-          <t>Source (click)</t>
-        </is>
-      </c>
-      <c r="D16" s="80" t="inlineStr">
-        <is>
-          <t>Ctrl+F (prove number)</t>
-        </is>
-      </c>
-      <c r="E16" s="81" t="inlineStr">
+      <c r="C18" s="80" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D18" s="80" t="inlineStr">
+        <is>
+          <t>Ctrl+F / proof</t>
+        </is>
+      </c>
+      <c r="E18" s="81" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>lululemon (LULU) — current</t>
-        </is>
-      </c>
-      <c r="B17" s="26" t="inlineStr">
-        <is>
-          <t>Distressed trough multiple on FY2025A EBITDA</t>
-        </is>
-      </c>
-      <c r="C17" s="63" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K</t>
-        </is>
-      </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "19.9%" → FY25 OM (EBIT $2,210,615). Ctrl+F "496,228" → Depreciation and amortization. Do not search the words Income from operations (17 hits).</t>
-        </is>
-      </c>
-      <c r="E17" s="82">
-        <f>(E10*E9-E8)/E5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>Nike (NKE)</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>Nike EV/EBITDA 12.0x equals StockAnalysis 11.97x, rounded; mature athletic benchmark.</t>
-        </is>
-      </c>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>StockAnalysis: NKE EV/EBITDA</t>
-        </is>
-      </c>
-      <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "EV / EBITDA" → 11.97. Model uses 12.0x.</t>
-        </is>
-      </c>
-      <c r="E18" s="83" t="n">
-        <v>12</v>
+      <c r="I18" s="81" t="inlineStr">
+        <is>
+          <t>EV ($000)</t>
+        </is>
+      </c>
+      <c r="J18" s="81" t="inlineStr">
+        <is>
+          <t>EBITDA ($000)</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>Deckers (DECK)</t>
+          <t>lululemon (LULU)</t>
         </is>
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>Deckers EV/EBITDA 8.0x equals StockAnalysis 7.95x, rounded; closest premium-footwear peer.</t>
-        </is>
-      </c>
-      <c r="C19" s="18" t="inlineStr">
-        <is>
-          <t>StockAnalysis: DECK EV/EBITDA</t>
+          <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
+        </is>
+      </c>
+      <c r="C19" s="82" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "EV / EBITDA" → 7.95. Model uses 8.0x.</t>
-        </is>
-      </c>
-      <c r="E19" s="83" t="n">
-        <v>8</v>
+          <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
+        </is>
+      </c>
+      <c r="E19" s="83">
+        <f>IF(J19&lt;=0,"n.m.",I19/J19)</f>
+        <v/>
+      </c>
+      <c r="I19" s="84" t="n">
+        <v>11890440</v>
+      </c>
+      <c r="J19" s="84" t="n">
+        <v>2548084</v>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>On Holding (ONON)</t>
+          <t>Under Armour (UAA)</t>
         </is>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>On Holding EV/EBITDA 14.0x equals StockAnalysis 14.03x, rounded; high-growth athletic peer.</t>
-        </is>
-      </c>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>StockAnalysis: ONON EV/EBITDA</t>
+          <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
+        </is>
+      </c>
+      <c r="C20" s="82" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "EV / EBITDA" → 14.03. Model uses 14.0x.</t>
-        </is>
-      </c>
-      <c r="E20" s="83" t="n">
-        <v>14</v>
+          <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
+        </is>
+      </c>
+      <c r="E20" s="83">
+        <f>IF(J20&lt;=0,"n.m.",I20/J20)</f>
+        <v/>
+      </c>
+      <c r="I20" s="84" t="n">
+        <v>3208397</v>
+      </c>
+      <c r="J20" s="84" t="n">
+        <v>-23230</v>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
@@ -4841,529 +4836,767 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>adidas (ADDYY) EV/EBITDA 9.3x equals StockAnalysis 9.31x; global incumbent.</t>
-        </is>
-      </c>
-      <c r="C21" s="18" t="inlineStr">
-        <is>
-          <t>StockAnalysis: adidas (ADR)</t>
+          <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
+        </is>
+      </c>
+      <c r="C21" s="82" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "EV / EBITDA" → 9.31. Model uses 9.3x.</t>
-        </is>
-      </c>
-      <c r="E21" s="83" t="n">
-        <v>9.300000000000001</v>
+          <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
+        </is>
+      </c>
+      <c r="E21" s="83">
+        <f>IF(J21&lt;=0,"n.m.",I21/J21)</f>
+        <v/>
+      </c>
+      <c r="I21" s="84" t="n">
+        <v>35661944</v>
+      </c>
+      <c r="J21" s="84" t="n">
+        <v>3857684</v>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>V.F. Corp (VFC)</t>
+          <t>Nike (NKE)</t>
         </is>
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>VFC EV/EBITDA 10.7x equals StockAnalysis 10.71x; challenged multi-brand apparel peer.</t>
-        </is>
-      </c>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>StockAnalysis: VFC EV/EBITDA</t>
+          <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
+        </is>
+      </c>
+      <c r="C22" s="82" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "EV / EBITDA" → 10.71. Model uses 10.7x.</t>
-        </is>
-      </c>
-      <c r="E22" s="83" t="n">
-        <v>10.7</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+          <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
+        </is>
+      </c>
+      <c r="E22" s="83">
+        <f>IF(J22&lt;=0,"n.m.",I22/J22)</f>
+        <v/>
+      </c>
+      <c r="I22" s="84" t="n">
+        <v>58972350</v>
+      </c>
+      <c r="J22" s="84" t="n">
+        <v>4647000</v>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Deckers (DECK)</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
+        </is>
+      </c>
+      <c r="C23" s="82" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
+        </is>
+      </c>
+      <c r="E23" s="83">
+        <f>IF(J23&lt;=0,"n.m.",I23/J23)</f>
+        <v/>
+      </c>
+      <c r="I23" s="84" t="n">
+        <v>10555510</v>
+      </c>
+      <c r="J23" s="84" t="n">
+        <v>1329439</v>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>Williams-Sonoma (WSM)</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
+        </is>
+      </c>
+      <c r="C24" s="82" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
+        </is>
+      </c>
+      <c r="E24" s="83">
+        <f>IF(J24&lt;=0,"n.m.",I24/J24)</f>
+        <v/>
+      </c>
+      <c r="I24" s="84" t="n">
+        <v>27284350</v>
+      </c>
+      <c r="J24" s="84" t="n">
+        <v>1768400</v>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>Crocs (CROX)</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
+        </is>
+      </c>
+      <c r="C25" s="82" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
+        </is>
+      </c>
+      <c r="E25" s="83">
+        <f>IF(J25&lt;=0,"n.m.",I25/J25)</f>
+        <v/>
+      </c>
+      <c r="I25" s="84" t="n">
+        <v>7153911</v>
+      </c>
+      <c r="J25" s="84" t="n">
+        <v>922278</v>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>Movado (MOV)</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
+        </is>
+      </c>
+      <c r="C26" s="82" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
+        </is>
+      </c>
+      <c r="E26" s="83">
+        <f>IF(J26&lt;=0,"n.m.",I26/J26)</f>
+        <v/>
+      </c>
+      <c r="I26" s="84" t="n">
+        <v>616045</v>
+      </c>
+      <c r="J26" s="84" t="n">
+        <v>62010</v>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>Levi Strauss (LEVI)</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
+        </is>
+      </c>
+      <c r="C27" s="82" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
+        </is>
+      </c>
+      <c r="E27" s="83">
+        <f>IF(J27&lt;=0,"n.m.",I27/J27)</f>
+        <v/>
+      </c>
+      <c r="I27" s="84" t="n">
+        <v>9422753</v>
+      </c>
+      <c r="J27" s="84" t="n">
+        <v>976700</v>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>La-Z-Boy (LZB)</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
+        </is>
+      </c>
+      <c r="C28" s="82" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
+        </is>
+      </c>
+      <c r="E28" s="83">
+        <f>IF(J28&lt;=0,"n.m.",I28/J28)</f>
+        <v/>
+      </c>
+      <c r="I28" s="84" t="n">
+        <v>1598873</v>
+      </c>
+      <c r="J28" s="84" t="n">
+        <v>235723</v>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>Kontoor (KTB)</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
+        </is>
+      </c>
+      <c r="C29" s="82" t="inlineStr">
+        <is>
+          <t>PitchBook Comps Set 04-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
+        </is>
+      </c>
+      <c r="E29" s="83">
+        <f>IF(J29&lt;=0,"n.m.",I29/J29)</f>
+        <v/>
+      </c>
+      <c r="I29" s="84" t="n">
+        <v>5236269</v>
+      </c>
+      <c r="J29" s="84" t="n">
+        <v>407521</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>ALO YOGA BUILD — no source prints EV/EBITDA (Firecrawl: Reuters + Forbes)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="26" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="26" t="inlineStr">
         <is>
           <t>Column E on the next two rows is $bn, not EV/EBITDA. The black formula is implied EV/Sales on an unclosed ask.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="42" customHeight="1">
-      <c r="A26" s="16" t="inlineStr">
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>Alo / Color Image 2023 Moelis ask ($bn)</t>
         </is>
       </c>
-      <c r="B26" s="19" t="inlineStr">
+      <c r="B33" s="19" t="inlineStr">
         <is>
           <t>Reuters: about $10 billion Moelis ask for Color Image. 2026 follow-up: no deal announced. Ask, not a print.
 Also: Reuters June 2026: no deal was announced on the 2023 process. The $10bn is still an ask.</t>
         </is>
       </c>
-      <c r="C26" s="22" t="inlineStr">
+      <c r="C33" s="22" t="inlineStr">
         <is>
           <t>Reuters: Alo parent $10bn Moelis ask
 Also: Reuters: Alo 2023 process — no deal</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
+      <c r="D33" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "at about $10 billion" and "hired investment bank Moelis". That is the 2023 ask, not a closed EV.
 Also: Ctrl+F "roughly $10 billion" and "No deal was announced". Still an ask.</t>
         </is>
       </c>
-      <c r="E26" s="84" t="n">
+      <c r="E33" s="85" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="16" t="inlineStr">
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t>Color Image parent sales, Forbes est. ($bn)</t>
         </is>
       </c>
-      <c r="B27" s="17" t="inlineStr">
+      <c r="B34" s="17" t="inlineStr">
         <is>
           <t>Forbes estimates Color Image parent sales nearly $2 billion. Mixed Alo + Bella+Canvas. Not Alo-only, not audited.</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C34" s="18" t="inlineStr">
         <is>
           <t>Forbes: Color Image nearly $2bn sales</t>
         </is>
       </c>
-      <c r="D27" s="19" t="inlineStr">
+      <c r="D34" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "nearly $2 billion". Forbes estimate for Color Image parent (Alo + Bella+Canvas), not Alo-only EBITDA.</t>
         </is>
       </c>
-      <c r="E27" s="84" t="n">
+      <c r="E34" s="85" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="72" t="inlineStr">
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="72" t="inlineStr">
         <is>
           <t>Alo implied EV/Sales (ask / parent sales)</t>
         </is>
       </c>
-      <c r="B28" s="26" t="inlineStr">
+      <c r="B35" s="26" t="inlineStr">
         <is>
           <t>5.0x = 10 / 2. Implied EV/Sales on an unclosed ask and parent sales. Not EV/EBITDA. Not the TV.</t>
         </is>
       </c>
-      <c r="C28" s="63" t="inlineStr">
+      <c r="C35" s="63" t="inlineStr">
         <is>
           <t>Comps: Alo ask / parent sales</t>
         </is>
       </c>
-      <c r="D28" s="19" t="inlineStr">
-        <is>
-          <t>No Ctrl+F for EV/EBITDA — Firecrawl found none on Reuters or Forbes. This cell is E26 / E27 (ask ÷ parent sales). Not the TV.</t>
-        </is>
-      </c>
-      <c r="E28" s="85">
-        <f>E26/E27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>No Ctrl+F for EV/EBITDA — Firecrawl found none on Reuters or Forbes. This cell is E33 / E34 (ask ÷ parent sales). Not the TV.</t>
+        </is>
+      </c>
+      <c r="E35" s="86">
+        <f>E33/E34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>Alo EV/EBITDA</t>
         </is>
       </c>
-      <c r="B29" s="26" t="inlineStr">
+      <c r="B36" s="26" t="inlineStr">
         <is>
           <t>No page prints Alo or Color Image EBITDA. PitchBook Alo column is blank. Cannot imply EV/EBITDA.</t>
         </is>
       </c>
-      <c r="C29" s="26" t="inlineStr">
+      <c r="C36" s="26" t="inlineStr">
         <is>
           <t>None — no EBITDA source</t>
         </is>
       </c>
-      <c r="D29" s="19" t="inlineStr">
+      <c r="D36" s="19" t="inlineStr">
         <is>
           <t>No Ctrl+F. Reuters, Forbes, and PitchBook do not print Alo EV/EBITDA.</t>
         </is>
       </c>
-      <c r="E29" s="86" t="inlineStr">
+      <c r="E36" s="87" t="inlineStr">
         <is>
           <t>n.a.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="14" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <t>Averages (live Excel AVERAGE — shown so TV is not a blended print)</t>
         </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t>Public 5-name mean (NKE / DECK / ONON / ADS / VFC)</t>
-        </is>
-      </c>
-      <c r="B32" s="26" t="inlineStr">
-        <is>
-          <t>10.8x simple mean. Too high for a 2.25% g / 15.5% OM terminal year — not the TV.</t>
-        </is>
-      </c>
-      <c r="C32" s="26" t="inlineStr">
-        <is>
-          <t>Derived: Excel AVERAGE of the five public prints</t>
-        </is>
-      </c>
-      <c r="D32" s="26" t="inlineStr">
-        <is>
-          <t>Math: (12.0+8.0+14.0+9.3+10.7)/5 = 10.8x. Do not use as FY30 exit.</t>
-        </is>
-      </c>
-      <c r="E32" s="82">
-        <f>AVERAGE(E18,E19,E20,E21,E22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="16" t="inlineStr">
-        <is>
-          <t>Mature public mean (DECK / ADS / VFC)</t>
-        </is>
-      </c>
-      <c r="B33" s="26" t="inlineStr">
-        <is>
-          <t>~9.3x closest mature set. Comps check only — selected exit is Gordon implied, below this tape.</t>
-        </is>
-      </c>
-      <c r="C33" s="26" t="inlineStr">
-        <is>
-          <t>Derived: Excel AVERAGE of Deckers, adidas, VFC</t>
-        </is>
-      </c>
-      <c r="D33" s="26" t="inlineStr">
-        <is>
-          <t>Math: (8.0+9.3+10.7)/3 = 9.3x. Not the selected FY30 exit.</t>
-        </is>
-      </c>
-      <c r="E33" s="82">
-        <f>AVERAGE(E19,E21,E22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="74" t="inlineStr">
-        <is>
-          <t>We do not average peers for terminal value, and we do not use Alo 5.0x EV/Sales as EV/EBITDA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="14" t="inlineStr">
-        <is>
-          <t>Terminal multiple selection (DCF exit method)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="16" t="inlineStr">
-        <is>
-          <t>Gordon Growth implied exit EV/EBITDA</t>
-        </is>
-      </c>
-      <c r="E37" s="62">
-        <f>DCF!E33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="72" t="inlineStr">
-        <is>
-          <t>Selected exit multiple (base case)</t>
-        </is>
-      </c>
-      <c r="E38" s="70">
-        <f>DCF!E48</f>
-        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
         <is>
+          <t>Core athletic / apparel mean (LULU / NKE / ADS / DECK / CROX / LEVI / KTB)</t>
+        </is>
+      </c>
+      <c r="B39" s="26" t="inlineStr">
+        <is>
+          <t>PitchBook core set, UAA out. Current tape — not a 2.25% g FY30 exit.</t>
+        </is>
+      </c>
+      <c r="C39" s="26" t="inlineStr">
+        <is>
+          <t>Derived: Excel AVERAGE of the seven core prints</t>
+        </is>
+      </c>
+      <c r="D39" s="26" t="inlineStr">
+        <is>
+          <t>Each E cell is I/J from the PitchBook extract. Do not use as FY30 exit.</t>
+        </is>
+      </c>
+      <c r="E39" s="83">
+        <f>AVERAGE(E19,E22,E21,E23,E25,E27,E29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>All positive-EBITDA mean (ex-UAA; includes WSM / MOV / LZB)</t>
+        </is>
+      </c>
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>Wider PitchBook tape. WSM/MOV/LZB are adjacent retail, not athletic. Not the TV.</t>
+        </is>
+      </c>
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>Derived: Excel AVERAGE of every positive-EBITDA row</t>
+        </is>
+      </c>
+      <c r="D40" s="26" t="inlineStr">
+        <is>
+          <t>UAA omitted because TTM EBITDA is negative. Not the selected FY30 exit.</t>
+        </is>
+      </c>
+      <c r="E40" s="83">
+        <f>AVERAGE(E19,E21,E22,E23,E24,E25,E26,E27,E28,E29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="74" t="inlineStr">
+        <is>
+          <t>We do not average peers for terminal value, and we do not use Alo 5.0x EV/Sales as EV/EBITDA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>Terminal multiple selection (DCF exit method)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>Gordon Growth implied exit EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="E44" s="62">
+        <f>DCF!E33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="72" t="inlineStr">
+        <is>
+          <t>Selected exit multiple (base case)</t>
+        </is>
+      </c>
+      <c r="E45" s="70">
+        <f>DCF!E48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
           <t>Spread (selected − Gordon implied)</t>
         </is>
       </c>
-      <c r="E39" s="62">
-        <f>E38-E37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="72" t="inlineStr">
+      <c r="E46" s="62">
+        <f>E45-E44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="72" t="inlineStr">
         <is>
           <t>Rationale for selected exit (Gordon identity, not a peer pick)</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="34" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="34" t="inlineStr">
         <is>
           <t>•  Selected exit = Gordon TV / FY30 EBITDA. Identity: (UFCF/EBITDA)×(1+g)/(WACC−g). Live formula, not a typed 8.0x</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="34" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="34" t="inlineStr">
         <is>
           <t>•  At base WACC 10.5% and g 2.25% that identity is ~6.0x — the stale “Gordon ~7x / pick Deckers 8.0x” overlay is gone</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="34" t="inlineStr">
-        <is>
-          <t>•  Deckers 8.0x is a public print, not a derivation of our exit. It is only the football-field cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="34" t="inlineStr">
-        <is>
-          <t>•  Public 5-name mean 10.8x and mature mean 9.3x are current trading tapes, not a 2.25% g terminal year</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="34" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="34" t="inlineStr">
+        <is>
+          <t>•  PitchBook pubcomps (04-Sep-2026) are the current tape: each multiple is daily EV / TTM EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="34" t="inlineStr">
+        <is>
+          <t>•  That tape is a check, not the exit. A 2.25% g / 15.5% OM year is not today’s NKE/WSM multiple</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="34" t="inlineStr">
         <is>
           <t>•  Alo has no EV/EBITDA print. Implied 5.0x is EV/Sales (unclosed $10bn ask / ~$2bn parent sales) — not the FY30 exit</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="34" t="inlineStr">
-        <is>
-          <t>•  Current LULU ~3.5–5x is a trough. Gordon 6.0x is a partial recovery, not a re-rate to ONON 14x</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="14" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="34" t="inlineStr">
+        <is>
+          <t>•  PitchBook LULU is ~4.7x TTM. Gordon 6.0x is a partial recovery, not a re-rate to WSM ~15x</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="inlineStr">
         <is>
           <t>Methodology / multiple ranges (FY2030E terminal EBITDA — football field)</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="80" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="80" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B49" s="80" t="inlineStr">
+      <c r="B56" s="80" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C49" s="80" t="inlineStr">
+      <c r="C56" s="80" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D49" s="80" t="inlineStr">
+      <c r="D56" s="80" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
-      <c r="E49" s="81" t="inlineStr">
+      <c r="E56" s="81" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="F49" s="81" t="inlineStr">
+      <c r="F56" s="81" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="G49" s="81" t="inlineStr">
+      <c r="G56" s="81" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="H49" s="81" t="inlineStr">
+      <c r="H56" s="81" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="42" customHeight="1">
-      <c r="A50" s="16" t="inlineStr">
+    <row r="57" ht="42" customHeight="1">
+      <c r="A57" s="16" t="inlineStr">
         <is>
           <t>EV / EBITDA (FY2030E terminal)</t>
         </is>
       </c>
-      <c r="B50" s="19" t="inlineStr">
+      <c r="B57" s="19" t="inlineStr">
         <is>
           <t>Lo: 5.0x on FY2030E EBITDA ≈ LULU current trough print. Floor of the range, not the selected exit.
 Hi: 8.0x = Deckers print as the high end of the range only. Selected exit is Gordon implied, not this cap.</t>
         </is>
       </c>
-      <c r="C50" s="87" t="inlineStr">
+      <c r="C57" s="88" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU EV/EBITDA
 Hi: StockAnalysis: DECK EV/EBITDA</t>
         </is>
       </c>
-      <c r="D50" s="19" t="inlineStr">
+      <c r="D57" s="19" t="inlineStr">
         <is>
           <t>Lo: Ctrl+F "EV / EBITDA" → LULU trough ~5x; football-field floor 5.0x
 Hi: Ctrl+F "EV / EBITDA" → 7.95. Football-field cap 8.0x (Deckers). Not the selected exit.</t>
         </is>
       </c>
-      <c r="E50" s="83" t="n">
+      <c r="E57" s="89" t="n">
         <v>5</v>
       </c>
-      <c r="F50" s="83" t="n">
+      <c r="F57" s="89" t="n">
         <v>8</v>
       </c>
-      <c r="G50" s="88">
-        <f>(E6*E50+E8)/E9</f>
-        <v/>
-      </c>
-      <c r="H50" s="88">
-        <f>(E6*F50+E8)/E9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="28" customHeight="1">
-      <c r="A51" s="72" t="inlineStr">
+      <c r="G57" s="90">
+        <f>(E6*E57+E8)/E9</f>
+        <v/>
+      </c>
+      <c r="H57" s="90">
+        <f>(E6*F57+E8)/E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="28" customHeight="1">
+      <c r="A58" s="72" t="inlineStr">
         <is>
           <t>DCF exit method (Gordon-implied on FY2030E EBITDA)</t>
         </is>
       </c>
-      <c r="B51" s="17" t="inlineStr">
+      <c r="B58" s="17" t="inlineStr">
         <is>
           <t>Selected exit is Gordon TV / FY30 EBITDA. Identity: (UFCF/EBITDA)×(1+g)/(WACC−g). Not Deckers and not a peer average.</t>
         </is>
       </c>
-      <c r="C51" s="18" t="inlineStr">
+      <c r="C58" s="18" t="inlineStr">
         <is>
           <t>DCF: Gordon implied exit (TV / FY30 EBITDA)</t>
         </is>
       </c>
-      <c r="D51" s="19" t="inlineStr">
+      <c r="D58" s="19" t="inlineStr">
         <is>
           <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
         </is>
       </c>
-      <c r="E51" s="85">
+      <c r="E58" s="86">
         <f>DCF!E48</f>
         <v/>
       </c>
-      <c r="G51" s="89">
-        <f>(E6*E51+E8)/E9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" ht="42" customHeight="1">
-      <c r="A52" s="16" t="inlineStr">
+      <c r="G58" s="91">
+        <f>(E6*E58+E8)/E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="42" customHeight="1">
+      <c r="A59" s="16" t="inlineStr">
         <is>
           <t>P / E (FY2026E EPS)</t>
         </is>
       </c>
-      <c r="B52" s="19" t="inlineStr">
+      <c r="B59" s="19" t="inlineStr">
         <is>
           <t>Lo: 10x P/E low on FY2026E EPS; trough earnings multiple after guidance reset and sentiment de-rating.
 Hi: 18x P/E high on FY2026E EPS; modest recovery case still below historical premium LULU multiples.</t>
         </is>
       </c>
-      <c r="C52" s="87" t="inlineStr">
+      <c r="C59" s="88" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU Forward P/E
 Hi: StockAnalysis: NKE Forward P/E</t>
         </is>
       </c>
-      <c r="D52" s="19" t="inlineStr">
+      <c r="D59" s="19" t="inlineStr">
         <is>
           <t>Lo: Ctrl+F "Forward PE" → LULU ~12.3x; low-case multiple assumption 10.0x
 Hi: Ctrl+F "Forward PE" → NKE peer benchmark; high-case assumption 18.0x</t>
         </is>
       </c>
-      <c r="E52" s="83" t="n">
+      <c r="E59" s="89" t="n">
         <v>10</v>
       </c>
-      <c r="F52" s="83" t="n">
+      <c r="F59" s="89" t="n">
         <v>18</v>
       </c>
-      <c r="G52" s="88">
-        <f>E7*E52</f>
-        <v/>
-      </c>
-      <c r="H52" s="88">
-        <f>E7*F52</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="16" t="inlineStr">
+      <c r="G59" s="90">
+        <f>E7*E59</f>
+        <v/>
+      </c>
+      <c r="H59" s="90">
+        <f>E7*F59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="inlineStr">
         <is>
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="E53" s="90" t="inlineStr">
+      <c r="E60" s="92" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F53" s="90" t="inlineStr">
+      <c r="F60" s="92" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G53" s="88">
+      <c r="G60" s="90">
         <f>Scenarios!F65</f>
         <v/>
       </c>
-      <c r="H53" s="88">
+      <c r="H60" s="90">
         <f>Scenarios!H65</f>
         <v/>
       </c>
     </row>
-    <row r="55" ht="28" customHeight="1">
-      <c r="A55" s="91" t="inlineStr">
+    <row r="62" ht="28" customHeight="1">
+      <c r="A62" s="93" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C55" s="63" t="inlineStr">
+      <c r="C62" s="63" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="D55" s="19" t="inlineStr">
+      <c r="D62" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E55" s="92" t="n">
+      <c r="E62" s="94" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="26" t="inlineStr">
-        <is>
-          <t>Note: public set is NKE, DECK, ONON, adidas, VFC (red). Alo is a private reference (implied 5.0x EV/Sales; EV/EBITDA n.a.). Selected TV is Gordon implied, not Alo.</t>
+    <row r="63">
+      <c r="A63" s="26" t="inlineStr">
+        <is>
+          <t>Note: pubcomps are PitchBook 04-Sep-2026 (EV/EBITDA = daily EV / TTM EBITDA). UAA excluded from the mean. Selected TV is Gordon implied, not the PitchBook average. Alo EV/EBITDA is n.a.</t>
         </is>
       </c>
     </row>
@@ -5380,22 +5613,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId20"/>
-    <hyperlink ref="C28" location="'Comps'!E26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId21"/>
-    <hyperlink ref="C51" location="'DCF'!E48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId14"/>
+    <hyperlink ref="C35" location="'Comps'!E33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId15"/>
+    <hyperlink ref="C58" location="'DCF'!E48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix #VALUE! errors on Revenue Drivers reconciliation rows
Comparable store revenue formulas were missing the leading '=' so Excel
treated them as text. Also link FY26+ prior-year store revenue to the
prior column's store channel total.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -3941,6 +3941,26 @@
       <c r="E28" s="56" t="n">
         <v>5049744</v>
       </c>
+      <c r="F28" s="35">
+        <f>E31</f>
+        <v/>
+      </c>
+      <c r="G28" s="35">
+        <f>F31</f>
+        <v/>
+      </c>
+      <c r="H28" s="35">
+        <f>G31</f>
+        <v/>
+      </c>
+      <c r="I28" s="35">
+        <f>H31</f>
+        <v/>
+      </c>
+      <c r="J28" s="35">
+        <f>I31</f>
+        <v/>
+      </c>
       <c r="K28" s="50" t="inlineStr">
         <is>
           <t>$000</t>
@@ -3956,30 +3976,25 @@
       <c r="E29" s="49" t="n">
         <v>5049744</v>
       </c>
-      <c r="F29" s="35" t="inlineStr">
-        <is>
-          <t>(E28*0.71*(1+F25)+E28*0.16*(1+F26)+E28*0.13*(1+F27))</t>
-        </is>
-      </c>
-      <c r="G29" s="35" t="inlineStr">
-        <is>
-          <t>(F28*0.71*(1+G25)+F28*0.16*(1+G26)+F28*0.13*(1+G27))</t>
-        </is>
-      </c>
-      <c r="H29" s="35" t="inlineStr">
-        <is>
-          <t>(G28*0.71*(1+H25)+G28*0.16*(1+H26)+G28*0.13*(1+H27))</t>
-        </is>
-      </c>
-      <c r="I29" s="35" t="inlineStr">
-        <is>
-          <t>(H28*0.71*(1+I25)+H28*0.16*(1+I26)+H28*0.13*(1+I27))</t>
-        </is>
-      </c>
-      <c r="J29" s="35" t="inlineStr">
-        <is>
-          <t>(I28*0.71*(1+J25)+I28*0.16*(1+J26)+I28*0.13*(1+J27))</t>
-        </is>
+      <c r="F29" s="35">
+        <f>E28*0.71*(1+F25)+E28*0.16*(1+F26)+E28*0.13*(1+F27)</f>
+        <v/>
+      </c>
+      <c r="G29" s="35">
+        <f>F28*0.71*(1+G25)+F28*0.16*(1+G26)+F28*0.13*(1+G27)</f>
+        <v/>
+      </c>
+      <c r="H29" s="35">
+        <f>G28*0.71*(1+H25)+G28*0.16*(1+H26)+G28*0.13*(1+H27)</f>
+        <v/>
+      </c>
+      <c r="I29" s="35">
+        <f>H28*0.71*(1+I25)+H28*0.16*(1+I26)+H28*0.13*(1+I27)</f>
+        <v/>
+      </c>
+      <c r="J29" s="35">
+        <f>I28*0.71*(1+J25)+I28*0.16*(1+J26)+I28*0.13*(1+J27)</f>
+        <v/>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">

</xml_diff>

<commit_message>
Split geo comp-sales docs; add RoW-specific justification and Ctrl+F anchor
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -3805,17 +3805,17 @@
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>FY26 Americas comp −4% vs FY25 −3% (10-K). China +14% vs +20% reported; RoW moderates from +9%.</t>
+          <t>FY25 Americas comp −3% per 10-K (traffic, conversion, AOV down). FY26 −4%: modest step-down before flat FY27 as promo clears.</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>FY2025 10-K: segment comp sales</t>
+          <t>FY2025 10-K: Americas comparable sales</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Americas comparable sales decreased 3%" / "China Mainland comparable sales increased 20%"</t>
+          <t>Ctrl+F "Americas comparable sales decreased 3%" → FY25 anchor. FY26 model −4% before stabilization.</t>
         </is>
       </c>
       <c r="E25" s="55" t="n">
@@ -3850,17 +3850,17 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>FY26 Americas comp −4% vs FY25 −3% (10-K). China +14% vs +20% reported; RoW moderates from +9%.</t>
+          <t>FY25 China comp +20% (+19% CCY) per 10-K. FY26 +14%: still fastest region but moderating as the store base scales.</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>FY2025 10-K: segment comp sales</t>
+          <t>FY2025 10-K: China Mainland comparable sales</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Americas comparable sales decreased 3%" / "China Mainland comparable sales increased 20%"</t>
+          <t>Ctrl+F "China Mainland comparable sales increased 20%" → FY25 anchor. FY26 model +14% on a larger base.</t>
         </is>
       </c>
       <c r="E26" s="55" t="n">
@@ -3895,17 +3895,17 @@
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>FY26 Americas comp −4% vs FY25 −3% (10-K). China +14% vs +20% reported; RoW moderates from +9%.</t>
+          <t>FY25 RoW comp +9% (+7% CCY) per 10-K. FY26 +7%: hold above CCY, fade to +4% by FY30 as APAC/Europe base matures.</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>FY2025 10-K: segment comp sales</t>
+          <t>FY2025 10-K: Rest of World comparable sales</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Americas comparable sales decreased 3%" / "China Mainland comparable sales increased 20%"</t>
+          <t>Ctrl+F "Rest of World comparable sales increased 9%" → FY25 +9% (+7% CCY). FY26 model +7%, fading to +4%.</t>
         </is>
       </c>
       <c r="E27" s="55" t="n">

</xml_diff>

<commit_message>
Move Revenue Drivers justification columns to the right of the data
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -510,13 +510,13 @@
     <xf numFmtId="0" fontId="27" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -2983,16 +2983,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3020,17 +3020,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="43" t="inlineStr">
+      <c r="I3" s="43" t="inlineStr">
         <is>
           <t>Justification (~20 words)</t>
         </is>
       </c>
-      <c r="C3" s="43" t="inlineStr">
+      <c r="J3" s="43" t="inlineStr">
         <is>
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D3" s="43" t="inlineStr">
+      <c r="K3" s="43" t="inlineStr">
         <is>
           <t>Ctrl+F (prove number)</t>
         </is>
@@ -3051,52 +3051,52 @@
       </c>
       <c r="B5" s="46" t="inlineStr">
         <is>
+          <t>FY2025A</t>
+        </is>
+      </c>
+      <c r="C5" s="47" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="D5" s="46" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="E5" s="46" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="F5" s="46" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="G5" s="46" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+      <c r="H5" s="46" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="I5" s="48" t="inlineStr">
+        <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C5" s="46" t="inlineStr">
+      <c r="J5" s="48" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D5" s="46" t="inlineStr">
+      <c r="K5" s="48" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
-        </is>
-      </c>
-      <c r="E5" s="47" t="inlineStr">
-        <is>
-          <t>FY2025A</t>
-        </is>
-      </c>
-      <c r="F5" s="48" t="inlineStr">
-        <is>
-          <t>FY2026E</t>
-        </is>
-      </c>
-      <c r="G5" s="47" t="inlineStr">
-        <is>
-          <t>FY2027E</t>
-        </is>
-      </c>
-      <c r="H5" s="47" t="inlineStr">
-        <is>
-          <t>FY2028E</t>
-        </is>
-      </c>
-      <c r="I5" s="47" t="inlineStr">
-        <is>
-          <t>FY2029E</t>
-        </is>
-      </c>
-      <c r="J5" s="47" t="inlineStr">
-        <is>
-          <t>FY2030E</t>
-        </is>
-      </c>
-      <c r="K5" s="47" t="inlineStr">
-        <is>
-          <t>Units</t>
         </is>
       </c>
     </row>
@@ -3106,8 +3106,20 @@
           <t xml:space="preserve">  Americas — beginning stores</t>
         </is>
       </c>
-      <c r="E6" s="49" t="n">
+      <c r="B6" s="49" t="n">
         <v>462</v>
+      </c>
+      <c r="C6" s="35">
+        <f>B9</f>
+        <v/>
+      </c>
+      <c r="D6" s="35">
+        <f>C9</f>
+        <v/>
+      </c>
+      <c r="E6" s="35">
+        <f>D9</f>
+        <v/>
       </c>
       <c r="F6" s="35">
         <f>E9</f>
@@ -3117,19 +3129,7 @@
         <f>F9</f>
         <v/>
       </c>
-      <c r="H6" s="35">
-        <f>G9</f>
-        <v/>
-      </c>
-      <c r="I6" s="35">
-        <f>H9</f>
-        <v/>
-      </c>
-      <c r="J6" s="35">
-        <f>I9</f>
-        <v/>
-      </c>
-      <c r="K6" s="50" t="inlineStr">
+      <c r="H6" s="50" t="inlineStr">
         <is>
           <t>stores</t>
         </is>
@@ -3141,39 +3141,39 @@
           <t xml:space="preserve">  Americas — openings</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="C7" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" s="51" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="51" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="50" t="inlineStr">
+        <is>
+          <t>stores</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>Store openings skew to China (+20 FY26) vs mature Americas (+8). Anchored to FY25 +44 net stores and 11% sq-ft growth.</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="J7" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: store count &amp; expansion</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="K7" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Total company-operated stores" → 811 (FY25). FY25 added 44 net stores; model skews openings to China.</t>
-        </is>
-      </c>
-      <c r="F7" s="51" t="n">
-        <v>8</v>
-      </c>
-      <c r="G7" s="51" t="n">
-        <v>7</v>
-      </c>
-      <c r="H7" s="51" t="n">
-        <v>6</v>
-      </c>
-      <c r="I7" s="51" t="n">
-        <v>5</v>
-      </c>
-      <c r="J7" s="51" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="50" t="inlineStr">
-        <is>
-          <t>stores</t>
         </is>
       </c>
     </row>
@@ -3183,39 +3183,39 @@
           <t xml:space="preserve">  Americas — closures</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="C8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="50" t="inlineStr">
+        <is>
+          <t>stores</t>
+        </is>
+      </c>
+      <c r="I8" s="17" t="inlineStr">
         <is>
           <t>Closures assume 2–3 per mature region annually as leases roll; immaterial vs openings in expansion markets.</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="J8" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: lease renewal / fleet</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="K8" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "lease" / store fleet — immaterial closures vs expansion; 2–3 per mature region.</t>
-        </is>
-      </c>
-      <c r="F8" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="G8" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="H8" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="I8" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="J8" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" s="50" t="inlineStr">
-        <is>
-          <t>stores</t>
         </is>
       </c>
     </row>
@@ -3225,13 +3225,20 @@
           <t xml:space="preserve">  Americas — ending stores</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Americas" → FY2025 ending stores 476.</t>
-        </is>
-      </c>
-      <c r="E9" s="49" t="n">
+      <c r="B9" s="49" t="n">
         <v>476</v>
+      </c>
+      <c r="C9" s="53">
+        <f>C6+C7-C8</f>
+        <v/>
+      </c>
+      <c r="D9" s="53">
+        <f>D6+D7-D8</f>
+        <v/>
+      </c>
+      <c r="E9" s="53">
+        <f>E6+E7-E8</f>
+        <v/>
       </c>
       <c r="F9" s="53">
         <f>F6+F7-F8</f>
@@ -3241,21 +3248,14 @@
         <f>G6+G7-G8</f>
         <v/>
       </c>
-      <c r="H9" s="53">
-        <f>H6+H7-H8</f>
-        <v/>
-      </c>
-      <c r="I9" s="53">
-        <f>I6+I7-I8</f>
-        <v/>
-      </c>
-      <c r="J9" s="53">
-        <f>J6+J7-J8</f>
-        <v/>
-      </c>
-      <c r="K9" s="50" t="inlineStr">
+      <c r="H9" s="50" t="inlineStr">
         <is>
           <t>stores</t>
+        </is>
+      </c>
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Americas" → FY2025 ending stores 476.</t>
         </is>
       </c>
     </row>
@@ -3265,8 +3265,20 @@
           <t xml:space="preserve">  China Mainland — beginning stores</t>
         </is>
       </c>
-      <c r="E10" s="49" t="n">
+      <c r="B10" s="49" t="n">
         <v>151</v>
+      </c>
+      <c r="C10" s="35">
+        <f>B13</f>
+        <v/>
+      </c>
+      <c r="D10" s="35">
+        <f>C13</f>
+        <v/>
+      </c>
+      <c r="E10" s="35">
+        <f>D13</f>
+        <v/>
       </c>
       <c r="F10" s="35">
         <f>E13</f>
@@ -3276,19 +3288,7 @@
         <f>F13</f>
         <v/>
       </c>
-      <c r="H10" s="35">
-        <f>G13</f>
-        <v/>
-      </c>
-      <c r="I10" s="35">
-        <f>H13</f>
-        <v/>
-      </c>
-      <c r="J10" s="35">
-        <f>I13</f>
-        <v/>
-      </c>
-      <c r="K10" s="50" t="inlineStr">
+      <c r="H10" s="50" t="inlineStr">
         <is>
           <t>stores</t>
         </is>
@@ -3300,39 +3300,39 @@
           <t xml:space="preserve">  China Mainland — openings</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="C11" s="51" t="n">
+        <v>20</v>
+      </c>
+      <c r="D11" s="51" t="n">
+        <v>18</v>
+      </c>
+      <c r="E11" s="51" t="n">
+        <v>16</v>
+      </c>
+      <c r="F11" s="51" t="n">
+        <v>14</v>
+      </c>
+      <c r="G11" s="51" t="n">
+        <v>12</v>
+      </c>
+      <c r="H11" s="50" t="inlineStr">
+        <is>
+          <t>stores</t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>Store openings skew to China (+20 FY26) vs mature Americas (+8). Anchored to FY25 +44 net stores and 11% sq-ft growth.</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="J11" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: store count &amp; expansion</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="K11" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Total company-operated stores" → 811 (FY25). FY25 added 44 net stores; model skews openings to China.</t>
-        </is>
-      </c>
-      <c r="F11" s="51" t="n">
-        <v>20</v>
-      </c>
-      <c r="G11" s="51" t="n">
-        <v>18</v>
-      </c>
-      <c r="H11" s="51" t="n">
-        <v>16</v>
-      </c>
-      <c r="I11" s="51" t="n">
-        <v>14</v>
-      </c>
-      <c r="J11" s="51" t="n">
-        <v>12</v>
-      </c>
-      <c r="K11" s="50" t="inlineStr">
-        <is>
-          <t>stores</t>
         </is>
       </c>
     </row>
@@ -3342,20 +3342,14 @@
           <t xml:space="preserve">  China Mainland — closures</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>Closures assume 2–3 per mature region annually as leases roll; immaterial vs openings in expansion markets.</t>
-        </is>
-      </c>
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: lease renewal / fleet</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "lease" / store fleet — immaterial closures vs expansion; 2–3 per mature region.</t>
-        </is>
+      <c r="C12" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="51" t="n">
+        <v>1</v>
       </c>
       <c r="F12" s="51" t="n">
         <v>1</v>
@@ -3363,18 +3357,24 @@
       <c r="G12" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="50" t="inlineStr">
+      <c r="H12" s="50" t="inlineStr">
         <is>
           <t>stores</t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>Closures assume 2–3 per mature region annually as leases roll; immaterial vs openings in expansion markets.</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: lease renewal / fleet</t>
+        </is>
+      </c>
+      <c r="K12" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "lease" / store fleet — immaterial closures vs expansion; 2–3 per mature region.</t>
         </is>
       </c>
     </row>
@@ -3384,13 +3384,20 @@
           <t xml:space="preserve">  China Mainland — ending stores</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "China Mainland" → FY2025 ending stores 172.</t>
-        </is>
-      </c>
-      <c r="E13" s="49" t="n">
+      <c r="B13" s="49" t="n">
         <v>172</v>
+      </c>
+      <c r="C13" s="53">
+        <f>C10+C11-C12</f>
+        <v/>
+      </c>
+      <c r="D13" s="53">
+        <f>D10+D11-D12</f>
+        <v/>
+      </c>
+      <c r="E13" s="53">
+        <f>E10+E11-E12</f>
+        <v/>
       </c>
       <c r="F13" s="53">
         <f>F10+F11-F12</f>
@@ -3400,21 +3407,14 @@
         <f>G10+G11-G12</f>
         <v/>
       </c>
-      <c r="H13" s="53">
-        <f>H10+H11-H12</f>
-        <v/>
-      </c>
-      <c r="I13" s="53">
-        <f>I10+I11-I12</f>
-        <v/>
-      </c>
-      <c r="J13" s="53">
-        <f>J10+J11-J12</f>
-        <v/>
-      </c>
-      <c r="K13" s="50" t="inlineStr">
+      <c r="H13" s="50" t="inlineStr">
         <is>
           <t>stores</t>
+        </is>
+      </c>
+      <c r="K13" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "China Mainland" → FY2025 ending stores 172.</t>
         </is>
       </c>
     </row>
@@ -3424,8 +3424,20 @@
           <t xml:space="preserve">  Rest of World — beginning stores</t>
         </is>
       </c>
-      <c r="E14" s="49" t="n">
+      <c r="B14" s="49" t="n">
         <v>154</v>
+      </c>
+      <c r="C14" s="35">
+        <f>B17</f>
+        <v/>
+      </c>
+      <c r="D14" s="35">
+        <f>C17</f>
+        <v/>
+      </c>
+      <c r="E14" s="35">
+        <f>D17</f>
+        <v/>
       </c>
       <c r="F14" s="35">
         <f>E17</f>
@@ -3435,19 +3447,7 @@
         <f>F17</f>
         <v/>
       </c>
-      <c r="H14" s="35">
-        <f>G17</f>
-        <v/>
-      </c>
-      <c r="I14" s="35">
-        <f>H17</f>
-        <v/>
-      </c>
-      <c r="J14" s="35">
-        <f>I17</f>
-        <v/>
-      </c>
-      <c r="K14" s="50" t="inlineStr">
+      <c r="H14" s="50" t="inlineStr">
         <is>
           <t>stores</t>
         </is>
@@ -3459,39 +3459,39 @@
           <t xml:space="preserve">  Rest of World — openings</t>
         </is>
       </c>
-      <c r="B15" s="17" t="inlineStr">
+      <c r="C15" s="51" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" s="51" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" s="50" t="inlineStr">
+        <is>
+          <t>stores</t>
+        </is>
+      </c>
+      <c r="I15" s="17" t="inlineStr">
         <is>
           <t>Store openings skew to China (+20 FY26) vs mature Americas (+8). Anchored to FY25 +44 net stores and 11% sq-ft growth.</t>
         </is>
       </c>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="J15" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: store count &amp; expansion</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="K15" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Total company-operated stores" → 811 (FY25). FY25 added 44 net stores; model skews openings to China.</t>
-        </is>
-      </c>
-      <c r="F15" s="51" t="n">
-        <v>7</v>
-      </c>
-      <c r="G15" s="51" t="n">
-        <v>6</v>
-      </c>
-      <c r="H15" s="51" t="n">
-        <v>5</v>
-      </c>
-      <c r="I15" s="51" t="n">
-        <v>5</v>
-      </c>
-      <c r="J15" s="51" t="n">
-        <v>4</v>
-      </c>
-      <c r="K15" s="50" t="inlineStr">
-        <is>
-          <t>stores</t>
         </is>
       </c>
     </row>
@@ -3501,20 +3501,14 @@
           <t xml:space="preserve">  Rest of World — closures</t>
         </is>
       </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>Closures assume 2–3 per mature region annually as leases roll; immaterial vs openings in expansion markets.</t>
-        </is>
-      </c>
-      <c r="C16" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: lease renewal / fleet</t>
-        </is>
-      </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "lease" / store fleet — immaterial closures vs expansion; 2–3 per mature region.</t>
-        </is>
+      <c r="C16" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="51" t="n">
+        <v>2</v>
       </c>
       <c r="F16" s="51" t="n">
         <v>2</v>
@@ -3522,18 +3516,24 @@
       <c r="G16" s="51" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="I16" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="J16" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="K16" s="50" t="inlineStr">
+      <c r="H16" s="50" t="inlineStr">
         <is>
           <t>stores</t>
+        </is>
+      </c>
+      <c r="I16" s="17" t="inlineStr">
+        <is>
+          <t>Closures assume 2–3 per mature region annually as leases roll; immaterial vs openings in expansion markets.</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: lease renewal / fleet</t>
+        </is>
+      </c>
+      <c r="K16" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "lease" / store fleet — immaterial closures vs expansion; 2–3 per mature region.</t>
         </is>
       </c>
     </row>
@@ -3543,13 +3543,20 @@
           <t xml:space="preserve">  Rest of World — ending stores</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Rest of World" → FY2025 ending stores 163.</t>
-        </is>
-      </c>
-      <c r="E17" s="49" t="n">
+      <c r="B17" s="49" t="n">
         <v>163</v>
+      </c>
+      <c r="C17" s="53">
+        <f>C14+C15-C16</f>
+        <v/>
+      </c>
+      <c r="D17" s="53">
+        <f>D14+D15-D16</f>
+        <v/>
+      </c>
+      <c r="E17" s="53">
+        <f>E14+E15-E16</f>
+        <v/>
       </c>
       <c r="F17" s="53">
         <f>F14+F15-F16</f>
@@ -3559,21 +3566,14 @@
         <f>G14+G15-G16</f>
         <v/>
       </c>
-      <c r="H17" s="53">
-        <f>H14+H15-H16</f>
-        <v/>
-      </c>
-      <c r="I17" s="53">
-        <f>I14+I15-I16</f>
-        <v/>
-      </c>
-      <c r="J17" s="53">
-        <f>J14+J15-J16</f>
-        <v/>
-      </c>
-      <c r="K17" s="50" t="inlineStr">
+      <c r="H17" s="50" t="inlineStr">
         <is>
           <t>stores</t>
+        </is>
+      </c>
+      <c r="K17" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Rest of World" → FY2025 ending stores 163.</t>
         </is>
       </c>
     </row>
@@ -3583,8 +3583,20 @@
           <t>Total ending stores</t>
         </is>
       </c>
-      <c r="E18" s="54" t="n">
+      <c r="B18" s="54" t="n">
         <v>811</v>
+      </c>
+      <c r="C18" s="53">
+        <f>C9+C13+C17</f>
+        <v/>
+      </c>
+      <c r="D18" s="53">
+        <f>D9+D13+D17</f>
+        <v/>
+      </c>
+      <c r="E18" s="53">
+        <f>E9+E13+E17</f>
+        <v/>
       </c>
       <c r="F18" s="53">
         <f>F9+F13+F17</f>
@@ -3594,18 +3606,6 @@
         <f>G9+G13+G17</f>
         <v/>
       </c>
-      <c r="H18" s="53">
-        <f>H9+H13+H17</f>
-        <v/>
-      </c>
-      <c r="I18" s="53">
-        <f>I9+I13+I17</f>
-        <v/>
-      </c>
-      <c r="J18" s="53">
-        <f>J9+J13+J17</f>
-        <v/>
-      </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="34" t="inlineStr">
@@ -3613,42 +3613,42 @@
           <t>Avg square feet per store</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="B19" s="51" t="n">
+        <v>4366</v>
+      </c>
+      <c r="C19" s="51" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D19" s="51" t="n">
+        <v>4425</v>
+      </c>
+      <c r="E19" s="51" t="n">
+        <v>4450</v>
+      </c>
+      <c r="F19" s="51" t="n">
+        <v>4475</v>
+      </c>
+      <c r="G19" s="51" t="n">
+        <v>4500</v>
+      </c>
+      <c r="H19" s="50" t="inlineStr">
+        <is>
+          <t>sq ft</t>
+        </is>
+      </c>
+      <c r="I19" s="17" t="inlineStr">
         <is>
           <t>4,367 avg sq ft/store = implied FY25 total sq ft / 811 stores. Modest expansion to 4,500 by FY30.</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="J19" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: sales per square foot</t>
         </is>
       </c>
-      <c r="D19" s="19" t="inlineStr">
+      <c r="K19" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "sales per square foot were $1,426" → implied 3.54M sq ft / 811 stores ≈ 4,367 sq ft.</t>
-        </is>
-      </c>
-      <c r="E19" s="51" t="n">
-        <v>4366</v>
-      </c>
-      <c r="F19" s="51" t="n">
-        <v>4400</v>
-      </c>
-      <c r="G19" s="51" t="n">
-        <v>4425</v>
-      </c>
-      <c r="H19" s="51" t="n">
-        <v>4450</v>
-      </c>
-      <c r="I19" s="51" t="n">
-        <v>4475</v>
-      </c>
-      <c r="J19" s="51" t="n">
-        <v>4500</v>
-      </c>
-      <c r="K19" s="50" t="inlineStr">
-        <is>
-          <t>sq ft</t>
         </is>
       </c>
     </row>
@@ -3658,6 +3658,18 @@
           <t>Total square footage (end stores × avg sq ft)</t>
         </is>
       </c>
+      <c r="B20" s="35">
+        <f>B18*B19</f>
+        <v/>
+      </c>
+      <c r="C20" s="35">
+        <f>C18*C19</f>
+        <v/>
+      </c>
+      <c r="D20" s="35">
+        <f>D18*D19</f>
+        <v/>
+      </c>
       <c r="E20" s="35">
         <f>E18*E19</f>
         <v/>
@@ -3670,19 +3682,7 @@
         <f>G18*G19</f>
         <v/>
       </c>
-      <c r="H20" s="35">
-        <f>H18*H19</f>
-        <v/>
-      </c>
-      <c r="I20" s="35">
-        <f>I18*I19</f>
-        <v/>
-      </c>
-      <c r="J20" s="35">
-        <f>J18*J19</f>
-        <v/>
-      </c>
-      <c r="K20" s="50" t="inlineStr">
+      <c r="H20" s="50" t="inlineStr">
         <is>
           <t>sq ft</t>
         </is>
@@ -3703,52 +3703,52 @@
       </c>
       <c r="B23" s="46" t="inlineStr">
         <is>
+          <t>FY2025A</t>
+        </is>
+      </c>
+      <c r="C23" s="47" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="D23" s="46" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="E23" s="46" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="F23" s="46" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="G23" s="46" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+      <c r="H23" s="46" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="I23" s="48" t="inlineStr">
+        <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C23" s="46" t="inlineStr">
+      <c r="J23" s="48" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D23" s="46" t="inlineStr">
+      <c r="K23" s="48" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
-        </is>
-      </c>
-      <c r="E23" s="47" t="inlineStr">
-        <is>
-          <t>FY2025A</t>
-        </is>
-      </c>
-      <c r="F23" s="48" t="inlineStr">
-        <is>
-          <t>FY2026E</t>
-        </is>
-      </c>
-      <c r="G23" s="47" t="inlineStr">
-        <is>
-          <t>FY2027E</t>
-        </is>
-      </c>
-      <c r="H23" s="47" t="inlineStr">
-        <is>
-          <t>FY2028E</t>
-        </is>
-      </c>
-      <c r="I23" s="47" t="inlineStr">
-        <is>
-          <t>FY2029E</t>
-        </is>
-      </c>
-      <c r="J23" s="47" t="inlineStr">
-        <is>
-          <t>FY2030E</t>
-        </is>
-      </c>
-      <c r="K23" s="47" t="inlineStr">
-        <is>
-          <t>Units</t>
         </is>
       </c>
     </row>
@@ -3758,42 +3758,42 @@
           <t>Sales per square foot ($)</t>
         </is>
       </c>
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="51" t="n">
+        <v>1426</v>
+      </c>
+      <c r="C24" s="51" t="n">
+        <v>1360</v>
+      </c>
+      <c r="D24" s="51" t="n">
+        <v>1380</v>
+      </c>
+      <c r="E24" s="51" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F24" s="51" t="n">
+        <v>1420</v>
+      </c>
+      <c r="G24" s="51" t="n">
+        <v>1440</v>
+      </c>
+      <c r="H24" s="50" t="inlineStr">
+        <is>
+          <t>$/sq ft</t>
+        </is>
+      </c>
+      <c r="I24" s="17" t="inlineStr">
         <is>
           <t>FY26 SPSF $1,380 reflects Americas traffic/conversion pressure; recovers toward $1,440 by FY30.</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="J24" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: comparable sales &amp; SPSF</t>
         </is>
       </c>
-      <c r="D24" s="19" t="inlineStr">
+      <c r="K24" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "sales per square foot were $1,426" → FY25 reported $1,426; FY26 model $1,380 on traffic pressure.</t>
-        </is>
-      </c>
-      <c r="E24" s="51" t="n">
-        <v>1426</v>
-      </c>
-      <c r="F24" s="51" t="n">
-        <v>1360</v>
-      </c>
-      <c r="G24" s="51" t="n">
-        <v>1380</v>
-      </c>
-      <c r="H24" s="51" t="n">
-        <v>1400</v>
-      </c>
-      <c r="I24" s="51" t="n">
-        <v>1420</v>
-      </c>
-      <c r="J24" s="51" t="n">
-        <v>1440</v>
-      </c>
-      <c r="K24" s="50" t="inlineStr">
-        <is>
-          <t>$/sq ft</t>
         </is>
       </c>
     </row>
@@ -3803,42 +3803,42 @@
           <t xml:space="preserve">  Americas — comparable sales growth</t>
         </is>
       </c>
-      <c r="B25" s="17" t="inlineStr">
+      <c r="B25" s="55" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="C25" s="55" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="D25" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="55" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F25" s="55" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G25" s="55" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H25" s="50" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I25" s="17" t="inlineStr">
         <is>
           <t>FY25 Americas comp −3% per 10-K (traffic, conversion, AOV down). FY26 −4%: modest step-down before flat FY27 as promo clears.</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="J25" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: Americas comparable sales</t>
         </is>
       </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="K25" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Americas comparable sales decreased 3%" → FY25 anchor. FY26 model −4% before stabilization.</t>
-        </is>
-      </c>
-      <c r="E25" s="55" t="n">
-        <v>-0.03</v>
-      </c>
-      <c r="F25" s="55" t="n">
-        <v>-0.04</v>
-      </c>
-      <c r="G25" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="55" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="I25" s="55" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="J25" s="55" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="K25" s="50" t="inlineStr">
-        <is>
-          <t>%</t>
         </is>
       </c>
     </row>
@@ -3848,42 +3848,42 @@
           <t xml:space="preserve">  China Mainland — comparable sales growth</t>
         </is>
       </c>
-      <c r="B26" s="17" t="inlineStr">
+      <c r="B26" s="55" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C26" s="55" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D26" s="55" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E26" s="55" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F26" s="55" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G26" s="55" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H26" s="50" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I26" s="17" t="inlineStr">
         <is>
           <t>FY25 China comp +20% (+19% CCY) per 10-K. FY26 +14%: still fastest region but moderating as the store base scales.</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="J26" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: China Mainland comparable sales</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
+      <c r="K26" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "China Mainland comparable sales increased 20%" → FY25 anchor. FY26 model +14% on a larger base.</t>
-        </is>
-      </c>
-      <c r="E26" s="55" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F26" s="55" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="G26" s="55" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="H26" s="55" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I26" s="55" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="J26" s="55" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="K26" s="50" t="inlineStr">
-        <is>
-          <t>%</t>
         </is>
       </c>
     </row>
@@ -3893,42 +3893,42 @@
           <t xml:space="preserve">  Rest of World — comparable sales growth</t>
         </is>
       </c>
-      <c r="B27" s="17" t="inlineStr">
+      <c r="B27" s="55" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="C27" s="55" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D27" s="55" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E27" s="55" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F27" s="55" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G27" s="55" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H27" s="50" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I27" s="17" t="inlineStr">
         <is>
           <t>FY25 RoW comp +9% (+7% CCY) per 10-K. FY26 +7%: hold above CCY, fade to +4% by FY30 as APAC/Europe base matures.</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="J27" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: Rest of World comparable sales</t>
         </is>
       </c>
-      <c r="D27" s="19" t="inlineStr">
+      <c r="K27" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Rest of World comparable sales increased 9%" → FY25 +9% (+7% CCY). FY26 model +7%, fading to +4%.</t>
-        </is>
-      </c>
-      <c r="E27" s="55" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="F27" s="55" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="G27" s="55" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="H27" s="55" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="I27" s="55" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="J27" s="55" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="K27" s="50" t="inlineStr">
-        <is>
-          <t>%</t>
         </is>
       </c>
     </row>
@@ -3938,8 +3938,20 @@
           <t>Prior-year store channel revenue ($000)</t>
         </is>
       </c>
-      <c r="E28" s="56" t="n">
+      <c r="B28" s="56" t="n">
         <v>5049744</v>
+      </c>
+      <c r="C28" s="35">
+        <f>B31</f>
+        <v/>
+      </c>
+      <c r="D28" s="35">
+        <f>C31</f>
+        <v/>
+      </c>
+      <c r="E28" s="35">
+        <f>D31</f>
+        <v/>
       </c>
       <c r="F28" s="35">
         <f>E31</f>
@@ -3949,19 +3961,7 @@
         <f>F31</f>
         <v/>
       </c>
-      <c r="H28" s="35">
-        <f>G31</f>
-        <v/>
-      </c>
-      <c r="I28" s="35">
-        <f>H31</f>
-        <v/>
-      </c>
-      <c r="J28" s="35">
-        <f>I31</f>
-        <v/>
-      </c>
-      <c r="K28" s="50" t="inlineStr">
+      <c r="H28" s="50" t="inlineStr">
         <is>
           <t>$000</t>
         </is>
@@ -3973,8 +3973,20 @@
           <t>Comparable store revenue ($000)</t>
         </is>
       </c>
-      <c r="E29" s="49" t="n">
+      <c r="B29" s="49" t="n">
         <v>5049744</v>
+      </c>
+      <c r="C29" s="35">
+        <f>B28*0.71*(1+C25)+B28*0.16*(1+C26)+B28*0.13*(1+C27)</f>
+        <v/>
+      </c>
+      <c r="D29" s="35">
+        <f>C28*0.71*(1+D25)+C28*0.16*(1+D26)+C28*0.13*(1+D27)</f>
+        <v/>
+      </c>
+      <c r="E29" s="35">
+        <f>D28*0.71*(1+E25)+D28*0.16*(1+E26)+D28*0.13*(1+E27)</f>
+        <v/>
       </c>
       <c r="F29" s="35">
         <f>E28*0.71*(1+F25)+E28*0.16*(1+F26)+E28*0.13*(1+F27)</f>
@@ -3984,18 +3996,6 @@
         <f>F28*0.71*(1+G25)+F28*0.16*(1+G26)+F28*0.13*(1+G27)</f>
         <v/>
       </c>
-      <c r="H29" s="35">
-        <f>G28*0.71*(1+H25)+G28*0.16*(1+H26)+G28*0.13*(1+H27)</f>
-        <v/>
-      </c>
-      <c r="I29" s="35">
-        <f>H28*0.71*(1+I25)+H28*0.16*(1+I26)+H28*0.13*(1+I27)</f>
-        <v/>
-      </c>
-      <c r="J29" s="35">
-        <f>I28*0.71*(1+J25)+I28*0.16*(1+J26)+I28*0.13*(1+J27)</f>
-        <v/>
-      </c>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="34" t="inlineStr">
@@ -4003,23 +4003,20 @@
           <t>Net new store revenue contribution ($000)</t>
         </is>
       </c>
-      <c r="B30" s="17" t="inlineStr">
-        <is>
-          <t>New-store contribution = net openings × sq ft × SPSF × 55% first-year ramp (standard retail maturity).</t>
-        </is>
-      </c>
-      <c r="C30" s="57" t="inlineStr">
-        <is>
-          <t>Revenue Drivers tab: formula</t>
-        </is>
-      </c>
-      <c r="D30" s="19" t="inlineStr">
-        <is>
-          <t>Formula: net openings × sq ft × SPSF / 1000 × 55% ramp. Not a sourced print.</t>
-        </is>
-      </c>
-      <c r="E30" s="35" t="n">
+      <c r="B30" s="35" t="n">
         <v>0</v>
+      </c>
+      <c r="C30" s="35">
+        <f>(C7-C8+C11-C12+C15-C16)*C19*C24/1000*0.55</f>
+        <v/>
+      </c>
+      <c r="D30" s="35">
+        <f>(D7-D8+D11-D12+D15-D16)*D19*D24/1000*0.55</f>
+        <v/>
+      </c>
+      <c r="E30" s="35">
+        <f>(E7-E8+E11-E12+E15-E16)*E19*E24/1000*0.55</f>
+        <v/>
       </c>
       <c r="F30" s="35">
         <f>(F7-F8+F11-F12+F15-F16)*F19*F24/1000*0.55</f>
@@ -4029,17 +4026,20 @@
         <f>(G7-G8+G11-G12+G15-G16)*G19*G24/1000*0.55</f>
         <v/>
       </c>
-      <c r="H30" s="35">
-        <f>(H7-H8+H11-H12+H15-H16)*H19*H24/1000*0.55</f>
-        <v/>
-      </c>
-      <c r="I30" s="35">
-        <f>(I7-I8+I11-I12+I15-I16)*I19*I24/1000*0.55</f>
-        <v/>
-      </c>
-      <c r="J30" s="35">
-        <f>(J7-J8+J11-J12+J15-J16)*J19*J24/1000*0.55</f>
-        <v/>
+      <c r="I30" s="17" t="inlineStr">
+        <is>
+          <t>New-store contribution = net openings × sq ft × SPSF × 55% first-year ramp (standard retail maturity).</t>
+        </is>
+      </c>
+      <c r="J30" s="57" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab: formula</t>
+        </is>
+      </c>
+      <c r="K30" s="19" t="inlineStr">
+        <is>
+          <t>Formula: net openings × sq ft × SPSF / 1000 × 55% ramp. Not a sourced print.</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -4048,8 +4048,20 @@
           <t>Store channel revenue ($000)</t>
         </is>
       </c>
-      <c r="E31" s="54" t="n">
+      <c r="B31" s="54" t="n">
         <v>5049744</v>
+      </c>
+      <c r="C31" s="53">
+        <f>C29+C30</f>
+        <v/>
+      </c>
+      <c r="D31" s="53">
+        <f>D29+D30</f>
+        <v/>
+      </c>
+      <c r="E31" s="53">
+        <f>E29+E30</f>
+        <v/>
       </c>
       <c r="F31" s="53">
         <f>F29+F30</f>
@@ -4059,18 +4071,6 @@
         <f>G29+G30</f>
         <v/>
       </c>
-      <c r="H31" s="53">
-        <f>H29+H30</f>
-        <v/>
-      </c>
-      <c r="I31" s="53">
-        <f>I29+I30</f>
-        <v/>
-      </c>
-      <c r="J31" s="53">
-        <f>J29+J30</f>
-        <v/>
-      </c>
     </row>
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="34" t="inlineStr">
@@ -4078,42 +4078,42 @@
           <t xml:space="preserve">  memo: fleet traffic (millions of visits)</t>
         </is>
       </c>
-      <c r="B32" s="17" t="inlineStr">
+      <c r="B32" s="58" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="C32" s="58" t="n">
+        <v>40</v>
+      </c>
+      <c r="D32" s="58" t="n">
+        <v>41</v>
+      </c>
+      <c r="E32" s="58" t="n">
+        <v>42</v>
+      </c>
+      <c r="F32" s="58" t="n">
+        <v>43</v>
+      </c>
+      <c r="G32" s="58" t="n">
+        <v>44</v>
+      </c>
+      <c r="H32" s="50" t="inlineStr">
+        <is>
+          <t>M visits</t>
+        </is>
+      </c>
+      <c r="I32" s="17" t="inlineStr">
         <is>
           <t>Fleet traffic memo line — not a separate FCF item. Calibrated to FY25 store productivity commentary.</t>
         </is>
       </c>
-      <c r="C32" s="18" t="inlineStr">
+      <c r="J32" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: store traffic commentary</t>
         </is>
       </c>
-      <c r="D32" s="19" t="inlineStr">
+      <c r="K32" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "store traffic" → lower traffic in Americas; memo line only.</t>
-        </is>
-      </c>
-      <c r="E32" s="58" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="F32" s="58" t="n">
-        <v>40</v>
-      </c>
-      <c r="G32" s="58" t="n">
-        <v>41</v>
-      </c>
-      <c r="H32" s="58" t="n">
-        <v>42</v>
-      </c>
-      <c r="I32" s="58" t="n">
-        <v>43</v>
-      </c>
-      <c r="J32" s="58" t="n">
-        <v>44</v>
-      </c>
-      <c r="K32" s="50" t="inlineStr">
-        <is>
-          <t>M visits</t>
         </is>
       </c>
     </row>
@@ -4123,38 +4123,38 @@
           <t xml:space="preserve">  memo: in-store conversion rate</t>
         </is>
       </c>
-      <c r="B33" s="17" t="inlineStr">
-        <is>
-          <t>In-store conversion memo — 10-K cites lower conversion in Americas; FY26 27% improving to 29%.</t>
-        </is>
-      </c>
-      <c r="C33" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: conversion rate commentary</t>
-        </is>
-      </c>
-      <c r="D33" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "conversion rates" → lower in Americas; in-store memo 27%→29%.</t>
-        </is>
+      <c r="B33" s="55" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C33" s="55" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="D33" s="55" t="n">
+        <v>0.275</v>
       </c>
       <c r="E33" s="55" t="n">
         <v>0.28</v>
       </c>
       <c r="F33" s="55" t="n">
-        <v>0.27</v>
+        <v>0.285</v>
       </c>
       <c r="G33" s="55" t="n">
-        <v>0.275</v>
-      </c>
-      <c r="H33" s="55" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="I33" s="55" t="n">
-        <v>0.285</v>
-      </c>
-      <c r="J33" s="55" t="n">
         <v>0.29</v>
+      </c>
+      <c r="I33" s="17" t="inlineStr">
+        <is>
+          <t>In-store conversion memo — 10-K cites lower conversion in Americas; FY26 27% improving to 29%.</t>
+        </is>
+      </c>
+      <c r="J33" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: conversion rate commentary</t>
+        </is>
+      </c>
+      <c r="K33" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "conversion rates" → lower in Americas; in-store memo 27%→29%.</t>
+        </is>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
@@ -4163,38 +4163,38 @@
           <t xml:space="preserve">  memo: in-store average transaction ($)</t>
         </is>
       </c>
-      <c r="B34" s="17" t="inlineStr">
-        <is>
-          <t>In-store average transaction $115–$122; supports SPSF and comp-sales bridge on the driver tab.</t>
-        </is>
-      </c>
-      <c r="C34" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: average order value commentary</t>
-        </is>
-      </c>
-      <c r="D34" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "average order value" → lower AOV in Americas; memo $115–$122.</t>
-        </is>
+      <c r="B34" s="59" t="n">
+        <v>118</v>
+      </c>
+      <c r="C34" s="59" t="n">
+        <v>115</v>
+      </c>
+      <c r="D34" s="59" t="n">
+        <v>116</v>
       </c>
       <c r="E34" s="59" t="n">
         <v>118</v>
       </c>
       <c r="F34" s="59" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="G34" s="59" t="n">
-        <v>116</v>
-      </c>
-      <c r="H34" s="59" t="n">
-        <v>118</v>
-      </c>
-      <c r="I34" s="59" t="n">
-        <v>120</v>
-      </c>
-      <c r="J34" s="59" t="n">
         <v>122</v>
+      </c>
+      <c r="I34" s="17" t="inlineStr">
+        <is>
+          <t>In-store average transaction $115–$122; supports SPSF and comp-sales bridge on the driver tab.</t>
+        </is>
+      </c>
+      <c r="J34" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: average order value commentary</t>
+        </is>
+      </c>
+      <c r="K34" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "average order value" → lower AOV in Americas; memo $115–$122.</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -4212,52 +4212,52 @@
       </c>
       <c r="B37" s="46" t="inlineStr">
         <is>
+          <t>FY2025A</t>
+        </is>
+      </c>
+      <c r="C37" s="47" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="D37" s="46" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="E37" s="46" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="F37" s="46" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="G37" s="46" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+      <c r="H37" s="46" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="I37" s="48" t="inlineStr">
+        <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C37" s="46" t="inlineStr">
+      <c r="J37" s="48" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D37" s="46" t="inlineStr">
+      <c r="K37" s="48" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
-        </is>
-      </c>
-      <c r="E37" s="47" t="inlineStr">
-        <is>
-          <t>FY2025A</t>
-        </is>
-      </c>
-      <c r="F37" s="48" t="inlineStr">
-        <is>
-          <t>FY2026E</t>
-        </is>
-      </c>
-      <c r="G37" s="47" t="inlineStr">
-        <is>
-          <t>FY2027E</t>
-        </is>
-      </c>
-      <c r="H37" s="47" t="inlineStr">
-        <is>
-          <t>FY2028E</t>
-        </is>
-      </c>
-      <c r="I37" s="47" t="inlineStr">
-        <is>
-          <t>FY2029E</t>
-        </is>
-      </c>
-      <c r="J37" s="47" t="inlineStr">
-        <is>
-          <t>FY2030E</t>
-        </is>
-      </c>
-      <c r="K37" s="47" t="inlineStr">
-        <is>
-          <t>Units</t>
         </is>
       </c>
     </row>
@@ -4267,42 +4267,42 @@
           <t>Unique digital sessions (millions)</t>
         </is>
       </c>
-      <c r="B38" s="17" t="inlineStr">
+      <c r="B38" s="51" t="n">
+        <v>485</v>
+      </c>
+      <c r="C38" s="51" t="n">
+        <v>485</v>
+      </c>
+      <c r="D38" s="51" t="n">
+        <v>505</v>
+      </c>
+      <c r="E38" s="51" t="n">
+        <v>525</v>
+      </c>
+      <c r="F38" s="51" t="n">
+        <v>545</v>
+      </c>
+      <c r="G38" s="51" t="n">
+        <v>560</v>
+      </c>
+      <c r="H38" s="50" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I38" s="17" t="inlineStr">
         <is>
           <t>485M FY25 sessions implied from reported e-comm revenue / conv / AOV. FY26 −3% on Americas softness.</t>
         </is>
       </c>
-      <c r="C38" s="18" t="inlineStr">
+      <c r="J38" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: e-commerce revenue</t>
         </is>
       </c>
-      <c r="D38" s="19" t="inlineStr">
+      <c r="K38" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "E-commerce" → 4,918,697 ($000). Sessions implied from revenue / conv / AOV.</t>
-        </is>
-      </c>
-      <c r="E38" s="51" t="n">
-        <v>485</v>
-      </c>
-      <c r="F38" s="51" t="n">
-        <v>485</v>
-      </c>
-      <c r="G38" s="51" t="n">
-        <v>505</v>
-      </c>
-      <c r="H38" s="51" t="n">
-        <v>525</v>
-      </c>
-      <c r="I38" s="51" t="n">
-        <v>545</v>
-      </c>
-      <c r="J38" s="51" t="n">
-        <v>560</v>
-      </c>
-      <c r="K38" s="50" t="inlineStr">
-        <is>
-          <t>M</t>
         </is>
       </c>
     </row>
@@ -4312,38 +4312,38 @@
           <t>Digital conversion rate</t>
         </is>
       </c>
-      <c r="B39" s="17" t="inlineStr">
+      <c r="B39" s="55" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="C39" s="55" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="D39" s="55" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="E39" s="55" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="F39" s="55" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="G39" s="55" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="I39" s="17" t="inlineStr">
         <is>
           <t>3.3% FY26 digital conversion vs 3.5% pressure cited in 10-K Americas; gradual recovery to 3.6%.</t>
         </is>
       </c>
-      <c r="C39" s="18" t="inlineStr">
+      <c r="J39" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: digital / traffic commentary</t>
         </is>
       </c>
-      <c r="D39" s="19" t="inlineStr">
+      <c r="K39" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "lower conversion rates" (Americas MD&amp;A). FY26 model 3.3% digital conversion.</t>
         </is>
-      </c>
-      <c r="E39" s="55" t="n">
-        <v>0.033</v>
-      </c>
-      <c r="F39" s="55" t="n">
-        <v>0.033</v>
-      </c>
-      <c r="G39" s="55" t="n">
-        <v>0.034</v>
-      </c>
-      <c r="H39" s="55" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="I39" s="55" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="J39" s="55" t="n">
-        <v>0.036</v>
       </c>
     </row>
     <row r="40" ht="28" customHeight="1">
@@ -4352,38 +4352,38 @@
           <t>Digital average order value ($)</t>
         </is>
       </c>
-      <c r="B40" s="17" t="inlineStr">
+      <c r="B40" s="59" t="n">
+        <v>307</v>
+      </c>
+      <c r="C40" s="59" t="n">
+        <v>305</v>
+      </c>
+      <c r="D40" s="59" t="n">
+        <v>308</v>
+      </c>
+      <c r="E40" s="59" t="n">
+        <v>310</v>
+      </c>
+      <c r="F40" s="59" t="n">
+        <v>312</v>
+      </c>
+      <c r="G40" s="59" t="n">
+        <v>315</v>
+      </c>
+      <c r="I40" s="17" t="inlineStr">
         <is>
           <t>AOV $305 FY26 on promo intensity; steps to $315 by FY30 as mix normalizes.</t>
         </is>
       </c>
-      <c r="C40" s="18" t="inlineStr">
+      <c r="J40" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: e-commerce revenue</t>
         </is>
       </c>
-      <c r="D40" s="19" t="inlineStr">
+      <c r="K40" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "average order value" (Americas MD&amp;A). FY26 model $305 AOV.</t>
         </is>
-      </c>
-      <c r="E40" s="59" t="n">
-        <v>307</v>
-      </c>
-      <c r="F40" s="59" t="n">
-        <v>305</v>
-      </c>
-      <c r="G40" s="59" t="n">
-        <v>308</v>
-      </c>
-      <c r="H40" s="59" t="n">
-        <v>310</v>
-      </c>
-      <c r="I40" s="59" t="n">
-        <v>312</v>
-      </c>
-      <c r="J40" s="59" t="n">
-        <v>315</v>
       </c>
     </row>
     <row r="41" ht="28" customHeight="1">
@@ -4392,13 +4392,20 @@
           <t>E-commerce revenue ($000)</t>
         </is>
       </c>
-      <c r="D41" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "E-commerce" → 4,918,697 ($000 FY2025). Forward = sessions × conversion × AOV.</t>
-        </is>
-      </c>
-      <c r="E41" s="54" t="n">
+      <c r="B41" s="54" t="n">
         <v>4918697</v>
+      </c>
+      <c r="C41" s="53">
+        <f>C38*1000000*C39*C40/1000</f>
+        <v/>
+      </c>
+      <c r="D41" s="53">
+        <f>D38*1000000*D39*D40/1000</f>
+        <v/>
+      </c>
+      <c r="E41" s="53">
+        <f>E38*1000000*E39*E40/1000</f>
+        <v/>
       </c>
       <c r="F41" s="53">
         <f>F38*1000000*F39*F40/1000</f>
@@ -4408,17 +4415,10 @@
         <f>G38*1000000*G39*G40/1000</f>
         <v/>
       </c>
-      <c r="H41" s="53">
-        <f>H38*1000000*H39*H40/1000</f>
-        <v/>
-      </c>
-      <c r="I41" s="53">
-        <f>I38*1000000*I39*I40/1000</f>
-        <v/>
-      </c>
-      <c r="J41" s="53">
-        <f>J38*1000000*J39*J40/1000</f>
-        <v/>
+      <c r="K41" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "E-commerce" → 4,918,697 ($000 FY2025). Forward = sessions × conversion × AOV.</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -4436,52 +4436,52 @@
       </c>
       <c r="B44" s="46" t="inlineStr">
         <is>
+          <t>FY2025A</t>
+        </is>
+      </c>
+      <c r="C44" s="47" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="D44" s="46" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="E44" s="46" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="F44" s="46" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="G44" s="46" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+      <c r="H44" s="46" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="I44" s="48" t="inlineStr">
+        <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C44" s="46" t="inlineStr">
+      <c r="J44" s="48" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D44" s="46" t="inlineStr">
+      <c r="K44" s="48" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
-        </is>
-      </c>
-      <c r="E44" s="47" t="inlineStr">
-        <is>
-          <t>FY2025A</t>
-        </is>
-      </c>
-      <c r="F44" s="48" t="inlineStr">
-        <is>
-          <t>FY2026E</t>
-        </is>
-      </c>
-      <c r="G44" s="47" t="inlineStr">
-        <is>
-          <t>FY2027E</t>
-        </is>
-      </c>
-      <c r="H44" s="47" t="inlineStr">
-        <is>
-          <t>FY2028E</t>
-        </is>
-      </c>
-      <c r="I44" s="47" t="inlineStr">
-        <is>
-          <t>FY2029E</t>
-        </is>
-      </c>
-      <c r="J44" s="47" t="inlineStr">
-        <is>
-          <t>FY2030E</t>
-        </is>
-      </c>
-      <c r="K44" s="47" t="inlineStr">
-        <is>
-          <t>Units</t>
         </is>
       </c>
     </row>
@@ -4491,47 +4491,47 @@
           <t>Other channels (wholesale / license / outlets) ($000)</t>
         </is>
       </c>
-      <c r="B45" s="17" t="inlineStr">
+      <c r="B45" s="56" t="n">
+        <v>1134159</v>
+      </c>
+      <c r="C45" s="35">
+        <f>B45*(1+-0.02)</f>
+        <v/>
+      </c>
+      <c r="D45" s="35">
+        <f>C45*(1+0.0)</f>
+        <v/>
+      </c>
+      <c r="E45" s="35">
+        <f>D45*(1+0.02)</f>
+        <v/>
+      </c>
+      <c r="F45" s="35">
+        <f>E45*(1+0.02)</f>
+        <v/>
+      </c>
+      <c r="G45" s="35">
+        <f>F45*(1+0.02)</f>
+        <v/>
+      </c>
+      <c r="H45" s="50" t="inlineStr">
+        <is>
+          <t>$000</t>
+        </is>
+      </c>
+      <c r="I45" s="17" t="inlineStr">
         <is>
           <t>Other channels (wholesale/license/outlets) held at FY25 $1.13B base; low-single-digit growth thereafter.</t>
         </is>
       </c>
-      <c r="C45" s="18" t="inlineStr">
+      <c r="J45" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: channel revenue table</t>
         </is>
       </c>
-      <c r="D45" s="19" t="inlineStr">
+      <c r="K45" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Company-operated stores" and "E-commerce" → residual other channels ≈ $1.13B.</t>
-        </is>
-      </c>
-      <c r="E45" s="56" t="n">
-        <v>1134159</v>
-      </c>
-      <c r="F45" s="35">
-        <f>E45*(1+-0.02)</f>
-        <v/>
-      </c>
-      <c r="G45" s="35">
-        <f>F45*(1+0.0)</f>
-        <v/>
-      </c>
-      <c r="H45" s="35">
-        <f>G45*(1+0.02)</f>
-        <v/>
-      </c>
-      <c r="I45" s="35">
-        <f>H45*(1+0.02)</f>
-        <v/>
-      </c>
-      <c r="J45" s="35">
-        <f>I45*(1+0.02)</f>
-        <v/>
-      </c>
-      <c r="K45" s="50" t="inlineStr">
-        <is>
-          <t>$000</t>
         </is>
       </c>
     </row>
@@ -4541,47 +4541,47 @@
           <t xml:space="preserve">  Americas net revenue ($000)</t>
         </is>
       </c>
-      <c r="B46" s="17" t="inlineStr">
+      <c r="B46" s="56" t="n">
+        <v>7847044</v>
+      </c>
+      <c r="C46" s="35">
+        <f>B46*(C31+C41+C45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="D46" s="35">
+        <f>B46*(D31+D41+D45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="E46" s="35">
+        <f>B46*(E31+E41+E45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="F46" s="35">
+        <f>B46*(F31+F41+F45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="G46" s="35">
+        <f>B46*(G31+G41+G45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="H46" s="50" t="inlineStr">
+        <is>
+          <t>$000</t>
+        </is>
+      </c>
+      <c r="I46" s="17" t="inlineStr">
         <is>
           <t>Geographic split scales with consolidated growth; FY25 Americas 70.7% of revenue per 10-K segment table.</t>
         </is>
       </c>
-      <c r="C46" s="18" t="inlineStr">
+      <c r="J46" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
-      <c r="D46" s="19" t="inlineStr">
+      <c r="K46" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Americas" segment table → $7,847,044 net revenue (70.7%).</t>
-        </is>
-      </c>
-      <c r="E46" s="56" t="n">
-        <v>7847044</v>
-      </c>
-      <c r="F46" s="35">
-        <f>E46*(F31+F41+F45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="G46" s="35">
-        <f>E46*(G31+G41+G45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="H46" s="35">
-        <f>E46*(H31+H41+H45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="I46" s="35">
-        <f>E46*(I31+I41+I45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="J46" s="35">
-        <f>E46*(J31+J41+J45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="K46" s="50" t="inlineStr">
-        <is>
-          <t>$000</t>
         </is>
       </c>
     </row>
@@ -4591,47 +4591,47 @@
           <t xml:space="preserve">  China Mainland net revenue ($000)</t>
         </is>
       </c>
-      <c r="B47" s="17" t="inlineStr">
+      <c r="B47" s="56" t="n">
+        <v>1754799</v>
+      </c>
+      <c r="C47" s="35">
+        <f>B47*(C31+C41+C45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="D47" s="35">
+        <f>B47*(D31+D41+D45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="E47" s="35">
+        <f>B47*(E31+E41+E45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="F47" s="35">
+        <f>B47*(F31+F41+F45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="G47" s="35">
+        <f>B47*(G31+G41+G45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="H47" s="50" t="inlineStr">
+        <is>
+          <t>$000</t>
+        </is>
+      </c>
+      <c r="I47" s="17" t="inlineStr">
         <is>
           <t>China 15.8% of FY25 revenue; fastest comp and store growth — expansion market in the driver schedule.</t>
         </is>
       </c>
-      <c r="C47" s="18" t="inlineStr">
+      <c r="J47" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
-      <c r="D47" s="19" t="inlineStr">
+      <c r="K47" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "China Mainland" segment → $1,754,799 net revenue (15.8%).</t>
-        </is>
-      </c>
-      <c r="E47" s="56" t="n">
-        <v>1754799</v>
-      </c>
-      <c r="F47" s="35">
-        <f>E47*(F31+F41+F45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="G47" s="35">
-        <f>E47*(G31+G41+G45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="H47" s="35">
-        <f>E47*(H31+H41+H45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="I47" s="35">
-        <f>E47*(I31+I41+I45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="J47" s="35">
-        <f>E47*(J31+J41+J45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="K47" s="50" t="inlineStr">
-        <is>
-          <t>$000</t>
         </is>
       </c>
     </row>
@@ -4641,47 +4641,47 @@
           <t xml:space="preserve">  Rest of World net revenue ($000)</t>
         </is>
       </c>
-      <c r="B48" s="17" t="inlineStr">
+      <c r="B48" s="56" t="n">
+        <v>1500757</v>
+      </c>
+      <c r="C48" s="35">
+        <f>B48*(C31+C41+C45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="D48" s="35">
+        <f>B48*(D31+D41+D45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="E48" s="35">
+        <f>B48*(E31+E41+E45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="F48" s="35">
+        <f>B48*(F31+F41+F45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="G48" s="35">
+        <f>B48*(G31+G41+G45)/(B31+B41+B45)</f>
+        <v/>
+      </c>
+      <c r="H48" s="50" t="inlineStr">
+        <is>
+          <t>$000</t>
+        </is>
+      </c>
+      <c r="I48" s="17" t="inlineStr">
         <is>
           <t>Rest of World 13.5% of FY25 revenue; mid-single-digit comps and steady openings.</t>
         </is>
       </c>
-      <c r="C48" s="18" t="inlineStr">
+      <c r="J48" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
-      <c r="D48" s="19" t="inlineStr">
+      <c r="K48" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Rest of World" segment → $1,500,757 net revenue (13.5%).</t>
-        </is>
-      </c>
-      <c r="E48" s="56" t="n">
-        <v>1500757</v>
-      </c>
-      <c r="F48" s="35">
-        <f>E48*(F31+F41+F45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="G48" s="35">
-        <f>E48*(G31+G41+G45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="H48" s="35">
-        <f>E48*(H31+H41+H45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="I48" s="35">
-        <f>E48*(I31+I41+I45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="J48" s="35">
-        <f>E48*(J31+J41+J45)/(E31+E41+E45)</f>
-        <v/>
-      </c>
-      <c r="K48" s="50" t="inlineStr">
-        <is>
-          <t>$000</t>
         </is>
       </c>
     </row>
@@ -4691,38 +4691,38 @@
           <t>Women's % of revenue</t>
         </is>
       </c>
-      <c r="B49" s="17" t="inlineStr">
+      <c r="B49" s="55" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="C49" s="55" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D49" s="55" t="n">
+        <v>0.615</v>
+      </c>
+      <c r="E49" s="55" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F49" s="55" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="G49" s="55" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I49" s="17" t="inlineStr">
         <is>
           <t>Women's mix fades 62.5%→60% as men's penetrates; FY25 reported 63% women's per 10-K category disclosure.</t>
         </is>
       </c>
-      <c r="C49" s="18" t="inlineStr">
+      <c r="J49" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: product category mix</t>
         </is>
       </c>
-      <c r="D49" s="19" t="inlineStr">
+      <c r="K49" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "women's, men's, and accessories" → 63% / 24% / 13% of net revenue.</t>
         </is>
-      </c>
-      <c r="E49" s="55" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="F49" s="55" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="G49" s="55" t="n">
-        <v>0.615</v>
-      </c>
-      <c r="H49" s="55" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="I49" s="55" t="n">
-        <v>0.605</v>
-      </c>
-      <c r="J49" s="55" t="n">
-        <v>0.6</v>
       </c>
     </row>
     <row r="50" ht="28" customHeight="1">
@@ -4731,38 +4731,38 @@
           <t>Men's % of revenue</t>
         </is>
       </c>
-      <c r="B50" s="17" t="inlineStr">
+      <c r="B50" s="55" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="C50" s="55" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D50" s="55" t="n">
+        <v>0.255</v>
+      </c>
+      <c r="E50" s="55" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F50" s="55" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="G50" s="55" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="I50" s="17" t="inlineStr">
         <is>
           <t>Men's mix rises 24.5%→27%; FY25 men's grew 4% vs women's 5% per 10-K category commentary.</t>
         </is>
       </c>
-      <c r="C50" s="18" t="inlineStr">
+      <c r="J50" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: product category mix</t>
         </is>
       </c>
-      <c r="D50" s="19" t="inlineStr">
+      <c r="K50" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "men's" category growth 4% in MD&amp;A; mix rises to 27% by FY30.</t>
         </is>
-      </c>
-      <c r="E50" s="55" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="F50" s="55" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G50" s="55" t="n">
-        <v>0.255</v>
-      </c>
-      <c r="H50" s="55" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="I50" s="55" t="n">
-        <v>0.265</v>
-      </c>
-      <c r="J50" s="55" t="n">
-        <v>0.27</v>
       </c>
     </row>
     <row r="51" ht="28" customHeight="1">
@@ -4771,20 +4771,14 @@
           <t>Accessories &amp; other % of revenue</t>
         </is>
       </c>
-      <c r="B51" s="17" t="inlineStr">
-        <is>
-          <t>Accessories steady at 13% of revenue; FY25 accessories +8% per 10-K category disclosure.</t>
-        </is>
-      </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: product category mix</t>
-        </is>
-      </c>
-      <c r="D51" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "accessories" +8% category growth; hold 13% mix.</t>
-        </is>
+      <c r="B51" s="55" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="C51" s="55" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D51" s="55" t="n">
+        <v>0.13</v>
       </c>
       <c r="E51" s="55" t="n">
         <v>0.13</v>
@@ -4795,14 +4789,20 @@
       <c r="G51" s="55" t="n">
         <v>0.13</v>
       </c>
-      <c r="H51" s="55" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="I51" s="55" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="J51" s="55" t="n">
-        <v>0.13</v>
+      <c r="I51" s="17" t="inlineStr">
+        <is>
+          <t>Accessories steady at 13% of revenue; FY25 accessories +8% per 10-K category disclosure.</t>
+        </is>
+      </c>
+      <c r="J51" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: product category mix</t>
+        </is>
+      </c>
+      <c r="K51" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "accessories" +8% category growth; hold 13% mix.</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -4820,52 +4820,52 @@
       </c>
       <c r="B54" s="46" t="inlineStr">
         <is>
+          <t>FY2025A</t>
+        </is>
+      </c>
+      <c r="C54" s="47" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="D54" s="46" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="E54" s="46" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="F54" s="46" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="G54" s="46" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+      <c r="H54" s="46" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="I54" s="48" t="inlineStr">
+        <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C54" s="46" t="inlineStr">
+      <c r="J54" s="48" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D54" s="46" t="inlineStr">
+      <c r="K54" s="48" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
-        </is>
-      </c>
-      <c r="E54" s="47" t="inlineStr">
-        <is>
-          <t>FY2025A</t>
-        </is>
-      </c>
-      <c r="F54" s="48" t="inlineStr">
-        <is>
-          <t>FY2026E</t>
-        </is>
-      </c>
-      <c r="G54" s="47" t="inlineStr">
-        <is>
-          <t>FY2027E</t>
-        </is>
-      </c>
-      <c r="H54" s="47" t="inlineStr">
-        <is>
-          <t>FY2028E</t>
-        </is>
-      </c>
-      <c r="I54" s="47" t="inlineStr">
-        <is>
-          <t>FY2029E</t>
-        </is>
-      </c>
-      <c r="J54" s="47" t="inlineStr">
-        <is>
-          <t>FY2030E</t>
-        </is>
-      </c>
-      <c r="K54" s="47" t="inlineStr">
-        <is>
-          <t>Units</t>
         </is>
       </c>
     </row>
@@ -4875,8 +4875,20 @@
           <t>Bottom-up total revenue ($000)</t>
         </is>
       </c>
-      <c r="E55" s="61" t="n">
+      <c r="B55" s="61" t="n">
         <v>11102600</v>
+      </c>
+      <c r="C55" s="62">
+        <f>C31+C41+C45</f>
+        <v/>
+      </c>
+      <c r="D55" s="62">
+        <f>D31+D41+D45</f>
+        <v/>
+      </c>
+      <c r="E55" s="62">
+        <f>E31+E41+E45</f>
+        <v/>
       </c>
       <c r="F55" s="62">
         <f>F31+F41+F45</f>
@@ -4886,18 +4898,6 @@
         <f>G31+G41+G45</f>
         <v/>
       </c>
-      <c r="H55" s="62">
-        <f>H31+H41+H45</f>
-        <v/>
-      </c>
-      <c r="I55" s="62">
-        <f>I31+I41+I45</f>
-        <v/>
-      </c>
-      <c r="J55" s="62">
-        <f>J31+J41+J45</f>
-        <v/>
-      </c>
     </row>
     <row r="56">
       <c r="A56" s="34" t="inlineStr">
@@ -4905,26 +4905,26 @@
           <t>Scenarios base-case revenue ($000)</t>
         </is>
       </c>
-      <c r="E56" s="56" t="n">
+      <c r="B56" s="56" t="n">
         <v>11102600</v>
       </c>
+      <c r="C56" s="35">
+        <f>Scenarios!G18</f>
+        <v/>
+      </c>
+      <c r="D56" s="35">
+        <f>Scenarios!G19</f>
+        <v/>
+      </c>
+      <c r="E56" s="35">
+        <f>Scenarios!G20</f>
+        <v/>
+      </c>
       <c r="F56" s="35">
-        <f>Scenarios!G18</f>
+        <f>Scenarios!G21</f>
         <v/>
       </c>
       <c r="G56" s="35">
-        <f>Scenarios!G19</f>
-        <v/>
-      </c>
-      <c r="H56" s="35">
-        <f>Scenarios!G20</f>
-        <v/>
-      </c>
-      <c r="I56" s="35">
-        <f>Scenarios!G21</f>
-        <v/>
-      </c>
-      <c r="J56" s="35">
         <f>Scenarios!G22</f>
         <v/>
       </c>
@@ -4935,6 +4935,18 @@
           <t>Variance (bottom-up − scenarios) ($000)</t>
         </is>
       </c>
+      <c r="B57" s="35">
+        <f>B55-B56</f>
+        <v/>
+      </c>
+      <c r="C57" s="35">
+        <f>C55-C56</f>
+        <v/>
+      </c>
+      <c r="D57" s="35">
+        <f>D55-D56</f>
+        <v/>
+      </c>
       <c r="E57" s="35">
         <f>E55-E56</f>
         <v/>
@@ -4947,18 +4959,6 @@
         <f>G55-G56</f>
         <v/>
       </c>
-      <c r="H57" s="35">
-        <f>H55-H56</f>
-        <v/>
-      </c>
-      <c r="I57" s="35">
-        <f>I55-I56</f>
-        <v/>
-      </c>
-      <c r="J57" s="35">
-        <f>J55-J56</f>
-        <v/>
-      </c>
     </row>
     <row r="58">
       <c r="A58" s="34" t="inlineStr">
@@ -4966,6 +4966,18 @@
           <t>Variance (%)</t>
         </is>
       </c>
+      <c r="B58" s="36">
+        <f>IF(B56=0,"",B57/B56)</f>
+        <v/>
+      </c>
+      <c r="C58" s="36">
+        <f>IF(C56=0,"",C57/C56)</f>
+        <v/>
+      </c>
+      <c r="D58" s="36">
+        <f>IF(D56=0,"",D57/D56)</f>
+        <v/>
+      </c>
       <c r="E58" s="36">
         <f>IF(E56=0,"",E57/E56)</f>
         <v/>
@@ -4978,18 +4990,6 @@
         <f>IF(G56=0,"",G57/G56)</f>
         <v/>
       </c>
-      <c r="H58" s="36">
-        <f>IF(H56=0,"",H57/H56)</f>
-        <v/>
-      </c>
-      <c r="I58" s="36">
-        <f>IF(I56=0,"",I57/I56)</f>
-        <v/>
-      </c>
-      <c r="J58" s="36">
-        <f>IF(J56=0,"",J57/J56)</f>
-        <v/>
-      </c>
     </row>
     <row r="59">
       <c r="A59" s="26" t="inlineStr">
@@ -5000,40 +5000,40 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6259,17 +6259,17 @@
     </row>
     <row r="55">
       <c r="A55" s="89" t="inlineStr"/>
-      <c r="B55" s="47" t="inlineStr">
+      <c r="B55" s="46" t="inlineStr">
         <is>
           <t>Gordon Growth</t>
         </is>
       </c>
-      <c r="C55" s="47" t="inlineStr">
+      <c r="C55" s="46" t="inlineStr">
         <is>
           <t>Exit Multiple</t>
         </is>
       </c>
-      <c r="D55" s="47" t="inlineStr">
+      <c r="D55" s="46" t="inlineStr">
         <is>
           <t>Variance</t>
         </is>

</xml_diff>

<commit_message>
Document comparable store revenue and net-new-store formula on Revenue Drivers
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -3967,7 +3967,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="28" customHeight="1">
       <c r="A29" s="34" t="inlineStr">
         <is>
           <t>Comparable store revenue ($000)</t>
@@ -3996,8 +3996,23 @@
         <f>F28*0.71*(1+G25)+F28*0.16*(1+G26)+F28*0.13*(1+G27)</f>
         <v/>
       </c>
-    </row>
-    <row r="30" ht="28" customHeight="1">
+      <c r="I29" s="17" t="inlineStr">
+        <is>
+          <t>Sales from existing stores open 12+ months, grown by regional comp % (Americas/China/RoW). Excludes new openings — those sit in the net-new-store line.</t>
+        </is>
+      </c>
+      <c r="J29" s="57" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab: comp formula</t>
+        </is>
+      </c>
+      <c r="K29" s="19" t="inlineStr">
+        <is>
+          <t>Prior-year store rev × geo-weighted comp (71% Americas, 16% China, 13% RoW). Existing stores only — not new openings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="56" customHeight="1">
       <c r="A30" s="34" t="inlineStr">
         <is>
           <t>Net new store revenue contribution ($000)</t>
@@ -4028,7 +4043,7 @@
       </c>
       <c r="I30" s="17" t="inlineStr">
         <is>
-          <t>New-store contribution = net openings × sq ft × SPSF × 55% first-year ramp (standard retail maturity).</t>
+          <t>Net new store $ = (Σ net openings by geo) × avg sq ft × SPSF ÷ 1,000 × 55% first-year ramp.</t>
         </is>
       </c>
       <c r="J30" s="57" t="inlineStr">
@@ -4036,10 +4051,11 @@
           <t>Revenue Drivers tab: formula</t>
         </is>
       </c>
-      <c r="K30" s="19" t="inlineStr">
-        <is>
-          <t>Formula: net openings × sq ft × SPSF / 1000 × 55% ramp. Not a sourced print.</t>
-        </is>
+      <c r="K30" s="19">
+        <f>(open−close Americas + open−close China + open−close RoW) × avg sq ft × SPSF / 1000 × 55%.
+Example FY27 (col D): (D7−D8+D11−D12+D15−D16)×D19×D24/1000×0.55.
+Net stores × sq ft/store × $/sq ft → annual sales; ÷1,000 for $000; ×55% first-year maturity ramp.</f>
+        <v/>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
Add casual formula side notes on Revenue Drivers tab
Wire drv_f_* explanations in columns I/J/K for every equation row,
including /1000 and ×0.55 on net-new-store revenue, plus Scenarios
reconciliation variance lines.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -523,6 +523,9 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -540,9 +543,6 @@
     </xf>
     <xf numFmtId="165" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Americas — beginning stores</t>
@@ -3134,6 +3134,20 @@
           <t>stores</t>
         </is>
       </c>
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
+        </is>
+      </c>
+      <c r="J6" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: beginning-stores formula</t>
+        </is>
+      </c>
+      <c r="K6" s="19">
+        <f>prior-year ending stores. Same count, new column — that's where the year starts.</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="34" t="inlineStr">
@@ -3141,19 +3155,19 @@
           <t xml:space="preserve">  Americas — openings</t>
         </is>
       </c>
-      <c r="C7" s="51" t="n">
+      <c r="C7" s="52" t="n">
         <v>8</v>
       </c>
-      <c r="D7" s="51" t="n">
+      <c r="D7" s="52" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="51" t="n">
+      <c r="E7" s="52" t="n">
         <v>6</v>
       </c>
-      <c r="F7" s="51" t="n">
+      <c r="F7" s="52" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="51" t="n">
+      <c r="G7" s="52" t="n">
         <v>4</v>
       </c>
       <c r="H7" s="50" t="inlineStr">
@@ -3183,19 +3197,19 @@
           <t xml:space="preserve">  Americas — closures</t>
         </is>
       </c>
-      <c r="C8" s="51" t="n">
+      <c r="C8" s="52" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="51" t="n">
+      <c r="D8" s="52" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="51" t="n">
+      <c r="E8" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="51" t="n">
+      <c r="F8" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="51" t="n">
+      <c r="G8" s="52" t="n">
         <v>2</v>
       </c>
       <c r="H8" s="50" t="inlineStr">
@@ -3220,7 +3234,7 @@
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="52" t="inlineStr">
+      <c r="A9" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">  Americas — ending stores</t>
         </is>
@@ -3228,23 +3242,23 @@
       <c r="B9" s="49" t="n">
         <v>476</v>
       </c>
-      <c r="C9" s="53">
+      <c r="C9" s="54">
         <f>C6+C7-C8</f>
         <v/>
       </c>
-      <c r="D9" s="53">
+      <c r="D9" s="54">
         <f>D6+D7-D8</f>
         <v/>
       </c>
-      <c r="E9" s="53">
+      <c r="E9" s="54">
         <f>E6+E7-E8</f>
         <v/>
       </c>
-      <c r="F9" s="53">
+      <c r="F9" s="54">
         <f>F6+F7-F8</f>
         <v/>
       </c>
-      <c r="G9" s="53">
+      <c r="G9" s="54">
         <f>G6+G7-G8</f>
         <v/>
       </c>
@@ -3253,13 +3267,22 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="K9" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Americas" → FY2025 ending stores 476.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
+        </is>
+      </c>
+      <c r="J9" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: ending-stores formula</t>
+        </is>
+      </c>
+      <c r="K9" s="19">
+        <f>beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  China Mainland — beginning stores</t>
@@ -3293,6 +3316,20 @@
           <t>stores</t>
         </is>
       </c>
+      <c r="I10" s="17" t="inlineStr">
+        <is>
+          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
+        </is>
+      </c>
+      <c r="J10" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: beginning-stores formula</t>
+        </is>
+      </c>
+      <c r="K10" s="19">
+        <f>prior-year ending stores. Same count, new column — that's where the year starts.</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="34" t="inlineStr">
@@ -3300,19 +3337,19 @@
           <t xml:space="preserve">  China Mainland — openings</t>
         </is>
       </c>
-      <c r="C11" s="51" t="n">
+      <c r="C11" s="52" t="n">
         <v>20</v>
       </c>
-      <c r="D11" s="51" t="n">
+      <c r="D11" s="52" t="n">
         <v>18</v>
       </c>
-      <c r="E11" s="51" t="n">
+      <c r="E11" s="52" t="n">
         <v>16</v>
       </c>
-      <c r="F11" s="51" t="n">
+      <c r="F11" s="52" t="n">
         <v>14</v>
       </c>
-      <c r="G11" s="51" t="n">
+      <c r="G11" s="52" t="n">
         <v>12</v>
       </c>
       <c r="H11" s="50" t="inlineStr">
@@ -3342,19 +3379,19 @@
           <t xml:space="preserve">  China Mainland — closures</t>
         </is>
       </c>
-      <c r="C12" s="51" t="n">
+      <c r="C12" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="51" t="n">
+      <c r="D12" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="51" t="n">
+      <c r="E12" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="51" t="n">
+      <c r="F12" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="51" t="n">
+      <c r="G12" s="52" t="n">
         <v>1</v>
       </c>
       <c r="H12" s="50" t="inlineStr">
@@ -3379,7 +3416,7 @@
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="52" t="inlineStr">
+      <c r="A13" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">  China Mainland — ending stores</t>
         </is>
@@ -3387,23 +3424,23 @@
       <c r="B13" s="49" t="n">
         <v>172</v>
       </c>
-      <c r="C13" s="53">
+      <c r="C13" s="54">
         <f>C10+C11-C12</f>
         <v/>
       </c>
-      <c r="D13" s="53">
+      <c r="D13" s="54">
         <f>D10+D11-D12</f>
         <v/>
       </c>
-      <c r="E13" s="53">
+      <c r="E13" s="54">
         <f>E10+E11-E12</f>
         <v/>
       </c>
-      <c r="F13" s="53">
+      <c r="F13" s="54">
         <f>F10+F11-F12</f>
         <v/>
       </c>
-      <c r="G13" s="53">
+      <c r="G13" s="54">
         <f>G10+G11-G12</f>
         <v/>
       </c>
@@ -3412,13 +3449,22 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="K13" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "China Mainland" → FY2025 ending stores 172.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
+        </is>
+      </c>
+      <c r="J13" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: ending-stores formula</t>
+        </is>
+      </c>
+      <c r="K13" s="19">
+        <f>beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
       <c r="A14" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rest of World — beginning stores</t>
@@ -3452,6 +3498,20 @@
           <t>stores</t>
         </is>
       </c>
+      <c r="I14" s="17" t="inlineStr">
+        <is>
+          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
+        </is>
+      </c>
+      <c r="J14" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: beginning-stores formula</t>
+        </is>
+      </c>
+      <c r="K14" s="19">
+        <f>prior-year ending stores. Same count, new column — that's where the year starts.</f>
+        <v/>
+      </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="34" t="inlineStr">
@@ -3459,19 +3519,19 @@
           <t xml:space="preserve">  Rest of World — openings</t>
         </is>
       </c>
-      <c r="C15" s="51" t="n">
+      <c r="C15" s="52" t="n">
         <v>7</v>
       </c>
-      <c r="D15" s="51" t="n">
+      <c r="D15" s="52" t="n">
         <v>6</v>
       </c>
-      <c r="E15" s="51" t="n">
+      <c r="E15" s="52" t="n">
         <v>5</v>
       </c>
-      <c r="F15" s="51" t="n">
+      <c r="F15" s="52" t="n">
         <v>5</v>
       </c>
-      <c r="G15" s="51" t="n">
+      <c r="G15" s="52" t="n">
         <v>4</v>
       </c>
       <c r="H15" s="50" t="inlineStr">
@@ -3501,19 +3561,19 @@
           <t xml:space="preserve">  Rest of World — closures</t>
         </is>
       </c>
-      <c r="C16" s="51" t="n">
+      <c r="C16" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="51" t="n">
+      <c r="D16" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="51" t="n">
+      <c r="E16" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="F16" s="51" t="n">
+      <c r="F16" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="51" t="n">
+      <c r="G16" s="52" t="n">
         <v>2</v>
       </c>
       <c r="H16" s="50" t="inlineStr">
@@ -3538,7 +3598,7 @@
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="52" t="inlineStr">
+      <c r="A17" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rest of World — ending stores</t>
         </is>
@@ -3546,23 +3606,23 @@
       <c r="B17" s="49" t="n">
         <v>163</v>
       </c>
-      <c r="C17" s="53">
+      <c r="C17" s="54">
         <f>C14+C15-C16</f>
         <v/>
       </c>
-      <c r="D17" s="53">
+      <c r="D17" s="54">
         <f>D14+D15-D16</f>
         <v/>
       </c>
-      <c r="E17" s="53">
+      <c r="E17" s="54">
         <f>E14+E15-E16</f>
         <v/>
       </c>
-      <c r="F17" s="53">
+      <c r="F17" s="54">
         <f>F14+F15-F16</f>
         <v/>
       </c>
-      <c r="G17" s="53">
+      <c r="G17" s="54">
         <f>G14+G15-G16</f>
         <v/>
       </c>
@@ -3571,39 +3631,62 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="K17" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Rest of World" → FY2025 ending stores 163.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="52" t="inlineStr">
+      <c r="I17" s="17" t="inlineStr">
+        <is>
+          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
+        </is>
+      </c>
+      <c r="J17" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: ending-stores formula</t>
+        </is>
+      </c>
+      <c r="K17" s="19">
+        <f>beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="53" t="inlineStr">
         <is>
           <t>Total ending stores</t>
         </is>
       </c>
-      <c r="B18" s="54" t="n">
+      <c r="B18" s="55" t="n">
         <v>811</v>
       </c>
-      <c r="C18" s="53">
+      <c r="C18" s="54">
         <f>C9+C13+C17</f>
         <v/>
       </c>
-      <c r="D18" s="53">
+      <c r="D18" s="54">
         <f>D9+D13+D17</f>
         <v/>
       </c>
-      <c r="E18" s="53">
+      <c r="E18" s="54">
         <f>E9+E13+E17</f>
         <v/>
       </c>
-      <c r="F18" s="53">
+      <c r="F18" s="54">
         <f>F9+F13+F17</f>
         <v/>
       </c>
-      <c r="G18" s="53">
+      <c r="G18" s="54">
         <f>G9+G13+G17</f>
+        <v/>
+      </c>
+      <c r="I18" s="17" t="inlineStr">
+        <is>
+          <t>Add up Americas + China + RoW ending stores. Should tie to the 10-K total company-operated count.</t>
+        </is>
+      </c>
+      <c r="J18" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: total-stores formula</t>
+        </is>
+      </c>
+      <c r="K18" s="19">
+        <f>Americas ending + China ending + RoW ending. Should foot to total company-operated stores.</f>
         <v/>
       </c>
     </row>
@@ -3613,22 +3696,22 @@
           <t>Avg square feet per store</t>
         </is>
       </c>
-      <c r="B19" s="51" t="n">
+      <c r="B19" s="52" t="n">
         <v>4366</v>
       </c>
-      <c r="C19" s="51" t="n">
+      <c r="C19" s="52" t="n">
         <v>4400</v>
       </c>
-      <c r="D19" s="51" t="n">
+      <c r="D19" s="52" t="n">
         <v>4425</v>
       </c>
-      <c r="E19" s="51" t="n">
+      <c r="E19" s="52" t="n">
         <v>4450</v>
       </c>
-      <c r="F19" s="51" t="n">
+      <c r="F19" s="52" t="n">
         <v>4475</v>
       </c>
-      <c r="G19" s="51" t="n">
+      <c r="G19" s="52" t="n">
         <v>4500</v>
       </c>
       <c r="H19" s="50" t="inlineStr">
@@ -3652,7 +3735,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="28" customHeight="1">
       <c r="A20" s="34" t="inlineStr">
         <is>
           <t>Total square footage (end stores × avg sq ft)</t>
@@ -3687,6 +3770,20 @@
           <t>sq ft</t>
         </is>
       </c>
+      <c r="I20" s="17" t="inlineStr">
+        <is>
+          <t>Ending stores times avg sq ft per box. Gives you total fleet square footage for the productivity math.</t>
+        </is>
+      </c>
+      <c r="J20" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: total-sqft formula</t>
+        </is>
+      </c>
+      <c r="K20" s="19">
+        <f>total ending stores × avg sq ft per store. Fleet size in square feet for the productivity lines.</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="44" t="inlineStr">
@@ -3758,22 +3855,22 @@
           <t>Sales per square foot ($)</t>
         </is>
       </c>
-      <c r="B24" s="51" t="n">
+      <c r="B24" s="52" t="n">
         <v>1426</v>
       </c>
-      <c r="C24" s="51" t="n">
+      <c r="C24" s="52" t="n">
         <v>1360</v>
       </c>
-      <c r="D24" s="51" t="n">
+      <c r="D24" s="52" t="n">
         <v>1380</v>
       </c>
-      <c r="E24" s="51" t="n">
+      <c r="E24" s="52" t="n">
         <v>1400</v>
       </c>
-      <c r="F24" s="51" t="n">
+      <c r="F24" s="52" t="n">
         <v>1420</v>
       </c>
-      <c r="G24" s="51" t="n">
+      <c r="G24" s="52" t="n">
         <v>1440</v>
       </c>
       <c r="H24" s="50" t="inlineStr">
@@ -3803,22 +3900,22 @@
           <t xml:space="preserve">  Americas — comparable sales growth</t>
         </is>
       </c>
-      <c r="B25" s="55" t="n">
+      <c r="B25" s="56" t="n">
         <v>-0.03</v>
       </c>
-      <c r="C25" s="55" t="n">
+      <c r="C25" s="56" t="n">
         <v>-0.04</v>
       </c>
-      <c r="D25" s="55" t="n">
+      <c r="D25" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="E25" s="55" t="n">
+      <c r="E25" s="56" t="n">
         <v>0.01</v>
       </c>
-      <c r="F25" s="55" t="n">
+      <c r="F25" s="56" t="n">
         <v>0.02</v>
       </c>
-      <c r="G25" s="55" t="n">
+      <c r="G25" s="56" t="n">
         <v>0.02</v>
       </c>
       <c r="H25" s="50" t="inlineStr">
@@ -3848,22 +3945,22 @@
           <t xml:space="preserve">  China Mainland — comparable sales growth</t>
         </is>
       </c>
-      <c r="B26" s="55" t="n">
+      <c r="B26" s="56" t="n">
         <v>0.2</v>
       </c>
-      <c r="C26" s="55" t="n">
+      <c r="C26" s="56" t="n">
         <v>0.14</v>
       </c>
-      <c r="D26" s="55" t="n">
+      <c r="D26" s="56" t="n">
         <v>0.12</v>
       </c>
-      <c r="E26" s="55" t="n">
+      <c r="E26" s="56" t="n">
         <v>0.1</v>
       </c>
-      <c r="F26" s="55" t="n">
+      <c r="F26" s="56" t="n">
         <v>0.08</v>
       </c>
-      <c r="G26" s="55" t="n">
+      <c r="G26" s="56" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="H26" s="50" t="inlineStr">
@@ -3893,22 +3990,22 @@
           <t xml:space="preserve">  Rest of World — comparable sales growth</t>
         </is>
       </c>
-      <c r="B27" s="55" t="n">
+      <c r="B27" s="56" t="n">
         <v>0.09</v>
       </c>
-      <c r="C27" s="55" t="n">
+      <c r="C27" s="56" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="D27" s="55" t="n">
+      <c r="D27" s="56" t="n">
         <v>0.06</v>
       </c>
-      <c r="E27" s="55" t="n">
+      <c r="E27" s="56" t="n">
         <v>0.05</v>
       </c>
-      <c r="F27" s="55" t="n">
+      <c r="F27" s="56" t="n">
         <v>0.04</v>
       </c>
-      <c r="G27" s="55" t="n">
+      <c r="G27" s="56" t="n">
         <v>0.04</v>
       </c>
       <c r="H27" s="50" t="inlineStr">
@@ -3932,13 +4029,13 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="28" customHeight="1">
       <c r="A28" s="34" t="inlineStr">
         <is>
           <t>Prior-year store channel revenue ($000)</t>
         </is>
       </c>
-      <c r="B28" s="56" t="n">
+      <c r="B28" s="57" t="n">
         <v>5049744</v>
       </c>
       <c r="C28" s="35">
@@ -3966,6 +4063,20 @@
           <t>$000</t>
         </is>
       </c>
+      <c r="I28" s="17" t="inlineStr">
+        <is>
+          <t>Last year's total store-channel revenue — the base you're growing comps off of, not the new boxes.</t>
+        </is>
+      </c>
+      <c r="J28" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: prior store-rev formula</t>
+        </is>
+      </c>
+      <c r="K28" s="19">
+        <f>prior column's total store-channel revenue. Base you're applying comps to — not new-store contribution.</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="34" t="inlineStr">
@@ -3998,21 +4109,20 @@
       </c>
       <c r="I29" s="17" t="inlineStr">
         <is>
-          <t>Sales from existing stores open 12+ months, grown by regional comp % (Americas/China/RoW). Excludes new openings — those sit in the net-new-store line.</t>
-        </is>
-      </c>
-      <c r="J29" s="57" t="inlineStr">
-        <is>
-          <t>Revenue Drivers tab: comp formula</t>
-        </is>
-      </c>
-      <c r="K29" s="19" t="inlineStr">
-        <is>
-          <t>Prior-year store rev × geo-weighted comp (71% Americas, 16% China, 13% RoW). Existing stores only — not new openings.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="56" customHeight="1">
+          <t>Existing-store sales only — prior store rev grown by geo comp %. New doors are a separate line, not in here.</t>
+        </is>
+      </c>
+      <c r="J29" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: comp-store formula</t>
+        </is>
+      </c>
+      <c r="K29" s="19">
+        <f>prior store rev×(71%×(1+Am comp)+16%×(1+China)+13%×(1+RoW)). Existing base only — new stores are on the next row.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1">
       <c r="A30" s="34" t="inlineStr">
         <is>
           <t>Net new store revenue contribution ($000)</t>
@@ -4043,48 +4153,60 @@
       </c>
       <c r="I30" s="17" t="inlineStr">
         <is>
-          <t>Net new store $ = (Σ net openings by geo) × avg sq ft × SPSF ÷ 1,000 × 55% first-year ramp.</t>
-        </is>
-      </c>
-      <c r="J30" s="57" t="inlineStr">
-        <is>
-          <t>Revenue Drivers tab: formula</t>
+          <t>Net new doors × sq ft × $/sq ft is plain dollars. /1000 → $000 on this tab. ×0.55 'cause year-one stores don't run full.</t>
+        </is>
+      </c>
+      <c r="J30" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: net-new-store formula</t>
         </is>
       </c>
       <c r="K30" s="19">
-        <f>(open−close Americas + open−close China + open−close RoW) × avg sq ft × SPSF / 1000 × 55%.
-Example FY27 (col D): (D7−D8+D11−D12+D15−D16)×D19×D24/1000×0.55.
-Net stores × sq ft/store × $/sq ft → annual sales; ÷1,000 for $000; ×55% first-year maturity ramp.</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="52" t="inlineStr">
+        <f>(open−close each geo)×sq ft×$/sq ft → raw annual $. /1000 flips that to $000 (this whole tab is thousands). ×0.55 = year-one haircut — new boxes don't run at full SPSF yet. FY27 ex: (D7−D8+D11−D12+D15−D16)×D19×D24/1000×0.55.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="53" t="inlineStr">
         <is>
           <t>Store channel revenue ($000)</t>
         </is>
       </c>
-      <c r="B31" s="54" t="n">
+      <c r="B31" s="55" t="n">
         <v>5049744</v>
       </c>
-      <c r="C31" s="53">
+      <c r="C31" s="54">
         <f>C29+C30</f>
         <v/>
       </c>
-      <c r="D31" s="53">
+      <c r="D31" s="54">
         <f>D29+D30</f>
         <v/>
       </c>
-      <c r="E31" s="53">
+      <c r="E31" s="54">
         <f>E29+E30</f>
         <v/>
       </c>
-      <c r="F31" s="53">
+      <c r="F31" s="54">
         <f>F29+F30</f>
         <v/>
       </c>
-      <c r="G31" s="53">
+      <c r="G31" s="54">
         <f>G29+G30</f>
+        <v/>
+      </c>
+      <c r="I31" s="17" t="inlineStr">
+        <is>
+          <t>Brick-and-mortar channel = comp store sales plus whatever the net new stores contributed. That's the whole store line.</t>
+        </is>
+      </c>
+      <c r="J31" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: store-channel formula</t>
+        </is>
+      </c>
+      <c r="K31" s="19">
+        <f>comparable store revenue + net new store revenue. Full brick-and-mortar channel for the year.</f>
         <v/>
       </c>
     </row>
@@ -4139,22 +4261,22 @@
           <t xml:space="preserve">  memo: in-store conversion rate</t>
         </is>
       </c>
-      <c r="B33" s="55" t="n">
+      <c r="B33" s="56" t="n">
         <v>0.28</v>
       </c>
-      <c r="C33" s="55" t="n">
+      <c r="C33" s="56" t="n">
         <v>0.27</v>
       </c>
-      <c r="D33" s="55" t="n">
+      <c r="D33" s="56" t="n">
         <v>0.275</v>
       </c>
-      <c r="E33" s="55" t="n">
+      <c r="E33" s="56" t="n">
         <v>0.28</v>
       </c>
-      <c r="F33" s="55" t="n">
+      <c r="F33" s="56" t="n">
         <v>0.285</v>
       </c>
-      <c r="G33" s="55" t="n">
+      <c r="G33" s="56" t="n">
         <v>0.29</v>
       </c>
       <c r="I33" s="17" t="inlineStr">
@@ -4283,22 +4405,22 @@
           <t>Unique digital sessions (millions)</t>
         </is>
       </c>
-      <c r="B38" s="51" t="n">
+      <c r="B38" s="52" t="n">
         <v>485</v>
       </c>
-      <c r="C38" s="51" t="n">
+      <c r="C38" s="52" t="n">
         <v>485</v>
       </c>
-      <c r="D38" s="51" t="n">
+      <c r="D38" s="52" t="n">
         <v>505</v>
       </c>
-      <c r="E38" s="51" t="n">
+      <c r="E38" s="52" t="n">
         <v>525</v>
       </c>
-      <c r="F38" s="51" t="n">
+      <c r="F38" s="52" t="n">
         <v>545</v>
       </c>
-      <c r="G38" s="51" t="n">
+      <c r="G38" s="52" t="n">
         <v>560</v>
       </c>
       <c r="H38" s="50" t="inlineStr">
@@ -4328,22 +4450,22 @@
           <t>Digital conversion rate</t>
         </is>
       </c>
-      <c r="B39" s="55" t="n">
+      <c r="B39" s="56" t="n">
         <v>0.033</v>
       </c>
-      <c r="C39" s="55" t="n">
+      <c r="C39" s="56" t="n">
         <v>0.033</v>
       </c>
-      <c r="D39" s="55" t="n">
+      <c r="D39" s="56" t="n">
         <v>0.034</v>
       </c>
-      <c r="E39" s="55" t="n">
+      <c r="E39" s="56" t="n">
         <v>0.035</v>
       </c>
-      <c r="F39" s="55" t="n">
+      <c r="F39" s="56" t="n">
         <v>0.035</v>
       </c>
-      <c r="G39" s="55" t="n">
+      <c r="G39" s="56" t="n">
         <v>0.036</v>
       </c>
       <c r="I39" s="17" t="inlineStr">
@@ -4403,38 +4525,47 @@
       </c>
     </row>
     <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="52" t="inlineStr">
+      <c r="A41" s="53" t="inlineStr">
         <is>
           <t>E-commerce revenue ($000)</t>
         </is>
       </c>
-      <c r="B41" s="54" t="n">
+      <c r="B41" s="55" t="n">
         <v>4918697</v>
       </c>
-      <c r="C41" s="53">
+      <c r="C41" s="54">
         <f>C38*1000000*C39*C40/1000</f>
         <v/>
       </c>
-      <c r="D41" s="53">
+      <c r="D41" s="54">
         <f>D38*1000000*D39*D40/1000</f>
         <v/>
       </c>
-      <c r="E41" s="53">
+      <c r="E41" s="54">
         <f>E38*1000000*E39*E40/1000</f>
         <v/>
       </c>
-      <c r="F41" s="53">
+      <c r="F41" s="54">
         <f>F38*1000000*F39*F40/1000</f>
         <v/>
       </c>
-      <c r="G41" s="53">
+      <c r="G41" s="54">
         <f>G38*1000000*G39*G40/1000</f>
         <v/>
       </c>
-      <c r="K41" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "E-commerce" → 4,918,697 ($000 FY2025). Forward = sessions × conversion × AOV.</t>
-        </is>
+      <c r="I41" s="17" t="inlineStr">
+        <is>
+          <t>Traffic × conversion × AOV is dollars. ×1M 'cause sessions are in millions; /1000 puts it in $000 like everything else.</t>
+        </is>
+      </c>
+      <c r="J41" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: e-comm formula</t>
+        </is>
+      </c>
+      <c r="K41" s="19">
+        <f>sessions×1,000,000×conversion×AOV/1000 → e-comm $000. ×1M 'cause sessions are millions; /1000 matches tab units.</f>
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -4501,13 +4632,13 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="28" customHeight="1">
+    <row r="45" ht="42" customHeight="1">
       <c r="A45" s="34" t="inlineStr">
         <is>
           <t>Other channels (wholesale / license / outlets) ($000)</t>
         </is>
       </c>
-      <c r="B45" s="56" t="n">
+      <c r="B45" s="57" t="n">
         <v>1134159</v>
       </c>
       <c r="C45" s="35">
@@ -4535,29 +4666,32 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I45" s="17" t="inlineStr">
-        <is>
-          <t>Other channels (wholesale/license/outlets) held at FY25 $1.13B base; low-single-digit growth thereafter.</t>
-        </is>
-      </c>
-      <c r="J45" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: channel revenue table</t>
+      <c r="I45" s="19" t="inlineStr">
+        <is>
+          <t>Other channels (wholesale/license/outlets) held at FY25 $1.13B base; low-single-digit growth thereafter.
+Formula: Take last year's other-channel revenue and grow it by your assumed %. Wholesale/license/outlets — not stores or dot-com.</t>
+        </is>
+      </c>
+      <c r="J45" s="22" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: channel revenue table
+Formula: Revenue Drivers: other-rev formula</t>
         </is>
       </c>
       <c r="K45" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Company-operated stores" and "E-commerce" → residual other channels ≈ $1.13B.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="28" customHeight="1">
+          <t>Ctrl+F "Company-operated stores" and "E-commerce" → residual other channels ≈ $1.13B.
+Formula: =prior other-channel rev × (1 + growth %). Wholesale/license/outlets — grown off last year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="42" customHeight="1">
       <c r="A46" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Americas net revenue ($000)</t>
         </is>
       </c>
-      <c r="B46" s="56" t="n">
+      <c r="B46" s="57" t="n">
         <v>7847044</v>
       </c>
       <c r="C46" s="35">
@@ -4585,29 +4719,32 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I46" s="17" t="inlineStr">
-        <is>
-          <t>Geographic split scales with consolidated growth; FY25 Americas 70.7% of revenue per 10-K segment table.</t>
-        </is>
-      </c>
-      <c r="J46" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: segmented net revenue</t>
+      <c r="I46" s="19" t="inlineStr">
+        <is>
+          <t>Geographic split scales with consolidated growth; FY25 Americas 70.7% of revenue per 10-K segment table.
+Formula: Hold the FY25 geo mix, scale each region by how much total revenue grew vs last year. Quick way to split the top line.</t>
+        </is>
+      </c>
+      <c r="J46" s="22" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: segmented net revenue
+Formula: Revenue Drivers: geo-scale formula</t>
         </is>
       </c>
       <c r="K46" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Americas" segment table → $7,847,044 net revenue (70.7%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="28" customHeight="1">
+          <t>Ctrl+F "Americas" segment table → $7,847,044 net revenue (70.7%).
+Formula: =FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="42" customHeight="1">
       <c r="A47" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  China Mainland net revenue ($000)</t>
         </is>
       </c>
-      <c r="B47" s="56" t="n">
+      <c r="B47" s="57" t="n">
         <v>1754799</v>
       </c>
       <c r="C47" s="35">
@@ -4635,29 +4772,32 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I47" s="17" t="inlineStr">
-        <is>
-          <t>China 15.8% of FY25 revenue; fastest comp and store growth — expansion market in the driver schedule.</t>
-        </is>
-      </c>
-      <c r="J47" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: segmented net revenue</t>
+      <c r="I47" s="19" t="inlineStr">
+        <is>
+          <t>China 15.8% of FY25 revenue; fastest comp and store growth — expansion market in the driver schedule.
+Formula: Hold the FY25 geo mix, scale each region by how much total revenue grew vs last year. Quick way to split the top line.</t>
+        </is>
+      </c>
+      <c r="J47" s="22" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: segmented net revenue
+Formula: Revenue Drivers: geo-scale formula</t>
         </is>
       </c>
       <c r="K47" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "China Mainland" segment → $1,754,799 net revenue (15.8%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="28" customHeight="1">
+          <t>Ctrl+F "China Mainland" segment → $1,754,799 net revenue (15.8%).
+Formula: =FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="42" customHeight="1">
       <c r="A48" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rest of World net revenue ($000)</t>
         </is>
       </c>
-      <c r="B48" s="56" t="n">
+      <c r="B48" s="57" t="n">
         <v>1500757</v>
       </c>
       <c r="C48" s="35">
@@ -4685,19 +4825,22 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I48" s="17" t="inlineStr">
-        <is>
-          <t>Rest of World 13.5% of FY25 revenue; mid-single-digit comps and steady openings.</t>
-        </is>
-      </c>
-      <c r="J48" s="18" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: segmented net revenue</t>
+      <c r="I48" s="19" t="inlineStr">
+        <is>
+          <t>Rest of World 13.5% of FY25 revenue; mid-single-digit comps and steady openings.
+Formula: Hold the FY25 geo mix, scale each region by how much total revenue grew vs last year. Quick way to split the top line.</t>
+        </is>
+      </c>
+      <c r="J48" s="22" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: segmented net revenue
+Formula: Revenue Drivers: geo-scale formula</t>
         </is>
       </c>
       <c r="K48" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Rest of World" segment → $1,500,757 net revenue (13.5%).</t>
+          <t>Ctrl+F "Rest of World" segment → $1,500,757 net revenue (13.5%).
+Formula: =FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
         </is>
       </c>
     </row>
@@ -4707,22 +4850,22 @@
           <t>Women's % of revenue</t>
         </is>
       </c>
-      <c r="B49" s="55" t="n">
+      <c r="B49" s="56" t="n">
         <v>0.63</v>
       </c>
-      <c r="C49" s="55" t="n">
+      <c r="C49" s="56" t="n">
         <v>0.62</v>
       </c>
-      <c r="D49" s="55" t="n">
+      <c r="D49" s="56" t="n">
         <v>0.615</v>
       </c>
-      <c r="E49" s="55" t="n">
+      <c r="E49" s="56" t="n">
         <v>0.61</v>
       </c>
-      <c r="F49" s="55" t="n">
+      <c r="F49" s="56" t="n">
         <v>0.605</v>
       </c>
-      <c r="G49" s="55" t="n">
+      <c r="G49" s="56" t="n">
         <v>0.6</v>
       </c>
       <c r="I49" s="17" t="inlineStr">
@@ -4747,22 +4890,22 @@
           <t>Men's % of revenue</t>
         </is>
       </c>
-      <c r="B50" s="55" t="n">
+      <c r="B50" s="56" t="n">
         <v>0.24</v>
       </c>
-      <c r="C50" s="55" t="n">
+      <c r="C50" s="56" t="n">
         <v>0.25</v>
       </c>
-      <c r="D50" s="55" t="n">
+      <c r="D50" s="56" t="n">
         <v>0.255</v>
       </c>
-      <c r="E50" s="55" t="n">
+      <c r="E50" s="56" t="n">
         <v>0.26</v>
       </c>
-      <c r="F50" s="55" t="n">
+      <c r="F50" s="56" t="n">
         <v>0.265</v>
       </c>
-      <c r="G50" s="55" t="n">
+      <c r="G50" s="56" t="n">
         <v>0.27</v>
       </c>
       <c r="I50" s="17" t="inlineStr">
@@ -4787,22 +4930,22 @@
           <t>Accessories &amp; other % of revenue</t>
         </is>
       </c>
-      <c r="B51" s="55" t="n">
+      <c r="B51" s="56" t="n">
         <v>0.13</v>
       </c>
-      <c r="C51" s="55" t="n">
+      <c r="C51" s="56" t="n">
         <v>0.13</v>
       </c>
-      <c r="D51" s="55" t="n">
+      <c r="D51" s="56" t="n">
         <v>0.13</v>
       </c>
-      <c r="E51" s="55" t="n">
+      <c r="E51" s="56" t="n">
         <v>0.13</v>
       </c>
-      <c r="F51" s="55" t="n">
+      <c r="F51" s="56" t="n">
         <v>0.13</v>
       </c>
-      <c r="G51" s="55" t="n">
+      <c r="G51" s="56" t="n">
         <v>0.13</v>
       </c>
       <c r="I51" s="17" t="inlineStr">
@@ -4885,7 +5028,7 @@
         </is>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="28" customHeight="1">
       <c r="A55" s="60" t="inlineStr">
         <is>
           <t>Bottom-up total revenue ($000)</t>
@@ -4914,14 +5057,28 @@
         <f>G31+G41+G45</f>
         <v/>
       </c>
-    </row>
-    <row r="56">
+      <c r="I55" s="17" t="inlineStr">
+        <is>
+          <t>Bottom-up total = store channel + e-comm + other. That's your driver-built revenue before you check Scenarios.</t>
+        </is>
+      </c>
+      <c r="J55" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: total-rev formula</t>
+        </is>
+      </c>
+      <c r="K55" s="19">
+        <f>store channel + e-commerce + other. Bottom-up top line before you reconcile to Scenarios.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="28" customHeight="1">
       <c r="A56" s="34" t="inlineStr">
         <is>
           <t>Scenarios base-case revenue ($000)</t>
         </is>
       </c>
-      <c r="B56" s="56" t="n">
+      <c r="B56" s="57" t="n">
         <v>11102600</v>
       </c>
       <c r="C56" s="35">
@@ -4944,8 +5101,22 @@
         <f>Scenarios!G22</f>
         <v/>
       </c>
-    </row>
-    <row r="57">
+      <c r="I56" s="17" t="inlineStr">
+        <is>
+          <t>Pulls the Scenarios base-case revenue path — that's still the number the DCF actually uses, not the driver total.</t>
+        </is>
+      </c>
+      <c r="J56" s="51" t="inlineStr">
+        <is>
+          <t>Scenarios tab: base revenue</t>
+        </is>
+      </c>
+      <c r="K56" s="19">
+        <f>Scenarios! base-case revenue. DCF still runs off this path — not the driver total.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" ht="28" customHeight="1">
       <c r="A57" s="34" t="inlineStr">
         <is>
           <t>Variance (bottom-up − scenarios) ($000)</t>
@@ -4975,8 +5146,22 @@
         <f>G55-G56</f>
         <v/>
       </c>
-    </row>
-    <row r="58">
+      <c r="I57" s="17" t="inlineStr">
+        <is>
+          <t>Driver-built revenue minus Scenarios revenue. Shows you how far off the bottom-up path is from what you're valuing on.</t>
+        </is>
+      </c>
+      <c r="J57" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: variance formula</t>
+        </is>
+      </c>
+      <c r="K57" s="19">
+        <f>bottom-up total − Scenarios revenue. Positive = drivers above Scenarios; negative = below.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="28" customHeight="1">
       <c r="A58" s="34" t="inlineStr">
         <is>
           <t>Variance (%)</t>
@@ -5004,6 +5189,20 @@
       </c>
       <c r="G58" s="36">
         <f>IF(G56=0,"",G57/G56)</f>
+        <v/>
+      </c>
+      <c r="I58" s="17" t="inlineStr">
+        <is>
+          <t>Variance as a percent of Scenarios revenue. Easy read on whether the driver schedule is close or way out of line.</t>
+        </is>
+      </c>
+      <c r="J58" s="51" t="inlineStr">
+        <is>
+          <t>Revenue Drivers: variance % formula</t>
+        </is>
+      </c>
+      <c r="K58" s="19">
+        <f>variance ÷ Scenarios revenue. Quick % read on how far the driver build is from the valuation path.</f>
         <v/>
       </c>
     </row>
@@ -6972,7 +7171,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C19" s="57" t="inlineStr">
+      <c r="C19" s="51" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7004,7 +7203,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C20" s="57" t="inlineStr">
+      <c r="C20" s="51" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7036,7 +7235,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C21" s="57" t="inlineStr">
+      <c r="C21" s="51" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7068,7 +7267,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C22" s="57" t="inlineStr">
+      <c r="C22" s="51" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7100,7 +7299,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C23" s="57" t="inlineStr">
+      <c r="C23" s="51" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7132,7 +7331,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C24" s="57" t="inlineStr">
+      <c r="C24" s="51" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7164,7 +7363,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C25" s="57" t="inlineStr">
+      <c r="C25" s="51" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7196,7 +7395,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C26" s="57" t="inlineStr">
+      <c r="C26" s="51" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7228,7 +7427,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C27" s="57" t="inlineStr">
+      <c r="C27" s="51" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7260,7 +7459,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C28" s="57" t="inlineStr">
+      <c r="C28" s="51" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7292,7 +7491,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C29" s="57" t="inlineStr">
+      <c r="C29" s="51" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>

</xml_diff>

<commit_message>
Fix Excel repair error: escape formula notes in Ctrl+F column
Notes that start with '=' were written as broken formulas on Revenue
Drivers (sheet4). Prefix with apostrophe so Excel treats them as text.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -3144,9 +3144,10 @@
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
       </c>
-      <c r="K6" s="19">
-        <f>prior-year ending stores. Same count, new column — that's where the year starts.</f>
-        <v/>
+      <c r="K6" s="19" t="inlineStr">
+        <is>
+          <t>'=prior-year ending stores. Same count, new column — that's where the year starts.</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
@@ -3277,9 +3278,10 @@
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
       </c>
-      <c r="K9" s="19">
-        <f>beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</f>
-        <v/>
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>'=beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
+        </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
@@ -3326,9 +3328,10 @@
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
       </c>
-      <c r="K10" s="19">
-        <f>prior-year ending stores. Same count, new column — that's where the year starts.</f>
-        <v/>
+      <c r="K10" s="19" t="inlineStr">
+        <is>
+          <t>'=prior-year ending stores. Same count, new column — that's where the year starts.</t>
+        </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
@@ -3459,9 +3462,10 @@
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
       </c>
-      <c r="K13" s="19">
-        <f>beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</f>
-        <v/>
+      <c r="K13" s="19" t="inlineStr">
+        <is>
+          <t>'=beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
+        </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
@@ -3508,9 +3512,10 @@
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
       </c>
-      <c r="K14" s="19">
-        <f>prior-year ending stores. Same count, new column — that's where the year starts.</f>
-        <v/>
+      <c r="K14" s="19" t="inlineStr">
+        <is>
+          <t>'=prior-year ending stores. Same count, new column — that's where the year starts.</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
@@ -3641,9 +3646,10 @@
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
       </c>
-      <c r="K17" s="19">
-        <f>beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</f>
-        <v/>
+      <c r="K17" s="19" t="inlineStr">
+        <is>
+          <t>'=beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
@@ -3685,9 +3691,10 @@
           <t>Revenue Drivers: total-stores formula</t>
         </is>
       </c>
-      <c r="K18" s="19">
-        <f>Americas ending + China ending + RoW ending. Should foot to total company-operated stores.</f>
-        <v/>
+      <c r="K18" s="19" t="inlineStr">
+        <is>
+          <t>'=Americas ending + China ending + RoW ending. Should foot to total company-operated stores.</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
@@ -3780,9 +3787,10 @@
           <t>Revenue Drivers: total-sqft formula</t>
         </is>
       </c>
-      <c r="K20" s="19">
-        <f>total ending stores × avg sq ft per store. Fleet size in square feet for the productivity lines.</f>
-        <v/>
+      <c r="K20" s="19" t="inlineStr">
+        <is>
+          <t>'=total ending stores × avg sq ft per store. Fleet size in square feet for the productivity lines.</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -4073,9 +4081,10 @@
           <t>Revenue Drivers: prior store-rev formula</t>
         </is>
       </c>
-      <c r="K28" s="19">
-        <f>prior column's total store-channel revenue. Base you're applying comps to — not new-store contribution.</f>
-        <v/>
+      <c r="K28" s="19" t="inlineStr">
+        <is>
+          <t>'=prior column's total store-channel revenue. Base you're applying comps to — not new-store contribution.</t>
+        </is>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
@@ -4117,9 +4126,10 @@
           <t>Revenue Drivers: comp-store formula</t>
         </is>
       </c>
-      <c r="K29" s="19">
-        <f>prior store rev×(71%×(1+Am comp)+16%×(1+China)+13%×(1+RoW)). Existing base only — new stores are on the next row.</f>
-        <v/>
+      <c r="K29" s="19" t="inlineStr">
+        <is>
+          <t>'=prior store rev×(71%×(1+Am comp)+16%×(1+China)+13%×(1+RoW)). Existing base only — new stores are on the next row.</t>
+        </is>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
@@ -4161,9 +4171,10 @@
           <t>Revenue Drivers: net-new-store formula</t>
         </is>
       </c>
-      <c r="K30" s="19">
-        <f>(open−close each geo)×sq ft×$/sq ft → raw annual $. /1000 flips that to $000 (this whole tab is thousands). ×0.55 = year-one haircut — new boxes don't run at full SPSF yet. FY27 ex: (D7−D8+D11−D12+D15−D16)×D19×D24/1000×0.55.</f>
-        <v/>
+      <c r="K30" s="19" t="inlineStr">
+        <is>
+          <t>'=(open−close each geo)×sq ft×$/sq ft → raw annual $. /1000 flips that to $000 (this whole tab is thousands). ×0.55 = year-one haircut — new boxes don't run at full SPSF yet. FY27 ex: (D7−D8+D11−D12+D15−D16)×D19×D24/1000×0.55.</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
@@ -4205,9 +4216,10 @@
           <t>Revenue Drivers: store-channel formula</t>
         </is>
       </c>
-      <c r="K31" s="19">
-        <f>comparable store revenue + net new store revenue. Full brick-and-mortar channel for the year.</f>
-        <v/>
+      <c r="K31" s="19" t="inlineStr">
+        <is>
+          <t>'=comparable store revenue + net new store revenue. Full brick-and-mortar channel for the year.</t>
+        </is>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
@@ -4563,9 +4575,10 @@
           <t>Revenue Drivers: e-comm formula</t>
         </is>
       </c>
-      <c r="K41" s="19">
-        <f>sessions×1,000,000×conversion×AOV/1000 → e-comm $000. ×1M 'cause sessions are millions; /1000 matches tab units.</f>
-        <v/>
+      <c r="K41" s="19" t="inlineStr">
+        <is>
+          <t>'=sessions×1,000,000×conversion×AOV/1000 → e-comm $000. ×1M 'cause sessions are millions; /1000 matches tab units.</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -5067,9 +5080,10 @@
           <t>Revenue Drivers: total-rev formula</t>
         </is>
       </c>
-      <c r="K55" s="19">
-        <f>store channel + e-commerce + other. Bottom-up top line before you reconcile to Scenarios.</f>
-        <v/>
+      <c r="K55" s="19" t="inlineStr">
+        <is>
+          <t>'=store channel + e-commerce + other. Bottom-up top line before you reconcile to Scenarios.</t>
+        </is>
       </c>
     </row>
     <row r="56" ht="28" customHeight="1">
@@ -5111,9 +5125,10 @@
           <t>Scenarios tab: base revenue</t>
         </is>
       </c>
-      <c r="K56" s="19">
-        <f>Scenarios! base-case revenue. DCF still runs off this path — not the driver total.</f>
-        <v/>
+      <c r="K56" s="19" t="inlineStr">
+        <is>
+          <t>'=Scenarios! base-case revenue. DCF still runs off this path — not the driver total.</t>
+        </is>
       </c>
     </row>
     <row r="57" ht="28" customHeight="1">
@@ -5156,9 +5171,10 @@
           <t>Revenue Drivers: variance formula</t>
         </is>
       </c>
-      <c r="K57" s="19">
-        <f>bottom-up total − Scenarios revenue. Positive = drivers above Scenarios; negative = below.</f>
-        <v/>
+      <c r="K57" s="19" t="inlineStr">
+        <is>
+          <t>'=bottom-up total − Scenarios revenue. Positive = drivers above Scenarios; negative = below.</t>
+        </is>
       </c>
     </row>
     <row r="58" ht="28" customHeight="1">
@@ -5201,9 +5217,10 @@
           <t>Revenue Drivers: variance % formula</t>
         </is>
       </c>
-      <c r="K58" s="19">
-        <f>variance ÷ Scenarios revenue. Quick % read on how far the driver build is from the valuation path.</f>
-        <v/>
+      <c r="K58" s="19" t="inlineStr">
+        <is>
+          <t>'=variance ÷ Scenarios revenue. Quick % read on how far the driver build is from the valuation path.</t>
+        </is>
       </c>
     </row>
     <row r="59">

</xml_diff>

<commit_message>
Move equation explanations into Justification column (I)
Formula notes were in Ctrl+F (K) where Excel ate them and users
wouldn't look. Now every formula row shows a Formula: line in col I.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -2990,7 +2990,7 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="36" customWidth="1" min="11" max="11"/>
   </cols>
@@ -3022,7 +3022,7 @@
     <row r="3">
       <c r="I3" s="43" t="inlineStr">
         <is>
-          <t>Justification (~20 words)</t>
+          <t>Justification + formula (~20 words)</t>
         </is>
       </c>
       <c r="J3" s="43" t="inlineStr">
@@ -3100,7 +3100,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1">
+    <row r="6" ht="56" customHeight="1">
       <c r="A6" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Americas — beginning stores</t>
@@ -3134,19 +3134,15 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I6" s="17" t="inlineStr">
-        <is>
-          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.
+Formula: prior-year ending stores. Same count, new column — that's where the year starts.</t>
         </is>
       </c>
       <c r="J6" s="51" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
-        </is>
-      </c>
-      <c r="K6" s="19" t="inlineStr">
-        <is>
-          <t>'=prior-year ending stores. Same count, new column — that's where the year starts.</t>
         </is>
       </c>
     </row>
@@ -3234,7 +3230,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="56" customHeight="1">
       <c r="A9" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">  Americas — ending stores</t>
@@ -3268,9 +3264,10 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I9" s="17" t="inlineStr">
-        <is>
-          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.
+Formula: beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
         </is>
       </c>
       <c r="J9" s="51" t="inlineStr">
@@ -3278,13 +3275,8 @@
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
       </c>
-      <c r="K9" s="19" t="inlineStr">
-        <is>
-          <t>'=beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
+    </row>
+    <row r="10" ht="56" customHeight="1">
       <c r="A10" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  China Mainland — beginning stores</t>
@@ -3318,19 +3310,15 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I10" s="17" t="inlineStr">
-        <is>
-          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
+      <c r="I10" s="19" t="inlineStr">
+        <is>
+          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.
+Formula: prior-year ending stores. Same count, new column — that's where the year starts.</t>
         </is>
       </c>
       <c r="J10" s="51" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
-        </is>
-      </c>
-      <c r="K10" s="19" t="inlineStr">
-        <is>
-          <t>'=prior-year ending stores. Same count, new column — that's where the year starts.</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3406,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="28" customHeight="1">
+    <row r="13" ht="56" customHeight="1">
       <c r="A13" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">  China Mainland — ending stores</t>
@@ -3452,9 +3440,10 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I13" s="17" t="inlineStr">
-        <is>
-          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
+      <c r="I13" s="19" t="inlineStr">
+        <is>
+          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.
+Formula: beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
         </is>
       </c>
       <c r="J13" s="51" t="inlineStr">
@@ -3462,13 +3451,8 @@
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
       </c>
-      <c r="K13" s="19" t="inlineStr">
-        <is>
-          <t>'=beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
+    </row>
+    <row r="14" ht="56" customHeight="1">
       <c r="A14" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rest of World — beginning stores</t>
@@ -3502,19 +3486,15 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I14" s="17" t="inlineStr">
-        <is>
-          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
+      <c r="I14" s="19" t="inlineStr">
+        <is>
+          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.
+Formula: prior-year ending stores. Same count, new column — that's where the year starts.</t>
         </is>
       </c>
       <c r="J14" s="51" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
-        </is>
-      </c>
-      <c r="K14" s="19" t="inlineStr">
-        <is>
-          <t>'=prior-year ending stores. Same count, new column — that's where the year starts.</t>
         </is>
       </c>
     </row>
@@ -3602,7 +3582,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="56" customHeight="1">
       <c r="A17" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rest of World — ending stores</t>
@@ -3636,9 +3616,10 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I17" s="17" t="inlineStr">
-        <is>
-          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
+      <c r="I17" s="19" t="inlineStr">
+        <is>
+          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.
+Formula: beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
         </is>
       </c>
       <c r="J17" s="51" t="inlineStr">
@@ -3646,13 +3627,8 @@
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
       </c>
-      <c r="K17" s="19" t="inlineStr">
-        <is>
-          <t>'=beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="28" customHeight="1">
+    </row>
+    <row r="18" ht="56" customHeight="1">
       <c r="A18" s="53" t="inlineStr">
         <is>
           <t>Total ending stores</t>
@@ -3681,19 +3657,15 @@
         <f>G9+G13+G17</f>
         <v/>
       </c>
-      <c r="I18" s="17" t="inlineStr">
-        <is>
-          <t>Add up Americas + China + RoW ending stores. Should tie to the 10-K total company-operated count.</t>
+      <c r="I18" s="19" t="inlineStr">
+        <is>
+          <t>Add up Americas + China + RoW ending stores. Should tie to the 10-K total company-operated count.
+Formula: Americas ending + China ending + RoW ending. Should foot to total company-operated stores.</t>
         </is>
       </c>
       <c r="J18" s="51" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-stores formula</t>
-        </is>
-      </c>
-      <c r="K18" s="19" t="inlineStr">
-        <is>
-          <t>'=Americas ending + China ending + RoW ending. Should foot to total company-operated stores.</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3714,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="28" customHeight="1">
+    <row r="20" ht="56" customHeight="1">
       <c r="A20" s="34" t="inlineStr">
         <is>
           <t>Total square footage (end stores × avg sq ft)</t>
@@ -3777,19 +3749,15 @@
           <t>sq ft</t>
         </is>
       </c>
-      <c r="I20" s="17" t="inlineStr">
-        <is>
-          <t>Ending stores times avg sq ft per box. Gives you total fleet square footage for the productivity math.</t>
+      <c r="I20" s="19" t="inlineStr">
+        <is>
+          <t>Ending stores times avg sq ft per box. Gives you total fleet square footage for the productivity math.
+Formula: total ending stores × avg sq ft per store. Fleet size in square feet for the productivity lines.</t>
         </is>
       </c>
       <c r="J20" s="51" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-sqft formula</t>
-        </is>
-      </c>
-      <c r="K20" s="19" t="inlineStr">
-        <is>
-          <t>'=total ending stores × avg sq ft per store. Fleet size in square feet for the productivity lines.</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4005,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
+    <row r="28" ht="56" customHeight="1">
       <c r="A28" s="34" t="inlineStr">
         <is>
           <t>Prior-year store channel revenue ($000)</t>
@@ -4071,9 +4039,10 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I28" s="17" t="inlineStr">
-        <is>
-          <t>Last year's total store-channel revenue — the base you're growing comps off of, not the new boxes.</t>
+      <c r="I28" s="19" t="inlineStr">
+        <is>
+          <t>Last year's total store-channel revenue — the base you're growing comps off of, not the new boxes.
+Formula: prior column's total store-channel revenue. Base you're applying comps to — not new-store contribution.</t>
         </is>
       </c>
       <c r="J28" s="51" t="inlineStr">
@@ -4081,13 +4050,8 @@
           <t>Revenue Drivers: prior store-rev formula</t>
         </is>
       </c>
-      <c r="K28" s="19" t="inlineStr">
-        <is>
-          <t>'=prior column's total store-channel revenue. Base you're applying comps to — not new-store contribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="28" customHeight="1">
+    </row>
+    <row r="29" ht="56" customHeight="1">
       <c r="A29" s="34" t="inlineStr">
         <is>
           <t>Comparable store revenue ($000)</t>
@@ -4116,9 +4080,10 @@
         <f>F28*0.71*(1+G25)+F28*0.16*(1+G26)+F28*0.13*(1+G27)</f>
         <v/>
       </c>
-      <c r="I29" s="17" t="inlineStr">
-        <is>
-          <t>Existing-store sales only — prior store rev grown by geo comp %. New doors are a separate line, not in here.</t>
+      <c r="I29" s="19" t="inlineStr">
+        <is>
+          <t>Existing-store sales only — prior store rev grown by geo comp %. New doors are a separate line, not in here.
+Formula: prior store rev×(71%×(1+Am comp)+16%×(1+China)+13%×(1+RoW)). Existing base only — new stores are on the next row.</t>
         </is>
       </c>
       <c r="J29" s="51" t="inlineStr">
@@ -4126,13 +4091,8 @@
           <t>Revenue Drivers: comp-store formula</t>
         </is>
       </c>
-      <c r="K29" s="19" t="inlineStr">
-        <is>
-          <t>'=prior store rev×(71%×(1+Am comp)+16%×(1+China)+13%×(1+RoW)). Existing base only — new stores are on the next row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="28" customHeight="1">
+    </row>
+    <row r="30" ht="56" customHeight="1">
       <c r="A30" s="34" t="inlineStr">
         <is>
           <t>Net new store revenue contribution ($000)</t>
@@ -4161,9 +4121,10 @@
         <f>(G7-G8+G11-G12+G15-G16)*G19*G24/1000*0.55</f>
         <v/>
       </c>
-      <c r="I30" s="17" t="inlineStr">
-        <is>
-          <t>Net new doors × sq ft × $/sq ft is plain dollars. /1000 → $000 on this tab. ×0.55 'cause year-one stores don't run full.</t>
+      <c r="I30" s="19" t="inlineStr">
+        <is>
+          <t>Net new doors × sq ft × $/sq ft is plain dollars. /1000 → $000 on this tab. ×0.55 'cause year-one stores don't run full.
+Formula: (open−close each geo)×sq ft×$/sq ft → raw annual $. /1000 flips that to $000 (this whole tab is thousands). ×0.55 = year-one haircut — new boxes don't run at full SPSF yet. FY27 ex: (D7−D8+D11−D12+D15−D16)×D19×D24/1000×0.55.</t>
         </is>
       </c>
       <c r="J30" s="51" t="inlineStr">
@@ -4171,13 +4132,8 @@
           <t>Revenue Drivers: net-new-store formula</t>
         </is>
       </c>
-      <c r="K30" s="19" t="inlineStr">
-        <is>
-          <t>'=(open−close each geo)×sq ft×$/sq ft → raw annual $. /1000 flips that to $000 (this whole tab is thousands). ×0.55 = year-one haircut — new boxes don't run at full SPSF yet. FY27 ex: (D7−D8+D11−D12+D15−D16)×D19×D24/1000×0.55.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1">
+    </row>
+    <row r="31" ht="56" customHeight="1">
       <c r="A31" s="53" t="inlineStr">
         <is>
           <t>Store channel revenue ($000)</t>
@@ -4206,19 +4162,15 @@
         <f>G29+G30</f>
         <v/>
       </c>
-      <c r="I31" s="17" t="inlineStr">
-        <is>
-          <t>Brick-and-mortar channel = comp store sales plus whatever the net new stores contributed. That's the whole store line.</t>
+      <c r="I31" s="19" t="inlineStr">
+        <is>
+          <t>Brick-and-mortar channel = comp store sales plus whatever the net new stores contributed. That's the whole store line.
+Formula: comparable store revenue + net new store revenue. Full brick-and-mortar channel for the year.</t>
         </is>
       </c>
       <c r="J31" s="51" t="inlineStr">
         <is>
           <t>Revenue Drivers: store-channel formula</t>
-        </is>
-      </c>
-      <c r="K31" s="19" t="inlineStr">
-        <is>
-          <t>'=comparable store revenue + net new store revenue. Full brick-and-mortar channel for the year.</t>
         </is>
       </c>
     </row>
@@ -4536,7 +4488,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="28" customHeight="1">
+    <row r="41" ht="56" customHeight="1">
       <c r="A41" s="53" t="inlineStr">
         <is>
           <t>E-commerce revenue ($000)</t>
@@ -4565,19 +4517,15 @@
         <f>G38*1000000*G39*G40/1000</f>
         <v/>
       </c>
-      <c r="I41" s="17" t="inlineStr">
-        <is>
-          <t>Traffic × conversion × AOV is dollars. ×1M 'cause sessions are in millions; /1000 puts it in $000 like everything else.</t>
+      <c r="I41" s="19" t="inlineStr">
+        <is>
+          <t>Traffic × conversion × AOV is dollars. ×1M 'cause sessions are in millions; /1000 puts it in $000 like everything else.
+Formula: sessions×1,000,000×conversion×AOV/1000 → e-comm $000. ×1M 'cause sessions are millions; /1000 matches tab units.</t>
         </is>
       </c>
       <c r="J41" s="51" t="inlineStr">
         <is>
           <t>Revenue Drivers: e-comm formula</t>
-        </is>
-      </c>
-      <c r="K41" s="19" t="inlineStr">
-        <is>
-          <t>'=sessions×1,000,000×conversion×AOV/1000 → e-comm $000. ×1M 'cause sessions are millions; /1000 matches tab units.</t>
         </is>
       </c>
     </row>
@@ -4645,7 +4593,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="42" customHeight="1">
+    <row r="45" ht="56" customHeight="1">
       <c r="A45" s="34" t="inlineStr">
         <is>
           <t>Other channels (wholesale / license / outlets) ($000)</t>
@@ -4682,23 +4630,21 @@
       <c r="I45" s="19" t="inlineStr">
         <is>
           <t>Other channels (wholesale/license/outlets) held at FY25 $1.13B base; low-single-digit growth thereafter.
-Formula: Take last year's other-channel revenue and grow it by your assumed %. Wholesale/license/outlets — not stores or dot-com.</t>
-        </is>
-      </c>
-      <c r="J45" s="22" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: channel revenue table
-Formula: Revenue Drivers: other-rev formula</t>
+Formula: prior other-channel rev × (1 + growth %). Wholesale/license/outlets — grown off last year.</t>
+        </is>
+      </c>
+      <c r="J45" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: channel revenue table</t>
         </is>
       </c>
       <c r="K45" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Company-operated stores" and "E-commerce" → residual other channels ≈ $1.13B.
-Formula: =prior other-channel rev × (1 + growth %). Wholesale/license/outlets — grown off last year.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="42" customHeight="1">
+          <t>Ctrl+F "Company-operated stores" and "E-commerce" → residual other channels ≈ $1.13B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="56" customHeight="1">
       <c r="A46" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Americas net revenue ($000)</t>
@@ -4735,23 +4681,21 @@
       <c r="I46" s="19" t="inlineStr">
         <is>
           <t>Geographic split scales with consolidated growth; FY25 Americas 70.7% of revenue per 10-K segment table.
-Formula: Hold the FY25 geo mix, scale each region by how much total revenue grew vs last year. Quick way to split the top line.</t>
-        </is>
-      </c>
-      <c r="J46" s="22" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: segmented net revenue
-Formula: Revenue Drivers: geo-scale formula</t>
+Formula: FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
+        </is>
+      </c>
+      <c r="J46" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
       <c r="K46" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Americas" segment table → $7,847,044 net revenue (70.7%).
-Formula: =FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="42" customHeight="1">
+          <t>Ctrl+F "Americas" segment table → $7,847,044 net revenue (70.7%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="56" customHeight="1">
       <c r="A47" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  China Mainland net revenue ($000)</t>
@@ -4788,23 +4732,21 @@
       <c r="I47" s="19" t="inlineStr">
         <is>
           <t>China 15.8% of FY25 revenue; fastest comp and store growth — expansion market in the driver schedule.
-Formula: Hold the FY25 geo mix, scale each region by how much total revenue grew vs last year. Quick way to split the top line.</t>
-        </is>
-      </c>
-      <c r="J47" s="22" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: segmented net revenue
-Formula: Revenue Drivers: geo-scale formula</t>
+Formula: FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
+        </is>
+      </c>
+      <c r="J47" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
       <c r="K47" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "China Mainland" segment → $1,754,799 net revenue (15.8%).
-Formula: =FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="42" customHeight="1">
+          <t>Ctrl+F "China Mainland" segment → $1,754,799 net revenue (15.8%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="56" customHeight="1">
       <c r="A48" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rest of World net revenue ($000)</t>
@@ -4841,19 +4783,17 @@
       <c r="I48" s="19" t="inlineStr">
         <is>
           <t>Rest of World 13.5% of FY25 revenue; mid-single-digit comps and steady openings.
-Formula: Hold the FY25 geo mix, scale each region by how much total revenue grew vs last year. Quick way to split the top line.</t>
-        </is>
-      </c>
-      <c r="J48" s="22" t="inlineStr">
-        <is>
-          <t>FY2025 10-K: segmented net revenue
-Formula: Revenue Drivers: geo-scale formula</t>
+Formula: FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
+        </is>
+      </c>
+      <c r="J48" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
       <c r="K48" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Rest of World" segment → $1,500,757 net revenue (13.5%).
-Formula: =FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
+          <t>Ctrl+F "Rest of World" segment → $1,500,757 net revenue (13.5%).</t>
         </is>
       </c>
     </row>
@@ -5041,7 +4981,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="28" customHeight="1">
+    <row r="55" ht="56" customHeight="1">
       <c r="A55" s="60" t="inlineStr">
         <is>
           <t>Bottom-up total revenue ($000)</t>
@@ -5070,9 +5010,10 @@
         <f>G31+G41+G45</f>
         <v/>
       </c>
-      <c r="I55" s="17" t="inlineStr">
-        <is>
-          <t>Bottom-up total = store channel + e-comm + other. That's your driver-built revenue before you check Scenarios.</t>
+      <c r="I55" s="19" t="inlineStr">
+        <is>
+          <t>Bottom-up total = store channel + e-comm + other. That's your driver-built revenue before you check Scenarios.
+Formula: store channel + e-commerce + other. Bottom-up top line before you reconcile to Scenarios.</t>
         </is>
       </c>
       <c r="J55" s="51" t="inlineStr">
@@ -5080,13 +5021,8 @@
           <t>Revenue Drivers: total-rev formula</t>
         </is>
       </c>
-      <c r="K55" s="19" t="inlineStr">
-        <is>
-          <t>'=store channel + e-commerce + other. Bottom-up top line before you reconcile to Scenarios.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="28" customHeight="1">
+    </row>
+    <row r="56" ht="56" customHeight="1">
       <c r="A56" s="34" t="inlineStr">
         <is>
           <t>Scenarios base-case revenue ($000)</t>
@@ -5115,9 +5051,10 @@
         <f>Scenarios!G22</f>
         <v/>
       </c>
-      <c r="I56" s="17" t="inlineStr">
-        <is>
-          <t>Pulls the Scenarios base-case revenue path — that's still the number the DCF actually uses, not the driver total.</t>
+      <c r="I56" s="19" t="inlineStr">
+        <is>
+          <t>Pulls the Scenarios base-case revenue path — that's still the number the DCF actually uses, not the driver total.
+Formula: Scenarios! base-case revenue. DCF still runs off this path — not the driver total.</t>
         </is>
       </c>
       <c r="J56" s="51" t="inlineStr">
@@ -5125,13 +5062,8 @@
           <t>Scenarios tab: base revenue</t>
         </is>
       </c>
-      <c r="K56" s="19" t="inlineStr">
-        <is>
-          <t>'=Scenarios! base-case revenue. DCF still runs off this path — not the driver total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="28" customHeight="1">
+    </row>
+    <row r="57" ht="56" customHeight="1">
       <c r="A57" s="34" t="inlineStr">
         <is>
           <t>Variance (bottom-up − scenarios) ($000)</t>
@@ -5161,9 +5093,10 @@
         <f>G55-G56</f>
         <v/>
       </c>
-      <c r="I57" s="17" t="inlineStr">
-        <is>
-          <t>Driver-built revenue minus Scenarios revenue. Shows you how far off the bottom-up path is from what you're valuing on.</t>
+      <c r="I57" s="19" t="inlineStr">
+        <is>
+          <t>Driver-built revenue minus Scenarios revenue. Shows you how far off the bottom-up path is from what you're valuing on.
+Formula: bottom-up total − Scenarios revenue. Positive = drivers above Scenarios; negative = below.</t>
         </is>
       </c>
       <c r="J57" s="51" t="inlineStr">
@@ -5171,13 +5104,8 @@
           <t>Revenue Drivers: variance formula</t>
         </is>
       </c>
-      <c r="K57" s="19" t="inlineStr">
-        <is>
-          <t>'=bottom-up total − Scenarios revenue. Positive = drivers above Scenarios; negative = below.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="28" customHeight="1">
+    </row>
+    <row r="58" ht="56" customHeight="1">
       <c r="A58" s="34" t="inlineStr">
         <is>
           <t>Variance (%)</t>
@@ -5207,19 +5135,15 @@
         <f>IF(G56=0,"",G57/G56)</f>
         <v/>
       </c>
-      <c r="I58" s="17" t="inlineStr">
-        <is>
-          <t>Variance as a percent of Scenarios revenue. Easy read on whether the driver schedule is close or way out of line.</t>
+      <c r="I58" s="19" t="inlineStr">
+        <is>
+          <t>Variance as a percent of Scenarios revenue. Easy read on whether the driver schedule is close or way out of line.
+Formula: variance ÷ Scenarios revenue. Quick % read on how far the driver build is from the valuation path.</t>
         </is>
       </c>
       <c r="J58" s="51" t="inlineStr">
         <is>
           <t>Revenue Drivers: variance % formula</t>
-        </is>
-      </c>
-      <c r="K58" s="19" t="inlineStr">
-        <is>
-          <t>'=variance ÷ Scenarios revenue. Quick % read on how far the driver build is from the valuation path.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add dedicated Equation column on Revenue Drivers tab
Column I now shows how every formula row is built. Justification,
Source, and Ctrl+F shift to J/K/L so equations are impossible to miss.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -399,7 +399,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -522,6 +522,9 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -2979,7 +2982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2990,9 +2993,10 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3011,6 +3015,7 @@
       <c r="I1" s="13" t="n"/>
       <c r="J1" s="13" t="n"/>
       <c r="K1" s="13" t="n"/>
+      <c r="L1" s="13" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="26" t="inlineStr">
@@ -3022,15 +3027,20 @@
     <row r="3">
       <c r="I3" s="43" t="inlineStr">
         <is>
-          <t>Justification + formula (~20 words)</t>
+          <t>Equation (every formula row)</t>
         </is>
       </c>
       <c r="J3" s="43" t="inlineStr">
         <is>
+          <t>Justification (~20 words)</t>
+        </is>
+      </c>
+      <c r="K3" s="43" t="inlineStr">
+        <is>
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="K3" s="43" t="inlineStr">
+      <c r="L3" s="43" t="inlineStr">
         <is>
           <t>Ctrl+F (prove number)</t>
         </is>
@@ -3084,23 +3094,28 @@
           <t>Units</t>
         </is>
       </c>
-      <c r="I5" s="48" t="inlineStr">
+      <c r="I5" s="47" t="inlineStr">
+        <is>
+          <t>Equation</t>
+        </is>
+      </c>
+      <c r="J5" s="48" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="J5" s="48" t="inlineStr">
+      <c r="K5" s="48" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="K5" s="48" t="inlineStr">
+      <c r="L5" s="48" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="56" customHeight="1">
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Americas — beginning stores</t>
@@ -3134,13 +3149,17 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I6" s="19" t="inlineStr">
-        <is>
-          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.
-Formula: prior-year ending stores. Same count, new column — that's where the year starts.</t>
-        </is>
-      </c>
-      <c r="J6" s="51" t="inlineStr">
+      <c r="I6" s="51" t="inlineStr">
+        <is>
+          <t>prior-year ending stores. Same count, new column — that's where the year starts.</t>
+        </is>
+      </c>
+      <c r="J6" s="17" t="inlineStr">
+        <is>
+          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
+        </is>
+      </c>
+      <c r="K6" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
@@ -3152,19 +3171,19 @@
           <t xml:space="preserve">  Americas — openings</t>
         </is>
       </c>
-      <c r="C7" s="52" t="n">
+      <c r="C7" s="53" t="n">
         <v>8</v>
       </c>
-      <c r="D7" s="52" t="n">
+      <c r="D7" s="53" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="52" t="n">
+      <c r="E7" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="F7" s="52" t="n">
+      <c r="F7" s="53" t="n">
         <v>5</v>
       </c>
-      <c r="G7" s="52" t="n">
+      <c r="G7" s="53" t="n">
         <v>4</v>
       </c>
       <c r="H7" s="50" t="inlineStr">
@@ -3172,17 +3191,17 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I7" s="17" t="inlineStr">
+      <c r="J7" s="17" t="inlineStr">
         <is>
           <t>Store openings skew to China (+20 FY26) vs mature Americas (+8). Anchored to FY25 +44 net stores and 11% sq-ft growth.</t>
         </is>
       </c>
-      <c r="J7" s="18" t="inlineStr">
+      <c r="K7" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: store count &amp; expansion</t>
         </is>
       </c>
-      <c r="K7" s="19" t="inlineStr">
+      <c r="L7" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Total company-operated stores" → 811 (FY25). FY25 added 44 net stores; model skews openings to China.</t>
         </is>
@@ -3194,19 +3213,19 @@
           <t xml:space="preserve">  Americas — closures</t>
         </is>
       </c>
-      <c r="C8" s="52" t="n">
+      <c r="C8" s="53" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="52" t="n">
+      <c r="D8" s="53" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="52" t="n">
+      <c r="E8" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="52" t="n">
+      <c r="F8" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="52" t="n">
+      <c r="G8" s="53" t="n">
         <v>2</v>
       </c>
       <c r="H8" s="50" t="inlineStr">
@@ -3214,24 +3233,24 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I8" s="17" t="inlineStr">
+      <c r="J8" s="17" t="inlineStr">
         <is>
           <t>Closures assume 2–3 per mature region annually as leases roll; immaterial vs openings in expansion markets.</t>
         </is>
       </c>
-      <c r="J8" s="18" t="inlineStr">
+      <c r="K8" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: lease renewal / fleet</t>
         </is>
       </c>
-      <c r="K8" s="19" t="inlineStr">
+      <c r="L8" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "lease" / store fleet — immaterial closures vs expansion; 2–3 per mature region.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="56" customHeight="1">
-      <c r="A9" s="53" t="inlineStr">
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="54" t="inlineStr">
         <is>
           <t xml:space="preserve">  Americas — ending stores</t>
         </is>
@@ -3239,23 +3258,23 @@
       <c r="B9" s="49" t="n">
         <v>476</v>
       </c>
-      <c r="C9" s="54">
+      <c r="C9" s="55">
         <f>C6+C7-C8</f>
         <v/>
       </c>
-      <c r="D9" s="54">
+      <c r="D9" s="55">
         <f>D6+D7-D8</f>
         <v/>
       </c>
-      <c r="E9" s="54">
+      <c r="E9" s="55">
         <f>E6+E7-E8</f>
         <v/>
       </c>
-      <c r="F9" s="54">
+      <c r="F9" s="55">
         <f>F6+F7-F8</f>
         <v/>
       </c>
-      <c r="G9" s="54">
+      <c r="G9" s="55">
         <f>G6+G7-G8</f>
         <v/>
       </c>
@@ -3264,19 +3283,23 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I9" s="19" t="inlineStr">
-        <is>
-          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.
-Formula: beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
-        </is>
-      </c>
-      <c r="J9" s="51" t="inlineStr">
+      <c r="I9" s="51" t="inlineStr">
+        <is>
+          <t>beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
+        </is>
+      </c>
+      <c r="J9" s="17" t="inlineStr">
+        <is>
+          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
+        </is>
+      </c>
+      <c r="K9" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="56" customHeight="1">
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  China Mainland — beginning stores</t>
@@ -3310,13 +3333,17 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I10" s="19" t="inlineStr">
-        <is>
-          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.
-Formula: prior-year ending stores. Same count, new column — that's where the year starts.</t>
-        </is>
-      </c>
-      <c r="J10" s="51" t="inlineStr">
+      <c r="I10" s="51" t="inlineStr">
+        <is>
+          <t>prior-year ending stores. Same count, new column — that's where the year starts.</t>
+        </is>
+      </c>
+      <c r="J10" s="17" t="inlineStr">
+        <is>
+          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
+        </is>
+      </c>
+      <c r="K10" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
@@ -3328,19 +3355,19 @@
           <t xml:space="preserve">  China Mainland — openings</t>
         </is>
       </c>
-      <c r="C11" s="52" t="n">
+      <c r="C11" s="53" t="n">
         <v>20</v>
       </c>
-      <c r="D11" s="52" t="n">
+      <c r="D11" s="53" t="n">
         <v>18</v>
       </c>
-      <c r="E11" s="52" t="n">
+      <c r="E11" s="53" t="n">
         <v>16</v>
       </c>
-      <c r="F11" s="52" t="n">
+      <c r="F11" s="53" t="n">
         <v>14</v>
       </c>
-      <c r="G11" s="52" t="n">
+      <c r="G11" s="53" t="n">
         <v>12</v>
       </c>
       <c r="H11" s="50" t="inlineStr">
@@ -3348,17 +3375,17 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I11" s="17" t="inlineStr">
+      <c r="J11" s="17" t="inlineStr">
         <is>
           <t>Store openings skew to China (+20 FY26) vs mature Americas (+8). Anchored to FY25 +44 net stores and 11% sq-ft growth.</t>
         </is>
       </c>
-      <c r="J11" s="18" t="inlineStr">
+      <c r="K11" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: store count &amp; expansion</t>
         </is>
       </c>
-      <c r="K11" s="19" t="inlineStr">
+      <c r="L11" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Total company-operated stores" → 811 (FY25). FY25 added 44 net stores; model skews openings to China.</t>
         </is>
@@ -3370,19 +3397,19 @@
           <t xml:space="preserve">  China Mainland — closures</t>
         </is>
       </c>
-      <c r="C12" s="52" t="n">
+      <c r="C12" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="52" t="n">
+      <c r="D12" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="52" t="n">
+      <c r="E12" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="52" t="n">
+      <c r="F12" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="52" t="n">
+      <c r="G12" s="53" t="n">
         <v>1</v>
       </c>
       <c r="H12" s="50" t="inlineStr">
@@ -3390,24 +3417,24 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I12" s="17" t="inlineStr">
+      <c r="J12" s="17" t="inlineStr">
         <is>
           <t>Closures assume 2–3 per mature region annually as leases roll; immaterial vs openings in expansion markets.</t>
         </is>
       </c>
-      <c r="J12" s="18" t="inlineStr">
+      <c r="K12" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: lease renewal / fleet</t>
         </is>
       </c>
-      <c r="K12" s="19" t="inlineStr">
+      <c r="L12" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "lease" / store fleet — immaterial closures vs expansion; 2–3 per mature region.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="56" customHeight="1">
-      <c r="A13" s="53" t="inlineStr">
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="54" t="inlineStr">
         <is>
           <t xml:space="preserve">  China Mainland — ending stores</t>
         </is>
@@ -3415,23 +3442,23 @@
       <c r="B13" s="49" t="n">
         <v>172</v>
       </c>
-      <c r="C13" s="54">
+      <c r="C13" s="55">
         <f>C10+C11-C12</f>
         <v/>
       </c>
-      <c r="D13" s="54">
+      <c r="D13" s="55">
         <f>D10+D11-D12</f>
         <v/>
       </c>
-      <c r="E13" s="54">
+      <c r="E13" s="55">
         <f>E10+E11-E12</f>
         <v/>
       </c>
-      <c r="F13" s="54">
+      <c r="F13" s="55">
         <f>F10+F11-F12</f>
         <v/>
       </c>
-      <c r="G13" s="54">
+      <c r="G13" s="55">
         <f>G10+G11-G12</f>
         <v/>
       </c>
@@ -3440,19 +3467,23 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I13" s="19" t="inlineStr">
-        <is>
-          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.
-Formula: beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
-        </is>
-      </c>
-      <c r="J13" s="51" t="inlineStr">
+      <c r="I13" s="51" t="inlineStr">
+        <is>
+          <t>beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
+        </is>
+      </c>
+      <c r="J13" s="17" t="inlineStr">
+        <is>
+          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
+        </is>
+      </c>
+      <c r="K13" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="56" customHeight="1">
+    <row r="14" ht="28" customHeight="1">
       <c r="A14" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rest of World — beginning stores</t>
@@ -3486,13 +3517,17 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I14" s="19" t="inlineStr">
-        <is>
-          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.
-Formula: prior-year ending stores. Same count, new column — that's where the year starts.</t>
-        </is>
-      </c>
-      <c r="J14" s="51" t="inlineStr">
+      <c r="I14" s="51" t="inlineStr">
+        <is>
+          <t>prior-year ending stores. Same count, new column — that's where the year starts.</t>
+        </is>
+      </c>
+      <c r="J14" s="17" t="inlineStr">
+        <is>
+          <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
+        </is>
+      </c>
+      <c r="K14" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
@@ -3504,19 +3539,19 @@
           <t xml:space="preserve">  Rest of World — openings</t>
         </is>
       </c>
-      <c r="C15" s="52" t="n">
+      <c r="C15" s="53" t="n">
         <v>7</v>
       </c>
-      <c r="D15" s="52" t="n">
+      <c r="D15" s="53" t="n">
         <v>6</v>
       </c>
-      <c r="E15" s="52" t="n">
+      <c r="E15" s="53" t="n">
         <v>5</v>
       </c>
-      <c r="F15" s="52" t="n">
+      <c r="F15" s="53" t="n">
         <v>5</v>
       </c>
-      <c r="G15" s="52" t="n">
+      <c r="G15" s="53" t="n">
         <v>4</v>
       </c>
       <c r="H15" s="50" t="inlineStr">
@@ -3524,17 +3559,17 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I15" s="17" t="inlineStr">
+      <c r="J15" s="17" t="inlineStr">
         <is>
           <t>Store openings skew to China (+20 FY26) vs mature Americas (+8). Anchored to FY25 +44 net stores and 11% sq-ft growth.</t>
         </is>
       </c>
-      <c r="J15" s="18" t="inlineStr">
+      <c r="K15" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: store count &amp; expansion</t>
         </is>
       </c>
-      <c r="K15" s="19" t="inlineStr">
+      <c r="L15" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Total company-operated stores" → 811 (FY25). FY25 added 44 net stores; model skews openings to China.</t>
         </is>
@@ -3546,19 +3581,19 @@
           <t xml:space="preserve">  Rest of World — closures</t>
         </is>
       </c>
-      <c r="C16" s="52" t="n">
+      <c r="C16" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="52" t="n">
+      <c r="D16" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="52" t="n">
+      <c r="E16" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="F16" s="52" t="n">
+      <c r="F16" s="53" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="52" t="n">
+      <c r="G16" s="53" t="n">
         <v>2</v>
       </c>
       <c r="H16" s="50" t="inlineStr">
@@ -3566,24 +3601,24 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I16" s="17" t="inlineStr">
+      <c r="J16" s="17" t="inlineStr">
         <is>
           <t>Closures assume 2–3 per mature region annually as leases roll; immaterial vs openings in expansion markets.</t>
         </is>
       </c>
-      <c r="J16" s="18" t="inlineStr">
+      <c r="K16" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: lease renewal / fleet</t>
         </is>
       </c>
-      <c r="K16" s="19" t="inlineStr">
+      <c r="L16" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "lease" / store fleet — immaterial closures vs expansion; 2–3 per mature region.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="56" customHeight="1">
-      <c r="A17" s="53" t="inlineStr">
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="54" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rest of World — ending stores</t>
         </is>
@@ -3591,23 +3626,23 @@
       <c r="B17" s="49" t="n">
         <v>163</v>
       </c>
-      <c r="C17" s="54">
+      <c r="C17" s="55">
         <f>C14+C15-C16</f>
         <v/>
       </c>
-      <c r="D17" s="54">
+      <c r="D17" s="55">
         <f>D14+D15-D16</f>
         <v/>
       </c>
-      <c r="E17" s="54">
+      <c r="E17" s="55">
         <f>E14+E15-E16</f>
         <v/>
       </c>
-      <c r="F17" s="54">
+      <c r="F17" s="55">
         <f>F14+F15-F16</f>
         <v/>
       </c>
-      <c r="G17" s="54">
+      <c r="G17" s="55">
         <f>G14+G15-G16</f>
         <v/>
       </c>
@@ -3616,54 +3651,62 @@
           <t>stores</t>
         </is>
       </c>
-      <c r="I17" s="19" t="inlineStr">
-        <is>
-          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.
-Formula: beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
-        </is>
-      </c>
-      <c r="J17" s="51" t="inlineStr">
+      <c r="I17" s="51" t="inlineStr">
+        <is>
+          <t>beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
+        </is>
+      </c>
+      <c r="J17" s="17" t="inlineStr">
+        <is>
+          <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
+        </is>
+      </c>
+      <c r="K17" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="56" customHeight="1">
-      <c r="A18" s="53" t="inlineStr">
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="54" t="inlineStr">
         <is>
           <t>Total ending stores</t>
         </is>
       </c>
-      <c r="B18" s="55" t="n">
+      <c r="B18" s="56" t="n">
         <v>811</v>
       </c>
-      <c r="C18" s="54">
+      <c r="C18" s="55">
         <f>C9+C13+C17</f>
         <v/>
       </c>
-      <c r="D18" s="54">
+      <c r="D18" s="55">
         <f>D9+D13+D17</f>
         <v/>
       </c>
-      <c r="E18" s="54">
+      <c r="E18" s="55">
         <f>E9+E13+E17</f>
         <v/>
       </c>
-      <c r="F18" s="54">
+      <c r="F18" s="55">
         <f>F9+F13+F17</f>
         <v/>
       </c>
-      <c r="G18" s="54">
+      <c r="G18" s="55">
         <f>G9+G13+G17</f>
         <v/>
       </c>
-      <c r="I18" s="19" t="inlineStr">
-        <is>
-          <t>Add up Americas + China + RoW ending stores. Should tie to the 10-K total company-operated count.
-Formula: Americas ending + China ending + RoW ending. Should foot to total company-operated stores.</t>
-        </is>
-      </c>
-      <c r="J18" s="51" t="inlineStr">
+      <c r="I18" s="51" t="inlineStr">
+        <is>
+          <t>Americas ending + China ending + RoW ending. Should foot to total company-operated stores.</t>
+        </is>
+      </c>
+      <c r="J18" s="17" t="inlineStr">
+        <is>
+          <t>Add up Americas + China + RoW ending stores. Should tie to the 10-K total company-operated count.</t>
+        </is>
+      </c>
+      <c r="K18" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-stores formula</t>
         </is>
@@ -3675,22 +3718,22 @@
           <t>Avg square feet per store</t>
         </is>
       </c>
-      <c r="B19" s="52" t="n">
+      <c r="B19" s="53" t="n">
         <v>4366</v>
       </c>
-      <c r="C19" s="52" t="n">
+      <c r="C19" s="53" t="n">
         <v>4400</v>
       </c>
-      <c r="D19" s="52" t="n">
+      <c r="D19" s="53" t="n">
         <v>4425</v>
       </c>
-      <c r="E19" s="52" t="n">
+      <c r="E19" s="53" t="n">
         <v>4450</v>
       </c>
-      <c r="F19" s="52" t="n">
+      <c r="F19" s="53" t="n">
         <v>4475</v>
       </c>
-      <c r="G19" s="52" t="n">
+      <c r="G19" s="53" t="n">
         <v>4500</v>
       </c>
       <c r="H19" s="50" t="inlineStr">
@@ -3698,23 +3741,23 @@
           <t>sq ft</t>
         </is>
       </c>
-      <c r="I19" s="17" t="inlineStr">
+      <c r="J19" s="17" t="inlineStr">
         <is>
           <t>4,367 avg sq ft/store = implied FY25 total sq ft / 811 stores. Modest expansion to 4,500 by FY30.</t>
         </is>
       </c>
-      <c r="J19" s="18" t="inlineStr">
+      <c r="K19" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: sales per square foot</t>
         </is>
       </c>
-      <c r="K19" s="19" t="inlineStr">
+      <c r="L19" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "sales per square foot were $1,426" → implied 3.54M sq ft / 811 stores ≈ 4,367 sq ft.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="56" customHeight="1">
+    <row r="20" ht="28" customHeight="1">
       <c r="A20" s="34" t="inlineStr">
         <is>
           <t>Total square footage (end stores × avg sq ft)</t>
@@ -3749,13 +3792,17 @@
           <t>sq ft</t>
         </is>
       </c>
-      <c r="I20" s="19" t="inlineStr">
-        <is>
-          <t>Ending stores times avg sq ft per box. Gives you total fleet square footage for the productivity math.
-Formula: total ending stores × avg sq ft per store. Fleet size in square feet for the productivity lines.</t>
-        </is>
-      </c>
-      <c r="J20" s="51" t="inlineStr">
+      <c r="I20" s="51" t="inlineStr">
+        <is>
+          <t>total ending stores × avg sq ft per store. Fleet size in square feet for the productivity lines.</t>
+        </is>
+      </c>
+      <c r="J20" s="17" t="inlineStr">
+        <is>
+          <t>Ending stores times avg sq ft per box. Gives you total fleet square footage for the productivity math.</t>
+        </is>
+      </c>
+      <c r="K20" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-sqft formula</t>
         </is>
@@ -3809,17 +3856,22 @@
           <t>Units</t>
         </is>
       </c>
-      <c r="I23" s="48" t="inlineStr">
+      <c r="I23" s="47" t="inlineStr">
+        <is>
+          <t>Equation</t>
+        </is>
+      </c>
+      <c r="J23" s="48" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="J23" s="48" t="inlineStr">
+      <c r="K23" s="48" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="K23" s="48" t="inlineStr">
+      <c r="L23" s="48" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
@@ -3831,22 +3883,22 @@
           <t>Sales per square foot ($)</t>
         </is>
       </c>
-      <c r="B24" s="52" t="n">
+      <c r="B24" s="53" t="n">
         <v>1426</v>
       </c>
-      <c r="C24" s="52" t="n">
+      <c r="C24" s="53" t="n">
         <v>1360</v>
       </c>
-      <c r="D24" s="52" t="n">
+      <c r="D24" s="53" t="n">
         <v>1380</v>
       </c>
-      <c r="E24" s="52" t="n">
+      <c r="E24" s="53" t="n">
         <v>1400</v>
       </c>
-      <c r="F24" s="52" t="n">
+      <c r="F24" s="53" t="n">
         <v>1420</v>
       </c>
-      <c r="G24" s="52" t="n">
+      <c r="G24" s="53" t="n">
         <v>1440</v>
       </c>
       <c r="H24" s="50" t="inlineStr">
@@ -3854,17 +3906,17 @@
           <t>$/sq ft</t>
         </is>
       </c>
-      <c r="I24" s="17" t="inlineStr">
+      <c r="J24" s="17" t="inlineStr">
         <is>
           <t>FY26 SPSF $1,380 reflects Americas traffic/conversion pressure; recovers toward $1,440 by FY30.</t>
         </is>
       </c>
-      <c r="J24" s="18" t="inlineStr">
+      <c r="K24" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: comparable sales &amp; SPSF</t>
         </is>
       </c>
-      <c r="K24" s="19" t="inlineStr">
+      <c r="L24" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "sales per square foot were $1,426" → FY25 reported $1,426; FY26 model $1,380 on traffic pressure.</t>
         </is>
@@ -3876,22 +3928,22 @@
           <t xml:space="preserve">  Americas — comparable sales growth</t>
         </is>
       </c>
-      <c r="B25" s="56" t="n">
+      <c r="B25" s="57" t="n">
         <v>-0.03</v>
       </c>
-      <c r="C25" s="56" t="n">
+      <c r="C25" s="57" t="n">
         <v>-0.04</v>
       </c>
-      <c r="D25" s="56" t="n">
+      <c r="D25" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="E25" s="56" t="n">
+      <c r="E25" s="57" t="n">
         <v>0.01</v>
       </c>
-      <c r="F25" s="56" t="n">
+      <c r="F25" s="57" t="n">
         <v>0.02</v>
       </c>
-      <c r="G25" s="56" t="n">
+      <c r="G25" s="57" t="n">
         <v>0.02</v>
       </c>
       <c r="H25" s="50" t="inlineStr">
@@ -3899,17 +3951,17 @@
           <t>%</t>
         </is>
       </c>
-      <c r="I25" s="17" t="inlineStr">
+      <c r="J25" s="17" t="inlineStr">
         <is>
           <t>FY25 Americas comp −3% per 10-K (traffic, conversion, AOV down). FY26 −4%: modest step-down before flat FY27 as promo clears.</t>
         </is>
       </c>
-      <c r="J25" s="18" t="inlineStr">
+      <c r="K25" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: Americas comparable sales</t>
         </is>
       </c>
-      <c r="K25" s="19" t="inlineStr">
+      <c r="L25" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Americas comparable sales decreased 3%" → FY25 anchor. FY26 model −4% before stabilization.</t>
         </is>
@@ -3921,22 +3973,22 @@
           <t xml:space="preserve">  China Mainland — comparable sales growth</t>
         </is>
       </c>
-      <c r="B26" s="56" t="n">
+      <c r="B26" s="57" t="n">
         <v>0.2</v>
       </c>
-      <c r="C26" s="56" t="n">
+      <c r="C26" s="57" t="n">
         <v>0.14</v>
       </c>
-      <c r="D26" s="56" t="n">
+      <c r="D26" s="57" t="n">
         <v>0.12</v>
       </c>
-      <c r="E26" s="56" t="n">
+      <c r="E26" s="57" t="n">
         <v>0.1</v>
       </c>
-      <c r="F26" s="56" t="n">
+      <c r="F26" s="57" t="n">
         <v>0.08</v>
       </c>
-      <c r="G26" s="56" t="n">
+      <c r="G26" s="57" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="H26" s="50" t="inlineStr">
@@ -3944,17 +3996,17 @@
           <t>%</t>
         </is>
       </c>
-      <c r="I26" s="17" t="inlineStr">
+      <c r="J26" s="17" t="inlineStr">
         <is>
           <t>FY25 China comp +20% (+19% CCY) per 10-K. FY26 +14%: still fastest region but moderating as the store base scales.</t>
         </is>
       </c>
-      <c r="J26" s="18" t="inlineStr">
+      <c r="K26" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: China Mainland comparable sales</t>
         </is>
       </c>
-      <c r="K26" s="19" t="inlineStr">
+      <c r="L26" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "China Mainland comparable sales increased 20%" → FY25 anchor. FY26 model +14% on a larger base.</t>
         </is>
@@ -3966,22 +4018,22 @@
           <t xml:space="preserve">  Rest of World — comparable sales growth</t>
         </is>
       </c>
-      <c r="B27" s="56" t="n">
+      <c r="B27" s="57" t="n">
         <v>0.09</v>
       </c>
-      <c r="C27" s="56" t="n">
+      <c r="C27" s="57" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="D27" s="56" t="n">
+      <c r="D27" s="57" t="n">
         <v>0.06</v>
       </c>
-      <c r="E27" s="56" t="n">
+      <c r="E27" s="57" t="n">
         <v>0.05</v>
       </c>
-      <c r="F27" s="56" t="n">
+      <c r="F27" s="57" t="n">
         <v>0.04</v>
       </c>
-      <c r="G27" s="56" t="n">
+      <c r="G27" s="57" t="n">
         <v>0.04</v>
       </c>
       <c r="H27" s="50" t="inlineStr">
@@ -3989,29 +4041,29 @@
           <t>%</t>
         </is>
       </c>
-      <c r="I27" s="17" t="inlineStr">
+      <c r="J27" s="17" t="inlineStr">
         <is>
           <t>FY25 RoW comp +9% (+7% CCY) per 10-K. FY26 +7%: hold above CCY, fade to +4% by FY30 as APAC/Europe base matures.</t>
         </is>
       </c>
-      <c r="J27" s="18" t="inlineStr">
+      <c r="K27" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: Rest of World comparable sales</t>
         </is>
       </c>
-      <c r="K27" s="19" t="inlineStr">
+      <c r="L27" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Rest of World comparable sales increased 9%" → FY25 +9% (+7% CCY). FY26 model +7%, fading to +4%.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="56" customHeight="1">
+    <row r="28" ht="28" customHeight="1">
       <c r="A28" s="34" t="inlineStr">
         <is>
           <t>Prior-year store channel revenue ($000)</t>
         </is>
       </c>
-      <c r="B28" s="57" t="n">
+      <c r="B28" s="58" t="n">
         <v>5049744</v>
       </c>
       <c r="C28" s="35">
@@ -4039,19 +4091,23 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I28" s="19" t="inlineStr">
-        <is>
-          <t>Last year's total store-channel revenue — the base you're growing comps off of, not the new boxes.
-Formula: prior column's total store-channel revenue. Base you're applying comps to — not new-store contribution.</t>
-        </is>
-      </c>
-      <c r="J28" s="51" t="inlineStr">
+      <c r="I28" s="51" t="inlineStr">
+        <is>
+          <t>prior column's total store-channel revenue. Base you're applying comps to — not new-store contribution.</t>
+        </is>
+      </c>
+      <c r="J28" s="17" t="inlineStr">
+        <is>
+          <t>Last year's total store-channel revenue — the base you're growing comps off of, not the new boxes.</t>
+        </is>
+      </c>
+      <c r="K28" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: prior store-rev formula</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="56" customHeight="1">
+    <row r="29" ht="28" customHeight="1">
       <c r="A29" s="34" t="inlineStr">
         <is>
           <t>Comparable store revenue ($000)</t>
@@ -4080,19 +4136,23 @@
         <f>F28*0.71*(1+G25)+F28*0.16*(1+G26)+F28*0.13*(1+G27)</f>
         <v/>
       </c>
-      <c r="I29" s="19" t="inlineStr">
-        <is>
-          <t>Existing-store sales only — prior store rev grown by geo comp %. New doors are a separate line, not in here.
-Formula: prior store rev×(71%×(1+Am comp)+16%×(1+China)+13%×(1+RoW)). Existing base only — new stores are on the next row.</t>
-        </is>
-      </c>
-      <c r="J29" s="51" t="inlineStr">
+      <c r="I29" s="51" t="inlineStr">
+        <is>
+          <t>prior store rev×(71%×(1+Am comp)+16%×(1+China)+13%×(1+RoW)). Existing base only — new stores are on the next row.</t>
+        </is>
+      </c>
+      <c r="J29" s="17" t="inlineStr">
+        <is>
+          <t>Existing-store sales only — prior store rev grown by geo comp %. New doors are a separate line, not in here.</t>
+        </is>
+      </c>
+      <c r="K29" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: comp-store formula</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="56" customHeight="1">
+    <row r="30" ht="28" customHeight="1">
       <c r="A30" s="34" t="inlineStr">
         <is>
           <t>Net new store revenue contribution ($000)</t>
@@ -4121,54 +4181,62 @@
         <f>(G7-G8+G11-G12+G15-G16)*G19*G24/1000*0.55</f>
         <v/>
       </c>
-      <c r="I30" s="19" t="inlineStr">
-        <is>
-          <t>Net new doors × sq ft × $/sq ft is plain dollars. /1000 → $000 on this tab. ×0.55 'cause year-one stores don't run full.
-Formula: (open−close each geo)×sq ft×$/sq ft → raw annual $. /1000 flips that to $000 (this whole tab is thousands). ×0.55 = year-one haircut — new boxes don't run at full SPSF yet. FY27 ex: (D7−D8+D11−D12+D15−D16)×D19×D24/1000×0.55.</t>
-        </is>
-      </c>
-      <c r="J30" s="51" t="inlineStr">
+      <c r="I30" s="51" t="inlineStr">
+        <is>
+          <t>(open−close each geo)×sq ft×$/sq ft → raw annual $. /1000 flips that to $000 (this whole tab is thousands). ×0.55 = year-one haircut — new boxes don't run at full SPSF yet. FY27 ex: (D7−D8+D11−D12+D15−D16)×D19×D24/1000×0.55.</t>
+        </is>
+      </c>
+      <c r="J30" s="17" t="inlineStr">
+        <is>
+          <t>Net new doors × sq ft × $/sq ft is plain dollars. /1000 → $000 on this tab. ×0.55 'cause year-one stores don't run full.</t>
+        </is>
+      </c>
+      <c r="K30" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: net-new-store formula</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="56" customHeight="1">
-      <c r="A31" s="53" t="inlineStr">
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="54" t="inlineStr">
         <is>
           <t>Store channel revenue ($000)</t>
         </is>
       </c>
-      <c r="B31" s="55" t="n">
+      <c r="B31" s="56" t="n">
         <v>5049744</v>
       </c>
-      <c r="C31" s="54">
+      <c r="C31" s="55">
         <f>C29+C30</f>
         <v/>
       </c>
-      <c r="D31" s="54">
+      <c r="D31" s="55">
         <f>D29+D30</f>
         <v/>
       </c>
-      <c r="E31" s="54">
+      <c r="E31" s="55">
         <f>E29+E30</f>
         <v/>
       </c>
-      <c r="F31" s="54">
+      <c r="F31" s="55">
         <f>F29+F30</f>
         <v/>
       </c>
-      <c r="G31" s="54">
+      <c r="G31" s="55">
         <f>G29+G30</f>
         <v/>
       </c>
-      <c r="I31" s="19" t="inlineStr">
-        <is>
-          <t>Brick-and-mortar channel = comp store sales plus whatever the net new stores contributed. That's the whole store line.
-Formula: comparable store revenue + net new store revenue. Full brick-and-mortar channel for the year.</t>
-        </is>
-      </c>
-      <c r="J31" s="51" t="inlineStr">
+      <c r="I31" s="51" t="inlineStr">
+        <is>
+          <t>comparable store revenue + net new store revenue. Full brick-and-mortar channel for the year.</t>
+        </is>
+      </c>
+      <c r="J31" s="17" t="inlineStr">
+        <is>
+          <t>Brick-and-mortar channel = comp store sales plus whatever the net new stores contributed. That's the whole store line.</t>
+        </is>
+      </c>
+      <c r="K31" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: store-channel formula</t>
         </is>
@@ -4180,22 +4248,22 @@
           <t xml:space="preserve">  memo: fleet traffic (millions of visits)</t>
         </is>
       </c>
-      <c r="B32" s="58" t="n">
+      <c r="B32" s="59" t="n">
         <v>42.5</v>
       </c>
-      <c r="C32" s="58" t="n">
+      <c r="C32" s="59" t="n">
         <v>40</v>
       </c>
-      <c r="D32" s="58" t="n">
+      <c r="D32" s="59" t="n">
         <v>41</v>
       </c>
-      <c r="E32" s="58" t="n">
+      <c r="E32" s="59" t="n">
         <v>42</v>
       </c>
-      <c r="F32" s="58" t="n">
+      <c r="F32" s="59" t="n">
         <v>43</v>
       </c>
-      <c r="G32" s="58" t="n">
+      <c r="G32" s="59" t="n">
         <v>44</v>
       </c>
       <c r="H32" s="50" t="inlineStr">
@@ -4203,17 +4271,17 @@
           <t>M visits</t>
         </is>
       </c>
-      <c r="I32" s="17" t="inlineStr">
+      <c r="J32" s="17" t="inlineStr">
         <is>
           <t>Fleet traffic memo line — not a separate FCF item. Calibrated to FY25 store productivity commentary.</t>
         </is>
       </c>
-      <c r="J32" s="18" t="inlineStr">
+      <c r="K32" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: store traffic commentary</t>
         </is>
       </c>
-      <c r="K32" s="19" t="inlineStr">
+      <c r="L32" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "store traffic" → lower traffic in Americas; memo line only.</t>
         </is>
@@ -4225,35 +4293,35 @@
           <t xml:space="preserve">  memo: in-store conversion rate</t>
         </is>
       </c>
-      <c r="B33" s="56" t="n">
+      <c r="B33" s="57" t="n">
         <v>0.28</v>
       </c>
-      <c r="C33" s="56" t="n">
+      <c r="C33" s="57" t="n">
         <v>0.27</v>
       </c>
-      <c r="D33" s="56" t="n">
+      <c r="D33" s="57" t="n">
         <v>0.275</v>
       </c>
-      <c r="E33" s="56" t="n">
+      <c r="E33" s="57" t="n">
         <v>0.28</v>
       </c>
-      <c r="F33" s="56" t="n">
+      <c r="F33" s="57" t="n">
         <v>0.285</v>
       </c>
-      <c r="G33" s="56" t="n">
+      <c r="G33" s="57" t="n">
         <v>0.29</v>
       </c>
-      <c r="I33" s="17" t="inlineStr">
+      <c r="J33" s="17" t="inlineStr">
         <is>
           <t>In-store conversion memo — 10-K cites lower conversion in Americas; FY26 27% improving to 29%.</t>
         </is>
       </c>
-      <c r="J33" s="18" t="inlineStr">
+      <c r="K33" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: conversion rate commentary</t>
         </is>
       </c>
-      <c r="K33" s="19" t="inlineStr">
+      <c r="L33" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "conversion rates" → lower in Americas; in-store memo 27%→29%.</t>
         </is>
@@ -4265,35 +4333,35 @@
           <t xml:space="preserve">  memo: in-store average transaction ($)</t>
         </is>
       </c>
-      <c r="B34" s="59" t="n">
+      <c r="B34" s="60" t="n">
         <v>118</v>
       </c>
-      <c r="C34" s="59" t="n">
+      <c r="C34" s="60" t="n">
         <v>115</v>
       </c>
-      <c r="D34" s="59" t="n">
+      <c r="D34" s="60" t="n">
         <v>116</v>
       </c>
-      <c r="E34" s="59" t="n">
+      <c r="E34" s="60" t="n">
         <v>118</v>
       </c>
-      <c r="F34" s="59" t="n">
+      <c r="F34" s="60" t="n">
         <v>120</v>
       </c>
-      <c r="G34" s="59" t="n">
+      <c r="G34" s="60" t="n">
         <v>122</v>
       </c>
-      <c r="I34" s="17" t="inlineStr">
+      <c r="J34" s="17" t="inlineStr">
         <is>
           <t>In-store average transaction $115–$122; supports SPSF and comp-sales bridge on the driver tab.</t>
         </is>
       </c>
-      <c r="J34" s="18" t="inlineStr">
+      <c r="K34" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: average order value commentary</t>
         </is>
       </c>
-      <c r="K34" s="19" t="inlineStr">
+      <c r="L34" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "average order value" → lower AOV in Americas; memo $115–$122.</t>
         </is>
@@ -4347,17 +4415,22 @@
           <t>Units</t>
         </is>
       </c>
-      <c r="I37" s="48" t="inlineStr">
+      <c r="I37" s="47" t="inlineStr">
+        <is>
+          <t>Equation</t>
+        </is>
+      </c>
+      <c r="J37" s="48" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="J37" s="48" t="inlineStr">
+      <c r="K37" s="48" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="K37" s="48" t="inlineStr">
+      <c r="L37" s="48" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
@@ -4369,22 +4442,22 @@
           <t>Unique digital sessions (millions)</t>
         </is>
       </c>
-      <c r="B38" s="52" t="n">
+      <c r="B38" s="53" t="n">
         <v>485</v>
       </c>
-      <c r="C38" s="52" t="n">
+      <c r="C38" s="53" t="n">
         <v>485</v>
       </c>
-      <c r="D38" s="52" t="n">
+      <c r="D38" s="53" t="n">
         <v>505</v>
       </c>
-      <c r="E38" s="52" t="n">
+      <c r="E38" s="53" t="n">
         <v>525</v>
       </c>
-      <c r="F38" s="52" t="n">
+      <c r="F38" s="53" t="n">
         <v>545</v>
       </c>
-      <c r="G38" s="52" t="n">
+      <c r="G38" s="53" t="n">
         <v>560</v>
       </c>
       <c r="H38" s="50" t="inlineStr">
@@ -4392,17 +4465,17 @@
           <t>M</t>
         </is>
       </c>
-      <c r="I38" s="17" t="inlineStr">
+      <c r="J38" s="17" t="inlineStr">
         <is>
           <t>485M FY25 sessions implied from reported e-comm revenue / conv / AOV. FY26 −3% on Americas softness.</t>
         </is>
       </c>
-      <c r="J38" s="18" t="inlineStr">
+      <c r="K38" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: e-commerce revenue</t>
         </is>
       </c>
-      <c r="K38" s="19" t="inlineStr">
+      <c r="L38" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "E-commerce" → 4,918,697 ($000). Sessions implied from revenue / conv / AOV.</t>
         </is>
@@ -4414,35 +4487,35 @@
           <t>Digital conversion rate</t>
         </is>
       </c>
-      <c r="B39" s="56" t="n">
+      <c r="B39" s="57" t="n">
         <v>0.033</v>
       </c>
-      <c r="C39" s="56" t="n">
+      <c r="C39" s="57" t="n">
         <v>0.033</v>
       </c>
-      <c r="D39" s="56" t="n">
+      <c r="D39" s="57" t="n">
         <v>0.034</v>
       </c>
-      <c r="E39" s="56" t="n">
+      <c r="E39" s="57" t="n">
         <v>0.035</v>
       </c>
-      <c r="F39" s="56" t="n">
+      <c r="F39" s="57" t="n">
         <v>0.035</v>
       </c>
-      <c r="G39" s="56" t="n">
+      <c r="G39" s="57" t="n">
         <v>0.036</v>
       </c>
-      <c r="I39" s="17" t="inlineStr">
+      <c r="J39" s="17" t="inlineStr">
         <is>
           <t>3.3% FY26 digital conversion vs 3.5% pressure cited in 10-K Americas; gradual recovery to 3.6%.</t>
         </is>
       </c>
-      <c r="J39" s="18" t="inlineStr">
+      <c r="K39" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: digital / traffic commentary</t>
         </is>
       </c>
-      <c r="K39" s="19" t="inlineStr">
+      <c r="L39" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "lower conversion rates" (Americas MD&amp;A). FY26 model 3.3% digital conversion.</t>
         </is>
@@ -4454,76 +4527,80 @@
           <t>Digital average order value ($)</t>
         </is>
       </c>
-      <c r="B40" s="59" t="n">
+      <c r="B40" s="60" t="n">
         <v>307</v>
       </c>
-      <c r="C40" s="59" t="n">
+      <c r="C40" s="60" t="n">
         <v>305</v>
       </c>
-      <c r="D40" s="59" t="n">
+      <c r="D40" s="60" t="n">
         <v>308</v>
       </c>
-      <c r="E40" s="59" t="n">
+      <c r="E40" s="60" t="n">
         <v>310</v>
       </c>
-      <c r="F40" s="59" t="n">
+      <c r="F40" s="60" t="n">
         <v>312</v>
       </c>
-      <c r="G40" s="59" t="n">
+      <c r="G40" s="60" t="n">
         <v>315</v>
       </c>
-      <c r="I40" s="17" t="inlineStr">
+      <c r="J40" s="17" t="inlineStr">
         <is>
           <t>AOV $305 FY26 on promo intensity; steps to $315 by FY30 as mix normalizes.</t>
         </is>
       </c>
-      <c r="J40" s="18" t="inlineStr">
+      <c r="K40" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: e-commerce revenue</t>
         </is>
       </c>
-      <c r="K40" s="19" t="inlineStr">
+      <c r="L40" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "average order value" (Americas MD&amp;A). FY26 model $305 AOV.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="56" customHeight="1">
-      <c r="A41" s="53" t="inlineStr">
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="54" t="inlineStr">
         <is>
           <t>E-commerce revenue ($000)</t>
         </is>
       </c>
-      <c r="B41" s="55" t="n">
+      <c r="B41" s="56" t="n">
         <v>4918697</v>
       </c>
-      <c r="C41" s="54">
+      <c r="C41" s="55">
         <f>C38*1000000*C39*C40/1000</f>
         <v/>
       </c>
-      <c r="D41" s="54">
+      <c r="D41" s="55">
         <f>D38*1000000*D39*D40/1000</f>
         <v/>
       </c>
-      <c r="E41" s="54">
+      <c r="E41" s="55">
         <f>E38*1000000*E39*E40/1000</f>
         <v/>
       </c>
-      <c r="F41" s="54">
+      <c r="F41" s="55">
         <f>F38*1000000*F39*F40/1000</f>
         <v/>
       </c>
-      <c r="G41" s="54">
+      <c r="G41" s="55">
         <f>G38*1000000*G39*G40/1000</f>
         <v/>
       </c>
-      <c r="I41" s="19" t="inlineStr">
-        <is>
-          <t>Traffic × conversion × AOV is dollars. ×1M 'cause sessions are in millions; /1000 puts it in $000 like everything else.
-Formula: sessions×1,000,000×conversion×AOV/1000 → e-comm $000. ×1M 'cause sessions are millions; /1000 matches tab units.</t>
-        </is>
-      </c>
-      <c r="J41" s="51" t="inlineStr">
+      <c r="I41" s="51" t="inlineStr">
+        <is>
+          <t>sessions×1,000,000×conversion×AOV/1000 → e-comm $000. ×1M 'cause sessions are millions; /1000 matches tab units.</t>
+        </is>
+      </c>
+      <c r="J41" s="17" t="inlineStr">
+        <is>
+          <t>Traffic × conversion × AOV is dollars. ×1M 'cause sessions are in millions; /1000 puts it in $000 like everything else.</t>
+        </is>
+      </c>
+      <c r="K41" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: e-comm formula</t>
         </is>
@@ -4577,29 +4654,34 @@
           <t>Units</t>
         </is>
       </c>
-      <c r="I44" s="48" t="inlineStr">
+      <c r="I44" s="47" t="inlineStr">
+        <is>
+          <t>Equation</t>
+        </is>
+      </c>
+      <c r="J44" s="48" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="J44" s="48" t="inlineStr">
+      <c r="K44" s="48" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="K44" s="48" t="inlineStr">
+      <c r="L44" s="48" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="56" customHeight="1">
+    <row r="45" ht="28" customHeight="1">
       <c r="A45" s="34" t="inlineStr">
         <is>
           <t>Other channels (wholesale / license / outlets) ($000)</t>
         </is>
       </c>
-      <c r="B45" s="57" t="n">
+      <c r="B45" s="58" t="n">
         <v>1134159</v>
       </c>
       <c r="C45" s="35">
@@ -4627,30 +4709,34 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I45" s="19" t="inlineStr">
-        <is>
-          <t>Other channels (wholesale/license/outlets) held at FY25 $1.13B base; low-single-digit growth thereafter.
-Formula: prior other-channel rev × (1 + growth %). Wholesale/license/outlets — grown off last year.</t>
-        </is>
-      </c>
-      <c r="J45" s="18" t="inlineStr">
+      <c r="I45" s="51" t="inlineStr">
+        <is>
+          <t>prior other-channel rev × (1 + growth %). Wholesale/license/outlets — grown off last year.</t>
+        </is>
+      </c>
+      <c r="J45" s="17" t="inlineStr">
+        <is>
+          <t>Other channels (wholesale/license/outlets) held at FY25 $1.13B base; low-single-digit growth thereafter.</t>
+        </is>
+      </c>
+      <c r="K45" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: channel revenue table</t>
         </is>
       </c>
-      <c r="K45" s="19" t="inlineStr">
+      <c r="L45" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Company-operated stores" and "E-commerce" → residual other channels ≈ $1.13B.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="56" customHeight="1">
+    <row r="46" ht="28" customHeight="1">
       <c r="A46" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Americas net revenue ($000)</t>
         </is>
       </c>
-      <c r="B46" s="57" t="n">
+      <c r="B46" s="58" t="n">
         <v>7847044</v>
       </c>
       <c r="C46" s="35">
@@ -4678,30 +4764,34 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I46" s="19" t="inlineStr">
-        <is>
-          <t>Geographic split scales with consolidated growth; FY25 Americas 70.7% of revenue per 10-K segment table.
-Formula: FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
-        </is>
-      </c>
-      <c r="J46" s="18" t="inlineStr">
+      <c r="I46" s="51" t="inlineStr">
+        <is>
+          <t>FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
+        </is>
+      </c>
+      <c r="J46" s="17" t="inlineStr">
+        <is>
+          <t>Geographic split scales with consolidated growth; FY25 Americas 70.7% of revenue per 10-K segment table.</t>
+        </is>
+      </c>
+      <c r="K46" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
-      <c r="K46" s="19" t="inlineStr">
+      <c r="L46" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Americas" segment table → $7,847,044 net revenue (70.7%).</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="56" customHeight="1">
+    <row r="47" ht="28" customHeight="1">
       <c r="A47" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  China Mainland net revenue ($000)</t>
         </is>
       </c>
-      <c r="B47" s="57" t="n">
+      <c r="B47" s="58" t="n">
         <v>1754799</v>
       </c>
       <c r="C47" s="35">
@@ -4729,30 +4819,34 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I47" s="19" t="inlineStr">
-        <is>
-          <t>China 15.8% of FY25 revenue; fastest comp and store growth — expansion market in the driver schedule.
-Formula: FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
-        </is>
-      </c>
-      <c r="J47" s="18" t="inlineStr">
+      <c r="I47" s="51" t="inlineStr">
+        <is>
+          <t>FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
+        </is>
+      </c>
+      <c r="J47" s="17" t="inlineStr">
+        <is>
+          <t>China 15.8% of FY25 revenue; fastest comp and store growth — expansion market in the driver schedule.</t>
+        </is>
+      </c>
+      <c r="K47" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
-      <c r="K47" s="19" t="inlineStr">
+      <c r="L47" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "China Mainland" segment → $1,754,799 net revenue (15.8%).</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="56" customHeight="1">
+    <row r="48" ht="28" customHeight="1">
       <c r="A48" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rest of World net revenue ($000)</t>
         </is>
       </c>
-      <c r="B48" s="57" t="n">
+      <c r="B48" s="58" t="n">
         <v>1500757</v>
       </c>
       <c r="C48" s="35">
@@ -4780,18 +4874,22 @@
           <t>$000</t>
         </is>
       </c>
-      <c r="I48" s="19" t="inlineStr">
-        <is>
-          <t>Rest of World 13.5% of FY25 revenue; mid-single-digit comps and steady openings.
-Formula: FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
-        </is>
-      </c>
-      <c r="J48" s="18" t="inlineStr">
+      <c r="I48" s="51" t="inlineStr">
+        <is>
+          <t>FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
+        </is>
+      </c>
+      <c r="J48" s="17" t="inlineStr">
+        <is>
+          <t>Rest of World 13.5% of FY25 revenue; mid-single-digit comps and steady openings.</t>
+        </is>
+      </c>
+      <c r="K48" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: segmented net revenue</t>
         </is>
       </c>
-      <c r="K48" s="19" t="inlineStr">
+      <c r="L48" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Rest of World" segment → $1,500,757 net revenue (13.5%).</t>
         </is>
@@ -4803,35 +4901,35 @@
           <t>Women's % of revenue</t>
         </is>
       </c>
-      <c r="B49" s="56" t="n">
+      <c r="B49" s="57" t="n">
         <v>0.63</v>
       </c>
-      <c r="C49" s="56" t="n">
+      <c r="C49" s="57" t="n">
         <v>0.62</v>
       </c>
-      <c r="D49" s="56" t="n">
+      <c r="D49" s="57" t="n">
         <v>0.615</v>
       </c>
-      <c r="E49" s="56" t="n">
+      <c r="E49" s="57" t="n">
         <v>0.61</v>
       </c>
-      <c r="F49" s="56" t="n">
+      <c r="F49" s="57" t="n">
         <v>0.605</v>
       </c>
-      <c r="G49" s="56" t="n">
+      <c r="G49" s="57" t="n">
         <v>0.6</v>
       </c>
-      <c r="I49" s="17" t="inlineStr">
+      <c r="J49" s="17" t="inlineStr">
         <is>
           <t>Women's mix fades 62.5%→60% as men's penetrates; FY25 reported 63% women's per 10-K category disclosure.</t>
         </is>
       </c>
-      <c r="J49" s="18" t="inlineStr">
+      <c r="K49" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: product category mix</t>
         </is>
       </c>
-      <c r="K49" s="19" t="inlineStr">
+      <c r="L49" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "women's, men's, and accessories" → 63% / 24% / 13% of net revenue.</t>
         </is>
@@ -4843,35 +4941,35 @@
           <t>Men's % of revenue</t>
         </is>
       </c>
-      <c r="B50" s="56" t="n">
+      <c r="B50" s="57" t="n">
         <v>0.24</v>
       </c>
-      <c r="C50" s="56" t="n">
+      <c r="C50" s="57" t="n">
         <v>0.25</v>
       </c>
-      <c r="D50" s="56" t="n">
+      <c r="D50" s="57" t="n">
         <v>0.255</v>
       </c>
-      <c r="E50" s="56" t="n">
+      <c r="E50" s="57" t="n">
         <v>0.26</v>
       </c>
-      <c r="F50" s="56" t="n">
+      <c r="F50" s="57" t="n">
         <v>0.265</v>
       </c>
-      <c r="G50" s="56" t="n">
+      <c r="G50" s="57" t="n">
         <v>0.27</v>
       </c>
-      <c r="I50" s="17" t="inlineStr">
+      <c r="J50" s="17" t="inlineStr">
         <is>
           <t>Men's mix rises 24.5%→27%; FY25 men's grew 4% vs women's 5% per 10-K category commentary.</t>
         </is>
       </c>
-      <c r="J50" s="18" t="inlineStr">
+      <c r="K50" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: product category mix</t>
         </is>
       </c>
-      <c r="K50" s="19" t="inlineStr">
+      <c r="L50" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "men's" category growth 4% in MD&amp;A; mix rises to 27% by FY30.</t>
         </is>
@@ -4883,35 +4981,35 @@
           <t>Accessories &amp; other % of revenue</t>
         </is>
       </c>
-      <c r="B51" s="56" t="n">
+      <c r="B51" s="57" t="n">
         <v>0.13</v>
       </c>
-      <c r="C51" s="56" t="n">
+      <c r="C51" s="57" t="n">
         <v>0.13</v>
       </c>
-      <c r="D51" s="56" t="n">
+      <c r="D51" s="57" t="n">
         <v>0.13</v>
       </c>
-      <c r="E51" s="56" t="n">
+      <c r="E51" s="57" t="n">
         <v>0.13</v>
       </c>
-      <c r="F51" s="56" t="n">
+      <c r="F51" s="57" t="n">
         <v>0.13</v>
       </c>
-      <c r="G51" s="56" t="n">
+      <c r="G51" s="57" t="n">
         <v>0.13</v>
       </c>
-      <c r="I51" s="17" t="inlineStr">
+      <c r="J51" s="17" t="inlineStr">
         <is>
           <t>Accessories steady at 13% of revenue; FY25 accessories +8% per 10-K category disclosure.</t>
         </is>
       </c>
-      <c r="J51" s="18" t="inlineStr">
+      <c r="K51" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: product category mix</t>
         </is>
       </c>
-      <c r="K51" s="19" t="inlineStr">
+      <c r="L51" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "accessories" +8% category growth; hold 13% mix.</t>
         </is>
@@ -4965,70 +5063,79 @@
           <t>Units</t>
         </is>
       </c>
-      <c r="I54" s="48" t="inlineStr">
+      <c r="I54" s="47" t="inlineStr">
+        <is>
+          <t>Equation</t>
+        </is>
+      </c>
+      <c r="J54" s="48" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="J54" s="48" t="inlineStr">
+      <c r="K54" s="48" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="K54" s="48" t="inlineStr">
+      <c r="L54" s="48" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="56" customHeight="1">
-      <c r="A55" s="60" t="inlineStr">
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="61" t="inlineStr">
         <is>
           <t>Bottom-up total revenue ($000)</t>
         </is>
       </c>
-      <c r="B55" s="61" t="n">
+      <c r="B55" s="62" t="n">
         <v>11102600</v>
       </c>
-      <c r="C55" s="62">
+      <c r="C55" s="63">
         <f>C31+C41+C45</f>
         <v/>
       </c>
-      <c r="D55" s="62">
+      <c r="D55" s="63">
         <f>D31+D41+D45</f>
         <v/>
       </c>
-      <c r="E55" s="62">
+      <c r="E55" s="63">
         <f>E31+E41+E45</f>
         <v/>
       </c>
-      <c r="F55" s="62">
+      <c r="F55" s="63">
         <f>F31+F41+F45</f>
         <v/>
       </c>
-      <c r="G55" s="62">
+      <c r="G55" s="63">
         <f>G31+G41+G45</f>
         <v/>
       </c>
-      <c r="I55" s="19" t="inlineStr">
-        <is>
-          <t>Bottom-up total = store channel + e-comm + other. That's your driver-built revenue before you check Scenarios.
-Formula: store channel + e-commerce + other. Bottom-up top line before you reconcile to Scenarios.</t>
-        </is>
-      </c>
-      <c r="J55" s="51" t="inlineStr">
+      <c r="I55" s="51" t="inlineStr">
+        <is>
+          <t>store channel + e-commerce + other. Bottom-up top line before you reconcile to Scenarios.</t>
+        </is>
+      </c>
+      <c r="J55" s="17" t="inlineStr">
+        <is>
+          <t>Bottom-up total = store channel + e-comm + other. That's your driver-built revenue before you check Scenarios.</t>
+        </is>
+      </c>
+      <c r="K55" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-rev formula</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="56" customHeight="1">
+    <row r="56" ht="28" customHeight="1">
       <c r="A56" s="34" t="inlineStr">
         <is>
           <t>Scenarios base-case revenue ($000)</t>
         </is>
       </c>
-      <c r="B56" s="57" t="n">
+      <c r="B56" s="58" t="n">
         <v>11102600</v>
       </c>
       <c r="C56" s="35">
@@ -5051,19 +5158,23 @@
         <f>Scenarios!G22</f>
         <v/>
       </c>
-      <c r="I56" s="19" t="inlineStr">
-        <is>
-          <t>Pulls the Scenarios base-case revenue path — that's still the number the DCF actually uses, not the driver total.
-Formula: Scenarios! base-case revenue. DCF still runs off this path — not the driver total.</t>
-        </is>
-      </c>
-      <c r="J56" s="51" t="inlineStr">
+      <c r="I56" s="51" t="inlineStr">
+        <is>
+          <t>Scenarios! base-case revenue. DCF still runs off this path — not the driver total.</t>
+        </is>
+      </c>
+      <c r="J56" s="17" t="inlineStr">
+        <is>
+          <t>Pulls the Scenarios base-case revenue path — that's still the number the DCF actually uses, not the driver total.</t>
+        </is>
+      </c>
+      <c r="K56" s="18" t="inlineStr">
         <is>
           <t>Scenarios tab: base revenue</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="56" customHeight="1">
+    <row r="57" ht="28" customHeight="1">
       <c r="A57" s="34" t="inlineStr">
         <is>
           <t>Variance (bottom-up − scenarios) ($000)</t>
@@ -5093,19 +5204,23 @@
         <f>G55-G56</f>
         <v/>
       </c>
-      <c r="I57" s="19" t="inlineStr">
-        <is>
-          <t>Driver-built revenue minus Scenarios revenue. Shows you how far off the bottom-up path is from what you're valuing on.
-Formula: bottom-up total − Scenarios revenue. Positive = drivers above Scenarios; negative = below.</t>
-        </is>
-      </c>
-      <c r="J57" s="51" t="inlineStr">
+      <c r="I57" s="51" t="inlineStr">
+        <is>
+          <t>bottom-up total − Scenarios revenue. Positive = drivers above Scenarios; negative = below.</t>
+        </is>
+      </c>
+      <c r="J57" s="17" t="inlineStr">
+        <is>
+          <t>Driver-built revenue minus Scenarios revenue. Shows you how far off the bottom-up path is from what you're valuing on.</t>
+        </is>
+      </c>
+      <c r="K57" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: variance formula</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="56" customHeight="1">
+    <row r="58" ht="28" customHeight="1">
       <c r="A58" s="34" t="inlineStr">
         <is>
           <t>Variance (%)</t>
@@ -5135,13 +5250,17 @@
         <f>IF(G56=0,"",G57/G56)</f>
         <v/>
       </c>
-      <c r="I58" s="19" t="inlineStr">
-        <is>
-          <t>Variance as a percent of Scenarios revenue. Easy read on whether the driver schedule is close or way out of line.
-Formula: variance ÷ Scenarios revenue. Quick % read on how far the driver build is from the valuation path.</t>
-        </is>
-      </c>
-      <c r="J58" s="51" t="inlineStr">
+      <c r="I58" s="51" t="inlineStr">
+        <is>
+          <t>variance ÷ Scenarios revenue. Quick % read on how far the driver build is from the valuation path.</t>
+        </is>
+      </c>
+      <c r="J58" s="17" t="inlineStr">
+        <is>
+          <t>Variance as a percent of Scenarios revenue. Easy read on whether the driver schedule is close or way out of line.</t>
+        </is>
+      </c>
+      <c r="K58" s="52" t="inlineStr">
         <is>
           <t>Revenue Drivers: variance % formula</t>
         </is>
@@ -5156,40 +5275,41 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId34"/>
+    <hyperlink ref="K56" location="'Scenarios'!G18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5236,69 +5356,69 @@
       <c r="J1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="B2" s="63" t="inlineStr">
+      <c r="B2" s="64" t="inlineStr">
         <is>
           <t>Justification (~20 words)</t>
         </is>
       </c>
-      <c r="C2" s="63" t="inlineStr">
+      <c r="C2" s="64" t="inlineStr">
         <is>
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D2" s="63" t="inlineStr">
+      <c r="D2" s="64" t="inlineStr">
         <is>
           <t>Ctrl+F (prove number)</t>
         </is>
       </c>
-      <c r="E2" s="64" t="inlineStr">
+      <c r="E2" s="65" t="inlineStr">
         <is>
           <t>FY2025A</t>
         </is>
       </c>
-      <c r="F2" s="65" t="inlineStr">
+      <c r="F2" s="66" t="inlineStr">
         <is>
           <t>FY2026E</t>
         </is>
       </c>
-      <c r="G2" s="65" t="inlineStr">
+      <c r="G2" s="66" t="inlineStr">
         <is>
           <t>FY2027E</t>
         </is>
       </c>
-      <c r="H2" s="65" t="inlineStr">
+      <c r="H2" s="66" t="inlineStr">
         <is>
           <t>FY2028E</t>
         </is>
       </c>
-      <c r="I2" s="65" t="inlineStr">
+      <c r="I2" s="66" t="inlineStr">
         <is>
           <t>FY2029E</t>
         </is>
       </c>
-      <c r="J2" s="65" t="inlineStr">
+      <c r="J2" s="66" t="inlineStr">
         <is>
           <t>FY2030E</t>
         </is>
       </c>
-      <c r="K2" s="66" t="inlineStr">
+      <c r="K2" s="67" t="inlineStr">
         <is>
           <t>Δ vs Scenarios</t>
         </is>
       </c>
-      <c r="L2" s="63" t="inlineStr">
+      <c r="L2" s="64" t="inlineStr">
         <is>
           <t>Alt. source</t>
         </is>
       </c>
-      <c r="M2" s="63" t="inlineStr">
+      <c r="M2" s="64" t="inlineStr">
         <is>
           <t>Alt. Ctrl+F</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="67" t="inlineStr">
+      <c r="A3" s="68" t="inlineStr">
         <is>
           <t>Forecast drivers linked to Scenarios tab → Base case (column G)</t>
         </is>
@@ -5308,12 +5428,12 @@
           <t>Ctrl+F "Net revenue" → 11,102,600 or "Depreciation and amortization" → 496,228 on this 10-K HTML file</t>
         </is>
       </c>
-      <c r="E3" s="68" t="inlineStr">
+      <c r="E3" s="69" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="K3" s="69" t="inlineStr">
+      <c r="K3" s="70" t="inlineStr">
         <is>
           <t>(should be 0)</t>
         </is>
@@ -5326,7 +5446,7 @@
 Ctrl+F: 1-page summary: justifications, Ctrl+F anchors, WACC, terminal multiple.</t>
         </is>
       </c>
-      <c r="C4" s="70" t="inlineStr">
+      <c r="C4" s="71" t="inlineStr">
         <is>
           <t>Revenue Drivers tab
 Ctrl+F: Bottom-up store / DTC / category schedule (FY26–30).</t>
@@ -5339,30 +5459,30 @@
           <t>Net revenue</t>
         </is>
       </c>
-      <c r="E5" s="71" t="n">
+      <c r="E5" s="72" t="n">
         <v>11102600</v>
       </c>
-      <c r="F5" s="72">
+      <c r="F5" s="73">
         <f>Scenarios!G18</f>
         <v/>
       </c>
-      <c r="G5" s="72">
+      <c r="G5" s="73">
         <f>Scenarios!G19</f>
         <v/>
       </c>
-      <c r="H5" s="72">
+      <c r="H5" s="73">
         <f>Scenarios!G20</f>
         <v/>
       </c>
-      <c r="I5" s="72">
+      <c r="I5" s="73">
         <f>Scenarios!G21</f>
         <v/>
       </c>
-      <c r="J5" s="72">
+      <c r="J5" s="73">
         <f>Scenarios!G22</f>
         <v/>
       </c>
-      <c r="K5" s="73">
+      <c r="K5" s="74">
         <f>IF(MAX(ABS(F5-Scenarios!$G$18),ABS(G5-Scenarios!$G$19),ABS(H5-Scenarios!$G$20),ABS(I5-Scenarios!$G$21),ABS(J5-Scenarios!$G$22))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5391,23 +5511,23 @@
 Also: Ctrl+F "Revenue Growth Forecast (3Y)" → 2.26%. That is the unique line (do not search "Net revenue"). Model FY27–30 uses 2.3%.</t>
         </is>
       </c>
-      <c r="F6" s="74">
+      <c r="F6" s="75">
         <f>F5/E5-1</f>
         <v/>
       </c>
-      <c r="G6" s="74">
+      <c r="G6" s="75">
         <f>G5/F5-1</f>
         <v/>
       </c>
-      <c r="H6" s="74">
+      <c r="H6" s="75">
         <f>H5/G5-1</f>
         <v/>
       </c>
-      <c r="I6" s="74">
+      <c r="I6" s="75">
         <f>I5/H5-1</f>
         <v/>
       </c>
-      <c r="J6" s="74">
+      <c r="J6" s="75">
         <f>J5/I5-1</f>
         <v/>
       </c>
@@ -5436,27 +5556,27 @@
 Also: Ctrl+F "19.9%" (one hit) → Operating margin decreased 380 basis points to 19.9%. That is FY25 OM. Do not search the words Income from operations (17 hits). Model FY30 15.5% is a partial-recovery assumption.</t>
         </is>
       </c>
-      <c r="F7" s="74">
+      <c r="F7" s="75">
         <f>Scenarios!G23</f>
         <v/>
       </c>
-      <c r="G7" s="74">
+      <c r="G7" s="75">
         <f>Scenarios!G24</f>
         <v/>
       </c>
-      <c r="H7" s="74">
+      <c r="H7" s="75">
         <f>Scenarios!G25</f>
         <v/>
       </c>
-      <c r="I7" s="74">
+      <c r="I7" s="75">
         <f>Scenarios!G26</f>
         <v/>
       </c>
-      <c r="J7" s="74">
+      <c r="J7" s="75">
         <f>Scenarios!G27</f>
         <v/>
       </c>
-      <c r="K7" s="73">
+      <c r="K7" s="74">
         <f>IF(MAX(ABS(F7-Scenarios!$G$23),ABS(G7-Scenarios!$G$24),ABS(H7-Scenarios!$G$25),ABS(I7-Scenarios!$G$26),ABS(J7-Scenarios!$G$27))&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5482,7 +5602,7 @@
           <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
         </is>
       </c>
-      <c r="E8" s="71" t="n">
+      <c r="E8" s="72" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="33">
@@ -5508,7 +5628,7 @@
           <t>EBIT (incl. FY26 refund)</t>
         </is>
       </c>
-      <c r="E9" s="75" t="n">
+      <c r="E9" s="76" t="n">
         <v>2210615</v>
       </c>
       <c r="F9" s="37">
@@ -5531,7 +5651,7 @@
         <f>Scenarios!G32</f>
         <v/>
       </c>
-      <c r="K9" s="76">
+      <c r="K9" s="77">
         <f>IF(MAX(ABS(F9-Scenarios!$G$28),ABS(G9-Scenarios!$G$29),ABS(H9-Scenarios!$G$30),ABS(I9-Scenarios!$G$31),ABS(J9-Scenarios!$G$32))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5542,26 +5662,26 @@
           <t>Reported EBIT margin % (incl. FY26 refund)</t>
         </is>
       </c>
-      <c r="E10" s="77" t="n">
+      <c r="E10" s="78" t="n">
         <v>0.1991078666258354</v>
       </c>
-      <c r="F10" s="74">
+      <c r="F10" s="75">
         <f>F9/F5</f>
         <v/>
       </c>
-      <c r="G10" s="74">
+      <c r="G10" s="75">
         <f>G9/G5</f>
         <v/>
       </c>
-      <c r="H10" s="74">
+      <c r="H10" s="75">
         <f>H9/H5</f>
         <v/>
       </c>
-      <c r="I10" s="74">
+      <c r="I10" s="75">
         <f>I9/I5</f>
         <v/>
       </c>
-      <c r="J10" s="74">
+      <c r="J10" s="75">
         <f>J9/J5</f>
         <v/>
       </c>
@@ -5572,23 +5692,23 @@
           <t>Less: cash taxes on EBIT</t>
         </is>
       </c>
-      <c r="F11" s="72">
+      <c r="F11" s="73">
         <f>-Scenarios!G28*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="G11" s="72">
+      <c r="G11" s="73">
         <f>-Scenarios!G29*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="H11" s="72">
+      <c r="H11" s="73">
         <f>-Scenarios!G30*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="I11" s="72">
+      <c r="I11" s="73">
         <f>-Scenarios!G31*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="J11" s="72">
+      <c r="J11" s="73">
         <f>-Scenarios!G32*Scenarios!$G$11</f>
         <v/>
       </c>
@@ -5619,7 +5739,7 @@
         <f>Scenarios!G37</f>
         <v/>
       </c>
-      <c r="K12" s="76">
+      <c r="K12" s="77">
         <f>IF(MAX(ABS(F12-Scenarios!$G$33),ABS(G12-Scenarios!$G$34),ABS(H12-Scenarios!$G$35),ABS(I12-Scenarios!$G$36),ABS(J12-Scenarios!$G$37))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5672,27 +5792,27 @@
           <t>Plus: depreciation &amp; amortization</t>
         </is>
       </c>
-      <c r="F14" s="72">
+      <c r="F14" s="73">
         <f>Scenarios!G38</f>
         <v/>
       </c>
-      <c r="G14" s="72">
+      <c r="G14" s="73">
         <f>Scenarios!G39</f>
         <v/>
       </c>
-      <c r="H14" s="72">
+      <c r="H14" s="73">
         <f>Scenarios!G40</f>
         <v/>
       </c>
-      <c r="I14" s="72">
+      <c r="I14" s="73">
         <f>Scenarios!G41</f>
         <v/>
       </c>
-      <c r="J14" s="72">
+      <c r="J14" s="73">
         <f>Scenarios!G42</f>
         <v/>
       </c>
-      <c r="K14" s="73">
+      <c r="K14" s="74">
         <f>IF(MAX(ABS(F14-Scenarios!$G$38),ABS(G14-Scenarios!$G$39),ABS(H14-Scenarios!$G$40),ABS(I14-Scenarios!$G$41),ABS(J14-Scenarios!$G$42))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5758,27 +5878,27 @@
           <t>Less: capital expenditures</t>
         </is>
       </c>
-      <c r="F16" s="72">
+      <c r="F16" s="73">
         <f>-Scenarios!G43</f>
         <v/>
       </c>
-      <c r="G16" s="72">
+      <c r="G16" s="73">
         <f>-Scenarios!G44</f>
         <v/>
       </c>
-      <c r="H16" s="72">
+      <c r="H16" s="73">
         <f>-Scenarios!G45</f>
         <v/>
       </c>
-      <c r="I16" s="72">
+      <c r="I16" s="73">
         <f>-Scenarios!G46</f>
         <v/>
       </c>
-      <c r="J16" s="72">
+      <c r="J16" s="73">
         <f>-Scenarios!G47</f>
         <v/>
       </c>
-      <c r="K16" s="73">
+      <c r="K16" s="74">
         <f>IF(MAX(ABS(F16+Scenarios!$G$43),ABS(G16+Scenarios!$G$44),ABS(H16+Scenarios!$G$45),ABS(I16+Scenarios!$G$46),ABS(J16+Scenarios!$G$47))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5888,30 +6008,30 @@
           <t>Ctrl+F "Accounts receivable, net" (one hit on the BS) → 190,657. 190,657 / 11,102,600 = 1.7% of sales. Lives inside the NWC line below.</t>
         </is>
       </c>
-      <c r="E19" s="71" t="n">
+      <c r="E19" s="72" t="n">
         <v>190657</v>
       </c>
-      <c r="F19" s="72">
+      <c r="F19" s="73">
         <f>Scenarios!G48</f>
         <v/>
       </c>
-      <c r="G19" s="72">
+      <c r="G19" s="73">
         <f>Scenarios!G49</f>
         <v/>
       </c>
-      <c r="H19" s="72">
+      <c r="H19" s="73">
         <f>Scenarios!G50</f>
         <v/>
       </c>
-      <c r="I19" s="72">
+      <c r="I19" s="73">
         <f>Scenarios!G51</f>
         <v/>
       </c>
-      <c r="J19" s="72">
+      <c r="J19" s="73">
         <f>Scenarios!G52</f>
         <v/>
       </c>
-      <c r="K19" s="73">
+      <c r="K19" s="74">
         <f>IF(MAX(ABS(F19-Scenarios!$G$48),ABS(G19-Scenarios!$G$49),ABS(H19-Scenarios!$G$50),ABS(I19-Scenarios!$G$51),ABS(J19-Scenarios!$G$52))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5922,27 +6042,27 @@
           <t>(Increase)/decrease in NWC (includes AR)</t>
         </is>
       </c>
-      <c r="F20" s="72">
+      <c r="F20" s="73">
         <f>-Scenarios!G53</f>
         <v/>
       </c>
-      <c r="G20" s="72">
+      <c r="G20" s="73">
         <f>-Scenarios!G54</f>
         <v/>
       </c>
-      <c r="H20" s="72">
+      <c r="H20" s="73">
         <f>-Scenarios!G55</f>
         <v/>
       </c>
-      <c r="I20" s="72">
+      <c r="I20" s="73">
         <f>-Scenarios!G56</f>
         <v/>
       </c>
-      <c r="J20" s="72">
+      <c r="J20" s="73">
         <f>-Scenarios!G57</f>
         <v/>
       </c>
-      <c r="K20" s="73">
+      <c r="K20" s="74">
         <f>IF(MAX(ABS(F20+Scenarios!$G$53),ABS(G20+Scenarios!$G$54),ABS(H20+Scenarios!$G$55),ABS(I20+Scenarios!$G$56),ABS(J20+Scenarios!$G$57))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5960,27 +6080,27 @@
           <t>Unlevered free cash flow</t>
         </is>
       </c>
-      <c r="F22" s="78">
+      <c r="F22" s="79">
         <f>Scenarios!G58</f>
         <v/>
       </c>
-      <c r="G22" s="78">
+      <c r="G22" s="79">
         <f>Scenarios!G59</f>
         <v/>
       </c>
-      <c r="H22" s="78">
+      <c r="H22" s="79">
         <f>Scenarios!G60</f>
         <v/>
       </c>
-      <c r="I22" s="78">
+      <c r="I22" s="79">
         <f>Scenarios!G61</f>
         <v/>
       </c>
-      <c r="J22" s="78">
+      <c r="J22" s="79">
         <f>Scenarios!G62</f>
         <v/>
       </c>
-      <c r="K22" s="76">
+      <c r="K22" s="77">
         <f>IF(MAX(ABS(F22-Scenarios!$G$58),ABS(G22-Scenarios!$G$59),ABS(H22-Scenarios!$G$60),ABS(I22-Scenarios!$G$61),ABS(J22-Scenarios!$G$62))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5991,19 +6111,19 @@
           <t>Discount period (years)</t>
         </is>
       </c>
-      <c r="F23" s="79" t="n">
+      <c r="F23" s="80" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="79" t="n">
+      <c r="G23" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="79" t="n">
+      <c r="H23" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="I23" s="79" t="n">
+      <c r="I23" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="J23" s="79" t="n">
+      <c r="J23" s="80" t="n">
         <v>5</v>
       </c>
     </row>
@@ -6013,23 +6133,23 @@
           <t>Discount factor @ WACC</t>
         </is>
       </c>
-      <c r="F24" s="80">
+      <c r="F24" s="81">
         <f>1/(1+Scenarios!$G$9)^F23</f>
         <v/>
       </c>
-      <c r="G24" s="80">
+      <c r="G24" s="81">
         <f>1/(1+Scenarios!$G$9)^G23</f>
         <v/>
       </c>
-      <c r="H24" s="80">
+      <c r="H24" s="81">
         <f>1/(1+Scenarios!$G$9)^H23</f>
         <v/>
       </c>
-      <c r="I24" s="80">
+      <c r="I24" s="81">
         <f>1/(1+Scenarios!$G$9)^I23</f>
         <v/>
       </c>
-      <c r="J24" s="80">
+      <c r="J24" s="81">
         <f>1/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
@@ -6067,13 +6187,13 @@
           <t>Scenarios linkage summary (column K should all read OK)</t>
         </is>
       </c>
-      <c r="K27" s="81">
+      <c r="K27" s="82">
         <f>IF(COUNTIF(K5:K22,"CHECK")=0,"ALL OK","REVIEW")</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="82" t="inlineStr">
+      <c r="A28" s="83" t="inlineStr">
         <is>
           <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
         </is>
@@ -6087,7 +6207,7 @@
           <t>Sum of PV of explicit FCF (FY26–FY30)</t>
         </is>
       </c>
-      <c r="E29" s="62">
+      <c r="E29" s="63">
         <f>SUM(F25:J25)</f>
         <v/>
       </c>
@@ -6113,7 +6233,7 @@
           <t>Ctrl+F "Q2 2026" → 24,269.613 and "Q2 2025" → 23,770.976. YoY = 2.1%. Model terminal g 2.25%.</t>
         </is>
       </c>
-      <c r="E30" s="74">
+      <c r="E30" s="75">
         <f>Scenarios!$G$10</f>
         <v/>
       </c>
@@ -6135,7 +6255,7 @@
           <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
         </is>
       </c>
-      <c r="E32" s="72">
+      <c r="E32" s="73">
         <f>J22*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
         <v/>
       </c>
@@ -6146,7 +6266,7 @@
           <t xml:space="preserve">  Implied exit EV/EBITDA = Gordon TV / FY30 EBITDA</t>
         </is>
       </c>
-      <c r="E33" s="83">
+      <c r="E33" s="84">
         <f>E32/E31</f>
         <v/>
       </c>
@@ -6157,7 +6277,7 @@
           <t xml:space="preserve">  memo: (UFCF₃₀ / EBITDA₃₀) × (1+g) / (WACC−g)</t>
         </is>
       </c>
-      <c r="E34" s="83">
+      <c r="E34" s="84">
         <f>J22/E31*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
         <v/>
       </c>
@@ -6168,7 +6288,7 @@
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="E35" s="62">
+      <c r="E35" s="63">
         <f>E32/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
@@ -6190,7 +6310,7 @@
           <t>Plus: cash &amp; equivalents (FY2025)</t>
         </is>
       </c>
-      <c r="C37" s="84" t="inlineStr">
+      <c r="C37" s="85" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -6200,7 +6320,7 @@
           <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
         </is>
       </c>
-      <c r="E37" s="71" t="n">
+      <c r="E37" s="72" t="n">
         <v>1807202</v>
       </c>
     </row>
@@ -6210,7 +6330,7 @@
           <t>Less: total debt</t>
         </is>
       </c>
-      <c r="C38" s="84" t="inlineStr">
+      <c r="C38" s="85" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -6220,7 +6340,7 @@
           <t>Ctrl+F "no borrowings were outstanding under this facility" → no funded term debt</t>
         </is>
       </c>
-      <c r="E38" s="71" t="n">
+      <c r="E38" s="72" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6241,7 +6361,7 @@
           <t>Diluted shares outstanding (000)</t>
         </is>
       </c>
-      <c r="C40" s="84" t="inlineStr">
+      <c r="C40" s="85" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -6251,7 +6371,7 @@
           <t>Ctrl+F "Diluted weighted-average number of shares outstanding" → 119,068 (000)</t>
         </is>
       </c>
-      <c r="E40" s="71" t="n">
+      <c r="E40" s="72" t="n">
         <v>111380</v>
       </c>
     </row>
@@ -6261,11 +6381,11 @@
           <t>Implied value per share</t>
         </is>
       </c>
-      <c r="E41" s="85">
+      <c r="E41" s="86">
         <f>E39/E40</f>
         <v/>
       </c>
-      <c r="K41" s="76">
+      <c r="K41" s="77">
         <f>IF(ABS(E41-Scenarios!$G$65)&lt;0.05,"OK","CHECK")</f>
         <v/>
       </c>
@@ -6276,7 +6396,7 @@
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C42" s="84" t="inlineStr">
+      <c r="C42" s="85" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -6286,7 +6406,7 @@
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E42" s="86" t="n">
+      <c r="E42" s="87" t="n">
         <v>100</v>
       </c>
     </row>
@@ -6296,7 +6416,7 @@
           <t>Implied upside / (downside)</t>
         </is>
       </c>
-      <c r="E43" s="87">
+      <c r="E43" s="88">
         <f>E41/E42-1</f>
         <v/>
       </c>
@@ -6307,13 +6427,13 @@
           <t xml:space="preserve">  memo: % of EV from terminal value</t>
         </is>
       </c>
-      <c r="E44" s="74">
+      <c r="E44" s="75">
         <f>E35/E36</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="82" t="inlineStr">
+      <c r="A46" s="83" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
@@ -6349,11 +6469,11 @@
           <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
         </is>
       </c>
-      <c r="E48" s="83">
+      <c r="E48" s="84">
         <f>E33</f>
         <v/>
       </c>
-      <c r="M48" s="84" t="inlineStr">
+      <c r="M48" s="85" t="inlineStr">
         <is>
           <t>Comps: Exit Multiple Build</t>
         </is>
@@ -6365,7 +6485,7 @@
           <t>Terminal value = Terminal EBITDA × exit multiple</t>
         </is>
       </c>
-      <c r="E49" s="72">
+      <c r="E49" s="73">
         <f>E31*E48</f>
         <v/>
       </c>
@@ -6376,7 +6496,7 @@
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="E50" s="72">
+      <c r="E50" s="73">
         <f>E49/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
@@ -6398,13 +6518,13 @@
           <t>Implied value per share (exit method)</t>
         </is>
       </c>
-      <c r="E52" s="88">
+      <c r="E52" s="89">
         <f>(E51+E37+E38)/E40</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="82" t="inlineStr">
+      <c r="A54" s="83" t="inlineStr">
         <is>
           <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
         </is>
@@ -6414,7 +6534,7 @@
       <c r="D54" s="13" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="89" t="inlineStr"/>
+      <c r="A55" s="90" t="inlineStr"/>
       <c r="B55" s="46" t="inlineStr">
         <is>
           <t>Gordon Growth</t>
@@ -6437,15 +6557,15 @@
           <t>Terminal value ($)</t>
         </is>
       </c>
-      <c r="B56" s="62">
+      <c r="B56" s="63">
         <f>E32</f>
         <v/>
       </c>
-      <c r="C56" s="62">
+      <c r="C56" s="63">
         <f>E49</f>
         <v/>
       </c>
-      <c r="D56" s="62">
+      <c r="D56" s="63">
         <f>B56-C56</f>
         <v/>
       </c>
@@ -6456,15 +6576,15 @@
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
       </c>
-      <c r="B57" s="90">
+      <c r="B57" s="91">
         <f>E33</f>
         <v/>
       </c>
-      <c r="C57" s="90">
+      <c r="C57" s="91">
         <f>E48</f>
         <v/>
       </c>
-      <c r="D57" s="90">
+      <c r="D57" s="91">
         <f>B57-C57</f>
         <v/>
       </c>
@@ -6475,9 +6595,9 @@
           <t>Terminal value variance (%)</t>
         </is>
       </c>
-      <c r="B58" s="74" t="inlineStr"/>
-      <c r="C58" s="74" t="inlineStr"/>
-      <c r="D58" s="74">
+      <c r="B58" s="75" t="inlineStr"/>
+      <c r="C58" s="75" t="inlineStr"/>
+      <c r="D58" s="75">
         <f>(B56-C56)/B56</f>
         <v/>
       </c>
@@ -6488,30 +6608,30 @@
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="B59" s="91">
+      <c r="B59" s="92">
         <f>E41</f>
         <v/>
       </c>
-      <c r="C59" s="91">
+      <c r="C59" s="92">
         <f>E52</f>
         <v/>
       </c>
-      <c r="D59" s="91">
+      <c r="D59" s="92">
         <f>B59-C59</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="60" t="inlineStr">
+      <c r="A60" s="61" t="inlineStr">
         <is>
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B60" s="92">
+      <c r="B60" s="93">
         <f>IF(ABS(D57)&lt;=1.5,"PASS","REVIEW")</f>
         <v/>
       </c>
-      <c r="C60" s="93">
+      <c r="C60" s="94">
         <f>TEXT(D57,"0.0")&amp;"x spread vs Gordon-implied exit"</f>
         <v/>
       </c>
@@ -6522,7 +6642,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="82" t="inlineStr">
+      <c r="A63" s="83" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
@@ -6536,7 +6656,7 @@
       <c r="H63" s="13" t="n"/>
     </row>
     <row r="64" ht="28" customHeight="1">
-      <c r="A64" s="94" t="inlineStr">
+      <c r="A64" s="95" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
@@ -6556,32 +6676,32 @@
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
       </c>
-      <c r="F64" s="95" t="n">
+      <c r="F64" s="96" t="n">
         <v>0.015</v>
       </c>
-      <c r="G64" s="95" t="n">
+      <c r="G64" s="96" t="n">
         <v>0.02</v>
       </c>
-      <c r="H64" s="95" t="n">
+      <c r="H64" s="96" t="n">
         <v>0.0225</v>
       </c>
-      <c r="I64" s="95" t="n">
+      <c r="I64" s="96" t="n">
         <v>0.025</v>
       </c>
-      <c r="J64" s="95" t="n">
+      <c r="J64" s="96" t="n">
         <v>0.03</v>
       </c>
-      <c r="L64" s="84" t="inlineStr">
+      <c r="L64" s="85" t="inlineStr">
         <is>
           <t>Scenarios: terminal g</t>
         </is>
       </c>
     </row>
     <row r="65" ht="28" customHeight="1">
-      <c r="A65" s="95" t="n">
+      <c r="A65" s="96" t="n">
         <v>0.095</v>
       </c>
-      <c r="C65" s="84" t="inlineStr">
+      <c r="C65" s="85" t="inlineStr">
         <is>
           <t>Damodaran: Historical Implied ERP</t>
         </is>
@@ -6591,34 +6711,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F65" s="96">
+      <c r="F65" s="97">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="G65" s="96">
+      <c r="G65" s="97">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="H65" s="96">
+      <c r="H65" s="97">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="I65" s="96">
+      <c r="I65" s="97">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="J65" s="96">
+      <c r="J65" s="97">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="L65" s="84" t="inlineStr">
+      <c r="L65" s="85" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="66" ht="28" customHeight="1">
-      <c r="A66" s="95" t="n">
+      <c r="A66" s="96" t="n">
         <v>0.1</v>
       </c>
       <c r="D66" s="19" t="inlineStr">
@@ -6626,34 +6746,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F66" s="96">
+      <c r="F66" s="97">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="G66" s="96">
+      <c r="G66" s="97">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="H66" s="96">
+      <c r="H66" s="97">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="I66" s="96">
+      <c r="I66" s="97">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="J66" s="96">
+      <c r="J66" s="97">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="L66" s="84" t="inlineStr">
+      <c r="L66" s="85" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="67" ht="28" customHeight="1">
-      <c r="A67" s="95" t="n">
+      <c r="A67" s="96" t="n">
         <v>0.105</v>
       </c>
       <c r="D67" s="19" t="inlineStr">
@@ -6661,34 +6781,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F67" s="96">
+      <c r="F67" s="97">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="G67" s="96">
+      <c r="G67" s="97">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="H67" s="97">
+      <c r="H67" s="98">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="I67" s="96">
+      <c r="I67" s="97">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="J67" s="96">
+      <c r="J67" s="97">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="L67" s="84" t="inlineStr">
+      <c r="L67" s="85" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="68" ht="28" customHeight="1">
-      <c r="A68" s="95" t="n">
+      <c r="A68" s="96" t="n">
         <v>0.11</v>
       </c>
       <c r="D68" s="19" t="inlineStr">
@@ -6696,34 +6816,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F68" s="96">
+      <c r="F68" s="97">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="G68" s="96">
+      <c r="G68" s="97">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="H68" s="96">
+      <c r="H68" s="97">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="I68" s="96">
+      <c r="I68" s="97">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="J68" s="96">
+      <c r="J68" s="97">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="L68" s="84" t="inlineStr">
+      <c r="L68" s="85" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="69" ht="28" customHeight="1">
-      <c r="A69" s="95" t="n">
+      <c r="A69" s="96" t="n">
         <v>0.115</v>
       </c>
       <c r="D69" s="19" t="inlineStr">
@@ -6731,27 +6851,27 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F69" s="96">
+      <c r="F69" s="97">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="G69" s="96">
+      <c r="G69" s="97">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="H69" s="96">
+      <c r="H69" s="97">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="I69" s="96">
+      <c r="I69" s="97">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="J69" s="96">
+      <c r="J69" s="97">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E37+E38)/E40</f>
         <v/>
       </c>
-      <c r="L69" s="84" t="inlineStr">
+      <c r="L69" s="85" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
@@ -6773,7 +6893,7 @@
           <t>Scenarios tab → Ctrl+F "WACC" and "Terminal growth" rows (base-case inputs)</t>
         </is>
       </c>
-      <c r="L70" s="84" t="inlineStr">
+      <c r="L70" s="85" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
@@ -6893,7 +7013,7 @@
           <t>FY2025A revenue</t>
         </is>
       </c>
-      <c r="C4" s="84" t="inlineStr">
+      <c r="C4" s="85" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -6903,7 +7023,7 @@
           <t>Ctrl+F "Net revenue" → 11,102,600 ($000) in FY2025 column</t>
         </is>
       </c>
-      <c r="E4" s="71" t="n">
+      <c r="E4" s="72" t="n">
         <v>11102600</v>
       </c>
     </row>
@@ -6913,7 +7033,7 @@
           <t>FY2025A EBITDA (EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="E5" s="72">
+      <c r="E5" s="73">
         <f>2210615+496228</f>
         <v/>
       </c>
@@ -6924,12 +7044,12 @@
           <t>FY2030E terminal EBITDA (DCF EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="C6" s="84" t="inlineStr">
+      <c r="C6" s="85" t="inlineStr">
         <is>
           <t>↳ DCF base case</t>
         </is>
       </c>
-      <c r="E6" s="72">
+      <c r="E6" s="73">
         <f>DCF!E31</f>
         <v/>
       </c>
@@ -6940,7 +7060,7 @@
           <t>FY2026E diluted EPS (guidance midpoint)</t>
         </is>
       </c>
-      <c r="C7" s="84" t="inlineStr">
+      <c r="C7" s="85" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
@@ -6950,7 +7070,7 @@
           <t>Ctrl+F "$9.48 to $9.73" → FY2026 diluted EPS guidance; model midpoint $9.61</t>
         </is>
       </c>
-      <c r="E7" s="86" t="n">
+      <c r="E7" s="87" t="n">
         <v>9.609999999999999</v>
       </c>
     </row>
@@ -6960,7 +7080,7 @@
           <t>Cash &amp; equivalents</t>
         </is>
       </c>
-      <c r="C8" s="84" t="inlineStr">
+      <c r="C8" s="85" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -6970,7 +7090,7 @@
           <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
         </is>
       </c>
-      <c r="E8" s="71" t="n">
+      <c r="E8" s="72" t="n">
         <v>1807202</v>
       </c>
     </row>
@@ -6980,7 +7100,7 @@
           <t>Diluted shares (000)</t>
         </is>
       </c>
-      <c r="C9" s="84" t="inlineStr">
+      <c r="C9" s="85" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -6990,7 +7110,7 @@
           <t>Ctrl+F "Diluted weighted-average number of shares outstanding" → 119,068 (000)</t>
         </is>
       </c>
-      <c r="E9" s="71" t="n">
+      <c r="E9" s="72" t="n">
         <v>111380</v>
       </c>
     </row>
@@ -7000,7 +7120,7 @@
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C10" s="84" t="inlineStr">
+      <c r="C10" s="85" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -7010,28 +7130,28 @@
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E10" s="86" t="n">
+      <c r="E10" s="87" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="93" t="inlineStr">
+      <c r="A11" s="94" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current EV / EBITDA</t>
         </is>
       </c>
-      <c r="E11" s="98">
+      <c r="E11" s="99">
         <f>(E10*E9-E8)/E5</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="93" t="inlineStr">
+      <c r="A12" s="94" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current P / E (FY2026E)</t>
         </is>
       </c>
-      <c r="E12" s="98">
+      <c r="E12" s="99">
         <f>E10/E7</f>
         <v/>
       </c>
@@ -7044,7 +7164,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="93" t="inlineStr">
+      <c r="A15" s="94" t="inlineStr">
         <is>
           <t>Peer / reference EV/EBITDA (forward / illustrative)</t>
         </is>
@@ -7065,37 +7185,37 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="99" t="inlineStr">
+      <c r="A18" s="100" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B18" s="99" t="inlineStr">
+      <c r="B18" s="100" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C18" s="99" t="inlineStr">
+      <c r="C18" s="100" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D18" s="99" t="inlineStr">
+      <c r="D18" s="100" t="inlineStr">
         <is>
           <t>Ctrl+F / proof</t>
         </is>
       </c>
-      <c r="E18" s="100" t="inlineStr">
+      <c r="E18" s="101" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="I18" s="100" t="inlineStr">
+      <c r="I18" s="101" t="inlineStr">
         <is>
           <t>EV ($000)</t>
         </is>
       </c>
-      <c r="J18" s="100" t="inlineStr">
+      <c r="J18" s="101" t="inlineStr">
         <is>
           <t>EBITDA ($000)</t>
         </is>
@@ -7112,7 +7232,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C19" s="51" t="inlineStr">
+      <c r="C19" s="52" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7122,14 +7242,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E19" s="101">
+      <c r="E19" s="102">
         <f>IF(J19&lt;=0,"n.m.",I19/J19)</f>
         <v/>
       </c>
-      <c r="I19" s="102" t="n">
+      <c r="I19" s="103" t="n">
         <v>11890440</v>
       </c>
-      <c r="J19" s="102" t="n">
+      <c r="J19" s="103" t="n">
         <v>2548084</v>
       </c>
     </row>
@@ -7144,7 +7264,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C20" s="51" t="inlineStr">
+      <c r="C20" s="52" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7154,14 +7274,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E20" s="101">
+      <c r="E20" s="102">
         <f>IF(J20&lt;=0,"n.m.",I20/J20)</f>
         <v/>
       </c>
-      <c r="I20" s="102" t="n">
+      <c r="I20" s="103" t="n">
         <v>3208397</v>
       </c>
-      <c r="J20" s="102" t="n">
+      <c r="J20" s="103" t="n">
         <v>-23230</v>
       </c>
     </row>
@@ -7176,7 +7296,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C21" s="51" t="inlineStr">
+      <c r="C21" s="52" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7186,14 +7306,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E21" s="101">
+      <c r="E21" s="102">
         <f>IF(J21&lt;=0,"n.m.",I21/J21)</f>
         <v/>
       </c>
-      <c r="I21" s="102" t="n">
+      <c r="I21" s="103" t="n">
         <v>35661944</v>
       </c>
-      <c r="J21" s="102" t="n">
+      <c r="J21" s="103" t="n">
         <v>3857684</v>
       </c>
     </row>
@@ -7208,7 +7328,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C22" s="51" t="inlineStr">
+      <c r="C22" s="52" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7218,14 +7338,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E22" s="101">
+      <c r="E22" s="102">
         <f>IF(J22&lt;=0,"n.m.",I22/J22)</f>
         <v/>
       </c>
-      <c r="I22" s="102" t="n">
+      <c r="I22" s="103" t="n">
         <v>58972350</v>
       </c>
-      <c r="J22" s="102" t="n">
+      <c r="J22" s="103" t="n">
         <v>4647000</v>
       </c>
     </row>
@@ -7240,7 +7360,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C23" s="51" t="inlineStr">
+      <c r="C23" s="52" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7250,14 +7370,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E23" s="101">
+      <c r="E23" s="102">
         <f>IF(J23&lt;=0,"n.m.",I23/J23)</f>
         <v/>
       </c>
-      <c r="I23" s="102" t="n">
+      <c r="I23" s="103" t="n">
         <v>10555510</v>
       </c>
-      <c r="J23" s="102" t="n">
+      <c r="J23" s="103" t="n">
         <v>1329439</v>
       </c>
     </row>
@@ -7272,7 +7392,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C24" s="51" t="inlineStr">
+      <c r="C24" s="52" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7282,14 +7402,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E24" s="101">
+      <c r="E24" s="102">
         <f>IF(J24&lt;=0,"n.m.",I24/J24)</f>
         <v/>
       </c>
-      <c r="I24" s="102" t="n">
+      <c r="I24" s="103" t="n">
         <v>27284350</v>
       </c>
-      <c r="J24" s="102" t="n">
+      <c r="J24" s="103" t="n">
         <v>1768400</v>
       </c>
     </row>
@@ -7304,7 +7424,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C25" s="51" t="inlineStr">
+      <c r="C25" s="52" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7314,14 +7434,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E25" s="101">
+      <c r="E25" s="102">
         <f>IF(J25&lt;=0,"n.m.",I25/J25)</f>
         <v/>
       </c>
-      <c r="I25" s="102" t="n">
+      <c r="I25" s="103" t="n">
         <v>7153911</v>
       </c>
-      <c r="J25" s="102" t="n">
+      <c r="J25" s="103" t="n">
         <v>922278</v>
       </c>
     </row>
@@ -7336,7 +7456,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C26" s="51" t="inlineStr">
+      <c r="C26" s="52" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7346,14 +7466,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E26" s="101">
+      <c r="E26" s="102">
         <f>IF(J26&lt;=0,"n.m.",I26/J26)</f>
         <v/>
       </c>
-      <c r="I26" s="102" t="n">
+      <c r="I26" s="103" t="n">
         <v>616045</v>
       </c>
-      <c r="J26" s="102" t="n">
+      <c r="J26" s="103" t="n">
         <v>62010</v>
       </c>
     </row>
@@ -7368,7 +7488,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C27" s="51" t="inlineStr">
+      <c r="C27" s="52" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7378,14 +7498,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E27" s="101">
+      <c r="E27" s="102">
         <f>IF(J27&lt;=0,"n.m.",I27/J27)</f>
         <v/>
       </c>
-      <c r="I27" s="102" t="n">
+      <c r="I27" s="103" t="n">
         <v>9422753</v>
       </c>
-      <c r="J27" s="102" t="n">
+      <c r="J27" s="103" t="n">
         <v>976700</v>
       </c>
     </row>
@@ -7400,7 +7520,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C28" s="51" t="inlineStr">
+      <c r="C28" s="52" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7410,14 +7530,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E28" s="101">
+      <c r="E28" s="102">
         <f>IF(J28&lt;=0,"n.m.",I28/J28)</f>
         <v/>
       </c>
-      <c r="I28" s="102" t="n">
+      <c r="I28" s="103" t="n">
         <v>1598873</v>
       </c>
-      <c r="J28" s="102" t="n">
+      <c r="J28" s="103" t="n">
         <v>235723</v>
       </c>
     </row>
@@ -7432,7 +7552,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C29" s="51" t="inlineStr">
+      <c r="C29" s="52" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7442,14 +7562,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E29" s="101">
+      <c r="E29" s="102">
         <f>IF(J29&lt;=0,"n.m.",I29/J29)</f>
         <v/>
       </c>
-      <c r="I29" s="102" t="n">
+      <c r="I29" s="103" t="n">
         <v>5236269</v>
       </c>
-      <c r="J29" s="102" t="n">
+      <c r="J29" s="103" t="n">
         <v>407521</v>
       </c>
     </row>
@@ -7491,7 +7611,7 @@
 Also: Ctrl+F "roughly $10 billion" and "No deal was announced". Still an ask.</t>
         </is>
       </c>
-      <c r="E33" s="103" t="n">
+      <c r="E33" s="104" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7516,12 +7636,12 @@
           <t>Ctrl+F "nearly $2 billion". Forbes estimate for Color Image parent (Alo + Bella+Canvas), not Alo-only EBITDA.</t>
         </is>
       </c>
-      <c r="E34" s="103" t="n">
+      <c r="E34" s="104" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
-      <c r="A35" s="60" t="inlineStr">
+      <c r="A35" s="61" t="inlineStr">
         <is>
           <t>Alo implied EV/Sales (ask / parent sales)</t>
         </is>
@@ -7531,7 +7651,7 @@
           <t>5.0x = 10 / 2. Implied EV/Sales on an unclosed ask and parent sales. Not EV/EBITDA. Not the TV.</t>
         </is>
       </c>
-      <c r="C35" s="84" t="inlineStr">
+      <c r="C35" s="85" t="inlineStr">
         <is>
           <t>Comps: Alo ask / parent sales</t>
         </is>
@@ -7541,7 +7661,7 @@
           <t>No Ctrl+F for EV/EBITDA — Firecrawl found none on Reuters or Forbes. This cell is E33 / E34 (ask ÷ parent sales). Not the TV.</t>
         </is>
       </c>
-      <c r="E35" s="104">
+      <c r="E35" s="105">
         <f>E33/E34</f>
         <v/>
       </c>
@@ -7567,7 +7687,7 @@
           <t>No Ctrl+F. Reuters, Forbes, and PitchBook do not print Alo EV/EBITDA.</t>
         </is>
       </c>
-      <c r="E36" s="105" t="inlineStr">
+      <c r="E36" s="106" t="inlineStr">
         <is>
           <t>n.a.</t>
         </is>
@@ -7601,7 +7721,7 @@
           <t>Each E cell is I/J from the PitchBook extract. Do not use as FY30 exit.</t>
         </is>
       </c>
-      <c r="E39" s="101">
+      <c r="E39" s="102">
         <f>AVERAGE(E19,E22,E21,E23,E25,E27,E29)</f>
         <v/>
       </c>
@@ -7627,13 +7747,13 @@
           <t>UAA omitted because TTM EBITDA is negative. Not the selected FY30 exit.</t>
         </is>
       </c>
-      <c r="E40" s="101">
+      <c r="E40" s="102">
         <f>AVERAGE(E19,E21,E22,E23,E24,E25,E26,E27,E28,E29)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="93" t="inlineStr">
+      <c r="A41" s="94" t="inlineStr">
         <is>
           <t>We do not average peers for terminal value, and we do not use Alo 5.0x EV/Sales as EV/EBITDA.</t>
         </is>
@@ -7652,18 +7772,18 @@
           <t>Gordon Growth implied exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="E44" s="83">
+      <c r="E44" s="84">
         <f>DCF!E33</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="60" t="inlineStr">
+      <c r="A45" s="61" t="inlineStr">
         <is>
           <t>Selected exit multiple (base case)</t>
         </is>
       </c>
-      <c r="E45" s="90">
+      <c r="E45" s="91">
         <f>DCF!E48</f>
         <v/>
       </c>
@@ -7674,13 +7794,13 @@
           <t>Spread (selected − Gordon implied)</t>
         </is>
       </c>
-      <c r="E46" s="83">
+      <c r="E46" s="84">
         <f>E45-E44</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="60" t="inlineStr">
+      <c r="A47" s="61" t="inlineStr">
         <is>
           <t>Rationale for selected exit (Gordon identity, not a peer pick)</t>
         </is>
@@ -7736,42 +7856,42 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="99" t="inlineStr">
+      <c r="A56" s="100" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B56" s="99" t="inlineStr">
+      <c r="B56" s="100" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C56" s="99" t="inlineStr">
+      <c r="C56" s="100" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D56" s="99" t="inlineStr">
+      <c r="D56" s="100" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
-      <c r="E56" s="100" t="inlineStr">
+      <c r="E56" s="101" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="F56" s="100" t="inlineStr">
+      <c r="F56" s="101" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="G56" s="100" t="inlineStr">
+      <c r="G56" s="101" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="H56" s="100" t="inlineStr">
+      <c r="H56" s="101" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
@@ -7789,7 +7909,7 @@
 Hi: 8.0x = Deckers print as the high end of the range only. Selected exit is Gordon implied, not this cap.</t>
         </is>
       </c>
-      <c r="C57" s="70" t="inlineStr">
+      <c r="C57" s="71" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU EV/EBITDA
 Hi: StockAnalysis: DECK EV/EBITDA</t>
@@ -7801,23 +7921,23 @@
 Hi: Ctrl+F "EV / EBITDA" → 7.95. Football-field cap 8.0x (Deckers). Not the selected exit.</t>
         </is>
       </c>
-      <c r="E57" s="106" t="n">
+      <c r="E57" s="107" t="n">
         <v>5</v>
       </c>
-      <c r="F57" s="106" t="n">
+      <c r="F57" s="107" t="n">
         <v>8</v>
       </c>
-      <c r="G57" s="107">
+      <c r="G57" s="108">
         <f>(E6*E57+E8)/E9</f>
         <v/>
       </c>
-      <c r="H57" s="107">
+      <c r="H57" s="108">
         <f>(E6*F57+E8)/E9</f>
         <v/>
       </c>
     </row>
     <row r="58" ht="28" customHeight="1">
-      <c r="A58" s="60" t="inlineStr">
+      <c r="A58" s="61" t="inlineStr">
         <is>
           <t>DCF exit method (Gordon-implied on FY2030E EBITDA)</t>
         </is>
@@ -7837,11 +7957,11 @@
           <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
         </is>
       </c>
-      <c r="E58" s="104">
+      <c r="E58" s="105">
         <f>DCF!E48</f>
         <v/>
       </c>
-      <c r="G58" s="108">
+      <c r="G58" s="109">
         <f>(E6*E58+E8)/E9</f>
         <v/>
       </c>
@@ -7858,7 +7978,7 @@
 Hi: 18x P/E high on FY2026E EPS; modest recovery case still below historical premium LULU multiples.</t>
         </is>
       </c>
-      <c r="C59" s="70" t="inlineStr">
+      <c r="C59" s="71" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU Forward P/E
 Hi: StockAnalysis: NKE Forward P/E</t>
@@ -7870,17 +7990,17 @@
 Hi: Ctrl+F "Forward PE" → NKE peer benchmark; high-case assumption 18.0x</t>
         </is>
       </c>
-      <c r="E59" s="106" t="n">
+      <c r="E59" s="107" t="n">
         <v>10</v>
       </c>
-      <c r="F59" s="106" t="n">
+      <c r="F59" s="107" t="n">
         <v>18</v>
       </c>
-      <c r="G59" s="107">
+      <c r="G59" s="108">
         <f>E7*E59</f>
         <v/>
       </c>
-      <c r="H59" s="107">
+      <c r="H59" s="108">
         <f>E7*F59</f>
         <v/>
       </c>
@@ -7891,32 +8011,32 @@
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="E60" s="109" t="inlineStr">
+      <c r="E60" s="110" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F60" s="109" t="inlineStr">
+      <c r="F60" s="110" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G60" s="107">
+      <c r="G60" s="108">
         <f>Scenarios!F65</f>
         <v/>
       </c>
-      <c r="H60" s="107">
+      <c r="H60" s="108">
         <f>Scenarios!H65</f>
         <v/>
       </c>
     </row>
     <row r="62" ht="28" customHeight="1">
-      <c r="A62" s="110" t="inlineStr">
+      <c r="A62" s="111" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C62" s="84" t="inlineStr">
+      <c r="C62" s="85" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -7926,7 +8046,7 @@
           <t>Ctrl+F "LULU" → Last Sale or Previous Close on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E62" s="111" t="n">
+      <c r="E62" s="112" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Plug geo revenue equation into Equation column with cell refs
Americas/China/RoW rows now show FY26 = FY25 × (total growth) plus
a FY26E example with actual row references (e.g. B46 × (C31+C41+C45)/...).

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -4730,7 +4730,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="28" customHeight="1">
+    <row r="46" ht="70" customHeight="1">
       <c r="A46" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Americas net revenue ($000)</t>
@@ -4766,7 +4766,9 @@
       </c>
       <c r="I46" s="51" t="inlineStr">
         <is>
-          <t>FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
+          <t>FY26 geo rev = FY25 geo rev × (FY26 total rev ÷ FY25 total rev).
+Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth.
+FY26E plugged: B46 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
         </is>
       </c>
       <c r="J46" s="17" t="inlineStr">
@@ -4785,7 +4787,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="28" customHeight="1">
+    <row r="47" ht="70" customHeight="1">
       <c r="A47" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  China Mainland net revenue ($000)</t>
@@ -4821,7 +4823,9 @@
       </c>
       <c r="I47" s="51" t="inlineStr">
         <is>
-          <t>FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
+          <t>FY26 geo rev = FY25 geo rev × (FY26 total rev ÷ FY25 total rev).
+Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth.
+FY26E plugged: B47 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
         </is>
       </c>
       <c r="J47" s="17" t="inlineStr">
@@ -4840,7 +4844,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="28" customHeight="1">
+    <row r="48" ht="70" customHeight="1">
       <c r="A48" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Rest of World net revenue ($000)</t>
@@ -4876,7 +4880,9 @@
       </c>
       <c r="I48" s="51" t="inlineStr">
         <is>
-          <t>FY25 geo rev × (this year's total rev ÷ FY25 total rev). Keeps mix, moves with consolidated growth.</t>
+          <t>FY26 geo rev = FY25 geo rev × (FY26 total rev ÷ FY25 total rev).
+Total rev = store channel + e-comm + other. Keeps FY25 geo mix; scales with consolidated growth.
+FY26E plugged: B48 × (C31+C41+C45) ÷ (B31+B41+B45)</t>
         </is>
       </c>
       <c r="J48" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Split WACC market equity into separate price and shares link rows
Give share price and shares outstanding their own Source (click) hyperlinks
on the WACC tab instead of stacking plain text under one NASDAQ link.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -23,8 +23,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="#,##0;(#,##0)"/>
-    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="#,##0;(#,##0)"/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="0.0x"/>
@@ -399,7 +399,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -443,58 +443,58 @@
     <xf numFmtId="2" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -503,10 +503,10 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="26" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="22" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="22" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -529,7 +529,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -538,37 +538,37 @@
     <xf numFmtId="0" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -595,13 +595,16 @@
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="35" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="35" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -610,7 +613,7 @@
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -629,23 +632,23 @@
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="45" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="45" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="46" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="46" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="46" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -660,27 +663,27 @@
     <xf numFmtId="164" fontId="48" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="49" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="166" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="49" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="167" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -693,10 +696,10 @@
     <xf numFmtId="169" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -705,7 +708,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="51" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="51" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1229,7 +1232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1404,127 +1407,174 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>Market value of equity (price × shares outstanding)</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>Market equity = $100 share price × 111,380k shares outstanding (FY25 10-K). Capital-structure weighting numerator.
-Also: 111,380k class A shares outstanding at FY25 year-end (10-K cover). Diluted WA 119,068 is for EPS, not market cap.</t>
-        </is>
-      </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>NASDAQ LULU last sale (current price)
-Also: LULU FY2025 10-K: shares outstanding</t>
+          <t>Share price ($)</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>$100 share price ≈ NASDAQ Last Sale after Q2 FY2026 guide cut; rounded from $100.61 close.</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>NASDAQ LULU last sale (current price)</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "closed at $100.61" → Last Sale $100.61 (NASDAQ). Model uses $100 rounded.
-Also: Ctrl+F "111,380 and 116,166 issued and outstanding" → 111,380k class A shares (FY25 10-K cover).</t>
-        </is>
-      </c>
-      <c r="E10" s="24">
-        <f>100.0*111380</f>
-        <v/>
+          <t>Ctrl+F "closed at $100.61" → Last Sale $100.61 (NASDAQ). Model uses $100 rounded.</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>Operating lease liabilities (ASC 842 debt equiv.)</t>
+          <t>Shares outstanding (000)</t>
         </is>
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>ASC 842 operating lease liabilities = current + non-current ($1,798,441k FY25). Treated as debt equivalent in WACC and EV bridge.</t>
+          <t>111,380k class A shares outstanding at FY25 year-end (10-K cover). Diluted WA 119,068 is for EPS, not market cap.</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K: operating lease liabilities</t>
+          <t>LULU FY2025 10-K: shares outstanding</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Current lease liabilities" → 298,724 | "Non-current lease liabilities" → 1,499,717 | sum = 1,798,441 ($000)</t>
-        </is>
-      </c>
-      <c r="E11" s="25" t="n">
-        <v>1798441</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  memo: current $298,724k + non-current $1,499,717k = $1,798,441k (FY25 10-K)</t>
-        </is>
+          <t>Ctrl+F "111,380 and 116,166 issued and outstanding" → 111,380k class A shares (FY25 10-K cover).</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="n">
+        <v>111380</v>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>Market value of equity</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Market equity = share price × shares outstanding. Capital-structure weighting numerator for relevered β and WACC weights.</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>WACC tab: price × shares</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Share price row × shares outstanding row on this tab.</t>
+        </is>
+      </c>
+      <c r="E12" s="27">
+        <f>E10*E11</f>
+        <v/>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="16" t="inlineStr">
         <is>
+          <t>Operating lease liabilities (ASC 842 debt equiv.)</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>ASC 842 operating lease liabilities = current + non-current ($1,798,441k FY25). Treated as debt equivalent in WACC and EV bridge.</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: operating lease liabilities</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Current lease liabilities" → 298,724 | "Non-current lease liabilities" → 1,499,717 | sum = 1,798,441 ($000)</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="n">
+        <v>1798441</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  memo: current $298,724k + non-current $1,499,717k = $1,798,441k (FY25 10-K)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
           <t>Funded debt (term loans / bonds)</t>
         </is>
       </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Funded term debt $0 — 10-K: no borrowings outstanding on the revolver. Leases are the only debt equivalent here.</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K (no funded debt)</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "no borrowings were outstanding under this facility" → funded debt $0</t>
         </is>
       </c>
-      <c r="E13" s="25" t="n">
+      <c r="E15" s="24" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="25" t="inlineStr">
         <is>
           <t>Total debt equivalents</t>
         </is>
       </c>
-      <c r="E14" s="28">
-        <f>E11+E13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="E16" s="27">
+        <f>E13+E15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Cost of equity (CAPM) — relevered</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="27" t="inlineStr">
+    <row r="19" ht="150" customHeight="1">
+      <c r="A19" s="25" t="inlineStr">
         <is>
           <t>Beta used (relevered for lease debt)</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Relevered β = βu × (1 + (1−T) × lease debt / market equity). No funded term loans — leases are the debt equivalent.</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>Damodaran: relevered β for lease debt</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>Relever Damodaran unlevered retail β for ASC 842 lease debt.
 Unlevered β (Damodaran Jan 2026)
@@ -1538,139 +1588,139 @@
   Ctrl+F "Beta (5Y)"  →  0.86</t>
         </is>
       </c>
-      <c r="E17" s="29">
-        <f>E6*(1+(1-E7)*E11/E10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="26" t="inlineStr">
+      <c r="E19" s="29">
+        <f>E6*(1+(1-E7)*E13/E12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: relever unlevered retail β for ASC 842 lease debt. βL = βu × (1 + (1−T) × D/E). No funded term loans.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="27" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="25" t="inlineStr">
         <is>
           <t>Cost of equity = rf + β × ERP</t>
         </is>
       </c>
-      <c r="E19" s="30">
-        <f>E3+E17*E4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="E21" s="30">
+        <f>E3+E19*E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>Cost of debt (lease-equivalent)</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="16" t="inlineStr">
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>Pre-tax cost of debt (lease-equivalent)</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>5.0% pre-tax lease-equivalent borrowing cost; cheaper than equity. No funded revolver borrowings per FY25 10-K.</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C24" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: lease liabilities &amp; no funded debt</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Current lease liabilities" + "Non-current lease liabilities" → debt equiv. 5.0% illustrative lease borrowing cost.</t>
         </is>
       </c>
-      <c r="E22" s="20" t="n">
+      <c r="E24" s="20" t="n">
         <v>0.05</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="E23" s="31">
-        <f>E22*(1-E7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="14" t="inlineStr">
+      <c r="E25" s="31">
+        <f>E24*(1-E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>WACC weights</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="16" t="inlineStr">
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>Equity weight</t>
         </is>
       </c>
-      <c r="B26" s="17" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>Equity weight = market cap ÷ (market cap + lease debt). ~86% at $100 and FY25 lease balance.</t>
         </is>
       </c>
-      <c r="C26" s="32" t="inlineStr">
+      <c r="C28" s="26" t="inlineStr">
         <is>
           <t>WACC tab: capital structure</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
+      <c r="D28" s="19" t="inlineStr">
         <is>
           <t>Equity weight = market cap ÷ (market cap + lease debt). Live formula on this tab.</t>
         </is>
       </c>
-      <c r="E26" s="33">
-        <f>E10/(E10+E14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="E28" s="32">
+        <f>E12/(E12+E16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>Debt weight (leases + funded)</t>
         </is>
       </c>
-      <c r="B27" s="17" t="inlineStr">
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>Debt weight = lease liabilities ÷ (market cap + lease debt). ~14% — ASC 842 leases, not bank debt.</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C29" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: operating lease liabilities</t>
         </is>
       </c>
-      <c r="D27" s="19" t="inlineStr">
+      <c r="D29" s="19" t="inlineStr">
         <is>
           <t>Debt weight = lease liabilities ÷ (market cap + lease debt). ~14% at FY25 balances.</t>
         </is>
       </c>
-      <c r="E27" s="33">
-        <f>E14/(E10+E14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="27" t="inlineStr">
+      <c r="E29" s="32">
+        <f>E16/(E12+E16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="25" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="E28" s="34">
-        <f>E26*E19+E27*E23</f>
+      <c r="E30" s="33">
+        <f>E28*E21+E29*E25</f>
         <v/>
       </c>
     </row>
@@ -1684,9 +1734,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1725,17 +1776,17 @@
       <c r="H1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="F2" s="35" t="inlineStr">
+      <c r="F2" s="34" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="G2" s="36" t="inlineStr">
+      <c r="G2" s="35" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="H2" s="37" t="inlineStr">
+      <c r="H2" s="36" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
@@ -1877,13 +1928,13 @@
           <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
         </is>
       </c>
-      <c r="F7" s="38" t="n">
+      <c r="F7" s="37" t="n">
         <v>134500</v>
       </c>
-      <c r="G7" s="38" t="n">
+      <c r="G7" s="37" t="n">
         <v>134500</v>
       </c>
-      <c r="H7" s="38" t="n">
+      <c r="H7" s="37" t="n">
         <v>134500</v>
       </c>
     </row>
@@ -1942,8 +1993,8 @@
       <c r="F9" s="20" t="n">
         <v>0.11</v>
       </c>
-      <c r="G9" s="33">
-        <f>WACC!E28</f>
+      <c r="G9" s="32">
+        <f>WACC!E30</f>
         <v/>
       </c>
       <c r="H9" s="20" t="n">
@@ -2055,7 +2106,7 @@
 Also: FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
+      <c r="C13" s="38" t="inlineStr">
         <is>
           <t>LULU 10-K: 2026 capex guide $725–745M
 Also: Q2 FY2026 outlook: $10.350B–$10.500B sales</t>
@@ -3012,20 +3063,20 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="27" t="inlineStr">
+      <c r="A64" s="25" t="inlineStr">
         <is>
           <t>Enterprise value (DCF)</t>
         </is>
       </c>
-      <c r="F64" s="28">
+      <c r="F64" s="27">
         <f>NPV(F9,F58,F59,F60,F61,F62)+(F62*(1+F10)/(F9-F10))/(1+F9)^5</f>
         <v/>
       </c>
-      <c r="G64" s="28">
+      <c r="G64" s="27">
         <f>NPV(G9,G58,G59,G60,G61,G62)+(G62*(1+G10)/(G9-G10))/(1+G9)^5</f>
         <v/>
       </c>
-      <c r="H64" s="28">
+      <c r="H64" s="27">
         <f>NPV(H9,H58,H59,H60,H61,H62)+(H62*(1+H10)/(H9-H10))/(1+H9)^5</f>
         <v/>
       </c>
@@ -3050,7 +3101,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="27" t="inlineStr">
+      <c r="A66" s="25" t="inlineStr">
         <is>
           <t>Upside / (downside) vs current</t>
         </is>
@@ -3069,7 +3120,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="26" t="inlineStr">
+      <c r="A68" s="28" t="inlineStr">
         <is>
           <t>Current price $100.00; cash $1,807,202 k; lease debt $1,798,441 k; funded debt $0; net cash $8,761 k.</t>
         </is>
@@ -3082,7 +3133,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
-    <hyperlink ref="C9" location="'WACC'!E28"/>
+    <hyperlink ref="C9" location="'WACC'!E30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
@@ -3136,7 +3187,7 @@
       <c r="L1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>FY2025A = Firecrawl-ingested 10-K anchors (blue). FY26–30 = red operational assumptions. Consolidated revenue cross-checks to Scenarios base case.</t>
         </is>
@@ -3277,7 +3328,7 @@
           <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
         </is>
       </c>
-      <c r="K6" s="32" t="inlineStr">
+      <c r="K6" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
@@ -3411,7 +3462,7 @@
           <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
         </is>
       </c>
-      <c r="K9" s="32" t="inlineStr">
+      <c r="K9" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
@@ -3461,7 +3512,7 @@
           <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
         </is>
       </c>
-      <c r="K10" s="32" t="inlineStr">
+      <c r="K10" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
@@ -3595,7 +3646,7 @@
           <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
         </is>
       </c>
-      <c r="K13" s="32" t="inlineStr">
+      <c r="K13" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
@@ -3645,7 +3696,7 @@
           <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
         </is>
       </c>
-      <c r="K14" s="32" t="inlineStr">
+      <c r="K14" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
@@ -3779,7 +3830,7 @@
           <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
         </is>
       </c>
-      <c r="K17" s="32" t="inlineStr">
+      <c r="K17" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
@@ -3824,7 +3875,7 @@
           <t>Add up Americas + China + RoW ending stores. Should tie to the 10-K total company-operated count.</t>
         </is>
       </c>
-      <c r="K18" s="32" t="inlineStr">
+      <c r="K18" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-stores formula</t>
         </is>
@@ -3920,7 +3971,7 @@
           <t>Ending stores times avg sq ft per box. Gives you total fleet square footage for the productivity math.</t>
         </is>
       </c>
-      <c r="K20" s="32" t="inlineStr">
+      <c r="K20" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-sqft formula</t>
         </is>
@@ -4219,7 +4270,7 @@
           <t>Last year's total store-channel revenue — the base you're growing comps off of, not the new boxes.</t>
         </is>
       </c>
-      <c r="K28" s="32" t="inlineStr">
+      <c r="K28" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: prior store-rev formula</t>
         </is>
@@ -4264,7 +4315,7 @@
           <t>Existing-store sales only — prior store rev grown by geo comp %. New doors are a separate line, not in here.</t>
         </is>
       </c>
-      <c r="K29" s="32" t="inlineStr">
+      <c r="K29" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: comp-store formula</t>
         </is>
@@ -4309,7 +4360,7 @@
           <t>Net new doors × sq ft × $/sq ft is plain dollars. /1000 → $000 on this tab. ×0.55 'cause year-one stores don't run full.</t>
         </is>
       </c>
-      <c r="K30" s="32" t="inlineStr">
+      <c r="K30" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: net-new-store formula</t>
         </is>
@@ -4354,7 +4405,7 @@
           <t>Brick-and-mortar channel = comp store sales plus whatever the net new stores contributed. That's the whole store line.</t>
         </is>
       </c>
-      <c r="K31" s="32" t="inlineStr">
+      <c r="K31" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: store-channel formula</t>
         </is>
@@ -4718,7 +4769,7 @@
           <t>Traffic × conversion × AOV is dollars. ×1M 'cause sessions are in millions; /1000 puts it in $000 like everything else.</t>
         </is>
       </c>
-      <c r="K41" s="32" t="inlineStr">
+      <c r="K41" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: e-comm formula</t>
         </is>
@@ -5247,7 +5298,7 @@
           <t>Bottom-up total = store channel + e-comm + other. That's your driver-built revenue before you check Scenarios.</t>
         </is>
       </c>
-      <c r="K55" s="32" t="inlineStr">
+      <c r="K55" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-rev formula</t>
         </is>
@@ -5338,7 +5389,7 @@
           <t>Driver-built revenue minus Scenarios revenue. Shows you how far off the bottom-up path is from what you're valuing on.</t>
         </is>
       </c>
-      <c r="K57" s="32" t="inlineStr">
+      <c r="K57" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: variance formula</t>
         </is>
@@ -5384,14 +5435,14 @@
           <t>Variance as a percent of Scenarios revenue. Easy read on whether the driver schedule is close or way out of line.</t>
         </is>
       </c>
-      <c r="K58" s="32" t="inlineStr">
+      <c r="K58" s="26" t="inlineStr">
         <is>
           <t>Revenue Drivers: variance % formula</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="26" t="inlineStr">
+      <c r="A59" s="28" t="inlineStr">
         <is>
           <t>Note: DCF / Scenarios consolidated revenue is the valuation anchor — drivers do not feed the DCF. A small variance vs Scenarios means the bottom-up path still hangs together, so the Scenarios case stays viable. Bigger gaps = revisit drivers or Scenarios assumptions.</t>
         </is>
@@ -5564,7 +5615,7 @@
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="38" t="inlineStr">
         <is>
           <t>Full Assumptions Guide (PDF)
 Ctrl+F: Every red assumption on every tab — justification, source link, Ctrl+F proof.</t>
@@ -5586,27 +5637,27 @@
       <c r="E5" s="75" t="n">
         <v>11102600</v>
       </c>
-      <c r="F5" s="24">
+      <c r="F5" s="76">
         <f>Scenarios!G18</f>
         <v/>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="76">
         <f>Scenarios!G19</f>
         <v/>
       </c>
-      <c r="H5" s="24">
+      <c r="H5" s="76">
         <f>Scenarios!G20</f>
         <v/>
       </c>
-      <c r="I5" s="24">
+      <c r="I5" s="76">
         <f>Scenarios!G21</f>
         <v/>
       </c>
-      <c r="J5" s="24">
+      <c r="J5" s="76">
         <f>Scenarios!G22</f>
         <v/>
       </c>
-      <c r="K5" s="76">
+      <c r="K5" s="77">
         <f>IF(MAX(ABS(F5-Scenarios!$G$18),ABS(G5-Scenarios!$G$19),ABS(H5-Scenarios!$G$20),ABS(I5-Scenarios!$G$21),ABS(J5-Scenarios!$G$22))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5623,7 +5674,7 @@
 Also: 2.3% FY27–30 growth matches StockAnalysis Revenue Growth Forecast (3Y) of 2.26%; next-year consensus is +2.64%.</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
+      <c r="C6" s="38" t="inlineStr">
         <is>
           <t>LULU Q2 FY2026 earnings release
 Also: StockAnalysis: LULU 3Y revenue forecast</t>
@@ -5635,23 +5686,23 @@
 Also: Ctrl+F "Revenue Growth Forecast (3Y)" → 2.26%. That is the unique line (do not search "Net revenue"). Model FY27–30 uses 2.3%.</t>
         </is>
       </c>
-      <c r="F6" s="33">
+      <c r="F6" s="32">
         <f>F5/E5-1</f>
         <v/>
       </c>
-      <c r="G6" s="33">
+      <c r="G6" s="32">
         <f>G5/F5-1</f>
         <v/>
       </c>
-      <c r="H6" s="33">
+      <c r="H6" s="32">
         <f>H5/G5-1</f>
         <v/>
       </c>
-      <c r="I6" s="33">
+      <c r="I6" s="32">
         <f>I5/H5-1</f>
         <v/>
       </c>
-      <c r="J6" s="33">
+      <c r="J6" s="32">
         <f>J5/I5-1</f>
         <v/>
       </c>
@@ -5668,7 +5719,7 @@
 Also: FY30 15.5% is a partial recovery vs the FY25 10-K OM of 19.9% (unique Ctrl+F). Still well below the FY24 23.7% peak.</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="38" t="inlineStr">
         <is>
           <t>Q2 FY2026 release: 18.8% OM minus 560bps tariffs
 Also: FY2025 10-K: Operating margin 19.9% (one hit)</t>
@@ -5680,27 +5731,27 @@
 Also: Ctrl+F "19.9%" (one hit) → Operating margin decreased 380 basis points to 19.9%. That is FY25 OM. Do not search the words Income from operations (17 hits). Model FY30 15.5% is a partial-recovery assumption.</t>
         </is>
       </c>
-      <c r="F7" s="33">
+      <c r="F7" s="32">
         <f>Scenarios!G23</f>
         <v/>
       </c>
-      <c r="G7" s="33">
+      <c r="G7" s="32">
         <f>Scenarios!G24</f>
         <v/>
       </c>
-      <c r="H7" s="33">
+      <c r="H7" s="32">
         <f>Scenarios!G25</f>
         <v/>
       </c>
-      <c r="I7" s="33">
+      <c r="I7" s="32">
         <f>Scenarios!G26</f>
         <v/>
       </c>
-      <c r="J7" s="33">
+      <c r="J7" s="32">
         <f>Scenarios!G27</f>
         <v/>
       </c>
-      <c r="K7" s="76">
+      <c r="K7" s="77">
         <f>IF(MAX(ABS(F7-Scenarios!$G$23),ABS(G7-Scenarios!$G$24),ABS(H7-Scenarios!$G$25),ABS(I7-Scenarios!$G$26),ABS(J7-Scenarios!$G$27))&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5729,53 +5780,53 @@
       <c r="E8" s="75" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="38">
+      <c r="F8" s="37">
         <f>Scenarios!$G$7</f>
         <v/>
       </c>
-      <c r="G8" s="38" t="n">
+      <c r="G8" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="38" t="n">
+      <c r="H8" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="38" t="n">
+      <c r="I8" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="38" t="n">
+      <c r="J8" s="37" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>EBIT (incl. FY26 refund)</t>
         </is>
       </c>
-      <c r="E9" s="77" t="n">
+      <c r="E9" s="78" t="n">
         <v>2210615</v>
       </c>
-      <c r="F9" s="28">
+      <c r="F9" s="27">
         <f>Scenarios!G28</f>
         <v/>
       </c>
-      <c r="G9" s="28">
+      <c r="G9" s="27">
         <f>Scenarios!G29</f>
         <v/>
       </c>
-      <c r="H9" s="28">
+      <c r="H9" s="27">
         <f>Scenarios!G30</f>
         <v/>
       </c>
-      <c r="I9" s="28">
+      <c r="I9" s="27">
         <f>Scenarios!G31</f>
         <v/>
       </c>
-      <c r="J9" s="28">
+      <c r="J9" s="27">
         <f>Scenarios!G32</f>
         <v/>
       </c>
-      <c r="K9" s="78">
+      <c r="K9" s="79">
         <f>IF(MAX(ABS(F9-Scenarios!$G$28),ABS(G9-Scenarios!$G$29),ABS(H9-Scenarios!$G$30),ABS(I9-Scenarios!$G$31),ABS(J9-Scenarios!$G$32))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5786,26 +5837,26 @@
           <t>Reported EBIT margin % (incl. FY26 refund)</t>
         </is>
       </c>
-      <c r="E10" s="79" t="n">
+      <c r="E10" s="80" t="n">
         <v>0.1991078666258354</v>
       </c>
-      <c r="F10" s="33">
+      <c r="F10" s="32">
         <f>F9/F5</f>
         <v/>
       </c>
-      <c r="G10" s="33">
+      <c r="G10" s="32">
         <f>G9/G5</f>
         <v/>
       </c>
-      <c r="H10" s="33">
+      <c r="H10" s="32">
         <f>H9/H5</f>
         <v/>
       </c>
-      <c r="I10" s="33">
+      <c r="I10" s="32">
         <f>I9/I5</f>
         <v/>
       </c>
-      <c r="J10" s="33">
+      <c r="J10" s="32">
         <f>J9/J5</f>
         <v/>
       </c>
@@ -5816,54 +5867,54 @@
           <t>Less: cash taxes on EBIT</t>
         </is>
       </c>
-      <c r="F11" s="24">
+      <c r="F11" s="76">
         <f>-Scenarios!G28*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="G11" s="24">
+      <c r="G11" s="76">
         <f>-Scenarios!G29*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="H11" s="24">
+      <c r="H11" s="76">
         <f>-Scenarios!G30*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="I11" s="24">
+      <c r="I11" s="76">
         <f>-Scenarios!G31*Scenarios!$G$11</f>
         <v/>
       </c>
-      <c r="J11" s="24">
+      <c r="J11" s="76">
         <f>-Scenarios!G32*Scenarios!$G$11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>NOPAT</t>
         </is>
       </c>
-      <c r="F12" s="28">
+      <c r="F12" s="27">
         <f>Scenarios!G33</f>
         <v/>
       </c>
-      <c r="G12" s="28">
+      <c r="G12" s="27">
         <f>Scenarios!G34</f>
         <v/>
       </c>
-      <c r="H12" s="28">
+      <c r="H12" s="27">
         <f>Scenarios!G35</f>
         <v/>
       </c>
-      <c r="I12" s="28">
+      <c r="I12" s="27">
         <f>Scenarios!G36</f>
         <v/>
       </c>
-      <c r="J12" s="28">
+      <c r="J12" s="27">
         <f>Scenarios!G37</f>
         <v/>
       </c>
-      <c r="K12" s="78">
+      <c r="K12" s="79">
         <f>IF(MAX(ABS(F12-Scenarios!$G$33),ABS(G12-Scenarios!$G$34),ABS(H12-Scenarios!$G$35),ABS(I12-Scenarios!$G$36),ABS(J12-Scenarios!$G$37))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5916,27 +5967,27 @@
           <t>Plus: depreciation &amp; amortization</t>
         </is>
       </c>
-      <c r="F14" s="24">
+      <c r="F14" s="76">
         <f>Scenarios!G38</f>
         <v/>
       </c>
-      <c r="G14" s="24">
+      <c r="G14" s="76">
         <f>Scenarios!G39</f>
         <v/>
       </c>
-      <c r="H14" s="24">
+      <c r="H14" s="76">
         <f>Scenarios!G40</f>
         <v/>
       </c>
-      <c r="I14" s="24">
+      <c r="I14" s="76">
         <f>Scenarios!G41</f>
         <v/>
       </c>
-      <c r="J14" s="24">
+      <c r="J14" s="76">
         <f>Scenarios!G42</f>
         <v/>
       </c>
-      <c r="K14" s="76">
+      <c r="K14" s="77">
         <f>IF(MAX(ABS(F14-Scenarios!$G$38),ABS(G14-Scenarios!$G$39),ABS(H14-Scenarios!$G$40),ABS(I14-Scenarios!$G$41),ABS(J14-Scenarios!$G$42))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -5953,7 +6004,7 @@
 Also: FY26 sales are $10.35–$10.50B (earnings). Use that $10.4B year as the 7% denominator, not FY25 $11.1B.</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="C15" s="38" t="inlineStr">
         <is>
           <t>LULU 10-K: 2026 capex guide $725–745M
 Also: Q2 FY2026 outlook: $10.350B–$10.500B sales</t>
@@ -6002,27 +6053,27 @@
           <t>Less: capital expenditures</t>
         </is>
       </c>
-      <c r="F16" s="24">
+      <c r="F16" s="76">
         <f>-Scenarios!G43</f>
         <v/>
       </c>
-      <c r="G16" s="24">
+      <c r="G16" s="76">
         <f>-Scenarios!G44</f>
         <v/>
       </c>
-      <c r="H16" s="24">
+      <c r="H16" s="76">
         <f>-Scenarios!G45</f>
         <v/>
       </c>
-      <c r="I16" s="24">
+      <c r="I16" s="76">
         <f>-Scenarios!G46</f>
         <v/>
       </c>
-      <c r="J16" s="24">
+      <c r="J16" s="76">
         <f>-Scenarios!G47</f>
         <v/>
       </c>
-      <c r="K16" s="76">
+      <c r="K16" s="77">
         <f>IF(MAX(ABS(F16+Scenarios!$G$43),ABS(G16+Scenarios!$G$44),ABS(H16+Scenarios!$G$45),ABS(I16+Scenarios!$G$46),ABS(J16+Scenarios!$G$47))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -6135,27 +6186,27 @@
       <c r="E19" s="75" t="n">
         <v>190657</v>
       </c>
-      <c r="F19" s="24">
+      <c r="F19" s="76">
         <f>Scenarios!G48</f>
         <v/>
       </c>
-      <c r="G19" s="24">
+      <c r="G19" s="76">
         <f>Scenarios!G49</f>
         <v/>
       </c>
-      <c r="H19" s="24">
+      <c r="H19" s="76">
         <f>Scenarios!G50</f>
         <v/>
       </c>
-      <c r="I19" s="24">
+      <c r="I19" s="76">
         <f>Scenarios!G51</f>
         <v/>
       </c>
-      <c r="J19" s="24">
+      <c r="J19" s="76">
         <f>Scenarios!G52</f>
         <v/>
       </c>
-      <c r="K19" s="76">
+      <c r="K19" s="77">
         <f>IF(MAX(ABS(F19-Scenarios!$G$48),ABS(G19-Scenarios!$G$49),ABS(H19-Scenarios!$G$50),ABS(I19-Scenarios!$G$51),ABS(J19-Scenarios!$G$52))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -6166,65 +6217,65 @@
           <t>(Increase)/decrease in NWC (includes AR)</t>
         </is>
       </c>
-      <c r="F20" s="24">
+      <c r="F20" s="76">
         <f>-Scenarios!G53</f>
         <v/>
       </c>
-      <c r="G20" s="24">
+      <c r="G20" s="76">
         <f>-Scenarios!G54</f>
         <v/>
       </c>
-      <c r="H20" s="24">
+      <c r="H20" s="76">
         <f>-Scenarios!G55</f>
         <v/>
       </c>
-      <c r="I20" s="24">
+      <c r="I20" s="76">
         <f>-Scenarios!G56</f>
         <v/>
       </c>
-      <c r="J20" s="24">
+      <c r="J20" s="76">
         <f>-Scenarios!G57</f>
         <v/>
       </c>
-      <c r="K20" s="76">
+      <c r="K20" s="77">
         <f>IF(MAX(ABS(F20+Scenarios!$G$53),ABS(G20+Scenarios!$G$54),ABS(H20+Scenarios!$G$55),ABS(I20+Scenarios!$G$56),ABS(J20+Scenarios!$G$57))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="26" t="inlineStr">
+      <c r="A21" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: NWC and AR are one line. 7.5% of Δsales already includes AR; UFCF does not take ΔAR separately.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>Unlevered free cash flow</t>
         </is>
       </c>
-      <c r="F22" s="80">
+      <c r="F22" s="81">
         <f>Scenarios!G58</f>
         <v/>
       </c>
-      <c r="G22" s="80">
+      <c r="G22" s="81">
         <f>Scenarios!G59</f>
         <v/>
       </c>
-      <c r="H22" s="80">
+      <c r="H22" s="81">
         <f>Scenarios!G60</f>
         <v/>
       </c>
-      <c r="I22" s="80">
+      <c r="I22" s="81">
         <f>Scenarios!G61</f>
         <v/>
       </c>
-      <c r="J22" s="80">
+      <c r="J22" s="81">
         <f>Scenarios!G62</f>
         <v/>
       </c>
-      <c r="K22" s="78">
+      <c r="K22" s="79">
         <f>IF(MAX(ABS(F22-Scenarios!$G$58),ABS(G22-Scenarios!$G$59),ABS(H22-Scenarios!$G$60),ABS(I22-Scenarios!$G$61),ABS(J22-Scenarios!$G$62))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -6235,19 +6286,19 @@
           <t>Discount period (years)</t>
         </is>
       </c>
-      <c r="F23" s="81" t="n">
+      <c r="F23" s="82" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="81" t="n">
+      <c r="G23" s="82" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="81" t="n">
+      <c r="H23" s="82" t="n">
         <v>3</v>
       </c>
-      <c r="I23" s="81" t="n">
+      <c r="I23" s="82" t="n">
         <v>4</v>
       </c>
-      <c r="J23" s="81" t="n">
+      <c r="J23" s="82" t="n">
         <v>5</v>
       </c>
     </row>
@@ -6257,50 +6308,50 @@
           <t>Discount factor @ WACC</t>
         </is>
       </c>
-      <c r="F24" s="82">
+      <c r="F24" s="83">
         <f>1/(1+Scenarios!$G$9)^F23</f>
         <v/>
       </c>
-      <c r="G24" s="82">
+      <c r="G24" s="83">
         <f>1/(1+Scenarios!$G$9)^G23</f>
         <v/>
       </c>
-      <c r="H24" s="82">
+      <c r="H24" s="83">
         <f>1/(1+Scenarios!$G$9)^H23</f>
         <v/>
       </c>
-      <c r="I24" s="82">
+      <c r="I24" s="83">
         <f>1/(1+Scenarios!$G$9)^I23</f>
         <v/>
       </c>
-      <c r="J24" s="82">
+      <c r="J24" s="83">
         <f>1/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>PV of unlevered FCF</t>
         </is>
       </c>
-      <c r="F25" s="28">
+      <c r="F25" s="27">
         <f>F22*F24</f>
         <v/>
       </c>
-      <c r="G25" s="28">
+      <c r="G25" s="27">
         <f>G22*G24</f>
         <v/>
       </c>
-      <c r="H25" s="28">
+      <c r="H25" s="27">
         <f>H22*H24</f>
         <v/>
       </c>
-      <c r="I25" s="28">
+      <c r="I25" s="27">
         <f>I22*I24</f>
         <v/>
       </c>
-      <c r="J25" s="28">
+      <c r="J25" s="27">
         <f>J22*J24</f>
         <v/>
       </c>
@@ -6311,13 +6362,13 @@
           <t>Scenarios linkage summary (column K should all read OK)</t>
         </is>
       </c>
-      <c r="K27" s="83">
+      <c r="K27" s="84">
         <f>IF(COUNTIF(K5:K22,"CHECK")=0,"ALL OK","REVIEW")</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="84" t="inlineStr">
+      <c r="A28" s="85" t="inlineStr">
         <is>
           <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
         </is>
@@ -6326,7 +6377,7 @@
       <c r="C28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="27" t="inlineStr">
+      <c r="A29" s="25" t="inlineStr">
         <is>
           <t>Sum of PV of explicit FCF (FY26–FY30)</t>
         </is>
@@ -6357,18 +6408,18 @@
           <t>Ctrl+F "Q2 2026" → 24,269.613 and "Q2 2025" → 23,770.976. YoY = 2.1%. Model terminal g 2.25%.</t>
         </is>
       </c>
-      <c r="E30" s="33">
+      <c r="E30" s="32">
         <f>Scenarios!$G$10</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="27" t="inlineStr">
+      <c r="A31" s="25" t="inlineStr">
         <is>
           <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="E31" s="28">
+      <c r="E31" s="27">
         <f>J9+J14</f>
         <v/>
       </c>
@@ -6379,7 +6430,7 @@
           <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
         </is>
       </c>
-      <c r="E32" s="24">
+      <c r="E32" s="76">
         <f>J22*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
         <v/>
       </c>
@@ -6390,7 +6441,7 @@
           <t xml:space="preserve">  Implied exit EV/EBITDA = Gordon TV / FY30 EBITDA</t>
         </is>
       </c>
-      <c r="E33" s="85">
+      <c r="E33" s="86">
         <f>E32/E31</f>
         <v/>
       </c>
@@ -6401,13 +6452,13 @@
           <t xml:space="preserve">  memo: (UFCF₃₀ / EBITDA₃₀) × (1+g) / (WACC−g)</t>
         </is>
       </c>
-      <c r="E34" s="85">
+      <c r="E34" s="86">
         <f>J22/E31*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="27" t="inlineStr">
+      <c r="A35" s="25" t="inlineStr">
         <is>
           <t>PV of terminal value</t>
         </is>
@@ -6418,12 +6469,12 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="27" t="inlineStr">
+      <c r="A36" s="25" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="E36" s="28">
+      <c r="E36" s="27">
         <f>E29+E35</f>
         <v/>
       </c>
@@ -6434,7 +6485,7 @@
           <t>Plus: cash &amp; equivalents (FY2025)</t>
         </is>
       </c>
-      <c r="C37" s="86" t="inlineStr">
+      <c r="C37" s="87" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -6474,26 +6525,26 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="26" t="inlineStr">
+      <c r="A39" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: funded term debt $0. Operating leases $298,724k current + $1,499,717k non-current = $1,798,441k (ASC 842 debt equivalent).</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="26" t="inlineStr">
+      <c r="A40" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: UFCF is pre-interest; rent stays in opex. We subtract lease liabilities in the bridge but do not add back implied lease interest to EBIT (simplified treatment).</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="27" t="inlineStr">
+      <c r="A41" s="25" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
       </c>
-      <c r="E41" s="28">
+      <c r="E41" s="27">
         <f>E36+E37+E38</f>
         <v/>
       </c>
@@ -6504,7 +6555,7 @@
           <t>Shares outstanding (000)</t>
         </is>
       </c>
-      <c r="C42" s="86" t="inlineStr">
+      <c r="C42" s="87" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -6519,16 +6570,16 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="27" t="inlineStr">
+      <c r="A43" s="25" t="inlineStr">
         <is>
           <t>Implied value per share</t>
         </is>
       </c>
-      <c r="E43" s="87">
+      <c r="E43" s="88">
         <f>E41/E42</f>
         <v/>
       </c>
-      <c r="K43" s="78">
+      <c r="K43" s="79">
         <f>IF(ABS(E43-Scenarios!$G$65)&lt;0.05,"OK","CHECK")</f>
         <v/>
       </c>
@@ -6539,7 +6590,7 @@
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C44" s="86" t="inlineStr">
+      <c r="C44" s="87" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -6549,17 +6600,17 @@
           <t>Ctrl+F "closed at $100.61" → Last Sale on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E44" s="88" t="n">
+      <c r="E44" s="89" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="27" t="inlineStr">
+      <c r="A45" s="25" t="inlineStr">
         <is>
           <t>Implied upside / (downside)</t>
         </is>
       </c>
-      <c r="E45" s="89">
+      <c r="E45" s="90">
         <f>E43/E44-1</f>
         <v/>
       </c>
@@ -6570,13 +6621,13 @@
           <t xml:space="preserve">  memo: % of EV from terminal value</t>
         </is>
       </c>
-      <c r="E46" s="33">
+      <c r="E46" s="32">
         <f>E35/E36</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="84" t="inlineStr">
+      <c r="A48" s="85" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
@@ -6612,11 +6663,11 @@
           <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
         </is>
       </c>
-      <c r="E50" s="85">
+      <c r="E50" s="86">
         <f>E33</f>
         <v/>
       </c>
-      <c r="M50" s="86" t="inlineStr">
+      <c r="M50" s="87" t="inlineStr">
         <is>
           <t>Comps: Exit Multiple Build</t>
         </is>
@@ -6628,7 +6679,7 @@
           <t>Terminal value = Terminal EBITDA × exit multiple</t>
         </is>
       </c>
-      <c r="E51" s="24">
+      <c r="E51" s="76">
         <f>E31*E50</f>
         <v/>
       </c>
@@ -6639,35 +6690,35 @@
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="E52" s="24">
+      <c r="E52" s="76">
         <f>E51/(1+Scenarios!$G$9)^J23</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="27" t="inlineStr">
+      <c r="A53" s="25" t="inlineStr">
         <is>
           <t>Enterprise value (exit method)</t>
         </is>
       </c>
-      <c r="E53" s="28">
+      <c r="E53" s="27">
         <f>E29+E52</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="27" t="inlineStr">
+      <c r="A54" s="25" t="inlineStr">
         <is>
           <t>Implied value per share (exit method)</t>
         </is>
       </c>
-      <c r="E54" s="90">
+      <c r="E54" s="91">
         <f>(E53+E37+E38)/E42</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="84" t="inlineStr">
+      <c r="A56" s="85" t="inlineStr">
         <is>
           <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
         </is>
@@ -6677,7 +6728,7 @@
       <c r="D56" s="13" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="91" t="inlineStr"/>
+      <c r="A57" s="92" t="inlineStr"/>
       <c r="B57" s="50" t="inlineStr">
         <is>
           <t>Gordon Growth</t>
@@ -6695,7 +6746,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="27" t="inlineStr">
+      <c r="A58" s="25" t="inlineStr">
         <is>
           <t>Terminal value ($)</t>
         </is>
@@ -6714,20 +6765,20 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="27" t="inlineStr">
+      <c r="A59" s="25" t="inlineStr">
         <is>
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
       </c>
-      <c r="B59" s="92">
+      <c r="B59" s="93">
         <f>E33</f>
         <v/>
       </c>
-      <c r="C59" s="92">
+      <c r="C59" s="93">
         <f>E50</f>
         <v/>
       </c>
-      <c r="D59" s="92">
+      <c r="D59" s="93">
         <f>B59-C59</f>
         <v/>
       </c>
@@ -6738,28 +6789,28 @@
           <t>Terminal value variance (%)</t>
         </is>
       </c>
-      <c r="B60" s="33" t="inlineStr"/>
-      <c r="C60" s="33" t="inlineStr"/>
-      <c r="D60" s="33">
+      <c r="B60" s="32" t="inlineStr"/>
+      <c r="C60" s="32" t="inlineStr"/>
+      <c r="D60" s="32">
         <f>(B58-C58)/B58</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="27" t="inlineStr">
+      <c r="A61" s="25" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="B61" s="93">
+      <c r="B61" s="94">
         <f>E43</f>
         <v/>
       </c>
-      <c r="C61" s="93">
+      <c r="C61" s="94">
         <f>E54</f>
         <v/>
       </c>
-      <c r="D61" s="93">
+      <c r="D61" s="94">
         <f>B61-C61</f>
         <v/>
       </c>
@@ -6770,22 +6821,22 @@
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B62" s="94">
+      <c r="B62" s="95">
         <f>IF(ABS(D59)&lt;=1.5,"PASS","REVIEW")</f>
         <v/>
       </c>
-      <c r="C62" s="95">
+      <c r="C62" s="96">
         <f>TEXT(D59,"0.0")&amp;"x spread vs Gordon-implied exit"</f>
         <v/>
       </c>
-      <c r="D62" s="26" t="inlineStr">
+      <c r="D62" s="28" t="inlineStr">
         <is>
           <t>Selected exit is the Gordon identity, so spread should be 0</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="84" t="inlineStr">
+      <c r="A65" s="85" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
@@ -6799,7 +6850,7 @@
       <c r="H65" s="13" t="n"/>
     </row>
     <row r="66" ht="28" customHeight="1">
-      <c r="A66" s="96" t="inlineStr">
+      <c r="A66" s="97" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
@@ -6819,32 +6870,32 @@
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
       </c>
-      <c r="F66" s="97" t="n">
+      <c r="F66" s="98" t="n">
         <v>0.015</v>
       </c>
-      <c r="G66" s="97" t="n">
+      <c r="G66" s="98" t="n">
         <v>0.02</v>
       </c>
-      <c r="H66" s="97" t="n">
+      <c r="H66" s="98" t="n">
         <v>0.0225</v>
       </c>
-      <c r="I66" s="97" t="n">
+      <c r="I66" s="98" t="n">
         <v>0.025</v>
       </c>
-      <c r="J66" s="97" t="n">
+      <c r="J66" s="98" t="n">
         <v>0.03</v>
       </c>
-      <c r="L66" s="86" t="inlineStr">
+      <c r="L66" s="87" t="inlineStr">
         <is>
           <t>Scenarios: terminal g</t>
         </is>
       </c>
     </row>
     <row r="67" ht="28" customHeight="1">
-      <c r="A67" s="97" t="n">
+      <c r="A67" s="98" t="n">
         <v>0.095</v>
       </c>
-      <c r="C67" s="86" t="inlineStr">
+      <c r="C67" s="87" t="inlineStr">
         <is>
           <t>Damodaran: Historical Implied ERP</t>
         </is>
@@ -6854,34 +6905,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F67" s="98">
+      <c r="F67" s="99">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="G67" s="98">
+      <c r="G67" s="99">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="H67" s="98">
+      <c r="H67" s="99">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="I67" s="98">
+      <c r="I67" s="99">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="J67" s="98">
+      <c r="J67" s="99">
         <f>(NPV(0.095,F22:J22)+(J22*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="L67" s="86" t="inlineStr">
+      <c r="L67" s="87" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="68" ht="28" customHeight="1">
-      <c r="A68" s="97" t="n">
+      <c r="A68" s="98" t="n">
         <v>0.1</v>
       </c>
       <c r="D68" s="19" t="inlineStr">
@@ -6889,34 +6940,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F68" s="98">
+      <c r="F68" s="99">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="G68" s="98">
+      <c r="G68" s="99">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="H68" s="98">
+      <c r="H68" s="99">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="I68" s="98">
+      <c r="I68" s="99">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="J68" s="98">
+      <c r="J68" s="99">
         <f>(NPV(0.1,F22:J22)+(J22*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="L68" s="86" t="inlineStr">
+      <c r="L68" s="87" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="69" ht="28" customHeight="1">
-      <c r="A69" s="97" t="n">
+      <c r="A69" s="98" t="n">
         <v>0.105</v>
       </c>
       <c r="D69" s="19" t="inlineStr">
@@ -6924,34 +6975,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F69" s="98">
+      <c r="F69" s="99">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="G69" s="98">
+      <c r="G69" s="99">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="H69" s="99">
+      <c r="H69" s="100">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="I69" s="98">
+      <c r="I69" s="99">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="J69" s="98">
+      <c r="J69" s="99">
         <f>(NPV(0.105,F22:J22)+(J22*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="L69" s="86" t="inlineStr">
+      <c r="L69" s="87" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="70" ht="28" customHeight="1">
-      <c r="A70" s="97" t="n">
+      <c r="A70" s="98" t="n">
         <v>0.11</v>
       </c>
       <c r="D70" s="19" t="inlineStr">
@@ -6959,34 +7010,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F70" s="98">
+      <c r="F70" s="99">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="G70" s="98">
+      <c r="G70" s="99">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="H70" s="98">
+      <c r="H70" s="99">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="I70" s="98">
+      <c r="I70" s="99">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="J70" s="98">
+      <c r="J70" s="99">
         <f>(NPV(0.11,F22:J22)+(J22*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="L70" s="86" t="inlineStr">
+      <c r="L70" s="87" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="71" ht="28" customHeight="1">
-      <c r="A71" s="97" t="n">
+      <c r="A71" s="98" t="n">
         <v>0.115</v>
       </c>
       <c r="D71" s="19" t="inlineStr">
@@ -6994,27 +7045,27 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F71" s="98">
+      <c r="F71" s="99">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="G71" s="98">
+      <c r="G71" s="99">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="H71" s="98">
+      <c r="H71" s="99">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="I71" s="98">
+      <c r="I71" s="99">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="J71" s="98">
+      <c r="J71" s="99">
         <f>(NPV(0.115,F22:J22)+(J22*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E37+E38)/E42</f>
         <v/>
       </c>
-      <c r="L71" s="86" t="inlineStr">
+      <c r="L71" s="87" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
@@ -7036,7 +7087,7 @@
           <t>Scenarios tab → Ctrl+F "WACC" and "Terminal growth" rows (base-case inputs)</t>
         </is>
       </c>
-      <c r="L72" s="86" t="inlineStr">
+      <c r="L72" s="87" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
@@ -7079,11 +7130,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId25"/>
     <hyperlink ref="L66" location="'Scenarios'!G10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId26"/>
-    <hyperlink ref="L67" location="'WACC'!E28"/>
-    <hyperlink ref="L68" location="'WACC'!E28"/>
-    <hyperlink ref="L69" location="'WACC'!E28"/>
-    <hyperlink ref="L70" location="'WACC'!E28"/>
-    <hyperlink ref="L71" location="'WACC'!E28"/>
+    <hyperlink ref="L67" location="'WACC'!E30"/>
+    <hyperlink ref="L68" location="'WACC'!E30"/>
+    <hyperlink ref="L69" location="'WACC'!E30"/>
+    <hyperlink ref="L70" location="'WACC'!E30"/>
+    <hyperlink ref="L71" location="'WACC'!E30"/>
     <hyperlink ref="C72" location="'Scenarios'!G9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId27"/>
   </hyperlinks>
@@ -7156,7 +7207,7 @@
           <t>FY2025A revenue</t>
         </is>
       </c>
-      <c r="C4" s="86" t="inlineStr">
+      <c r="C4" s="87" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -7176,7 +7227,7 @@
           <t>FY2025A EBITDA (EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="76">
         <f>2210615+496228</f>
         <v/>
       </c>
@@ -7187,12 +7238,12 @@
           <t>FY2030E terminal EBITDA (DCF EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="C6" s="86" t="inlineStr">
+      <c r="C6" s="87" t="inlineStr">
         <is>
           <t>↳ DCF base case</t>
         </is>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="76">
         <f>DCF!E31</f>
         <v/>
       </c>
@@ -7203,7 +7254,7 @@
           <t>FY2026E diluted EPS (guidance midpoint)</t>
         </is>
       </c>
-      <c r="C7" s="86" t="inlineStr">
+      <c r="C7" s="87" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
@@ -7213,7 +7264,7 @@
           <t>Ctrl+F "$9.48 to $9.73" → FY2026 diluted EPS guidance; model midpoint $9.61</t>
         </is>
       </c>
-      <c r="E7" s="88" t="n">
+      <c r="E7" s="89" t="n">
         <v>9.609999999999999</v>
       </c>
     </row>
@@ -7223,7 +7274,7 @@
           <t>Cash &amp; equivalents</t>
         </is>
       </c>
-      <c r="C8" s="86" t="inlineStr">
+      <c r="C8" s="87" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -7243,7 +7294,7 @@
           <t>Shares outstanding (000)</t>
         </is>
       </c>
-      <c r="C9" s="86" t="inlineStr">
+      <c r="C9" s="87" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -7263,7 +7314,7 @@
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C10" s="86" t="inlineStr">
+      <c r="C10" s="87" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -7273,28 +7324,28 @@
           <t>Ctrl+F "closed at $100.61" → Last Sale on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E10" s="88" t="n">
+      <c r="E10" s="89" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="95" t="inlineStr">
+      <c r="A11" s="96" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current EV / EBITDA</t>
         </is>
       </c>
-      <c r="E11" s="100">
+      <c r="E11" s="101">
         <f>(E10*E9-E8)/E5</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="95" t="inlineStr">
+      <c r="A12" s="96" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current P / E (FY2026E)</t>
         </is>
       </c>
-      <c r="E12" s="100">
+      <c r="E12" s="101">
         <f>E10/E7</f>
         <v/>
       </c>
@@ -7307,7 +7358,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="95" t="inlineStr">
+      <c r="A15" s="96" t="inlineStr">
         <is>
           <t>Peer / reference EV/EBITDA (forward / illustrative)</t>
         </is>
@@ -7321,44 +7372,44 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="26" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>EV/EBITDA is a black formula (I/J). UAA is shown but excluded from averages (negative TTM EBITDA).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="101" t="inlineStr">
+      <c r="A18" s="102" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B18" s="101" t="inlineStr">
+      <c r="B18" s="102" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C18" s="101" t="inlineStr">
+      <c r="C18" s="102" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D18" s="101" t="inlineStr">
+      <c r="D18" s="102" t="inlineStr">
         <is>
           <t>Ctrl+F / proof</t>
         </is>
       </c>
-      <c r="E18" s="102" t="inlineStr">
+      <c r="E18" s="103" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="I18" s="102" t="inlineStr">
+      <c r="I18" s="103" t="inlineStr">
         <is>
           <t>EV ($000)</t>
         </is>
       </c>
-      <c r="J18" s="102" t="inlineStr">
+      <c r="J18" s="103" t="inlineStr">
         <is>
           <t>EBITDA ($000)</t>
         </is>
@@ -7375,7 +7426,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C19" s="32" t="inlineStr">
+      <c r="C19" s="26" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7385,14 +7436,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E19" s="103">
+      <c r="E19" s="104">
         <f>IF(J19&lt;=0,"n.m.",I19/J19)</f>
         <v/>
       </c>
-      <c r="I19" s="104" t="n">
+      <c r="I19" s="105" t="n">
         <v>11890440</v>
       </c>
-      <c r="J19" s="104" t="n">
+      <c r="J19" s="105" t="n">
         <v>2548084</v>
       </c>
     </row>
@@ -7407,7 +7458,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C20" s="32" t="inlineStr">
+      <c r="C20" s="26" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7417,14 +7468,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E20" s="103">
+      <c r="E20" s="104">
         <f>IF(J20&lt;=0,"n.m.",I20/J20)</f>
         <v/>
       </c>
-      <c r="I20" s="104" t="n">
+      <c r="I20" s="105" t="n">
         <v>3208397</v>
       </c>
-      <c r="J20" s="104" t="n">
+      <c r="J20" s="105" t="n">
         <v>-23230</v>
       </c>
     </row>
@@ -7439,7 +7490,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C21" s="32" t="inlineStr">
+      <c r="C21" s="26" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7449,14 +7500,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E21" s="103">
+      <c r="E21" s="104">
         <f>IF(J21&lt;=0,"n.m.",I21/J21)</f>
         <v/>
       </c>
-      <c r="I21" s="104" t="n">
+      <c r="I21" s="105" t="n">
         <v>35661944</v>
       </c>
-      <c r="J21" s="104" t="n">
+      <c r="J21" s="105" t="n">
         <v>3857684</v>
       </c>
     </row>
@@ -7471,7 +7522,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C22" s="32" t="inlineStr">
+      <c r="C22" s="26" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7481,14 +7532,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E22" s="103">
+      <c r="E22" s="104">
         <f>IF(J22&lt;=0,"n.m.",I22/J22)</f>
         <v/>
       </c>
-      <c r="I22" s="104" t="n">
+      <c r="I22" s="105" t="n">
         <v>58972350</v>
       </c>
-      <c r="J22" s="104" t="n">
+      <c r="J22" s="105" t="n">
         <v>4647000</v>
       </c>
     </row>
@@ -7503,7 +7554,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C23" s="32" t="inlineStr">
+      <c r="C23" s="26" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7513,14 +7564,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E23" s="103">
+      <c r="E23" s="104">
         <f>IF(J23&lt;=0,"n.m.",I23/J23)</f>
         <v/>
       </c>
-      <c r="I23" s="104" t="n">
+      <c r="I23" s="105" t="n">
         <v>10555510</v>
       </c>
-      <c r="J23" s="104" t="n">
+      <c r="J23" s="105" t="n">
         <v>1329439</v>
       </c>
     </row>
@@ -7535,7 +7586,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C24" s="32" t="inlineStr">
+      <c r="C24" s="26" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7545,14 +7596,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E24" s="103">
+      <c r="E24" s="104">
         <f>IF(J24&lt;=0,"n.m.",I24/J24)</f>
         <v/>
       </c>
-      <c r="I24" s="104" t="n">
+      <c r="I24" s="105" t="n">
         <v>27284350</v>
       </c>
-      <c r="J24" s="104" t="n">
+      <c r="J24" s="105" t="n">
         <v>1768400</v>
       </c>
     </row>
@@ -7567,7 +7618,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C25" s="32" t="inlineStr">
+      <c r="C25" s="26" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7577,14 +7628,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E25" s="103">
+      <c r="E25" s="104">
         <f>IF(J25&lt;=0,"n.m.",I25/J25)</f>
         <v/>
       </c>
-      <c r="I25" s="104" t="n">
+      <c r="I25" s="105" t="n">
         <v>7153911</v>
       </c>
-      <c r="J25" s="104" t="n">
+      <c r="J25" s="105" t="n">
         <v>922278</v>
       </c>
     </row>
@@ -7599,7 +7650,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C26" s="32" t="inlineStr">
+      <c r="C26" s="26" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7609,14 +7660,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E26" s="103">
+      <c r="E26" s="104">
         <f>IF(J26&lt;=0,"n.m.",I26/J26)</f>
         <v/>
       </c>
-      <c r="I26" s="104" t="n">
+      <c r="I26" s="105" t="n">
         <v>616045</v>
       </c>
-      <c r="J26" s="104" t="n">
+      <c r="J26" s="105" t="n">
         <v>62010</v>
       </c>
     </row>
@@ -7631,7 +7682,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C27" s="32" t="inlineStr">
+      <c r="C27" s="26" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7641,14 +7692,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E27" s="103">
+      <c r="E27" s="104">
         <f>IF(J27&lt;=0,"n.m.",I27/J27)</f>
         <v/>
       </c>
-      <c r="I27" s="104" t="n">
+      <c r="I27" s="105" t="n">
         <v>9422753</v>
       </c>
-      <c r="J27" s="104" t="n">
+      <c r="J27" s="105" t="n">
         <v>976700</v>
       </c>
     </row>
@@ -7663,7 +7714,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C28" s="32" t="inlineStr">
+      <c r="C28" s="26" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7673,14 +7724,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E28" s="103">
+      <c r="E28" s="104">
         <f>IF(J28&lt;=0,"n.m.",I28/J28)</f>
         <v/>
       </c>
-      <c r="I28" s="104" t="n">
+      <c r="I28" s="105" t="n">
         <v>1598873</v>
       </c>
-      <c r="J28" s="104" t="n">
+      <c r="J28" s="105" t="n">
         <v>235723</v>
       </c>
     </row>
@@ -7695,7 +7746,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C29" s="32" t="inlineStr">
+      <c r="C29" s="26" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7705,14 +7756,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E29" s="103">
+      <c r="E29" s="104">
         <f>IF(J29&lt;=0,"n.m.",I29/J29)</f>
         <v/>
       </c>
-      <c r="I29" s="104" t="n">
+      <c r="I29" s="105" t="n">
         <v>5236269</v>
       </c>
-      <c r="J29" s="104" t="n">
+      <c r="J29" s="105" t="n">
         <v>407521</v>
       </c>
     </row>
@@ -7724,7 +7775,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="26" t="inlineStr">
+      <c r="A32" s="28" t="inlineStr">
         <is>
           <t>Column E on the next two rows is $bn, not EV/EBITDA. The black formula is implied EV/Sales on an unclosed ask.</t>
         </is>
@@ -7742,7 +7793,7 @@
 Also: Reuters June 2026: no deal was announced on the 2023 process. The $10bn is still an ask.</t>
         </is>
       </c>
-      <c r="C33" s="23" t="inlineStr">
+      <c r="C33" s="38" t="inlineStr">
         <is>
           <t>Reuters: Alo parent $10bn Moelis ask
 Also: Reuters: Alo 2023 process — no deal</t>
@@ -7754,7 +7805,7 @@
 Also: Ctrl+F "roughly $10 billion" and "No deal was announced". Still an ask.</t>
         </is>
       </c>
-      <c r="E33" s="105" t="n">
+      <c r="E33" s="106" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7779,7 +7830,7 @@
           <t>Ctrl+F "nearly $2 billion". Forbes estimate for Color Image parent (Alo + Bella+Canvas), not Alo-only EBITDA.</t>
         </is>
       </c>
-      <c r="E34" s="105" t="n">
+      <c r="E34" s="106" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7789,12 +7840,12 @@
           <t>Alo implied EV/Sales (ask / parent sales)</t>
         </is>
       </c>
-      <c r="B35" s="26" t="inlineStr">
+      <c r="B35" s="28" t="inlineStr">
         <is>
           <t>5.0x = 10 / 2. Implied EV/Sales on an unclosed ask and parent sales. Not EV/EBITDA. Not the TV.</t>
         </is>
       </c>
-      <c r="C35" s="86" t="inlineStr">
+      <c r="C35" s="87" t="inlineStr">
         <is>
           <t>Comps: Alo ask / parent sales</t>
         </is>
@@ -7804,7 +7855,7 @@
           <t>No Ctrl+F for EV/EBITDA — Firecrawl found none on Reuters or Forbes. This cell is E33 / E34 (ask ÷ parent sales). Not the TV.</t>
         </is>
       </c>
-      <c r="E35" s="106">
+      <c r="E35" s="107">
         <f>E33/E34</f>
         <v/>
       </c>
@@ -7815,12 +7866,12 @@
           <t>Alo EV/EBITDA</t>
         </is>
       </c>
-      <c r="B36" s="26" t="inlineStr">
+      <c r="B36" s="28" t="inlineStr">
         <is>
           <t>No page prints Alo or Color Image EBITDA. PitchBook Alo column is blank. Cannot imply EV/EBITDA.</t>
         </is>
       </c>
-      <c r="C36" s="26" t="inlineStr">
+      <c r="C36" s="28" t="inlineStr">
         <is>
           <t>None — no EBITDA source</t>
         </is>
@@ -7830,7 +7881,7 @@
           <t>No Ctrl+F. Reuters, Forbes, and PitchBook do not print Alo EV/EBITDA.</t>
         </is>
       </c>
-      <c r="E36" s="107" t="inlineStr">
+      <c r="E36" s="108" t="inlineStr">
         <is>
           <t>n.a.</t>
         </is>
@@ -7849,22 +7900,22 @@
           <t>Core athletic / apparel mean (LULU / NKE / ADS / DECK / CROX / LEVI / KTB)</t>
         </is>
       </c>
-      <c r="B39" s="26" t="inlineStr">
+      <c r="B39" s="28" t="inlineStr">
         <is>
           <t>PitchBook core set, UAA out. Current tape — not a 2.25% g FY30 exit.</t>
         </is>
       </c>
-      <c r="C39" s="26" t="inlineStr">
+      <c r="C39" s="28" t="inlineStr">
         <is>
           <t>Derived: Excel AVERAGE of the seven core prints</t>
         </is>
       </c>
-      <c r="D39" s="26" t="inlineStr">
+      <c r="D39" s="28" t="inlineStr">
         <is>
           <t>Each E cell is I/J from the PitchBook extract. Do not use as FY30 exit.</t>
         </is>
       </c>
-      <c r="E39" s="103">
+      <c r="E39" s="104">
         <f>AVERAGE(E19,E22,E21,E23,E25,E27,E29)</f>
         <v/>
       </c>
@@ -7875,28 +7926,28 @@
           <t>All positive-EBITDA mean (ex-UAA; includes WSM / MOV / LZB)</t>
         </is>
       </c>
-      <c r="B40" s="26" t="inlineStr">
+      <c r="B40" s="28" t="inlineStr">
         <is>
           <t>Wider PitchBook tape. WSM/MOV/LZB are adjacent retail, not athletic. Not the TV.</t>
         </is>
       </c>
-      <c r="C40" s="26" t="inlineStr">
+      <c r="C40" s="28" t="inlineStr">
         <is>
           <t>Derived: Excel AVERAGE of every positive-EBITDA row</t>
         </is>
       </c>
-      <c r="D40" s="26" t="inlineStr">
+      <c r="D40" s="28" t="inlineStr">
         <is>
           <t>UAA omitted because TTM EBITDA is negative. Not the selected FY30 exit.</t>
         </is>
       </c>
-      <c r="E40" s="103">
+      <c r="E40" s="104">
         <f>AVERAGE(E19,E21,E22,E23,E24,E25,E26,E27,E28,E29)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="95" t="inlineStr">
+      <c r="A41" s="96" t="inlineStr">
         <is>
           <t>We do not average peers for terminal value, and we do not use Alo 5.0x EV/Sales as EV/EBITDA.</t>
         </is>
@@ -7915,7 +7966,7 @@
           <t>Gordon Growth implied exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="E44" s="85">
+      <c r="E44" s="86">
         <f>DCF!E33</f>
         <v/>
       </c>
@@ -7926,7 +7977,7 @@
           <t>Selected exit multiple (base case)</t>
         </is>
       </c>
-      <c r="E45" s="92">
+      <c r="E45" s="93">
         <f>DCF!E50</f>
         <v/>
       </c>
@@ -7937,7 +7988,7 @@
           <t>Spread (selected − Gordon implied)</t>
         </is>
       </c>
-      <c r="E46" s="85">
+      <c r="E46" s="86">
         <f>E45-E44</f>
         <v/>
       </c>
@@ -7999,42 +8050,42 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="101" t="inlineStr">
+      <c r="A56" s="102" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B56" s="101" t="inlineStr">
+      <c r="B56" s="102" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C56" s="101" t="inlineStr">
+      <c r="C56" s="102" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D56" s="101" t="inlineStr">
+      <c r="D56" s="102" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
-      <c r="E56" s="102" t="inlineStr">
+      <c r="E56" s="103" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="F56" s="102" t="inlineStr">
+      <c r="F56" s="103" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="G56" s="102" t="inlineStr">
+      <c r="G56" s="103" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="H56" s="102" t="inlineStr">
+      <c r="H56" s="103" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
@@ -8064,17 +8115,17 @@
 Hi: Ctrl+F "EV / EBITDA" → 7.95. Football-field cap 8.0x (Deckers). Not the selected exit.</t>
         </is>
       </c>
-      <c r="E57" s="108" t="n">
+      <c r="E57" s="109" t="n">
         <v>5</v>
       </c>
-      <c r="F57" s="108" t="n">
+      <c r="F57" s="109" t="n">
         <v>8</v>
       </c>
-      <c r="G57" s="109">
+      <c r="G57" s="110">
         <f>(E6*E57+E8)/E9</f>
         <v/>
       </c>
-      <c r="H57" s="109">
+      <c r="H57" s="110">
         <f>(E6*F57+E8)/E9</f>
         <v/>
       </c>
@@ -8100,11 +8151,11 @@
           <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
         </is>
       </c>
-      <c r="E58" s="106">
+      <c r="E58" s="107">
         <f>DCF!E50</f>
         <v/>
       </c>
-      <c r="G58" s="110">
+      <c r="G58" s="111">
         <f>(E6*E58+E8)/E9</f>
         <v/>
       </c>
@@ -8133,17 +8184,17 @@
 Hi: Ctrl+F "Forward PE" → NKE peer benchmark; high-case assumption 18.0x</t>
         </is>
       </c>
-      <c r="E59" s="108" t="n">
+      <c r="E59" s="109" t="n">
         <v>10</v>
       </c>
-      <c r="F59" s="108" t="n">
+      <c r="F59" s="109" t="n">
         <v>18</v>
       </c>
-      <c r="G59" s="109">
+      <c r="G59" s="110">
         <f>E7*E59</f>
         <v/>
       </c>
-      <c r="H59" s="109">
+      <c r="H59" s="110">
         <f>E7*F59</f>
         <v/>
       </c>
@@ -8154,32 +8205,32 @@
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="E60" s="111" t="inlineStr">
+      <c r="E60" s="112" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F60" s="111" t="inlineStr">
+      <c r="F60" s="112" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G60" s="109">
+      <c r="G60" s="110">
         <f>Scenarios!F65</f>
         <v/>
       </c>
-      <c r="H60" s="109">
+      <c r="H60" s="110">
         <f>Scenarios!H65</f>
         <v/>
       </c>
     </row>
     <row r="62" ht="28" customHeight="1">
-      <c r="A62" s="112" t="inlineStr">
+      <c r="A62" s="113" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C62" s="86" t="inlineStr">
+      <c r="C62" s="87" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -8189,12 +8240,12 @@
           <t>Ctrl+F "closed at $100.61" → Last Sale on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E62" s="113" t="n">
+      <c r="E62" s="114" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="26" t="inlineStr">
+      <c r="A63" s="28" t="inlineStr">
         <is>
           <t>Note: pubcomps are PitchBook 04-Sep-2026 (EV/EBITDA = daily EV / TTM EBITDA). UAA excluded from the mean. Selected TV is Gordon implied, not the PitchBook average. Alo EV/EBITDA is n.a.</t>
         </is>

</xml_diff>

<commit_message>
Clarify 0.86 is levered beta (βL), not unlevered βu
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1328,12 +1328,12 @@
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>Observed Beta (5Y) — not used in WACC</t>
+          <t>Observed Beta (5Y) — levered βL, not used in WACC</t>
         </is>
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>StockAnalysis Beta (5Y) is 0.86. Company 5Y print; too calm after the guide cut, so not the WACC input.</t>
+          <t>StockAnalysis Beta (5Y) 0.86 is levered equity β (βL) from regressions — not unlevered βu. Too calm post-guide-cut; not the WACC input.</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Beta (5Y)" → 0.86. Company 5Y beta. Not the WACC input.</t>
+          <t>Ctrl+F "Beta (5Y)" → 0.86. This is levered equity β (βL), not unlevered βu. Shown for reference only.</t>
         </is>
       </c>
       <c r="E5" s="21" t="n">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Damodaran unlevered Retail (Special Lines) β 0.95 is the starting point; we relever it for ASC 842 lease debt.</t>
+          <t>Damodaran unlevered Retail (Special Lines) βu 0.95 is the starting point; we relever it for ASC 842 lease debt. Do not confuse with company βL 0.86.</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95. Relever for ASC 842 lease debt on the next row.</t>
+          <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95 (βu). Do not use levered column 1.09 or company βL 0.86 here.</t>
         </is>
       </c>
       <c r="E6" s="22" t="n">
@@ -1576,16 +1576,17 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Relever Damodaran unlevered retail β for ASC 842 lease debt.
-Unlevered β (Damodaran Jan 2026)
+          <t>Relever Damodaran unlevered retail βu for ASC 842 lease debt.
+Unlevered βu (Damodaran Jan 2026)
   Ctrl+F "Retail (Special Lines)"  →  Unlevered beta 0.95
   Do not take the levered Beta column (1.09)
 Lease debt equivalent (FY25 10-K)
   Ctrl+F "Current lease liabilities"  →  298,724
   Ctrl+F "Non-current lease liabilities"  →  1,499,717
   Sum = 1,798,441 ($000). No funded term loans.
-Company 5Y (StockAnalysis) — shown, not used
-  Ctrl+F "Beta (5Y)"  →  0.86</t>
+Company 5Y (StockAnalysis) — levered βL, not βu; not used
+  Ctrl+F "Beta (5Y)"  →  0.86 = equity beta (βL), not unlevered
+  0.86 is not a substitute for βu 0.95 on the relever row above</t>
         </is>
       </c>
       <c r="E19" s="29">

</xml_diff>

<commit_message>
WACC beta: unlever company βL 0.86 then relever for lease debt
Replace Damodaran 0.95 input with Hamada chain: βu from observed
βL using funded D/E (zero), then relever βu for ASC 842 lease
liabilities. Damodaran sector β kept as benchmark reference only.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -437,29 +437,29 @@
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="2" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="2" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -1232,7 +1232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1328,400 +1328,435 @@
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>Observed Beta (5Y) — levered βL, not used in WACC</t>
+          <t>Tax rate</t>
         </is>
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>StockAnalysis Beta (5Y) 0.86 is levered equity β (βL) from regressions — not unlevered βu. Too calm post-guide-cut; not the WACC input.</t>
+          <t>30% cash tax matches FY2026 guidance (“approximately 30%”); FY25 effective was 29.5%.</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>StockAnalysis: LULU Beta (5Y)</t>
+          <t>Q2 FY2026 outlook: tax rate ≈ 30%</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Beta (5Y)" → 0.86. This is levered equity β (βL), not unlevered βu. Shown for reference only.</t>
-        </is>
-      </c>
-      <c r="E5" s="21" t="n">
-        <v>0.86</v>
-      </c>
-    </row>
-    <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>Unlevered retail beta (Damodaran Special Lines)</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Damodaran unlevered Retail (Special Lines) βu 0.95 is the starting point; we relever it for ASC 842 lease debt. Do not confuse with company βL 0.86.</t>
-        </is>
-      </c>
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>Damodaran: US betas by sector (Jan 2026)</t>
-        </is>
-      </c>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95 (βu). Do not use levered column 1.09 or company βL 0.86 here.</t>
-        </is>
-      </c>
-      <c r="E6" s="22" t="n">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Tax rate</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>30% cash tax matches FY2026 guidance (“approximately 30%”); FY25 effective was 29.5%.</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>Q2 FY2026 outlook: tax rate ≈ 30%</t>
-        </is>
-      </c>
-      <c r="D7" s="19" t="inlineStr">
-        <is>
           <t>Ctrl+F "a tax rate of approximately 30%" on the FY2026 outlook paragraph.</t>
         </is>
       </c>
-      <c r="E7" s="20" t="n">
+      <c r="E5" s="20" t="n">
         <v>0.3</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Capital structure (market values)</t>
         </is>
       </c>
     </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Share price ($)</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>$100 share price ≈ NASDAQ Last Sale after Q2 FY2026 guide cut; rounded from $100.61 close.</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>NASDAQ LULU last sale (current price)</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "closed at $100.61" → Last Sale $100.61 (NASDAQ). Model uses $100 rounded.</t>
+        </is>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Shares outstanding (000)</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>111,380k class A shares outstanding at FY25 year-end (10-K cover). Diluted WA 119,068 is for EPS, not market cap.</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: shares outstanding</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "111,380 and 116,166 issued and outstanding" → 111,380k class A shares (FY25 10-K cover).</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>111380</v>
+      </c>
+    </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>Share price ($)</t>
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>Market value of equity</t>
         </is>
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>$100 share price ≈ NASDAQ Last Sale after Q2 FY2026 guide cut; rounded from $100.61 close.</t>
-        </is>
-      </c>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>NASDAQ LULU last sale (current price)</t>
+          <t>Market equity = share price × shares outstanding. Capital-structure weighting numerator for relevered β and WACC weights.</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>WACC tab: price × shares</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "closed at $100.61" → Last Sale $100.61 (NASDAQ). Model uses $100 rounded.</t>
-        </is>
-      </c>
-      <c r="E10" s="23" t="n">
-        <v>100</v>
+          <t>Share price row × shares outstanding row on this tab.</t>
+        </is>
+      </c>
+      <c r="E10" s="25">
+        <f>E8*E9</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>Shares outstanding (000)</t>
+          <t>Operating lease liabilities (ASC 842 debt equiv.)</t>
         </is>
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>111,380k class A shares outstanding at FY25 year-end (10-K cover). Diluted WA 119,068 is for EPS, not market cap.</t>
+          <t>ASC 842 operating lease liabilities = current + non-current ($1,798,441k FY25). Treated as debt equivalent in WACC and EV bridge.</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K: shares outstanding</t>
+          <t>LULU FY2025 10-K: operating lease liabilities</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "111,380 and 116,166 issued and outstanding" → 111,380k class A shares (FY25 10-K cover).</t>
-        </is>
-      </c>
-      <c r="E11" s="24" t="n">
-        <v>111380</v>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="25" t="inlineStr">
-        <is>
-          <t>Market value of equity</t>
-        </is>
-      </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>Market equity = share price × shares outstanding. Capital-structure weighting numerator for relevered β and WACC weights.</t>
-        </is>
-      </c>
-      <c r="C12" s="26" t="inlineStr">
-        <is>
-          <t>WACC tab: price × shares</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>Share price row × shares outstanding row on this tab.</t>
-        </is>
-      </c>
-      <c r="E12" s="27">
-        <f>E10*E11</f>
-        <v/>
+          <t>Ctrl+F "Current lease liabilities" → 298,724 | "Non-current lease liabilities" → 1,499,717 | sum = 1,798,441 ($000)</t>
+        </is>
+      </c>
+      <c r="E11" s="22" t="n">
+        <v>1798441</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  memo: current $298,724k + non-current $1,499,717k = $1,798,441k (FY25 10-K)</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Operating lease liabilities (ASC 842 debt equiv.)</t>
+          <t>Funded debt (term loans / bonds)</t>
         </is>
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>ASC 842 operating lease liabilities = current + non-current ($1,798,441k FY25). Treated as debt equivalent in WACC and EV bridge.</t>
+          <t>Funded term debt $0 — 10-K: no borrowings outstanding on the revolver. Leases are the only debt equivalent here.</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K: operating lease liabilities</t>
+          <t>LULU FY2025 10-K (no funded debt)</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Current lease liabilities" → 298,724 | "Non-current lease liabilities" → 1,499,717 | sum = 1,798,441 ($000)</t>
-        </is>
-      </c>
-      <c r="E13" s="24" t="n">
-        <v>1798441</v>
+          <t>Ctrl+F "no borrowings were outstanding under this facility" → funded debt $0</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  memo: current $298,724k + non-current $1,499,717k = $1,798,441k (FY25 10-K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>Funded debt (term loans / bonds)</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>Funded term debt $0 — 10-K: no borrowings outstanding on the revolver. Leases are the only debt equivalent here.</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K (no funded debt)</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "no borrowings were outstanding under this facility" → funded debt $0</t>
-        </is>
-      </c>
-      <c r="E15" s="24" t="n">
-        <v>0</v>
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>Total debt equivalents</t>
+        </is>
+      </c>
+      <c r="E14" s="25">
+        <f>E11+E13</f>
+        <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr">
-        <is>
-          <t>Total debt equivalents</t>
-        </is>
-      </c>
-      <c r="E16" s="27">
-        <f>E13+E15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>Cost of equity (CAPM) — relevered</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="150" customHeight="1">
-      <c r="A19" s="25" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Beta (unlever → relever)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Observed Beta (5Y) — levered βL</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>StockAnalysis Beta (5Y) 0.86 is levered equity βL — the starting point for the unlever / relever chain below.</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>StockAnalysis: LULU Beta (5Y)</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Beta (5Y)" → 0.86. Levered equity βL (StockAnalysis).</t>
+        </is>
+      </c>
+      <c r="E17" s="27" t="n">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Unlevered βu (Hamada; funded D/E only)</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>βu = βL ÷ [1 + (1−T) × funded D/E]. No term loans → funded D/E = 0, so βu = 0.86.</t>
+        </is>
+      </c>
+      <c r="C18" s="24" t="inlineStr">
+        <is>
+          <t>WACC tab: Hamada unlever (funded D/E)</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>βu = E[βL] ÷ (1 + (1−T) × E[funded debt] ÷ E[market equity]). Funded debt = $0 → βu = 0.86.</t>
+        </is>
+      </c>
+      <c r="E18" s="28">
+        <f>E17/(1+(1-E5)*E13/E10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Sector βu benchmark (Damodaran Special Lines) — not used</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Damodaran unlevered Retail (Special Lines) βu 0.95 shown as a sector benchmark only — not the WACC input.</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Damodaran: US betas by sector (Jan 2026)</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95 (βu). Sector benchmark only — not used in WACC.</t>
+        </is>
+      </c>
+      <c r="E19" s="27" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="20" ht="150" customHeight="1">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>Beta used (relevered for lease debt)</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>Relevered β = βu × (1 + (1−T) × lease debt / market equity). No funded term loans — leases are the debt equivalent.</t>
-        </is>
-      </c>
-      <c r="C19" s="18" t="inlineStr">
-        <is>
-          <t>Damodaran: relevered β for lease debt</t>
-        </is>
-      </c>
-      <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>Relever Damodaran unlevered retail βu for ASC 842 lease debt.
-Unlevered βu (Damodaran Jan 2026)
-  Ctrl+F "Retail (Special Lines)"  →  Unlevered beta 0.95
-  Do not take the levered Beta column (1.09)
-Lease debt equivalent (FY25 10-K)
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>βL = βu × [1 + (1−T) × total debt equiv. / E]. Relevers company βu for ASC 842 lease liabilities in WACC.</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>WACC tab: Hamada relever (total D/E incl. leases)</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Company β: unlever observed βL, then relever for ASC 842 lease debt.
+Step 1 — Observed levered βL (StockAnalysis)
+  Ctrl+F "Beta (5Y)"  →  0.86
+Step 2 — Unlever (Hamada; funded debt only)
+  βu = βL ÷ [1 + (1−T) × D_funded/E]
+  Funded debt $0 (10-K) → βu = 0.86
+Step 3 — Relever (total debt equiv. incl. leases)
+  βL = βu × [1 + (1−T) × D_total/E]
   Ctrl+F "Current lease liabilities"  →  298,724
   Ctrl+F "Non-current lease liabilities"  →  1,499,717
-  Sum = 1,798,441 ($000). No funded term loans.
-Company 5Y (StockAnalysis) — levered βL, not βu; not used
-  Ctrl+F "Beta (5Y)"  →  0.86 = equity beta (βL), not unlevered
-  0.86 is not a substitute for βu 0.95 on the relever row above</t>
-        </is>
-      </c>
-      <c r="E19" s="29">
-        <f>E6*(1+(1-E7)*E13/E12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  memo: relever unlevered retail β for ASC 842 lease debt. βL = βu × (1 + (1−T) × D/E). No funded term loans.</t>
-        </is>
+  D_total = 1,798,441 ($000) + funded debt $0
+Sector benchmark (Damodaran) — not used
+  Ctrl+F "Retail (Special Lines)"  →  Unlevered beta 0.95</t>
+        </is>
+      </c>
+      <c r="E20" s="29">
+        <f>E18*(1+(1-E5)*E14/E10)</f>
+        <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  memo: βu strips funded debt only (none). βL relevers for ASC 842 leases. βL = βu × (1 + (1−T) × D/E).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>Cost of equity (CAPM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
         <is>
           <t>Cost of equity = rf + β × ERP</t>
         </is>
       </c>
-      <c r="E21" s="30">
-        <f>E3+E19*E4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="E23" s="30">
+        <f>E3+E20*E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>Cost of debt (lease-equivalent)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="16" t="inlineStr">
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>Pre-tax cost of debt (lease-equivalent)</t>
         </is>
       </c>
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>5.0% pre-tax lease-equivalent borrowing cost; cheaper than equity. No funded revolver borrowings per FY25 10-K.</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C26" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: lease liabilities &amp; no funded debt</t>
         </is>
       </c>
-      <c r="D24" s="19" t="inlineStr">
+      <c r="D26" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Current lease liabilities" + "Non-current lease liabilities" → debt equiv. 5.0% illustrative lease borrowing cost.</t>
         </is>
       </c>
-      <c r="E24" s="20" t="n">
+      <c r="E26" s="20" t="n">
         <v>0.05</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="E25" s="31">
-        <f>E24*(1-E7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="E27" s="31">
+        <f>E26*(1-E5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>WACC weights</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="16" t="inlineStr">
+    <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>Equity weight</t>
         </is>
       </c>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>Equity weight = market cap ÷ (market cap + lease debt). ~86% at $100 and FY25 lease balance.</t>
         </is>
       </c>
-      <c r="C28" s="26" t="inlineStr">
+      <c r="C30" s="24" t="inlineStr">
         <is>
           <t>WACC tab: capital structure</t>
         </is>
       </c>
-      <c r="D28" s="19" t="inlineStr">
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>Equity weight = market cap ÷ (market cap + lease debt). Live formula on this tab.</t>
         </is>
       </c>
-      <c r="E28" s="32">
-        <f>E12/(E12+E16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="E30" s="32">
+        <f>E10/(E10+E14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>Debt weight (leases + funded)</t>
         </is>
       </c>
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>Debt weight = lease liabilities ÷ (market cap + lease debt). ~14% — ASC 842 leases, not bank debt.</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
+      <c r="C31" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: operating lease liabilities</t>
         </is>
       </c>
-      <c r="D29" s="19" t="inlineStr">
+      <c r="D31" s="19" t="inlineStr">
         <is>
           <t>Debt weight = lease liabilities ÷ (market cap + lease debt). ~14% at FY25 balances.</t>
         </is>
       </c>
-      <c r="E29" s="32">
-        <f>E16/(E12+E16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="25" t="inlineStr">
+      <c r="E31" s="32">
+        <f>E14/(E10+E14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="23" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="E30" s="33">
-        <f>E28*E21+E29*E25</f>
+      <c r="E32" s="33">
+        <f>E30*E23+E31*E27</f>
         <v/>
       </c>
     </row>
@@ -1730,15 +1765,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1988,14 +2022,14 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>WACC tab → cell E (green) = rf 4.8% + β 0.95 × ERP 6.0% = 10.5%</t>
+          <t>WACC tab → green cell = rf 4.8% + relevered β × ERP 6.0%</t>
         </is>
       </c>
       <c r="F9" s="20" t="n">
         <v>0.11</v>
       </c>
       <c r="G9" s="32">
-        <f>WACC!E30</f>
+        <f>WACC!E32</f>
         <v/>
       </c>
       <c r="H9" s="20" t="n">
@@ -3064,20 +3098,20 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="25" t="inlineStr">
+      <c r="A64" s="23" t="inlineStr">
         <is>
           <t>Enterprise value (DCF)</t>
         </is>
       </c>
-      <c r="F64" s="27">
+      <c r="F64" s="25">
         <f>NPV(F9,F58,F59,F60,F61,F62)+(F62*(1+F10)/(F9-F10))/(1+F9)^5</f>
         <v/>
       </c>
-      <c r="G64" s="27">
+      <c r="G64" s="25">
         <f>NPV(G9,G58,G59,G60,G61,G62)+(G62*(1+G10)/(G9-G10))/(1+G9)^5</f>
         <v/>
       </c>
-      <c r="H64" s="27">
+      <c r="H64" s="25">
         <f>NPV(H9,H58,H59,H60,H61,H62)+(H62*(1+H10)/(H9-H10))/(1+H9)^5</f>
         <v/>
       </c>
@@ -3102,7 +3136,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="25" t="inlineStr">
+      <c r="A66" s="23" t="inlineStr">
         <is>
           <t>Upside / (downside) vs current</t>
         </is>
@@ -3121,7 +3155,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="28" t="inlineStr">
+      <c r="A68" s="26" t="inlineStr">
         <is>
           <t>Current price $100.00; cash $1,807,202 k; lease debt $1,798,441 k; funded debt $0; net cash $8,761 k.</t>
         </is>
@@ -3134,7 +3168,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
-    <hyperlink ref="C9" location="'WACC'!E30"/>
+    <hyperlink ref="C9" location="'WACC'!E32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
@@ -3188,7 +3222,7 @@
       <c r="L1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>FY2025A = Firecrawl-ingested 10-K anchors (blue). FY26–30 = red operational assumptions. Consolidated revenue cross-checks to Scenarios base case.</t>
         </is>
@@ -3329,7 +3363,7 @@
           <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
         </is>
       </c>
-      <c r="K6" s="26" t="inlineStr">
+      <c r="K6" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
@@ -3463,7 +3497,7 @@
           <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
         </is>
       </c>
-      <c r="K9" s="26" t="inlineStr">
+      <c r="K9" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
@@ -3513,7 +3547,7 @@
           <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
         </is>
       </c>
-      <c r="K10" s="26" t="inlineStr">
+      <c r="K10" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
@@ -3647,7 +3681,7 @@
           <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
         </is>
       </c>
-      <c r="K13" s="26" t="inlineStr">
+      <c r="K13" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
@@ -3697,7 +3731,7 @@
           <t>Beginning stores = last year's ending count. Same number, just carried forward into the new fiscal year.</t>
         </is>
       </c>
-      <c r="K14" s="26" t="inlineStr">
+      <c r="K14" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: beginning-stores formula</t>
         </is>
@@ -3831,7 +3865,7 @@
           <t>Simple roll-forward: where you started, plus openings, minus closures. That's your ending store count for the year.</t>
         </is>
       </c>
-      <c r="K17" s="26" t="inlineStr">
+      <c r="K17" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: ending-stores formula</t>
         </is>
@@ -3876,7 +3910,7 @@
           <t>Add up Americas + China + RoW ending stores. Should tie to the 10-K total company-operated count.</t>
         </is>
       </c>
-      <c r="K18" s="26" t="inlineStr">
+      <c r="K18" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-stores formula</t>
         </is>
@@ -3972,7 +4006,7 @@
           <t>Ending stores times avg sq ft per box. Gives you total fleet square footage for the productivity math.</t>
         </is>
       </c>
-      <c r="K20" s="26" t="inlineStr">
+      <c r="K20" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-sqft formula</t>
         </is>
@@ -4271,7 +4305,7 @@
           <t>Last year's total store-channel revenue — the base you're growing comps off of, not the new boxes.</t>
         </is>
       </c>
-      <c r="K28" s="26" t="inlineStr">
+      <c r="K28" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: prior store-rev formula</t>
         </is>
@@ -4316,7 +4350,7 @@
           <t>Existing-store sales only — prior store rev grown by geo comp %. New doors are a separate line, not in here.</t>
         </is>
       </c>
-      <c r="K29" s="26" t="inlineStr">
+      <c r="K29" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: comp-store formula</t>
         </is>
@@ -4361,7 +4395,7 @@
           <t>Net new doors × sq ft × $/sq ft is plain dollars. /1000 → $000 on this tab. ×0.55 'cause year-one stores don't run full.</t>
         </is>
       </c>
-      <c r="K30" s="26" t="inlineStr">
+      <c r="K30" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: net-new-store formula</t>
         </is>
@@ -4406,7 +4440,7 @@
           <t>Brick-and-mortar channel = comp store sales plus whatever the net new stores contributed. That's the whole store line.</t>
         </is>
       </c>
-      <c r="K31" s="26" t="inlineStr">
+      <c r="K31" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: store-channel formula</t>
         </is>
@@ -4770,7 +4804,7 @@
           <t>Traffic × conversion × AOV is dollars. ×1M 'cause sessions are in millions; /1000 puts it in $000 like everything else.</t>
         </is>
       </c>
-      <c r="K41" s="26" t="inlineStr">
+      <c r="K41" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: e-comm formula</t>
         </is>
@@ -5299,7 +5333,7 @@
           <t>Bottom-up total = store channel + e-comm + other. That's your driver-built revenue before you check Scenarios.</t>
         </is>
       </c>
-      <c r="K55" s="26" t="inlineStr">
+      <c r="K55" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: total-rev formula</t>
         </is>
@@ -5390,7 +5424,7 @@
           <t>Driver-built revenue minus Scenarios revenue. Shows you how far off the bottom-up path is from what you're valuing on.</t>
         </is>
       </c>
-      <c r="K57" s="26" t="inlineStr">
+      <c r="K57" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: variance formula</t>
         </is>
@@ -5436,14 +5470,14 @@
           <t>Variance as a percent of Scenarios revenue. Easy read on whether the driver schedule is close or way out of line.</t>
         </is>
       </c>
-      <c r="K58" s="26" t="inlineStr">
+      <c r="K58" s="24" t="inlineStr">
         <is>
           <t>Revenue Drivers: variance % formula</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="28" t="inlineStr">
+      <c r="A59" s="26" t="inlineStr">
         <is>
           <t>Note: DCF / Scenarios consolidated revenue is the valuation anchor — drivers do not feed the DCF. A small variance vs Scenarios means the bottom-up path still hangs together, so the Scenarios case stays viable. Bigger gaps = revisit drivers or Scenarios assumptions.</t>
         </is>
@@ -5799,7 +5833,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="25" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>EBIT (incl. FY26 refund)</t>
         </is>
@@ -5807,23 +5841,23 @@
       <c r="E9" s="78" t="n">
         <v>2210615</v>
       </c>
-      <c r="F9" s="27">
+      <c r="F9" s="25">
         <f>Scenarios!G28</f>
         <v/>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="25">
         <f>Scenarios!G29</f>
         <v/>
       </c>
-      <c r="H9" s="27">
+      <c r="H9" s="25">
         <f>Scenarios!G30</f>
         <v/>
       </c>
-      <c r="I9" s="27">
+      <c r="I9" s="25">
         <f>Scenarios!G31</f>
         <v/>
       </c>
-      <c r="J9" s="27">
+      <c r="J9" s="25">
         <f>Scenarios!G32</f>
         <v/>
       </c>
@@ -5890,28 +5924,28 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>NOPAT</t>
         </is>
       </c>
-      <c r="F12" s="27">
+      <c r="F12" s="25">
         <f>Scenarios!G33</f>
         <v/>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="25">
         <f>Scenarios!G34</f>
         <v/>
       </c>
-      <c r="H12" s="27">
+      <c r="H12" s="25">
         <f>Scenarios!G35</f>
         <v/>
       </c>
-      <c r="I12" s="27">
+      <c r="I12" s="25">
         <f>Scenarios!G36</f>
         <v/>
       </c>
-      <c r="J12" s="27">
+      <c r="J12" s="25">
         <f>Scenarios!G37</f>
         <v/>
       </c>
@@ -6244,14 +6278,14 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: NWC and AR are one line. 7.5% of Δsales already includes AR; UFCF does not take ΔAR separately.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="inlineStr">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t>Unlevered free cash flow</t>
         </is>
@@ -6331,28 +6365,28 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="25" t="inlineStr">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>PV of unlevered FCF</t>
         </is>
       </c>
-      <c r="F25" s="27">
+      <c r="F25" s="25">
         <f>F22*F24</f>
         <v/>
       </c>
-      <c r="G25" s="27">
+      <c r="G25" s="25">
         <f>G22*G24</f>
         <v/>
       </c>
-      <c r="H25" s="27">
+      <c r="H25" s="25">
         <f>H22*H24</f>
         <v/>
       </c>
-      <c r="I25" s="27">
+      <c r="I25" s="25">
         <f>I22*I24</f>
         <v/>
       </c>
-      <c r="J25" s="27">
+      <c r="J25" s="25">
         <f>J22*J24</f>
         <v/>
       </c>
@@ -6378,7 +6412,7 @@
       <c r="C28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="25" t="inlineStr">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>Sum of PV of explicit FCF (FY26–FY30)</t>
         </is>
@@ -6415,12 +6449,12 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="25" t="inlineStr">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>Terminal EBITDA (FY2030E EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="E31" s="27">
+      <c r="E31" s="25">
         <f>J9+J14</f>
         <v/>
       </c>
@@ -6459,7 +6493,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="25" t="inlineStr">
+      <c r="A35" s="23" t="inlineStr">
         <is>
           <t>PV of terminal value</t>
         </is>
@@ -6470,12 +6504,12 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="25" t="inlineStr">
+      <c r="A36" s="23" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="E36" s="27">
+      <c r="E36" s="25">
         <f>E29+E35</f>
         <v/>
       </c>
@@ -6526,26 +6560,26 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="28" t="inlineStr">
+      <c r="A39" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: funded term debt $0. Operating leases $298,724k current + $1,499,717k non-current = $1,798,441k (ASC 842 debt equivalent).</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="28" t="inlineStr">
+      <c r="A40" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: UFCF is pre-interest; rent stays in opex. We subtract lease liabilities in the bridge but do not add back implied lease interest to EBIT (simplified treatment).</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="25" t="inlineStr">
+      <c r="A41" s="23" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
       </c>
-      <c r="E41" s="27">
+      <c r="E41" s="25">
         <f>E36+E37+E38</f>
         <v/>
       </c>
@@ -6571,7 +6605,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="25" t="inlineStr">
+      <c r="A43" s="23" t="inlineStr">
         <is>
           <t>Implied value per share</t>
         </is>
@@ -6606,7 +6640,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="25" t="inlineStr">
+      <c r="A45" s="23" t="inlineStr">
         <is>
           <t>Implied upside / (downside)</t>
         </is>
@@ -6697,18 +6731,18 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="25" t="inlineStr">
+      <c r="A53" s="23" t="inlineStr">
         <is>
           <t>Enterprise value (exit method)</t>
         </is>
       </c>
-      <c r="E53" s="27">
+      <c r="E53" s="25">
         <f>E29+E52</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="25" t="inlineStr">
+      <c r="A54" s="23" t="inlineStr">
         <is>
           <t>Implied value per share (exit method)</t>
         </is>
@@ -6747,7 +6781,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="25" t="inlineStr">
+      <c r="A58" s="23" t="inlineStr">
         <is>
           <t>Terminal value ($)</t>
         </is>
@@ -6766,7 +6800,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="25" t="inlineStr">
+      <c r="A59" s="23" t="inlineStr">
         <is>
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
@@ -6798,7 +6832,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="25" t="inlineStr">
+      <c r="A61" s="23" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
@@ -6830,7 +6864,7 @@
         <f>TEXT(D59,"0.0")&amp;"x spread vs Gordon-implied exit"</f>
         <v/>
       </c>
-      <c r="D62" s="28" t="inlineStr">
+      <c r="D62" s="26" t="inlineStr">
         <is>
           <t>Selected exit is the Gordon identity, so spread should be 0</t>
         </is>
@@ -7131,11 +7165,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId25"/>
     <hyperlink ref="L66" location="'Scenarios'!G10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId26"/>
-    <hyperlink ref="L67" location="'WACC'!E30"/>
-    <hyperlink ref="L68" location="'WACC'!E30"/>
-    <hyperlink ref="L69" location="'WACC'!E30"/>
-    <hyperlink ref="L70" location="'WACC'!E30"/>
-    <hyperlink ref="L71" location="'WACC'!E30"/>
+    <hyperlink ref="L67" location="'WACC'!E32"/>
+    <hyperlink ref="L68" location="'WACC'!E32"/>
+    <hyperlink ref="L69" location="'WACC'!E32"/>
+    <hyperlink ref="L70" location="'WACC'!E32"/>
+    <hyperlink ref="L71" location="'WACC'!E32"/>
     <hyperlink ref="C72" location="'Scenarios'!G9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId27"/>
   </hyperlinks>
@@ -7373,7 +7407,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t>EV/EBITDA is a black formula (I/J). UAA is shown but excluded from averages (negative TTM EBITDA).</t>
         </is>
@@ -7427,7 +7461,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7459,7 +7493,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C20" s="26" t="inlineStr">
+      <c r="C20" s="24" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7491,7 +7525,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C21" s="26" t="inlineStr">
+      <c r="C21" s="24" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7523,7 +7557,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C22" s="26" t="inlineStr">
+      <c r="C22" s="24" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7555,7 +7589,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C23" s="26" t="inlineStr">
+      <c r="C23" s="24" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7587,7 +7621,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C24" s="26" t="inlineStr">
+      <c r="C24" s="24" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7619,7 +7653,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C25" s="26" t="inlineStr">
+      <c r="C25" s="24" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7651,7 +7685,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C26" s="26" t="inlineStr">
+      <c r="C26" s="24" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7683,7 +7717,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C27" s="26" t="inlineStr">
+      <c r="C27" s="24" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7715,7 +7749,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C28" s="26" t="inlineStr">
+      <c r="C28" s="24" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7747,7 +7781,7 @@
           <t>PitchBook Comps Set 04-Sep-2026. Multiple = daily EV / TTM EBITDA. UAA excluded from the mean (negative EBITDA).</t>
         </is>
       </c>
-      <c r="C29" s="26" t="inlineStr">
+      <c r="C29" s="24" t="inlineStr">
         <is>
           <t>PitchBook Comps Set 04-Sep-2026</t>
         </is>
@@ -7776,7 +7810,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="28" t="inlineStr">
+      <c r="A32" s="26" t="inlineStr">
         <is>
           <t>Column E on the next two rows is $bn, not EV/EBITDA. The black formula is implied EV/Sales on an unclosed ask.</t>
         </is>
@@ -7841,7 +7875,7 @@
           <t>Alo implied EV/Sales (ask / parent sales)</t>
         </is>
       </c>
-      <c r="B35" s="28" t="inlineStr">
+      <c r="B35" s="26" t="inlineStr">
         <is>
           <t>5.0x = 10 / 2. Implied EV/Sales on an unclosed ask and parent sales. Not EV/EBITDA. Not the TV.</t>
         </is>
@@ -7867,12 +7901,12 @@
           <t>Alo EV/EBITDA</t>
         </is>
       </c>
-      <c r="B36" s="28" t="inlineStr">
+      <c r="B36" s="26" t="inlineStr">
         <is>
           <t>No page prints Alo or Color Image EBITDA. PitchBook Alo column is blank. Cannot imply EV/EBITDA.</t>
         </is>
       </c>
-      <c r="C36" s="28" t="inlineStr">
+      <c r="C36" s="26" t="inlineStr">
         <is>
           <t>None — no EBITDA source</t>
         </is>
@@ -7901,17 +7935,17 @@
           <t>Core athletic / apparel mean (LULU / NKE / ADS / DECK / CROX / LEVI / KTB)</t>
         </is>
       </c>
-      <c r="B39" s="28" t="inlineStr">
+      <c r="B39" s="26" t="inlineStr">
         <is>
           <t>PitchBook core set, UAA out. Current tape — not a 2.25% g FY30 exit.</t>
         </is>
       </c>
-      <c r="C39" s="28" t="inlineStr">
+      <c r="C39" s="26" t="inlineStr">
         <is>
           <t>Derived: Excel AVERAGE of the seven core prints</t>
         </is>
       </c>
-      <c r="D39" s="28" t="inlineStr">
+      <c r="D39" s="26" t="inlineStr">
         <is>
           <t>Each E cell is I/J from the PitchBook extract. Do not use as FY30 exit.</t>
         </is>
@@ -7927,17 +7961,17 @@
           <t>All positive-EBITDA mean (ex-UAA; includes WSM / MOV / LZB)</t>
         </is>
       </c>
-      <c r="B40" s="28" t="inlineStr">
+      <c r="B40" s="26" t="inlineStr">
         <is>
           <t>Wider PitchBook tape. WSM/MOV/LZB are adjacent retail, not athletic. Not the TV.</t>
         </is>
       </c>
-      <c r="C40" s="28" t="inlineStr">
+      <c r="C40" s="26" t="inlineStr">
         <is>
           <t>Derived: Excel AVERAGE of every positive-EBITDA row</t>
         </is>
       </c>
-      <c r="D40" s="28" t="inlineStr">
+      <c r="D40" s="26" t="inlineStr">
         <is>
           <t>UAA omitted because TTM EBITDA is negative. Not the selected FY30 exit.</t>
         </is>
@@ -8246,7 +8280,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="28" t="inlineStr">
+      <c r="A63" s="26" t="inlineStr">
         <is>
           <t>Note: pubcomps are PitchBook 04-Sep-2026 (EV/EBITDA = daily EV / TTM EBITDA). UAA excluded from the mean. Selected TV is Gordon implied, not the PitchBook average. Alo EV/EBITDA is n.a.</t>
         </is>

</xml_diff>

<commit_message>
WACC beta: unlever at StockAnalysis D/E 0.45, relever at lease D/E
Strip observed βL 0.86 using StockAnalysis total-debt/book-equity
ratio (0.45, $2.14B debt), then relever βu to FY25 lease debt over
market equity for WACC capital structure (~0.73 used β).

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1232,7 +1232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>StockAnalysis Beta (5Y) 0.86 is levered equity βL — the starting point for the unlever / relever chain below.</t>
+          <t>StockAnalysis Beta (5Y) 0.86 is levered equity βL — observed while D/E ≈ 0.45 (total debt incl. leases).</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -1536,227 +1536,280 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>Unlevered βu (Hamada; funded D/E only)</t>
+          <t>D/E for unlever (StockAnalysis; total debt / book equity)</t>
         </is>
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>βu = βL ÷ [1 + (1−T) × funded D/E]. No term loans → funded D/E = 0, so βu = 0.86.</t>
-        </is>
-      </c>
-      <c r="C18" s="24" t="inlineStr">
-        <is>
-          <t>WACC tab: Hamada unlever (funded D/E)</t>
+          <t>StockAnalysis D/E 0.45 = $2.14B total debt ÷ $4.79B book equity — leverage embedded in the 0.86 regression βL.</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>StockAnalysis: LULU Debt / Equity</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>βu = E[βL] ÷ (1 + (1−T) × E[funded debt] ÷ E[market equity]). Funded debt = $0 → βu = 0.86.</t>
-        </is>
-      </c>
-      <c r="E18" s="28">
-        <f>E17/(1+(1-E5)*E13/E10)</f>
-        <v/>
+          <t>Ctrl+F "Debt / Equity" → 0.45 | "Total Debt" → 2.14B (leases; StockAnalysis FY25).</t>
+        </is>
+      </c>
+      <c r="E18" s="27" t="n">
+        <v>0.45</v>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
+          <t>Unlevered βu</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>βu = βL ÷ [1 + (1−T) × D/E]. Strip StockAnalysis 0.45 D/E → βu ≈ 0.65.</t>
+        </is>
+      </c>
+      <c r="C19" s="24" t="inlineStr">
+        <is>
+          <t>WACC tab: Hamada unlever</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>βu = E[βL] ÷ (1 + (1−T) × E[D/E unlever]). With 0.45 D/E → βu ≈ 0.65.</t>
+        </is>
+      </c>
+      <c r="E19" s="28">
+        <f>E17/(1+(1-E5)*E18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>D/E for relever (WACC lease debt / market equity)</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>WACC target D/E = FY25 lease debt equiv. ÷ market equity — real ASC 842 debt for relever step.</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>WACC tab: lease debt / market equity</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>D/E = E[total debt equiv.] ÷ E[market equity]. FY25 10-K leases ÷ $100 × shares.</t>
+        </is>
+      </c>
+      <c r="E20" s="28">
+        <f>E14/E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
           <t>Sector βu benchmark (Damodaran Special Lines) — not used</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>Damodaran unlevered Retail (Special Lines) βu 0.95 shown as a sector benchmark only — not the WACC input.</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>Damodaran: US betas by sector (Jan 2026)</t>
         </is>
       </c>
-      <c r="D19" s="19" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95 (βu). Sector benchmark only — not used in WACC.</t>
         </is>
       </c>
-      <c r="E19" s="27" t="n">
+      <c r="E21" s="27" t="n">
         <v>0.95</v>
       </c>
     </row>
-    <row r="20" ht="150" customHeight="1">
-      <c r="A20" s="23" t="inlineStr">
-        <is>
-          <t>Beta used (relevered for lease debt)</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>βL = βu × [1 + (1−T) × total debt equiv. / E]. Relevers company βu for ASC 842 lease liabilities in WACC.</t>
-        </is>
-      </c>
-      <c r="C20" s="24" t="inlineStr">
+    <row r="22" ht="150" customHeight="1">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>Beta used (relevered for WACC capital structure)</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>βL = βu × [1 + (1−T) × WACC D/E]. Relevers to FY25 lease debt in market-value capital structure.</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
         <is>
           <t>WACC tab: Hamada relever (total D/E incl. leases)</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>Company β: unlever observed βL, then relever for ASC 842 lease debt.
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Company β: unlever at StockAnalysis D/E, relever at WACC lease debt.
 Step 1 — Observed levered βL (StockAnalysis)
   Ctrl+F "Beta (5Y)"  →  0.86
-Step 2 — Unlever (Hamada; funded debt only)
-  βu = βL ÷ [1 + (1−T) × D_funded/E]
-  Funded debt $0 (10-K) → βu = 0.86
-Step 3 — Relever (total debt equiv. incl. leases)
-  βL = βu × [1 + (1−T) × D_total/E]
+Step 2 — D/E embedded in that β (StockAnalysis)
+  Ctrl+F "Debt / Equity"  →  0.45
+  Ctrl+F "Total Debt"  →  2.14B (leases; no term loans)
+Step 3 — Unlever (Hamada)
+  βu = βL ÷ [1 + (1−T) × 0.45]  →  ≈ 0.65
+Step 4 — Relever (WACC real debt / market equity)
+  D/E = FY25 lease debt equiv. ÷ market cap
   Ctrl+F "Current lease liabilities"  →  298,724
   Ctrl+F "Non-current lease liabilities"  →  1,499,717
-  D_total = 1,798,441 ($000) + funded debt $0
+  βL = βu × [1 + (1−T) × D/E]  →  ≈ 0.73
 Sector benchmark (Damodaran) — not used
   Ctrl+F "Retail (Special Lines)"  →  Unlevered beta 0.95</t>
         </is>
       </c>
-      <c r="E20" s="29">
-        <f>E18*(1+(1-E5)*E14/E10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  memo: βu strips funded debt only (none). βL relevers for ASC 842 leases. βL = βu × (1 + (1−T) × D/E).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+      <c r="E22" s="29">
+        <f>E19*(1+(1-E5)*E20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  memo: Unlever strips StockAnalysis 0.45 D/E ($2.14B debt). Relever uses FY25 10-K lease debt / market cap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>Cost of equity (CAPM)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="23" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>Cost of equity = rf + β × ERP</t>
         </is>
       </c>
-      <c r="E23" s="30">
-        <f>E3+E20*E4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="14" t="inlineStr">
+      <c r="E25" s="30">
+        <f>E3+E22*E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>Cost of debt (lease-equivalent)</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="16" t="inlineStr">
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>Pre-tax cost of debt (lease-equivalent)</t>
         </is>
       </c>
-      <c r="B26" s="17" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>5.0% pre-tax lease-equivalent borrowing cost; cheaper than equity. No funded revolver borrowings per FY25 10-K.</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C28" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: lease liabilities &amp; no funded debt</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
+      <c r="D28" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Current lease liabilities" + "Non-current lease liabilities" → debt equiv. 5.0% illustrative lease borrowing cost.</t>
         </is>
       </c>
-      <c r="E26" s="20" t="n">
+      <c r="E28" s="20" t="n">
         <v>0.05</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="E27" s="31">
-        <f>E26*(1-E5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="E29" s="31">
+        <f>E28*(1-E5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>WACC weights</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="16" t="inlineStr">
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>Equity weight</t>
         </is>
       </c>
-      <c r="B30" s="17" t="inlineStr">
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>Equity weight = market cap ÷ (market cap + lease debt). ~86% at $100 and FY25 lease balance.</t>
         </is>
       </c>
-      <c r="C30" s="24" t="inlineStr">
+      <c r="C32" s="24" t="inlineStr">
         <is>
           <t>WACC tab: capital structure</t>
         </is>
       </c>
-      <c r="D30" s="19" t="inlineStr">
+      <c r="D32" s="19" t="inlineStr">
         <is>
           <t>Equity weight = market cap ÷ (market cap + lease debt). Live formula on this tab.</t>
         </is>
       </c>
-      <c r="E30" s="32">
+      <c r="E32" s="32">
         <f>E10/(E10+E14)</f>
         <v/>
       </c>
     </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="16" t="inlineStr">
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>Debt weight (leases + funded)</t>
         </is>
       </c>
-      <c r="B31" s="17" t="inlineStr">
+      <c r="B33" s="17" t="inlineStr">
         <is>
           <t>Debt weight = lease liabilities ÷ (market cap + lease debt). ~14% — ASC 842 leases, not bank debt.</t>
         </is>
       </c>
-      <c r="C31" s="18" t="inlineStr">
+      <c r="C33" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: operating lease liabilities</t>
         </is>
       </c>
-      <c r="D31" s="19" t="inlineStr">
+      <c r="D33" s="19" t="inlineStr">
         <is>
           <t>Debt weight = lease liabilities ÷ (market cap + lease debt). ~14% at FY25 balances.</t>
         </is>
       </c>
-      <c r="E31" s="32">
+      <c r="E33" s="32">
         <f>E14/(E10+E14)</f>
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="23" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="23" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="E32" s="33">
-        <f>E30*E23+E31*E27</f>
+      <c r="E34" s="33">
+        <f>E32*E25+E33*E29</f>
         <v/>
       </c>
     </row>
@@ -1770,9 +1823,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2029,7 +2083,7 @@
         <v>0.11</v>
       </c>
       <c r="G9" s="32">
-        <f>WACC!E32</f>
+        <f>WACC!E34</f>
         <v/>
       </c>
       <c r="H9" s="20" t="n">
@@ -3168,7 +3222,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
-    <hyperlink ref="C9" location="'WACC'!E32"/>
+    <hyperlink ref="C9" location="'WACC'!E34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
@@ -7165,11 +7219,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId25"/>
     <hyperlink ref="L66" location="'Scenarios'!G10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId26"/>
-    <hyperlink ref="L67" location="'WACC'!E32"/>
-    <hyperlink ref="L68" location="'WACC'!E32"/>
-    <hyperlink ref="L69" location="'WACC'!E32"/>
-    <hyperlink ref="L70" location="'WACC'!E32"/>
-    <hyperlink ref="L71" location="'WACC'!E32"/>
+    <hyperlink ref="L67" location="'WACC'!E34"/>
+    <hyperlink ref="L68" location="'WACC'!E34"/>
+    <hyperlink ref="L69" location="'WACC'!E34"/>
+    <hyperlink ref="L70" location="'WACC'!E34"/>
+    <hyperlink ref="L71" location="'WACC'!E34"/>
     <hyperlink ref="C72" location="'Scenarios'!G9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId27"/>
   </hyperlinks>

</xml_diff>

<commit_message>
WACC beta: same lease D/E for unlever and relever (10-K debt)
Use FY25 lease debt / market equity for both Hamada steps so β
strips and re-applies our capital structure. β used = 0.86; keep
StockAnalysis 0.45 book D/E as reference only.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1516,7 +1516,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>StockAnalysis Beta (5Y) 0.86 is levered equity βL — observed while D/E ≈ 0.45 (total debt incl. leases).</t>
+          <t>StockAnalysis Beta (5Y) 0.86 is levered equity βL — strip WACC D/E, then relever to the same lease-debt capital structure.</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -1536,26 +1536,27 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>D/E for unlever (StockAnalysis; total debt / book equity)</t>
+          <t>D/E (lease debt / market equity)</t>
         </is>
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>StockAnalysis D/E 0.45 = $2.14B total debt ÷ $4.79B book equity — leverage embedded in the 0.86 regression βL.</t>
-        </is>
-      </c>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>StockAnalysis: LULU Debt / Equity</t>
+          <t>D/E = FY25 lease debt equiv. ÷ market equity (~0.16). Same ratio for unlever and relever — our 10-K debt numbers.</t>
+        </is>
+      </c>
+      <c r="C18" s="24" t="inlineStr">
+        <is>
+          <t>WACC tab: lease debt / market equity</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Debt / Equity" → 0.45 | "Total Debt" → 2.14B (leases; StockAnalysis FY25).</t>
-        </is>
-      </c>
-      <c r="E18" s="27" t="n">
-        <v>0.45</v>
+          <t>D/E = E[total debt equiv.] ÷ E[market equity]. FY25 10-K leases ($1,798,441k) ÷ market cap.</t>
+        </is>
+      </c>
+      <c r="E18" s="28">
+        <f>E14/E10</f>
+        <v/>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
@@ -1566,7 +1567,7 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>βu = βL ÷ [1 + (1−T) × D/E]. Strip StockAnalysis 0.45 D/E → βu ≈ 0.65.</t>
+          <t>βu = βL ÷ [1 + (1−T) × D/E]. Strips lease leverage embedded in the 0.86 regression using WACC D/E.</t>
         </is>
       </c>
       <c r="C19" s="24" t="inlineStr">
@@ -1576,7 +1577,7 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>βu = E[βL] ÷ (1 + (1−T) × E[D/E unlever]). With 0.45 D/E → βu ≈ 0.65.</t>
+          <t>βu = E[βL] ÷ (1 + (1−T) × E[D/E]). Same D/E as relever row.</t>
         </is>
       </c>
       <c r="E19" s="28">
@@ -1587,52 +1588,51 @@
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>D/E for relever (WACC lease debt / market equity)</t>
+          <t>Sector βu benchmark (Damodaran Special Lines) — not used</t>
         </is>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>WACC target D/E = FY25 lease debt equiv. ÷ market equity — real ASC 842 debt for relever step.</t>
-        </is>
-      </c>
-      <c r="C20" s="24" t="inlineStr">
-        <is>
-          <t>WACC tab: lease debt / market equity</t>
+          <t>Damodaran unlevered Retail (Special Lines) βu 0.95 shown as a sector benchmark only — not the WACC input.</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Damodaran: US betas by sector (Jan 2026)</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>D/E = E[total debt equiv.] ÷ E[market equity]. FY25 10-K leases ÷ $100 × shares.</t>
-        </is>
-      </c>
-      <c r="E20" s="28">
-        <f>E14/E10</f>
-        <v/>
+          <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95 (βu). Sector benchmark only — not used in WACC.</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="n">
+        <v>0.95</v>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>Sector βu benchmark (Damodaran Special Lines) — not used</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="inlineStr">
-        <is>
-          <t>Damodaran unlevered Retail (Special Lines) βu 0.95 shown as a sector benchmark only — not the WACC input.</t>
+          <t>StockAnalysis D/E (book; reference only)</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>StockAnalysis 0.45 D/E is book debt / book equity ($2.14B / $4.79B). Shown for reference; Hamada uses market D/E above.</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>Damodaran: US betas by sector (Jan 2026)</t>
+          <t>StockAnalysis: LULU statistics</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95 (βu). Sector benchmark only — not used in WACC.</t>
+          <t>Ctrl+F "Debt / Equity" → 0.45 | "Total Debt" → 2.14B. Reference only — not used in unlever formula.</t>
         </is>
       </c>
       <c r="E21" s="27" t="n">
-        <v>0.95</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="22" ht="150" customHeight="1">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>βL = βu × [1 + (1−T) × WACC D/E]. Relevers to FY25 lease debt in market-value capital structure.</t>
+          <t>βL = βu × [1 + (1−T) × D/E]. Relevers to the same FY25 lease debt / market equity. β used = 0.86 when D/E matches.</t>
         </is>
       </c>
       <c r="C22" s="24" t="inlineStr">
@@ -1653,32 +1653,32 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Company β: unlever at StockAnalysis D/E, relever at WACC lease debt.
-Step 1 — Observed levered βL (StockAnalysis)
+          <t>Company β: unlever then relever using WACC lease debt / market equity.
+Observed levered βL (StockAnalysis)
   Ctrl+F "Beta (5Y)"  →  0.86
-Step 2 — D/E embedded in that β (StockAnalysis)
-  Ctrl+F "Debt / Equity"  →  0.45
-  Ctrl+F "Total Debt"  →  2.14B (leases; no term loans)
-Step 3 — Unlever (Hamada)
-  βu = βL ÷ [1 + (1−T) × 0.45]  →  ≈ 0.65
-Step 4 — Relever (WACC real debt / market equity)
-  D/E = FY25 lease debt equiv. ÷ market cap
+D/E (same for unlever and relever)
+  = total debt equiv. ÷ market equity
   Ctrl+F "Current lease liabilities"  →  298,724
   Ctrl+F "Non-current lease liabilities"  →  1,499,717
-  βL = βu × [1 + (1−T) × D/E]  →  ≈ 0.73
+  Sum = 1,798,441 ($000) ÷ market cap
+Unlever:  βu = βL ÷ [1 + (1−T) × D/E]
+Relever:  βL = βu × [1 + (1−T) × D/E]
+Same D/E both steps → β used = 0.86
+StockAnalysis D/E 0.45 (book) — reference only, not used here
+  Ctrl+F "Debt / Equity"  →  0.45 | "Total Debt"  →  2.14B
 Sector benchmark (Damodaran) — not used
   Ctrl+F "Retail (Special Lines)"  →  Unlevered beta 0.95</t>
         </is>
       </c>
       <c r="E22" s="29">
-        <f>E19*(1+(1-E5)*E20)</f>
+        <f>E19*(1+(1-E5)*E18)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: Unlever strips StockAnalysis 0.45 D/E ($2.14B debt). Relever uses FY25 10-K lease debt / market cap.</t>
+          <t xml:space="preserve">  memo: Unlever and relever use the same D/E (FY25 lease debt ÷ market cap). β used = observed 0.86 when capital structure is unchanged.</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId12"/>

</xml_diff>

<commit_message>
WACC beta: unlever at StockAnalysis source D/E, relever at WACC D/E
Unlever βL 0.86 using StockAnalysis 0.45 D/E ($2.14B debt on same
page as beta). Relever βu to FY25 10-K lease debt / market equity.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1516,7 +1516,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>StockAnalysis Beta (5Y) 0.86 is levered equity βL — strip WACC D/E, then relever to the same lease-debt capital structure.</t>
+          <t>StockAnalysis Beta (5Y) 0.86 is levered equity βL — observed alongside D/E 0.45 and $2.14B total debt on the same page.</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -1536,27 +1536,26 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>D/E (lease debt / market equity)</t>
+          <t>D/E for unlever (StockAnalysis; source of βL)</t>
         </is>
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>D/E = FY25 lease debt equiv. ÷ market equity (~0.16). Same ratio for unlever and relever — our 10-K debt numbers.</t>
-        </is>
-      </c>
-      <c r="C18" s="24" t="inlineStr">
-        <is>
-          <t>WACC tab: lease debt / market equity</t>
+          <t>Unlever D/E = StockAnalysis 0.45 ($2.14B total debt ÷ $4.79B book equity) — leverage embedded in the source βL.</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>StockAnalysis: LULU Debt / Equity</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>D/E = E[total debt equiv.] ÷ E[market equity]. FY25 10-K leases ($1,798,441k) ÷ market cap.</t>
-        </is>
-      </c>
-      <c r="E18" s="28">
-        <f>E14/E10</f>
-        <v/>
+          <t>Ctrl+F "Debt / Equity" → 0.45 | "Total Debt" → 2.14B. Source D/E for unlever step.</t>
+        </is>
+      </c>
+      <c r="E18" s="27" t="n">
+        <v>0.45</v>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
@@ -1567,17 +1566,17 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>βu = βL ÷ [1 + (1−T) × D/E]. Strips lease leverage embedded in the 0.86 regression using WACC D/E.</t>
+          <t>βu = βL ÷ [1 + (1−T) × D/E_source]. Strip StockAnalysis 0.45 D/E → βu ≈ 0.65.</t>
         </is>
       </c>
       <c r="C19" s="24" t="inlineStr">
         <is>
-          <t>WACC tab: Hamada unlever</t>
+          <t>WACC tab: Hamada unlever (source D/E)</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>βu = E[βL] ÷ (1 + (1−T) × E[D/E]). Same D/E as relever row.</t>
+          <t>βu = E[βL] ÷ (1 + (1−T) × E[D/E source]). With StockAnalysis 0.45 → βu ≈ 0.65.</t>
         </is>
       </c>
       <c r="E19" s="28">
@@ -1588,51 +1587,52 @@
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>Sector βu benchmark (Damodaran Special Lines) — not used</t>
+          <t>D/E for relever (WACC: FY25 lease debt / market equity)</t>
         </is>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Damodaran unlevered Retail (Special Lines) βu 0.95 shown as a sector benchmark only — not the WACC input.</t>
-        </is>
-      </c>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>Damodaran: US betas by sector (Jan 2026)</t>
+          <t>Relever D/E = FY25 10-K lease debt equiv. ÷ market equity — WACC capital structure we model.</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>WACC tab: FY25 lease debt / market equity</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95 (βu). Sector benchmark only — not used in WACC.</t>
-        </is>
-      </c>
-      <c r="E20" s="27" t="n">
-        <v>0.95</v>
+          <t>D/E = E[total debt equiv.] ÷ E[market equity]. FY25 10-K leases ÷ market cap for relever.</t>
+        </is>
+      </c>
+      <c r="E20" s="28">
+        <f>E14/E10</f>
+        <v/>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>StockAnalysis D/E (book; reference only)</t>
-        </is>
-      </c>
-      <c r="B21" s="26" t="inlineStr">
-        <is>
-          <t>StockAnalysis 0.45 D/E is book debt / book equity ($2.14B / $4.79B). Shown for reference; Hamada uses market D/E above.</t>
+          <t>Sector βu benchmark (Damodaran Special Lines) — not used</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Damodaran unlevered Retail (Special Lines) βu 0.95 shown as a sector benchmark only — not the WACC input.</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>StockAnalysis: LULU statistics</t>
+          <t>Damodaran: US betas by sector (Jan 2026)</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Debt / Equity" → 0.45 | "Total Debt" → 2.14B. Reference only — not used in unlever formula.</t>
+          <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95 (βu). Sector benchmark only — not used in WACC.</t>
         </is>
       </c>
       <c r="E21" s="27" t="n">
-        <v>0.45</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="22" ht="150" customHeight="1">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>βL = βu × [1 + (1−T) × D/E]. Relevers to the same FY25 lease debt / market equity. β used = 0.86 when D/E matches.</t>
+          <t>βL = βu × [1 + (1−T) × D/E_WACC]. Relevers to FY25 lease debt / market cap (~0.73 used β).</t>
         </is>
       </c>
       <c r="C22" s="24" t="inlineStr">
@@ -1653,32 +1653,31 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Company β: unlever then relever using WACC lease debt / market equity.
-Observed levered βL (StockAnalysis)
+          <t>Unlever at source D/E (StockAnalysis) → relever at WACC D/E (10-K leases).
+Observed levered βL (same source as D/E below)
   Ctrl+F "Beta (5Y)"  →  0.86
-D/E (same for unlever and relever)
-  = total debt equiv. ÷ market equity
+Step 1 — Unlever (source leverage)
+  Ctrl+F "Debt / Equity"  →  0.45
+  Ctrl+F "Total Debt"  →  2.14B (leases on StockAnalysis)
+  βu = 0.86 ÷ [1 + (1−T) × 0.45]  →  ≈ 0.65
+Step 2 — Relever (WACC capital structure)
+  D/E = FY25 lease debt equiv. ÷ market equity
   Ctrl+F "Current lease liabilities"  →  298,724
   Ctrl+F "Non-current lease liabilities"  →  1,499,717
-  Sum = 1,798,441 ($000) ÷ market cap
-Unlever:  βu = βL ÷ [1 + (1−T) × D/E]
-Relever:  βL = βu × [1 + (1−T) × D/E]
-Same D/E both steps → β used = 0.86
-StockAnalysis D/E 0.45 (book) — reference only, not used here
-  Ctrl+F "Debt / Equity"  →  0.45 | "Total Debt"  →  2.14B
+  βL = βu × [1 + (1−T) × D/E]  →  ≈ 0.73
 Sector benchmark (Damodaran) — not used
   Ctrl+F "Retail (Special Lines)"  →  Unlevered beta 0.95</t>
         </is>
       </c>
       <c r="E22" s="29">
-        <f>E19*(1+(1-E5)*E18)</f>
+        <f>E19*(1+(1-E5)*E20)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: Unlever and relever use the same D/E (FY25 lease debt ÷ market cap). β used = observed 0.86 when capital structure is unchanged.</t>
+          <t xml:space="preserve">  memo: Unlever strips StockAnalysis 0.45 D/E ($2.14B debt). Relever applies FY25 10-K lease debt / market cap.</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1822,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId12"/>

</xml_diff>

<commit_message>
Expand WACC beta walkthrough: 0.86 unlever at source D/E, relever at WACC
Step-by-step justifications, Ctrl+F block, and memo lines explaining
Hamada (1-T)=0.70, StockAnalysis D/E 0.45, and FY25 lease relever.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1232,7 +1232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>30% cash tax matches FY2026 guidance (“approximately 30%”); FY25 effective was 29.5%.</t>
+          <t>30% cash tax matches FY2026 guidance (“approximately 30%”). Also sets (1−T) = 0.70 in the Hamada β unlever/relever formulas.</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>StockAnalysis Beta (5Y) 0.86 is levered equity βL — observed alongside D/E 0.45 and $2.14B total debt on the same page.</t>
+          <t>Step 0: StockAnalysis Beta (5Y) = 0.86. This is levered equity βL from a 5-year regression vs the market — not unlevered.</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Beta (5Y)" → 0.86. Levered equity βL (StockAnalysis).</t>
+          <t>Ctrl+F "Beta (5Y)" → 0.86. Levered equity βL — starting point (StockAnalysis).</t>
         </is>
       </c>
       <c r="E17" s="27" t="n">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>Unlever D/E = StockAnalysis 0.45 ($2.14B total debt ÷ $4.79B book equity) — leverage embedded in the source βL.</t>
+          <t>Step 1a: Source D/E = 0.45 on StockAnalysis ($2.14B total debt ÷ $4.79B book equity) — the leverage paired with βL on that page.</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Debt / Equity" → 0.45 | "Total Debt" → 2.14B. Source D/E for unlever step.</t>
+          <t>Ctrl+F "Debt / Equity" → 0.45. = $2.14B total debt ÷ $4.79B book equity (source page).</t>
         </is>
       </c>
       <c r="E18" s="27" t="n">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>βu = βL ÷ [1 + (1−T) × D/E_source]. Strip StockAnalysis 0.45 D/E → βu ≈ 0.65.</t>
+          <t>Step 1b: βu = 0.86 ÷ [1 + (1−T)×0.45]. With T=30% → (1−T)=0.70. Denominator = 1.315 → βu ≈ 0.65 (pure business risk).</t>
         </is>
       </c>
       <c r="C19" s="24" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>βu = E[βL] ÷ (1 + (1−T) × E[D/E source]). With StockAnalysis 0.45 → βu ≈ 0.65.</t>
+          <t>Formula: βu = βL ÷ [1 + (1−T) × D/E]. (1−T) = 0.70 at 30% tax. 0.86 ÷ 1.315 ≈ 0.65.</t>
         </is>
       </c>
       <c r="E19" s="28">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Relever D/E = FY25 10-K lease debt equiv. ÷ market equity — WACC capital structure we model.</t>
+          <t>Step 2a: WACC D/E = FY25 lease debt ($1,798,441k) ÷ market cap ($100 × 111,380k shares) ≈ 0.16 — our modeled capital structure.</t>
         </is>
       </c>
       <c r="C20" s="24" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>D/E = E[total debt equiv.] ÷ E[market equity]. FY25 10-K leases ÷ market cap for relever.</t>
+          <t>Formula: D/E = E[lease debt] ÷ E[market equity]. 1,798,441 ÷ 11,138,000 ≈ 0.16 (10-K + NASDAQ).</t>
         </is>
       </c>
       <c r="E20" s="28">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>Damodaran unlevered Retail (Special Lines) βu 0.95 shown as a sector benchmark only — not the WACC input.</t>
+          <t>Benchmark only: Damodaran unlevered Retail (Special Lines) βu = 0.95. Not used — we derive βu from company βL instead.</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Retail (Special Lines)" → Unlevered beta 0.95 (βu). Sector benchmark only — not used in WACC.</t>
+          <t>Ctrl+F "Retail (Special Lines)" → 0.95 βu. Sector benchmark — not used in WACC.</t>
         </is>
       </c>
       <c r="E21" s="27" t="n">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>βL = βu × [1 + (1−T) × D/E_WACC]. Relevers to FY25 lease debt / market cap (~0.73 used β).</t>
+          <t>Step 2b: β used = 0.65 × [1 + 0.70×0.16] ≈ 0.73. This relevered βL feeds CAPM: CoE = rf + β×ERP.</t>
         </is>
       </c>
       <c r="C22" s="24" t="inlineStr">
@@ -1653,20 +1653,26 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Unlever at source D/E (StockAnalysis) → relever at WACC D/E (10-K leases).
-Observed levered βL (same source as D/E below)
+          <t>HOW WE GET β USED IN WACC (Hamada)
+STEP 0 — Start with observed levered βL (StockAnalysis)
   Ctrl+F "Beta (5Y)"  →  0.86
-Step 1 — Unlever (source leverage)
-  Ctrl+F "Debt / Equity"  →  0.45
-  Ctrl+F "Total Debt"  →  2.14B (leases on StockAnalysis)
-  βu = 0.86 ÷ [1 + (1−T) × 0.45]  →  ≈ 0.65
-Step 2 — Relever (WACC capital structure)
-  D/E = FY25 lease debt equiv. ÷ market equity
+  5-year regression vs market. Already includes equity risk at source leverage.
+STEP 1 — UNLEVER at source D/E (strip leverage from βL)
+  Ctrl+F "Debt / Equity"  →  0.45  (= $2.14B debt ÷ $4.79B book equity)
+  Ctrl+F "Total Debt"  →  2.14B
+  Formula:  βu = βL ÷ [1 + (1−T) × D/E]
+  (1−T) = 0.70  because tax rate T = 30% on this tab
+  0.45 = source D/E from StockAnalysis (same page as βL)
+  βu = 0.86 ÷ [1 + 0.70 × 0.45] = 0.86 ÷ 1.315  ≈  0.65
+STEP 2 — RELEVER at WACC D/E (our modeled lease debt)
+  D/E = FY25 lease debt equiv. ÷ market equity (rows above)
   Ctrl+F "Current lease liabilities"  →  298,724
   Ctrl+F "Non-current lease liabilities"  →  1,499,717
-  βL = βu × [1 + (1−T) × D/E]  →  ≈ 0.73
-Sector benchmark (Damodaran) — not used
-  Ctrl+F "Retail (Special Lines)"  →  Unlevered beta 0.95</t>
+  Sum = 1,798,441 ($000). Market cap = $100 × 111,380k shares.
+  D/E ≈ 0.16.  Formula:  β used = βu × [1 + 0.70 × D/E]
+  β used = 0.65 × [1 + 0.70 × 0.16]  ≈  0.73  →  CoE = rf + β × ERP
+Benchmark (not used): Damodaran Retail βu 0.95
+  Ctrl+F "Retail (Special Lines)"  →  0.95</t>
         </is>
       </c>
       <c r="E22" s="29">
@@ -1677,138 +1683,159 @@
     <row r="23">
       <c r="A23" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  memo: Unlever strips StockAnalysis 0.45 D/E ($2.14B debt). Relever applies FY25 10-K lease debt / market cap.</t>
+          <t xml:space="preserve">  β walkthrough (Hamada):</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>Cost of equity (CAPM)</t>
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (0) StockAnalysis βL = 0.86 (levered; 5Y regression vs market).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="inlineStr">
-        <is>
-          <t>Cost of equity = rf + β × ERP</t>
-        </is>
-      </c>
-      <c r="E25" s="30">
-        <f>E3+E22*E4</f>
-        <v/>
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (1) Unlever at source D/E = 0.45 [(1−T)=0.70 at 30% tax] → βu = 0.86 ÷ 1.315 ≈ 0.65.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (2) Relever at WACC D/E = FY25 lease debt ÷ market cap ≈ 0.16 → β used ≈ 0.73 in CAPM below.</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
+          <t>Cost of equity (CAPM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>Cost of equity = rf + β × ERP</t>
+        </is>
+      </c>
+      <c r="E28" s="30">
+        <f>E3+E22*E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
           <t>Cost of debt (lease-equivalent)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="16" t="inlineStr">
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>Pre-tax cost of debt (lease-equivalent)</t>
         </is>
       </c>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>5.0% pre-tax lease-equivalent borrowing cost; cheaper than equity. No funded revolver borrowings per FY25 10-K.</t>
         </is>
       </c>
-      <c r="C28" s="18" t="inlineStr">
+      <c r="C31" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: lease liabilities &amp; no funded debt</t>
         </is>
       </c>
-      <c r="D28" s="19" t="inlineStr">
+      <c r="D31" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Current lease liabilities" + "Non-current lease liabilities" → debt equiv. 5.0% illustrative lease borrowing cost.</t>
         </is>
       </c>
-      <c r="E28" s="20" t="n">
+      <c r="E31" s="20" t="n">
         <v>0.05</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="E29" s="31">
-        <f>E28*(1-E5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="E32" s="31">
+        <f>E31*(1-E5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
         <is>
           <t>WACC weights</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="16" t="inlineStr">
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="16" t="inlineStr">
         <is>
           <t>Equity weight</t>
         </is>
       </c>
-      <c r="B32" s="17" t="inlineStr">
+      <c r="B35" s="17" t="inlineStr">
         <is>
           <t>Equity weight = market cap ÷ (market cap + lease debt). ~86% at $100 and FY25 lease balance.</t>
         </is>
       </c>
-      <c r="C32" s="24" t="inlineStr">
+      <c r="C35" s="24" t="inlineStr">
         <is>
           <t>WACC tab: capital structure</t>
         </is>
       </c>
-      <c r="D32" s="19" t="inlineStr">
+      <c r="D35" s="19" t="inlineStr">
         <is>
           <t>Equity weight = market cap ÷ (market cap + lease debt). Live formula on this tab.</t>
         </is>
       </c>
-      <c r="E32" s="32">
+      <c r="E35" s="32">
         <f>E10/(E10+E14)</f>
         <v/>
       </c>
     </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="16" t="inlineStr">
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>Debt weight (leases + funded)</t>
         </is>
       </c>
-      <c r="B33" s="17" t="inlineStr">
+      <c r="B36" s="17" t="inlineStr">
         <is>
           <t>Debt weight = lease liabilities ÷ (market cap + lease debt). ~14% — ASC 842 leases, not bank debt.</t>
         </is>
       </c>
-      <c r="C33" s="18" t="inlineStr">
+      <c r="C36" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: operating lease liabilities</t>
         </is>
       </c>
-      <c r="D33" s="19" t="inlineStr">
+      <c r="D36" s="19" t="inlineStr">
         <is>
           <t>Debt weight = lease liabilities ÷ (market cap + lease debt). ~14% at FY25 balances.</t>
         </is>
       </c>
-      <c r="E33" s="32">
+      <c r="E36" s="32">
         <f>E14/(E10+E14)</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="23" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="23" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="E34" s="33">
-        <f>E32*E25+E33*E29</f>
+      <c r="E37" s="33">
+        <f>E35*E28+E36*E32</f>
         <v/>
       </c>
     </row>
@@ -1824,8 +1851,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2082,7 +2109,7 @@
         <v>0.11</v>
       </c>
       <c r="G9" s="32">
-        <f>WACC!E34</f>
+        <f>WACC!E37</f>
         <v/>
       </c>
       <c r="H9" s="20" t="n">
@@ -3221,7 +3248,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
-    <hyperlink ref="C9" location="'WACC'!E34"/>
+    <hyperlink ref="C9" location="'WACC'!E37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
@@ -7218,11 +7245,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId25"/>
     <hyperlink ref="L66" location="'Scenarios'!G10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId26"/>
-    <hyperlink ref="L67" location="'WACC'!E34"/>
-    <hyperlink ref="L68" location="'WACC'!E34"/>
-    <hyperlink ref="L69" location="'WACC'!E34"/>
-    <hyperlink ref="L70" location="'WACC'!E34"/>
-    <hyperlink ref="L71" location="'WACC'!E34"/>
+    <hyperlink ref="L67" location="'WACC'!E37"/>
+    <hyperlink ref="L68" location="'WACC'!E37"/>
+    <hyperlink ref="L69" location="'WACC'!E37"/>
+    <hyperlink ref="L70" location="'WACC'!E37"/>
+    <hyperlink ref="L71" location="'WACC'!E37"/>
     <hyperlink ref="C72" location="'Scenarios'!G9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId27"/>
   </hyperlinks>

</xml_diff>

<commit_message>
WACC beta: Yahoo Key Statistics source with paired debt and market cap
Firecrawl verified Yahoo pairs Beta (5Y Monthly) 0.86 with Total
Debt (mrq) $2.14B and Market Cap $11.14B on one page. Unlever
using market D/E (debt÷mkt cap); relever to FY25 lease/WACC D/E.
Book D/E 44.69% kept as reference only.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1232,7 +1232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1511,22 +1511,22 @@
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>Observed Beta (5Y) — levered βL</t>
+          <t>Observed Beta (5Y Monthly) — levered βL</t>
         </is>
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>Step 0: StockAnalysis Beta (5Y) = 0.86. This is levered equity βL from a 5-year regression vs the market — not unlevered.</t>
+          <t>Yahoo Beta (5Y Monthly) = 0.86. Levered equity βL from ~60 monthly returns vs S&amp;P 500 — not unlevered.</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>StockAnalysis: LULU Beta (5Y)</t>
+          <t>Yahoo Finance: LULU Beta (5Y Monthly)</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Beta (5Y)" → 0.86. Levered equity βL — starting point (StockAnalysis).</t>
+          <t>Ctrl+F "Beta (5Y Monthly)" → 0.86. Levered βL (Yahoo Key Statistics).</t>
         </is>
       </c>
       <c r="E17" s="27" t="n">
@@ -1536,306 +1536,387 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>D/E for unlever (StockAnalysis; source of βL)</t>
+          <t>Yahoo Total Debt (mrq)</t>
         </is>
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>Step 1a: Source D/E = 0.45 on StockAnalysis ($2.14B total debt ÷ $4.79B book equity) — the leverage paired with βL on that page.</t>
+          <t>Yahoo Total Debt (mrq) = $2.14B on the same Key Statistics page as βL. Most recent quarter balance sheet.</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>StockAnalysis: LULU Debt / Equity</t>
+          <t>Yahoo Finance: LULU Total Debt (mrq)</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Debt / Equity" → 0.45. = $2.14B total debt ÷ $4.79B book equity (source page).</t>
-        </is>
-      </c>
-      <c r="E18" s="27" t="n">
-        <v>0.45</v>
+          <t>Ctrl+F "Total Debt (mrq)" → 2.14B. Same page as beta.</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="n">
+        <v>2140000</v>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>Unlevered βu</t>
+          <t>Yahoo Market Cap (same page as βL)</t>
         </is>
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>Step 1b: βu = 0.86 ÷ [1 + (1−T)×0.45]. With T=30% → (1−T)=0.70. Denominator = 1.315 → βu ≈ 0.65 (pure business risk).</t>
-        </is>
-      </c>
-      <c r="C19" s="24" t="inlineStr">
-        <is>
-          <t>WACC tab: Hamada unlever (source D/E)</t>
+          <t>Yahoo Market Cap = $11.14B on the same page as βL and Total Debt (mrq). Market value of equity.</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Yahoo Finance: LULU Market Cap</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Formula: βu = βL ÷ [1 + (1−T) × D/E]. (1−T) = 0.70 at 30% tax. 0.86 ÷ 1.315 ≈ 0.65.</t>
-        </is>
-      </c>
-      <c r="E19" s="28">
-        <f>E17/(1+(1-E5)*E18)</f>
-        <v/>
+          <t>Ctrl+F "Market Cap" → 11.14B. Same page as beta and debt.</t>
+        </is>
+      </c>
+      <c r="E19" s="22" t="n">
+        <v>11140000</v>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>D/E for relever (WACC: FY25 lease debt / market equity)</t>
+          <t>D/E for unlever (Yahoo debt mrq ÷ Yahoo market cap)</t>
         </is>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Step 2a: WACC D/E = FY25 lease debt ($1,798,441k) ÷ market cap ($100 × 111,380k shares) ≈ 0.16 — our modeled capital structure.</t>
-        </is>
-      </c>
-      <c r="C20" s="24" t="inlineStr">
-        <is>
-          <t>WACC tab: FY25 lease debt / market equity</t>
+          <t>Unlever D/E = Yahoo debt (mrq) ÷ Yahoo market cap ≈ 0.19. Market-value D/E from the beta source page (Hamada convention).</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Yahoo Finance: debt (mrq) ÷ market cap</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Formula: D/E = E[lease debt] ÷ E[market equity]. 1,798,441 ÷ 11,138,000 ≈ 0.16 (10-K + NASDAQ).</t>
+          <t>Formula: D/E = E[Yahoo debt mrq] ÷ E[Yahoo market cap]. 2.14B ÷ 11.14B ≈ 0.19.</t>
         </is>
       </c>
       <c r="E20" s="28">
-        <f>E14/E10</f>
+        <f>E18/E19</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
+          <t>Yahoo book D/E (mrq) — reference only</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Yahoo Total Debt/Equity (mrq) = 44.69% is book D/E on the same page — shown for reference, not used in Hamada.</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Yahoo Finance: Total Debt/Equity (mrq)</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Total Debt/Equity (mrq)" → 44.69%. Book D/E — reference only, not in Hamada.</t>
+        </is>
+      </c>
+      <c r="E21" s="27" t="n">
+        <v>0.4469</v>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>Unlevered βu</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>βu = 0.86 ÷ [1 + 0.70 × 0.19]. Strip Yahoo market D/E from βL → βu ≈ 0.76. No vendor publishes D/E inside the regression.</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>WACC tab: Hamada unlever (Yahoo market D/E)</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>βu = E[βL] ÷ (1 + 0.70 × E[D/E Yahoo]). 0.86 ÷ 1.134 ≈ 0.76. Regression does not publish embedded D/E.</t>
+        </is>
+      </c>
+      <c r="E22" s="28">
+        <f>E17/(1+(1-E5)*E20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>D/E for relever (WACC: FY25 lease debt / market equity)</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>Relever D/E = FY25 10-K lease debt ÷ our market cap ≈ 0.16 — WACC capital structure we model.</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>WACC tab: FY25 lease debt / market equity</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>D/E = E[FY25 lease debt] ÷ E[market cap]. 1,798,441 ÷ 11,138,000 ≈ 0.16 (10-K + model).</t>
+        </is>
+      </c>
+      <c r="E23" s="28">
+        <f>E14/E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
           <t>Sector βu benchmark (Damodaran Special Lines) — not used</t>
         </is>
       </c>
-      <c r="B21" s="17" t="inlineStr">
-        <is>
-          <t>Benchmark only: Damodaran unlevered Retail (Special Lines) βu = 0.95. Not used — we derive βu from company βL instead.</t>
-        </is>
-      </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>Benchmark only: Damodaran unlevered Retail (Special Lines) βu = 0.95. Not used — we derive βu from Yahoo βL.</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
         <is>
           <t>Damodaran: US betas by sector (Jan 2026)</t>
         </is>
       </c>
-      <c r="D21" s="19" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Retail (Special Lines)" → 0.95 βu. Sector benchmark — not used in WACC.</t>
         </is>
       </c>
-      <c r="E21" s="27" t="n">
+      <c r="E24" s="27" t="n">
         <v>0.95</v>
       </c>
     </row>
-    <row r="22" ht="150" customHeight="1">
-      <c r="A22" s="23" t="inlineStr">
+    <row r="25" ht="150" customHeight="1">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>Beta used (relevered for WACC capital structure)</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
-        <is>
-          <t>Step 2b: β used = 0.65 × [1 + 0.70×0.16] ≈ 0.73. This relevered βL feeds CAPM: CoE = rf + β×ERP.</t>
-        </is>
-      </c>
-      <c r="C22" s="24" t="inlineStr">
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>β used = βu × [1 + 0.70 × WACC D/E] ≈ 0.84. Relevered βL feeds CAPM: CoE = rf + β×ERP.</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr">
         <is>
           <t>WACC tab: Hamada relever (total D/E incl. leases)</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>HOW WE GET β USED IN WACC (Hamada)
-STEP 0 — Start with observed levered βL (StockAnalysis)
-  Ctrl+F "Beta (5Y)"  →  0.86
-  5-year regression vs market. Already includes equity risk at source leverage.
-STEP 1 — UNLEVER at source D/E (strip leverage from βL)
-  Ctrl+F "Debt / Equity"  →  0.45  (= $2.14B debt ÷ $4.79B book equity)
-  Ctrl+F "Total Debt"  →  2.14B
-  Formula:  βu = βL ÷ [1 + (1−T) × D/E]
-  (1−T) = 0.70  because tax rate T = 30% on this tab
-  0.45 = source D/E from StockAnalysis (same page as βL)
-  βu = 0.86 ÷ [1 + 0.70 × 0.45] = 0.86 ÷ 1.315  ≈  0.65
-STEP 2 — RELEVER at WACC D/E (our modeled lease debt)
-  D/E = FY25 lease debt equiv. ÷ market equity (rows above)
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>YAHOO KEY STATISTICS — βL + debt + equity on ONE page
+(No vendor publishes the D/E embedded inside the regression.)
+Observed levered βL
+  Ctrl+F "Beta (5Y Monthly)"  →  0.86
+  ~60 monthly returns vs S&amp;P 500 (Yahoo label)
+Paired inputs on same page (mrq = most recent quarter)
+  Ctrl+F "Total Debt (mrq)"  →  2.14B
+  Ctrl+F "Market Cap"  →  11.14B
+  Ctrl+F "Total Debt/Equity (mrq)"  →  44.69%  (book; reference only)
+STEP 1 — UNLEVER (market D/E from Yahoo page)
+  D/E = Total Debt (mrq) ÷ Market Cap = 2.14 ÷ 11.14 ≈  0.19
+  βu = 0.86 ÷ [1 + 0.70 × 0.19] = 0.86 ÷ 1.134  ≈  0.76
+  (1−T) = 0.70 at 30% tax on this tab
+STEP 2 — RELEVER (WACC: FY25 10-K lease debt / our market cap)
   Ctrl+F "Current lease liabilities"  →  298,724
   Ctrl+F "Non-current lease liabilities"  →  1,499,717
-  Sum = 1,798,441 ($000). Market cap = $100 × 111,380k shares.
-  D/E ≈ 0.16.  Formula:  β used = βu × [1 + 0.70 × D/E]
-  β used = 0.65 × [1 + 0.70 × 0.16]  ≈  0.73  →  CoE = rf + β × ERP
-Benchmark (not used): Damodaran Retail βu 0.95
-  Ctrl+F "Retail (Special Lines)"  →  0.95</t>
-        </is>
-      </c>
-      <c r="E22" s="29">
-        <f>E19*(1+(1-E5)*E20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  β walkthrough (Hamada):</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  (0) StockAnalysis βL = 0.86 (levered; 5Y regression vs market).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  (1) Unlever at source D/E = 0.45 [(1−T)=0.70 at 30% tax] → βu = 0.86 ÷ 1.315 ≈ 0.65.</t>
-        </is>
+  D/E ≈ 0.16.  β used = 0.76 × 1.113  ≈  0.84
+Benchmark (not used): Damodaran Retail βu 0.95</t>
+        </is>
+      </c>
+      <c r="E25" s="29">
+        <f>E22*(1+(1-E5)*E23)</f>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (2) Relever at WACC D/E = FY25 lease debt ÷ market cap ≈ 0.16 → β used ≈ 0.73 in CAPM below.</t>
+          <t xml:space="preserve">  β walkthrough (Hamada; Yahoo Key Statistics source):</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (0) Yahoo βL = 0.86 (Beta 5Y Monthly). No vendor publishes D/E inside the regression.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (1) Unlever at Yahoo market D/E = $2.14B debt (mrq) ÷ $11.14B mkt cap ≈ 0.19 → βu ≈ 0.76.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (2) Relever at WACC D/E = FY25 10-K leases ÷ our market cap ≈ 0.16 → β used ≈ 0.84.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Book D/E 44.69% on Yahoo page is reference only (not used in formula).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
         <is>
           <t>Cost of equity (CAPM)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="23" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="23" t="inlineStr">
         <is>
           <t>Cost of equity = rf + β × ERP</t>
         </is>
       </c>
-      <c r="E28" s="30">
-        <f>E3+E22*E4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="14" t="inlineStr">
-        <is>
-          <t>Cost of debt (lease-equivalent)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>Pre-tax cost of debt (lease-equivalent)</t>
-        </is>
-      </c>
-      <c r="B31" s="17" t="inlineStr">
-        <is>
-          <t>5.0% pre-tax lease-equivalent borrowing cost; cheaper than equity. No funded revolver borrowings per FY25 10-K.</t>
-        </is>
-      </c>
-      <c r="C31" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K: lease liabilities &amp; no funded debt</t>
-        </is>
-      </c>
-      <c r="D31" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Current lease liabilities" + "Non-current lease liabilities" → debt equiv. 5.0% illustrative lease borrowing cost.</t>
-        </is>
-      </c>
-      <c r="E31" s="20" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t>After-tax cost of debt</t>
-        </is>
-      </c>
-      <c r="E32" s="31">
-        <f>E31*(1-E5)</f>
+      <c r="E32" s="30">
+        <f>E3+E25*E4</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>WACC weights</t>
+          <t>Cost of debt (lease-equivalent)</t>
         </is>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="16" t="inlineStr">
         <is>
+          <t>Pre-tax cost of debt (lease-equivalent)</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>5.0% pre-tax lease-equivalent borrowing cost; cheaper than equity. No funded revolver borrowings per FY25 10-K.</t>
+        </is>
+      </c>
+      <c r="C35" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: lease liabilities &amp; no funded debt</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Current lease liabilities" + "Non-current lease liabilities" → debt equiv. 5.0% illustrative lease borrowing cost.</t>
+        </is>
+      </c>
+      <c r="E35" s="20" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>After-tax cost of debt</t>
+        </is>
+      </c>
+      <c r="E36" s="31">
+        <f>E35*(1-E5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>WACC weights</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
           <t>Equity weight</t>
         </is>
       </c>
-      <c r="B35" s="17" t="inlineStr">
+      <c r="B39" s="17" t="inlineStr">
         <is>
           <t>Equity weight = market cap ÷ (market cap + lease debt). ~86% at $100 and FY25 lease balance.</t>
         </is>
       </c>
-      <c r="C35" s="24" t="inlineStr">
+      <c r="C39" s="24" t="inlineStr">
         <is>
           <t>WACC tab: capital structure</t>
         </is>
       </c>
-      <c r="D35" s="19" t="inlineStr">
+      <c r="D39" s="19" t="inlineStr">
         <is>
           <t>Equity weight = market cap ÷ (market cap + lease debt). Live formula on this tab.</t>
         </is>
       </c>
-      <c r="E35" s="32">
+      <c r="E39" s="32">
         <f>E10/(E10+E14)</f>
         <v/>
       </c>
     </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="16" t="inlineStr">
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>Debt weight (leases + funded)</t>
         </is>
       </c>
-      <c r="B36" s="17" t="inlineStr">
+      <c r="B40" s="17" t="inlineStr">
         <is>
           <t>Debt weight = lease liabilities ÷ (market cap + lease debt). ~14% — ASC 842 leases, not bank debt.</t>
         </is>
       </c>
-      <c r="C36" s="18" t="inlineStr">
+      <c r="C40" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: operating lease liabilities</t>
         </is>
       </c>
-      <c r="D36" s="19" t="inlineStr">
+      <c r="D40" s="19" t="inlineStr">
         <is>
           <t>Debt weight = lease liabilities ÷ (market cap + lease debt). ~14% at FY25 balances.</t>
         </is>
       </c>
-      <c r="E36" s="32">
+      <c r="E40" s="32">
         <f>E14/(E10+E14)</f>
         <v/>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="23" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="23" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
       </c>
-      <c r="E37" s="33">
-        <f>E35*E28+E36*E32</f>
+      <c r="E41" s="33">
+        <f>E39*E32+E40*E36</f>
         <v/>
       </c>
     </row>
@@ -1850,9 +1931,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2109,7 +2193,7 @@
         <v>0.11</v>
       </c>
       <c r="G9" s="32">
-        <f>WACC!E37</f>
+        <f>WACC!E41</f>
         <v/>
       </c>
       <c r="H9" s="20" t="n">
@@ -3248,7 +3332,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
-    <hyperlink ref="C9" location="'WACC'!E37"/>
+    <hyperlink ref="C9" location="'WACC'!E41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId8"/>
@@ -7245,11 +7329,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId25"/>
     <hyperlink ref="L66" location="'Scenarios'!G10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId26"/>
-    <hyperlink ref="L67" location="'WACC'!E37"/>
-    <hyperlink ref="L68" location="'WACC'!E37"/>
-    <hyperlink ref="L69" location="'WACC'!E37"/>
-    <hyperlink ref="L70" location="'WACC'!E37"/>
-    <hyperlink ref="L71" location="'WACC'!E37"/>
+    <hyperlink ref="L67" location="'WACC'!E41"/>
+    <hyperlink ref="L68" location="'WACC'!E41"/>
+    <hyperlink ref="L69" location="'WACC'!E41"/>
+    <hyperlink ref="L70" location="'WACC'!E41"/>
+    <hyperlink ref="L71" location="'WACC'!E41"/>
     <hyperlink ref="C72" location="'Scenarios'!G9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId27"/>
   </hyperlinks>

</xml_diff>

<commit_message>
Fix NWC Ctrl+F docs, add evidence links, collapse DCF WC detail
- Per-driver Ctrl+F strings (DSO/DIO/DPO/prepaid/accrual) no longer overwritten
- Strengthen justifications with FY25 10-K markdown/inventory outlook evidence
- Add sc_dnwc bridge documentation with Scenarios cross-link
- Collapse DCF working-capital detail rows by default; ΔNWC stays visible

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -2349,7 +2349,7 @@
         <v>0.045</v>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
+    <row r="14" ht="112" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Gross margin %</t>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>Gross margin % isolates COGS = Rev × (1 − GM%). FY25 anchor 56.6% = 6,284,132 ÷ 11,102,600 on the 10-K.</t>
+          <t>GM% isolates COGS for inventory/AP drivers. FY25 56.6% = 6,284,132 ÷ 11,102,600; held near reported level in base case.</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
@@ -2367,7 +2367,13 @@
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Gross profit" → 6,284,132 | Ctrl+F "Net revenue" → 11,102,600 | GM = 56.6%. Ctrl+F "Cost of goods sold" → 4,818,468.</t>
+          <t>Ctrl+F "Gross profit"
+→ 6,284,132 ($000)
+Ctrl+F "Net revenue"
+→ 11,102,600 ($000)
+Ctrl+F "Cost of goods sold"
+→ 4,818,468 ($000)
+GM = 6,284,132 ÷ 11,102,600 = 56.6%</t>
         </is>
       </c>
       <c r="F14" s="20" t="n">
@@ -2380,7 +2386,7 @@
         <v>0.575</v>
       </c>
     </row>
-    <row r="15" ht="150" customHeight="1">
+    <row r="15" ht="98" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
           <t>DSO (days) — flat vs FY25</t>
@@ -2388,7 +2394,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>DSO flat at FY25 (AR ÷ Rev) × 365 ≈ 6.3 days. AR balance = (DSO ÷ 365) × projected revenue.</t>
+          <t>DSO flat ~6.3 days: LULU is DTC-heavy (minimal wholesale AR). FY22–FY25 DSO ran 6.0–6.3 days — no structural change assumed.</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
@@ -2398,24 +2404,12 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
-Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
+          <t>Ctrl+F "Accounts receivable, net"
+→ 190,657 ($000)
 Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 11,102,600 ($000)
+DSO = (190,657 ÷ 11,102,600) × 365 ≈ 6.3 days
+Flat: ~6.0–6.3 days FY22–FY25 (DTC model; immaterial wholesale AR).</t>
         </is>
       </c>
       <c r="F15" s="39" t="n">
@@ -2428,7 +2422,7 @@
         <v>6.267883648875038</v>
       </c>
     </row>
-    <row r="16" ht="150" customHeight="1">
+    <row r="16" ht="84" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
           <t>FY25 DIO anchor (days)</t>
@@ -2436,7 +2430,7 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>DIO FY25 anchor ≈ 129 days = (Inventories ÷ COGS) × 365. Declines 1 day/yr (−5 days over FY26–30) to clear excess stock.</t>
+          <t>DIO FY25 ≈129 days anchors on elevated inventory (1,700,753 vs 1,442,081 FY24). Inventory ÷ COGS × 365 on the 10-K balance sheet.</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
@@ -2446,24 +2440,11 @@
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
+          <t>Ctrl+F "Inventories"
+→ 1,700,753 ($000)  |  FY24: 1,442,081
 Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
-Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 4,818,468 ($000)
+DIO = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days</t>
         </is>
       </c>
       <c r="F16" s="39" t="n">
@@ -2476,7 +2457,7 @@
         <v>128.8324100108167</v>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
+    <row r="17" ht="70" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
           <t>DIO decline (days / forecast yr)</t>
@@ -2484,17 +2465,20 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>One day of DIO improvement per forecast year — five days total by FY30 vs the FY25 anchor.</t>
-        </is>
-      </c>
-      <c r="C17" s="24" t="inlineStr">
-        <is>
-          <t>Scenarios: DIO clearance path (−5 days / 5 yrs)</t>
+          <t>−1 DIO day/yr tied to 10-K: unit inventories expected to decrease and markdown % to fall — gradual clearance, not a shock write-down.</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: inventory &amp; markdown outlook</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Model assumption: −1 day DIO per forecast year (−5 days FY26–30 vs FY25 anchor). No 10-K Ctrl+F.</t>
+          <t>Ctrl+F "reduce the percentage of markdowns"
+→ Americas plan to cut promo/markdown intensity
+Ctrl+F "On a unit basis, we expect inventories to slightly decrease"
+Model: −1 DIO day/yr (−5 days FY26–30 vs FY25 anchor)</t>
         </is>
       </c>
       <c r="F17" s="40" t="n">
@@ -2507,7 +2491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" ht="150" customHeight="1">
+    <row r="18" ht="84" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
           <t>DPO (days) — flat vs FY25</t>
@@ -2515,7 +2499,7 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>DPO flat at FY25 (AP ÷ COGS) × 365 ≈ 25.1 days. AP balance = (DPO ÷ 365) × projected COGS.</t>
+          <t>DPO flat ~25 days at FY25 vendor leverage (331,421 ÷ 4,818,468 × 365). AP scales with projected COGS; payment terms unchanged.</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
@@ -2525,24 +2509,11 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
+          <t>Ctrl+F "Accounts payable"
+→ 331,421 ($000)
 Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
-Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 4,818,468 ($000)
+DPO = (331,421 ÷ 4,818,468) × 365 ≈ 25.1 days (held flat)</t>
         </is>
       </c>
       <c r="F18" s="39" t="n">
@@ -2555,7 +2526,7 @@
         <v>25.10521290169407</v>
       </c>
     </row>
-    <row r="19" ht="150" customHeight="1">
+    <row r="19" ht="84" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Prepaid expenses (% of revenue)</t>
@@ -2563,7 +2534,7 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>Prepaid / other current assets held at FY25 % of revenue (564,089 ÷ 11,102,600 ≈ 5.1%).</t>
+          <t>OCA held at FY25 5.1% of revenue — prepaids + income-tax receivables (211,620 + 352,469) are the main non-AR/inventory current assets.</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
@@ -2573,24 +2544,11 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
-Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
-Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+          <t>Ctrl+F "Prepaid expenses and other current assets"
+→ 211,620 ($000)
+Ctrl+F "Prepaid and receivable income taxes"
+→ 352,469 ($000)
+OCA residual (ex-cash/AR/inv) = 564,089 ≈ 5.1% of revenue</t>
         </is>
       </c>
       <c r="F19" s="20" t="n">
@@ -2603,7 +2561,7 @@
         <v>0.05080692810692991</v>
       </c>
     </row>
-    <row r="20" ht="150" customHeight="1">
+    <row r="20" ht="84" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Accrued liabilities (% of revenue)</t>
@@ -2611,7 +2569,7 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Accrued liabilities held at FY25 % of revenue (662,982 ÷ 11,102,600 ≈ 6.0%).</t>
+          <t>Accrued liabilities flat at FY25 6.0% of revenue (662,982 ÷ 11,102,600). Stable comp, marketing, and operating accrual mix.</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
@@ -2621,24 +2579,11 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
-Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
+          <t>Ctrl+F "Accrued liabilities and other"
+→ 662,982 ($000)
 Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 11,102,600 ($000)
+662,982 ÷ 11,102,600 ≈ 6.0% of revenue (held flat)</t>
         </is>
       </c>
       <c r="F20" s="20" t="n">
@@ -4732,9 +4677,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7088,7 +7034,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M85"/>
@@ -7302,7 +7248,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="150" customHeight="1">
+    <row r="7" ht="112" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Gross margin %</t>
@@ -7310,7 +7256,7 @@
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Gross margin % isolates COGS = Rev × (1 − GM%). FY25 anchor 56.6% = 6,284,132 ÷ 11,102,600 on the 10-K.</t>
+          <t>GM% isolates COGS for inventory/AP drivers. FY25 56.6% = 6,284,132 ÷ 11,102,600; held near reported level in base case.</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
@@ -7320,24 +7266,13 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
+          <t>Ctrl+F "Gross profit"
+→ 6,284,132 ($000)
+Ctrl+F "Net revenue"
+→ 11,102,600 ($000)
 Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
-Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 4,818,468 ($000)
+GM = 6,284,132 ÷ 11,102,600 = 56.6%</t>
         </is>
       </c>
       <c r="E7" s="81" t="n">
@@ -7772,11 +7707,11 @@
     <row r="19">
       <c r="A19" s="51" t="inlineStr">
         <is>
-          <t>Working capital schedule (driver-based)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="150" customHeight="1">
+          <t>Working capital schedule (driver-based)  [click − to collapse detail]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" hidden="1" outlineLevel="1" ht="98" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  DSO (days) — flat vs FY25</t>
@@ -7784,7 +7719,7 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>DSO flat at FY25 (AR ÷ Rev) × 365 ≈ 6.3 days. AR balance = (DSO ÷ 365) × projected revenue.</t>
+          <t>DSO flat ~6.3 days: LULU is DTC-heavy (minimal wholesale AR). FY22–FY25 DSO ran 6.0–6.3 days — no structural change assumed.</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
@@ -7794,24 +7729,12 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
-Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
+          <t>Ctrl+F "Accounts receivable, net"
+→ 190,657 ($000)
 Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 11,102,600 ($000)
+DSO = (190,657 ÷ 11,102,600) × 365 ≈ 6.3 days
+Flat: ~6.0–6.3 days FY22–FY25 (DTC model; immaterial wholesale AR).</t>
         </is>
       </c>
       <c r="E20" s="84" t="n">
@@ -7842,7 +7765,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="150" customHeight="1">
+    <row r="21" hidden="1" outlineLevel="1" ht="98" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Accounts receivable, net</t>
@@ -7850,7 +7773,7 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>DSO flat at FY25 (AR ÷ Rev) × 365 ≈ 6.3 days. AR balance = (DSO ÷ 365) × projected revenue.</t>
+          <t>DSO flat ~6.3 days: LULU is DTC-heavy (minimal wholesale AR). FY22–FY25 DSO ran 6.0–6.3 days — no structural change assumed.</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
@@ -7860,24 +7783,12 @@
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
-Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
+          <t>Ctrl+F "Accounts receivable, net"
+→ 190,657 ($000)
 Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 11,102,600 ($000)
+DSO = (190,657 ÷ 11,102,600) × 365 ≈ 6.3 days
+Flat: ~6.0–6.3 days FY22–FY25 (DTC model; immaterial wholesale AR).</t>
         </is>
       </c>
       <c r="E21" s="78" t="n">
@@ -7908,7 +7819,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="150" customHeight="1">
+    <row r="22" hidden="1" outlineLevel="1" ht="140" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  DIO (days) — FY25 anchor, −1 day/yr</t>
@@ -7916,36 +7827,27 @@
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>DIO FY25 anchor ≈ 129 days = (Inventories ÷ COGS) × 365. Declines 1 day/yr (−5 days over FY26–30) to clear excess stock.
-Also: One day of DIO improvement per forecast year — five days total by FY30 vs the FY25 anchor.</t>
+          <t>DIO FY25 ≈129 days anchors on elevated inventory (1,700,753 vs 1,442,081 FY24). Inventory ÷ COGS × 365 on the 10-K balance sheet.
+Also: −1 DIO day/yr tied to 10-K: unit inventories expected to decrease and markdown % to fall — gradual clearance, not a shock write-down.</t>
         </is>
       </c>
       <c r="C22" s="38" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: Inventories &amp; COGS
-Also: Scenarios: DIO clearance path (−5 days / 5 yrs)</t>
+Also: LULU FY2025 10-K: inventory &amp; markdown outlook</t>
         </is>
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
+          <t>Ctrl+F "Inventories"
+→ 1,700,753 ($000)  |  FY24: 1,442,081
 Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
-Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 4,818,468 ($000)
+DIO = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days
+Also: Ctrl+F "reduce the percentage of markdowns"
+→ Americas plan to cut promo/markdown intensity
+Ctrl+F "On a unit basis, we expect inventories to slightly decrease"
+Model: −1 DIO day/yr (−5 days FY26–30 vs FY25 anchor)</t>
         </is>
       </c>
       <c r="E22" s="84" t="n">
@@ -7976,7 +7878,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="150" customHeight="1">
+    <row r="23" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Inventories</t>
@@ -7984,7 +7886,7 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>DIO FY25 anchor ≈ 129 days = (Inventories ÷ COGS) × 365. Declines 1 day/yr (−5 days over FY26–30) to clear excess stock.</t>
+          <t>DIO FY25 ≈129 days anchors on elevated inventory (1,700,753 vs 1,442,081 FY24). Inventory ÷ COGS × 365 on the 10-K balance sheet.</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
@@ -7994,24 +7896,11 @@
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
+          <t>Ctrl+F "Inventories"
+→ 1,700,753 ($000)  |  FY24: 1,442,081
 Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
-Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 4,818,468 ($000)
+DIO = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days</t>
         </is>
       </c>
       <c r="E23" s="78" t="n">
@@ -8042,7 +7931,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="150" customHeight="1">
+    <row r="24" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  DPO (days) — flat vs FY25</t>
@@ -8050,7 +7939,7 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>DPO flat at FY25 (AP ÷ COGS) × 365 ≈ 25.1 days. AP balance = (DPO ÷ 365) × projected COGS.</t>
+          <t>DPO flat ~25 days at FY25 vendor leverage (331,421 ÷ 4,818,468 × 365). AP scales with projected COGS; payment terms unchanged.</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
@@ -8060,24 +7949,11 @@
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
+          <t>Ctrl+F "Accounts payable"
+→ 331,421 ($000)
 Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
-Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 4,818,468 ($000)
+DPO = (331,421 ÷ 4,818,468) × 365 ≈ 25.1 days (held flat)</t>
         </is>
       </c>
       <c r="E24" s="84" t="n">
@@ -8108,7 +7984,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="150" customHeight="1">
+    <row r="25" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Accounts payable</t>
@@ -8116,7 +7992,7 @@
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>DPO flat at FY25 (AP ÷ COGS) × 365 ≈ 25.1 days. AP balance = (DPO ÷ 365) × projected COGS.</t>
+          <t>DPO flat ~25 days at FY25 vendor leverage (331,421 ÷ 4,818,468 × 365). AP scales with projected COGS; payment terms unchanged.</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
@@ -8126,24 +8002,11 @@
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
+          <t>Ctrl+F "Accounts payable"
+→ 331,421 ($000)
 Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
-Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 4,818,468 ($000)
+DPO = (331,421 ÷ 4,818,468) × 365 ≈ 25.1 days (held flat)</t>
         </is>
       </c>
       <c r="E25" s="78" t="n">
@@ -8174,7 +8037,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="150" customHeight="1">
+    <row r="26" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A26" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Prepaid expenses (% of revenue)</t>
@@ -8182,7 +8045,7 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>Prepaid / other current assets held at FY25 % of revenue (564,089 ÷ 11,102,600 ≈ 5.1%).</t>
+          <t>OCA held at FY25 5.1% of revenue — prepaids + income-tax receivables (211,620 + 352,469) are the main non-AR/inventory current assets.</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
@@ -8192,24 +8055,11 @@
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
-Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
-Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+          <t>Ctrl+F "Prepaid expenses and other current assets"
+→ 211,620 ($000)
+Ctrl+F "Prepaid and receivable income taxes"
+→ 352,469 ($000)
+OCA residual (ex-cash/AR/inv) = 564,089 ≈ 5.1% of revenue</t>
         </is>
       </c>
       <c r="E26" s="81" t="n">
@@ -8236,7 +8086,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="150" customHeight="1">
+    <row r="27" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Prepaid expenses (other current assets)</t>
@@ -8244,7 +8094,7 @@
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>Prepaid / other current assets held at FY25 % of revenue (564,089 ÷ 11,102,600 ≈ 5.1%).</t>
+          <t>OCA held at FY25 5.1% of revenue — prepaids + income-tax receivables (211,620 + 352,469) are the main non-AR/inventory current assets.</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
@@ -8254,24 +8104,11 @@
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
-Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
-Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+          <t>Ctrl+F "Prepaid expenses and other current assets"
+→ 211,620 ($000)
+Ctrl+F "Prepaid and receivable income taxes"
+→ 352,469 ($000)
+OCA residual (ex-cash/AR/inv) = 564,089 ≈ 5.1% of revenue</t>
         </is>
       </c>
       <c r="E27" s="78" t="n">
@@ -8302,7 +8139,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="150" customHeight="1">
+    <row r="28" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Accrued liabilities (% of revenue)</t>
@@ -8310,7 +8147,7 @@
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>Accrued liabilities held at FY25 % of revenue (662,982 ÷ 11,102,600 ≈ 6.0%).</t>
+          <t>Accrued liabilities flat at FY25 6.0% of revenue (662,982 ÷ 11,102,600). Stable comp, marketing, and operating accrual mix.</t>
         </is>
       </c>
       <c r="C28" s="18" t="inlineStr">
@@ -8320,24 +8157,11 @@
       </c>
       <c r="D28" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
-Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
+          <t>Ctrl+F "Accrued liabilities and other"
+→ 662,982 ($000)
 Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 11,102,600 ($000)
+662,982 ÷ 11,102,600 ≈ 6.0% of revenue (held flat)</t>
         </is>
       </c>
       <c r="E28" s="81" t="n">
@@ -8364,7 +8188,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="150" customHeight="1">
+    <row r="29" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A29" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Accrued liabilities and other</t>
@@ -8372,7 +8196,7 @@
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>Accrued liabilities held at FY25 % of revenue (662,982 ÷ 11,102,600 ≈ 6.0%).</t>
+          <t>Accrued liabilities flat at FY25 6.0% of revenue (662,982 ÷ 11,102,600). Stable comp, marketing, and operating accrual mix.</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
@@ -8382,24 +8206,11 @@
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>FY25 WORKING CAPITAL ANCHORS (Form 10-K)
-Ctrl+F "Accounts receivable, net"
-  → 190,657 ($000)
-Ctrl+F "Inventories"
-  → 1,700,753 ($000)
-Ctrl+F "Accounts payable"
-  → 331,421 ($000)
-Ctrl+F "Accrued liabilities and other"
-  → 662,982 ($000)
-Ctrl+F "Cost of goods sold"
-  → 4,818,468 ($000)
+          <t>Ctrl+F "Accrued liabilities and other"
+→ 662,982 ($000)
 Ctrl+F "Net revenue"
-  → 11,102,600 ($000)
-Derived drivers
-  DSO ≈ 6.3 days  |  DIO ≈ 129 days  |  DPO ≈ 25.1 days
-  Prepaids ≈ 5.1% of revenue  |  Accruals ≈ 6.0% of revenue
-  DIO −1 day/yr (−5 days by FY30)  |  DSO &amp; DPO flat
-  ΔNWC = prior-year NWC − current-year NWC</t>
+→ 11,102,600 ($000)
+662,982 ÷ 11,102,600 ≈ 6.0% of revenue (held flat)</t>
         </is>
       </c>
       <c r="E29" s="78" t="n">
@@ -8430,7 +8241,7 @@
         <v/>
       </c>
     </row>
-    <row r="30">
+    <row r="30" hidden="1" outlineLevel="1">
       <c r="A30" s="16" t="inlineStr">
         <is>
           <t>Current operating assets (AR + inv + prepaids)</t>
@@ -8461,7 +8272,7 @@
         <v/>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="1" outlineLevel="1">
       <c r="A31" s="16" t="inlineStr">
         <is>
           <t>Current operating liabilities (AP + accruals)</t>
@@ -8492,7 +8303,7 @@
         <v/>
       </c>
     </row>
-    <row r="32">
+    <row r="32" hidden="1" outlineLevel="1">
       <c r="A32" s="23" t="inlineStr">
         <is>
           <t>Net working capital</t>
@@ -8526,33 +8337,50 @@
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="16" t="inlineStr">
+    <row r="33" ht="56" customHeight="1">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t>ΔNWC (prior yr − current yr)</t>
         </is>
       </c>
-      <c r="F33" s="79">
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>ΔNWC = prior − current. FY26 releases WC (sales down + DIO improves); FY27–30 absorbs cash as revenue grows — standard unlevered FCF bridge.</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>Scenarios tab: NWC roll-forward (driver schedule)</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="inlineStr">
+        <is>
+          <t>No single Ctrl+F — derived roll-forward.
+FY26: revenue −6.1% + DIO −1 day → NWC falls → ΔNWC positive (WC release).
+FY27–30: revenue +2.3%/yr → AR &amp; inventory rebuild → ΔNWC negative (WC build).</t>
+        </is>
+      </c>
+      <c r="F33" s="25">
         <f>Scenarios!G118</f>
         <v/>
       </c>
-      <c r="G33" s="79">
+      <c r="G33" s="25">
         <f>Scenarios!G119</f>
         <v/>
       </c>
-      <c r="H33" s="79">
+      <c r="H33" s="25">
         <f>Scenarios!G120</f>
         <v/>
       </c>
-      <c r="I33" s="79">
+      <c r="I33" s="25">
         <f>Scenarios!G121</f>
         <v/>
       </c>
-      <c r="J33" s="79">
+      <c r="J33" s="25">
         <f>Scenarios!G122</f>
         <v/>
       </c>
-      <c r="K33" s="80">
+      <c r="K33" s="83">
         <f>IF(MAX(ABS(F33-Scenarios!$G$118),ABS(G33-Scenarios!$G$119),ABS(H33-Scenarios!$G$120),ABS(I33-Scenarios!$G$121),ABS(J33-Scenarios!$G$122))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -9451,6 +9279,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId35"/>
+    <hyperlink ref="C33" location="'Scenarios'!A118"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId38"/>

</xml_diff>

<commit_message>
Lead NWC justifications with % of revenue (or not) per line item
Each NWC driver and balance row now opens column B with whether it is a
% of revenue and the FY25 implied percent. Added sc_ar, sc_inventory,
sc_ap, sc_coa, sc_col, and sc_nwc keys for distinct line-item docs.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -2357,7 +2357,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>GM% isolates COGS for inventory/AP drivers. FY25 56.6% = 6,284,132 ÷ 11,102,600; held near reported level in base case.</t>
+          <t>56.6% of revenue (gross margin). Isolates COGS for inventory/AP drivers; base case held near FY25 reported GM.</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
@@ -2367,13 +2367,13 @@
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Gross profit"
+          <t>56.6% of revenue (gross margin).
+Ctrl+F "Gross profit"
 → 6,284,132 ($000)
 Ctrl+F "Net revenue"
 → 11,102,600 ($000)
 Ctrl+F "Cost of goods sold"
-→ 4,818,468 ($000)
-GM = 6,284,132 ÷ 11,102,600 = 56.6%</t>
+→ 4,818,468 ($000)</t>
         </is>
       </c>
       <c r="F14" s="20" t="n">
@@ -2386,7 +2386,7 @@
         <v>0.575</v>
       </c>
     </row>
-    <row r="15" ht="98" customHeight="1">
+    <row r="15" ht="84" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
           <t>DSO (days) — flat vs FY25</t>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>DSO flat ~6.3 days: LULU is DTC-heavy (minimal wholesale AR). FY22–FY25 DSO ran 6.0–6.3 days — no structural change assumed.</t>
+          <t>Not % of revenue — DSO (days), flat ~6.3. Implied AR ≈1.7% of sales via (DSO÷365)×revenue.</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
@@ -2408,8 +2408,7 @@
 → 190,657 ($000)
 Ctrl+F "Net revenue"
 → 11,102,600 ($000)
-DSO = (190,657 ÷ 11,102,600) × 365 ≈ 6.3 days
-Flat: ~6.0–6.3 days FY22–FY25 (DTC model; immaterial wholesale AR).</t>
+Not % of revenue — DSO ≈ 6.3 days. Implied AR ≈ 1.7% of sales.</t>
         </is>
       </c>
       <c r="F15" s="39" t="n">
@@ -2430,7 +2429,7 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>DIO FY25 ≈129 days anchors on elevated inventory (1,700,753 vs 1,442,081 FY24). Inventory ÷ COGS × 365 on the 10-K balance sheet.</t>
+          <t>Not % of revenue — DIO (days), FY25 anchor ~129. Implied inventory ~15.3% of sales / 35.3% of COGS.</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
@@ -2444,7 +2443,7 @@
 → 1,700,753 ($000)  |  FY24: 1,442,081
 Ctrl+F "Cost of goods sold"
 → 4,818,468 ($000)
-DIO = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days</t>
+Not % of revenue — DIO ≈ 129 days. Implied ~15.3% of sales / 35.3% of COGS.</t>
         </is>
       </c>
       <c r="F16" s="39" t="n">
@@ -2457,7 +2456,7 @@
         <v>128.8324100108167</v>
       </c>
     </row>
-    <row r="17" ht="70" customHeight="1">
+    <row r="17" ht="56" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
           <t>DIO decline (days / forecast yr)</t>
@@ -2465,7 +2464,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>−1 DIO day/yr tied to 10-K: unit inventories expected to decrease and markdown % to fall — gradual clearance, not a shock write-down.</t>
+          <t>Not % of revenue — DIO falls 1 day/yr (−5 days by FY30). 10-K: fewer markdowns; unit inventories down.</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -2475,10 +2474,9 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "reduce the percentage of markdowns"
-→ Americas plan to cut promo/markdown intensity
-Ctrl+F "On a unit basis, we expect inventories to slightly decrease"
-Model: −1 DIO day/yr (−5 days FY26–30 vs FY25 anchor)</t>
+          <t>Not % of revenue — DIO −1 day/yr (−5 days FY26–30).
+Ctrl+F "reduce the percentage of markdowns"
+Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
         </is>
       </c>
       <c r="F17" s="40" t="n">
@@ -2499,7 +2497,7 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>DPO flat ~25 days at FY25 vendor leverage (331,421 ÷ 4,818,468 × 365). AP scales with projected COGS; payment terms unchanged.</t>
+          <t>Not % of revenue — DPO (days), flat ~25.1. Implied AP ≈3.0% of sales / 6.9% of COGS.</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
@@ -2513,7 +2511,7 @@
 → 331,421 ($000)
 Ctrl+F "Cost of goods sold"
 → 4,818,468 ($000)
-DPO = (331,421 ÷ 4,818,468) × 365 ≈ 25.1 days (held flat)</t>
+Not % of revenue — DPO ≈ 25.1 days. Implied AP ≈ 3.0% of sales / 6.9% of COGS.</t>
         </is>
       </c>
       <c r="F18" s="39" t="n">
@@ -2534,7 +2532,7 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>OCA held at FY25 5.1% of revenue — prepaids + income-tax receivables (211,620 + 352,469) are the main non-AR/inventory current assets.</t>
+          <t>5.1% of revenue (flat). FY25 other current assets (prepaids + tax receivables) ÷ net revenue.</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
@@ -2548,7 +2546,7 @@
 → 211,620 ($000)
 Ctrl+F "Prepaid and receivable income taxes"
 → 352,469 ($000)
-OCA residual (ex-cash/AR/inv) = 564,089 ≈ 5.1% of revenue</t>
+5.1% of revenue (flat). OCA residual = 564,089 ÷ 11,102,600.</t>
         </is>
       </c>
       <c r="F19" s="20" t="n">
@@ -2569,7 +2567,7 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Accrued liabilities flat at FY25 6.0% of revenue (662,982 ÷ 11,102,600). Stable comp, marketing, and operating accrual mix.</t>
+          <t>6.0% of revenue (flat). FY25 accrued liabilities ÷ net revenue; comp/marketing accrual mix.</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
@@ -2583,7 +2581,7 @@
 → 662,982 ($000)
 Ctrl+F "Net revenue"
 → 11,102,600 ($000)
-662,982 ÷ 11,102,600 ≈ 6.0% of revenue (held flat)</t>
+6.0% of revenue (flat). 662,982 ÷ 11,102,600.</t>
         </is>
       </c>
       <c r="F20" s="20" t="n">
@@ -7256,7 +7254,7 @@
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>GM% isolates COGS for inventory/AP drivers. FY25 56.6% = 6,284,132 ÷ 11,102,600; held near reported level in base case.</t>
+          <t>56.6% of revenue (gross margin). Isolates COGS for inventory/AP drivers; base case held near FY25 reported GM.</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
@@ -7266,13 +7264,13 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Gross profit"
+          <t>56.6% of revenue (gross margin).
+Ctrl+F "Gross profit"
 → 6,284,132 ($000)
 Ctrl+F "Net revenue"
 → 11,102,600 ($000)
 Ctrl+F "Cost of goods sold"
-→ 4,818,468 ($000)
-GM = 6,284,132 ÷ 11,102,600 = 56.6%</t>
+→ 4,818,468 ($000)</t>
         </is>
       </c>
       <c r="E7" s="81" t="n">
@@ -7711,7 +7709,7 @@
         </is>
       </c>
     </row>
-    <row r="20" hidden="1" outlineLevel="1" ht="98" customHeight="1">
+    <row r="20" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  DSO (days) — flat vs FY25</t>
@@ -7719,7 +7717,7 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>DSO flat ~6.3 days: LULU is DTC-heavy (minimal wholesale AR). FY22–FY25 DSO ran 6.0–6.3 days — no structural change assumed.</t>
+          <t>Not % of revenue — DSO (days), flat ~6.3. Implied AR ≈1.7% of sales via (DSO÷365)×revenue.</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
@@ -7733,8 +7731,7 @@
 → 190,657 ($000)
 Ctrl+F "Net revenue"
 → 11,102,600 ($000)
-DSO = (190,657 ÷ 11,102,600) × 365 ≈ 6.3 days
-Flat: ~6.0–6.3 days FY22–FY25 (DTC model; immaterial wholesale AR).</t>
+Not % of revenue — DSO ≈ 6.3 days. Implied AR ≈ 1.7% of sales.</t>
         </is>
       </c>
       <c r="E20" s="84" t="n">
@@ -7765,7 +7762,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" hidden="1" outlineLevel="1" ht="98" customHeight="1">
+    <row r="21" hidden="1" outlineLevel="1" ht="84" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Accounts receivable, net</t>
@@ -7773,7 +7770,7 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>DSO flat ~6.3 days: LULU is DTC-heavy (minimal wholesale AR). FY22–FY25 DSO ran 6.0–6.3 days — no structural change assumed.</t>
+          <t>Implied ~1.7% of revenue (not a direct % plug). Balance = (DSO÷365)×revenue; DSO flat at FY25.</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
@@ -7787,8 +7784,7 @@
 → 190,657 ($000)
 Ctrl+F "Net revenue"
 → 11,102,600 ($000)
-DSO = (190,657 ÷ 11,102,600) × 365 ≈ 6.3 days
-Flat: ~6.0–6.3 days FY22–FY25 (DTC model; immaterial wholesale AR).</t>
+Implied ~1.7% of revenue (= 190,657 ÷ 11,102,600); forecast via DSO×revenue.</t>
         </is>
       </c>
       <c r="E21" s="78" t="n">
@@ -7819,7 +7815,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" hidden="1" outlineLevel="1" ht="140" customHeight="1">
+    <row r="22" hidden="1" outlineLevel="1" ht="126" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  DIO (days) — FY25 anchor, −1 day/yr</t>
@@ -7827,8 +7823,8 @@
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>DIO FY25 ≈129 days anchors on elevated inventory (1,700,753 vs 1,442,081 FY24). Inventory ÷ COGS × 365 on the 10-K balance sheet.
-Also: −1 DIO day/yr tied to 10-K: unit inventories expected to decrease and markdown % to fall — gradual clearance, not a shock write-down.</t>
+          <t>Not % of revenue — DIO (days), FY25 anchor ~129. Implied inventory ~15.3% of sales / 35.3% of COGS.
+Also: Not % of revenue — DIO falls 1 day/yr (−5 days by FY30). 10-K: fewer markdowns; unit inventories down.</t>
         </is>
       </c>
       <c r="C22" s="38" t="inlineStr">
@@ -7843,11 +7839,10 @@
 → 1,700,753 ($000)  |  FY24: 1,442,081
 Ctrl+F "Cost of goods sold"
 → 4,818,468 ($000)
-DIO = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days
-Also: Ctrl+F "reduce the percentage of markdowns"
-→ Americas plan to cut promo/markdown intensity
-Ctrl+F "On a unit basis, we expect inventories to slightly decrease"
-Model: −1 DIO day/yr (−5 days FY26–30 vs FY25 anchor)</t>
+Not % of revenue — DIO ≈ 129 days. Implied ~15.3% of sales / 35.3% of COGS.
+Also: Not % of revenue — DIO −1 day/yr (−5 days FY26–30).
+Ctrl+F "reduce the percentage of markdowns"
+Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
         </is>
       </c>
       <c r="E22" s="84" t="n">
@@ -7886,21 +7881,21 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>DIO FY25 ≈129 days anchors on elevated inventory (1,700,753 vs 1,442,081 FY24). Inventory ÷ COGS × 365 on the 10-K balance sheet.</t>
+          <t>Not % of revenue (DIO×COGS balance). FY25 ≈15.3% of sales; improves as DIO declines 1 day/yr.</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K: Inventories &amp; COGS</t>
+          <t>LULU FY2025 10-K: Inventories</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Inventories"
-→ 1,700,753 ($000)  |  FY24: 1,442,081
-Ctrl+F "Cost of goods sold"
-→ 4,818,468 ($000)
-DIO = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days</t>
+→ 1,700,753 ($000)
+Ctrl+F "Net revenue"
+→ 11,102,600 ($000)
+Not % of revenue (DIO×COGS). FY25 ≈ 15.3% of sales (= 1,700,753 ÷ 11,102,600).</t>
         </is>
       </c>
       <c r="E23" s="78" t="n">
@@ -7939,7 +7934,7 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>DPO flat ~25 days at FY25 vendor leverage (331,421 ÷ 4,818,468 × 365). AP scales with projected COGS; payment terms unchanged.</t>
+          <t>Not % of revenue — DPO (days), flat ~25.1. Implied AP ≈3.0% of sales / 6.9% of COGS.</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
@@ -7953,7 +7948,7 @@
 → 331,421 ($000)
 Ctrl+F "Cost of goods sold"
 → 4,818,468 ($000)
-DPO = (331,421 ÷ 4,818,468) × 365 ≈ 25.1 days (held flat)</t>
+Not % of revenue — DPO ≈ 25.1 days. Implied AP ≈ 3.0% of sales / 6.9% of COGS.</t>
         </is>
       </c>
       <c r="E24" s="84" t="n">
@@ -7992,21 +7987,21 @@
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>DPO flat ~25 days at FY25 vendor leverage (331,421 ÷ 4,818,468 × 365). AP scales with projected COGS; payment terms unchanged.</t>
+          <t>Implied ~3.0% of revenue (not a direct % plug). Balance = (DPO÷365)×COGS; DPO flat at FY25.</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K: Accounts payable &amp; COGS</t>
+          <t>LULU FY2025 10-K: Accounts payable</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Accounts payable"
 → 331,421 ($000)
-Ctrl+F "Cost of goods sold"
-→ 4,818,468 ($000)
-DPO = (331,421 ÷ 4,818,468) × 365 ≈ 25.1 days (held flat)</t>
+Ctrl+F "Net revenue"
+→ 11,102,600 ($000)
+Implied ~3.0% of revenue (= 331,421 ÷ 11,102,600); forecast via DPO×COGS.</t>
         </is>
       </c>
       <c r="E25" s="78" t="n">
@@ -8045,7 +8040,7 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>OCA held at FY25 5.1% of revenue — prepaids + income-tax receivables (211,620 + 352,469) are the main non-AR/inventory current assets.</t>
+          <t>5.1% of revenue (flat). FY25 other current assets (prepaids + tax receivables) ÷ net revenue.</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
@@ -8059,7 +8054,7 @@
 → 211,620 ($000)
 Ctrl+F "Prepaid and receivable income taxes"
 → 352,469 ($000)
-OCA residual (ex-cash/AR/inv) = 564,089 ≈ 5.1% of revenue</t>
+5.1% of revenue (flat). OCA residual = 564,089 ÷ 11,102,600.</t>
         </is>
       </c>
       <c r="E26" s="81" t="n">
@@ -8094,7 +8089,7 @@
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>OCA held at FY25 5.1% of revenue — prepaids + income-tax receivables (211,620 + 352,469) are the main non-AR/inventory current assets.</t>
+          <t>5.1% of revenue (flat). FY25 other current assets (prepaids + tax receivables) ÷ net revenue.</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
@@ -8108,7 +8103,7 @@
 → 211,620 ($000)
 Ctrl+F "Prepaid and receivable income taxes"
 → 352,469 ($000)
-OCA residual (ex-cash/AR/inv) = 564,089 ≈ 5.1% of revenue</t>
+5.1% of revenue (flat). OCA residual = 564,089 ÷ 11,102,600.</t>
         </is>
       </c>
       <c r="E27" s="78" t="n">
@@ -8147,7 +8142,7 @@
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>Accrued liabilities flat at FY25 6.0% of revenue (662,982 ÷ 11,102,600). Stable comp, marketing, and operating accrual mix.</t>
+          <t>6.0% of revenue (flat). FY25 accrued liabilities ÷ net revenue; comp/marketing accrual mix.</t>
         </is>
       </c>
       <c r="C28" s="18" t="inlineStr">
@@ -8161,7 +8156,7 @@
 → 662,982 ($000)
 Ctrl+F "Net revenue"
 → 11,102,600 ($000)
-662,982 ÷ 11,102,600 ≈ 6.0% of revenue (held flat)</t>
+6.0% of revenue (flat). 662,982 ÷ 11,102,600.</t>
         </is>
       </c>
       <c r="E28" s="81" t="n">
@@ -8196,7 +8191,7 @@
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>Accrued liabilities flat at FY25 6.0% of revenue (662,982 ÷ 11,102,600). Stable comp, marketing, and operating accrual mix.</t>
+          <t>6.0% of revenue (flat). FY25 accrued liabilities ÷ net revenue; comp/marketing accrual mix.</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
@@ -8210,7 +8205,7 @@
 → 662,982 ($000)
 Ctrl+F "Net revenue"
 → 11,102,600 ($000)
-662,982 ÷ 11,102,600 ≈ 6.0% of revenue (held flat)</t>
+6.0% of revenue (flat). 662,982 ÷ 11,102,600.</t>
         </is>
       </c>
       <c r="E29" s="78" t="n">
@@ -8241,10 +8236,26 @@
         <v/>
       </c>
     </row>
-    <row r="30" hidden="1" outlineLevel="1">
+    <row r="30" hidden="1" outlineLevel="1" ht="42" customHeight="1">
       <c r="A30" s="16" t="inlineStr">
         <is>
           <t>Current operating assets (AR + inv + prepaids)</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>Not one % — sum ≈22.1% of FY25 sales (AR ~1.7% + inventory ~15.3% + prepaids 5.1%).</t>
+        </is>
+      </c>
+      <c r="C30" s="24" t="inlineStr">
+        <is>
+          <t>Scenarios tab: AR + inventory + prepaids</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Not one % of revenue — sum of line items.
+FY25: AR ~1.7% + inventory ~15.3% + prepaids 5.1% ≈ 22.1% of sales.</t>
         </is>
       </c>
       <c r="F30" s="79">
@@ -8272,10 +8283,26 @@
         <v/>
       </c>
     </row>
-    <row r="31" hidden="1" outlineLevel="1">
+    <row r="31" hidden="1" outlineLevel="1" ht="42" customHeight="1">
       <c r="A31" s="16" t="inlineStr">
         <is>
           <t>Current operating liabilities (AP + accruals)</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>Not one % — sum ≈9.0% of FY25 sales (AP ~3.0% + accrued liabilities 6.0%).</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>Scenarios tab: AP + accrued liabilities</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>Not one % of revenue — sum of line items.
+FY25: AP ~3.0% + accrued liabilities 6.0% ≈ 9.0% of sales.</t>
         </is>
       </c>
       <c r="F31" s="79">
@@ -8303,10 +8330,26 @@
         <v/>
       </c>
     </row>
-    <row r="32" hidden="1" outlineLevel="1">
+    <row r="32" hidden="1" outlineLevel="1" ht="42" customHeight="1">
       <c r="A32" s="23" t="inlineStr">
         <is>
           <t>Net working capital</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Not one % — net ≈13.2% of FY25 sales ($1,461,096k). COA minus COL; rolls forward each year.</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: working-capital components</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>Not one % of revenue — net balance.
+FY25 NWC ≈ 13.2% of sales ($1,461,096k = COA − COL).</t>
         </is>
       </c>
       <c r="E32" s="82" t="n">
@@ -8345,7 +8388,7 @@
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>ΔNWC = prior − current. FY26 releases WC (sales down + DIO improves); FY27–30 absorbs cash as revenue grows — standard unlevered FCF bridge.</t>
+          <t>Not % of revenue — $ change in NWC year-over-year. Prior-year NWC minus current-year NWC for the FCF bridge.</t>
         </is>
       </c>
       <c r="C33" s="18" t="inlineStr">
@@ -8355,7 +8398,7 @@
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>No single Ctrl+F — derived roll-forward.
+          <t>Not % of revenue — $ change year-over-year.
 FY26: revenue −6.1% + DIO −1 day → NWC falls → ΔNWC positive (WC release).
 FY27–30: revenue +2.3%/yr → AR &amp; inventory rebuild → ΔNWC negative (WC build).</t>
         </is>
@@ -9278,29 +9321,30 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId36"/>
     <hyperlink ref="C33" location="'Scenarios'!A118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId45"/>
     <hyperlink ref="C63" location="'DCF'!E46"/>
     <hyperlink ref="M63" location="'Comps'!A45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId46"/>
     <hyperlink ref="L79" location="'Scenarios'!G10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId47"/>
     <hyperlink ref="L80" location="'WACC'!E41"/>
     <hyperlink ref="L81" location="'WACC'!E41"/>
     <hyperlink ref="L82" location="'WACC'!E41"/>
     <hyperlink ref="L83" location="'WACC'!E41"/>
     <hyperlink ref="L84" location="'WACC'!E41"/>
     <hyperlink ref="C85" location="'Scenarios'!G9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L85" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L85" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Document DIO anchor and Inventories balance formulas in NWC justifications
Spell out FY25 DIO = (Inventories ÷ COGS) × 365 and forecast
Inventories_t = (DIO_t ÷ 365) × COGS_t with COGS_t = Revenue × (1 − GM%).

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -2421,7 +2421,7 @@
         <v>6.267883648875038</v>
       </c>
     </row>
-    <row r="16" ht="84" customHeight="1">
+    <row r="16" ht="140" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
           <t>FY25 DIO anchor (days)</t>
@@ -2429,7 +2429,10 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — DIO (days), FY25 anchor ~129. Implied inventory ~15.3% of sales / 35.3% of COGS.</t>
+          <t>Not % of revenue — DIO (days).
+FY25 anchor: DIO = (Inventories ÷ COGS) × 365
+  = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days (FY24 inv: 1,442,081).
+Forecast path: DIO_t = FY25 DIO − (1 day × year t); flat across scenarios.</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
@@ -2439,11 +2442,15 @@
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Inventories"
+          <t>Not % of revenue — DIO (days).
+FY25 anchor formula:
+  DIO = (Inventories ÷ COGS) × 365
+Ctrl+F "Inventories"
 → 1,700,753 ($000)  |  FY24: 1,442,081
 Ctrl+F "Cost of goods sold"
 → 4,818,468 ($000)
-Not % of revenue — DIO ≈ 129 days. Implied ~15.3% of sales / 35.3% of COGS.</t>
+  = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days
+Forecast: DIO_t = FY25 DIO − (1 × year t)</t>
         </is>
       </c>
       <c r="F16" s="39" t="n">
@@ -2456,7 +2463,7 @@
         <v>128.8324100108167</v>
       </c>
     </row>
-    <row r="17" ht="56" customHeight="1">
+    <row r="17" ht="70" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
           <t>DIO decline (days / forecast yr)</t>
@@ -2464,7 +2471,10 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — DIO falls 1 day/yr (−5 days by FY30). 10-K: fewer markdowns; unit inventories down.</t>
+          <t>Not % of revenue — subtract 1 DIO day per forecast year (−5 days FY26–30).
+Feeds Inventories = (DIO_t ÷ 365) × COGS_t.
+Ctrl+F "reduce the percentage of markdowns"
+Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -2475,6 +2485,7 @@
       <c r="D17" s="19" t="inlineStr">
         <is>
           <t>Not % of revenue — DIO −1 day/yr (−5 days FY26–30).
+Feeds Inventories_t = (DIO_t ÷ 365) × COGS_t.
 Ctrl+F "reduce the percentage of markdowns"
 Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
         </is>
@@ -7815,7 +7826,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" hidden="1" outlineLevel="1" ht="126" customHeight="1">
+    <row r="22" hidden="1" outlineLevel="1" ht="150" customHeight="1">
       <c r="A22" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  DIO (days) — FY25 anchor, −1 day/yr</t>
@@ -7823,8 +7834,14 @@
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue — DIO (days), FY25 anchor ~129. Implied inventory ~15.3% of sales / 35.3% of COGS.
-Also: Not % of revenue — DIO falls 1 day/yr (−5 days by FY30). 10-K: fewer markdowns; unit inventories down.</t>
+          <t>Not % of revenue — DIO (days).
+FY25 anchor: DIO = (Inventories ÷ COGS) × 365
+  = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days (FY24 inv: 1,442,081).
+Forecast path: DIO_t = FY25 DIO − (1 day × year t); flat across scenarios.
+Also: Not % of revenue — subtract 1 DIO day per forecast year (−5 days FY26–30).
+Feeds Inventories = (DIO_t ÷ 365) × COGS_t.
+Ctrl+F "reduce the percentage of markdowns"
+Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
         </is>
       </c>
       <c r="C22" s="38" t="inlineStr">
@@ -7835,12 +7852,17 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Inventories"
+          <t>Not % of revenue — DIO (days).
+FY25 anchor formula:
+  DIO = (Inventories ÷ COGS) × 365
+Ctrl+F "Inventories"
 → 1,700,753 ($000)  |  FY24: 1,442,081
 Ctrl+F "Cost of goods sold"
 → 4,818,468 ($000)
-Not % of revenue — DIO ≈ 129 days. Implied ~15.3% of sales / 35.3% of COGS.
+  = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days
+Forecast: DIO_t = FY25 DIO − (1 × year t)
 Also: Not % of revenue — DIO −1 day/yr (−5 days FY26–30).
+Feeds Inventories_t = (DIO_t ÷ 365) × COGS_t.
 Ctrl+F "reduce the percentage of markdowns"
 Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
         </is>
@@ -7873,7 +7895,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" hidden="1" outlineLevel="1" ht="84" customHeight="1">
+    <row r="23" hidden="1" outlineLevel="1" ht="112" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Inventories</t>
@@ -7881,7 +7903,13 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue (DIO×COGS balance). FY25 ≈15.3% of sales; improves as DIO declines 1 day/yr.</t>
+          <t>Not % of revenue — $ balance (not a direct % plug).
+Inventories_t = (DIO_t ÷ 365) × COGS_t
+COGS_t = Revenue_t × (1 − GM%). FY25 check: (129 ÷ 365) × 4,818,468 ≈ 1,700,753.
+Ctrl+F "Inventories"
+→ 1,700,753 ($000)
+Ctrl+F "Cost of goods sold"
+→ 4,818,468 ($000)</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
@@ -7891,11 +7919,13 @@
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Inventories"
+          <t>Not % of revenue — Inventories_t = (DIO_t ÷ 365) × COGS_t.
+COGS_t = Revenue_t × (1 − GM%).
+Ctrl+F "Inventories"
 → 1,700,753 ($000)
-Ctrl+F "Net revenue"
-→ 11,102,600 ($000)
-Not % of revenue (DIO×COGS). FY25 ≈ 15.3% of sales (= 1,700,753 ÷ 11,102,600).</t>
+Ctrl+F "Cost of goods sold"
+→ 4,818,468 ($000)
+FY25 proof: (129 ÷ 365) × 4,818,468 ≈ 1,700,753</t>
         </is>
       </c>
       <c r="E23" s="78" t="n">
@@ -8247,7 +8277,7 @@
           <t>Not one % — sum ≈22.1% of FY25 sales (AR ~1.7% + inventory ~15.3% + prepaids 5.1%).</t>
         </is>
       </c>
-      <c r="C30" s="24" t="inlineStr">
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>Scenarios tab: AR + inventory + prepaids</t>
         </is>
@@ -8294,7 +8324,7 @@
           <t>Not one % — sum ≈9.0% of FY25 sales (AP ~3.0% + accrued liabilities 6.0%).</t>
         </is>
       </c>
-      <c r="C31" s="24" t="inlineStr">
+      <c r="C31" s="18" t="inlineStr">
         <is>
           <t>Scenarios tab: AP + accrued liabilities</t>
         </is>
@@ -9321,6 +9351,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId34"/>
+    <hyperlink ref="C30" location="'Scenarios'!A103"/>
+    <hyperlink ref="C31" location="'Scenarios'!A108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId36"/>
     <hyperlink ref="C33" location="'Scenarios'!A118"/>

</xml_diff>

<commit_message>
Add DTC/store rationale for flat DSO on AR justification
Explain that DSO stays ~6 days because most revenue is company-operated
stores and e-commerce (cash at sale); AR is a small predictable wholesale residual.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — DSO (days), flat ~6.3. Implied AR ≈1.7% of sales via (DSO÷365)×revenue.</t>
+          <t>Not % of revenue — DSO (days), flat ~6.3. Mostly own stores/DTC (cash at register); AR is small wholesale residual — predictable ~6 days FY22–25.</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
@@ -7728,7 +7728,7 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — DSO (days), flat ~6.3. Implied AR ≈1.7% of sales via (DSO÷365)×revenue.</t>
+          <t>Not % of revenue — DSO (days), flat ~6.3. Mostly own stores/DTC (cash at register); AR is small wholesale residual — predictable ~6 days FY22–25.</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
@@ -7781,7 +7781,7 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>Implied ~1.7% of revenue (not a direct % plug). Balance = (DSO÷365)×revenue; DSO flat at FY25.</t>
+          <t>Implied ~1.7% of revenue (not a direct % plug). AR = (DSO÷365)×revenue; flat DSO because sales are mostly own-store/DTC, not credit wholesale.</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Collapse documentation columns by default on all model tabs
Group and hide Justification | Source | Ctrl+F (B–D) on WACC, Scenarios,
DCF, and Comps; also L–M alt-source on DCF and I–L equation/docs on Revenue
Drivers so users see labels and numbers first.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1241,16 +1241,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="2" max="2"/>
+    <col hidden="1" outlineLevel="1" width="18" customWidth="1" min="3" max="3"/>
+    <col hidden="1" outlineLevel="1" width="40" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Justification (~20 words)</t>
+          <t>Justification (~20 words)  [cols B–D: click + to expand]</t>
         </is>
       </c>
       <c r="C2" s="15" t="inlineStr">
@@ -1957,16 +1957,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col hidden="1" outlineLevel="1" width="26" customWidth="1" min="2" max="2"/>
+    <col hidden="1" outlineLevel="1" width="16" customWidth="1" min="3" max="3"/>
+    <col hidden="1" outlineLevel="1" width="38" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>Justification (~20 words)</t>
+          <t>Justification (~20 words)  [cols B–D: click + to expand]</t>
         </is>
       </c>
       <c r="C3" s="15" t="inlineStr">
@@ -2386,7 +2386,7 @@
         <v>0.575</v>
       </c>
     </row>
-    <row r="15" ht="84" customHeight="1">
+    <row r="15" ht="150" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
           <t>DSO (days) — flat vs FY25</t>
@@ -2404,11 +2404,16 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts receivable, net"
+          <t>Not % of revenue — DSO (days), flat ~6.3.
+Why flat: ~90%+ revenue is company-operated stores + e-commerce (cash/card at sale);
+AR is a small, stable wholesale/license residual — predictable collection, not trade credit.
+Ctrl+F "Accounts receivable, net"
 → 190,657 ($000)
 Ctrl+F "Net revenue"
 → 11,102,600 ($000)
-Not % of revenue — DSO ≈ 6.3 days. Implied AR ≈ 1.7% of sales.</t>
+DSO = (190,657 ÷ 11,102,600) × 365 ≈ 6.3 days (~6.0–6.3 FY22–25).
+Ctrl+F "company-operated stores"
+Ctrl+F "E-commerce"</t>
         </is>
       </c>
       <c r="F15" s="39" t="n">
@@ -4698,7 +4703,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L59"/>
@@ -4712,10 +4717,10 @@
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="36" customWidth="1" min="12" max="12"/>
+    <col hidden="1" outlineLevel="1" width="40" customWidth="1" min="9" max="9"/>
+    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="10" max="10"/>
+    <col hidden="1" outlineLevel="1" width="16" customWidth="1" min="11" max="11"/>
+    <col hidden="1" outlineLevel="1" width="36" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4820,7 +4825,7 @@
       </c>
       <c r="J5" s="55" t="inlineStr">
         <is>
-          <t>Justification</t>
+          <t>Justification  [cols I–L: click + to expand]</t>
         </is>
       </c>
       <c r="K5" s="55" t="inlineStr">
@@ -5582,7 +5587,7 @@
       </c>
       <c r="J23" s="55" t="inlineStr">
         <is>
-          <t>Justification</t>
+          <t>Justification  [cols I–L: click + to expand]</t>
         </is>
       </c>
       <c r="K23" s="55" t="inlineStr">
@@ -6141,7 +6146,7 @@
       </c>
       <c r="J37" s="55" t="inlineStr">
         <is>
-          <t>Justification</t>
+          <t>Justification  [cols I–L: click + to expand]</t>
         </is>
       </c>
       <c r="K37" s="55" t="inlineStr">
@@ -6380,7 +6385,7 @@
       </c>
       <c r="J44" s="55" t="inlineStr">
         <is>
-          <t>Justification</t>
+          <t>Justification  [cols I–L: click + to expand]</t>
         </is>
       </c>
       <c r="K44" s="55" t="inlineStr">
@@ -6795,7 +6800,7 @@
       </c>
       <c r="J54" s="55" t="inlineStr">
         <is>
-          <t>Justification</t>
+          <t>Justification  [cols I–L: click + to expand]</t>
         </is>
       </c>
       <c r="K54" s="55" t="inlineStr">
@@ -7050,9 +7055,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col hidden="1" outlineLevel="1" width="26" customWidth="1" min="2" max="2"/>
+    <col hidden="1" outlineLevel="1" width="16" customWidth="1" min="3" max="3"/>
+    <col hidden="1" outlineLevel="1" width="36" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
@@ -7060,8 +7065,8 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="36" customWidth="1" min="13" max="13"/>
+    <col hidden="1" outlineLevel="1" width="16" customWidth="1" min="12" max="12"/>
+    <col hidden="1" outlineLevel="1" width="36" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -7083,7 +7088,7 @@
     <row r="2">
       <c r="B2" s="70" t="inlineStr">
         <is>
-          <t>Justification (~20 words)</t>
+          <t>Justification (~20 words)  [cols B–D: click + to expand]</t>
         </is>
       </c>
       <c r="C2" s="70" t="inlineStr">
@@ -7133,7 +7138,7 @@
       </c>
       <c r="L2" s="70" t="inlineStr">
         <is>
-          <t>Alt. source</t>
+          <t>Alt. source  [cols L–M: click + to expand]</t>
         </is>
       </c>
       <c r="M2" s="70" t="inlineStr">
@@ -7720,7 +7725,7 @@
         </is>
       </c>
     </row>
-    <row r="20" hidden="1" outlineLevel="1" ht="84" customHeight="1">
+    <row r="20" hidden="1" outlineLevel="1" ht="150" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  DSO (days) — flat vs FY25</t>
@@ -7738,11 +7743,16 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts receivable, net"
+          <t>Not % of revenue — DSO (days), flat ~6.3.
+Why flat: ~90%+ revenue is company-operated stores + e-commerce (cash/card at sale);
+AR is a small, stable wholesale/license residual — predictable collection, not trade credit.
+Ctrl+F "Accounts receivable, net"
 → 190,657 ($000)
 Ctrl+F "Net revenue"
 → 11,102,600 ($000)
-Not % of revenue — DSO ≈ 6.3 days. Implied AR ≈ 1.7% of sales.</t>
+DSO = (190,657 ÷ 11,102,600) × 365 ≈ 6.3 days (~6.0–6.3 FY22–25).
+Ctrl+F "company-operated stores"
+Ctrl+F "E-commerce"</t>
         </is>
       </c>
       <c r="E20" s="84" t="n">
@@ -7773,7 +7783,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" hidden="1" outlineLevel="1" ht="84" customHeight="1">
+    <row r="21" hidden="1" outlineLevel="1" ht="98" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Accounts receivable, net</t>
@@ -7791,11 +7801,12 @@
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Accounts receivable, net"
+          <t>Implied ~1.7% of revenue (= 190,657 ÷ 11,102,600); not a direct % plug.
+AR_t = (DSO ÷ 365) × Revenue_t. DSO flat because own-store/DTC dominates — AR scales predictably with sales.
+Ctrl+F "Accounts receivable, net"
 → 190,657 ($000)
 Ctrl+F "Net revenue"
-→ 11,102,600 ($000)
-Implied ~1.7% of revenue (= 190,657 ÷ 11,102,600); forecast via DSO×revenue.</t>
+→ 11,102,600 ($000)</t>
         </is>
       </c>
       <c r="E21" s="78" t="n">
@@ -9385,16 +9396,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="2" max="2"/>
+    <col hidden="1" outlineLevel="1" width="18" customWidth="1" min="3" max="3"/>
+    <col hidden="1" outlineLevel="1" width="44" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -9420,7 +9431,7 @@
     <row r="2">
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Justification (~20 words)</t>
+          <t>Justification (~20 words)  [cols B–D: click + to expand]</t>
         </is>
       </c>
       <c r="C2" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Add 5-phase NOPAT Bridge tab and wire normalized tax into DCF
Implements the EBIT-to-NOPAT normalization pipeline: operating adjustments,
lease interest reclass, channel EBIT forecasting, and unlevered t_operating
with glide to marginal rate. Scenarios base-case NOPAT links to the bridge;
bear/bull use bridge t_operating on their EBIT paths. DCF tax row uses
unlevered tax expense. Adds np_* documentation and assumptions memo section.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WACC" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Drivers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOPAT Bridge" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
     <numFmt numFmtId="168" formatCode="0.000"/>
     <numFmt numFmtId="169" formatCode="0.0x"/>
   </numFmts>
-  <fonts count="52">
+  <fonts count="53">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -246,6 +247,28 @@
     </font>
     <font>
       <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="001F2A44"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <color rgb="00000000"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <color rgb="00C8102E"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
       <i val="1"/>
       <color rgb="000000CC"/>
       <sz val="8"/>
@@ -256,12 +279,6 @@
       <color rgb="000000CC"/>
       <sz val="8"/>
       <u val="single"/>
-    </font>
-    <font>
-      <name val="Garamond"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Garamond"/>
@@ -280,11 +297,6 @@
       <i val="1"/>
       <color rgb="00F2F2F2"/>
       <sz val="7"/>
-    </font>
-    <font>
-      <name val="Garamond"/>
-      <color rgb="00000000"/>
-      <sz val="8"/>
     </font>
     <font>
       <name val="Garamond"/>
@@ -309,12 +321,6 @@
       <b val="1"/>
       <color rgb="00006100"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Garamond"/>
-      <b val="1"/>
-      <color rgb="001F2A44"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Garamond"/>
@@ -399,7 +405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -580,29 +586,14 @@
     <xf numFmtId="166" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="166" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -610,16 +601,40 @@
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="166" fontId="35" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="35" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -634,26 +649,26 @@
     <xf numFmtId="168" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="45" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="47" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="46" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="46" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -663,31 +678,31 @@
     <xf numFmtId="165" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="48" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="49" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="49" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="50" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -702,7 +717,7 @@
     <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -720,7 +735,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="51" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="52" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1161,7 +1176,7 @@
     <row r="15">
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>WACC  •  Revenue Drivers  •  Scenarios  •  DCF  •  Comps / Football Field</t>
+          <t>WACC  •  Revenue Drivers  •  NOPAT Bridge  •  Scenarios  •  DCF  •  Comps / Football Field</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1190,7 @@
     <row r="17" ht="36" customHeight="1">
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>LULU_Assumptions_Memo.pdf — full guide: every red assumption on WACC, Scenarios, Revenue Drivers, DCF, Comps &amp; 3-Statement
+          <t>LULU_Assumptions_Memo.pdf — full guide: every red assumption on WACC, Scenarios, Revenue Drivers, NOPAT Bridge, DCF, Comps &amp; 3-Statement
 Ctrl+F: Open for justification, clickable source links, and Ctrl+F proof for every assumption.</t>
         </is>
       </c>
@@ -3099,15 +3114,15 @@
         </is>
       </c>
       <c r="F48" s="42">
-        <f>F43*(1-F11)</f>
+        <f>F43*(1-'NOPAT Bridge'!F$35)</f>
         <v/>
       </c>
       <c r="G48" s="42">
-        <f>G43*(1-G11)</f>
+        <f>'NOPAT Bridge'!F37</f>
         <v/>
       </c>
       <c r="H48" s="42">
-        <f>H43*(1-H11)</f>
+        <f>H43*(1-'NOPAT Bridge'!F$35)</f>
         <v/>
       </c>
     </row>
@@ -3118,15 +3133,15 @@
         </is>
       </c>
       <c r="F49" s="42">
-        <f>F44*(1-F11)</f>
+        <f>F44*(1-'NOPAT Bridge'!G$35)</f>
         <v/>
       </c>
       <c r="G49" s="42">
-        <f>G44*(1-G11)</f>
+        <f>'NOPAT Bridge'!G37</f>
         <v/>
       </c>
       <c r="H49" s="42">
-        <f>H44*(1-H11)</f>
+        <f>H44*(1-'NOPAT Bridge'!G$35)</f>
         <v/>
       </c>
     </row>
@@ -3137,15 +3152,15 @@
         </is>
       </c>
       <c r="F50" s="42">
-        <f>F45*(1-F11)</f>
+        <f>F45*(1-'NOPAT Bridge'!H$35)</f>
         <v/>
       </c>
       <c r="G50" s="42">
-        <f>G45*(1-G11)</f>
+        <f>'NOPAT Bridge'!H37</f>
         <v/>
       </c>
       <c r="H50" s="42">
-        <f>H45*(1-H11)</f>
+        <f>H45*(1-'NOPAT Bridge'!H$35)</f>
         <v/>
       </c>
     </row>
@@ -3156,15 +3171,15 @@
         </is>
       </c>
       <c r="F51" s="42">
-        <f>F46*(1-F11)</f>
+        <f>F46*(1-'NOPAT Bridge'!I$35)</f>
         <v/>
       </c>
       <c r="G51" s="42">
-        <f>G46*(1-G11)</f>
+        <f>'NOPAT Bridge'!I37</f>
         <v/>
       </c>
       <c r="H51" s="42">
-        <f>H46*(1-H11)</f>
+        <f>H46*(1-'NOPAT Bridge'!I$35)</f>
         <v/>
       </c>
     </row>
@@ -3175,15 +3190,15 @@
         </is>
       </c>
       <c r="F52" s="42">
-        <f>F47*(1-F11)</f>
+        <f>F47*(1-'NOPAT Bridge'!J$35)</f>
         <v/>
       </c>
       <c r="G52" s="42">
-        <f>G47*(1-G11)</f>
+        <f>'NOPAT Bridge'!J37</f>
         <v/>
       </c>
       <c r="H52" s="42">
-        <f>H47*(1-H11)</f>
+        <f>H47*(1-'NOPAT Bridge'!J$35)</f>
         <v/>
       </c>
     </row>
@@ -7051,6 +7066,1382 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col hidden="1" outlineLevel="1" width="26" customWidth="1" min="2" max="2"/>
+    <col hidden="1" outlineLevel="1" width="16" customWidth="1" min="3" max="3"/>
+    <col hidden="1" outlineLevel="1" width="38" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>NOPAT NORMALIZATION PIPELINE (BASE CASE)</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="13" t="n"/>
+      <c r="H1" s="13" t="n"/>
+      <c r="I1" s="13" t="n"/>
+      <c r="J1" s="13" t="n"/>
+    </row>
+    <row r="2">
+      <c r="B2" s="50" t="inlineStr">
+        <is>
+          <t>Justification  [cols B–D: click + to expand]</t>
+        </is>
+      </c>
+      <c r="C2" s="50" t="inlineStr">
+        <is>
+          <t>Source (click)</t>
+        </is>
+      </c>
+      <c r="D2" s="50" t="inlineStr">
+        <is>
+          <t>Ctrl+F (prove number)</t>
+        </is>
+      </c>
+      <c r="E2" s="70" t="inlineStr">
+        <is>
+          <t>FY2025A</t>
+        </is>
+      </c>
+      <c r="F2" s="71" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="G2" s="71" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="H2" s="71" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="I2" s="71" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="J2" s="71" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="51" t="inlineStr">
+        <is>
+          <t>Reported EBIT → Normalized NOPAT (5-phase pipeline)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Phases 1–4 clean and forecast operating profit; Phase 5 is the agent workflow summary below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="51" t="inlineStr">
+        <is>
+          <t>Driver assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Phase 1: Add back SBC? (1 = yes; diluted-shares / UFCF convention)</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Not % of revenue — SBC add-back flag (1 = yes). UFCF uses diluted shares; add back non-cash SBC to EBIT. FY25 SBC $62,203k scaled with revenue in forecast.</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>LULU CF statement (10-K): stock-based compensation</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Stock-based compensation expense"
+→ 62,203 ($000). Flag = 1 adds back to EBIT (diluted-shares UFCF convention).</t>
+        </is>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Phase 3: Store-channel EBIT margin %</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>18.6% EBIT margin on store-channel revenue. Calibrated so FY25 channel EBIT ≈ reported EBIT.</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge tab: channel margin calibration</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Channel margin assumption — calibrated so FY25 store rev × 18.6% + e-comm × 23.6% + other × 9.1% ≈ reported EBIT.</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="G8" s="20" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="I8" s="20" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="J8" s="20" t="n">
+        <v>0.186</v>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Phase 3: E-commerce EBIT margin %</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>23.6% EBIT margin on e-commerce revenue. Higher than stores (no occupancy).</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge tab: channel margin calibration</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>E-commerce EBIT margin 23.6% — higher than stores (no occupancy drag).</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="G9" s="20" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="I9" s="20" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="J9" s="20" t="n">
+        <v>0.236</v>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Phase 3: Other-channels EBIT margin %</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>9.1% EBIT margin on wholesale/license/outlets — lower-margin residual channel.</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge tab: channel margin calibration</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Other channels 9.1% — wholesale/license/outlets residual margin.</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="F10" s="20" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="G10" s="20" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="I10" s="20" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="J10" s="20" t="n">
+        <v>0.091</v>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Phase 4: Terminal marginal tax rate</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>30% statutory marginal rate. t_operating transitions here over the 5-year forecast.</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>Q2 FY2026 outlook: tax rate ≈ 30%</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "a tax rate of approximately 30%" → terminal marginal rate for t_operating glide path.</t>
+        </is>
+      </c>
+      <c r="E11" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F11" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G11" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H11" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I11" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J11" s="20" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Phase 2: R&amp;D / software amortization period (years)</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Not % of revenue — amortization period (years) if R&amp;D/software is capitalized. LULU: no separate R&amp;D cap.</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge: capitalization convention</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Amortization period if R&amp;D capitalized (3–5 yr convention). LULU: no separate R&amp;D capitalization.</t>
+        </is>
+      </c>
+      <c r="E12" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="H12" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="I12" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="J12" s="40" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" hidden="1" outlineLevel="1">
+      <c r="A14" s="72" t="inlineStr">
+        <is>
+          <t>Phase 1 — Operating normalization</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Reported operating income (EBIT)</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>FY25: reported operating income from 10-K. Forecast: Scenarios base-case EBIT (margin path).</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: Income from operations</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Income from operations" → 2,210,615 ($000). Forecast links to Scenarios EBIT.</t>
+        </is>
+      </c>
+      <c r="E15" s="73" t="n">
+        <v>2210615</v>
+      </c>
+      <c r="F15" s="74">
+        <f>Scenarios!G43</f>
+        <v/>
+      </c>
+      <c r="G15" s="74">
+        <f>Scenarios!G44</f>
+        <v/>
+      </c>
+      <c r="H15" s="74">
+        <f>Scenarios!G45</f>
+        <v/>
+      </c>
+      <c r="I15" s="74">
+        <f>Scenarios!G46</f>
+        <v/>
+      </c>
+      <c r="J15" s="74">
+        <f>Scenarios!G47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>+ Impairment / intangible amortization (add-back)</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Add back intangible amortization / impairments. FY25 = other operating expense amortization run-rate.</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: amortization of intangible assets</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Amortization of intangible assets" → other operating expense run-rate (add-back).</t>
+        </is>
+      </c>
+      <c r="E16" s="73" t="n">
+        <v>6961</v>
+      </c>
+      <c r="F16" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>+ Restructuring costs (add-back)</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Add back restructuring (severance, store closures). LULU FY25: none identified.</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: restructuring charges</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "restructuring" → none material in FY25 10-K.</t>
+        </is>
+      </c>
+      <c r="E17" s="73" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>+ Legal / M&amp;A one-offs (add-back)</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>Strip one-off legal / M&amp;A advisory fees. LULU FY25: none identified.</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: SG&amp;A one-offs</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>One-off legal/M&amp;A fees in SG&amp;A — none identified FY25.</t>
+        </is>
+      </c>
+      <c r="E18" s="73" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" hidden="1" outlineLevel="1" ht="42" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>+ Stock-based compensation (add-back if flag = 1)</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Not % of revenue — SBC add-back flag (1 = yes). UFCF uses diluted shares; add back non-cash SBC to EBIT. FY25 SBC $62,203k scaled with revenue in forecast.</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>LULU CF statement (10-K): stock-based compensation</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Stock-based compensation expense"
+→ 62,203 ($000). Flag = 1 adds back to EBIT (diluted-shares UFCF convention).</t>
+        </is>
+      </c>
+      <c r="E19" s="73" t="n">
+        <v>62203</v>
+      </c>
+      <c r="F19" s="74">
+        <f>Scenarios!G23/11102600*62203*$E$7</f>
+        <v/>
+      </c>
+      <c r="G19" s="74">
+        <f>Scenarios!G24/11102600*62203*$E$7</f>
+        <v/>
+      </c>
+      <c r="H19" s="74">
+        <f>Scenarios!G25/11102600*62203*$E$7</f>
+        <v/>
+      </c>
+      <c r="I19" s="74">
+        <f>Scenarios!G26/11102600*62203*$E$7</f>
+        <v/>
+      </c>
+      <c r="J19" s="74">
+        <f>Scenarios!G27/11102600*62203*$E$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A20" s="23">
+        <f> Adjusted EBIT (Phase 1)</f>
+        <v/>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Phase 1 adjusted EBIT = reported + non-recurring add-backs + optional SBC.</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge tab: Phase 1 subtotal</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Sum of reported EBIT + Phase 1 add-backs on this tab.</t>
+        </is>
+      </c>
+      <c r="F20" s="25">
+        <f>F15+F16+F17+F18+F19</f>
+        <v/>
+      </c>
+      <c r="G20" s="25">
+        <f>G15+G16+G17+G18+G19</f>
+        <v/>
+      </c>
+      <c r="H20" s="25">
+        <f>H15+H16+H17+H18+H19</f>
+        <v/>
+      </c>
+      <c r="I20" s="25">
+        <f>I15+I16+I17+I18+I19</f>
+        <v/>
+      </c>
+      <c r="J20" s="25">
+        <f>J15+J16+J17+J18+J19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" hidden="1" outlineLevel="1">
+      <c r="A21" s="72" t="inlineStr">
+        <is>
+          <t>Phase 2 — Lease &amp; capitalization (ASC 842 / IFRS 16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" hidden="1" outlineLevel="1" ht="42" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>+ Implied lease interest expense (reclass from rent)</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>Not % of revenue — implied lease interest ($1,028k FY25). Reclass from rent to unlevered EBIT; scales with revenue in forecast.</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: interest on lease liabilities (supplemental)</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "Interest paid on lease liabilities"
+→ 1,028 ($000) supplemental cash-flow disclosure. Reclass to unlevered EBIT.</t>
+        </is>
+      </c>
+      <c r="E22" s="73" t="n">
+        <v>1028</v>
+      </c>
+      <c r="F22" s="74">
+        <f>1028*(Scenarios!G23/11102600)</f>
+        <v/>
+      </c>
+      <c r="G22" s="74">
+        <f>1028*(Scenarios!G24/11102600)</f>
+        <v/>
+      </c>
+      <c r="H22" s="74">
+        <f>1028*(Scenarios!G25/11102600)</f>
+        <v/>
+      </c>
+      <c r="I22" s="74">
+        <f>1028*(Scenarios!G26/11102600)</f>
+        <v/>
+      </c>
+      <c r="J22" s="74">
+        <f>1028*(Scenarios!G27/11102600)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>+ Capitalize R&amp;D / software (current-year expense)</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>Capitalize multi-year software/R&amp;D. LULU: immaterial separate R&amp;D line — held at $0.</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: R&amp;D / software expense</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>R&amp;D / software capitalization — LULU immaterial; held at $0.</t>
+        </is>
+      </c>
+      <c r="E23" s="73" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>− Amortization of prior capitalized intangibles</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>Amortization of prior capitalized intangibles. LULU: flows through existing D&amp;A.</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: intangible amortization</t>
+        </is>
+      </c>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>Amortization of prior capitalized intangibles — netted in D&amp;A line.</t>
+        </is>
+      </c>
+      <c r="E24" s="73" t="n">
+        <v>6961</v>
+      </c>
+      <c r="F24" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A25" s="23">
+        <f> EBIT after lease &amp; capitalization (Phase 2)</f>
+        <v/>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Phase 2 EBIT = Phase 1 + lease interest reclass + R&amp;D cap − amortization.</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge tab: Phase 2 subtotal</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>Phase 1 + lease interest + R&amp;D cap − amortization.</t>
+        </is>
+      </c>
+      <c r="F25" s="25">
+        <f>F20+F22+F23-F24</f>
+        <v/>
+      </c>
+      <c r="G25" s="25">
+        <f>G20+G22+G23-G24</f>
+        <v/>
+      </c>
+      <c r="H25" s="25">
+        <f>H20+H22+H23-H24</f>
+        <v/>
+      </c>
+      <c r="I25" s="25">
+        <f>I20+I22+I23-I24</f>
+        <v/>
+      </c>
+      <c r="J25" s="25">
+        <f>J20+J22+J23-J24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" hidden="1" outlineLevel="1">
+      <c r="A26" s="72" t="inlineStr">
+        <is>
+          <t>Phase 3 — Segment / channel EBIT (driver-based)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Store-channel revenue</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>Not % of revenue — store-channel revenue from Revenue Drivers tab.</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab: store-channel revenue</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab → store-channel revenue row.</t>
+        </is>
+      </c>
+      <c r="E27" s="73" t="n">
+        <v>5049744</v>
+      </c>
+      <c r="F27" s="74">
+        <f>'Revenue Drivers'!F31</f>
+        <v/>
+      </c>
+      <c r="G27" s="74">
+        <f>'Revenue Drivers'!G31</f>
+        <v/>
+      </c>
+      <c r="H27" s="74">
+        <f>'Revenue Drivers'!H31</f>
+        <v/>
+      </c>
+      <c r="I27" s="74">
+        <f>'Revenue Drivers'!I31</f>
+        <v/>
+      </c>
+      <c r="J27" s="74">
+        <f>'Revenue Drivers'!J31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  E-commerce revenue</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Not % of revenue — e-commerce revenue from Revenue Drivers tab.</t>
+        </is>
+      </c>
+      <c r="C28" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab: e-commerce revenue</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab → e-commerce revenue row.</t>
+        </is>
+      </c>
+      <c r="E28" s="73" t="n">
+        <v>4918697</v>
+      </c>
+      <c r="F28" s="74">
+        <f>'Revenue Drivers'!F41</f>
+        <v/>
+      </c>
+      <c r="G28" s="74">
+        <f>'Revenue Drivers'!G41</f>
+        <v/>
+      </c>
+      <c r="H28" s="74">
+        <f>'Revenue Drivers'!H41</f>
+        <v/>
+      </c>
+      <c r="I28" s="74">
+        <f>'Revenue Drivers'!I41</f>
+        <v/>
+      </c>
+      <c r="J28" s="74">
+        <f>'Revenue Drivers'!J41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Other channels revenue</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>Not % of revenue — wholesale/license/outlet revenue from Revenue Drivers tab.</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab: other channels revenue</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab → other channels revenue row.</t>
+        </is>
+      </c>
+      <c r="E29" s="73" t="n">
+        <v>1134159</v>
+      </c>
+      <c r="F29" s="74">
+        <f>'Revenue Drivers'!F45</f>
+        <v/>
+      </c>
+      <c r="G29" s="74">
+        <f>'Revenue Drivers'!G45</f>
+        <v/>
+      </c>
+      <c r="H29" s="74">
+        <f>'Revenue Drivers'!H45</f>
+        <v/>
+      </c>
+      <c r="I29" s="74">
+        <f>'Revenue Drivers'!I45</f>
+        <v/>
+      </c>
+      <c r="J29" s="74">
+        <f>'Revenue Drivers'!J45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Channel EBIT (= Sum Rev_i x Margin_i)</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>Phase 3 channel EBIT = Σ(Revenue_i × Margin_i). FY26 adds Scenarios tariff refund.</t>
+        </is>
+      </c>
+      <c r="C30" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge tab: channel EBIT formula</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Σ channel revenue × margin. FY26 adds Scenarios tariff refund cell.</t>
+        </is>
+      </c>
+      <c r="F30" s="69">
+        <f>F27*E$8+F28*E$9+F29*E$10+Scenarios!G7</f>
+        <v/>
+      </c>
+      <c r="G30" s="69">
+        <f>G27*E$8+G28*E$9+G29*E$10</f>
+        <v/>
+      </c>
+      <c r="H30" s="69">
+        <f>H27*E$8+H28*E$9+H29*E$10</f>
+        <v/>
+      </c>
+      <c r="I30" s="69">
+        <f>I27*E$8+I28*E$9+I29*E$10</f>
+        <v/>
+      </c>
+      <c r="J30" s="69">
+        <f>J27*E$8+J28*E$9+J29*E$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A31" s="23">
+        <f> EBIT after channel mix (Phase 3)</f>
+        <v/>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>Channel-mix EBIT output (Phase 3). Check row vs Scenarios shows channel vs margin-path gap.</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge tab: Phase 3 subtotal</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>Channel EBIT subtotal (Phase 3). Compare Check row vs Scenarios.</t>
+        </is>
+      </c>
+      <c r="E31" s="75" t="n">
+        <v>2203273.345</v>
+      </c>
+      <c r="F31" s="25">
+        <f>F30</f>
+        <v/>
+      </c>
+      <c r="G31" s="25">
+        <f>G30</f>
+        <v/>
+      </c>
+      <c r="H31" s="25">
+        <f>H30</f>
+        <v/>
+      </c>
+      <c r="I31" s="25">
+        <f>I30</f>
+        <v/>
+      </c>
+      <c r="J31" s="25">
+        <f>J30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A32" s="23">
+        <f> Normalized EBIT (tax base for NOPAT)</f>
+        <v/>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>FY25: Phases 1–2 walk-through. Forecast: Scenarios base EBIT — tax base for NOPAT.</t>
+        </is>
+      </c>
+      <c r="C32" s="24" t="inlineStr">
+        <is>
+          <t>Scenarios tab: base-case EBIT (forecast)</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>FY25: Phase 1–2 formula. Forecast: Scenarios base EBIT (tax base).</t>
+        </is>
+      </c>
+      <c r="E32" s="25">
+        <f>E20+E22+E23-E24</f>
+        <v/>
+      </c>
+      <c r="F32" s="25">
+        <f>Scenarios!G43</f>
+        <v/>
+      </c>
+      <c r="G32" s="25">
+        <f>Scenarios!G44</f>
+        <v/>
+      </c>
+      <c r="H32" s="25">
+        <f>Scenarios!G45</f>
+        <v/>
+      </c>
+      <c r="I32" s="25">
+        <f>Scenarios!G46</f>
+        <v/>
+      </c>
+      <c r="J32" s="25">
+        <f>Scenarios!G47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" hidden="1" outlineLevel="1">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Check vs Scenarios EBIT (base case)</t>
+        </is>
+      </c>
+      <c r="F33" s="74">
+        <f>F32-Scenarios!G43</f>
+        <v/>
+      </c>
+      <c r="G33" s="74">
+        <f>G32-Scenarios!G44</f>
+        <v/>
+      </c>
+      <c r="H33" s="74">
+        <f>H32-Scenarios!G45</f>
+        <v/>
+      </c>
+      <c r="I33" s="74">
+        <f>I32-Scenarios!G46</f>
+        <v/>
+      </c>
+      <c r="J33" s="74">
+        <f>J32-Scenarios!G47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" hidden="1" outlineLevel="1">
+      <c r="A34" s="72" t="inlineStr">
+        <is>
+          <t>Phase 4 — Tax normalization to NOPAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" hidden="1" outlineLevel="1" ht="70" customHeight="1">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>Operating effective tax rate (t_operating)</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Operating effective tax rate: (tax + interest shield) ÷ (EBT + interest). Transitions from FY25 t_operating toward 30% marginal over 5 years.</t>
+        </is>
+      </c>
+      <c r="C35" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: income tax &amp; interest expense</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>t_operating = (tax + interest×30%) ÷ (EBT + interest).
+Ctrl+F "Income tax expense" → 659,784
+Ctrl+F "Income before income tax expense" → 2,238,967
+Ctrl+F "Interest paid on lease liabilities" → 1,028</t>
+        </is>
+      </c>
+      <c r="E35" s="76" t="n">
+        <v>0.2946847649213503</v>
+      </c>
+      <c r="F35" s="32">
+        <f>0.29468476492135026+(F$11-0.29468476492135026)*1/5</f>
+        <v/>
+      </c>
+      <c r="G35" s="32">
+        <f>0.29468476492135026+(G$11-0.29468476492135026)*2/5</f>
+        <v/>
+      </c>
+      <c r="H35" s="32">
+        <f>0.29468476492135026+(H$11-0.29468476492135026)*3/5</f>
+        <v/>
+      </c>
+      <c r="I35" s="32">
+        <f>0.29468476492135026+(I$11-0.29468476492135026)*4/5</f>
+        <v/>
+      </c>
+      <c r="J35" s="32">
+        <f>0.29468476492135026+(J$11-0.29468476492135026)*5/5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>Unlevered tax on normalized EBIT</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>Unlevered tax = normalized EBIT × t_operating. Strips debt-interest tax shield from GAAP rate.</t>
+        </is>
+      </c>
+      <c r="C36" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge tab: unlevered tax expense</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>Normalized EBIT × t_operating — unlevered tax (no debt shield).</t>
+        </is>
+      </c>
+      <c r="F36" s="74">
+        <f>F32*F35</f>
+        <v/>
+      </c>
+      <c r="G36" s="74">
+        <f>G32*G35</f>
+        <v/>
+      </c>
+      <c r="H36" s="74">
+        <f>H32*H35</f>
+        <v/>
+      </c>
+      <c r="I36" s="74">
+        <f>I32*I35</f>
+        <v/>
+      </c>
+      <c r="J36" s="74">
+        <f>J32*J35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A37" s="23" t="inlineStr">
+        <is>
+          <t>NORMALIZED NOPAT</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>NORMALIZED NOPAT = EBIT_norm × (1 − t_operating). Scenarios base case links here.</t>
+        </is>
+      </c>
+      <c r="C37" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge tab: normalized NOPAT</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
+        <is>
+          <t>EBIT_norm − unlevered tax. Scenarios base-case NOPAT links to this row.</t>
+        </is>
+      </c>
+      <c r="F37" s="25">
+        <f>F32-F36</f>
+        <v/>
+      </c>
+      <c r="G37" s="25">
+        <f>G32-G36</f>
+        <v/>
+      </c>
+      <c r="H37" s="25">
+        <f>H32-H36</f>
+        <v/>
+      </c>
+      <c r="I37" s="25">
+        <f>I32-I36</f>
+        <v/>
+      </c>
+      <c r="J37" s="25">
+        <f>J32-J36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="72" t="inlineStr">
+        <is>
+          <t>Phase 5 — Agent workflow (execution steps)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="60" t="inlineStr">
+        <is>
+          <t>1. Clean base</t>
+        </is>
+      </c>
+      <c r="B40" s="77" t="inlineStr">
+        <is>
+          <t>SEC 10-K income statement</t>
+        </is>
+      </c>
+      <c r="D40" s="26" t="inlineStr">
+        <is>
+          <t>Add back impairments, restructuring, M&amp;A; optional SBC add-back.</t>
+        </is>
+      </c>
+      <c r="F40" s="78" t="inlineStr">
+        <is>
+          <t>EBIT_adj (Phase 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="60" t="inlineStr">
+        <is>
+          <t>2. Capitalize R&amp;D</t>
+        </is>
+      </c>
+      <c r="B41" s="77" t="inlineStr">
+        <is>
+          <t>SG&amp;A footnotes</t>
+        </is>
+      </c>
+      <c r="D41" s="26" t="inlineStr">
+        <is>
+          <t>Capitalize multi-year software/R&amp;D; amortize over N years.</t>
+        </is>
+      </c>
+      <c r="F41" s="78" t="inlineStr">
+        <is>
+          <t>EBIT_lease-adj (Phase 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="60" t="inlineStr">
+        <is>
+          <t>3. Lease shift</t>
+        </is>
+      </c>
+      <c r="B42" s="77" t="inlineStr">
+        <is>
+          <t>ASC 842 lease footnote</t>
+        </is>
+      </c>
+      <c r="D42" s="26" t="inlineStr">
+        <is>
+          <t>Add implied lease interest; standardize to unlevered EBIT.</t>
+        </is>
+      </c>
+      <c r="F42" s="78" t="inlineStr">
+        <is>
+          <t>EBIT_capitalized</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="60" t="inlineStr">
+        <is>
+          <t>4. Segment mix</t>
+        </is>
+      </c>
+      <c r="B43" s="77" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab</t>
+        </is>
+      </c>
+      <c r="D43" s="26" t="inlineStr">
+        <is>
+          <t>Blend store / e-comm / other EBIT margins by channel revenue share.</t>
+        </is>
+      </c>
+      <c r="F43" s="78" t="inlineStr">
+        <is>
+          <t>Forecast EBIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="60" t="inlineStr">
+        <is>
+          <t>5. NOPAT bridge</t>
+        </is>
+      </c>
+      <c r="B44" s="77" t="inlineStr">
+        <is>
+          <t>Normalized EBIT &amp; t_operating</t>
+        </is>
+      </c>
+      <c r="D44" s="26" t="inlineStr">
+        <is>
+          <t>NOPAT = EBIT x (1 - t); transition t toward marginal rate.</t>
+        </is>
+      </c>
+      <c r="F44" s="78" t="inlineStr">
+        <is>
+          <t>Normalized NOPAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="26" t="inlineStr">
+        <is>
+          <t>Scenarios base-case NOPAT (col G) links to NORMALIZED NOPAT above. Bear/bull apply the same t_operating to their EBIT paths.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId18"/>
+    <hyperlink ref="C27" location="'Revenue Drivers'!B31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId19"/>
+    <hyperlink ref="C28" location="'Revenue Drivers'!B41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId20"/>
+    <hyperlink ref="C29" location="'Revenue Drivers'!B45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId24"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7086,69 +8477,69 @@
       <c r="J1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="B2" s="70" t="inlineStr">
+      <c r="B2" s="79" t="inlineStr">
         <is>
           <t>Justification (~20 words)  [cols B–D: click + to expand]</t>
         </is>
       </c>
-      <c r="C2" s="70" t="inlineStr">
+      <c r="C2" s="79" t="inlineStr">
         <is>
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D2" s="70" t="inlineStr">
+      <c r="D2" s="79" t="inlineStr">
         <is>
           <t>Ctrl+F (prove number)</t>
         </is>
       </c>
-      <c r="E2" s="71" t="inlineStr">
+      <c r="E2" s="70" t="inlineStr">
         <is>
           <t>FY2025A</t>
         </is>
       </c>
-      <c r="F2" s="72" t="inlineStr">
+      <c r="F2" s="71" t="inlineStr">
         <is>
           <t>FY2026E</t>
         </is>
       </c>
-      <c r="G2" s="72" t="inlineStr">
+      <c r="G2" s="71" t="inlineStr">
         <is>
           <t>FY2027E</t>
         </is>
       </c>
-      <c r="H2" s="72" t="inlineStr">
+      <c r="H2" s="71" t="inlineStr">
         <is>
           <t>FY2028E</t>
         </is>
       </c>
-      <c r="I2" s="72" t="inlineStr">
+      <c r="I2" s="71" t="inlineStr">
         <is>
           <t>FY2029E</t>
         </is>
       </c>
-      <c r="J2" s="72" t="inlineStr">
+      <c r="J2" s="71" t="inlineStr">
         <is>
           <t>FY2030E</t>
         </is>
       </c>
-      <c r="K2" s="73" t="inlineStr">
+      <c r="K2" s="80" t="inlineStr">
         <is>
           <t>Δ vs Scenarios</t>
         </is>
       </c>
-      <c r="L2" s="70" t="inlineStr">
+      <c r="L2" s="79" t="inlineStr">
         <is>
           <t>Alt. source  [cols L–M: click + to expand]</t>
         </is>
       </c>
-      <c r="M2" s="70" t="inlineStr">
+      <c r="M2" s="79" t="inlineStr">
         <is>
           <t>Alt. Ctrl+F</t>
         </is>
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="74" t="inlineStr">
+      <c r="A3" s="81" t="inlineStr">
         <is>
           <t>Forecast drivers linked to Scenarios tab → Base case (column G)</t>
         </is>
@@ -7158,12 +8549,12 @@
           <t>Ctrl+F "Net revenue" → 11,102,600 or "Depreciation and amortization" → 496,228 on this 10-K HTML file</t>
         </is>
       </c>
-      <c r="E3" s="75" t="inlineStr">
+      <c r="E3" s="82" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
       </c>
-      <c r="K3" s="76" t="inlineStr">
+      <c r="K3" s="83" t="inlineStr">
         <is>
           <t>(should be 0)</t>
         </is>
@@ -7176,7 +8567,13 @@
 Ctrl+F: Every red assumption on every tab — justification, source link, Ctrl+F proof.</t>
         </is>
       </c>
-      <c r="C4" s="77" t="inlineStr">
+      <c r="C4" s="84" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge tab
+Ctrl+F: 5-phase EBIT normalization → normalized NOPAT (base case).</t>
+        </is>
+      </c>
+      <c r="D4" s="84" t="inlineStr">
         <is>
           <t>Revenue Drivers tab
 Ctrl+F: Bottom-up store / DTC / category schedule (FY26–30).</t>
@@ -7189,30 +8586,30 @@
           <t>Net revenue</t>
         </is>
       </c>
-      <c r="E5" s="78" t="n">
+      <c r="E5" s="73" t="n">
         <v>11102600</v>
       </c>
-      <c r="F5" s="79">
+      <c r="F5" s="74">
         <f>Scenarios!G23</f>
         <v/>
       </c>
-      <c r="G5" s="79">
+      <c r="G5" s="74">
         <f>Scenarios!G24</f>
         <v/>
       </c>
-      <c r="H5" s="79">
+      <c r="H5" s="74">
         <f>Scenarios!G25</f>
         <v/>
       </c>
-      <c r="I5" s="79">
+      <c r="I5" s="74">
         <f>Scenarios!G26</f>
         <v/>
       </c>
-      <c r="J5" s="79">
+      <c r="J5" s="74">
         <f>Scenarios!G27</f>
         <v/>
       </c>
-      <c r="K5" s="80">
+      <c r="K5" s="85">
         <f>IF(MAX(ABS(F5-Scenarios!$G$23),ABS(G5-Scenarios!$G$24),ABS(H5-Scenarios!$G$25),ABS(I5-Scenarios!$G$26),ABS(J5-Scenarios!$G$27))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -7289,7 +8686,7 @@
 → 4,818,468 ($000)</t>
         </is>
       </c>
-      <c r="E7" s="81" t="n">
+      <c r="E7" s="76" t="n">
         <v>0.566005440167168</v>
       </c>
       <c r="F7" s="20">
@@ -7319,30 +8716,30 @@
           <t>Cost of goods sold (COGS)</t>
         </is>
       </c>
-      <c r="E8" s="78" t="n">
+      <c r="E8" s="73" t="n">
         <v>4818468</v>
       </c>
-      <c r="F8" s="79">
+      <c r="F8" s="74">
         <f>Scenarios!G33</f>
         <v/>
       </c>
-      <c r="G8" s="79">
+      <c r="G8" s="74">
         <f>Scenarios!G34</f>
         <v/>
       </c>
-      <c r="H8" s="79">
+      <c r="H8" s="74">
         <f>Scenarios!G35</f>
         <v/>
       </c>
-      <c r="I8" s="79">
+      <c r="I8" s="74">
         <f>Scenarios!G36</f>
         <v/>
       </c>
-      <c r="J8" s="79">
+      <c r="J8" s="74">
         <f>Scenarios!G37</f>
         <v/>
       </c>
-      <c r="K8" s="80">
+      <c r="K8" s="85">
         <f>IF(MAX(ABS(F8-Scenarios!$G$33),ABS(G8-Scenarios!$G$34),ABS(H8-Scenarios!$G$35),ABS(I8-Scenarios!$G$36),ABS(J8-Scenarios!$G$37))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -7391,7 +8788,7 @@
         <f>Scenarios!G42</f>
         <v/>
       </c>
-      <c r="K9" s="80">
+      <c r="K9" s="85">
         <f>IF(MAX(ABS(F9-Scenarios!$G$38),ABS(G9-Scenarios!$G$39),ABS(H9-Scenarios!$G$40),ABS(I9-Scenarios!$G$41),ABS(J9-Scenarios!$G$42))&lt;0.0001,"OK","CHECK")</f>
         <v/>
       </c>
@@ -7417,7 +8814,7 @@
           <t>Ctrl+F "134.5 million" → IEEPA tariff refunds reduced COGS. Add this dollar amount to FY26 EBIT only. Full-year boost = 134.5 / FY26 sales ≈ 1.3ppt, not 5.6ppt.</t>
         </is>
       </c>
-      <c r="E10" s="78" t="n">
+      <c r="E10" s="73" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="37">
@@ -7443,7 +8840,7 @@
           <t>EBIT (incl. FY26 refund)</t>
         </is>
       </c>
-      <c r="E11" s="82" t="n">
+      <c r="E11" s="75" t="n">
         <v>2210615</v>
       </c>
       <c r="F11" s="25">
@@ -7466,7 +8863,7 @@
         <f>Scenarios!G47</f>
         <v/>
       </c>
-      <c r="K11" s="83">
+      <c r="K11" s="86">
         <f>IF(MAX(ABS(F11-Scenarios!$G$43),ABS(G11-Scenarios!$G$44),ABS(H11-Scenarios!$G$45),ABS(I11-Scenarios!$G$46),ABS(J11-Scenarios!$G$47))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -7477,7 +8874,7 @@
           <t>Reported EBIT margin % (incl. FY26 refund)</t>
         </is>
       </c>
-      <c r="E12" s="81" t="n">
+      <c r="E12" s="76" t="n">
         <v>0.1991078666258354</v>
       </c>
       <c r="F12" s="32">
@@ -7504,27 +8901,27 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Less: cash taxes on EBIT</t>
-        </is>
-      </c>
-      <c r="F13" s="79">
-        <f>-Scenarios!G43*Scenarios!$G$11</f>
-        <v/>
-      </c>
-      <c r="G13" s="79">
-        <f>-Scenarios!G44*Scenarios!$G$11</f>
-        <v/>
-      </c>
-      <c r="H13" s="79">
-        <f>-Scenarios!G45*Scenarios!$G$11</f>
-        <v/>
-      </c>
-      <c r="I13" s="79">
-        <f>-Scenarios!G46*Scenarios!$G$11</f>
-        <v/>
-      </c>
-      <c r="J13" s="79">
-        <f>-Scenarios!G47*Scenarios!$G$11</f>
+          <t>Less: unlevered tax (t_operating from NOPAT Bridge)</t>
+        </is>
+      </c>
+      <c r="F13" s="74">
+        <f>-'NOPAT Bridge'!F36</f>
+        <v/>
+      </c>
+      <c r="G13" s="74">
+        <f>-'NOPAT Bridge'!G36</f>
+        <v/>
+      </c>
+      <c r="H13" s="74">
+        <f>-'NOPAT Bridge'!H36</f>
+        <v/>
+      </c>
+      <c r="I13" s="74">
+        <f>-'NOPAT Bridge'!I36</f>
+        <v/>
+      </c>
+      <c r="J13" s="74">
+        <f>-'NOPAT Bridge'!J36</f>
         <v/>
       </c>
     </row>
@@ -7554,7 +8951,7 @@
         <f>Scenarios!G52</f>
         <v/>
       </c>
-      <c r="K14" s="83">
+      <c r="K14" s="86">
         <f>IF(MAX(ABS(F14-Scenarios!$G$48),ABS(G14-Scenarios!$G$49),ABS(H14-Scenarios!$G$50),ABS(I14-Scenarios!$G$51),ABS(J14-Scenarios!$G$52))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -7607,27 +9004,27 @@
           <t>Plus: depreciation &amp; amortization</t>
         </is>
       </c>
-      <c r="F16" s="79">
+      <c r="F16" s="74">
         <f>Scenarios!G53</f>
         <v/>
       </c>
-      <c r="G16" s="79">
+      <c r="G16" s="74">
         <f>Scenarios!G54</f>
         <v/>
       </c>
-      <c r="H16" s="79">
+      <c r="H16" s="74">
         <f>Scenarios!G55</f>
         <v/>
       </c>
-      <c r="I16" s="79">
+      <c r="I16" s="74">
         <f>Scenarios!G56</f>
         <v/>
       </c>
-      <c r="J16" s="79">
+      <c r="J16" s="74">
         <f>Scenarios!G57</f>
         <v/>
       </c>
-      <c r="K16" s="80">
+      <c r="K16" s="85">
         <f>IF(MAX(ABS(F16-Scenarios!$G$53),ABS(G16-Scenarios!$G$54),ABS(H16-Scenarios!$G$55),ABS(I16-Scenarios!$G$56),ABS(J16-Scenarios!$G$57))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -7693,27 +9090,27 @@
           <t>Less: capital expenditures</t>
         </is>
       </c>
-      <c r="F18" s="79">
+      <c r="F18" s="74">
         <f>-Scenarios!G58</f>
         <v/>
       </c>
-      <c r="G18" s="79">
+      <c r="G18" s="74">
         <f>-Scenarios!G59</f>
         <v/>
       </c>
-      <c r="H18" s="79">
+      <c r="H18" s="74">
         <f>-Scenarios!G60</f>
         <v/>
       </c>
-      <c r="I18" s="79">
+      <c r="I18" s="74">
         <f>-Scenarios!G61</f>
         <v/>
       </c>
-      <c r="J18" s="79">
+      <c r="J18" s="74">
         <f>-Scenarios!G62</f>
         <v/>
       </c>
-      <c r="K18" s="80">
+      <c r="K18" s="85">
         <f>IF(MAX(ABS(F18+Scenarios!$G$58),ABS(G18+Scenarios!$G$59),ABS(H18+Scenarios!$G$60),ABS(I18+Scenarios!$G$61),ABS(J18+Scenarios!$G$62))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -7755,7 +9152,7 @@
 Ctrl+F "E-commerce"</t>
         </is>
       </c>
-      <c r="E20" s="84" t="n">
+      <c r="E20" s="87" t="n">
         <v>6.267883648875038</v>
       </c>
       <c r="F20" s="28">
@@ -7778,7 +9175,7 @@
         <f>Scenarios!G67</f>
         <v/>
       </c>
-      <c r="K20" s="80">
+      <c r="K20" s="85">
         <f>IF(MAX(ABS(F20-Scenarios!$G$63),ABS(G20-Scenarios!$G$64),ABS(H20-Scenarios!$G$65),ABS(I20-Scenarios!$G$66),ABS(J20-Scenarios!$G$67))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -7809,30 +9206,30 @@
 → 11,102,600 ($000)</t>
         </is>
       </c>
-      <c r="E21" s="78" t="n">
+      <c r="E21" s="73" t="n">
         <v>190657</v>
       </c>
-      <c r="F21" s="79">
+      <c r="F21" s="74">
         <f>Scenarios!G68</f>
         <v/>
       </c>
-      <c r="G21" s="79">
+      <c r="G21" s="74">
         <f>Scenarios!G69</f>
         <v/>
       </c>
-      <c r="H21" s="79">
+      <c r="H21" s="74">
         <f>Scenarios!G70</f>
         <v/>
       </c>
-      <c r="I21" s="79">
+      <c r="I21" s="74">
         <f>Scenarios!G71</f>
         <v/>
       </c>
-      <c r="J21" s="79">
+      <c r="J21" s="74">
         <f>Scenarios!G72</f>
         <v/>
       </c>
-      <c r="K21" s="80">
+      <c r="K21" s="85">
         <f>IF(MAX(ABS(F21-Scenarios!$G$68),ABS(G21-Scenarios!$G$69),ABS(H21-Scenarios!$G$70),ABS(I21-Scenarios!$G$71),ABS(J21-Scenarios!$G$72))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -7878,7 +9275,7 @@
 Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
         </is>
       </c>
-      <c r="E22" s="84" t="n">
+      <c r="E22" s="87" t="n">
         <v>128.8324100108167</v>
       </c>
       <c r="F22" s="28">
@@ -7901,7 +9298,7 @@
         <f>Scenarios!G77</f>
         <v/>
       </c>
-      <c r="K22" s="80">
+      <c r="K22" s="85">
         <f>IF(MAX(ABS(F22-Scenarios!$G$73),ABS(G22-Scenarios!$G$74),ABS(H22-Scenarios!$G$75),ABS(I22-Scenarios!$G$76),ABS(J22-Scenarios!$G$77))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -7939,30 +9336,30 @@
 FY25 proof: (129 ÷ 365) × 4,818,468 ≈ 1,700,753</t>
         </is>
       </c>
-      <c r="E23" s="78" t="n">
+      <c r="E23" s="73" t="n">
         <v>1700753</v>
       </c>
-      <c r="F23" s="79">
+      <c r="F23" s="74">
         <f>Scenarios!G78</f>
         <v/>
       </c>
-      <c r="G23" s="79">
+      <c r="G23" s="74">
         <f>Scenarios!G79</f>
         <v/>
       </c>
-      <c r="H23" s="79">
+      <c r="H23" s="74">
         <f>Scenarios!G80</f>
         <v/>
       </c>
-      <c r="I23" s="79">
+      <c r="I23" s="74">
         <f>Scenarios!G81</f>
         <v/>
       </c>
-      <c r="J23" s="79">
+      <c r="J23" s="74">
         <f>Scenarios!G82</f>
         <v/>
       </c>
-      <c r="K23" s="80">
+      <c r="K23" s="85">
         <f>IF(MAX(ABS(F23-Scenarios!$G$78),ABS(G23-Scenarios!$G$79),ABS(H23-Scenarios!$G$80),ABS(I23-Scenarios!$G$81),ABS(J23-Scenarios!$G$82))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -7992,7 +9389,7 @@
 Not % of revenue — DPO ≈ 25.1 days. Implied AP ≈ 3.0% of sales / 6.9% of COGS.</t>
         </is>
       </c>
-      <c r="E24" s="84" t="n">
+      <c r="E24" s="87" t="n">
         <v>25.10521290169407</v>
       </c>
       <c r="F24" s="28">
@@ -8015,7 +9412,7 @@
         <f>Scenarios!G87</f>
         <v/>
       </c>
-      <c r="K24" s="80">
+      <c r="K24" s="85">
         <f>IF(MAX(ABS(F24-Scenarios!$G$83),ABS(G24-Scenarios!$G$84),ABS(H24-Scenarios!$G$85),ABS(I24-Scenarios!$G$86),ABS(J24-Scenarios!$G$87))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -8045,30 +9442,30 @@
 Implied ~3.0% of revenue (= 331,421 ÷ 11,102,600); forecast via DPO×COGS.</t>
         </is>
       </c>
-      <c r="E25" s="78" t="n">
+      <c r="E25" s="73" t="n">
         <v>331421</v>
       </c>
-      <c r="F25" s="79">
+      <c r="F25" s="74">
         <f>Scenarios!G88</f>
         <v/>
       </c>
-      <c r="G25" s="79">
+      <c r="G25" s="74">
         <f>Scenarios!G89</f>
         <v/>
       </c>
-      <c r="H25" s="79">
+      <c r="H25" s="74">
         <f>Scenarios!G90</f>
         <v/>
       </c>
-      <c r="I25" s="79">
+      <c r="I25" s="74">
         <f>Scenarios!G91</f>
         <v/>
       </c>
-      <c r="J25" s="79">
+      <c r="J25" s="74">
         <f>Scenarios!G92</f>
         <v/>
       </c>
-      <c r="K25" s="80">
+      <c r="K25" s="85">
         <f>IF(MAX(ABS(F25-Scenarios!$G$88),ABS(G25-Scenarios!$G$89),ABS(H25-Scenarios!$G$90),ABS(I25-Scenarios!$G$91),ABS(J25-Scenarios!$G$92))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -8098,7 +9495,7 @@
 5.1% of revenue (flat). OCA residual = 564,089 ÷ 11,102,600.</t>
         </is>
       </c>
-      <c r="E26" s="81" t="n">
+      <c r="E26" s="76" t="n">
         <v>0.05080692810692991</v>
       </c>
       <c r="F26" s="20">
@@ -8147,30 +9544,30 @@
 5.1% of revenue (flat). OCA residual = 564,089 ÷ 11,102,600.</t>
         </is>
       </c>
-      <c r="E27" s="78" t="n">
+      <c r="E27" s="73" t="n">
         <v>564089</v>
       </c>
-      <c r="F27" s="79">
+      <c r="F27" s="74">
         <f>Scenarios!G93</f>
         <v/>
       </c>
-      <c r="G27" s="79">
+      <c r="G27" s="74">
         <f>Scenarios!G94</f>
         <v/>
       </c>
-      <c r="H27" s="79">
+      <c r="H27" s="74">
         <f>Scenarios!G95</f>
         <v/>
       </c>
-      <c r="I27" s="79">
+      <c r="I27" s="74">
         <f>Scenarios!G96</f>
         <v/>
       </c>
-      <c r="J27" s="79">
+      <c r="J27" s="74">
         <f>Scenarios!G97</f>
         <v/>
       </c>
-      <c r="K27" s="80">
+      <c r="K27" s="85">
         <f>IF(MAX(ABS(F27-Scenarios!$G$93),ABS(G27-Scenarios!$G$94),ABS(H27-Scenarios!$G$95),ABS(I27-Scenarios!$G$96),ABS(J27-Scenarios!$G$97))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -8200,7 +9597,7 @@
 6.0% of revenue (flat). 662,982 ÷ 11,102,600.</t>
         </is>
       </c>
-      <c r="E28" s="81" t="n">
+      <c r="E28" s="76" t="n">
         <v>0.05971412101669879</v>
       </c>
       <c r="F28" s="20">
@@ -8249,30 +9646,30 @@
 6.0% of revenue (flat). 662,982 ÷ 11,102,600.</t>
         </is>
       </c>
-      <c r="E29" s="78" t="n">
+      <c r="E29" s="73" t="n">
         <v>662982</v>
       </c>
-      <c r="F29" s="79">
+      <c r="F29" s="74">
         <f>Scenarios!G98</f>
         <v/>
       </c>
-      <c r="G29" s="79">
+      <c r="G29" s="74">
         <f>Scenarios!G99</f>
         <v/>
       </c>
-      <c r="H29" s="79">
+      <c r="H29" s="74">
         <f>Scenarios!G100</f>
         <v/>
       </c>
-      <c r="I29" s="79">
+      <c r="I29" s="74">
         <f>Scenarios!G101</f>
         <v/>
       </c>
-      <c r="J29" s="79">
+      <c r="J29" s="74">
         <f>Scenarios!G102</f>
         <v/>
       </c>
-      <c r="K29" s="80">
+      <c r="K29" s="85">
         <f>IF(MAX(ABS(F29-Scenarios!$G$98),ABS(G29-Scenarios!$G$99),ABS(H29-Scenarios!$G$100),ABS(I29-Scenarios!$G$101),ABS(J29-Scenarios!$G$102))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -8299,27 +9696,27 @@
 FY25: AR ~1.7% + inventory ~15.3% + prepaids 5.1% ≈ 22.1% of sales.</t>
         </is>
       </c>
-      <c r="F30" s="79">
+      <c r="F30" s="74">
         <f>Scenarios!G103</f>
         <v/>
       </c>
-      <c r="G30" s="79">
+      <c r="G30" s="74">
         <f>Scenarios!G104</f>
         <v/>
       </c>
-      <c r="H30" s="79">
+      <c r="H30" s="74">
         <f>Scenarios!G105</f>
         <v/>
       </c>
-      <c r="I30" s="79">
+      <c r="I30" s="74">
         <f>Scenarios!G106</f>
         <v/>
       </c>
-      <c r="J30" s="79">
+      <c r="J30" s="74">
         <f>Scenarios!G107</f>
         <v/>
       </c>
-      <c r="K30" s="80">
+      <c r="K30" s="85">
         <f>IF(MAX(ABS(F30-Scenarios!$G$103),ABS(G30-Scenarios!$G$104),ABS(H30-Scenarios!$G$105),ABS(I30-Scenarios!$G$106),ABS(J30-Scenarios!$G$107))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -8346,27 +9743,27 @@
 FY25: AP ~3.0% + accrued liabilities 6.0% ≈ 9.0% of sales.</t>
         </is>
       </c>
-      <c r="F31" s="79">
+      <c r="F31" s="74">
         <f>Scenarios!G108</f>
         <v/>
       </c>
-      <c r="G31" s="79">
+      <c r="G31" s="74">
         <f>Scenarios!G109</f>
         <v/>
       </c>
-      <c r="H31" s="79">
+      <c r="H31" s="74">
         <f>Scenarios!G110</f>
         <v/>
       </c>
-      <c r="I31" s="79">
+      <c r="I31" s="74">
         <f>Scenarios!G111</f>
         <v/>
       </c>
-      <c r="J31" s="79">
+      <c r="J31" s="74">
         <f>Scenarios!G112</f>
         <v/>
       </c>
-      <c r="K31" s="80">
+      <c r="K31" s="85">
         <f>IF(MAX(ABS(F31-Scenarios!$G$108),ABS(G31-Scenarios!$G$109),ABS(H31-Scenarios!$G$110),ABS(I31-Scenarios!$G$111),ABS(J31-Scenarios!$G$112))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -8393,7 +9790,7 @@
 FY25 NWC ≈ 13.2% of sales ($1,461,096k = COA − COL).</t>
         </is>
       </c>
-      <c r="E32" s="82" t="n">
+      <c r="E32" s="75" t="n">
         <v>1461096</v>
       </c>
       <c r="F32" s="25">
@@ -8416,7 +9813,7 @@
         <f>Scenarios!G117</f>
         <v/>
       </c>
-      <c r="K32" s="83">
+      <c r="K32" s="86">
         <f>IF(MAX(ABS(F32-Scenarios!$G$113),ABS(G32-Scenarios!$G$114),ABS(H32-Scenarios!$G$115),ABS(I32-Scenarios!$G$116),ABS(J32-Scenarios!$G$117))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -8464,7 +9861,7 @@
         <f>Scenarios!G122</f>
         <v/>
       </c>
-      <c r="K33" s="83">
+      <c r="K33" s="86">
         <f>IF(MAX(ABS(F33-Scenarios!$G$118),ABS(G33-Scenarios!$G$119),ABS(H33-Scenarios!$G$120),ABS(I33-Scenarios!$G$121),ABS(J33-Scenarios!$G$122))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -8482,27 +9879,27 @@
           <t>Unlevered free cash flow</t>
         </is>
       </c>
-      <c r="F35" s="85">
+      <c r="F35" s="88">
         <f>Scenarios!G123</f>
         <v/>
       </c>
-      <c r="G35" s="85">
+      <c r="G35" s="88">
         <f>Scenarios!G124</f>
         <v/>
       </c>
-      <c r="H35" s="85">
+      <c r="H35" s="88">
         <f>Scenarios!G125</f>
         <v/>
       </c>
-      <c r="I35" s="85">
+      <c r="I35" s="88">
         <f>Scenarios!G126</f>
         <v/>
       </c>
-      <c r="J35" s="85">
+      <c r="J35" s="88">
         <f>Scenarios!G127</f>
         <v/>
       </c>
-      <c r="K35" s="83">
+      <c r="K35" s="86">
         <f>IF(MAX(ABS(F35-Scenarios!$G$123),ABS(G35-Scenarios!$G$124),ABS(H35-Scenarios!$G$125),ABS(I35-Scenarios!$G$126),ABS(J35-Scenarios!$G$127))&lt;0.5,"OK","CHECK")</f>
         <v/>
       </c>
@@ -8513,19 +9910,19 @@
           <t>Discount period (years)</t>
         </is>
       </c>
-      <c r="F36" s="86" t="n">
+      <c r="F36" s="89" t="n">
         <v>1</v>
       </c>
-      <c r="G36" s="86" t="n">
+      <c r="G36" s="89" t="n">
         <v>2</v>
       </c>
-      <c r="H36" s="86" t="n">
+      <c r="H36" s="89" t="n">
         <v>3</v>
       </c>
-      <c r="I36" s="86" t="n">
+      <c r="I36" s="89" t="n">
         <v>4</v>
       </c>
-      <c r="J36" s="86" t="n">
+      <c r="J36" s="89" t="n">
         <v>5</v>
       </c>
     </row>
@@ -8535,23 +9932,23 @@
           <t>Discount factor @ WACC</t>
         </is>
       </c>
-      <c r="F37" s="87">
+      <c r="F37" s="90">
         <f>1/(1+Scenarios!$G$9)^F36</f>
         <v/>
       </c>
-      <c r="G37" s="87">
+      <c r="G37" s="90">
         <f>1/(1+Scenarios!$G$9)^G36</f>
         <v/>
       </c>
-      <c r="H37" s="87">
+      <c r="H37" s="90">
         <f>1/(1+Scenarios!$G$9)^H36</f>
         <v/>
       </c>
-      <c r="I37" s="87">
+      <c r="I37" s="90">
         <f>1/(1+Scenarios!$G$9)^I36</f>
         <v/>
       </c>
-      <c r="J37" s="87">
+      <c r="J37" s="90">
         <f>1/(1+Scenarios!$G$9)^J36</f>
         <v/>
       </c>
@@ -8589,13 +9986,13 @@
           <t>Scenarios linkage summary (column K should all read OK)</t>
         </is>
       </c>
-      <c r="K40" s="88">
+      <c r="K40" s="91">
         <f>IF(COUNTIF(K5:K35,"CHECK")=0,"ALL OK","REVIEW")</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="89" t="inlineStr">
+      <c r="A41" s="92" t="inlineStr">
         <is>
           <t>VALUATION — GORDON GROWTH (PERPETUITY) METHOD</t>
         </is>
@@ -8657,7 +10054,7 @@
           <t>Terminal value = FCF₅×(1+g)/(WACC−g)</t>
         </is>
       </c>
-      <c r="E45" s="79">
+      <c r="E45" s="74">
         <f>J35*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
         <v/>
       </c>
@@ -8668,7 +10065,7 @@
           <t xml:space="preserve">  Implied exit EV/EBITDA = Gordon TV / FY30 EBITDA</t>
         </is>
       </c>
-      <c r="E46" s="90">
+      <c r="E46" s="93">
         <f>E45/E44</f>
         <v/>
       </c>
@@ -8679,7 +10076,7 @@
           <t xml:space="preserve">  memo: (UFCF₃₀ / EBITDA₃₀) × (1+g) / (WACC−g)</t>
         </is>
       </c>
-      <c r="E47" s="90">
+      <c r="E47" s="93">
         <f>J35/E44*(1+Scenarios!$G$10)/(Scenarios!$G$9-Scenarios!$G$10)</f>
         <v/>
       </c>
@@ -8712,7 +10109,7 @@
           <t>Plus: cash &amp; equivalents (FY2025)</t>
         </is>
       </c>
-      <c r="C50" s="91" t="inlineStr">
+      <c r="C50" s="94" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -8722,7 +10119,7 @@
           <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
         </is>
       </c>
-      <c r="E50" s="78" t="n">
+      <c r="E50" s="73" t="n">
         <v>1807202</v>
       </c>
     </row>
@@ -8747,7 +10144,7 @@
           <t>Ctrl+F "Current lease liabilities" → 298,724 | "Non-current lease liabilities" → 1,499,717 | sum 1,798,441 ($000). Funded debt: "no borrowings were outstanding"</t>
         </is>
       </c>
-      <c r="E51" s="78" t="n">
+      <c r="E51" s="73" t="n">
         <v>-1798441</v>
       </c>
     </row>
@@ -8782,7 +10179,7 @@
           <t>Shares outstanding (000)</t>
         </is>
       </c>
-      <c r="C55" s="91" t="inlineStr">
+      <c r="C55" s="94" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -8792,7 +10189,7 @@
           <t>Ctrl+F "111,380 and 116,166 issued and outstanding" → 111,380k class A (FY25 10-K cover)</t>
         </is>
       </c>
-      <c r="E55" s="78" t="n">
+      <c r="E55" s="73" t="n">
         <v>111380</v>
       </c>
     </row>
@@ -8802,11 +10199,11 @@
           <t>Implied value per share</t>
         </is>
       </c>
-      <c r="E56" s="92">
+      <c r="E56" s="95">
         <f>E54/E55</f>
         <v/>
       </c>
-      <c r="K56" s="83">
+      <c r="K56" s="86">
         <f>IF(ABS(E56-Scenarios!$G$130)&lt;0.05,"OK","CHECK")</f>
         <v/>
       </c>
@@ -8817,7 +10214,7 @@
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C57" s="91" t="inlineStr">
+      <c r="C57" s="94" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -8827,7 +10224,7 @@
           <t>Ctrl+F "closed at $100.61" → Last Sale on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E57" s="93" t="n">
+      <c r="E57" s="96" t="n">
         <v>100</v>
       </c>
     </row>
@@ -8837,7 +10234,7 @@
           <t>Implied upside / (downside)</t>
         </is>
       </c>
-      <c r="E58" s="94">
+      <c r="E58" s="97">
         <f>E56/E57-1</f>
         <v/>
       </c>
@@ -8854,7 +10251,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="89" t="inlineStr">
+      <c r="A61" s="92" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
@@ -8890,11 +10287,11 @@
           <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
         </is>
       </c>
-      <c r="E63" s="90">
+      <c r="E63" s="93">
         <f>E46</f>
         <v/>
       </c>
-      <c r="M63" s="91" t="inlineStr">
+      <c r="M63" s="94" t="inlineStr">
         <is>
           <t>Comps: Exit Multiple Build</t>
         </is>
@@ -8906,7 +10303,7 @@
           <t>Terminal value = Terminal EBITDA × exit multiple</t>
         </is>
       </c>
-      <c r="E64" s="79">
+      <c r="E64" s="74">
         <f>E44*E63</f>
         <v/>
       </c>
@@ -8917,7 +10314,7 @@
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="E65" s="79">
+      <c r="E65" s="74">
         <f>E64/(1+Scenarios!$G$9)^J36</f>
         <v/>
       </c>
@@ -8939,13 +10336,13 @@
           <t>Implied value per share (exit method)</t>
         </is>
       </c>
-      <c r="E67" s="95">
+      <c r="E67" s="98">
         <f>(E66+E50+E51)/E55</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="89" t="inlineStr">
+      <c r="A69" s="92" t="inlineStr">
         <is>
           <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
         </is>
@@ -8955,7 +10352,7 @@
       <c r="D69" s="13" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="96" t="inlineStr"/>
+      <c r="A70" s="99" t="inlineStr"/>
       <c r="B70" s="53" t="inlineStr">
         <is>
           <t>Gordon Growth</t>
@@ -8997,15 +10394,15 @@
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
       </c>
-      <c r="B72" s="97">
+      <c r="B72" s="100">
         <f>E46</f>
         <v/>
       </c>
-      <c r="C72" s="97">
+      <c r="C72" s="100">
         <f>E63</f>
         <v/>
       </c>
-      <c r="D72" s="97">
+      <c r="D72" s="100">
         <f>B72-C72</f>
         <v/>
       </c>
@@ -9029,15 +10426,15 @@
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="B74" s="98">
+      <c r="B74" s="101">
         <f>E56</f>
         <v/>
       </c>
-      <c r="C74" s="98">
+      <c r="C74" s="101">
         <f>E67</f>
         <v/>
       </c>
-      <c r="D74" s="98">
+      <c r="D74" s="101">
         <f>B74-C74</f>
         <v/>
       </c>
@@ -9048,11 +10445,11 @@
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B75" s="99">
+      <c r="B75" s="102">
         <f>IF(ABS(D72)&lt;=1.5,"PASS","REVIEW")</f>
         <v/>
       </c>
-      <c r="C75" s="100">
+      <c r="C75" s="103">
         <f>TEXT(D72,"0.0")&amp;"x spread vs Gordon-implied exit"</f>
         <v/>
       </c>
@@ -9063,7 +10460,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="89" t="inlineStr">
+      <c r="A78" s="92" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
@@ -9077,7 +10474,7 @@
       <c r="H78" s="13" t="n"/>
     </row>
     <row r="79" ht="28" customHeight="1">
-      <c r="A79" s="101" t="inlineStr">
+      <c r="A79" s="104" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
@@ -9097,32 +10494,32 @@
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
       </c>
-      <c r="F79" s="102" t="n">
+      <c r="F79" s="105" t="n">
         <v>0.015</v>
       </c>
-      <c r="G79" s="102" t="n">
+      <c r="G79" s="105" t="n">
         <v>0.02</v>
       </c>
-      <c r="H79" s="102" t="n">
+      <c r="H79" s="105" t="n">
         <v>0.0225</v>
       </c>
-      <c r="I79" s="102" t="n">
+      <c r="I79" s="105" t="n">
         <v>0.025</v>
       </c>
-      <c r="J79" s="102" t="n">
+      <c r="J79" s="105" t="n">
         <v>0.03</v>
       </c>
-      <c r="L79" s="91" t="inlineStr">
+      <c r="L79" s="94" t="inlineStr">
         <is>
           <t>Scenarios: terminal g</t>
         </is>
       </c>
     </row>
     <row r="80" ht="28" customHeight="1">
-      <c r="A80" s="102" t="n">
+      <c r="A80" s="105" t="n">
         <v>0.095</v>
       </c>
-      <c r="C80" s="91" t="inlineStr">
+      <c r="C80" s="94" t="inlineStr">
         <is>
           <t>Damodaran: Historical Implied ERP</t>
         </is>
@@ -9132,34 +10529,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F80" s="103">
+      <c r="F80" s="106">
         <f>(NPV(0.095,F35:J35)+(J35*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="G80" s="103">
+      <c r="G80" s="106">
         <f>(NPV(0.095,F35:J35)+(J35*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="H80" s="103">
+      <c r="H80" s="106">
         <f>(NPV(0.095,F35:J35)+(J35*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="I80" s="103">
+      <c r="I80" s="106">
         <f>(NPV(0.095,F35:J35)+(J35*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="J80" s="103">
+      <c r="J80" s="106">
         <f>(NPV(0.095,F35:J35)+(J35*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="L80" s="91" t="inlineStr">
+      <c r="L80" s="94" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="81" ht="28" customHeight="1">
-      <c r="A81" s="102" t="n">
+      <c r="A81" s="105" t="n">
         <v>0.1</v>
       </c>
       <c r="D81" s="19" t="inlineStr">
@@ -9167,34 +10564,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F81" s="103">
+      <c r="F81" s="106">
         <f>(NPV(0.1,F35:J35)+(J35*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="G81" s="103">
+      <c r="G81" s="106">
         <f>(NPV(0.1,F35:J35)+(J35*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="H81" s="103">
+      <c r="H81" s="106">
         <f>(NPV(0.1,F35:J35)+(J35*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="I81" s="103">
+      <c r="I81" s="106">
         <f>(NPV(0.1,F35:J35)+(J35*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="J81" s="103">
+      <c r="J81" s="106">
         <f>(NPV(0.1,F35:J35)+(J35*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="L81" s="91" t="inlineStr">
+      <c r="L81" s="94" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="82" ht="28" customHeight="1">
-      <c r="A82" s="102" t="n">
+      <c r="A82" s="105" t="n">
         <v>0.105</v>
       </c>
       <c r="D82" s="19" t="inlineStr">
@@ -9202,34 +10599,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F82" s="103">
+      <c r="F82" s="106">
         <f>(NPV(0.105,F35:J35)+(J35*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="G82" s="103">
+      <c r="G82" s="106">
         <f>(NPV(0.105,F35:J35)+(J35*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="H82" s="104">
+      <c r="H82" s="107">
         <f>(NPV(0.105,F35:J35)+(J35*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="I82" s="103">
+      <c r="I82" s="106">
         <f>(NPV(0.105,F35:J35)+(J35*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="J82" s="103">
+      <c r="J82" s="106">
         <f>(NPV(0.105,F35:J35)+(J35*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="L82" s="91" t="inlineStr">
+      <c r="L82" s="94" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="83" ht="28" customHeight="1">
-      <c r="A83" s="102" t="n">
+      <c r="A83" s="105" t="n">
         <v>0.11</v>
       </c>
       <c r="D83" s="19" t="inlineStr">
@@ -9237,34 +10634,34 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F83" s="103">
+      <c r="F83" s="106">
         <f>(NPV(0.11,F35:J35)+(J35*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="G83" s="103">
+      <c r="G83" s="106">
         <f>(NPV(0.11,F35:J35)+(J35*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="H83" s="103">
+      <c r="H83" s="106">
         <f>(NPV(0.11,F35:J35)+(J35*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="I83" s="103">
+      <c r="I83" s="106">
         <f>(NPV(0.11,F35:J35)+(J35*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="J83" s="103">
+      <c r="J83" s="106">
         <f>(NPV(0.11,F35:J35)+(J35*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="L83" s="91" t="inlineStr">
+      <c r="L83" s="94" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="84" ht="28" customHeight="1">
-      <c r="A84" s="102" t="n">
+      <c r="A84" s="105" t="n">
         <v>0.115</v>
       </c>
       <c r="D84" s="19" t="inlineStr">
@@ -9272,27 +10669,27 @@
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F84" s="103">
+      <c r="F84" s="106">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="G84" s="103">
+      <c r="G84" s="106">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="H84" s="103">
+      <c r="H84" s="106">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="I84" s="103">
+      <c r="I84" s="106">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="J84" s="103">
+      <c r="J84" s="106">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="L84" s="91" t="inlineStr">
+      <c r="L84" s="94" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
@@ -9314,7 +10711,7 @@
           <t>Scenarios tab → Ctrl+F "WACC" and "Terminal growth" rows (base-case inputs)</t>
         </is>
       </c>
-      <c r="L85" s="91" t="inlineStr">
+      <c r="L85" s="94" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
@@ -9329,7 +10726,8 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId2"/>
-    <hyperlink ref="C4" location="'Revenue Drivers'!A1"/>
+    <hyperlink ref="C4" location="'NOPAT Bridge'!A1"/>
+    <hyperlink ref="D4" location="'Revenue Drivers'!A1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId5"/>
@@ -9393,7 +10791,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
@@ -9458,7 +10856,7 @@
           <t>FY2025A revenue</t>
         </is>
       </c>
-      <c r="C4" s="91" t="inlineStr">
+      <c r="C4" s="94" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -9468,7 +10866,7 @@
           <t>Ctrl+F "Net revenue" → 11,102,600 ($000) in FY2025 column</t>
         </is>
       </c>
-      <c r="E4" s="78" t="n">
+      <c r="E4" s="73" t="n">
         <v>11102600</v>
       </c>
     </row>
@@ -9478,7 +10876,7 @@
           <t>FY2025A EBITDA (EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="E5" s="79">
+      <c r="E5" s="74">
         <f>2210615+496228</f>
         <v/>
       </c>
@@ -9489,12 +10887,12 @@
           <t>FY2030E terminal EBITDA (DCF EBIT + D&amp;A)</t>
         </is>
       </c>
-      <c r="C6" s="91" t="inlineStr">
+      <c r="C6" s="94" t="inlineStr">
         <is>
           <t>↳ DCF base case</t>
         </is>
       </c>
-      <c r="E6" s="79">
+      <c r="E6" s="74">
         <f>DCF!E44</f>
         <v/>
       </c>
@@ -9505,7 +10903,7 @@
           <t>FY2026E diluted EPS (guidance midpoint)</t>
         </is>
       </c>
-      <c r="C7" s="91" t="inlineStr">
+      <c r="C7" s="94" t="inlineStr">
         <is>
           <t>Release</t>
         </is>
@@ -9515,7 +10913,7 @@
           <t>Ctrl+F "$9.48 to $9.73" → FY2026 diluted EPS guidance; model midpoint $9.61</t>
         </is>
       </c>
-      <c r="E7" s="93" t="n">
+      <c r="E7" s="96" t="n">
         <v>9.609999999999999</v>
       </c>
     </row>
@@ -9525,7 +10923,7 @@
           <t>Cash &amp; equivalents</t>
         </is>
       </c>
-      <c r="C8" s="91" t="inlineStr">
+      <c r="C8" s="94" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -9535,7 +10933,7 @@
           <t>Ctrl+F "Cash and cash equivalents" → 1,807,202 ($000) FY2025</t>
         </is>
       </c>
-      <c r="E8" s="78" t="n">
+      <c r="E8" s="73" t="n">
         <v>1807202</v>
       </c>
     </row>
@@ -9545,7 +10943,7 @@
           <t>Shares outstanding (000)</t>
         </is>
       </c>
-      <c r="C9" s="91" t="inlineStr">
+      <c r="C9" s="94" t="inlineStr">
         <is>
           <t>10-K</t>
         </is>
@@ -9555,7 +10953,7 @@
           <t>Ctrl+F "111,380 and 116,166 issued and outstanding" → 111,380k class A (FY25 10-K cover)</t>
         </is>
       </c>
-      <c r="E9" s="78" t="n">
+      <c r="E9" s="73" t="n">
         <v>111380</v>
       </c>
     </row>
@@ -9565,7 +10963,7 @@
           <t>Current share price</t>
         </is>
       </c>
-      <c r="C10" s="91" t="inlineStr">
+      <c r="C10" s="94" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -9575,28 +10973,28 @@
           <t>Ctrl+F "closed at $100.61" → Last Sale on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E10" s="93" t="n">
+      <c r="E10" s="96" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="100" t="inlineStr">
+      <c r="A11" s="103" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current EV / EBITDA</t>
         </is>
       </c>
-      <c r="E11" s="105">
+      <c r="E11" s="108">
         <f>(E10*E9-E8)/E5</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="100" t="inlineStr">
+      <c r="A12" s="103" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current P / E (FY2026E)</t>
         </is>
       </c>
-      <c r="E12" s="105">
+      <c r="E12" s="108">
         <f>E10/E7</f>
         <v/>
       </c>
@@ -9609,7 +11007,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="100" t="inlineStr">
+      <c r="A15" s="103" t="inlineStr">
         <is>
           <t>Peer / reference EV/EBITDA (forward / illustrative)</t>
         </is>
@@ -9630,37 +11028,37 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="106" t="inlineStr">
+      <c r="A18" s="109" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B18" s="106" t="inlineStr">
+      <c r="B18" s="109" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C18" s="106" t="inlineStr">
+      <c r="C18" s="109" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D18" s="106" t="inlineStr">
+      <c r="D18" s="109" t="inlineStr">
         <is>
           <t>Ctrl+F / proof</t>
         </is>
       </c>
-      <c r="E18" s="107" t="inlineStr">
+      <c r="E18" s="110" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="I18" s="107" t="inlineStr">
+      <c r="I18" s="110" t="inlineStr">
         <is>
           <t>EV ($000)</t>
         </is>
       </c>
-      <c r="J18" s="107" t="inlineStr">
+      <c r="J18" s="110" t="inlineStr">
         <is>
           <t>EBITDA ($000)</t>
         </is>
@@ -9687,14 +11085,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E19" s="108">
+      <c r="E19" s="111">
         <f>IF(J19&lt;=0,"n.m.",I19/J19)</f>
         <v/>
       </c>
-      <c r="I19" s="109" t="n">
+      <c r="I19" s="112" t="n">
         <v>11890440</v>
       </c>
-      <c r="J19" s="109" t="n">
+      <c r="J19" s="112" t="n">
         <v>2548084</v>
       </c>
     </row>
@@ -9719,14 +11117,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E20" s="108">
+      <c r="E20" s="111">
         <f>IF(J20&lt;=0,"n.m.",I20/J20)</f>
         <v/>
       </c>
-      <c r="I20" s="109" t="n">
+      <c r="I20" s="112" t="n">
         <v>3208397</v>
       </c>
-      <c r="J20" s="109" t="n">
+      <c r="J20" s="112" t="n">
         <v>-23230</v>
       </c>
     </row>
@@ -9751,14 +11149,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E21" s="108">
+      <c r="E21" s="111">
         <f>IF(J21&lt;=0,"n.m.",I21/J21)</f>
         <v/>
       </c>
-      <c r="I21" s="109" t="n">
+      <c r="I21" s="112" t="n">
         <v>35661944</v>
       </c>
-      <c r="J21" s="109" t="n">
+      <c r="J21" s="112" t="n">
         <v>3857684</v>
       </c>
     </row>
@@ -9783,14 +11181,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E22" s="108">
+      <c r="E22" s="111">
         <f>IF(J22&lt;=0,"n.m.",I22/J22)</f>
         <v/>
       </c>
-      <c r="I22" s="109" t="n">
+      <c r="I22" s="112" t="n">
         <v>58972350</v>
       </c>
-      <c r="J22" s="109" t="n">
+      <c r="J22" s="112" t="n">
         <v>4647000</v>
       </c>
     </row>
@@ -9815,14 +11213,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E23" s="108">
+      <c r="E23" s="111">
         <f>IF(J23&lt;=0,"n.m.",I23/J23)</f>
         <v/>
       </c>
-      <c r="I23" s="109" t="n">
+      <c r="I23" s="112" t="n">
         <v>10555510</v>
       </c>
-      <c r="J23" s="109" t="n">
+      <c r="J23" s="112" t="n">
         <v>1329439</v>
       </c>
     </row>
@@ -9847,14 +11245,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E24" s="108">
+      <c r="E24" s="111">
         <f>IF(J24&lt;=0,"n.m.",I24/J24)</f>
         <v/>
       </c>
-      <c r="I24" s="109" t="n">
+      <c r="I24" s="112" t="n">
         <v>27284350</v>
       </c>
-      <c r="J24" s="109" t="n">
+      <c r="J24" s="112" t="n">
         <v>1768400</v>
       </c>
     </row>
@@ -9879,14 +11277,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E25" s="108">
+      <c r="E25" s="111">
         <f>IF(J25&lt;=0,"n.m.",I25/J25)</f>
         <v/>
       </c>
-      <c r="I25" s="109" t="n">
+      <c r="I25" s="112" t="n">
         <v>7153911</v>
       </c>
-      <c r="J25" s="109" t="n">
+      <c r="J25" s="112" t="n">
         <v>922278</v>
       </c>
     </row>
@@ -9911,14 +11309,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E26" s="108">
+      <c r="E26" s="111">
         <f>IF(J26&lt;=0,"n.m.",I26/J26)</f>
         <v/>
       </c>
-      <c r="I26" s="109" t="n">
+      <c r="I26" s="112" t="n">
         <v>616045</v>
       </c>
-      <c r="J26" s="109" t="n">
+      <c r="J26" s="112" t="n">
         <v>62010</v>
       </c>
     </row>
@@ -9943,14 +11341,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E27" s="108">
+      <c r="E27" s="111">
         <f>IF(J27&lt;=0,"n.m.",I27/J27)</f>
         <v/>
       </c>
-      <c r="I27" s="109" t="n">
+      <c r="I27" s="112" t="n">
         <v>9422753</v>
       </c>
-      <c r="J27" s="109" t="n">
+      <c r="J27" s="112" t="n">
         <v>976700</v>
       </c>
     </row>
@@ -9975,14 +11373,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E28" s="108">
+      <c r="E28" s="111">
         <f>IF(J28&lt;=0,"n.m.",I28/J28)</f>
         <v/>
       </c>
-      <c r="I28" s="109" t="n">
+      <c r="I28" s="112" t="n">
         <v>1598873</v>
       </c>
-      <c r="J28" s="109" t="n">
+      <c r="J28" s="112" t="n">
         <v>235723</v>
       </c>
     </row>
@@ -10007,14 +11405,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E29" s="108">
+      <c r="E29" s="111">
         <f>IF(J29&lt;=0,"n.m.",I29/J29)</f>
         <v/>
       </c>
-      <c r="I29" s="109" t="n">
+      <c r="I29" s="112" t="n">
         <v>5236269</v>
       </c>
-      <c r="J29" s="109" t="n">
+      <c r="J29" s="112" t="n">
         <v>407521</v>
       </c>
     </row>
@@ -10056,7 +11454,7 @@
 Also: Ctrl+F "roughly $10 billion" and "No deal was announced". Still an ask.</t>
         </is>
       </c>
-      <c r="E33" s="110" t="n">
+      <c r="E33" s="113" t="n">
         <v>10</v>
       </c>
     </row>
@@ -10081,7 +11479,7 @@
           <t>Ctrl+F "nearly $2 billion". Forbes estimate for Color Image parent (Alo + Bella+Canvas), not Alo-only EBITDA.</t>
         </is>
       </c>
-      <c r="E34" s="110" t="n">
+      <c r="E34" s="113" t="n">
         <v>2</v>
       </c>
     </row>
@@ -10096,7 +11494,7 @@
           <t>5.0x = 10 / 2. Implied EV/Sales on an unclosed ask and parent sales. Not EV/EBITDA. Not the TV.</t>
         </is>
       </c>
-      <c r="C35" s="91" t="inlineStr">
+      <c r="C35" s="94" t="inlineStr">
         <is>
           <t>Comps: Alo ask / parent sales</t>
         </is>
@@ -10106,7 +11504,7 @@
           <t>No Ctrl+F for EV/EBITDA — Firecrawl found none on Reuters or Forbes. This cell is E33 / E34 (ask ÷ parent sales). Not the TV.</t>
         </is>
       </c>
-      <c r="E35" s="111">
+      <c r="E35" s="114">
         <f>E33/E34</f>
         <v/>
       </c>
@@ -10132,7 +11530,7 @@
           <t>No Ctrl+F. Reuters, Forbes, and PitchBook do not print Alo EV/EBITDA.</t>
         </is>
       </c>
-      <c r="E36" s="112" t="inlineStr">
+      <c r="E36" s="115" t="inlineStr">
         <is>
           <t>n.a.</t>
         </is>
@@ -10166,7 +11564,7 @@
           <t>Each E cell is I/J from the PitchBook extract. Do not use as FY30 exit.</t>
         </is>
       </c>
-      <c r="E39" s="108">
+      <c r="E39" s="111">
         <f>AVERAGE(E19,E22,E21,E23,E25,E27,E29)</f>
         <v/>
       </c>
@@ -10192,13 +11590,13 @@
           <t>UAA omitted because TTM EBITDA is negative. Not the selected FY30 exit.</t>
         </is>
       </c>
-      <c r="E40" s="108">
+      <c r="E40" s="111">
         <f>AVERAGE(E19,E21,E22,E23,E24,E25,E26,E27,E28,E29)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="100" t="inlineStr">
+      <c r="A41" s="103" t="inlineStr">
         <is>
           <t>We do not average peers for terminal value, and we do not use Alo 5.0x EV/Sales as EV/EBITDA.</t>
         </is>
@@ -10217,7 +11615,7 @@
           <t>Gordon Growth implied exit EV/EBITDA</t>
         </is>
       </c>
-      <c r="E44" s="90">
+      <c r="E44" s="93">
         <f>DCF!E46</f>
         <v/>
       </c>
@@ -10228,7 +11626,7 @@
           <t>Selected exit multiple (base case)</t>
         </is>
       </c>
-      <c r="E45" s="97">
+      <c r="E45" s="100">
         <f>DCF!E63</f>
         <v/>
       </c>
@@ -10239,7 +11637,7 @@
           <t>Spread (selected − Gordon implied)</t>
         </is>
       </c>
-      <c r="E46" s="90">
+      <c r="E46" s="93">
         <f>E45-E44</f>
         <v/>
       </c>
@@ -10301,42 +11699,42 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="106" t="inlineStr">
+      <c r="A56" s="109" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B56" s="106" t="inlineStr">
+      <c r="B56" s="109" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C56" s="106" t="inlineStr">
+      <c r="C56" s="109" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D56" s="106" t="inlineStr">
+      <c r="D56" s="109" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
-      <c r="E56" s="107" t="inlineStr">
+      <c r="E56" s="110" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="F56" s="107" t="inlineStr">
+      <c r="F56" s="110" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="G56" s="107" t="inlineStr">
+      <c r="G56" s="110" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="H56" s="107" t="inlineStr">
+      <c r="H56" s="110" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
@@ -10354,7 +11752,7 @@
 Hi: 8.0x = Deckers print as the high end of the range only. Selected exit is Gordon implied, not this cap.</t>
         </is>
       </c>
-      <c r="C57" s="77" t="inlineStr">
+      <c r="C57" s="84" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU EV/EBITDA
 Hi: StockAnalysis: DECK EV/EBITDA</t>
@@ -10366,17 +11764,17 @@
 Hi: Ctrl+F "EV / EBITDA" → 7.95. Football-field cap 8.0x (Deckers). Not the selected exit.</t>
         </is>
       </c>
-      <c r="E57" s="113" t="n">
+      <c r="E57" s="116" t="n">
         <v>5</v>
       </c>
-      <c r="F57" s="113" t="n">
+      <c r="F57" s="116" t="n">
         <v>8</v>
       </c>
-      <c r="G57" s="114">
+      <c r="G57" s="117">
         <f>(E6*E57+E8)/E9</f>
         <v/>
       </c>
-      <c r="H57" s="114">
+      <c r="H57" s="117">
         <f>(E6*F57+E8)/E9</f>
         <v/>
       </c>
@@ -10402,11 +11800,11 @@
           <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
         </is>
       </c>
-      <c r="E58" s="111">
+      <c r="E58" s="114">
         <f>DCF!E63</f>
         <v/>
       </c>
-      <c r="G58" s="115">
+      <c r="G58" s="118">
         <f>(E6*E58+E8)/E9</f>
         <v/>
       </c>
@@ -10423,7 +11821,7 @@
 Hi: 18x P/E high on FY2026E EPS; modest recovery case still below historical premium LULU multiples.</t>
         </is>
       </c>
-      <c r="C59" s="77" t="inlineStr">
+      <c r="C59" s="84" t="inlineStr">
         <is>
           <t>Lo: StockAnalysis: LULU Forward P/E
 Hi: StockAnalysis: NKE Forward P/E</t>
@@ -10435,17 +11833,17 @@
 Hi: Ctrl+F "Forward PE" → NKE peer benchmark; high-case assumption 18.0x</t>
         </is>
       </c>
-      <c r="E59" s="113" t="n">
+      <c r="E59" s="116" t="n">
         <v>10</v>
       </c>
-      <c r="F59" s="113" t="n">
+      <c r="F59" s="116" t="n">
         <v>18</v>
       </c>
-      <c r="G59" s="114">
+      <c r="G59" s="117">
         <f>E7*E59</f>
         <v/>
       </c>
-      <c r="H59" s="114">
+      <c r="H59" s="117">
         <f>E7*F59</f>
         <v/>
       </c>
@@ -10456,32 +11854,32 @@
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="E60" s="116" t="inlineStr">
+      <c r="E60" s="119" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F60" s="116" t="inlineStr">
+      <c r="F60" s="119" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G60" s="114">
+      <c r="G60" s="117">
         <f>Scenarios!F130</f>
         <v/>
       </c>
-      <c r="H60" s="114">
+      <c r="H60" s="117">
         <f>Scenarios!H130</f>
         <v/>
       </c>
     </row>
     <row r="62" ht="28" customHeight="1">
-      <c r="A62" s="117" t="inlineStr">
+      <c r="A62" s="120" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
       </c>
-      <c r="C62" s="91" t="inlineStr">
+      <c r="C62" s="94" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
@@ -10491,7 +11889,7 @@
           <t>Ctrl+F "closed at $100.61" → Last Sale on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E62" s="118" t="n">
+      <c r="E62" s="121" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add per-sector EBIT rows with margin justifications on NOPAT Bridge
Phase 3 now breaks out store, e-comm, and other channel EBIT with
formula, FY25 calibration math, 10-K source links, and Ctrl+F proof.
Margin assumption docs enhanced with channel revenue anchors.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -3114,15 +3114,15 @@
         </is>
       </c>
       <c r="F48" s="42">
-        <f>F43*(1-'NOPAT Bridge'!F$35)</f>
+        <f>F43*(1-'NOPAT Bridge'!F$38)</f>
         <v/>
       </c>
       <c r="G48" s="42">
-        <f>'NOPAT Bridge'!F37</f>
+        <f>'NOPAT Bridge'!F40</f>
         <v/>
       </c>
       <c r="H48" s="42">
-        <f>H43*(1-'NOPAT Bridge'!F$35)</f>
+        <f>H43*(1-'NOPAT Bridge'!F$38)</f>
         <v/>
       </c>
     </row>
@@ -3133,15 +3133,15 @@
         </is>
       </c>
       <c r="F49" s="42">
-        <f>F44*(1-'NOPAT Bridge'!G$35)</f>
+        <f>F44*(1-'NOPAT Bridge'!G$38)</f>
         <v/>
       </c>
       <c r="G49" s="42">
-        <f>'NOPAT Bridge'!G37</f>
+        <f>'NOPAT Bridge'!G40</f>
         <v/>
       </c>
       <c r="H49" s="42">
-        <f>H44*(1-'NOPAT Bridge'!G$35)</f>
+        <f>H44*(1-'NOPAT Bridge'!G$38)</f>
         <v/>
       </c>
     </row>
@@ -3152,15 +3152,15 @@
         </is>
       </c>
       <c r="F50" s="42">
-        <f>F45*(1-'NOPAT Bridge'!H$35)</f>
+        <f>F45*(1-'NOPAT Bridge'!H$38)</f>
         <v/>
       </c>
       <c r="G50" s="42">
-        <f>'NOPAT Bridge'!H37</f>
+        <f>'NOPAT Bridge'!H40</f>
         <v/>
       </c>
       <c r="H50" s="42">
-        <f>H45*(1-'NOPAT Bridge'!H$35)</f>
+        <f>H45*(1-'NOPAT Bridge'!H$38)</f>
         <v/>
       </c>
     </row>
@@ -3171,15 +3171,15 @@
         </is>
       </c>
       <c r="F51" s="42">
-        <f>F46*(1-'NOPAT Bridge'!I$35)</f>
+        <f>F46*(1-'NOPAT Bridge'!I$38)</f>
         <v/>
       </c>
       <c r="G51" s="42">
-        <f>'NOPAT Bridge'!I37</f>
+        <f>'NOPAT Bridge'!I40</f>
         <v/>
       </c>
       <c r="H51" s="42">
-        <f>H46*(1-'NOPAT Bridge'!I$35)</f>
+        <f>H46*(1-'NOPAT Bridge'!I$38)</f>
         <v/>
       </c>
     </row>
@@ -3190,15 +3190,15 @@
         </is>
       </c>
       <c r="F52" s="42">
-        <f>F47*(1-'NOPAT Bridge'!J$35)</f>
+        <f>F47*(1-'NOPAT Bridge'!J$38)</f>
         <v/>
       </c>
       <c r="G52" s="42">
-        <f>'NOPAT Bridge'!J37</f>
+        <f>'NOPAT Bridge'!J40</f>
         <v/>
       </c>
       <c r="H52" s="42">
-        <f>H47*(1-'NOPAT Bridge'!J$35)</f>
+        <f>H47*(1-'NOPAT Bridge'!J$38)</f>
         <v/>
       </c>
     </row>
@@ -7066,7 +7066,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -7206,7 +7206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="56" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Phase 3: Store-channel EBIT margin %</t>
@@ -7214,17 +7214,22 @@
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>18.6% EBIT margin on store-channel revenue. Calibrated so FY25 channel EBIT ≈ reported EBIT.</t>
-        </is>
-      </c>
-      <c r="C8" s="24" t="inlineStr">
-        <is>
-          <t>NOPAT Bridge tab: channel margin calibration</t>
+          <t>18.6% of store-channel revenue (EBIT margin assumption).
+EBIT_store = Rev_store × Margin_store
+FY25 check: 5,049,744 × 18.6% ≈ 939,252 ($000).
+Calibrated so Σ channel EBIT ≈ consolidated EBIT 2,210,615 (10-K).</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: company-operated stores net revenue</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Channel margin assumption — calibrated so FY25 store rev × 18.6% + e-comm × 23.6% + other × 9.1% ≈ reported EBIT.</t>
+          <t>Ctrl+F "Company-operated stores"
+→ 5,049,744 ($000) net revenue
+× 18.6% margin assumption → store EBIT ≈ 939,252 ($000)</t>
         </is>
       </c>
       <c r="E8" s="20" t="n">
@@ -7246,7 +7251,7 @@
         <v>0.186</v>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
+    <row r="9" ht="56" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Phase 3: E-commerce EBIT margin %</t>
@@ -7254,17 +7259,22 @@
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>23.6% EBIT margin on e-commerce revenue. Higher than stores (no occupancy).</t>
-        </is>
-      </c>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>NOPAT Bridge tab: channel margin calibration</t>
+          <t>23.6% of e-commerce revenue (EBIT margin assumption).
+EBIT_e-comm = Rev_e-comm × Margin_e-comm
+FY25 check: 4,918,697 × 23.6% ≈ 1,160,812 ($000).
+Higher than stores — no occupancy; fulfillment + digital marketing only.</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: e-commerce net revenue</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>E-commerce EBIT margin 23.6% — higher than stores (no occupancy drag).</t>
+          <t>Ctrl+F "E-commerce"
+→ 4,918,697 ($000) net revenue
+× 23.6% margin assumption → e-comm EBIT ≈ 1,160,812 ($000)</t>
         </is>
       </c>
       <c r="E9" s="20" t="n">
@@ -7286,7 +7296,7 @@
         <v>0.236</v>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
+    <row r="10" ht="56" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Phase 3: Other-channels EBIT margin %</t>
@@ -7294,17 +7304,22 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>9.1% EBIT margin on wholesale/license/outlets — lower-margin residual channel.</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>NOPAT Bridge tab: channel margin calibration</t>
+          <t>9.1% of other-channel revenue (EBIT margin assumption).
+EBIT_other = Rev_other × Margin_other
+FY25 check: 1,134,159 × 9.1% ≈ 103,209 ($000).
+Wholesale/license/outlets — lower-margin residual channel.</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: other channels (residual)</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Other channels 9.1% — wholesale/license/outlets residual margin.</t>
+          <t>Ctrl+F "Net revenue" → 11,102,600
+Minus stores + e-comm → other channels ≈ 1,134,159 ($000)
+× 9.1% margin assumption → other EBIT ≈ 103,209 ($000)</t>
         </is>
       </c>
       <c r="E10" s="20" t="n">
@@ -7981,188 +7996,337 @@
         <v/>
       </c>
     </row>
-    <row r="30" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A30" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Channel EBIT (= Sum Rev_i x Margin_i)</t>
+    <row r="30" hidden="1" outlineLevel="1" ht="56" customHeight="1">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Store-channel EBIT (= Rev × store margin)</t>
         </is>
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>Phase 3 channel EBIT = Σ(Revenue_i × Margin_i). FY26 adds Scenarios tariff refund.</t>
-        </is>
-      </c>
-      <c r="C30" s="24" t="inlineStr">
-        <is>
-          <t>NOPAT Bridge tab: channel EBIT formula</t>
+          <t>18.6% of store-channel revenue.
+EBIT_store,t = Rev_store,t × Margin_store
+FY25: 5,049,744 × 18.6% ≈ 939,252 ($000).
+Margin from driver assumptions row above; ties to 10-K store revenue.</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: company-operated stores net revenue</t>
         </is>
       </c>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>Σ channel revenue × margin. FY26 adds Scenarios tariff refund cell.</t>
-        </is>
-      </c>
-      <c r="F30" s="69">
-        <f>F27*E$8+F28*E$9+F29*E$10+Scenarios!G7</f>
-        <v/>
-      </c>
-      <c r="G30" s="69">
-        <f>G27*E$8+G28*E$9+G29*E$10</f>
-        <v/>
-      </c>
-      <c r="H30" s="69">
-        <f>H27*E$8+H28*E$9+H29*E$10</f>
-        <v/>
-      </c>
-      <c r="I30" s="69">
-        <f>I27*E$8+I28*E$9+I29*E$10</f>
-        <v/>
-      </c>
-      <c r="J30" s="69">
-        <f>J27*E$8+J28*E$9+J29*E$10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A31" s="23">
+          <t>Ctrl+F "Company-operated stores"
+→ 5,049,744 ($000)
+EBIT = Rev × 18.6% → ≈ 939,252 ($000)</t>
+        </is>
+      </c>
+      <c r="E30" s="74" t="n">
+        <v>939252.384</v>
+      </c>
+      <c r="F30" s="74">
+        <f>F27*E$8</f>
+        <v/>
+      </c>
+      <c r="G30" s="74">
+        <f>G27*E$8</f>
+        <v/>
+      </c>
+      <c r="H30" s="74">
+        <f>H27*E$8</f>
+        <v/>
+      </c>
+      <c r="I30" s="74">
+        <f>I27*E$8</f>
+        <v/>
+      </c>
+      <c r="J30" s="74">
+        <f>J27*E$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" hidden="1" outlineLevel="1" ht="56" customHeight="1">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  E-commerce EBIT (= Rev × e-comm margin)</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>23.6% of e-commerce revenue.
+EBIT_e-comm,t = Rev_e-comm,t × Margin_e-comm
+FY25: 4,918,697 × 23.6% ≈ 1,160,812 ($000).
+Higher than stores — no brick-and-mortar occupancy drag.</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: e-commerce net revenue</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "E-commerce"
+→ 4,918,697 ($000)
+EBIT = Rev × 23.6% → ≈ 1,160,812 ($000)</t>
+        </is>
+      </c>
+      <c r="E31" s="74" t="n">
+        <v>1160812.492</v>
+      </c>
+      <c r="F31" s="74">
+        <f>F28*E$9</f>
+        <v/>
+      </c>
+      <c r="G31" s="74">
+        <f>G28*E$9</f>
+        <v/>
+      </c>
+      <c r="H31" s="74">
+        <f>H28*E$9</f>
+        <v/>
+      </c>
+      <c r="I31" s="74">
+        <f>I28*E$9</f>
+        <v/>
+      </c>
+      <c r="J31" s="74">
+        <f>J28*E$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" hidden="1" outlineLevel="1" ht="42" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Other-channels EBIT (= Rev × other margin)</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>9.1% of other-channel revenue.
+EBIT_other,t = Rev_other,t × Margin_other
+FY25: 1,134,159 × 9.1% ≈ 103,209 ($000).
+Wholesale/license/outlets — lowest channel margin.</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>FY2025 10-K: other channels (residual)</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>Other rev = 11,102,600 − 5,049,744 − 4,918,697 ≈ 1,134,159 ($000)
+EBIT = Rev × 9.1% → ≈ 103,209 ($000)</t>
+        </is>
+      </c>
+      <c r="E32" s="74" t="n">
+        <v>103208.469</v>
+      </c>
+      <c r="F32" s="74">
+        <f>F29*E$10</f>
+        <v/>
+      </c>
+      <c r="G32" s="74">
+        <f>G29*E$10</f>
+        <v/>
+      </c>
+      <c r="H32" s="74">
+        <f>H29*E$10</f>
+        <v/>
+      </c>
+      <c r="I32" s="74">
+        <f>I29*E$10</f>
+        <v/>
+      </c>
+      <c r="J32" s="74">
+        <f>J29*E$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Channel EBIT (sum of sector EBIT)</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>Phase 3 channel EBIT = Σ sector EBIT_i. FY26 adds Scenarios tariff refund.</t>
+        </is>
+      </c>
+      <c r="C33" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge tab: sector EBIT subtotal</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="inlineStr">
+        <is>
+          <t>Sum of sector EBIT rows. FY26 adds Scenarios tariff refund cell.</t>
+        </is>
+      </c>
+      <c r="F33" s="69">
+        <f>F30+F31+F32+Scenarios!G7</f>
+        <v/>
+      </c>
+      <c r="G33" s="69">
+        <f>G30+G31+G32</f>
+        <v/>
+      </c>
+      <c r="H33" s="69">
+        <f>H30+H31+H32</f>
+        <v/>
+      </c>
+      <c r="I33" s="69">
+        <f>I30+I31+I32</f>
+        <v/>
+      </c>
+      <c r="J33" s="69">
+        <f>J30+J31+J32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A34" s="23">
         <f> EBIT after channel mix (Phase 3)</f>
         <v/>
       </c>
-      <c r="B31" s="17" t="inlineStr">
+      <c r="B34" s="17" t="inlineStr">
         <is>
           <t>Channel-mix EBIT output (Phase 3). Check row vs Scenarios shows channel vs margin-path gap.</t>
         </is>
       </c>
-      <c r="C31" s="24" t="inlineStr">
+      <c r="C34" s="24" t="inlineStr">
         <is>
           <t>NOPAT Bridge tab: Phase 3 subtotal</t>
         </is>
       </c>
-      <c r="D31" s="19" t="inlineStr">
+      <c r="D34" s="19" t="inlineStr">
         <is>
           <t>Channel EBIT subtotal (Phase 3). Compare Check row vs Scenarios.</t>
         </is>
       </c>
-      <c r="E31" s="75" t="n">
+      <c r="E34" s="75" t="n">
         <v>2203273.345</v>
       </c>
-      <c r="F31" s="25">
-        <f>F30</f>
-        <v/>
-      </c>
-      <c r="G31" s="25">
-        <f>G30</f>
-        <v/>
-      </c>
-      <c r="H31" s="25">
-        <f>H30</f>
-        <v/>
-      </c>
-      <c r="I31" s="25">
-        <f>I30</f>
-        <v/>
-      </c>
-      <c r="J31" s="25">
-        <f>J30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A32" s="23">
+      <c r="F34" s="25">
+        <f>F33</f>
+        <v/>
+      </c>
+      <c r="G34" s="25">
+        <f>G33</f>
+        <v/>
+      </c>
+      <c r="H34" s="25">
+        <f>H33</f>
+        <v/>
+      </c>
+      <c r="I34" s="25">
+        <f>I33</f>
+        <v/>
+      </c>
+      <c r="J34" s="25">
+        <f>J33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A35" s="23">
         <f> Normalized EBIT (tax base for NOPAT)</f>
         <v/>
       </c>
-      <c r="B32" s="17" t="inlineStr">
+      <c r="B35" s="17" t="inlineStr">
         <is>
           <t>FY25: Phases 1–2 walk-through. Forecast: Scenarios base EBIT — tax base for NOPAT.</t>
         </is>
       </c>
-      <c r="C32" s="24" t="inlineStr">
+      <c r="C35" s="24" t="inlineStr">
         <is>
           <t>Scenarios tab: base-case EBIT (forecast)</t>
         </is>
       </c>
-      <c r="D32" s="19" t="inlineStr">
+      <c r="D35" s="19" t="inlineStr">
         <is>
           <t>FY25: Phase 1–2 formula. Forecast: Scenarios base EBIT (tax base).</t>
         </is>
       </c>
-      <c r="E32" s="25">
+      <c r="E35" s="25">
         <f>E20+E22+E23-E24</f>
         <v/>
       </c>
-      <c r="F32" s="25">
+      <c r="F35" s="25">
         <f>Scenarios!G43</f>
         <v/>
       </c>
-      <c r="G32" s="25">
+      <c r="G35" s="25">
         <f>Scenarios!G44</f>
         <v/>
       </c>
-      <c r="H32" s="25">
+      <c r="H35" s="25">
         <f>Scenarios!G45</f>
         <v/>
       </c>
-      <c r="I32" s="25">
+      <c r="I35" s="25">
         <f>Scenarios!G46</f>
         <v/>
       </c>
-      <c r="J32" s="25">
+      <c r="J35" s="25">
         <f>Scenarios!G47</f>
         <v/>
       </c>
     </row>
-    <row r="33" hidden="1" outlineLevel="1">
-      <c r="A33" s="16" t="inlineStr">
+    <row r="36" hidden="1" outlineLevel="1">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Check vs Scenarios EBIT (base case)</t>
         </is>
       </c>
-      <c r="F33" s="74">
-        <f>F32-Scenarios!G43</f>
-        <v/>
-      </c>
-      <c r="G33" s="74">
-        <f>G32-Scenarios!G44</f>
-        <v/>
-      </c>
-      <c r="H33" s="74">
-        <f>H32-Scenarios!G45</f>
-        <v/>
-      </c>
-      <c r="I33" s="74">
-        <f>I32-Scenarios!G46</f>
-        <v/>
-      </c>
-      <c r="J33" s="74">
-        <f>J32-Scenarios!G47</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" hidden="1" outlineLevel="1">
-      <c r="A34" s="72" t="inlineStr">
+      <c r="F36" s="74">
+        <f>F35-Scenarios!G43</f>
+        <v/>
+      </c>
+      <c r="G36" s="74">
+        <f>G35-Scenarios!G44</f>
+        <v/>
+      </c>
+      <c r="H36" s="74">
+        <f>H35-Scenarios!G45</f>
+        <v/>
+      </c>
+      <c r="I36" s="74">
+        <f>I35-Scenarios!G46</f>
+        <v/>
+      </c>
+      <c r="J36" s="74">
+        <f>J35-Scenarios!G47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" hidden="1" outlineLevel="1">
+      <c r="A37" s="72" t="inlineStr">
         <is>
           <t>Phase 4 — Tax normalization to NOPAT</t>
         </is>
       </c>
     </row>
-    <row r="35" hidden="1" outlineLevel="1" ht="70" customHeight="1">
-      <c r="A35" s="16" t="inlineStr">
+    <row r="38" hidden="1" outlineLevel="1" ht="70" customHeight="1">
+      <c r="A38" s="16" t="inlineStr">
         <is>
           <t>Operating effective tax rate (t_operating)</t>
         </is>
       </c>
-      <c r="B35" s="17" t="inlineStr">
+      <c r="B38" s="17" t="inlineStr">
         <is>
           <t>Operating effective tax rate: (tax + interest shield) ÷ (EBT + interest). Transitions from FY25 t_operating toward 30% marginal over 5 years.</t>
         </is>
       </c>
-      <c r="C35" s="18" t="inlineStr">
+      <c r="C38" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: income tax &amp; interest expense</t>
         </is>
       </c>
-      <c r="D35" s="19" t="inlineStr">
+      <c r="D38" s="19" t="inlineStr">
         <is>
           <t>t_operating = (tax + interest×30%) ÷ (EBT + interest).
 Ctrl+F "Income tax expense" → 659,784
@@ -8170,233 +8334,233 @@
 Ctrl+F "Interest paid on lease liabilities" → 1,028</t>
         </is>
       </c>
-      <c r="E35" s="76" t="n">
+      <c r="E38" s="76" t="n">
         <v>0.2946847649213503</v>
       </c>
-      <c r="F35" s="32">
+      <c r="F38" s="32">
         <f>0.29468476492135026+(F$11-0.29468476492135026)*1/5</f>
         <v/>
       </c>
-      <c r="G35" s="32">
+      <c r="G38" s="32">
         <f>0.29468476492135026+(G$11-0.29468476492135026)*2/5</f>
         <v/>
       </c>
-      <c r="H35" s="32">
+      <c r="H38" s="32">
         <f>0.29468476492135026+(H$11-0.29468476492135026)*3/5</f>
         <v/>
       </c>
-      <c r="I35" s="32">
+      <c r="I38" s="32">
         <f>0.29468476492135026+(I$11-0.29468476492135026)*4/5</f>
         <v/>
       </c>
-      <c r="J35" s="32">
+      <c r="J38" s="32">
         <f>0.29468476492135026+(J$11-0.29468476492135026)*5/5</f>
         <v/>
       </c>
     </row>
-    <row r="36" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A36" s="16" t="inlineStr">
+    <row r="39" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A39" s="16" t="inlineStr">
         <is>
           <t>Unlevered tax on normalized EBIT</t>
         </is>
       </c>
-      <c r="B36" s="17" t="inlineStr">
+      <c r="B39" s="17" t="inlineStr">
         <is>
           <t>Unlevered tax = normalized EBIT × t_operating. Strips debt-interest tax shield from GAAP rate.</t>
         </is>
       </c>
-      <c r="C36" s="24" t="inlineStr">
+      <c r="C39" s="24" t="inlineStr">
         <is>
           <t>NOPAT Bridge tab: unlevered tax expense</t>
         </is>
       </c>
-      <c r="D36" s="19" t="inlineStr">
+      <c r="D39" s="19" t="inlineStr">
         <is>
           <t>Normalized EBIT × t_operating — unlevered tax (no debt shield).</t>
         </is>
       </c>
-      <c r="F36" s="74">
-        <f>F32*F35</f>
-        <v/>
-      </c>
-      <c r="G36" s="74">
-        <f>G32*G35</f>
-        <v/>
-      </c>
-      <c r="H36" s="74">
-        <f>H32*H35</f>
-        <v/>
-      </c>
-      <c r="I36" s="74">
-        <f>I32*I35</f>
-        <v/>
-      </c>
-      <c r="J36" s="74">
-        <f>J32*J35</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A37" s="23" t="inlineStr">
+      <c r="F39" s="74">
+        <f>F35*F38</f>
+        <v/>
+      </c>
+      <c r="G39" s="74">
+        <f>G35*G38</f>
+        <v/>
+      </c>
+      <c r="H39" s="74">
+        <f>H35*H38</f>
+        <v/>
+      </c>
+      <c r="I39" s="74">
+        <f>I35*I38</f>
+        <v/>
+      </c>
+      <c r="J39" s="74">
+        <f>J35*J38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A40" s="23" t="inlineStr">
         <is>
           <t>NORMALIZED NOPAT</t>
         </is>
       </c>
-      <c r="B37" s="17" t="inlineStr">
+      <c r="B40" s="17" t="inlineStr">
         <is>
           <t>NORMALIZED NOPAT = EBIT_norm × (1 − t_operating). Scenarios base case links here.</t>
         </is>
       </c>
-      <c r="C37" s="24" t="inlineStr">
+      <c r="C40" s="24" t="inlineStr">
         <is>
           <t>NOPAT Bridge tab: normalized NOPAT</t>
         </is>
       </c>
-      <c r="D37" s="19" t="inlineStr">
+      <c r="D40" s="19" t="inlineStr">
         <is>
           <t>EBIT_norm − unlevered tax. Scenarios base-case NOPAT links to this row.</t>
         </is>
       </c>
-      <c r="F37" s="25">
-        <f>F32-F36</f>
-        <v/>
-      </c>
-      <c r="G37" s="25">
-        <f>G32-G36</f>
-        <v/>
-      </c>
-      <c r="H37" s="25">
-        <f>H32-H36</f>
-        <v/>
-      </c>
-      <c r="I37" s="25">
-        <f>I32-I36</f>
-        <v/>
-      </c>
-      <c r="J37" s="25">
-        <f>J32-J36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="72" t="inlineStr">
+      <c r="F40" s="25">
+        <f>F35-F39</f>
+        <v/>
+      </c>
+      <c r="G40" s="25">
+        <f>G35-G39</f>
+        <v/>
+      </c>
+      <c r="H40" s="25">
+        <f>H35-H39</f>
+        <v/>
+      </c>
+      <c r="I40" s="25">
+        <f>I35-I39</f>
+        <v/>
+      </c>
+      <c r="J40" s="25">
+        <f>J35-J39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="72" t="inlineStr">
         <is>
           <t>Phase 5 — Agent workflow (execution steps)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="60" t="inlineStr">
-        <is>
-          <t>1. Clean base</t>
-        </is>
-      </c>
-      <c r="B40" s="77" t="inlineStr">
-        <is>
-          <t>SEC 10-K income statement</t>
-        </is>
-      </c>
-      <c r="D40" s="26" t="inlineStr">
-        <is>
-          <t>Add back impairments, restructuring, M&amp;A; optional SBC add-back.</t>
-        </is>
-      </c>
-      <c r="F40" s="78" t="inlineStr">
-        <is>
-          <t>EBIT_adj (Phase 1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="60" t="inlineStr">
-        <is>
-          <t>2. Capitalize R&amp;D</t>
-        </is>
-      </c>
-      <c r="B41" s="77" t="inlineStr">
-        <is>
-          <t>SG&amp;A footnotes</t>
-        </is>
-      </c>
-      <c r="D41" s="26" t="inlineStr">
-        <is>
-          <t>Capitalize multi-year software/R&amp;D; amortize over N years.</t>
-        </is>
-      </c>
-      <c r="F41" s="78" t="inlineStr">
-        <is>
-          <t>EBIT_lease-adj (Phase 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="60" t="inlineStr">
-        <is>
-          <t>3. Lease shift</t>
-        </is>
-      </c>
-      <c r="B42" s="77" t="inlineStr">
-        <is>
-          <t>ASC 842 lease footnote</t>
-        </is>
-      </c>
-      <c r="D42" s="26" t="inlineStr">
-        <is>
-          <t>Add implied lease interest; standardize to unlevered EBIT.</t>
-        </is>
-      </c>
-      <c r="F42" s="78" t="inlineStr">
-        <is>
-          <t>EBIT_capitalized</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="60" t="inlineStr">
         <is>
-          <t>4. Segment mix</t>
+          <t>1. Clean base</t>
         </is>
       </c>
       <c r="B43" s="77" t="inlineStr">
         <is>
-          <t>Revenue Drivers tab</t>
+          <t>SEC 10-K income statement</t>
         </is>
       </c>
       <c r="D43" s="26" t="inlineStr">
         <is>
-          <t>Blend store / e-comm / other EBIT margins by channel revenue share.</t>
+          <t>Add back impairments, restructuring, M&amp;A; optional SBC add-back.</t>
         </is>
       </c>
       <c r="F43" s="78" t="inlineStr">
         <is>
-          <t>Forecast EBIT</t>
+          <t>EBIT_adj (Phase 1)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="60" t="inlineStr">
         <is>
+          <t>2. Capitalize R&amp;D</t>
+        </is>
+      </c>
+      <c r="B44" s="77" t="inlineStr">
+        <is>
+          <t>SG&amp;A footnotes</t>
+        </is>
+      </c>
+      <c r="D44" s="26" t="inlineStr">
+        <is>
+          <t>Capitalize multi-year software/R&amp;D; amortize over N years.</t>
+        </is>
+      </c>
+      <c r="F44" s="78" t="inlineStr">
+        <is>
+          <t>EBIT_lease-adj (Phase 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="60" t="inlineStr">
+        <is>
+          <t>3. Lease shift</t>
+        </is>
+      </c>
+      <c r="B45" s="77" t="inlineStr">
+        <is>
+          <t>ASC 842 lease footnote</t>
+        </is>
+      </c>
+      <c r="D45" s="26" t="inlineStr">
+        <is>
+          <t>Add implied lease interest; standardize to unlevered EBIT.</t>
+        </is>
+      </c>
+      <c r="F45" s="78" t="inlineStr">
+        <is>
+          <t>EBIT_capitalized</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="60" t="inlineStr">
+        <is>
+          <t>4. Segment mix</t>
+        </is>
+      </c>
+      <c r="B46" s="77" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab</t>
+        </is>
+      </c>
+      <c r="D46" s="26" t="inlineStr">
+        <is>
+          <t>Blend store / e-comm / other EBIT margins by channel revenue share.</t>
+        </is>
+      </c>
+      <c r="F46" s="78" t="inlineStr">
+        <is>
+          <t>Forecast EBIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="60" t="inlineStr">
+        <is>
           <t>5. NOPAT bridge</t>
         </is>
       </c>
-      <c r="B44" s="77" t="inlineStr">
+      <c r="B47" s="77" t="inlineStr">
         <is>
           <t>Normalized EBIT &amp; t_operating</t>
         </is>
       </c>
-      <c r="D44" s="26" t="inlineStr">
+      <c r="D47" s="26" t="inlineStr">
         <is>
           <t>NOPAT = EBIT x (1 - t); transition t toward marginal rate.</t>
         </is>
       </c>
-      <c r="F44" s="78" t="inlineStr">
+      <c r="F47" s="78" t="inlineStr">
         <is>
           <t>Normalized NOPAT</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="26" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="26" t="inlineStr">
         <is>
           <t>Scenarios base-case NOPAT (col G) links to NORMALIZED NOPAT above. Bear/bull apply the same t_operating to their EBIT paths.</t>
         </is>
@@ -8405,32 +8569,38 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId21"/>
     <hyperlink ref="C27" location="'Revenue Drivers'!B31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId22"/>
     <hyperlink ref="C28" location="'Revenue Drivers'!B41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId23"/>
     <hyperlink ref="C29" location="'Revenue Drivers'!B45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8905,23 +9075,23 @@
         </is>
       </c>
       <c r="F13" s="74">
-        <f>-'NOPAT Bridge'!F36</f>
+        <f>-'NOPAT Bridge'!F39</f>
         <v/>
       </c>
       <c r="G13" s="74">
-        <f>-'NOPAT Bridge'!G36</f>
+        <f>-'NOPAT Bridge'!G39</f>
         <v/>
       </c>
       <c r="H13" s="74">
-        <f>-'NOPAT Bridge'!H36</f>
+        <f>-'NOPAT Bridge'!H39</f>
         <v/>
       </c>
       <c r="I13" s="74">
-        <f>-'NOPAT Bridge'!I36</f>
+        <f>-'NOPAT Bridge'!I39</f>
         <v/>
       </c>
       <c r="J13" s="74">
-        <f>-'NOPAT Bridge'!J36</f>
+        <f>-'NOPAT Bridge'!J39</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Lead NOPAT Bridge channel margin justifications with per-channel EBIT %
Clarify that 18.6%/23.6%/9.1% are EBIT as a percent of each channel's
own revenue, not the Scenarios 13.2%-15.5% consolidated EBIT margin.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -7214,7 +7214,8 @@
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>18.6% of store-channel revenue (EBIT margin assumption).
+          <t>Not % of consolidated revenue — EBIT as % of store-channel revenue only (not the Scenarios 13.2%–15.5% consolidated margin).
+18.6% margin assumption.
 EBIT_store = Rev_store × Margin_store
 FY25 check: 5,049,744 × 18.6% ≈ 939,252 ($000).
 Calibrated so Σ channel EBIT ≈ consolidated EBIT 2,210,615 (10-K).</t>
@@ -7259,7 +7260,8 @@
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>23.6% of e-commerce revenue (EBIT margin assumption).
+          <t>Not % of consolidated revenue — EBIT as % of e-commerce revenue only (not the Scenarios 13.2%–15.5% consolidated margin).
+23.6% margin assumption.
 EBIT_e-comm = Rev_e-comm × Margin_e-comm
 FY25 check: 4,918,697 × 23.6% ≈ 1,160,812 ($000).
 Higher than stores — no occupancy; fulfillment + digital marketing only.</t>
@@ -7304,7 +7306,8 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>9.1% of other-channel revenue (EBIT margin assumption).
+          <t>Not % of consolidated revenue — EBIT as % of other-channel revenue only (not the Scenarios 13.2%–15.5% consolidated margin).
+9.1% margin assumption.
 EBIT_other = Rev_other × Margin_other
 FY25 check: 1,134,159 × 9.1% ≈ 103,209 ($000).
 Wholesale/license/outlets — lower-margin residual channel.</t>

</xml_diff>

<commit_message>
Add without/with FY26 DCF impact columns to NOPAT Bridge Phase 5
Phase 5 workflow table now shows what each step looks like with and
without applied on FY26 DCF EBIT/NOPAT, including a tariff refund row.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -259,6 +259,12 @@
     </font>
     <font>
       <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="00C8102E"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
       <color rgb="00000000"/>
       <sz val="8"/>
     </font>
@@ -285,12 +291,6 @@
       <i val="1"/>
       <color rgb="00F2F2F2"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Garamond"/>
-      <b val="1"/>
-      <color rgb="00C8102E"/>
-      <sz val="8"/>
     </font>
     <font>
       <name val="Garamond"/>
@@ -611,27 +611,27 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -656,7 +656,7 @@
     <xf numFmtId="169" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="47" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -7066,15 +7066,15 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
-    <col hidden="1" outlineLevel="1" width="26" customWidth="1" min="2" max="2"/>
-    <col hidden="1" outlineLevel="1" width="16" customWidth="1" min="3" max="3"/>
-    <col hidden="1" outlineLevel="1" width="38" customWidth="1" min="4" max="4"/>
+    <col hidden="1" outlineLevel="1" width="22" customWidth="1" min="2" max="2"/>
+    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="3" max="3"/>
+    <col hidden="1" outlineLevel="1" width="28" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
@@ -7206,7 +7206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" ht="56" customHeight="1">
+    <row r="8" ht="70" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Phase 3: Store-channel EBIT margin %</t>
@@ -7228,7 +7228,8 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Company-operated stores"
+          <t>Not consolidated EBIT margin — EBIT ÷ store revenue only (cf. Scenarios 13.2%–15.5%).
+Ctrl+F "Company-operated stores"
 → 5,049,744 ($000) net revenue
 × 18.6% margin assumption → store EBIT ≈ 939,252 ($000)</t>
         </is>
@@ -7252,7 +7253,7 @@
         <v>0.186</v>
       </c>
     </row>
-    <row r="9" ht="56" customHeight="1">
+    <row r="9" ht="70" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Phase 3: E-commerce EBIT margin %</t>
@@ -7274,7 +7275,8 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "E-commerce"
+          <t>Not consolidated EBIT margin — EBIT ÷ e-commerce revenue only (cf. Scenarios 13.2%–15.5%).
+Ctrl+F "E-commerce"
 → 4,918,697 ($000) net revenue
 × 23.6% margin assumption → e-comm EBIT ≈ 1,160,812 ($000)</t>
         </is>
@@ -7298,7 +7300,7 @@
         <v>0.236</v>
       </c>
     </row>
-    <row r="10" ht="56" customHeight="1">
+    <row r="10" ht="70" customHeight="1">
       <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Phase 3: Other-channels EBIT margin %</t>
@@ -7320,7 +7322,8 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Net revenue" → 11,102,600
+          <t>Not consolidated EBIT margin — EBIT ÷ other-channel revenue only (cf. Scenarios 13.2%–15.5%).
+Ctrl+F "Net revenue" → 11,102,600
 Minus stores + e-comm → other channels ≈ 1,134,159 ($000)
 × 9.1% margin assumption → other EBIT ≈ 103,209 ($000)</t>
         </is>
@@ -7999,7 +8002,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" hidden="1" outlineLevel="1" ht="56" customHeight="1">
+    <row r="30" hidden="1" outlineLevel="1" ht="70" customHeight="1">
       <c r="A30" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Store-channel EBIT (= Rev × store margin)</t>
@@ -8007,8 +8010,8 @@
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>18.6% of store-channel revenue.
-EBIT_store,t = Rev_store,t × Margin_store
+          <t>Not % of consolidated revenue — store EBIT ÷ store revenue only (not Scenarios consolidated EBIT margin).
+EBIT_store,t = Rev_store,t × 18.6%
 FY25: 5,049,744 × 18.6% ≈ 939,252 ($000).
 Margin from driver assumptions row above; ties to 10-K store revenue.</t>
         </is>
@@ -8020,7 +8023,8 @@
       </c>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Company-operated stores"
+          <t>Not consolidated EBIT margin — store EBIT ÷ store revenue only.
+Ctrl+F "Company-operated stores"
 → 5,049,744 ($000)
 EBIT = Rev × 18.6% → ≈ 939,252 ($000)</t>
         </is>
@@ -8049,7 +8053,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" hidden="1" outlineLevel="1" ht="56" customHeight="1">
+    <row r="31" hidden="1" outlineLevel="1" ht="70" customHeight="1">
       <c r="A31" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  E-commerce EBIT (= Rev × e-comm margin)</t>
@@ -8057,8 +8061,8 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>23.6% of e-commerce revenue.
-EBIT_e-comm,t = Rev_e-comm,t × Margin_e-comm
+          <t>Not % of consolidated revenue — e-commerce EBIT ÷ e-commerce revenue only (not Scenarios consolidated EBIT margin).
+EBIT_e-comm,t = Rev_e-comm,t × 23.6%
 FY25: 4,918,697 × 23.6% ≈ 1,160,812 ($000).
 Higher than stores — no brick-and-mortar occupancy drag.</t>
         </is>
@@ -8070,7 +8074,8 @@
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "E-commerce"
+          <t>Not consolidated EBIT margin — e-commerce EBIT ÷ e-commerce revenue only.
+Ctrl+F "E-commerce"
 → 4,918,697 ($000)
 EBIT = Rev × 23.6% → ≈ 1,160,812 ($000)</t>
         </is>
@@ -8099,7 +8104,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" hidden="1" outlineLevel="1" ht="42" customHeight="1">
+    <row r="32" hidden="1" outlineLevel="1" ht="56" customHeight="1">
       <c r="A32" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Other-channels EBIT (= Rev × other margin)</t>
@@ -8107,8 +8112,8 @@
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>9.1% of other-channel revenue.
-EBIT_other,t = Rev_other,t × Margin_other
+          <t>Not % of consolidated revenue — other-channel EBIT ÷ other revenue only (not Scenarios consolidated EBIT margin).
+EBIT_other,t = Rev_other,t × 9.1%
 FY25: 1,134,159 × 9.1% ≈ 103,209 ($000).
 Wholesale/license/outlets — lowest channel margin.</t>
         </is>
@@ -8120,7 +8125,8 @@
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>Other rev = 11,102,600 − 5,049,744 − 4,918,697 ≈ 1,134,159 ($000)
+          <t>Not consolidated EBIT margin — other-channel EBIT ÷ other revenue only.
+Other rev = 11,102,600 − 5,049,744 − 4,918,697 ≈ 1,134,159 ($000)
 EBIT = Rev × 9.1% → ≈ 103,209 ($000)</t>
         </is>
       </c>
@@ -8453,117 +8459,198 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="60" t="inlineStr">
-        <is>
-          <t>1. Clean base</t>
-        </is>
-      </c>
       <c r="B43" s="77" t="inlineStr">
         <is>
-          <t>SEC 10-K income statement</t>
-        </is>
-      </c>
-      <c r="D43" s="26" t="inlineStr">
-        <is>
-          <t>Add back impairments, restructuring, M&amp;A; optional SBC add-back.</t>
-        </is>
-      </c>
-      <c r="F43" s="78" t="inlineStr">
-        <is>
-          <t>EBIT_adj (Phase 1)</t>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C43" s="77" t="inlineStr">
+        <is>
+          <t>Without applied (FY26 DCF)</t>
+        </is>
+      </c>
+      <c r="D43" s="77" t="inlineStr">
+        <is>
+          <t>With applied (FY26 DCF)</t>
+        </is>
+      </c>
+      <c r="F43" s="77" t="inlineStr">
+        <is>
+          <t>Output</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="60" t="inlineStr">
         <is>
-          <t>2. Capitalize R&amp;D</t>
-        </is>
-      </c>
-      <c r="B44" s="77" t="inlineStr">
-        <is>
-          <t>SG&amp;A footnotes</t>
-        </is>
-      </c>
-      <c r="D44" s="26" t="inlineStr">
-        <is>
-          <t>Capitalize multi-year software/R&amp;D; amortize over N years.</t>
-        </is>
-      </c>
-      <c r="F44" s="78" t="inlineStr">
-        <is>
-          <t>EBIT_lease-adj (Phase 2)</t>
+          <t>1. Clean base</t>
+        </is>
+      </c>
+      <c r="B44" s="78" t="inlineStr">
+        <is>
+          <t>SEC 10-K income statement</t>
+        </is>
+      </c>
+      <c r="C44" s="78" t="inlineStr">
+        <is>
+          <t>FY26 EBIT = Rev × 13.2% + tariff. No impairment/SBC/restructuring add-backs in forecast.</t>
+        </is>
+      </c>
+      <c r="D44" s="78" t="inlineStr">
+        <is>
+          <t>Would lift EBIT by adding back one-offs + SBC — runs on FY25 history only; FY26 DCF unchanged.</t>
+        </is>
+      </c>
+      <c r="F44" s="79" t="inlineStr">
+        <is>
+          <t>EBIT_adj (Phase 1)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="60" t="inlineStr">
         <is>
-          <t>3. Lease shift</t>
-        </is>
-      </c>
-      <c r="B45" s="77" t="inlineStr">
-        <is>
-          <t>ASC 842 lease footnote</t>
-        </is>
-      </c>
-      <c r="D45" s="26" t="inlineStr">
-        <is>
-          <t>Add implied lease interest; standardize to unlevered EBIT.</t>
-        </is>
-      </c>
-      <c r="F45" s="78" t="inlineStr">
-        <is>
-          <t>EBIT_capitalized</t>
+          <t>2. Capitalize R&amp;D</t>
+        </is>
+      </c>
+      <c r="B45" s="78" t="inlineStr">
+        <is>
+          <t>SG&amp;A footnotes</t>
+        </is>
+      </c>
+      <c r="C45" s="78" t="inlineStr">
+        <is>
+          <t>R&amp;D/software expensed in full each year. LULU = $0 cap; no FY26 EBIT change.</t>
+        </is>
+      </c>
+      <c r="D45" s="78" t="inlineStr">
+        <is>
+          <t>Would spread expense over 4 yrs (cap + amort) — higher near-term EBIT; not wired to FY26 DCF.</t>
+        </is>
+      </c>
+      <c r="F45" s="79" t="inlineStr">
+        <is>
+          <t>EBIT_capitalized (Phase 2)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="60" t="inlineStr">
         <is>
-          <t>4. Segment mix</t>
-        </is>
-      </c>
-      <c r="B46" s="77" t="inlineStr">
-        <is>
-          <t>Revenue Drivers tab</t>
-        </is>
-      </c>
-      <c r="D46" s="26" t="inlineStr">
-        <is>
-          <t>Blend store / e-comm / other EBIT margins by channel revenue share.</t>
-        </is>
-      </c>
-      <c r="F46" s="78" t="inlineStr">
-        <is>
-          <t>Forecast EBIT</t>
+          <t>3. Lease shift</t>
+        </is>
+      </c>
+      <c r="B46" s="78" t="inlineStr">
+        <is>
+          <t>ASC 842 lease footnote</t>
+        </is>
+      </c>
+      <c r="C46" s="78" t="inlineStr">
+        <is>
+          <t>Rent stays in operating costs; no lease-interest add-back. FY26 DCF EBIT unchanged.</t>
+        </is>
+      </c>
+      <c r="D46" s="78" t="inlineStr">
+        <is>
+          <t>Would add implied lease interest to EBIT (unlevered) — FY25 bridge only; FY26 DCF same.</t>
+        </is>
+      </c>
+      <c r="F46" s="79" t="inlineStr">
+        <is>
+          <t>EBIT_lease-adj (Phase 2)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="60" t="inlineStr">
         <is>
+          <t>4. Segment mix</t>
+        </is>
+      </c>
+      <c r="B47" s="78" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab</t>
+        </is>
+      </c>
+      <c r="C47" s="78" t="inlineStr">
+        <is>
+          <t>DCF uses consolidated 13.2% on total revenue (+ tariff). Channel EBIT not used.</t>
+        </is>
+      </c>
+      <c r="D47" s="78" t="inlineStr">
+        <is>
+          <t>Channel EBIT = Σ(Rev_i × margin_i) — higher illustrative EBIT; check row shows gap vs Scenarios.</t>
+        </is>
+      </c>
+      <c r="F47" s="79" t="inlineStr">
+        <is>
+          <t>Forecast EBIT (Phase 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="60" t="inlineStr">
+        <is>
           <t>5. NOPAT bridge</t>
         </is>
       </c>
-      <c r="B47" s="77" t="inlineStr">
+      <c r="B48" s="78" t="inlineStr">
         <is>
           <t>Normalized EBIT &amp; t_operating</t>
         </is>
       </c>
-      <c r="D47" s="26" t="inlineStr">
-        <is>
-          <t>NOPAT = EBIT x (1 - t); transition t toward marginal rate.</t>
-        </is>
-      </c>
-      <c r="F47" s="78" t="inlineStr">
+      <c r="C48" s="78" t="inlineStr">
+        <is>
+          <t>NOPAT = EBIT × (1 − 30%) flat sc_tax. Same EBIT as Scenarios.</t>
+        </is>
+      </c>
+      <c r="D48" s="78" t="inlineStr">
+        <is>
+          <t>NOPAT = EBIT × (1 − t_operating). Same EBIT; ~29.6% FY26 tax → slightly higher NOPAT.</t>
+        </is>
+      </c>
+      <c r="F48" s="79" t="inlineStr">
         <is>
           <t>Normalized NOPAT</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="26" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="60" t="inlineStr">
+        <is>
+          <t>6. Tariff refund (Scenarios)</t>
+        </is>
+      </c>
+      <c r="B49" s="78" t="inlineStr">
+        <is>
+          <t>Q2 FY2026 earnings release</t>
+        </is>
+      </c>
+      <c r="C49" s="78" t="inlineStr">
+        <is>
+          <t>EBIT = Rev × 13.2% only — run-rate margin, no IEEPA refund.</t>
+        </is>
+      </c>
+      <c r="D49" s="78" t="inlineStr">
+        <is>
+          <t>+ $134,500k in FY26 only — DCF uses this; EBIT and NOPAT both higher vs without.</t>
+        </is>
+      </c>
+      <c r="F49" s="79" t="inlineStr">
+        <is>
+          <t>Scenarios EBIT (FY26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="26" t="inlineStr">
+        <is>
+          <t>FY26 DCF EBIT is built on Scenarios (13.2% + tariff). Phases 1–4 are FY25 documentation or illustrative channel math — only Phase 5 tax and the tariff row change NOPAT vs a flat 30%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="26" t="inlineStr">
         <is>
           <t>Scenarios base-case NOPAT (col G) links to NORMALIZED NOPAT above. Bear/bull apply the same t_operating to their EBIT paths.</t>
         </is>
@@ -8650,17 +8737,17 @@
       <c r="J1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="B2" s="79" t="inlineStr">
+      <c r="B2" s="77" t="inlineStr">
         <is>
           <t>Justification (~20 words)  [cols B–D: click + to expand]</t>
         </is>
       </c>
-      <c r="C2" s="79" t="inlineStr">
+      <c r="C2" s="77" t="inlineStr">
         <is>
           <t>Source (click)</t>
         </is>
       </c>
-      <c r="D2" s="79" t="inlineStr">
+      <c r="D2" s="77" t="inlineStr">
         <is>
           <t>Ctrl+F (prove number)</t>
         </is>
@@ -8700,12 +8787,12 @@
           <t>Δ vs Scenarios</t>
         </is>
       </c>
-      <c r="L2" s="79" t="inlineStr">
+      <c r="L2" s="77" t="inlineStr">
         <is>
           <t>Alt. source  [cols L–M: click + to expand]</t>
         </is>
       </c>
-      <c r="M2" s="79" t="inlineStr">
+      <c r="M2" s="77" t="inlineStr">
         <is>
           <t>Alt. Ctrl+F</t>
         </is>

</xml_diff>

<commit_message>
Simplify NOPAT Bridge Phase 5: DCF unchanged for steps 1–4
Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -8493,12 +8493,12 @@
       </c>
       <c r="C44" s="78" t="inlineStr">
         <is>
-          <t>FY26 EBIT = Rev × 13.2% + tariff. No impairment/SBC/restructuring add-backs in forecast.</t>
+          <t>EBIT = 13.2% × rev + tariff; no add-backs.</t>
         </is>
       </c>
       <c r="D44" s="78" t="inlineStr">
         <is>
-          <t>Would lift EBIT by adding back one-offs + SBC — runs on FY25 history only; FY26 DCF unchanged.</t>
+          <t>DCF unchanged.</t>
         </is>
       </c>
       <c r="F44" s="79" t="inlineStr">
@@ -8520,12 +8520,12 @@
       </c>
       <c r="C45" s="78" t="inlineStr">
         <is>
-          <t>R&amp;D/software expensed in full each year. LULU = $0 cap; no FY26 EBIT change.</t>
+          <t>R&amp;D/software expensed in full each year ($0 for LULU).</t>
         </is>
       </c>
       <c r="D45" s="78" t="inlineStr">
         <is>
-          <t>Would spread expense over 4 yrs (cap + amort) — higher near-term EBIT; not wired to FY26 DCF.</t>
+          <t>DCF unchanged.</t>
         </is>
       </c>
       <c r="F45" s="79" t="inlineStr">
@@ -8547,12 +8547,12 @@
       </c>
       <c r="C46" s="78" t="inlineStr">
         <is>
-          <t>Rent stays in operating costs; no lease-interest add-back. FY26 DCF EBIT unchanged.</t>
+          <t>Rent in opex; no implied lease-interest add-back.</t>
         </is>
       </c>
       <c r="D46" s="78" t="inlineStr">
         <is>
-          <t>Would add implied lease interest to EBIT (unlevered) — FY25 bridge only; FY26 DCF same.</t>
+          <t>DCF unchanged.</t>
         </is>
       </c>
       <c r="F46" s="79" t="inlineStr">
@@ -8574,12 +8574,12 @@
       </c>
       <c r="C47" s="78" t="inlineStr">
         <is>
-          <t>DCF uses consolidated 13.2% on total revenue (+ tariff). Channel EBIT not used.</t>
+          <t>DCF uses consolidated 13.2% on total revenue (+ tariff).</t>
         </is>
       </c>
       <c r="D47" s="78" t="inlineStr">
         <is>
-          <t>Channel EBIT = Σ(Rev_i × margin_i) — higher illustrative EBIT; check row shows gap vs Scenarios.</t>
+          <t>DCF unchanged.</t>
         </is>
       </c>
       <c r="F47" s="79" t="inlineStr">
@@ -8601,12 +8601,12 @@
       </c>
       <c r="C48" s="78" t="inlineStr">
         <is>
-          <t>NOPAT = EBIT × (1 − 30%) flat sc_tax. Same EBIT as Scenarios.</t>
+          <t>NOPAT = EBIT × (1 − 30%) flat sc_tax.</t>
         </is>
       </c>
       <c r="D48" s="78" t="inlineStr">
         <is>
-          <t>NOPAT = EBIT × (1 − t_operating). Same EBIT; ~29.6% FY26 tax → slightly higher NOPAT.</t>
+          <t>NOPAT = EBIT × (1 − t_operating) — same EBIT, slightly higher NOPAT.</t>
         </is>
       </c>
       <c r="F48" s="79" t="inlineStr">
@@ -8628,12 +8628,12 @@
       </c>
       <c r="C49" s="78" t="inlineStr">
         <is>
-          <t>EBIT = Rev × 13.2% only — run-rate margin, no IEEPA refund.</t>
+          <t>EBIT = Rev × 13.2% only (no refund).</t>
         </is>
       </c>
       <c r="D49" s="78" t="inlineStr">
         <is>
-          <t>+ $134,500k in FY26 only — DCF uses this; EBIT and NOPAT both higher vs without.</t>
+          <t>+ $134,500k in FY26 — DCF uses this.</t>
         </is>
       </c>
       <c r="F49" s="79" t="inlineStr">
@@ -8645,7 +8645,7 @@
     <row r="50">
       <c r="A50" s="26" t="inlineStr">
         <is>
-          <t>FY26 DCF EBIT is built on Scenarios (13.2% + tariff). Phases 1–4 are FY25 documentation or illustrative channel math — only Phase 5 tax and the tariff row change NOPAT vs a flat 30%.</t>
+          <t>Steps 1–4: DCF unchanged on FY26. Step 5 changes NOPAT only (tax). Step 6 changes FY26 EBIT (+ tariff).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Share Repurchase & EPS Accretion schedule below DCF valuation
Pulls UFCF years 1-5, allocates 75% to buybacks, grows share price at
10.5% CoE, rolls forward shares retired, and computes accretive EPS.
Guardrail: implied value per share still uses Day-1 diluted shares (111.4M).

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -405,7 +405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -666,6 +666,15 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="34" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -8702,7 +8711,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M85"/>
+  <dimension ref="A1:M103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -10510,473 +10519,788 @@
         <v/>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="92" t="inlineStr">
-        <is>
-          <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
-        </is>
-      </c>
-      <c r="B61" s="13" t="n"/>
-      <c r="C61" s="13" t="n"/>
-    </row>
     <row r="62">
-      <c r="A62" s="15" t="inlineStr">
-        <is>
-          <t>Exit multiple is the Gordon identity — not a peer pick or an average</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="28" customHeight="1">
-      <c r="A63" s="16" t="inlineStr">
-        <is>
-          <t>Selected exit EV/EBITDA (Gordon implied)</t>
-        </is>
-      </c>
-      <c r="B63" s="17" t="inlineStr">
-        <is>
-          <t>Selected exit is Gordon TV / FY30 EBITDA. Identity: (UFCF/EBITDA)×(1+g)/(WACC−g). Not Deckers and not a peer average.</t>
-        </is>
-      </c>
-      <c r="C63" s="18" t="inlineStr">
-        <is>
-          <t>DCF: Gordon implied exit (TV / FY30 EBITDA)</t>
-        </is>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
-        </is>
-      </c>
-      <c r="E63" s="93">
-        <f>E46</f>
-        <v/>
-      </c>
-      <c r="M63" s="94" t="inlineStr">
-        <is>
-          <t>Comps: Exit Multiple Build</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="16" t="inlineStr">
-        <is>
-          <t>Terminal value = Terminal EBITDA × exit multiple</t>
-        </is>
-      </c>
-      <c r="E64" s="74">
-        <f>E44*E63</f>
-        <v/>
+      <c r="A62" s="92" t="inlineStr">
+        <is>
+          <t>SHARE REPURCHASE &amp; EPS ACCRETION SCHEDULE</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="n"/>
+      <c r="C62" s="13" t="n"/>
+      <c r="D62" s="13" t="n"/>
+      <c r="E62" s="13" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="26" t="inlineStr">
+        <is>
+          <t>Guardrail: implied value per share above still divides equity value by Day-1 shares (E55 = 111,380k). This schedule does not change intrinsic DCF per share.</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
-          <t>PV of terminal value</t>
-        </is>
-      </c>
-      <c r="E65" s="74">
-        <f>E64/(1+Scenarios!$G$9)^J36</f>
+          <t>FCF allocated to buybacks</t>
+        </is>
+      </c>
+      <c r="E65" s="20" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F65" s="20">
+        <f>$E$65</f>
+        <v/>
+      </c>
+      <c r="G65" s="20">
+        <f>$E$65</f>
+        <v/>
+      </c>
+      <c r="H65" s="20">
+        <f>$E$65</f>
+        <v/>
+      </c>
+      <c r="I65" s="20">
+        <f>$E$65</f>
+        <v/>
+      </c>
+      <c r="J65" s="20">
+        <f>$E$65</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="23" t="inlineStr">
-        <is>
-          <t>Enterprise value (exit method)</t>
-        </is>
-      </c>
-      <c r="E66" s="25">
-        <f>E42+E65</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="23" t="inlineStr">
-        <is>
-          <t>Implied value per share (exit method)</t>
-        </is>
-      </c>
-      <c r="E67" s="98">
-        <f>(E66+E50+E51)/E55</f>
+      <c r="A66" s="16" t="inlineStr">
+        <is>
+          <t>Cost of equity — share-price growth rate</t>
+        </is>
+      </c>
+      <c r="E66" s="20" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="F66" s="20">
+        <f>$E$66</f>
+        <v/>
+      </c>
+      <c r="G66" s="20">
+        <f>$E$66</f>
+        <v/>
+      </c>
+      <c r="H66" s="20">
+        <f>$E$66</f>
+        <v/>
+      </c>
+      <c r="I66" s="20">
+        <f>$E$66</f>
+        <v/>
+      </c>
+      <c r="J66" s="20">
+        <f>$E$66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="16" t="inlineStr">
+        <is>
+          <t>Unlevered free cash flow (from DCF above)</t>
+        </is>
+      </c>
+      <c r="F68" s="74">
+        <f>F35</f>
+        <v/>
+      </c>
+      <c r="G68" s="74">
+        <f>G35</f>
+        <v/>
+      </c>
+      <c r="H68" s="74">
+        <f>H35</f>
+        <v/>
+      </c>
+      <c r="I68" s="74">
+        <f>I35</f>
+        <v/>
+      </c>
+      <c r="J68" s="74">
+        <f>J35</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="92" t="inlineStr">
-        <is>
-          <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
-        </is>
-      </c>
-      <c r="B69" s="13" t="n"/>
-      <c r="C69" s="13" t="n"/>
-      <c r="D69" s="13" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="99" t="inlineStr"/>
-      <c r="B70" s="53" t="inlineStr">
-        <is>
-          <t>Gordon Growth</t>
-        </is>
-      </c>
-      <c r="C70" s="53" t="inlineStr">
-        <is>
-          <t>Exit Multiple</t>
-        </is>
-      </c>
-      <c r="D70" s="53" t="inlineStr">
-        <is>
-          <t>Variance</t>
-        </is>
+      <c r="A69" s="16" t="inlineStr">
+        <is>
+          <t>Available repurchase cash (= UFCF × allocation)</t>
+        </is>
+      </c>
+      <c r="E69" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="74">
+        <f>F68*F65</f>
+        <v/>
+      </c>
+      <c r="G69" s="74">
+        <f>G68*G65</f>
+        <v/>
+      </c>
+      <c r="H69" s="74">
+        <f>H68*H65</f>
+        <v/>
+      </c>
+      <c r="I69" s="74">
+        <f>I68*I65</f>
+        <v/>
+      </c>
+      <c r="J69" s="74">
+        <f>J68*J65</f>
+        <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="23" t="inlineStr">
-        <is>
-          <t>Terminal value ($)</t>
-        </is>
-      </c>
-      <c r="B71" s="69">
-        <f>E45</f>
-        <v/>
-      </c>
-      <c r="C71" s="69">
-        <f>E64</f>
-        <v/>
-      </c>
-      <c r="D71" s="69">
-        <f>B71-C71</f>
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t>Projected share price ($)</t>
+        </is>
+      </c>
+      <c r="E71" s="98" t="n">
+        <v>100</v>
+      </c>
+      <c r="F71" s="98">
+        <f>E71*(1+$E$66)</f>
+        <v/>
+      </c>
+      <c r="G71" s="98">
+        <f>F71*(1+$E$66)</f>
+        <v/>
+      </c>
+      <c r="H71" s="98">
+        <f>G71*(1+$E$66)</f>
+        <v/>
+      </c>
+      <c r="I71" s="98">
+        <f>H71*(1+$E$66)</f>
+        <v/>
+      </c>
+      <c r="J71" s="98">
+        <f>I71*(1+$E$66)</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="23" t="inlineStr">
-        <is>
-          <t>Exit EV/EBITDA (implied vs selected)</t>
-        </is>
-      </c>
-      <c r="B72" s="100">
-        <f>E46</f>
-        <v/>
-      </c>
-      <c r="C72" s="100">
-        <f>E63</f>
-        <v/>
-      </c>
-      <c r="D72" s="100">
-        <f>B72-C72</f>
+      <c r="A72" s="16" t="inlineStr">
+        <is>
+          <t>Shares retired (000)</t>
+        </is>
+      </c>
+      <c r="E72" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="74">
+        <f>F69/F71</f>
+        <v/>
+      </c>
+      <c r="G72" s="74">
+        <f>G69/G71</f>
+        <v/>
+      </c>
+      <c r="H72" s="74">
+        <f>H69/H71</f>
+        <v/>
+      </c>
+      <c r="I72" s="74">
+        <f>I69/I71</f>
+        <v/>
+      </c>
+      <c r="J72" s="74">
+        <f>J69/J71</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="16" t="inlineStr">
         <is>
-          <t>Terminal value variance (%)</t>
-        </is>
-      </c>
-      <c r="B73" s="32" t="inlineStr"/>
-      <c r="C73" s="32" t="inlineStr"/>
-      <c r="D73" s="32">
-        <f>(B71-C71)/B71</f>
+          <t>Beginning shares (000)</t>
+        </is>
+      </c>
+      <c r="E73" s="22" t="n">
+        <v>111380</v>
+      </c>
+      <c r="F73" s="74">
+        <f>$E$73</f>
+        <v/>
+      </c>
+      <c r="G73" s="74">
+        <f>F74</f>
+        <v/>
+      </c>
+      <c r="H73" s="74">
+        <f>G74</f>
+        <v/>
+      </c>
+      <c r="I73" s="74">
+        <f>H74</f>
+        <v/>
+      </c>
+      <c r="J73" s="74">
+        <f>I74</f>
         <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="23" t="inlineStr">
         <is>
+          <t>Ending shares (000)</t>
+        </is>
+      </c>
+      <c r="E74" s="99" t="n">
+        <v>111380</v>
+      </c>
+      <c r="F74" s="25">
+        <f>F73-F72</f>
+        <v/>
+      </c>
+      <c r="G74" s="25">
+        <f>G73-G72</f>
+        <v/>
+      </c>
+      <c r="H74" s="25">
+        <f>H73-H72</f>
+        <v/>
+      </c>
+      <c r="I74" s="25">
+        <f>I73-I72</f>
+        <v/>
+      </c>
+      <c r="J74" s="25">
+        <f>J73-J72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="16" t="inlineStr">
+        <is>
+          <t>Projected net income ($000)</t>
+        </is>
+      </c>
+      <c r="E76" s="22" t="n">
+        <v>1579183</v>
+      </c>
+      <c r="F76" s="74">
+        <f>('NOPAT Bridge'!F35-'NOPAT Bridge'!F22)*(1-'NOPAT Bridge'!F$38)</f>
+        <v/>
+      </c>
+      <c r="G76" s="74">
+        <f>('NOPAT Bridge'!G35-'NOPAT Bridge'!G22)*(1-'NOPAT Bridge'!G$38)</f>
+        <v/>
+      </c>
+      <c r="H76" s="74">
+        <f>('NOPAT Bridge'!H35-'NOPAT Bridge'!H22)*(1-'NOPAT Bridge'!H$38)</f>
+        <v/>
+      </c>
+      <c r="I76" s="74">
+        <f>('NOPAT Bridge'!I35-'NOPAT Bridge'!I22)*(1-'NOPAT Bridge'!I$38)</f>
+        <v/>
+      </c>
+      <c r="J76" s="74">
+        <f>('NOPAT Bridge'!J35-'NOPAT Bridge'!J22)*(1-'NOPAT Bridge'!J$38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="23" t="inlineStr">
+        <is>
+          <t>Accretive EPS ($/share) = Net income ÷ ending shares</t>
+        </is>
+      </c>
+      <c r="E77" s="100" t="n">
+        <v>14.1783354282636</v>
+      </c>
+      <c r="F77" s="100">
+        <f>F76/F74</f>
+        <v/>
+      </c>
+      <c r="G77" s="100">
+        <f>G76/G74</f>
+        <v/>
+      </c>
+      <c r="H77" s="100">
+        <f>H76/H74</f>
+        <v/>
+      </c>
+      <c r="I77" s="100">
+        <f>I76/I74</f>
+        <v/>
+      </c>
+      <c r="J77" s="100">
+        <f>J76/J74</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="92" t="inlineStr">
+        <is>
+          <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
+        </is>
+      </c>
+      <c r="B79" s="13" t="n"/>
+      <c r="C79" s="13" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="15" t="inlineStr">
+        <is>
+          <t>Exit multiple is the Gordon identity — not a peer pick or an average</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="28" customHeight="1">
+      <c r="A81" s="16" t="inlineStr">
+        <is>
+          <t>Selected exit EV/EBITDA (Gordon implied)</t>
+        </is>
+      </c>
+      <c r="B81" s="17" t="inlineStr">
+        <is>
+          <t>Selected exit is Gordon TV / FY30 EBITDA. Identity: (UFCF/EBITDA)×(1+g)/(WACC−g). Not Deckers and not a peer average.</t>
+        </is>
+      </c>
+      <c r="C81" s="18" t="inlineStr">
+        <is>
+          <t>DCF: Gordon implied exit (TV / FY30 EBITDA)</t>
+        </is>
+      </c>
+      <c r="D81" s="19" t="inlineStr">
+        <is>
+          <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
+        </is>
+      </c>
+      <c r="E81" s="93">
+        <f>E46</f>
+        <v/>
+      </c>
+      <c r="M81" s="94" t="inlineStr">
+        <is>
+          <t>Comps: Exit Multiple Build</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="16" t="inlineStr">
+        <is>
+          <t>Terminal value = Terminal EBITDA × exit multiple</t>
+        </is>
+      </c>
+      <c r="E82" s="74">
+        <f>E44*E81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="16" t="inlineStr">
+        <is>
+          <t>PV of terminal value</t>
+        </is>
+      </c>
+      <c r="E83" s="74">
+        <f>E82/(1+Scenarios!$G$9)^J36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="23" t="inlineStr">
+        <is>
+          <t>Enterprise value (exit method)</t>
+        </is>
+      </c>
+      <c r="E84" s="25">
+        <f>E42+E83</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="23" t="inlineStr">
+        <is>
+          <t>Implied value per share (exit method)</t>
+        </is>
+      </c>
+      <c r="E85" s="101">
+        <f>(E84+E50+E51)/E55</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="92" t="inlineStr">
+        <is>
+          <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
+        </is>
+      </c>
+      <c r="B87" s="13" t="n"/>
+      <c r="C87" s="13" t="n"/>
+      <c r="D87" s="13" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="102" t="inlineStr"/>
+      <c r="B88" s="53" t="inlineStr">
+        <is>
+          <t>Gordon Growth</t>
+        </is>
+      </c>
+      <c r="C88" s="53" t="inlineStr">
+        <is>
+          <t>Exit Multiple</t>
+        </is>
+      </c>
+      <c r="D88" s="53" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="23" t="inlineStr">
+        <is>
+          <t>Terminal value ($)</t>
+        </is>
+      </c>
+      <c r="B89" s="69">
+        <f>E45</f>
+        <v/>
+      </c>
+      <c r="C89" s="69">
+        <f>E82</f>
+        <v/>
+      </c>
+      <c r="D89" s="69">
+        <f>B89-C89</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="23" t="inlineStr">
+        <is>
+          <t>Exit EV/EBITDA (implied vs selected)</t>
+        </is>
+      </c>
+      <c r="B90" s="103">
+        <f>E46</f>
+        <v/>
+      </c>
+      <c r="C90" s="103">
+        <f>E81</f>
+        <v/>
+      </c>
+      <c r="D90" s="103">
+        <f>B90-C90</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="16" t="inlineStr">
+        <is>
+          <t>Terminal value variance (%)</t>
+        </is>
+      </c>
+      <c r="B91" s="32" t="inlineStr"/>
+      <c r="C91" s="32" t="inlineStr"/>
+      <c r="D91" s="32">
+        <f>(B89-C89)/B89</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="23" t="inlineStr">
+        <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="B74" s="101">
+      <c r="B92" s="104">
         <f>E56</f>
         <v/>
       </c>
-      <c r="C74" s="101">
-        <f>E67</f>
-        <v/>
-      </c>
-      <c r="D74" s="101">
-        <f>B74-C74</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="67" t="inlineStr">
+      <c r="C92" s="104">
+        <f>E85</f>
+        <v/>
+      </c>
+      <c r="D92" s="104">
+        <f>B92-C92</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="67" t="inlineStr">
         <is>
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B75" s="102">
-        <f>IF(ABS(D72)&lt;=1.5,"PASS","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="C75" s="103">
-        <f>TEXT(D72,"0.0")&amp;"x spread vs Gordon-implied exit"</f>
-        <v/>
-      </c>
-      <c r="D75" s="26" t="inlineStr">
+      <c r="B93" s="105">
+        <f>IF(ABS(D90)&lt;=1.5,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="C93" s="106">
+        <f>TEXT(D90,"0.0")&amp;"x spread vs Gordon-implied exit"</f>
+        <v/>
+      </c>
+      <c r="D93" s="26" t="inlineStr">
         <is>
           <t>Selected exit is the Gordon identity, so spread should be 0</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="92" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="92" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
       </c>
-      <c r="B78" s="13" t="n"/>
-      <c r="C78" s="13" t="n"/>
-      <c r="D78" s="13" t="n"/>
-      <c r="E78" s="13" t="n"/>
-      <c r="F78" s="13" t="n"/>
-      <c r="G78" s="13" t="n"/>
-      <c r="H78" s="13" t="n"/>
-    </row>
-    <row r="79" ht="28" customHeight="1">
-      <c r="A79" s="104" t="inlineStr">
+      <c r="B96" s="13" t="n"/>
+      <c r="C96" s="13" t="n"/>
+      <c r="D96" s="13" t="n"/>
+      <c r="E96" s="13" t="n"/>
+      <c r="F96" s="13" t="n"/>
+      <c r="G96" s="13" t="n"/>
+      <c r="H96" s="13" t="n"/>
+    </row>
+    <row r="97" ht="28" customHeight="1">
+      <c r="A97" s="107" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
       </c>
-      <c r="B79" s="17" t="inlineStr">
+      <c r="B97" s="17" t="inlineStr">
         <is>
           <t>Terminal-g axis 1.5–3.0% brackets 2.25% base; bounded by long-run real GDP and inflation benchmarks.</t>
         </is>
       </c>
-      <c r="C79" s="18" t="inlineStr">
+      <c r="C97" s="18" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="D79" s="19" t="inlineStr">
+      <c r="D97" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
       </c>
-      <c r="F79" s="105" t="n">
+      <c r="F97" s="108" t="n">
         <v>0.015</v>
       </c>
-      <c r="G79" s="105" t="n">
+      <c r="G97" s="108" t="n">
         <v>0.02</v>
       </c>
-      <c r="H79" s="105" t="n">
+      <c r="H97" s="108" t="n">
         <v>0.0225</v>
       </c>
-      <c r="I79" s="105" t="n">
+      <c r="I97" s="108" t="n">
         <v>0.025</v>
       </c>
-      <c r="J79" s="105" t="n">
+      <c r="J97" s="108" t="n">
         <v>0.03</v>
       </c>
-      <c r="L79" s="94" t="inlineStr">
+      <c r="L97" s="94" t="inlineStr">
         <is>
           <t>Scenarios: terminal g</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="28" customHeight="1">
-      <c r="A80" s="105" t="n">
+    <row r="98" ht="28" customHeight="1">
+      <c r="A98" s="108" t="n">
         <v>0.095</v>
       </c>
-      <c r="C80" s="94" t="inlineStr">
+      <c r="C98" s="94" t="inlineStr">
         <is>
           <t>Damodaran: Historical Implied ERP</t>
         </is>
       </c>
-      <c r="D80" s="19" t="inlineStr">
+      <c r="D98" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F80" s="106">
+      <c r="F98" s="109">
         <f>(NPV(0.095,F35:J35)+(J35*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="G80" s="106">
+      <c r="G98" s="109">
         <f>(NPV(0.095,F35:J35)+(J35*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="H80" s="106">
+      <c r="H98" s="109">
         <f>(NPV(0.095,F35:J35)+(J35*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="I80" s="106">
+      <c r="I98" s="109">
         <f>(NPV(0.095,F35:J35)+(J35*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="J80" s="106">
+      <c r="J98" s="109">
         <f>(NPV(0.095,F35:J35)+(J35*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="L80" s="94" t="inlineStr">
+      <c r="L98" s="94" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="28" customHeight="1">
-      <c r="A81" s="105" t="n">
+    <row r="99" ht="28" customHeight="1">
+      <c r="A99" s="108" t="n">
         <v>0.1</v>
       </c>
-      <c r="D81" s="19" t="inlineStr">
+      <c r="D99" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F81" s="106">
+      <c r="F99" s="109">
         <f>(NPV(0.1,F35:J35)+(J35*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="G81" s="106">
+      <c r="G99" s="109">
         <f>(NPV(0.1,F35:J35)+(J35*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="H81" s="106">
+      <c r="H99" s="109">
         <f>(NPV(0.1,F35:J35)+(J35*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="I81" s="106">
+      <c r="I99" s="109">
         <f>(NPV(0.1,F35:J35)+(J35*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="J81" s="106">
+      <c r="J99" s="109">
         <f>(NPV(0.1,F35:J35)+(J35*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="L81" s="94" t="inlineStr">
+      <c r="L99" s="94" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="28" customHeight="1">
-      <c r="A82" s="105" t="n">
+    <row r="100" ht="28" customHeight="1">
+      <c r="A100" s="108" t="n">
         <v>0.105</v>
       </c>
-      <c r="D82" s="19" t="inlineStr">
+      <c r="D100" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F82" s="106">
+      <c r="F100" s="109">
         <f>(NPV(0.105,F35:J35)+(J35*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="G82" s="106">
+      <c r="G100" s="109">
         <f>(NPV(0.105,F35:J35)+(J35*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="H82" s="107">
+      <c r="H100" s="110">
         <f>(NPV(0.105,F35:J35)+(J35*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="I82" s="106">
+      <c r="I100" s="109">
         <f>(NPV(0.105,F35:J35)+(J35*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="J82" s="106">
+      <c r="J100" s="109">
         <f>(NPV(0.105,F35:J35)+(J35*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="L82" s="94" t="inlineStr">
+      <c r="L100" s="94" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="28" customHeight="1">
-      <c r="A83" s="105" t="n">
+    <row r="101" ht="28" customHeight="1">
+      <c r="A101" s="108" t="n">
         <v>0.11</v>
       </c>
-      <c r="D83" s="19" t="inlineStr">
+      <c r="D101" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F83" s="106">
+      <c r="F101" s="109">
         <f>(NPV(0.11,F35:J35)+(J35*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="G83" s="106">
+      <c r="G101" s="109">
         <f>(NPV(0.11,F35:J35)+(J35*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="H83" s="106">
+      <c r="H101" s="109">
         <f>(NPV(0.11,F35:J35)+(J35*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="I83" s="106">
+      <c r="I101" s="109">
         <f>(NPV(0.11,F35:J35)+(J35*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="J83" s="106">
+      <c r="J101" s="109">
         <f>(NPV(0.11,F35:J35)+(J35*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="L83" s="94" t="inlineStr">
+      <c r="L101" s="94" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="28" customHeight="1">
-      <c r="A84" s="105" t="n">
+    <row r="102" ht="28" customHeight="1">
+      <c r="A102" s="108" t="n">
         <v>0.115</v>
       </c>
-      <c r="D84" s="19" t="inlineStr">
+      <c r="D102" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
         </is>
       </c>
-      <c r="F84" s="106">
+      <c r="F102" s="109">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="G84" s="106">
+      <c r="G102" s="109">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="H84" s="106">
+      <c r="H102" s="109">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="I84" s="106">
+      <c r="I102" s="109">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="J84" s="106">
+      <c r="J102" s="109">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="L84" s="94" t="inlineStr">
+      <c r="L102" s="94" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="28" customHeight="1">
-      <c r="B85" s="17" t="inlineStr">
+    <row r="103" ht="28" customHeight="1">
+      <c r="B103" s="17" t="inlineStr">
         <is>
           <t>Red WACC and g grid values bracket base case ±100bps discount rate and ±75bps terminal growth for sensitivity.</t>
         </is>
       </c>
-      <c r="C85" s="18" t="inlineStr">
+      <c r="C103" s="18" t="inlineStr">
         <is>
           <t>Scenarios: WACC &amp; terminal g</t>
         </is>
       </c>
-      <c r="D85" s="19" t="inlineStr">
+      <c r="D103" s="19" t="inlineStr">
         <is>
           <t>Scenarios tab → Ctrl+F "WACC" and "Terminal growth" rows (base-case inputs)</t>
         </is>
       </c>
-      <c r="L85" s="94" t="inlineStr">
+      <c r="L103" s="94" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="M85" s="19" t="inlineStr">
+      <c r="M103" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
@@ -11034,18 +11358,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId45"/>
-    <hyperlink ref="C63" location="'DCF'!E46"/>
-    <hyperlink ref="M63" location="'Comps'!A45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId46"/>
-    <hyperlink ref="L79" location="'Scenarios'!G10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId47"/>
-    <hyperlink ref="L80" location="'WACC'!E41"/>
-    <hyperlink ref="L81" location="'WACC'!E41"/>
-    <hyperlink ref="L82" location="'WACC'!E41"/>
-    <hyperlink ref="L83" location="'WACC'!E41"/>
-    <hyperlink ref="L84" location="'WACC'!E41"/>
-    <hyperlink ref="C85" location="'Scenarios'!G9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L85" r:id="rId48"/>
+    <hyperlink ref="C81" location="'DCF'!E46"/>
+    <hyperlink ref="M81" location="'Comps'!A45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId46"/>
+    <hyperlink ref="L97" location="'Scenarios'!G10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId47"/>
+    <hyperlink ref="L98" location="'WACC'!E41"/>
+    <hyperlink ref="L99" location="'WACC'!E41"/>
+    <hyperlink ref="L100" location="'WACC'!E41"/>
+    <hyperlink ref="L101" location="'WACC'!E41"/>
+    <hyperlink ref="L102" location="'WACC'!E41"/>
+    <hyperlink ref="C103" location="'Scenarios'!G9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L103" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11238,23 +11562,23 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="103" t="inlineStr">
+      <c r="A11" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current EV / EBITDA</t>
         </is>
       </c>
-      <c r="E11" s="108">
+      <c r="E11" s="111">
         <f>(E10*E9-E8)/E5</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="103" t="inlineStr">
+      <c r="A12" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: current P / E (FY2026E)</t>
         </is>
       </c>
-      <c r="E12" s="108">
+      <c r="E12" s="111">
         <f>E10/E7</f>
         <v/>
       </c>
@@ -11267,7 +11591,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="103" t="inlineStr">
+      <c r="A15" s="106" t="inlineStr">
         <is>
           <t>Peer / reference EV/EBITDA (forward / illustrative)</t>
         </is>
@@ -11288,37 +11612,37 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="109" t="inlineStr">
+      <c r="A18" s="112" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B18" s="109" t="inlineStr">
+      <c r="B18" s="112" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C18" s="109" t="inlineStr">
+      <c r="C18" s="112" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D18" s="109" t="inlineStr">
+      <c r="D18" s="112" t="inlineStr">
         <is>
           <t>Ctrl+F / proof</t>
         </is>
       </c>
-      <c r="E18" s="110" t="inlineStr">
+      <c r="E18" s="113" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="I18" s="110" t="inlineStr">
+      <c r="I18" s="113" t="inlineStr">
         <is>
           <t>EV ($000)</t>
         </is>
       </c>
-      <c r="J18" s="110" t="inlineStr">
+      <c r="J18" s="113" t="inlineStr">
         <is>
           <t>EBITDA ($000)</t>
         </is>
@@ -11345,14 +11669,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E19" s="111">
+      <c r="E19" s="114">
         <f>IF(J19&lt;=0,"n.m.",I19/J19)</f>
         <v/>
       </c>
-      <c r="I19" s="112" t="n">
+      <c r="I19" s="115" t="n">
         <v>11890440</v>
       </c>
-      <c r="J19" s="112" t="n">
+      <c r="J19" s="115" t="n">
         <v>2548084</v>
       </c>
     </row>
@@ -11377,14 +11701,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E20" s="111">
+      <c r="E20" s="114">
         <f>IF(J20&lt;=0,"n.m.",I20/J20)</f>
         <v/>
       </c>
-      <c r="I20" s="112" t="n">
+      <c r="I20" s="115" t="n">
         <v>3208397</v>
       </c>
-      <c r="J20" s="112" t="n">
+      <c r="J20" s="115" t="n">
         <v>-23230</v>
       </c>
     </row>
@@ -11409,14 +11733,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E21" s="111">
+      <c r="E21" s="114">
         <f>IF(J21&lt;=0,"n.m.",I21/J21)</f>
         <v/>
       </c>
-      <c r="I21" s="112" t="n">
+      <c r="I21" s="115" t="n">
         <v>35661944</v>
       </c>
-      <c r="J21" s="112" t="n">
+      <c r="J21" s="115" t="n">
         <v>3857684</v>
       </c>
     </row>
@@ -11441,14 +11765,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E22" s="111">
+      <c r="E22" s="114">
         <f>IF(J22&lt;=0,"n.m.",I22/J22)</f>
         <v/>
       </c>
-      <c r="I22" s="112" t="n">
+      <c r="I22" s="115" t="n">
         <v>58972350</v>
       </c>
-      <c r="J22" s="112" t="n">
+      <c r="J22" s="115" t="n">
         <v>4647000</v>
       </c>
     </row>
@@ -11473,14 +11797,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E23" s="111">
+      <c r="E23" s="114">
         <f>IF(J23&lt;=0,"n.m.",I23/J23)</f>
         <v/>
       </c>
-      <c r="I23" s="112" t="n">
+      <c r="I23" s="115" t="n">
         <v>10555510</v>
       </c>
-      <c r="J23" s="112" t="n">
+      <c r="J23" s="115" t="n">
         <v>1329439</v>
       </c>
     </row>
@@ -11505,14 +11829,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E24" s="111">
+      <c r="E24" s="114">
         <f>IF(J24&lt;=0,"n.m.",I24/J24)</f>
         <v/>
       </c>
-      <c r="I24" s="112" t="n">
+      <c r="I24" s="115" t="n">
         <v>27284350</v>
       </c>
-      <c r="J24" s="112" t="n">
+      <c r="J24" s="115" t="n">
         <v>1768400</v>
       </c>
     </row>
@@ -11537,14 +11861,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E25" s="111">
+      <c r="E25" s="114">
         <f>IF(J25&lt;=0,"n.m.",I25/J25)</f>
         <v/>
       </c>
-      <c r="I25" s="112" t="n">
+      <c r="I25" s="115" t="n">
         <v>7153911</v>
       </c>
-      <c r="J25" s="112" t="n">
+      <c r="J25" s="115" t="n">
         <v>922278</v>
       </c>
     </row>
@@ -11569,14 +11893,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E26" s="111">
+      <c r="E26" s="114">
         <f>IF(J26&lt;=0,"n.m.",I26/J26)</f>
         <v/>
       </c>
-      <c r="I26" s="112" t="n">
+      <c r="I26" s="115" t="n">
         <v>616045</v>
       </c>
-      <c r="J26" s="112" t="n">
+      <c r="J26" s="115" t="n">
         <v>62010</v>
       </c>
     </row>
@@ -11601,14 +11925,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E27" s="111">
+      <c r="E27" s="114">
         <f>IF(J27&lt;=0,"n.m.",I27/J27)</f>
         <v/>
       </c>
-      <c r="I27" s="112" t="n">
+      <c r="I27" s="115" t="n">
         <v>9422753</v>
       </c>
-      <c r="J27" s="112" t="n">
+      <c r="J27" s="115" t="n">
         <v>976700</v>
       </c>
     </row>
@@ -11633,14 +11957,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E28" s="111">
+      <c r="E28" s="114">
         <f>IF(J28&lt;=0,"n.m.",I28/J28)</f>
         <v/>
       </c>
-      <c r="I28" s="112" t="n">
+      <c r="I28" s="115" t="n">
         <v>1598873</v>
       </c>
-      <c r="J28" s="112" t="n">
+      <c r="J28" s="115" t="n">
         <v>235723</v>
       </c>
     </row>
@@ -11665,14 +11989,14 @@
           <t>No public HTML. PitchBook Comps Set 04-Sep-2026. Prove daily EV and TTM EBITDA on that screen; E = I/J.</t>
         </is>
       </c>
-      <c r="E29" s="111">
+      <c r="E29" s="114">
         <f>IF(J29&lt;=0,"n.m.",I29/J29)</f>
         <v/>
       </c>
-      <c r="I29" s="112" t="n">
+      <c r="I29" s="115" t="n">
         <v>5236269</v>
       </c>
-      <c r="J29" s="112" t="n">
+      <c r="J29" s="115" t="n">
         <v>407521</v>
       </c>
     </row>
@@ -11714,7 +12038,7 @@
 Also: Ctrl+F "roughly $10 billion" and "No deal was announced". Still an ask.</t>
         </is>
       </c>
-      <c r="E33" s="113" t="n">
+      <c r="E33" s="116" t="n">
         <v>10</v>
       </c>
     </row>
@@ -11739,7 +12063,7 @@
           <t>Ctrl+F "nearly $2 billion". Forbes estimate for Color Image parent (Alo + Bella+Canvas), not Alo-only EBITDA.</t>
         </is>
       </c>
-      <c r="E34" s="113" t="n">
+      <c r="E34" s="116" t="n">
         <v>2</v>
       </c>
     </row>
@@ -11764,7 +12088,7 @@
           <t>No Ctrl+F for EV/EBITDA — Firecrawl found none on Reuters or Forbes. This cell is E33 / E34 (ask ÷ parent sales). Not the TV.</t>
         </is>
       </c>
-      <c r="E35" s="114">
+      <c r="E35" s="117">
         <f>E33/E34</f>
         <v/>
       </c>
@@ -11790,7 +12114,7 @@
           <t>No Ctrl+F. Reuters, Forbes, and PitchBook do not print Alo EV/EBITDA.</t>
         </is>
       </c>
-      <c r="E36" s="115" t="inlineStr">
+      <c r="E36" s="118" t="inlineStr">
         <is>
           <t>n.a.</t>
         </is>
@@ -11824,7 +12148,7 @@
           <t>Each E cell is I/J from the PitchBook extract. Do not use as FY30 exit.</t>
         </is>
       </c>
-      <c r="E39" s="111">
+      <c r="E39" s="114">
         <f>AVERAGE(E19,E22,E21,E23,E25,E27,E29)</f>
         <v/>
       </c>
@@ -11850,13 +12174,13 @@
           <t>UAA omitted because TTM EBITDA is negative. Not the selected FY30 exit.</t>
         </is>
       </c>
-      <c r="E40" s="111">
+      <c r="E40" s="114">
         <f>AVERAGE(E19,E21,E22,E23,E24,E25,E26,E27,E28,E29)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="103" t="inlineStr">
+      <c r="A41" s="106" t="inlineStr">
         <is>
           <t>We do not average peers for terminal value, and we do not use Alo 5.0x EV/Sales as EV/EBITDA.</t>
         </is>
@@ -11886,8 +12210,8 @@
           <t>Selected exit multiple (base case)</t>
         </is>
       </c>
-      <c r="E45" s="100">
-        <f>DCF!E63</f>
+      <c r="E45" s="103">
+        <f>DCF!E81</f>
         <v/>
       </c>
     </row>
@@ -11959,42 +12283,42 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="109" t="inlineStr">
+      <c r="A56" s="112" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B56" s="109" t="inlineStr">
+      <c r="B56" s="112" t="inlineStr">
         <is>
           <t>Justification</t>
         </is>
       </c>
-      <c r="C56" s="109" t="inlineStr">
+      <c r="C56" s="112" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D56" s="109" t="inlineStr">
+      <c r="D56" s="112" t="inlineStr">
         <is>
           <t>Ctrl+F</t>
         </is>
       </c>
-      <c r="E56" s="110" t="inlineStr">
+      <c r="E56" s="113" t="inlineStr">
         <is>
           <t>Low mult.</t>
         </is>
       </c>
-      <c r="F56" s="110" t="inlineStr">
+      <c r="F56" s="113" t="inlineStr">
         <is>
           <t>High mult.</t>
         </is>
       </c>
-      <c r="G56" s="110" t="inlineStr">
+      <c r="G56" s="113" t="inlineStr">
         <is>
           <t>Implied px (low)</t>
         </is>
       </c>
-      <c r="H56" s="110" t="inlineStr">
+      <c r="H56" s="113" t="inlineStr">
         <is>
           <t>Implied px (high)</t>
         </is>
@@ -12024,17 +12348,17 @@
 Hi: Ctrl+F "EV / EBITDA" → 7.95. Football-field cap 8.0x (Deckers). Not the selected exit.</t>
         </is>
       </c>
-      <c r="E57" s="116" t="n">
+      <c r="E57" s="119" t="n">
         <v>5</v>
       </c>
-      <c r="F57" s="116" t="n">
+      <c r="F57" s="119" t="n">
         <v>8</v>
       </c>
-      <c r="G57" s="117">
+      <c r="G57" s="120">
         <f>(E6*E57+E8)/E9</f>
         <v/>
       </c>
-      <c r="H57" s="117">
+      <c r="H57" s="120">
         <f>(E6*F57+E8)/E9</f>
         <v/>
       </c>
@@ -12060,11 +12384,11 @@
           <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
         </is>
       </c>
-      <c r="E58" s="114">
-        <f>DCF!E63</f>
-        <v/>
-      </c>
-      <c r="G58" s="118">
+      <c r="E58" s="117">
+        <f>DCF!E81</f>
+        <v/>
+      </c>
+      <c r="G58" s="121">
         <f>(E6*E58+E8)/E9</f>
         <v/>
       </c>
@@ -12093,17 +12417,17 @@
 Hi: Ctrl+F "Forward PE" → NKE peer benchmark; high-case assumption 18.0x</t>
         </is>
       </c>
-      <c r="E59" s="116" t="n">
+      <c r="E59" s="119" t="n">
         <v>10</v>
       </c>
-      <c r="F59" s="116" t="n">
+      <c r="F59" s="119" t="n">
         <v>18</v>
       </c>
-      <c r="G59" s="117">
+      <c r="G59" s="120">
         <f>E7*E59</f>
         <v/>
       </c>
-      <c r="H59" s="117">
+      <c r="H59" s="120">
         <f>E7*F59</f>
         <v/>
       </c>
@@ -12114,27 +12438,27 @@
           <t>DCF (bear – bull)</t>
         </is>
       </c>
-      <c r="E60" s="119" t="inlineStr">
+      <c r="E60" s="122" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F60" s="119" t="inlineStr">
+      <c r="F60" s="122" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G60" s="117">
+      <c r="G60" s="120">
         <f>Scenarios!F130</f>
         <v/>
       </c>
-      <c r="H60" s="117">
+      <c r="H60" s="120">
         <f>Scenarios!H130</f>
         <v/>
       </c>
     </row>
     <row r="62" ht="28" customHeight="1">
-      <c r="A62" s="120" t="inlineStr">
+      <c r="A62" s="123" t="inlineStr">
         <is>
           <t>Current price</t>
         </is>
@@ -12149,7 +12473,7 @@
           <t>Ctrl+F "closed at $100.61" → Last Sale on NASDAQ quote page</t>
         </is>
       </c>
-      <c r="E62" s="121" t="n">
+      <c r="E62" s="124" t="n">
         <v>100</v>
       </c>
     </row>
@@ -12179,7 +12503,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId14"/>
     <hyperlink ref="C35" location="'Comps'!E33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId15"/>
-    <hyperlink ref="C58" location="'DCF'!E63"/>
+    <hyperlink ref="C58" location="'DCF'!E81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId18"/>

</xml_diff>

<commit_message>
Align NOPAT Bridge SBC documentation with Convention A (flag = 0)
SBC stays expensed in Scenarios EBIT/NOPAT; DCF uses basic shares.
Update flag, memo, Phase 1 formula, and assumptions memo text.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -3123,15 +3123,15 @@
         </is>
       </c>
       <c r="F48" s="42">
-        <f>F43*(1-'NOPAT Bridge'!F$38)</f>
+        <f>F43*(1-'NOPAT Bridge'!F$39)</f>
         <v/>
       </c>
       <c r="G48" s="42">
-        <f>'NOPAT Bridge'!F40</f>
+        <f>'NOPAT Bridge'!F41</f>
         <v/>
       </c>
       <c r="H48" s="42">
-        <f>H43*(1-'NOPAT Bridge'!F$38)</f>
+        <f>H43*(1-'NOPAT Bridge'!F$39)</f>
         <v/>
       </c>
     </row>
@@ -3142,15 +3142,15 @@
         </is>
       </c>
       <c r="F49" s="42">
-        <f>F44*(1-'NOPAT Bridge'!G$38)</f>
+        <f>F44*(1-'NOPAT Bridge'!G$39)</f>
         <v/>
       </c>
       <c r="G49" s="42">
-        <f>'NOPAT Bridge'!G40</f>
+        <f>'NOPAT Bridge'!G41</f>
         <v/>
       </c>
       <c r="H49" s="42">
-        <f>H44*(1-'NOPAT Bridge'!G$38)</f>
+        <f>H44*(1-'NOPAT Bridge'!G$39)</f>
         <v/>
       </c>
     </row>
@@ -3161,15 +3161,15 @@
         </is>
       </c>
       <c r="F50" s="42">
-        <f>F45*(1-'NOPAT Bridge'!H$38)</f>
+        <f>F45*(1-'NOPAT Bridge'!H$39)</f>
         <v/>
       </c>
       <c r="G50" s="42">
-        <f>'NOPAT Bridge'!H40</f>
+        <f>'NOPAT Bridge'!H41</f>
         <v/>
       </c>
       <c r="H50" s="42">
-        <f>H45*(1-'NOPAT Bridge'!H$38)</f>
+        <f>H45*(1-'NOPAT Bridge'!H$39)</f>
         <v/>
       </c>
     </row>
@@ -3180,15 +3180,15 @@
         </is>
       </c>
       <c r="F51" s="42">
-        <f>F46*(1-'NOPAT Bridge'!I$38)</f>
+        <f>F46*(1-'NOPAT Bridge'!I$39)</f>
         <v/>
       </c>
       <c r="G51" s="42">
-        <f>'NOPAT Bridge'!I40</f>
+        <f>'NOPAT Bridge'!I41</f>
         <v/>
       </c>
       <c r="H51" s="42">
-        <f>H46*(1-'NOPAT Bridge'!I$38)</f>
+        <f>H46*(1-'NOPAT Bridge'!I$39)</f>
         <v/>
       </c>
     </row>
@@ -3199,15 +3199,15 @@
         </is>
       </c>
       <c r="F52" s="42">
-        <f>F47*(1-'NOPAT Bridge'!J$38)</f>
+        <f>F47*(1-'NOPAT Bridge'!J$39)</f>
         <v/>
       </c>
       <c r="G52" s="42">
-        <f>'NOPAT Bridge'!J40</f>
+        <f>'NOPAT Bridge'!J41</f>
         <v/>
       </c>
       <c r="H52" s="42">
-        <f>H47*(1-'NOPAT Bridge'!J$38)</f>
+        <f>H47*(1-'NOPAT Bridge'!J$39)</f>
         <v/>
       </c>
     </row>
@@ -7075,7 +7075,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -7177,12 +7177,14 @@
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Phase 1: Add back SBC? (1 = yes; diluted-shares / UFCF convention)</t>
+          <t>Phase 1: Add back SBC? (0 = no — Convention A: expense stays in EBIT)</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — SBC add-back flag (1 = yes). UFCF uses diluted shares; add back non-cash SBC to EBIT. FY25 SBC $62,203k scaled with revenue in forecast.</t>
+          <t>Not % of revenue — SBC add-back flag. Set to 0 (Convention A).
+SBC stays inside Scenarios EBIT/NOPAT as a real economic cost; DCF uses basic shares (111.4M).
+FY25 reference: $62,203k (10-K). Flag = 1 would add back (Convention B + diluted shares) — not used.</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
@@ -7193,35 +7195,42 @@
       <c r="D7" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Stock-based compensation expense"
-→ 62,203 ($000). Flag = 1 adds back to EBIT (diluted-shares UFCF convention).</t>
+→ 62,203 ($000) FY25 reference. Flag = 0: SBC stays in EBIT (Convention A); DCF IV uses basic 111,380k shares.</t>
         </is>
       </c>
       <c r="E7" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H7" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" s="40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" s="40" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>Convention A: SBC is a real economic cost (captures shareholder dilution). Forecast NOPAT uses Scenarios EBIT with SBC expensed. DCF implied value uses basic shares (111.4M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Phase 3: Store-channel EBIT margin %</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Not % of consolidated revenue — EBIT as % of store-channel revenue only (not the Scenarios 13.2%–15.5% consolidated margin).
 18.6% margin assumption.
@@ -7230,12 +7239,12 @@
 Calibrated so Σ channel EBIT ≈ consolidated EBIT 2,210,615 (10-K).</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: company-operated stores net revenue</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>Not consolidated EBIT margin — EBIT ÷ store revenue only (cf. Scenarios 13.2%–15.5%).
 Ctrl+F "Company-operated stores"
@@ -7243,32 +7252,32 @@
 × 18.6% margin assumption → store EBIT ≈ 939,252 ($000)</t>
         </is>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E9" s="20" t="n">
         <v>0.186</v>
       </c>
-      <c r="F8" s="20" t="n">
+      <c r="F9" s="20" t="n">
         <v>0.186</v>
       </c>
-      <c r="G8" s="20" t="n">
+      <c r="G9" s="20" t="n">
         <v>0.186</v>
       </c>
-      <c r="H8" s="20" t="n">
+      <c r="H9" s="20" t="n">
         <v>0.186</v>
       </c>
-      <c r="I8" s="20" t="n">
+      <c r="I9" s="20" t="n">
         <v>0.186</v>
       </c>
-      <c r="J8" s="20" t="n">
+      <c r="J9" s="20" t="n">
         <v>0.186</v>
       </c>
     </row>
-    <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+    <row r="10" ht="70" customHeight="1">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Phase 3: E-commerce EBIT margin %</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Not % of consolidated revenue — EBIT as % of e-commerce revenue only (not the Scenarios 13.2%–15.5% consolidated margin).
 23.6% margin assumption.
@@ -7277,12 +7286,12 @@
 Higher than stores — no occupancy; fulfillment + digital marketing only.</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: e-commerce net revenue</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>Not consolidated EBIT margin — EBIT ÷ e-commerce revenue only (cf. Scenarios 13.2%–15.5%).
 Ctrl+F "E-commerce"
@@ -7290,32 +7299,32 @@
 × 23.6% margin assumption → e-comm EBIT ≈ 1,160,812 ($000)</t>
         </is>
       </c>
-      <c r="E9" s="20" t="n">
+      <c r="E10" s="20" t="n">
         <v>0.236</v>
       </c>
-      <c r="F9" s="20" t="n">
+      <c r="F10" s="20" t="n">
         <v>0.236</v>
       </c>
-      <c r="G9" s="20" t="n">
+      <c r="G10" s="20" t="n">
         <v>0.236</v>
       </c>
-      <c r="H9" s="20" t="n">
+      <c r="H10" s="20" t="n">
         <v>0.236</v>
       </c>
-      <c r="I9" s="20" t="n">
+      <c r="I10" s="20" t="n">
         <v>0.236</v>
       </c>
-      <c r="J9" s="20" t="n">
+      <c r="J10" s="20" t="n">
         <v>0.236</v>
       </c>
     </row>
-    <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Phase 3: Other-channels EBIT margin %</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>Not % of consolidated revenue — EBIT as % of other-channel revenue only (not the Scenarios 13.2%–15.5% consolidated margin).
 9.1% margin assumption.
@@ -7324,12 +7333,12 @@
 Wholesale/license/outlets — lower-margin residual channel.</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: other channels (residual)</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>Not consolidated EBIT margin — EBIT ÷ other-channel revenue only (cf. Scenarios 13.2%–15.5%).
 Ctrl+F "Net revenue" → 11,102,600
@@ -7337,220 +7346,180 @@
 × 9.1% margin assumption → other EBIT ≈ 103,209 ($000)</t>
         </is>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E11" s="20" t="n">
         <v>0.091</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F11" s="20" t="n">
         <v>0.091</v>
       </c>
-      <c r="G10" s="20" t="n">
+      <c r="G11" s="20" t="n">
         <v>0.091</v>
       </c>
-      <c r="H10" s="20" t="n">
+      <c r="H11" s="20" t="n">
         <v>0.091</v>
       </c>
-      <c r="I10" s="20" t="n">
+      <c r="I11" s="20" t="n">
         <v>0.091</v>
       </c>
-      <c r="J10" s="20" t="n">
+      <c r="J11" s="20" t="n">
         <v>0.091</v>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
-        <is>
-          <t>Phase 4: Terminal marginal tax rate</t>
-        </is>
-      </c>
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>30% statutory marginal rate. t_operating transitions here over the 5-year forecast.</t>
-        </is>
-      </c>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>Q2 FY2026 outlook: tax rate ≈ 30%</t>
-        </is>
-      </c>
-      <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "a tax rate of approximately 30%" → terminal marginal rate for t_operating glide path.</t>
-        </is>
-      </c>
-      <c r="E11" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F11" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G11" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="H11" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="I11" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J11" s="20" t="n">
-        <v>0.3</v>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
+          <t>Phase 4: Terminal marginal tax rate</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>30% statutory marginal rate. t_operating transitions here over the 5-year forecast.</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Q2 FY2026 outlook: tax rate ≈ 30%</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Ctrl+F "a tax rate of approximately 30%" → terminal marginal rate for t_operating glide path.</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F12" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G12" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H12" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I12" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J12" s="20" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
           <t>Phase 2: R&amp;D / software amortization period (years)</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>Not % of revenue — amortization period (years) if R&amp;D/software is capitalized. LULU: no separate R&amp;D cap.</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
         <is>
           <t>NOPAT Bridge: capitalization convention</t>
         </is>
       </c>
-      <c r="D12" s="19" t="inlineStr">
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>Amortization period if R&amp;D capitalized (3–5 yr convention). LULU: no separate R&amp;D capitalization.</t>
         </is>
       </c>
-      <c r="E12" s="40" t="n">
+      <c r="E13" s="40" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="40" t="n">
+      <c r="F13" s="40" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="40" t="n">
+      <c r="G13" s="40" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="40" t="n">
+      <c r="H13" s="40" t="n">
         <v>4</v>
       </c>
-      <c r="I12" s="40" t="n">
+      <c r="I13" s="40" t="n">
         <v>4</v>
       </c>
-      <c r="J12" s="40" t="n">
+      <c r="J13" s="40" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="14" hidden="1" outlineLevel="1">
-      <c r="A14" s="72" t="inlineStr">
+    <row r="15" hidden="1" outlineLevel="1">
+      <c r="A15" s="72" t="inlineStr">
         <is>
           <t>Phase 1 — Operating normalization</t>
         </is>
-      </c>
-    </row>
-    <row r="15" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>Reported operating income (EBIT)</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>FY25: reported operating income from 10-K. Forecast: Scenarios base-case EBIT (margin path).</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K: Income from operations</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>Ctrl+F "Income from operations" → 2,210,615 ($000). Forecast links to Scenarios EBIT.</t>
-        </is>
-      </c>
-      <c r="E15" s="73" t="n">
-        <v>2210615</v>
-      </c>
-      <c r="F15" s="74">
-        <f>Scenarios!G43</f>
-        <v/>
-      </c>
-      <c r="G15" s="74">
-        <f>Scenarios!G44</f>
-        <v/>
-      </c>
-      <c r="H15" s="74">
-        <f>Scenarios!G45</f>
-        <v/>
-      </c>
-      <c r="I15" s="74">
-        <f>Scenarios!G46</f>
-        <v/>
-      </c>
-      <c r="J15" s="74">
-        <f>Scenarios!G47</f>
-        <v/>
       </c>
     </row>
     <row r="16" hidden="1" outlineLevel="1" ht="28" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>+ Impairment / intangible amortization (add-back)</t>
+          <t>Reported operating income (EBIT)</t>
         </is>
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Add back intangible amortization / impairments. FY25 = other operating expense amortization run-rate.</t>
+          <t>FY25: reported operating income from 10-K. Forecast: Scenarios base-case EBIT (margin path).</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K: amortization of intangible assets</t>
+          <t>LULU FY2025 10-K: Income from operations</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Amortization of intangible assets" → other operating expense run-rate (add-back).</t>
+          <t>Ctrl+F "Income from operations" → 2,210,615 ($000). Forecast links to Scenarios EBIT.</t>
         </is>
       </c>
       <c r="E16" s="73" t="n">
-        <v>6961</v>
-      </c>
-      <c r="F16" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="74" t="n">
-        <v>0</v>
+        <v>2210615</v>
+      </c>
+      <c r="F16" s="74">
+        <f>Scenarios!G43</f>
+        <v/>
+      </c>
+      <c r="G16" s="74">
+        <f>Scenarios!G44</f>
+        <v/>
+      </c>
+      <c r="H16" s="74">
+        <f>Scenarios!G45</f>
+        <v/>
+      </c>
+      <c r="I16" s="74">
+        <f>Scenarios!G46</f>
+        <v/>
+      </c>
+      <c r="J16" s="74">
+        <f>Scenarios!G47</f>
+        <v/>
       </c>
     </row>
     <row r="17" hidden="1" outlineLevel="1" ht="28" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>+ Restructuring costs (add-back)</t>
+          <t>+ Impairment / intangible amortization (add-back)</t>
         </is>
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>Add back restructuring (severance, store closures). LULU FY25: none identified.</t>
+          <t>Add back intangible amortization / impairments. FY25 = other operating expense amortization run-rate.</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K: restructuring charges</t>
+          <t>LULU FY2025 10-K: amortization of intangible assets</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "restructuring" → none material in FY25 10-K.</t>
+          <t>Ctrl+F "Amortization of intangible assets" → other operating expense run-rate (add-back).</t>
         </is>
       </c>
       <c r="E17" s="73" t="n">
-        <v>0</v>
+        <v>6961</v>
       </c>
       <c r="F17" s="74" t="n">
         <v>0</v>
@@ -7571,22 +7540,22 @@
     <row r="18" hidden="1" outlineLevel="1" ht="28" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>+ Legal / M&amp;A one-offs (add-back)</t>
+          <t>+ Restructuring costs (add-back)</t>
         </is>
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>Strip one-off legal / M&amp;A advisory fees. LULU FY25: none identified.</t>
+          <t>Add back restructuring (severance, store closures). LULU FY25: none identified.</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K: SG&amp;A one-offs</t>
+          <t>LULU FY2025 10-K: restructuring charges</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>One-off legal/M&amp;A fees in SG&amp;A — none identified FY25.</t>
+          <t>Ctrl+F "restructuring" → none material in FY25 10-K.</t>
         </is>
       </c>
       <c r="E18" s="73" t="n">
@@ -7608,209 +7577,212 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" hidden="1" outlineLevel="1" ht="42" customHeight="1">
+    <row r="19" hidden="1" outlineLevel="1" ht="28" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>+ Stock-based compensation (add-back if flag = 1)</t>
+          <t>+ Legal / M&amp;A one-offs (add-back)</t>
         </is>
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — SBC add-back flag (1 = yes). UFCF uses diluted shares; add back non-cash SBC to EBIT. FY25 SBC $62,203k scaled with revenue in forecast.</t>
+          <t>Strip one-off legal / M&amp;A advisory fees. LULU FY25: none identified.</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
+          <t>LULU FY2025 10-K: SG&amp;A one-offs</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>One-off legal/M&amp;A fees in SG&amp;A — none identified FY25.</t>
+        </is>
+      </c>
+      <c r="E19" s="73" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" hidden="1" outlineLevel="1" ht="42" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>+ Stock-based compensation (add-back only if flag = 1)</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Not % of revenue — SBC add-back flag. Set to 0 (Convention A).
+SBC stays inside Scenarios EBIT/NOPAT as a real economic cost; DCF uses basic shares (111.4M).
+FY25 reference: $62,203k (10-K). Flag = 1 would add back (Convention B + diluted shares) — not used.</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
           <t>LULU CF statement (10-K): stock-based compensation</t>
         </is>
       </c>
-      <c r="D19" s="19" t="inlineStr">
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Stock-based compensation expense"
-→ 62,203 ($000). Flag = 1 adds back to EBIT (diluted-shares UFCF convention).</t>
-        </is>
-      </c>
-      <c r="E19" s="73" t="n">
-        <v>62203</v>
-      </c>
-      <c r="F19" s="74">
+→ 62,203 ($000) FY25 reference. Flag = 0: SBC stays in EBIT (Convention A); DCF IV uses basic 111,380k shares.</t>
+        </is>
+      </c>
+      <c r="E20" s="74">
+        <f>62203*$E$7</f>
+        <v/>
+      </c>
+      <c r="F20" s="74">
         <f>Scenarios!G23/11102600*62203*$E$7</f>
         <v/>
       </c>
-      <c r="G19" s="74">
+      <c r="G20" s="74">
         <f>Scenarios!G24/11102600*62203*$E$7</f>
         <v/>
       </c>
-      <c r="H19" s="74">
+      <c r="H20" s="74">
         <f>Scenarios!G25/11102600*62203*$E$7</f>
         <v/>
       </c>
-      <c r="I19" s="74">
+      <c r="I20" s="74">
         <f>Scenarios!G26/11102600*62203*$E$7</f>
         <v/>
       </c>
-      <c r="J19" s="74">
+      <c r="J20" s="74">
         <f>Scenarios!G27/11102600*62203*$E$7</f>
         <v/>
       </c>
     </row>
-    <row r="20" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A20" s="23">
+    <row r="21" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A21" s="23">
         <f> Adjusted EBIT (Phase 1)</f>
         <v/>
       </c>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>Phase 1 adjusted EBIT = reported + non-recurring add-backs + optional SBC.</t>
-        </is>
-      </c>
-      <c r="C20" s="24" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Phase 1 adjusted EBIT = reported + non-recurring add-backs. SBC add-back = 0 when flag = 0.</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
         <is>
           <t>NOPAT Bridge tab: Phase 1 subtotal</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>Sum of reported EBIT + Phase 1 add-backs on this tab.</t>
         </is>
       </c>
-      <c r="F20" s="25">
-        <f>F15+F16+F17+F18+F19</f>
-        <v/>
-      </c>
-      <c r="G20" s="25">
-        <f>G15+G16+G17+G18+G19</f>
-        <v/>
-      </c>
-      <c r="H20" s="25">
-        <f>H15+H16+H17+H18+H19</f>
-        <v/>
-      </c>
-      <c r="I20" s="25">
-        <f>I15+I16+I17+I18+I19</f>
-        <v/>
-      </c>
-      <c r="J20" s="25">
-        <f>J15+J16+J17+J18+J19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" hidden="1" outlineLevel="1">
-      <c r="A21" s="72" t="inlineStr">
+      <c r="F21" s="25">
+        <f>F16+F17+F18+F19+F20</f>
+        <v/>
+      </c>
+      <c r="G21" s="25">
+        <f>G16+G17+G18+G19+G20</f>
+        <v/>
+      </c>
+      <c r="H21" s="25">
+        <f>H16+H17+H18+H19+H20</f>
+        <v/>
+      </c>
+      <c r="I21" s="25">
+        <f>I16+I17+I18+I19+I20</f>
+        <v/>
+      </c>
+      <c r="J21" s="25">
+        <f>J16+J17+J18+J19+J20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" hidden="1" outlineLevel="1">
+      <c r="A22" s="72" t="inlineStr">
         <is>
           <t>Phase 2 — Lease &amp; capitalization (ASC 842 / IFRS 16)</t>
         </is>
       </c>
     </row>
-    <row r="22" hidden="1" outlineLevel="1" ht="42" customHeight="1">
-      <c r="A22" s="16" t="inlineStr">
+    <row r="23" hidden="1" outlineLevel="1" ht="42" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>+ Implied lease interest expense (reclass from rent)</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>Not % of revenue — implied lease interest ($1,028k FY25). Reclass from rent to unlevered EBIT; scales with revenue in forecast.</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: interest on lease liabilities (supplemental)</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
+      <c r="D23" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "Interest paid on lease liabilities"
 → 1,028 ($000) supplemental cash-flow disclosure. Reclass to unlevered EBIT.</t>
         </is>
       </c>
-      <c r="E22" s="73" t="n">
+      <c r="E23" s="73" t="n">
         <v>1028</v>
       </c>
-      <c r="F22" s="74">
+      <c r="F23" s="74">
         <f>1028*(Scenarios!G23/11102600)</f>
         <v/>
       </c>
-      <c r="G22" s="74">
+      <c r="G23" s="74">
         <f>1028*(Scenarios!G24/11102600)</f>
         <v/>
       </c>
-      <c r="H22" s="74">
+      <c r="H23" s="74">
         <f>1028*(Scenarios!G25/11102600)</f>
         <v/>
       </c>
-      <c r="I22" s="74">
+      <c r="I23" s="74">
         <f>1028*(Scenarios!G26/11102600)</f>
         <v/>
       </c>
-      <c r="J22" s="74">
+      <c r="J23" s="74">
         <f>1028*(Scenarios!G27/11102600)</f>
         <v/>
-      </c>
-    </row>
-    <row r="23" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>+ Capitalize R&amp;D / software (current-year expense)</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>Capitalize multi-year software/R&amp;D. LULU: immaterial separate R&amp;D line — held at $0.</t>
-        </is>
-      </c>
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>LULU FY2025 10-K: R&amp;D / software expense</t>
-        </is>
-      </c>
-      <c r="D23" s="19" t="inlineStr">
-        <is>
-          <t>R&amp;D / software capitalization — LULU immaterial; held at $0.</t>
-        </is>
-      </c>
-      <c r="E23" s="73" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="74" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="74" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="24" hidden="1" outlineLevel="1" ht="28" customHeight="1">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>− Amortization of prior capitalized intangibles</t>
+          <t>+ Capitalize R&amp;D / software (current-year expense)</t>
         </is>
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>Amortization of prior capitalized intangibles. LULU: flows through existing D&amp;A.</t>
+          <t>Capitalize multi-year software/R&amp;D. LULU: immaterial separate R&amp;D line — held at $0.</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>LULU FY2025 10-K: intangible amortization</t>
+          <t>LULU FY2025 10-K: R&amp;D / software expense</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>Amortization of prior capitalized intangibles — netted in D&amp;A line.</t>
+          <t>R&amp;D / software capitalization — LULU immaterial; held at $0.</t>
         </is>
       </c>
       <c r="E24" s="73" t="n">
-        <v>6961</v>
+        <v>0</v>
       </c>
       <c r="F24" s="74" t="n">
         <v>0</v>
@@ -7829,195 +7801,235 @@
       </c>
     </row>
     <row r="25" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A25" s="23">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>− Amortization of prior capitalized intangibles</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Amortization of prior capitalized intangibles. LULU: flows through existing D&amp;A.</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>LULU FY2025 10-K: intangible amortization</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>Amortization of prior capitalized intangibles — netted in D&amp;A line.</t>
+        </is>
+      </c>
+      <c r="E25" s="73" t="n">
+        <v>6961</v>
+      </c>
+      <c r="F25" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A26" s="23">
         <f> EBIT after lease &amp; capitalization (Phase 2)</f>
         <v/>
       </c>
-      <c r="B25" s="17" t="inlineStr">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>Phase 2 EBIT = Phase 1 + lease interest reclass + R&amp;D cap − amortization.</t>
         </is>
       </c>
-      <c r="C25" s="24" t="inlineStr">
+      <c r="C26" s="24" t="inlineStr">
         <is>
           <t>NOPAT Bridge tab: Phase 2 subtotal</t>
         </is>
       </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="D26" s="19" t="inlineStr">
         <is>
           <t>Phase 1 + lease interest + R&amp;D cap − amortization.</t>
         </is>
       </c>
-      <c r="F25" s="25">
-        <f>F20+F22+F23-F24</f>
-        <v/>
-      </c>
-      <c r="G25" s="25">
-        <f>G20+G22+G23-G24</f>
-        <v/>
-      </c>
-      <c r="H25" s="25">
-        <f>H20+H22+H23-H24</f>
-        <v/>
-      </c>
-      <c r="I25" s="25">
-        <f>I20+I22+I23-I24</f>
-        <v/>
-      </c>
-      <c r="J25" s="25">
-        <f>J20+J22+J23-J24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" hidden="1" outlineLevel="1">
-      <c r="A26" s="72" t="inlineStr">
+      <c r="F26" s="25">
+        <f>F21+F23+F24-F25</f>
+        <v/>
+      </c>
+      <c r="G26" s="25">
+        <f>G21+G23+G24-G25</f>
+        <v/>
+      </c>
+      <c r="H26" s="25">
+        <f>H21+H23+H24-H25</f>
+        <v/>
+      </c>
+      <c r="I26" s="25">
+        <f>I21+I23+I24-I25</f>
+        <v/>
+      </c>
+      <c r="J26" s="25">
+        <f>J21+J23+J24-J25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" hidden="1" outlineLevel="1">
+      <c r="A27" s="72" t="inlineStr">
         <is>
           <t>Phase 3 — Segment / channel EBIT (driver-based)</t>
         </is>
-      </c>
-    </row>
-    <row r="27" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Store-channel revenue</t>
-        </is>
-      </c>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>Not % of revenue — store-channel revenue from Revenue Drivers tab.</t>
-        </is>
-      </c>
-      <c r="C27" s="18" t="inlineStr">
-        <is>
-          <t>Revenue Drivers tab: store-channel revenue</t>
-        </is>
-      </c>
-      <c r="D27" s="19" t="inlineStr">
-        <is>
-          <t>Revenue Drivers tab → store-channel revenue row.</t>
-        </is>
-      </c>
-      <c r="E27" s="73" t="n">
-        <v>5049744</v>
-      </c>
-      <c r="F27" s="74">
-        <f>'Revenue Drivers'!F31</f>
-        <v/>
-      </c>
-      <c r="G27" s="74">
-        <f>'Revenue Drivers'!G31</f>
-        <v/>
-      </c>
-      <c r="H27" s="74">
-        <f>'Revenue Drivers'!H31</f>
-        <v/>
-      </c>
-      <c r="I27" s="74">
-        <f>'Revenue Drivers'!I31</f>
-        <v/>
-      </c>
-      <c r="J27" s="74">
-        <f>'Revenue Drivers'!J31</f>
-        <v/>
       </c>
     </row>
     <row r="28" hidden="1" outlineLevel="1" ht="28" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  E-commerce revenue</t>
+          <t xml:space="preserve">  Store-channel revenue</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — e-commerce revenue from Revenue Drivers tab.</t>
+          <t>Not % of revenue — store-channel revenue from Revenue Drivers tab.</t>
         </is>
       </c>
       <c r="C28" s="18" t="inlineStr">
         <is>
-          <t>Revenue Drivers tab: e-commerce revenue</t>
+          <t>Revenue Drivers tab: store-channel revenue</t>
         </is>
       </c>
       <c r="D28" s="19" t="inlineStr">
         <is>
-          <t>Revenue Drivers tab → e-commerce revenue row.</t>
+          <t>Revenue Drivers tab → store-channel revenue row.</t>
         </is>
       </c>
       <c r="E28" s="73" t="n">
-        <v>4918697</v>
+        <v>5049744</v>
       </c>
       <c r="F28" s="74">
-        <f>'Revenue Drivers'!F41</f>
+        <f>'Revenue Drivers'!F31</f>
         <v/>
       </c>
       <c r="G28" s="74">
-        <f>'Revenue Drivers'!G41</f>
+        <f>'Revenue Drivers'!G31</f>
         <v/>
       </c>
       <c r="H28" s="74">
-        <f>'Revenue Drivers'!H41</f>
+        <f>'Revenue Drivers'!H31</f>
         <v/>
       </c>
       <c r="I28" s="74">
-        <f>'Revenue Drivers'!I41</f>
+        <f>'Revenue Drivers'!I31</f>
         <v/>
       </c>
       <c r="J28" s="74">
-        <f>'Revenue Drivers'!J41</f>
+        <f>'Revenue Drivers'!J31</f>
         <v/>
       </c>
     </row>
     <row r="29" hidden="1" outlineLevel="1" ht="28" customHeight="1">
       <c r="A29" s="16" t="inlineStr">
         <is>
+          <t xml:space="preserve">  E-commerce revenue</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>Not % of revenue — e-commerce revenue from Revenue Drivers tab.</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab: e-commerce revenue</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>Revenue Drivers tab → e-commerce revenue row.</t>
+        </is>
+      </c>
+      <c r="E29" s="73" t="n">
+        <v>4918697</v>
+      </c>
+      <c r="F29" s="74">
+        <f>'Revenue Drivers'!F41</f>
+        <v/>
+      </c>
+      <c r="G29" s="74">
+        <f>'Revenue Drivers'!G41</f>
+        <v/>
+      </c>
+      <c r="H29" s="74">
+        <f>'Revenue Drivers'!H41</f>
+        <v/>
+      </c>
+      <c r="I29" s="74">
+        <f>'Revenue Drivers'!I41</f>
+        <v/>
+      </c>
+      <c r="J29" s="74">
+        <f>'Revenue Drivers'!J41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Other channels revenue</t>
         </is>
       </c>
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>Not % of revenue — wholesale/license/outlet revenue from Revenue Drivers tab.</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>Revenue Drivers tab: other channels revenue</t>
         </is>
       </c>
-      <c r="D29" s="19" t="inlineStr">
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>Revenue Drivers tab → other channels revenue row.</t>
         </is>
       </c>
-      <c r="E29" s="73" t="n">
+      <c r="E30" s="73" t="n">
         <v>1134159</v>
       </c>
-      <c r="F29" s="74">
+      <c r="F30" s="74">
         <f>'Revenue Drivers'!F45</f>
         <v/>
       </c>
-      <c r="G29" s="74">
+      <c r="G30" s="74">
         <f>'Revenue Drivers'!G45</f>
         <v/>
       </c>
-      <c r="H29" s="74">
+      <c r="H30" s="74">
         <f>'Revenue Drivers'!H45</f>
         <v/>
       </c>
-      <c r="I29" s="74">
+      <c r="I30" s="74">
         <f>'Revenue Drivers'!I45</f>
         <v/>
       </c>
-      <c r="J29" s="74">
+      <c r="J30" s="74">
         <f>'Revenue Drivers'!J45</f>
         <v/>
       </c>
     </row>
-    <row r="30" hidden="1" outlineLevel="1" ht="70" customHeight="1">
-      <c r="A30" s="16" t="inlineStr">
+    <row r="31" hidden="1" outlineLevel="1" ht="70" customHeight="1">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Store-channel EBIT (= Rev × store margin)</t>
         </is>
       </c>
-      <c r="B30" s="17" t="inlineStr">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>Not % of consolidated revenue — store EBIT ÷ store revenue only (not Scenarios consolidated EBIT margin).
 EBIT_store,t = Rev_store,t × 18.6%
@@ -8025,12 +8037,12 @@
 Margin from driver assumptions row above; ties to 10-K store revenue.</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
+      <c r="C31" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: company-operated stores net revenue</t>
         </is>
       </c>
-      <c r="D30" s="19" t="inlineStr">
+      <c r="D31" s="19" t="inlineStr">
         <is>
           <t>Not consolidated EBIT margin — store EBIT ÷ store revenue only.
 Ctrl+F "Company-operated stores"
@@ -8038,37 +8050,37 @@
 EBIT = Rev × 18.6% → ≈ 939,252 ($000)</t>
         </is>
       </c>
-      <c r="E30" s="74" t="n">
+      <c r="E31" s="74" t="n">
         <v>939252.384</v>
       </c>
-      <c r="F30" s="74">
-        <f>F27*E$8</f>
-        <v/>
-      </c>
-      <c r="G30" s="74">
-        <f>G27*E$8</f>
-        <v/>
-      </c>
-      <c r="H30" s="74">
-        <f>H27*E$8</f>
-        <v/>
-      </c>
-      <c r="I30" s="74">
-        <f>I27*E$8</f>
-        <v/>
-      </c>
-      <c r="J30" s="74">
-        <f>J27*E$8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" hidden="1" outlineLevel="1" ht="70" customHeight="1">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="F31" s="74">
+        <f>F28*E$9</f>
+        <v/>
+      </c>
+      <c r="G31" s="74">
+        <f>G28*E$9</f>
+        <v/>
+      </c>
+      <c r="H31" s="74">
+        <f>H28*E$9</f>
+        <v/>
+      </c>
+      <c r="I31" s="74">
+        <f>I28*E$9</f>
+        <v/>
+      </c>
+      <c r="J31" s="74">
+        <f>J28*E$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" hidden="1" outlineLevel="1" ht="70" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  E-commerce EBIT (= Rev × e-comm margin)</t>
         </is>
       </c>
-      <c r="B31" s="17" t="inlineStr">
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>Not % of consolidated revenue — e-commerce EBIT ÷ e-commerce revenue only (not Scenarios consolidated EBIT margin).
 EBIT_e-comm,t = Rev_e-comm,t × 23.6%
@@ -8076,12 +8088,12 @@
 Higher than stores — no brick-and-mortar occupancy drag.</t>
         </is>
       </c>
-      <c r="C31" s="18" t="inlineStr">
+      <c r="C32" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: e-commerce net revenue</t>
         </is>
       </c>
-      <c r="D31" s="19" t="inlineStr">
+      <c r="D32" s="19" t="inlineStr">
         <is>
           <t>Not consolidated EBIT margin — e-commerce EBIT ÷ e-commerce revenue only.
 Ctrl+F "E-commerce"
@@ -8089,37 +8101,37 @@
 EBIT = Rev × 23.6% → ≈ 1,160,812 ($000)</t>
         </is>
       </c>
-      <c r="E31" s="74" t="n">
+      <c r="E32" s="74" t="n">
         <v>1160812.492</v>
       </c>
-      <c r="F31" s="74">
-        <f>F28*E$9</f>
-        <v/>
-      </c>
-      <c r="G31" s="74">
-        <f>G28*E$9</f>
-        <v/>
-      </c>
-      <c r="H31" s="74">
-        <f>H28*E$9</f>
-        <v/>
-      </c>
-      <c r="I31" s="74">
-        <f>I28*E$9</f>
-        <v/>
-      </c>
-      <c r="J31" s="74">
-        <f>J28*E$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" hidden="1" outlineLevel="1" ht="56" customHeight="1">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="F32" s="74">
+        <f>F29*E$10</f>
+        <v/>
+      </c>
+      <c r="G32" s="74">
+        <f>G29*E$10</f>
+        <v/>
+      </c>
+      <c r="H32" s="74">
+        <f>H29*E$10</f>
+        <v/>
+      </c>
+      <c r="I32" s="74">
+        <f>I29*E$10</f>
+        <v/>
+      </c>
+      <c r="J32" s="74">
+        <f>J29*E$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" hidden="1" outlineLevel="1" ht="56" customHeight="1">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Other-channels EBIT (= Rev × other margin)</t>
         </is>
       </c>
-      <c r="B32" s="17" t="inlineStr">
+      <c r="B33" s="17" t="inlineStr">
         <is>
           <t>Not % of consolidated revenue — other-channel EBIT ÷ other revenue only (not Scenarios consolidated EBIT margin).
 EBIT_other,t = Rev_other,t × 9.1%
@@ -8127,224 +8139,224 @@
 Wholesale/license/outlets — lowest channel margin.</t>
         </is>
       </c>
-      <c r="C32" s="18" t="inlineStr">
+      <c r="C33" s="18" t="inlineStr">
         <is>
           <t>FY2025 10-K: other channels (residual)</t>
         </is>
       </c>
-      <c r="D32" s="19" t="inlineStr">
+      <c r="D33" s="19" t="inlineStr">
         <is>
           <t>Not consolidated EBIT margin — other-channel EBIT ÷ other revenue only.
 Other rev = 11,102,600 − 5,049,744 − 4,918,697 ≈ 1,134,159 ($000)
 EBIT = Rev × 9.1% → ≈ 103,209 ($000)</t>
         </is>
       </c>
-      <c r="E32" s="74" t="n">
+      <c r="E33" s="74" t="n">
         <v>103208.469</v>
       </c>
-      <c r="F32" s="74">
-        <f>F29*E$10</f>
-        <v/>
-      </c>
-      <c r="G32" s="74">
-        <f>G29*E$10</f>
-        <v/>
-      </c>
-      <c r="H32" s="74">
-        <f>H29*E$10</f>
-        <v/>
-      </c>
-      <c r="I32" s="74">
-        <f>I29*E$10</f>
-        <v/>
-      </c>
-      <c r="J32" s="74">
-        <f>J29*E$10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A33" s="23" t="inlineStr">
+      <c r="F33" s="74">
+        <f>F30*E$11</f>
+        <v/>
+      </c>
+      <c r="G33" s="74">
+        <f>G30*E$11</f>
+        <v/>
+      </c>
+      <c r="H33" s="74">
+        <f>H30*E$11</f>
+        <v/>
+      </c>
+      <c r="I33" s="74">
+        <f>I30*E$11</f>
+        <v/>
+      </c>
+      <c r="J33" s="74">
+        <f>J30*E$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A34" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  Channel EBIT (sum of sector EBIT)</t>
         </is>
       </c>
-      <c r="B33" s="17" t="inlineStr">
+      <c r="B34" s="17" t="inlineStr">
         <is>
           <t>Phase 3 channel EBIT = Σ sector EBIT_i. FY26 adds Scenarios tariff refund.</t>
         </is>
       </c>
-      <c r="C33" s="24" t="inlineStr">
+      <c r="C34" s="24" t="inlineStr">
         <is>
           <t>NOPAT Bridge tab: sector EBIT subtotal</t>
         </is>
       </c>
-      <c r="D33" s="19" t="inlineStr">
+      <c r="D34" s="19" t="inlineStr">
         <is>
           <t>Sum of sector EBIT rows. FY26 adds Scenarios tariff refund cell.</t>
         </is>
       </c>
-      <c r="F33" s="69">
-        <f>F30+F31+F32+Scenarios!G7</f>
-        <v/>
-      </c>
-      <c r="G33" s="69">
-        <f>G30+G31+G32</f>
-        <v/>
-      </c>
-      <c r="H33" s="69">
-        <f>H30+H31+H32</f>
-        <v/>
-      </c>
-      <c r="I33" s="69">
-        <f>I30+I31+I32</f>
-        <v/>
-      </c>
-      <c r="J33" s="69">
-        <f>J30+J31+J32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A34" s="23">
-        <f> EBIT after channel mix (Phase 3)</f>
-        <v/>
-      </c>
-      <c r="B34" s="17" t="inlineStr">
-        <is>
-          <t>Channel-mix EBIT output (Phase 3). Check row vs Scenarios shows channel vs margin-path gap.</t>
-        </is>
-      </c>
-      <c r="C34" s="24" t="inlineStr">
-        <is>
-          <t>NOPAT Bridge tab: Phase 3 subtotal</t>
-        </is>
-      </c>
-      <c r="D34" s="19" t="inlineStr">
-        <is>
-          <t>Channel EBIT subtotal (Phase 3). Compare Check row vs Scenarios.</t>
-        </is>
-      </c>
-      <c r="E34" s="75" t="n">
-        <v>2203273.345</v>
-      </c>
-      <c r="F34" s="25">
-        <f>F33</f>
-        <v/>
-      </c>
-      <c r="G34" s="25">
-        <f>G33</f>
-        <v/>
-      </c>
-      <c r="H34" s="25">
-        <f>H33</f>
-        <v/>
-      </c>
-      <c r="I34" s="25">
-        <f>I33</f>
-        <v/>
-      </c>
-      <c r="J34" s="25">
-        <f>J33</f>
+      <c r="F34" s="69">
+        <f>F31+F32+F33+Scenarios!G7</f>
+        <v/>
+      </c>
+      <c r="G34" s="69">
+        <f>G31+G32+G33</f>
+        <v/>
+      </c>
+      <c r="H34" s="69">
+        <f>H31+H32+H33</f>
+        <v/>
+      </c>
+      <c r="I34" s="69">
+        <f>I31+I32+I33</f>
+        <v/>
+      </c>
+      <c r="J34" s="69">
+        <f>J31+J32+J33</f>
         <v/>
       </c>
     </row>
     <row r="35" hidden="1" outlineLevel="1" ht="28" customHeight="1">
       <c r="A35" s="23">
+        <f> EBIT after channel mix (Phase 3)</f>
+        <v/>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Channel-mix EBIT output (Phase 3). Check row vs Scenarios shows channel vs margin-path gap.</t>
+        </is>
+      </c>
+      <c r="C35" s="24" t="inlineStr">
+        <is>
+          <t>NOPAT Bridge tab: Phase 3 subtotal</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>Channel EBIT subtotal (Phase 3). Compare Check row vs Scenarios.</t>
+        </is>
+      </c>
+      <c r="E35" s="75" t="n">
+        <v>2203273.345</v>
+      </c>
+      <c r="F35" s="25">
+        <f>F34</f>
+        <v/>
+      </c>
+      <c r="G35" s="25">
+        <f>G34</f>
+        <v/>
+      </c>
+      <c r="H35" s="25">
+        <f>H34</f>
+        <v/>
+      </c>
+      <c r="I35" s="25">
+        <f>I34</f>
+        <v/>
+      </c>
+      <c r="J35" s="25">
+        <f>J34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A36" s="23">
         <f> Normalized EBIT (tax base for NOPAT)</f>
         <v/>
       </c>
-      <c r="B35" s="17" t="inlineStr">
-        <is>
-          <t>FY25: Phases 1–2 walk-through. Forecast: Scenarios base EBIT — tax base for NOPAT.</t>
-        </is>
-      </c>
-      <c r="C35" s="24" t="inlineStr">
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>FY25: Phases 1–2 walk-through (SBC not added back; flag = 0). Forecast: Scenarios base EBIT — tax base for NOPAT.</t>
+        </is>
+      </c>
+      <c r="C36" s="24" t="inlineStr">
         <is>
           <t>Scenarios tab: base-case EBIT (forecast)</t>
         </is>
       </c>
-      <c r="D35" s="19" t="inlineStr">
+      <c r="D36" s="19" t="inlineStr">
         <is>
           <t>FY25: Phase 1–2 formula. Forecast: Scenarios base EBIT (tax base).</t>
         </is>
       </c>
-      <c r="E35" s="25">
-        <f>E20+E22+E23-E24</f>
-        <v/>
-      </c>
-      <c r="F35" s="25">
+      <c r="E36" s="25">
+        <f>E21+E23+E24-E25</f>
+        <v/>
+      </c>
+      <c r="F36" s="25">
         <f>Scenarios!G43</f>
         <v/>
       </c>
-      <c r="G35" s="25">
+      <c r="G36" s="25">
         <f>Scenarios!G44</f>
         <v/>
       </c>
-      <c r="H35" s="25">
+      <c r="H36" s="25">
         <f>Scenarios!G45</f>
         <v/>
       </c>
-      <c r="I35" s="25">
+      <c r="I36" s="25">
         <f>Scenarios!G46</f>
         <v/>
       </c>
-      <c r="J35" s="25">
+      <c r="J36" s="25">
         <f>Scenarios!G47</f>
         <v/>
       </c>
     </row>
-    <row r="36" hidden="1" outlineLevel="1">
-      <c r="A36" s="16" t="inlineStr">
+    <row r="37" hidden="1" outlineLevel="1">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  Check vs Scenarios EBIT (base case)</t>
         </is>
       </c>
-      <c r="F36" s="74">
-        <f>F35-Scenarios!G43</f>
-        <v/>
-      </c>
-      <c r="G36" s="74">
-        <f>G35-Scenarios!G44</f>
-        <v/>
-      </c>
-      <c r="H36" s="74">
-        <f>H35-Scenarios!G45</f>
-        <v/>
-      </c>
-      <c r="I36" s="74">
-        <f>I35-Scenarios!G46</f>
-        <v/>
-      </c>
-      <c r="J36" s="74">
-        <f>J35-Scenarios!G47</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" hidden="1" outlineLevel="1">
-      <c r="A37" s="72" t="inlineStr">
+      <c r="F37" s="74">
+        <f>F36-Scenarios!G43</f>
+        <v/>
+      </c>
+      <c r="G37" s="74">
+        <f>G36-Scenarios!G44</f>
+        <v/>
+      </c>
+      <c r="H37" s="74">
+        <f>H36-Scenarios!G45</f>
+        <v/>
+      </c>
+      <c r="I37" s="74">
+        <f>I36-Scenarios!G46</f>
+        <v/>
+      </c>
+      <c r="J37" s="74">
+        <f>J36-Scenarios!G47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" hidden="1" outlineLevel="1">
+      <c r="A38" s="72" t="inlineStr">
         <is>
           <t>Phase 4 — Tax normalization to NOPAT</t>
         </is>
       </c>
     </row>
-    <row r="38" hidden="1" outlineLevel="1" ht="70" customHeight="1">
-      <c r="A38" s="16" t="inlineStr">
+    <row r="39" hidden="1" outlineLevel="1" ht="70" customHeight="1">
+      <c r="A39" s="16" t="inlineStr">
         <is>
           <t>Operating effective tax rate (t_operating)</t>
         </is>
       </c>
-      <c r="B38" s="17" t="inlineStr">
+      <c r="B39" s="17" t="inlineStr">
         <is>
           <t>Operating effective tax rate: (tax + interest shield) ÷ (EBT + interest). Transitions from FY25 t_operating toward 30% marginal over 5 years.</t>
         </is>
       </c>
-      <c r="C38" s="18" t="inlineStr">
+      <c r="C39" s="18" t="inlineStr">
         <is>
           <t>LULU FY2025 10-K: income tax &amp; interest expense</t>
         </is>
       </c>
-      <c r="D38" s="19" t="inlineStr">
+      <c r="D39" s="19" t="inlineStr">
         <is>
           <t>t_operating = (tax + interest×30%) ÷ (EBT + interest).
 Ctrl+F "Income tax expense" → 659,784
@@ -8352,184 +8364,157 @@
 Ctrl+F "Interest paid on lease liabilities" → 1,028</t>
         </is>
       </c>
-      <c r="E38" s="76" t="n">
+      <c r="E39" s="76" t="n">
         <v>0.2946847649213503</v>
       </c>
-      <c r="F38" s="32">
-        <f>0.29468476492135026+(F$11-0.29468476492135026)*1/5</f>
-        <v/>
-      </c>
-      <c r="G38" s="32">
-        <f>0.29468476492135026+(G$11-0.29468476492135026)*2/5</f>
-        <v/>
-      </c>
-      <c r="H38" s="32">
-        <f>0.29468476492135026+(H$11-0.29468476492135026)*3/5</f>
-        <v/>
-      </c>
-      <c r="I38" s="32">
-        <f>0.29468476492135026+(I$11-0.29468476492135026)*4/5</f>
-        <v/>
-      </c>
-      <c r="J38" s="32">
-        <f>0.29468476492135026+(J$11-0.29468476492135026)*5/5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="F39" s="32">
+        <f>0.29468476492135026+(F$12-0.29468476492135026)*1/5</f>
+        <v/>
+      </c>
+      <c r="G39" s="32">
+        <f>0.29468476492135026+(G$12-0.29468476492135026)*2/5</f>
+        <v/>
+      </c>
+      <c r="H39" s="32">
+        <f>0.29468476492135026+(H$12-0.29468476492135026)*3/5</f>
+        <v/>
+      </c>
+      <c r="I39" s="32">
+        <f>0.29468476492135026+(I$12-0.29468476492135026)*4/5</f>
+        <v/>
+      </c>
+      <c r="J39" s="32">
+        <f>0.29468476492135026+(J$12-0.29468476492135026)*5/5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>Unlevered tax on normalized EBIT</t>
         </is>
       </c>
-      <c r="B39" s="17" t="inlineStr">
+      <c r="B40" s="17" t="inlineStr">
         <is>
           <t>Unlevered tax = normalized EBIT × t_operating. Strips debt-interest tax shield from GAAP rate.</t>
         </is>
       </c>
-      <c r="C39" s="24" t="inlineStr">
+      <c r="C40" s="24" t="inlineStr">
         <is>
           <t>NOPAT Bridge tab: unlevered tax expense</t>
         </is>
       </c>
-      <c r="D39" s="19" t="inlineStr">
+      <c r="D40" s="19" t="inlineStr">
         <is>
           <t>Normalized EBIT × t_operating — unlevered tax (no debt shield).</t>
         </is>
       </c>
-      <c r="F39" s="74">
-        <f>F35*F38</f>
-        <v/>
-      </c>
-      <c r="G39" s="74">
-        <f>G35*G38</f>
-        <v/>
-      </c>
-      <c r="H39" s="74">
-        <f>H35*H38</f>
-        <v/>
-      </c>
-      <c r="I39" s="74">
-        <f>I35*I38</f>
-        <v/>
-      </c>
-      <c r="J39" s="74">
-        <f>J35*J38</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" hidden="1" outlineLevel="1" ht="28" customHeight="1">
-      <c r="A40" s="23" t="inlineStr">
+      <c r="F40" s="74">
+        <f>F36*F39</f>
+        <v/>
+      </c>
+      <c r="G40" s="74">
+        <f>G36*G39</f>
+        <v/>
+      </c>
+      <c r="H40" s="74">
+        <f>H36*H39</f>
+        <v/>
+      </c>
+      <c r="I40" s="74">
+        <f>I36*I39</f>
+        <v/>
+      </c>
+      <c r="J40" s="74">
+        <f>J36*J39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" hidden="1" outlineLevel="1" ht="28" customHeight="1">
+      <c r="A41" s="23" t="inlineStr">
         <is>
           <t>NORMALIZED NOPAT</t>
         </is>
       </c>
-      <c r="B40" s="17" t="inlineStr">
+      <c r="B41" s="17" t="inlineStr">
         <is>
           <t>NORMALIZED NOPAT = EBIT_norm × (1 − t_operating). Scenarios base case links here.</t>
         </is>
       </c>
-      <c r="C40" s="24" t="inlineStr">
+      <c r="C41" s="24" t="inlineStr">
         <is>
           <t>NOPAT Bridge tab: normalized NOPAT</t>
         </is>
       </c>
-      <c r="D40" s="19" t="inlineStr">
+      <c r="D41" s="19" t="inlineStr">
         <is>
           <t>EBIT_norm − unlevered tax. Scenarios base-case NOPAT links to this row.</t>
         </is>
       </c>
-      <c r="F40" s="25">
-        <f>F35-F39</f>
-        <v/>
-      </c>
-      <c r="G40" s="25">
-        <f>G35-G39</f>
-        <v/>
-      </c>
-      <c r="H40" s="25">
-        <f>H35-H39</f>
-        <v/>
-      </c>
-      <c r="I40" s="25">
-        <f>I35-I39</f>
-        <v/>
-      </c>
-      <c r="J40" s="25">
-        <f>J35-J39</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="72" t="inlineStr">
+      <c r="F41" s="25">
+        <f>F36-F40</f>
+        <v/>
+      </c>
+      <c r="G41" s="25">
+        <f>G36-G40</f>
+        <v/>
+      </c>
+      <c r="H41" s="25">
+        <f>H36-H40</f>
+        <v/>
+      </c>
+      <c r="I41" s="25">
+        <f>I36-I40</f>
+        <v/>
+      </c>
+      <c r="J41" s="25">
+        <f>J36-J40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="72" t="inlineStr">
         <is>
           <t>Phase 5 — Agent workflow (execution steps)</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="77" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="77" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="C43" s="77" t="inlineStr">
+      <c r="C44" s="77" t="inlineStr">
         <is>
           <t>Without applied (FY26 DCF)</t>
         </is>
       </c>
-      <c r="D43" s="77" t="inlineStr">
+      <c r="D44" s="77" t="inlineStr">
         <is>
           <t>With applied (FY26 DCF)</t>
         </is>
       </c>
-      <c r="F43" s="77" t="inlineStr">
+      <c r="F44" s="77" t="inlineStr">
         <is>
           <t>Output</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="60" t="inlineStr">
-        <is>
-          <t>1. Clean base</t>
-        </is>
-      </c>
-      <c r="B44" s="78" t="inlineStr">
-        <is>
-          <t>SEC 10-K income statement</t>
-        </is>
-      </c>
-      <c r="C44" s="78" t="inlineStr">
-        <is>
-          <t>EBIT = 13.2% × rev + tariff; no add-backs.</t>
-        </is>
-      </c>
-      <c r="D44" s="78" t="inlineStr">
-        <is>
-          <t>DCF unchanged.</t>
-        </is>
-      </c>
-      <c r="F44" s="79" t="inlineStr">
-        <is>
-          <t>EBIT_adj (Phase 1)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="60" t="inlineStr">
         <is>
-          <t>2. Capitalize R&amp;D</t>
+          <t>1. Clean base</t>
         </is>
       </c>
       <c r="B45" s="78" t="inlineStr">
         <is>
-          <t>SG&amp;A footnotes</t>
+          <t>SEC 10-K income statement</t>
         </is>
       </c>
       <c r="C45" s="78" t="inlineStr">
         <is>
-          <t>R&amp;D/software expensed in full each year ($0 for LULU).</t>
+          <t>EBIT = 13.2% × rev + tariff; SBC stays expensed (flag = 0).</t>
         </is>
       </c>
       <c r="D45" s="78" t="inlineStr">
@@ -8539,24 +8524,24 @@
       </c>
       <c r="F45" s="79" t="inlineStr">
         <is>
-          <t>EBIT_capitalized (Phase 2)</t>
+          <t>EBIT_adj (Phase 1)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="60" t="inlineStr">
         <is>
-          <t>3. Lease shift</t>
+          <t>2. Capitalize R&amp;D</t>
         </is>
       </c>
       <c r="B46" s="78" t="inlineStr">
         <is>
-          <t>ASC 842 lease footnote</t>
+          <t>SG&amp;A footnotes</t>
         </is>
       </c>
       <c r="C46" s="78" t="inlineStr">
         <is>
-          <t>Rent in opex; no implied lease-interest add-back.</t>
+          <t>R&amp;D/software expensed in full each year ($0 for LULU).</t>
         </is>
       </c>
       <c r="D46" s="78" t="inlineStr">
@@ -8566,24 +8551,24 @@
       </c>
       <c r="F46" s="79" t="inlineStr">
         <is>
-          <t>EBIT_lease-adj (Phase 2)</t>
+          <t>EBIT_capitalized (Phase 2)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="60" t="inlineStr">
         <is>
-          <t>4. Segment mix</t>
+          <t>3. Lease shift</t>
         </is>
       </c>
       <c r="B47" s="78" t="inlineStr">
         <is>
-          <t>Revenue Drivers tab</t>
+          <t>ASC 842 lease footnote</t>
         </is>
       </c>
       <c r="C47" s="78" t="inlineStr">
         <is>
-          <t>DCF uses consolidated 13.2% on total revenue (+ tariff).</t>
+          <t>Rent in opex; no implied lease-interest add-back.</t>
         </is>
       </c>
       <c r="D47" s="78" t="inlineStr">
@@ -8593,73 +8578,100 @@
       </c>
       <c r="F47" s="79" t="inlineStr">
         <is>
-          <t>Forecast EBIT (Phase 3)</t>
+          <t>EBIT_lease-adj (Phase 2)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="60" t="inlineStr">
         <is>
-          <t>5. NOPAT bridge</t>
+          <t>4. Segment mix</t>
         </is>
       </c>
       <c r="B48" s="78" t="inlineStr">
         <is>
-          <t>Normalized EBIT &amp; t_operating</t>
+          <t>Revenue Drivers tab</t>
         </is>
       </c>
       <c r="C48" s="78" t="inlineStr">
         <is>
-          <t>NOPAT = EBIT × (1 − 30%) flat sc_tax.</t>
+          <t>DCF uses consolidated 13.2% on total revenue (+ tariff).</t>
         </is>
       </c>
       <c r="D48" s="78" t="inlineStr">
         <is>
-          <t>NOPAT = EBIT × (1 − t_operating) — same EBIT, slightly higher NOPAT.</t>
+          <t>DCF unchanged.</t>
         </is>
       </c>
       <c r="F48" s="79" t="inlineStr">
         <is>
-          <t>Normalized NOPAT</t>
+          <t>Forecast EBIT (Phase 3)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="60" t="inlineStr">
         <is>
+          <t>5. NOPAT bridge</t>
+        </is>
+      </c>
+      <c r="B49" s="78" t="inlineStr">
+        <is>
+          <t>Normalized EBIT &amp; t_operating</t>
+        </is>
+      </c>
+      <c r="C49" s="78" t="inlineStr">
+        <is>
+          <t>NOPAT = EBIT × (1 − 30%) flat sc_tax.</t>
+        </is>
+      </c>
+      <c r="D49" s="78" t="inlineStr">
+        <is>
+          <t>NOPAT = EBIT × (1 − t_operating) — same EBIT, slightly higher NOPAT.</t>
+        </is>
+      </c>
+      <c r="F49" s="79" t="inlineStr">
+        <is>
+          <t>Normalized NOPAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="60" t="inlineStr">
+        <is>
           <t>6. Tariff refund (Scenarios)</t>
         </is>
       </c>
-      <c r="B49" s="78" t="inlineStr">
+      <c r="B50" s="78" t="inlineStr">
         <is>
           <t>Q2 FY2026 earnings release</t>
         </is>
       </c>
-      <c r="C49" s="78" t="inlineStr">
+      <c r="C50" s="78" t="inlineStr">
         <is>
           <t>EBIT = Rev × 13.2% only (no refund).</t>
         </is>
       </c>
-      <c r="D49" s="78" t="inlineStr">
+      <c r="D50" s="78" t="inlineStr">
         <is>
           <t>+ $134,500k in FY26 — DCF uses this.</t>
         </is>
       </c>
-      <c r="F49" s="79" t="inlineStr">
+      <c r="F50" s="79" t="inlineStr">
         <is>
           <t>Scenarios EBIT (FY26)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="26" t="inlineStr">
-        <is>
-          <t>Steps 1–4: DCF unchanged on FY26. Step 5 changes NOPAT only (tax). Step 6 changes FY26 EBIT (+ tariff).</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="26" t="inlineStr">
+        <is>
+          <t>Steps 1–4: DCF unchanged on FY26. Step 5 changes NOPAT only (tax). Step 6 changes FY26 EBIT (+ tariff).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="26" t="inlineStr">
         <is>
           <t>Scenarios base-case NOPAT (col G) links to NORMALIZED NOPAT above. Bear/bull apply the same t_operating to their EBIT paths.</t>
         </is>
@@ -8668,38 +8680,37 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId21"/>
-    <hyperlink ref="C27" location="'Revenue Drivers'!B31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId22"/>
-    <hyperlink ref="C28" location="'Revenue Drivers'!B41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId23"/>
-    <hyperlink ref="C29" location="'Revenue Drivers'!B45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId20"/>
+    <hyperlink ref="C28" location="'Revenue Drivers'!B31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId21"/>
+    <hyperlink ref="C29" location="'Revenue Drivers'!B41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId22"/>
+    <hyperlink ref="C30" location="'Revenue Drivers'!B45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9174,23 +9185,23 @@
         </is>
       </c>
       <c r="F13" s="74">
-        <f>-'NOPAT Bridge'!F39</f>
+        <f>-'NOPAT Bridge'!F40</f>
         <v/>
       </c>
       <c r="G13" s="74">
-        <f>-'NOPAT Bridge'!G39</f>
+        <f>-'NOPAT Bridge'!G40</f>
         <v/>
       </c>
       <c r="H13" s="74">
-        <f>-'NOPAT Bridge'!H39</f>
+        <f>-'NOPAT Bridge'!H40</f>
         <v/>
       </c>
       <c r="I13" s="74">
-        <f>-'NOPAT Bridge'!I39</f>
+        <f>-'NOPAT Bridge'!I40</f>
         <v/>
       </c>
       <c r="J13" s="74">
-        <f>-'NOPAT Bridge'!J39</f>
+        <f>-'NOPAT Bridge'!J40</f>
         <v/>
       </c>
     </row>
@@ -10784,23 +10795,23 @@
         <v>1579183</v>
       </c>
       <c r="F76" s="74">
-        <f>('NOPAT Bridge'!F35-'NOPAT Bridge'!F22)*(1-'NOPAT Bridge'!F$38)</f>
+        <f>('NOPAT Bridge'!F36-'NOPAT Bridge'!F23)*(1-'NOPAT Bridge'!F$39)</f>
         <v/>
       </c>
       <c r="G76" s="74">
-        <f>('NOPAT Bridge'!G35-'NOPAT Bridge'!G22)*(1-'NOPAT Bridge'!G$38)</f>
+        <f>('NOPAT Bridge'!G36-'NOPAT Bridge'!G23)*(1-'NOPAT Bridge'!G$39)</f>
         <v/>
       </c>
       <c r="H76" s="74">
-        <f>('NOPAT Bridge'!H35-'NOPAT Bridge'!H22)*(1-'NOPAT Bridge'!H$38)</f>
+        <f>('NOPAT Bridge'!H36-'NOPAT Bridge'!H23)*(1-'NOPAT Bridge'!H$39)</f>
         <v/>
       </c>
       <c r="I76" s="74">
-        <f>('NOPAT Bridge'!I35-'NOPAT Bridge'!I22)*(1-'NOPAT Bridge'!I$38)</f>
+        <f>('NOPAT Bridge'!I36-'NOPAT Bridge'!I23)*(1-'NOPAT Bridge'!I$39)</f>
         <v/>
       </c>
       <c r="J76" s="74">
-        <f>('NOPAT Bridge'!J35-'NOPAT Bridge'!J22)*(1-'NOPAT Bridge'!J$38)</f>
+        <f>('NOPAT Bridge'!J36-'NOPAT Bridge'!J23)*(1-'NOPAT Bridge'!J$39)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Option A: link 3-statement assumptions to Scenarios col G
- Add scenario_links.py with Scenarios Base mirror sheet and row map
- Wire Assumptions red inputs (rev growth, GM, margin path, tax, capex/D&A)
  to DCF Scenarios column G via local mirror; derive SG&A from clean OM path
- Extend pitch_values.py to export all FY26-30 IS/BS/CF lines
- Refactor build_pitch.py with pitch_financial_slide() helper and GIS footnote
- Add recalc_workbook.py for headless LibreOffice recalc with mirror sync

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -11121,7 +11121,7 @@
       </c>
       <c r="D98" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
+          <t>WACC tab → green WACC cell ~9.0%. Sensitivity WACC axis brackets base ±100bps.</t>
         </is>
       </c>
       <c r="F98" s="109">
@@ -11156,7 +11156,7 @@
       </c>
       <c r="D99" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
+          <t>WACC tab → green WACC cell ~9.0%. Sensitivity WACC axis brackets base ±100bps.</t>
         </is>
       </c>
       <c r="F99" s="109">
@@ -11191,7 +11191,7 @@
       </c>
       <c r="D100" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
+          <t>WACC tab → green WACC cell ~9.0%. Sensitivity WACC axis brackets base ±100bps.</t>
         </is>
       </c>
       <c r="F100" s="109">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="D101" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
+          <t>WACC tab → green WACC cell ~9.0%. Sensitivity WACC axis brackets base ±100bps.</t>
         </is>
       </c>
       <c r="F101" s="109">
@@ -11261,7 +11261,7 @@
       </c>
       <c r="D102" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "4.23%" (2025 implied ERP). Sensitivity WACC axis brackets the 10.5% base.</t>
+          <t>WACC tab → green WACC cell ~9.0%. Sensitivity WACC axis brackets base ±100bps.</t>
         </is>
       </c>
       <c r="F102" s="109">
@@ -12254,7 +12254,7 @@
     <row r="49">
       <c r="A49" s="41" t="inlineStr">
         <is>
-          <t>•  At base WACC 10.5% and g 2.25% that identity is ~6.0x — the stale “Gordon ~7x / pick Deckers 8.0x” overlay is gone</t>
+          <t>•  At base WACC ~9.0% and g 2.25% that identity is ~7.4x FY30 EBITDA — not a peer average</t>
         </is>
       </c>
     </row>
@@ -12282,7 +12282,7 @@
     <row r="53">
       <c r="A53" s="41" t="inlineStr">
         <is>
-          <t>•  PitchBook LULU is ~4.7x TTM. Gordon 6.0x is a partial recovery, not a re-rate to WSM ~15x</t>
+          <t>•  PitchBook LULU is ~4.7x TTM. Gordon ~7.4x is a partial recovery, not a re-rate to WSM ~15x</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix buyback-linked EPS on 3-statement slides and align to $500M/yr
- Correct Scenarios pitch-bridge EPS (was NI×1000/shares → ~$9,777)
- Add diluted shares row with $500M/yr retirement at repurchase price path
- Recompute forecast EPS via align_buyback_eps (FY30 $12.93 diluted)
- Update IS/BS/CF slide footnotes; sync Risk/Timeline narrative EPS

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>Funded term debt $0 — 10-K: no borrowings outstanding on the revolver. Leases are the only debt equivalent here.</t>
+          <t>Funded term debt $0; 10-K: no borrowings outstanding on the revolver. Leases are the only debt equivalent here.</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>Yahoo Beta (5Y Monthly) = 0.86. Levered equity βL from ~60 monthly returns vs S&amp;P 500 — not unlevered.</t>
+          <t>Yahoo Beta (5Y Monthly) = 0.86. Levered equity βL from ~60 monthly returns vs S&amp;P 500; not unlevered.</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>Yahoo Total Debt/Equity (mrq) = 44.69% is book D/E on the same page — shown for reference, not used in Hamada.</t>
+          <t>Yahoo Total Debt/Equity (mrq) = 44.69% is book D/E on the same page; shown for reference, not used in Hamada.</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
@@ -1666,7 +1666,7 @@
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Total Debt/Equity (mrq)" → 44.69%. Book D/E — reference only, not in Hamada.</t>
+          <t>Ctrl+F "Total Debt/Equity (mrq)" → 44.69%. Book D/E; reference only, not in Hamada.</t>
         </is>
       </c>
       <c r="E21" s="27" t="n">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>Relever D/E = FY25 10-K lease debt ÷ our market cap ≈ 0.16 — WACC capital structure we model.</t>
+          <t>Relever D/E = FY25 10-K lease debt ÷ our market cap ≈ 0.16; WACC capital structure we model.</t>
         </is>
       </c>
       <c r="C23" s="24" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>Benchmark only: Damodaran unlevered Retail (Special Lines) βu = 0.95. Not used — we derive βu from Yahoo βL.</t>
+          <t>Benchmark only: Damodaran unlevered Retail (Special Lines) βu = 0.95. Not used; we derive βu from Yahoo βL.</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "Retail (Special Lines)" → 0.95 βu. Sector benchmark — not used in WACC.</t>
+          <t>Ctrl+F "Retail (Special Lines)" → 0.95 βu. Sector benchmark; not used in WACC.</t>
         </is>
       </c>
       <c r="E24" s="27" t="n">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>YAHOO KEY STATISTICS — βL + debt + equity on ONE page
+          <t>YAHOO KEY STATISTICS; βL + debt + equity on ONE page
 (No vendor publishes the D/E embedded inside the regression.)
 Observed levered βL
   Ctrl+F "Beta (5Y Monthly)"  →  0.86
@@ -1930,7 +1930,7 @@
       </c>
       <c r="B40" s="17" t="inlineStr">
         <is>
-          <t>Debt weight = lease liabilities ÷ (market cap + lease debt). ~14% — ASC 842 leases, not bank debt.</t>
+          <t>Debt weight = lease liabilities ÷ (market cap + lease debt). ~14%; ASC 842 leases, not bank debt.</t>
         </is>
       </c>
       <c r="C40" s="18" t="inlineStr">
@@ -1987,7 +1987,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Add back $134.5M in FY26 only — already recognized (reduced COGS). +130bps on FY26 sales, not +560bps (that was Q2-only).</t>
+          <t>Add back $134.5M in FY26 only; already recognized (reduced COGS). +130bps on FY26 sales, not +560bps (that was Q2-only).</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — DSO (days), flat ~6.3. Mostly own stores/DTC (cash at register); AR is small wholesale residual — predictable ~6 days FY22–25.</t>
+          <t>Not % of revenue; DSO (days), flat ~6.3. Mostly own stores/DTC (cash at register); AR is small wholesale residual; predictable ~6 days FY22–25.</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
@@ -2431,9 +2431,9 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue — DSO (days), flat ~6.3.
+          <t>Not % of revenue; DSO (days), flat ~6.3.
 Why flat: ~90%+ revenue is company-operated stores + e-commerce (cash/card at sale);
-AR is a small, stable wholesale/license residual — predictable collection, not trade credit.
+AR is a small, stable wholesale/license residual; predictable collection, not trade credit.
 Ctrl+F "Accounts receivable, net"
 → 190,657 ($000)
 Ctrl+F "Net revenue"
@@ -2461,7 +2461,7 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — DIO (days).
+          <t>Not % of revenue; DIO (days).
 FY25 anchor: DIO = (Inventories ÷ COGS) × 365
   = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days (FY24 inv: 1,442,081).
 Forecast path: DIO_t = FY25 DIO − (1 day × year t); flat across scenarios.</t>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue — DIO (days).
+          <t>Not % of revenue; DIO (days).
 FY25 anchor formula:
   DIO = (Inventories ÷ COGS) × 365
 Ctrl+F "Inventories"
@@ -2503,7 +2503,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — subtract 1 DIO day per forecast year (−5 days FY26–30).
+          <t>Not % of revenue; subtract 1 DIO day per forecast year (−5 days FY26–30).
 Feeds Inventories = (DIO_t ÷ 365) × COGS_t.
 Ctrl+F "reduce the percentage of markdowns"
 Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
@@ -2516,7 +2516,7 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue — DIO −1 day/yr (−5 days FY26–30).
+          <t>Not % of revenue; DIO −1 day/yr (−5 days FY26–30).
 Feeds Inventories_t = (DIO_t ÷ 365) × COGS_t.
 Ctrl+F "reduce the percentage of markdowns"
 Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
@@ -2540,7 +2540,7 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — DPO (days), flat ~25.1. Implied AP ≈3.0% of sales / 6.9% of COGS.</t>
+          <t>Not % of revenue; DPO (days), flat ~25.1. Implied AP ≈3.0% of sales / 6.9% of COGS.</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
@@ -2554,7 +2554,7 @@
 → 331,421 ($000)
 Ctrl+F "Cost of goods sold"
 → 4,818,468 ($000)
-Not % of revenue — DPO ≈ 25.1 days. Implied AP ≈ 3.0% of sales / 6.9% of COGS.</t>
+Not % of revenue; DPO ≈ 25.1 days. Implied AP ≈ 3.0% of sales / 6.9% of COGS.</t>
         </is>
       </c>
       <c r="F18" s="39" t="n">
@@ -5585,100 +5585,195 @@
     <row r="183">
       <c r="A183" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted EPS ($) – year 1</t>
-        </is>
-      </c>
-      <c r="F183" s="49">
-        <f>F143*1000/111380</f>
-        <v/>
-      </c>
-      <c r="G183" s="49">
-        <f>G143*1000/111380</f>
-        <v/>
-      </c>
-      <c r="H183" s="49">
-        <f>H143*1000/111380</f>
+          <t xml:space="preserve">  Diluted shares (000) – year 1</t>
+        </is>
+      </c>
+      <c r="F183" s="42">
+        <f>119068-F21/100</f>
+        <v/>
+      </c>
+      <c r="G183" s="42">
+        <f>119068-G21/100</f>
+        <v/>
+      </c>
+      <c r="H183" s="42">
+        <f>119068-ROUND(H22*H153,0)/100</f>
         <v/>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted EPS ($) – year 2</t>
-        </is>
-      </c>
-      <c r="F184" s="49">
-        <f>F144*1000/111380</f>
-        <v/>
-      </c>
-      <c r="G184" s="49">
-        <f>G144*1000/111380</f>
-        <v/>
-      </c>
-      <c r="H184" s="49">
-        <f>H144*1000/111380</f>
+          <t xml:space="preserve">  Diluted shares (000) – year 2</t>
+        </is>
+      </c>
+      <c r="F184" s="42">
+        <f>F183-F21/108</f>
+        <v/>
+      </c>
+      <c r="G184" s="42">
+        <f>G183-G21/108</f>
+        <v/>
+      </c>
+      <c r="H184" s="42">
+        <f>H183-ROUND(H22*H154,0)/108</f>
         <v/>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted EPS ($) – year 3</t>
-        </is>
-      </c>
-      <c r="F185" s="49">
-        <f>F145*1000/111380</f>
-        <v/>
-      </c>
-      <c r="G185" s="49">
-        <f>G145*1000/111380</f>
-        <v/>
-      </c>
-      <c r="H185" s="49">
-        <f>H145*1000/111380</f>
+          <t xml:space="preserve">  Diluted shares (000) – year 3</t>
+        </is>
+      </c>
+      <c r="F185" s="42">
+        <f>F184-F21/115</f>
+        <v/>
+      </c>
+      <c r="G185" s="42">
+        <f>G184-G21/115</f>
+        <v/>
+      </c>
+      <c r="H185" s="42">
+        <f>H184-ROUND(H22*H155,0)/115</f>
         <v/>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Diluted EPS ($) – year 4</t>
-        </is>
-      </c>
-      <c r="F186" s="49">
-        <f>F146*1000/111380</f>
-        <v/>
-      </c>
-      <c r="G186" s="49">
-        <f>G146*1000/111380</f>
-        <v/>
-      </c>
-      <c r="H186" s="49">
-        <f>H146*1000/111380</f>
+          <t xml:space="preserve">  Diluted shares (000) – year 4</t>
+        </is>
+      </c>
+      <c r="F186" s="42">
+        <f>F185-F21/122</f>
+        <v/>
+      </c>
+      <c r="G186" s="42">
+        <f>G185-G21/122</f>
+        <v/>
+      </c>
+      <c r="H186" s="42">
+        <f>H185-ROUND(H22*H156,0)/122</f>
         <v/>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="41" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Diluted shares (000) – year 5</t>
+        </is>
+      </c>
+      <c r="F187" s="42">
+        <f>F186-F21/130</f>
+        <v/>
+      </c>
+      <c r="G187" s="42">
+        <f>G186-G21/130</f>
+        <v/>
+      </c>
+      <c r="H187" s="42">
+        <f>H186-ROUND(H22*H157,0)/130</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Diluted EPS ($) – year 1</t>
+        </is>
+      </c>
+      <c r="F188" s="49">
+        <f>F143/F183</f>
+        <v/>
+      </c>
+      <c r="G188" s="49">
+        <f>G143/G183</f>
+        <v/>
+      </c>
+      <c r="H188" s="49">
+        <f>H143/H183</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Diluted EPS ($) – year 2</t>
+        </is>
+      </c>
+      <c r="F189" s="49">
+        <f>F144/F184</f>
+        <v/>
+      </c>
+      <c r="G189" s="49">
+        <f>G144/G184</f>
+        <v/>
+      </c>
+      <c r="H189" s="49">
+        <f>H144/H184</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Diluted EPS ($) – year 3</t>
+        </is>
+      </c>
+      <c r="F190" s="49">
+        <f>F145/F185</f>
+        <v/>
+      </c>
+      <c r="G190" s="49">
+        <f>G145/G185</f>
+        <v/>
+      </c>
+      <c r="H190" s="49">
+        <f>H145/H185</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Diluted EPS ($) – year 4</t>
+        </is>
+      </c>
+      <c r="F191" s="49">
+        <f>F146/F186</f>
+        <v/>
+      </c>
+      <c r="G191" s="49">
+        <f>G146/G186</f>
+        <v/>
+      </c>
+      <c r="H191" s="49">
+        <f>H146/H186</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="41" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Diluted EPS ($) – year 5</t>
         </is>
       </c>
-      <c r="F187" s="49">
-        <f>F147*1000/111380</f>
-        <v/>
-      </c>
-      <c r="G187" s="49">
-        <f>G147*1000/111380</f>
-        <v/>
-      </c>
-      <c r="H187" s="49">
-        <f>H147*1000/111380</f>
-        <v/>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" s="26" t="inlineStr">
+      <c r="F192" s="49">
+        <f>F147/F187</f>
+        <v/>
+      </c>
+      <c r="G192" s="49">
+        <f>G147/G187</f>
+        <v/>
+      </c>
+      <c r="H192" s="49">
+        <f>H147/H187</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  memo: pitch deck pulls cols G (base) &amp; H (bull) from this block via pitch_values.py</t>
         </is>
@@ -5883,7 +5978,7 @@
       </c>
       <c r="I6" s="59" t="inlineStr">
         <is>
-          <t>prior-year ending stores. Same count, new column — that's where the year starts.</t>
+          <t>prior-year ending stores. Same count, new column; that's where the year starts.</t>
         </is>
       </c>
       <c r="J6" s="17" t="inlineStr">
@@ -5977,7 +6072,7 @@
       </c>
       <c r="L8" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "lease" / store fleet — immaterial closures vs expansion; 2–3 per mature region.</t>
+          <t>Ctrl+F "lease" / store fleet; immaterial closures vs expansion; 2–3 per mature region.</t>
         </is>
       </c>
     </row>
@@ -6017,7 +6112,7 @@
       </c>
       <c r="I9" s="59" t="inlineStr">
         <is>
-          <t>beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
+          <t>beginning stores + openings − closures. Roll-forward; nothing fancy, just how many doors you end with.</t>
         </is>
       </c>
       <c r="J9" s="17" t="inlineStr">
@@ -6067,7 +6162,7 @@
       </c>
       <c r="I10" s="59" t="inlineStr">
         <is>
-          <t>prior-year ending stores. Same count, new column — that's where the year starts.</t>
+          <t>prior-year ending stores. Same count, new column; that's where the year starts.</t>
         </is>
       </c>
       <c r="J10" s="17" t="inlineStr">
@@ -6161,7 +6256,7 @@
       </c>
       <c r="L12" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "lease" / store fleet — immaterial closures vs expansion; 2–3 per mature region.</t>
+          <t>Ctrl+F "lease" / store fleet; immaterial closures vs expansion; 2–3 per mature region.</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6296,7 @@
       </c>
       <c r="I13" s="59" t="inlineStr">
         <is>
-          <t>beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
+          <t>beginning stores + openings − closures. Roll-forward; nothing fancy, just how many doors you end with.</t>
         </is>
       </c>
       <c r="J13" s="17" t="inlineStr">
@@ -6251,7 +6346,7 @@
       </c>
       <c r="I14" s="59" t="inlineStr">
         <is>
-          <t>prior-year ending stores. Same count, new column — that's where the year starts.</t>
+          <t>prior-year ending stores. Same count, new column; that's where the year starts.</t>
         </is>
       </c>
       <c r="J14" s="17" t="inlineStr">
@@ -6345,7 +6440,7 @@
       </c>
       <c r="L16" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+F "lease" / store fleet — immaterial closures vs expansion; 2–3 per mature region.</t>
+          <t>Ctrl+F "lease" / store fleet; immaterial closures vs expansion; 2–3 per mature region.</t>
         </is>
       </c>
     </row>
@@ -6385,7 +6480,7 @@
       </c>
       <c r="I17" s="59" t="inlineStr">
         <is>
-          <t>beginning stores + openings − closures. Roll-forward — nothing fancy, just how many doors you end with.</t>
+          <t>beginning stores + openings − closures. Roll-forward; nothing fancy, just how many doors you end with.</t>
         </is>
       </c>
       <c r="J17" s="17" t="inlineStr">
@@ -6825,12 +6920,12 @@
       </c>
       <c r="I28" s="59" t="inlineStr">
         <is>
-          <t>prior column's total store-channel revenue. Base you're applying comps to — not new-store contribution.</t>
+          <t>prior column's total store-channel revenue. Base you're applying comps to; not new-store contribution.</t>
         </is>
       </c>
       <c r="J28" s="17" t="inlineStr">
         <is>
-          <t>Last year's total store-channel revenue — the base you're growing comps off of, not the new boxes.</t>
+          <t>Last year's total store-channel revenue; the base you're growing comps off of, not the new boxes.</t>
         </is>
       </c>
       <c r="K28" s="24" t="inlineStr">
@@ -6870,12 +6965,12 @@
       </c>
       <c r="I29" s="59" t="inlineStr">
         <is>
-          <t>prior store rev×(71%×(1+Am comp)+16%×(1+China)+13%×(1+RoW)). Existing base only — new stores are on the next row.</t>
+          <t>prior store rev×(71%×(1+Am comp)+16%×(1+China)+13%×(1+RoW)). Existing base only; new stores are on the next row.</t>
         </is>
       </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
-          <t>Existing-store sales only — prior store rev grown by geo comp %. New doors are a separate line, not in here.</t>
+          <t>Existing-store sales only; prior store rev grown by geo comp %. New doors are a separate line, not in here.</t>
         </is>
       </c>
       <c r="K29" s="24" t="inlineStr">
@@ -6915,7 +7010,7 @@
       </c>
       <c r="I30" s="59" t="inlineStr">
         <is>
-          <t>(open−close each geo)×sq ft×$/sq ft → raw annual $. /1000 flips that to $000 (this whole tab is thousands). ×0.55 = year-one haircut — new boxes don't run at full SPSF yet. FY27 ex: (D7−D8+D11−D12+D15−D16)×D19×D24/1000×0.55.</t>
+          <t>(open−close each geo)×sq ft×$/sq ft → raw annual $. /1000 flips that to $000 (this whole tab is thousands). ×0.55 = year-one haircut; new boxes don't run at full SPSF yet. FY27 ex: (D7−D8+D11−D12+D15−D16)×D19×D24/1000×0.55.</t>
         </is>
       </c>
       <c r="J30" s="17" t="inlineStr">
@@ -7005,7 +7100,7 @@
       </c>
       <c r="J32" s="17" t="inlineStr">
         <is>
-          <t>Fleet traffic memo line — not a separate FCF item. Calibrated to FY25 store productivity commentary.</t>
+          <t>Fleet traffic memo line; not a separate FCF item. Calibrated to FY25 store productivity commentary.</t>
         </is>
       </c>
       <c r="K32" s="18" t="inlineStr">
@@ -7045,7 +7140,7 @@
       </c>
       <c r="J33" s="17" t="inlineStr">
         <is>
-          <t>In-store conversion memo — 10-K cites lower conversion in Americas; FY26 27% improving to 29%.</t>
+          <t>In-store conversion memo; 10-K cites lower conversion in Americas; FY26 27% improving to 29%.</t>
         </is>
       </c>
       <c r="K33" s="18" t="inlineStr">
@@ -7443,7 +7538,7 @@
       </c>
       <c r="I45" s="59" t="inlineStr">
         <is>
-          <t>prior other-channel rev × (1 + growth %). Wholesale/license/outlets — grown off last year.</t>
+          <t>prior other-channel rev × (1 + growth %). Wholesale/license/outlets; grown off last year.</t>
         </is>
       </c>
       <c r="J45" s="17" t="inlineStr">
@@ -7562,7 +7657,7 @@
       </c>
       <c r="J47" s="17" t="inlineStr">
         <is>
-          <t>China 15.8% of FY25 revenue; fastest comp and store growth — expansion market in the driver schedule.</t>
+          <t>China 15.8% of FY25 revenue; fastest comp and store growth; expansion market in the driver schedule.</t>
         </is>
       </c>
       <c r="K47" s="18" t="inlineStr">
@@ -7898,12 +7993,12 @@
       </c>
       <c r="I56" s="59" t="inlineStr">
         <is>
-          <t>Scenarios! base-case revenue. DCF still runs off this path — not the driver total.</t>
+          <t>Scenarios! base-case revenue. DCF still runs off this path; not the driver total.</t>
         </is>
       </c>
       <c r="J56" s="17" t="inlineStr">
         <is>
-          <t>Pulls the Scenarios base-case revenue path — that's still the number the DCF actually uses, not the driver total.</t>
+          <t>Pulls the Scenarios base-case revenue path; that's still the number the DCF actually uses, not the driver total.</t>
         </is>
       </c>
       <c r="K56" s="18" t="inlineStr">
@@ -8166,9 +8261,9 @@
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — SBC add-back flag. Set to 0 (Convention A).
+          <t>Not % of revenue; SBC add-back flag. Set to 0 (Convention A).
 SBC stays inside Scenarios EBIT/NOPAT as a real economic cost; DCF uses basic shares (111.4M).
-FY25 reference: $62,203k (10-K). Flag = 1 would add back (Convention B + diluted shares) — not used.</t>
+FY25 reference: $62,203k (10-K). Flag = 1 would add back (Convention B + diluted shares); not used.</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
@@ -8216,7 +8311,7 @@
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>Not % of consolidated revenue — EBIT as % of store-channel revenue only (not the Scenarios 13.2%–15.5% consolidated margin).
+          <t>Not % of consolidated revenue; EBIT as % of store-channel revenue only (not the Scenarios 13.2%–15.5% consolidated margin).
 18.6% margin assumption.
 EBIT_store = Rev_store × Margin_store
 FY25 check: 5,049,744 × 18.6% ≈ 939,252 ($000).
@@ -8230,7 +8325,7 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Not consolidated EBIT margin — EBIT ÷ store revenue only (cf. Scenarios 13.2%–15.5%).
+          <t>Not consolidated EBIT margin; EBIT ÷ store revenue only (cf. Scenarios 13.2%–15.5%).
 Ctrl+F "Company-operated stores"
 → 5,049,744 ($000) net revenue
 × 18.6% margin assumption → store EBIT ≈ 939,252 ($000)</t>
@@ -8263,11 +8358,11 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>Not % of consolidated revenue — EBIT as % of e-commerce revenue only (not the Scenarios 13.2%–15.5% consolidated margin).
+          <t>Not % of consolidated revenue; EBIT as % of e-commerce revenue only (not the Scenarios 13.2%–15.5% consolidated margin).
 23.6% margin assumption.
 EBIT_e-comm = Rev_e-comm × Margin_e-comm
 FY25 check: 4,918,697 × 23.6% ≈ 1,160,812 ($000).
-Higher than stores — no occupancy; fulfillment + digital marketing only.</t>
+Higher than stores; no occupancy; fulfillment + digital marketing only.</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
@@ -8277,7 +8372,7 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Not consolidated EBIT margin — EBIT ÷ e-commerce revenue only (cf. Scenarios 13.2%–15.5%).
+          <t>Not consolidated EBIT margin; EBIT ÷ e-commerce revenue only (cf. Scenarios 13.2%–15.5%).
 Ctrl+F "E-commerce"
 → 4,918,697 ($000) net revenue
 × 23.6% margin assumption → e-comm EBIT ≈ 1,160,812 ($000)</t>
@@ -8310,11 +8405,11 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>Not % of consolidated revenue — EBIT as % of other-channel revenue only (not the Scenarios 13.2%–15.5% consolidated margin).
+          <t>Not % of consolidated revenue; EBIT as % of other-channel revenue only (not the Scenarios 13.2%–15.5% consolidated margin).
 9.1% margin assumption.
 EBIT_other = Rev_other × Margin_other
 FY25 check: 1,134,159 × 9.1% ≈ 103,209 ($000).
-Wholesale/license/outlets — lower-margin residual channel.</t>
+Wholesale/license/outlets; lower-margin residual channel.</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
@@ -8324,7 +8419,7 @@
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Not consolidated EBIT margin — EBIT ÷ other-channel revenue only (cf. Scenarios 13.2%–15.5%).
+          <t>Not consolidated EBIT margin; EBIT ÷ other-channel revenue only (cf. Scenarios 13.2%–15.5%).
 Ctrl+F "Net revenue" → 11,102,600
 Minus stores + e-comm → other channels ≈ 1,134,159 ($000)
 × 9.1% margin assumption → other EBIT ≈ 103,209 ($000)</t>
@@ -8397,7 +8492,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — amortization period (years) if R&amp;D/software is capitalized. LULU: no separate R&amp;D cap.</t>
+          <t>Not % of revenue; amortization period (years) if R&amp;D/software is capitalized. LULU: no separate R&amp;D cap.</t>
         </is>
       </c>
       <c r="C13" s="24" t="inlineStr">
@@ -8579,7 +8674,7 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>One-off legal/M&amp;A fees in SG&amp;A — none identified FY25.</t>
+          <t>One-off legal/M&amp;A fees in SG&amp;A; none identified FY25.</t>
         </is>
       </c>
       <c r="E19" s="74" t="n">
@@ -8609,9 +8704,9 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — SBC add-back flag. Set to 0 (Convention A).
+          <t>Not % of revenue; SBC add-back flag. Set to 0 (Convention A).
 SBC stays inside Scenarios EBIT/NOPAT as a real economic cost; DCF uses basic shares (111.4M).
-FY25 reference: $62,203k (10-K). Flag = 1 would add back (Convention B + diluted shares) — not used.</t>
+FY25 reference: $62,203k (10-K). Flag = 1 would add back (Convention B + diluted shares); not used.</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
@@ -8706,7 +8801,7 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — implied lease interest ($1,028k FY25). Reclass from rent to unlevered EBIT; scales with revenue in forecast.</t>
+          <t>Not % of revenue; implied lease interest ($1,028k FY25). Reclass from rent to unlevered EBIT; scales with revenue in forecast.</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
@@ -8752,7 +8847,7 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>Capitalize multi-year software/R&amp;D. LULU: immaterial separate R&amp;D line — held at $0.</t>
+          <t>Capitalize multi-year software/R&amp;D. LULU: immaterial separate R&amp;D line; held at $0.</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
@@ -8762,7 +8857,7 @@
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>R&amp;D / software capitalization — LULU immaterial; held at $0.</t>
+          <t>R&amp;D / software capitalization; LULU immaterial; held at $0.</t>
         </is>
       </c>
       <c r="E24" s="74" t="n">
@@ -8802,7 +8897,7 @@
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Amortization of prior capitalized intangibles — netted in D&amp;A line.</t>
+          <t>Amortization of prior capitalized intangibles; netted in D&amp;A line.</t>
         </is>
       </c>
       <c r="E25" s="74" t="n">
@@ -8880,7 +8975,7 @@
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — store-channel revenue from Revenue Drivers tab.</t>
+          <t>Not % of revenue; store-channel revenue from Revenue Drivers tab.</t>
         </is>
       </c>
       <c r="C28" s="18" t="inlineStr">
@@ -8925,7 +9020,7 @@
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — e-commerce revenue from Revenue Drivers tab.</t>
+          <t>Not % of revenue; e-commerce revenue from Revenue Drivers tab.</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
@@ -8970,7 +9065,7 @@
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — wholesale/license/outlet revenue from Revenue Drivers tab.</t>
+          <t>Not % of revenue; wholesale/license/outlet revenue from Revenue Drivers tab.</t>
         </is>
       </c>
       <c r="C30" s="18" t="inlineStr">
@@ -9015,7 +9110,7 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>Not % of consolidated revenue — store EBIT ÷ store revenue only (not Scenarios consolidated EBIT margin).
+          <t>Not % of consolidated revenue; store EBIT ÷ store revenue only (not Scenarios consolidated EBIT margin).
 EBIT_store,t = Rev_store,t × 18.6%
 FY25: 5,049,744 × 18.6% ≈ 939,252 ($000).
 Margin from driver assumptions row above; ties to 10-K store revenue.</t>
@@ -9028,7 +9123,7 @@
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Not consolidated EBIT margin — store EBIT ÷ store revenue only.
+          <t>Not consolidated EBIT margin; store EBIT ÷ store revenue only.
 Ctrl+F "Company-operated stores"
 → 5,049,744 ($000)
 EBIT = Rev × 18.6% → ≈ 939,252 ($000)</t>
@@ -9066,10 +9161,10 @@
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>Not % of consolidated revenue — e-commerce EBIT ÷ e-commerce revenue only (not Scenarios consolidated EBIT margin).
+          <t>Not % of consolidated revenue; e-commerce EBIT ÷ e-commerce revenue only (not Scenarios consolidated EBIT margin).
 EBIT_e-comm,t = Rev_e-comm,t × 23.6%
 FY25: 4,918,697 × 23.6% ≈ 1,160,812 ($000).
-Higher than stores — no brick-and-mortar occupancy drag.</t>
+Higher than stores; no brick-and-mortar occupancy drag.</t>
         </is>
       </c>
       <c r="C32" s="18" t="inlineStr">
@@ -9079,7 +9174,7 @@
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>Not consolidated EBIT margin — e-commerce EBIT ÷ e-commerce revenue only.
+          <t>Not consolidated EBIT margin; e-commerce EBIT ÷ e-commerce revenue only.
 Ctrl+F "E-commerce"
 → 4,918,697 ($000)
 EBIT = Rev × 23.6% → ≈ 1,160,812 ($000)</t>
@@ -9117,10 +9212,10 @@
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>Not % of consolidated revenue — other-channel EBIT ÷ other revenue only (not Scenarios consolidated EBIT margin).
+          <t>Not % of consolidated revenue; other-channel EBIT ÷ other revenue only (not Scenarios consolidated EBIT margin).
 EBIT_other,t = Rev_other,t × 9.1%
 FY25: 1,134,159 × 9.1% ≈ 103,209 ($000).
-Wholesale/license/outlets — lowest channel margin.</t>
+Wholesale/license/outlets; lowest channel margin.</t>
         </is>
       </c>
       <c r="C33" s="18" t="inlineStr">
@@ -9130,7 +9225,7 @@
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Not consolidated EBIT margin — other-channel EBIT ÷ other revenue only.
+          <t>Not consolidated EBIT margin; other-channel EBIT ÷ other revenue only.
 Other rev = 11,102,600 − 5,049,744 − 4,918,697 ≈ 1,134,159 ($000)
 EBIT = Rev × 9.1% → ≈ 103,209 ($000)</t>
         </is>
@@ -9252,7 +9347,7 @@
       </c>
       <c r="B36" s="17" t="inlineStr">
         <is>
-          <t>FY25: Phases 1–2 walk-through (SBC not added back; flag = 0). Forecast: Scenarios base EBIT — tax base for NOPAT.</t>
+          <t>FY25: Phases 1–2 walk-through (SBC not added back; flag = 0). Forecast: Scenarios base EBIT; tax base for NOPAT.</t>
         </is>
       </c>
       <c r="C36" s="24" t="inlineStr">
@@ -9390,7 +9485,7 @@
       </c>
       <c r="D40" s="19" t="inlineStr">
         <is>
-          <t>Normalized EBIT × t_operating — unlevered tax (no debt shield).</t>
+          <t>Normalized EBIT × t_operating; unlevered tax (no debt shield).</t>
         </is>
       </c>
       <c r="F40" s="75">
@@ -9706,7 +9801,7 @@
     <outlinePr applyStyles="1" summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M103"/>
+  <dimension ref="A1:M104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -10065,7 +10160,7 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>Add back $134.5M in FY26 only — already recognized (reduced COGS). +130bps on FY26 sales, not +560bps (that was Q2-only).</t>
+          <t>Add back $134.5M in FY26 only; already recognized (reduced COGS). +130bps on FY26 sales, not +560bps (that was Q2-only).</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
@@ -10394,7 +10489,7 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — DSO (days), flat ~6.3. Mostly own stores/DTC (cash at register); AR is small wholesale residual — predictable ~6 days FY22–25.</t>
+          <t>Not % of revenue; DSO (days), flat ~6.3. Mostly own stores/DTC (cash at register); AR is small wholesale residual; predictable ~6 days FY22–25.</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
@@ -10404,9 +10499,9 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue — DSO (days), flat ~6.3.
+          <t>Not % of revenue; DSO (days), flat ~6.3.
 Why flat: ~90%+ revenue is company-operated stores + e-commerce (cash/card at sale);
-AR is a small, stable wholesale/license residual — predictable collection, not trade credit.
+AR is a small, stable wholesale/license residual; predictable collection, not trade credit.
 Ctrl+F "Accounts receivable, net"
 → 190,657 ($000)
 Ctrl+F "Net revenue"
@@ -10463,7 +10558,7 @@
       <c r="D21" s="19" t="inlineStr">
         <is>
           <t>Implied ~1.7% of revenue (= 190,657 ÷ 11,102,600); not a direct % plug.
-AR_t = (DSO ÷ 365) × Revenue_t. DSO flat because own-store/DTC dominates — AR scales predictably with sales.
+AR_t = (DSO ÷ 365) × Revenue_t. DSO flat because own-store/DTC dominates; AR scales predictably with sales.
 Ctrl+F "Accounts receivable, net"
 → 190,657 ($000)
 Ctrl+F "Net revenue"
@@ -10506,11 +10601,11 @@
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue — DIO (days).
+          <t>Not % of revenue; DIO (days).
 FY25 anchor: DIO = (Inventories ÷ COGS) × 365
   = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days (FY24 inv: 1,442,081).
 Forecast path: DIO_t = FY25 DIO − (1 day × year t); flat across scenarios.
-Also: Not % of revenue — subtract 1 DIO day per forecast year (−5 days FY26–30).
+Also: Not % of revenue; subtract 1 DIO day per forecast year (−5 days FY26–30).
 Feeds Inventories = (DIO_t ÷ 365) × COGS_t.
 Ctrl+F "reduce the percentage of markdowns"
 Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
@@ -10524,7 +10619,7 @@
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue — DIO (days).
+          <t>Not % of revenue; DIO (days).
 FY25 anchor formula:
   DIO = (Inventories ÷ COGS) × 365
 Ctrl+F "Inventories"
@@ -10533,7 +10628,7 @@
 → 4,818,468 ($000)
   = (1,700,753 ÷ 4,818,468) × 365 ≈ 129 days
 Forecast: DIO_t = FY25 DIO − (1 × year t)
-Also: Not % of revenue — DIO −1 day/yr (−5 days FY26–30).
+Also: Not % of revenue; DIO −1 day/yr (−5 days FY26–30).
 Feeds Inventories_t = (DIO_t ÷ 365) × COGS_t.
 Ctrl+F "reduce the percentage of markdowns"
 Ctrl+F "On a unit basis, we expect inventories to slightly decrease"</t>
@@ -10575,7 +10670,7 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — $ balance (not a direct % plug).
+          <t>Not % of revenue; $ balance (not a direct % plug).
 Inventories_t = (DIO_t ÷ 365) × COGS_t
 COGS_t = Revenue_t × (1 − GM%). FY25 check: (129 ÷ 365) × 4,818,468 ≈ 1,700,753.
 Ctrl+F "Inventories"
@@ -10591,7 +10686,7 @@
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue — Inventories_t = (DIO_t ÷ 365) × COGS_t.
+          <t>Not % of revenue; Inventories_t = (DIO_t ÷ 365) × COGS_t.
 COGS_t = Revenue_t × (1 − GM%).
 Ctrl+F "Inventories"
 → 1,700,753 ($000)
@@ -10636,7 +10731,7 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — DPO (days), flat ~25.1. Implied AP ≈3.0% of sales / 6.9% of COGS.</t>
+          <t>Not % of revenue; DPO (days), flat ~25.1. Implied AP ≈3.0% of sales / 6.9% of COGS.</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
@@ -10650,7 +10745,7 @@
 → 331,421 ($000)
 Ctrl+F "Cost of goods sold"
 → 4,818,468 ($000)
-Not % of revenue — DPO ≈ 25.1 days. Implied AP ≈ 3.0% of sales / 6.9% of COGS.</t>
+Not % of revenue; DPO ≈ 25.1 days. Implied AP ≈ 3.0% of sales / 6.9% of COGS.</t>
         </is>
       </c>
       <c r="E24" s="88" t="n">
@@ -10946,7 +11041,7 @@
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>Not one % — sum ≈22.1% of FY25 sales (AR ~1.7% + inventory ~15.3% + prepaids 5.1%).</t>
+          <t>Not one %; sum ≈22.1% of FY25 sales (AR ~1.7% + inventory ~15.3% + prepaids 5.1%).</t>
         </is>
       </c>
       <c r="C30" s="18" t="inlineStr">
@@ -10956,7 +11051,7 @@
       </c>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>Not one % of revenue — sum of line items.
+          <t>Not one % of revenue; sum of line items.
 FY25: AR ~1.7% + inventory ~15.3% + prepaids 5.1% ≈ 22.1% of sales.</t>
         </is>
       </c>
@@ -10993,7 +11088,7 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>Not one % — sum ≈9.0% of FY25 sales (AP ~3.0% + accrued liabilities 6.0%).</t>
+          <t>Not one %; sum ≈9.0% of FY25 sales (AP ~3.0% + accrued liabilities 6.0%).</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
@@ -11003,7 +11098,7 @@
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Not one % of revenue — sum of line items.
+          <t>Not one % of revenue; sum of line items.
 FY25: AP ~3.0% + accrued liabilities 6.0% ≈ 9.0% of sales.</t>
         </is>
       </c>
@@ -11040,7 +11135,7 @@
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>Not one % — net ≈13.2% of FY25 sales ($1,461,096k). COA minus COL; rolls forward each year.</t>
+          <t>Not one %; net ≈13.2% of FY25 sales ($1,461,096k). COA minus COL; rolls forward each year.</t>
         </is>
       </c>
       <c r="C32" s="18" t="inlineStr">
@@ -11050,7 +11145,7 @@
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>Not one % of revenue — net balance.
+          <t>Not one % of revenue; net balance.
 FY25 NWC ≈ 13.2% of sales ($1,461,096k = COA − COL).</t>
         </is>
       </c>
@@ -11090,7 +11185,7 @@
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>Not % of revenue — $ change in NWC year-over-year. Prior-year NWC minus current-year NWC for the FCF bridge.</t>
+          <t>Not % of revenue; $ change in NWC year-over-year. Prior-year NWC minus current-year NWC for the FCF bridge.</t>
         </is>
       </c>
       <c r="C33" s="18" t="inlineStr">
@@ -11100,7 +11195,7 @@
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Not % of revenue — $ change year-over-year.
+          <t>Not % of revenue; $ change year-over-year.
 FY26: revenue −6.1% + DIO −1 day → NWC falls → ΔNWC positive (WC release).
 FY27–30: revenue +2.3%/yr → AR &amp; inventory rebuild → ΔNWC negative (WC build).</t>
         </is>
@@ -11535,29 +11630,29 @@
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
-          <t>FCF allocated to buybacks</t>
-        </is>
-      </c>
-      <c r="E65" s="20" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F65" s="20">
+          <t>Annual repurchase budget ($000) — base case</t>
+        </is>
+      </c>
+      <c r="E65" s="37" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F65" s="37">
         <f>$E$65</f>
         <v/>
       </c>
-      <c r="G65" s="20">
+      <c r="G65" s="37">
         <f>$E$65</f>
         <v/>
       </c>
-      <c r="H65" s="20">
+      <c r="H65" s="37">
         <f>$E$65</f>
         <v/>
       </c>
-      <c r="I65" s="20">
+      <c r="I65" s="37">
         <f>$E$65</f>
         <v/>
       </c>
-      <c r="J65" s="20">
+      <c r="J65" s="37">
         <f>$E$65</f>
         <v/>
       </c>
@@ -11622,521 +11717,513 @@
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
         <is>
-          <t>Available repurchase cash (= UFCF × allocation)</t>
+          <t>Repurchase cash deployed (= fixed budget)</t>
         </is>
       </c>
       <c r="E69" s="75" t="n">
         <v>0</v>
       </c>
       <c r="F69" s="75">
-        <f>F68*F65</f>
+        <f>F65</f>
         <v/>
       </c>
       <c r="G69" s="75">
-        <f>G68*G65</f>
+        <f>G65</f>
         <v/>
       </c>
       <c r="H69" s="75">
-        <f>H68*H65</f>
+        <f>H65</f>
         <v/>
       </c>
       <c r="I69" s="75">
-        <f>I68*I65</f>
+        <f>I65</f>
         <v/>
       </c>
       <c r="J69" s="75">
-        <f>J68*J65</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="16" t="inlineStr">
-        <is>
-          <t>Projected share price ($)</t>
-        </is>
-      </c>
-      <c r="E71" s="99" t="n">
-        <v>100</v>
-      </c>
-      <c r="F71" s="99">
-        <f>E71*(1+$E$66)</f>
-        <v/>
-      </c>
-      <c r="G71" s="99">
-        <f>F71*(1+$E$66)</f>
-        <v/>
-      </c>
-      <c r="H71" s="99">
-        <f>G71*(1+$E$66)</f>
-        <v/>
-      </c>
-      <c r="I71" s="99">
-        <f>H71*(1+$E$66)</f>
-        <v/>
-      </c>
-      <c r="J71" s="99">
-        <f>I71*(1+$E$66)</f>
+        <f>J65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="16" t="inlineStr">
+        <is>
+          <t>Repurchase as % of UFCF (derived)</t>
+        </is>
+      </c>
+      <c r="F70" s="32">
+        <f>F69/F68</f>
+        <v/>
+      </c>
+      <c r="G70" s="32">
+        <f>G69/G68</f>
+        <v/>
+      </c>
+      <c r="H70" s="32">
+        <f>H69/H68</f>
+        <v/>
+      </c>
+      <c r="I70" s="32">
+        <f>I69/I68</f>
+        <v/>
+      </c>
+      <c r="J70" s="32">
+        <f>J69/J68</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
         <is>
-          <t>Shares retired (000)</t>
-        </is>
-      </c>
-      <c r="E72" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="F72" s="75">
-        <f>F69/F71</f>
-        <v/>
-      </c>
-      <c r="G72" s="75">
-        <f>G69/G71</f>
-        <v/>
-      </c>
-      <c r="H72" s="75">
-        <f>H69/H71</f>
-        <v/>
-      </c>
-      <c r="I72" s="75">
-        <f>I69/I71</f>
-        <v/>
-      </c>
-      <c r="J72" s="75">
-        <f>J69/J71</f>
+          <t>Projected share price ($)</t>
+        </is>
+      </c>
+      <c r="E72" s="99" t="n">
+        <v>100</v>
+      </c>
+      <c r="F72" s="99">
+        <f>E72*(1+$E$66)</f>
+        <v/>
+      </c>
+      <c r="G72" s="99">
+        <f>F72*(1+$E$66)</f>
+        <v/>
+      </c>
+      <c r="H72" s="99">
+        <f>G72*(1+$E$66)</f>
+        <v/>
+      </c>
+      <c r="I72" s="99">
+        <f>H72*(1+$E$66)</f>
+        <v/>
+      </c>
+      <c r="J72" s="99">
+        <f>I72*(1+$E$66)</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="16" t="inlineStr">
         <is>
+          <t>Shares retired (000)</t>
+        </is>
+      </c>
+      <c r="E73" s="75" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="75">
+        <f>F69/F72</f>
+        <v/>
+      </c>
+      <c r="G73" s="75">
+        <f>G69/G72</f>
+        <v/>
+      </c>
+      <c r="H73" s="75">
+        <f>H69/H72</f>
+        <v/>
+      </c>
+      <c r="I73" s="75">
+        <f>I69/I72</f>
+        <v/>
+      </c>
+      <c r="J73" s="75">
+        <f>J69/J72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="16" t="inlineStr">
+        <is>
           <t>Beginning shares (000)</t>
         </is>
       </c>
-      <c r="E73" s="22" t="n">
+      <c r="E74" s="22" t="n">
         <v>111380</v>
       </c>
-      <c r="F73" s="75">
-        <f>$E$73</f>
-        <v/>
-      </c>
-      <c r="G73" s="75">
-        <f>F74</f>
-        <v/>
-      </c>
-      <c r="H73" s="75">
-        <f>G74</f>
-        <v/>
-      </c>
-      <c r="I73" s="75">
-        <f>H74</f>
-        <v/>
-      </c>
-      <c r="J73" s="75">
-        <f>I74</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="23" t="inlineStr">
+      <c r="F74" s="75">
+        <f>$E$74</f>
+        <v/>
+      </c>
+      <c r="G74" s="75">
+        <f>F75</f>
+        <v/>
+      </c>
+      <c r="H74" s="75">
+        <f>G75</f>
+        <v/>
+      </c>
+      <c r="I74" s="75">
+        <f>H75</f>
+        <v/>
+      </c>
+      <c r="J74" s="75">
+        <f>I75</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="23" t="inlineStr">
         <is>
           <t>Ending shares (000)</t>
         </is>
       </c>
-      <c r="E74" s="100" t="n">
+      <c r="E75" s="100" t="n">
         <v>111380</v>
       </c>
-      <c r="F74" s="25">
-        <f>F73-F72</f>
-        <v/>
-      </c>
-      <c r="G74" s="25">
-        <f>G73-G72</f>
-        <v/>
-      </c>
-      <c r="H74" s="25">
-        <f>H73-H72</f>
-        <v/>
-      </c>
-      <c r="I74" s="25">
-        <f>I73-I72</f>
-        <v/>
-      </c>
-      <c r="J74" s="25">
-        <f>J73-J72</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="16" t="inlineStr">
+      <c r="F75" s="25">
+        <f>F74-F73</f>
+        <v/>
+      </c>
+      <c r="G75" s="25">
+        <f>G74-G73</f>
+        <v/>
+      </c>
+      <c r="H75" s="25">
+        <f>H74-H73</f>
+        <v/>
+      </c>
+      <c r="I75" s="25">
+        <f>I74-I73</f>
+        <v/>
+      </c>
+      <c r="J75" s="25">
+        <f>J74-J73</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="16" t="inlineStr">
         <is>
           <t>Projected net income ($000)</t>
         </is>
       </c>
-      <c r="E76" s="22" t="n">
+      <c r="E77" s="22" t="n">
         <v>1579183</v>
       </c>
-      <c r="F76" s="75">
+      <c r="F77" s="75">
         <f>('NOPAT Bridge'!F36-'NOPAT Bridge'!F23)*(1-'NOPAT Bridge'!F$39)</f>
         <v/>
       </c>
-      <c r="G76" s="75">
+      <c r="G77" s="75">
         <f>('NOPAT Bridge'!G36-'NOPAT Bridge'!G23)*(1-'NOPAT Bridge'!G$39)</f>
         <v/>
       </c>
-      <c r="H76" s="75">
+      <c r="H77" s="75">
         <f>('NOPAT Bridge'!H36-'NOPAT Bridge'!H23)*(1-'NOPAT Bridge'!H$39)</f>
         <v/>
       </c>
-      <c r="I76" s="75">
+      <c r="I77" s="75">
         <f>('NOPAT Bridge'!I36-'NOPAT Bridge'!I23)*(1-'NOPAT Bridge'!I$39)</f>
         <v/>
       </c>
-      <c r="J76" s="75">
+      <c r="J77" s="75">
         <f>('NOPAT Bridge'!J36-'NOPAT Bridge'!J23)*(1-'NOPAT Bridge'!J$39)</f>
         <v/>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="23" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="23" t="inlineStr">
         <is>
           <t>Accretive EPS ($/share) = Net income ÷ ending shares</t>
         </is>
       </c>
-      <c r="E77" s="101" t="n">
+      <c r="E78" s="101" t="n">
         <v>14.1783354282636</v>
       </c>
-      <c r="F77" s="101">
-        <f>F76/F74</f>
-        <v/>
-      </c>
-      <c r="G77" s="101">
-        <f>G76/G74</f>
-        <v/>
-      </c>
-      <c r="H77" s="101">
-        <f>H76/H74</f>
-        <v/>
-      </c>
-      <c r="I77" s="101">
-        <f>I76/I74</f>
-        <v/>
-      </c>
-      <c r="J77" s="101">
-        <f>J76/J74</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="93" t="inlineStr">
+      <c r="F78" s="101">
+        <f>F77/F75</f>
+        <v/>
+      </c>
+      <c r="G78" s="101">
+        <f>G77/G75</f>
+        <v/>
+      </c>
+      <c r="H78" s="101">
+        <f>H77/H75</f>
+        <v/>
+      </c>
+      <c r="I78" s="101">
+        <f>I77/I75</f>
+        <v/>
+      </c>
+      <c r="J78" s="101">
+        <f>J77/J75</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="93" t="inlineStr">
         <is>
           <t>CROSS-CHECK — EXIT MULTIPLE METHOD</t>
         </is>
       </c>
-      <c r="B79" s="13" t="n"/>
-      <c r="C79" s="13" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="15" t="inlineStr">
+      <c r="B80" s="13" t="n"/>
+      <c r="C80" s="13" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="15" t="inlineStr">
         <is>
           <t>Exit multiple is the Gordon identity — not a peer pick or an average</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="28" customHeight="1">
-      <c r="A81" s="16" t="inlineStr">
+    <row r="82" ht="28" customHeight="1">
+      <c r="A82" s="16" t="inlineStr">
         <is>
           <t>Selected exit EV/EBITDA (Gordon implied)</t>
         </is>
       </c>
-      <c r="B81" s="17" t="inlineStr">
+      <c r="B82" s="17" t="inlineStr">
         <is>
           <t>Selected exit is Gordon TV / FY30 EBITDA. Identity: (UFCF/EBITDA)×(1+g)/(WACC−g). Not Deckers and not a peer average.</t>
         </is>
       </c>
-      <c r="C81" s="18" t="inlineStr">
+      <c r="C82" s="18" t="inlineStr">
         <is>
           <t>DCF: Gordon implied exit (TV / FY30 EBITDA)</t>
         </is>
       </c>
-      <c r="D81" s="19" t="inlineStr">
+      <c r="D82" s="19" t="inlineStr">
         <is>
           <t>No peer Ctrl+F. This cell = Gordon TV / FY30 EBITDA = (UFCF/EBITDA)×(1+g)/(WACC−g). WACC and g are sourced on those rows.</t>
         </is>
       </c>
-      <c r="E81" s="94">
+      <c r="E82" s="94">
         <f>E46</f>
         <v/>
       </c>
-      <c r="M81" s="95" t="inlineStr">
+      <c r="M82" s="95" t="inlineStr">
         <is>
           <t>Comps: Exit Multiple Build</t>
         </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="16" t="inlineStr">
-        <is>
-          <t>Terminal value = Terminal EBITDA × exit multiple</t>
-        </is>
-      </c>
-      <c r="E82" s="75">
-        <f>E44*E81</f>
-        <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="16" t="inlineStr">
         <is>
+          <t>Terminal value = Terminal EBITDA × exit multiple</t>
+        </is>
+      </c>
+      <c r="E83" s="75">
+        <f>E44*E82</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="16" t="inlineStr">
+        <is>
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="E83" s="75">
-        <f>E82/(1+Scenarios!$G$9)^J36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="23" t="inlineStr">
-        <is>
-          <t>Enterprise value (exit method)</t>
-        </is>
-      </c>
-      <c r="E84" s="25">
-        <f>E42+E83</f>
+      <c r="E84" s="75">
+        <f>E83/(1+Scenarios!$G$9)^J36</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="23" t="inlineStr">
         <is>
+          <t>Enterprise value (exit method)</t>
+        </is>
+      </c>
+      <c r="E85" s="25">
+        <f>E42+E84</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="23" t="inlineStr">
+        <is>
           <t>Implied value per share (exit method)</t>
         </is>
       </c>
-      <c r="E85" s="102">
-        <f>(E84+E50+E51)/E55</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="93" t="inlineStr">
+      <c r="E86" s="102">
+        <f>(E85+E50+E51)/E55</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="93" t="inlineStr">
         <is>
           <t>TERMINAL VALUE RECONCILIATION (GORDON vs EXIT MULTIPLE)</t>
         </is>
       </c>
-      <c r="B87" s="13" t="n"/>
-      <c r="C87" s="13" t="n"/>
-      <c r="D87" s="13" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="103" t="inlineStr"/>
-      <c r="B88" s="54" t="inlineStr">
+      <c r="B88" s="13" t="n"/>
+      <c r="C88" s="13" t="n"/>
+      <c r="D88" s="13" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="103" t="inlineStr"/>
+      <c r="B89" s="54" t="inlineStr">
         <is>
           <t>Gordon Growth</t>
         </is>
       </c>
-      <c r="C88" s="54" t="inlineStr">
+      <c r="C89" s="54" t="inlineStr">
         <is>
           <t>Exit Multiple</t>
         </is>
       </c>
-      <c r="D88" s="54" t="inlineStr">
+      <c r="D89" s="54" t="inlineStr">
         <is>
           <t>Variance</t>
         </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="23" t="inlineStr">
-        <is>
-          <t>Terminal value ($)</t>
-        </is>
-      </c>
-      <c r="B89" s="70">
-        <f>E45</f>
-        <v/>
-      </c>
-      <c r="C89" s="70">
-        <f>E82</f>
-        <v/>
-      </c>
-      <c r="D89" s="70">
-        <f>B89-C89</f>
-        <v/>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="23" t="inlineStr">
         <is>
+          <t>Terminal value ($)</t>
+        </is>
+      </c>
+      <c r="B90" s="70">
+        <f>E45</f>
+        <v/>
+      </c>
+      <c r="C90" s="70">
+        <f>E83</f>
+        <v/>
+      </c>
+      <c r="D90" s="70">
+        <f>B90-C90</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="23" t="inlineStr">
+        <is>
           <t>Exit EV/EBITDA (implied vs selected)</t>
         </is>
       </c>
-      <c r="B90" s="104">
+      <c r="B91" s="104">
         <f>E46</f>
         <v/>
       </c>
-      <c r="C90" s="104">
-        <f>E81</f>
-        <v/>
-      </c>
-      <c r="D90" s="104">
-        <f>B90-C90</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="16" t="inlineStr">
+      <c r="C91" s="104">
+        <f>E82</f>
+        <v/>
+      </c>
+      <c r="D91" s="104">
+        <f>B91-C91</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="16" t="inlineStr">
         <is>
           <t>Terminal value variance (%)</t>
         </is>
       </c>
-      <c r="B91" s="32" t="inlineStr"/>
-      <c r="C91" s="32" t="inlineStr"/>
-      <c r="D91" s="32">
-        <f>(B89-C89)/B89</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="23" t="inlineStr">
+      <c r="B92" s="32" t="inlineStr"/>
+      <c r="C92" s="32" t="inlineStr"/>
+      <c r="D92" s="32">
+        <f>(B90-C90)/B90</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="23" t="inlineStr">
         <is>
           <t>Implied share price</t>
         </is>
       </c>
-      <c r="B92" s="105">
+      <c r="B93" s="105">
         <f>E56</f>
         <v/>
       </c>
-      <c r="C92" s="105">
-        <f>E85</f>
-        <v/>
-      </c>
-      <c r="D92" s="105">
-        <f>B92-C92</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="68" t="inlineStr">
+      <c r="C93" s="105">
+        <f>E86</f>
+        <v/>
+      </c>
+      <c r="D93" s="105">
+        <f>B93-C93</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="68" t="inlineStr">
         <is>
           <t>Sanity check: multiples within ±1.5 turns?</t>
         </is>
       </c>
-      <c r="B93" s="106">
-        <f>IF(ABS(D90)&lt;=1.5,"PASS","REVIEW")</f>
-        <v/>
-      </c>
-      <c r="C93" s="107">
-        <f>TEXT(D90,"0.0")&amp;"x spread vs Gordon-implied exit"</f>
-        <v/>
-      </c>
-      <c r="D93" s="26" t="inlineStr">
+      <c r="B94" s="106">
+        <f>IF(ABS(D91)&lt;=1.5,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+      <c r="C94" s="107">
+        <f>TEXT(D91,"0.0")&amp;"x spread vs Gordon-implied exit"</f>
+        <v/>
+      </c>
+      <c r="D94" s="26" t="inlineStr">
         <is>
           <t>Selected exit is the Gordon identity, so spread should be 0</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="93" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="93" t="inlineStr">
         <is>
           <t>SENSITIVITY — IMPLIED SHARE PRICE (WACC vs terminal growth)</t>
         </is>
       </c>
-      <c r="B96" s="13" t="n"/>
-      <c r="C96" s="13" t="n"/>
-      <c r="D96" s="13" t="n"/>
-      <c r="E96" s="13" t="n"/>
-      <c r="F96" s="13" t="n"/>
-      <c r="G96" s="13" t="n"/>
-      <c r="H96" s="13" t="n"/>
-    </row>
-    <row r="97" ht="28" customHeight="1">
-      <c r="A97" s="108" t="inlineStr">
+      <c r="B97" s="13" t="n"/>
+      <c r="C97" s="13" t="n"/>
+      <c r="D97" s="13" t="n"/>
+      <c r="E97" s="13" t="n"/>
+      <c r="F97" s="13" t="n"/>
+      <c r="G97" s="13" t="n"/>
+      <c r="H97" s="13" t="n"/>
+    </row>
+    <row r="98" ht="28" customHeight="1">
+      <c r="A98" s="108" t="inlineStr">
         <is>
           <t>WACC \ g</t>
         </is>
       </c>
-      <c r="B97" s="17" t="inlineStr">
+      <c r="B98" s="17" t="inlineStr">
         <is>
           <t>Terminal-g axis 1.5–3.0% brackets 2.25% base; bounded by long-run real GDP and inflation benchmarks.</t>
         </is>
       </c>
-      <c r="C97" s="18" t="inlineStr">
+      <c r="C98" s="18" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="D97" s="19" t="inlineStr">
+      <c r="D98" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
       </c>
-      <c r="F97" s="109" t="n">
+      <c r="F98" s="109" t="n">
         <v>0.015</v>
       </c>
-      <c r="G97" s="109" t="n">
+      <c r="G98" s="109" t="n">
         <v>0.02</v>
       </c>
-      <c r="H97" s="109" t="n">
+      <c r="H98" s="109" t="n">
         <v>0.0225</v>
       </c>
-      <c r="I97" s="109" t="n">
+      <c r="I98" s="109" t="n">
         <v>0.025</v>
       </c>
-      <c r="J97" s="109" t="n">
+      <c r="J98" s="109" t="n">
         <v>0.03</v>
       </c>
-      <c r="L97" s="95" t="inlineStr">
+      <c r="L98" s="95" t="inlineStr">
         <is>
           <t>Scenarios: terminal g</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="28" customHeight="1">
-      <c r="A98" s="109" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="C98" s="95" t="inlineStr">
-        <is>
-          <t>Damodaran: Historical Implied ERP</t>
-        </is>
-      </c>
-      <c r="D98" s="19" t="inlineStr">
-        <is>
-          <t>WACC tab → green WACC cell ~9.0%. Sensitivity WACC axis brackets base ±100bps.</t>
-        </is>
-      </c>
-      <c r="F98" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E50+E51)/E55</f>
-        <v/>
-      </c>
-      <c r="G98" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E50+E51)/E55</f>
-        <v/>
-      </c>
-      <c r="H98" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E50+E51)/E55</f>
-        <v/>
-      </c>
-      <c r="I98" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E50+E51)/E55</f>
-        <v/>
-      </c>
-      <c r="J98" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E50+E51)/E55</f>
-        <v/>
-      </c>
-      <c r="L98" s="95" t="inlineStr">
-        <is>
-          <t>WACC tab</t>
         </is>
       </c>
     </row>
     <row r="99" ht="28" customHeight="1">
       <c r="A99" s="109" t="n">
-        <v>0.1</v>
+        <v>0.095</v>
+      </c>
+      <c r="C99" s="95" t="inlineStr">
+        <is>
+          <t>Damodaran: Historical Implied ERP</t>
+        </is>
       </c>
       <c r="D99" s="19" t="inlineStr">
         <is>
@@ -12144,23 +12231,23 @@
         </is>
       </c>
       <c r="F99" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E50+E51)/E55</f>
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="G99" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E50+E51)/E55</f>
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="H99" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E50+E51)/E55</f>
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="I99" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E50+E51)/E55</f>
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="J99" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E50+E51)/E55</f>
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="L99" s="95" t="inlineStr">
@@ -12171,7 +12258,7 @@
     </row>
     <row r="100" ht="28" customHeight="1">
       <c r="A100" s="109" t="n">
-        <v>0.105</v>
+        <v>0.1</v>
       </c>
       <c r="D100" s="19" t="inlineStr">
         <is>
@@ -12179,23 +12266,23 @@
         </is>
       </c>
       <c r="F100" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E50+E51)/E55</f>
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="G100" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E50+E51)/E55</f>
-        <v/>
-      </c>
-      <c r="H100" s="111">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E50+E51)/E55</f>
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E50+E51)/E55</f>
+        <v/>
+      </c>
+      <c r="H100" s="110">
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="I100" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E50+E51)/E55</f>
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="J100" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E50+E51)/E55</f>
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="L100" s="95" t="inlineStr">
@@ -12206,7 +12293,7 @@
     </row>
     <row r="101" ht="28" customHeight="1">
       <c r="A101" s="109" t="n">
-        <v>0.11</v>
+        <v>0.105</v>
       </c>
       <c r="D101" s="19" t="inlineStr">
         <is>
@@ -12214,23 +12301,23 @@
         </is>
       </c>
       <c r="F101" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E50+E51)/E55</f>
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="G101" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E50+E51)/E55</f>
-        <v/>
-      </c>
-      <c r="H101" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E50+E51)/E55</f>
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E50+E51)/E55</f>
+        <v/>
+      </c>
+      <c r="H101" s="111">
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="I101" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E50+E51)/E55</f>
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="J101" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E50+E51)/E55</f>
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E50+E51)/E55</f>
         <v/>
       </c>
       <c r="L101" s="95" t="inlineStr">
@@ -12241,61 +12328,96 @@
     </row>
     <row r="102" ht="28" customHeight="1">
       <c r="A102" s="109" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="D102" s="19" t="inlineStr">
+        <is>
+          <t>WACC tab → green WACC cell ~9.0%. Sensitivity WACC axis brackets base ±100bps.</t>
+        </is>
+      </c>
+      <c r="F102" s="110">
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E50+E51)/E55</f>
+        <v/>
+      </c>
+      <c r="G102" s="110">
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E50+E51)/E55</f>
+        <v/>
+      </c>
+      <c r="H102" s="110">
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E50+E51)/E55</f>
+        <v/>
+      </c>
+      <c r="I102" s="110">
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E50+E51)/E55</f>
+        <v/>
+      </c>
+      <c r="J102" s="110">
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E50+E51)/E55</f>
+        <v/>
+      </c>
+      <c r="L102" s="95" t="inlineStr">
+        <is>
+          <t>WACC tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="28" customHeight="1">
+      <c r="A103" s="109" t="n">
         <v>0.115</v>
       </c>
-      <c r="D102" s="19" t="inlineStr">
+      <c r="D103" s="19" t="inlineStr">
         <is>
           <t>WACC tab → green WACC cell ~9.0%. Sensitivity WACC axis brackets base ±100bps.</t>
         </is>
       </c>
-      <c r="F102" s="110">
+      <c r="F103" s="110">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="G102" s="110">
+      <c r="G103" s="110">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="H102" s="110">
+      <c r="H103" s="110">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="I102" s="110">
+      <c r="I103" s="110">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="J102" s="110">
+      <c r="J103" s="110">
         <f>(NPV(0.115,F35:J35)+(J35*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E50+E51)/E55</f>
         <v/>
       </c>
-      <c r="L102" s="95" t="inlineStr">
+      <c r="L103" s="95" t="inlineStr">
         <is>
           <t>WACC tab</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="28" customHeight="1">
-      <c r="B103" s="17" t="inlineStr">
+    <row r="104" ht="28" customHeight="1">
+      <c r="B104" s="17" t="inlineStr">
         <is>
           <t>Red WACC and g grid values bracket base case ±100bps discount rate and ±75bps terminal growth for sensitivity.</t>
         </is>
       </c>
-      <c r="C103" s="18" t="inlineStr">
+      <c r="C104" s="18" t="inlineStr">
         <is>
           <t>Scenarios: WACC &amp; terminal g</t>
         </is>
       </c>
-      <c r="D103" s="19" t="inlineStr">
+      <c r="D104" s="19" t="inlineStr">
         <is>
           <t>Scenarios tab → Ctrl+F "WACC" and "Terminal growth" rows (base-case inputs)</t>
         </is>
       </c>
-      <c r="L103" s="95" t="inlineStr">
+      <c r="L104" s="95" t="inlineStr">
         <is>
           <t>FRED: Real GDP (GDPC1)</t>
         </is>
       </c>
-      <c r="M103" s="19" t="inlineStr">
+      <c r="M104" s="19" t="inlineStr">
         <is>
           <t>Ctrl+F "GDPC1" → bounds terminal-g sensitivity grid 1.5%–3.0%</t>
         </is>
@@ -12353,18 +12475,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId45"/>
-    <hyperlink ref="C81" location="'DCF'!E46"/>
-    <hyperlink ref="M81" location="'Comps'!A45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId46"/>
-    <hyperlink ref="L97" location="'Scenarios'!G10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId47"/>
-    <hyperlink ref="L98" location="'WACC'!E41"/>
+    <hyperlink ref="C82" location="'DCF'!E46"/>
+    <hyperlink ref="M82" location="'Comps'!A45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId46"/>
+    <hyperlink ref="L98" location="'Scenarios'!G10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId47"/>
     <hyperlink ref="L99" location="'WACC'!E41"/>
     <hyperlink ref="L100" location="'WACC'!E41"/>
     <hyperlink ref="L101" location="'WACC'!E41"/>
     <hyperlink ref="L102" location="'WACC'!E41"/>
-    <hyperlink ref="C103" location="'Scenarios'!G9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L103" r:id="rId48"/>
+    <hyperlink ref="L103" location="'WACC'!E41"/>
+    <hyperlink ref="C104" location="'Scenarios'!G9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L104" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13024,7 +13146,7 @@
       <c r="C33" s="38" t="inlineStr">
         <is>
           <t>Reuters: Alo parent $10bn Moelis ask
-Also: Reuters: Alo 2023 process — no deal</t>
+Also: Reuters: Alo 2023 process; no deal</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -13206,7 +13328,7 @@
         </is>
       </c>
       <c r="E45" s="104">
-        <f>DCF!E81</f>
+        <f>DCF!E82</f>
         <v/>
       </c>
     </row>
@@ -13380,7 +13502,7 @@
         </is>
       </c>
       <c r="E58" s="118">
-        <f>DCF!E81</f>
+        <f>DCF!E82</f>
         <v/>
       </c>
       <c r="G58" s="122">
@@ -13498,7 +13620,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId14"/>
     <hyperlink ref="C35" location="'Comps'!E33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId15"/>
-    <hyperlink ref="C58" location="'DCF'!E81"/>
+    <hyperlink ref="C58" location="'DCF'!E82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId18"/>

</xml_diff>

<commit_message>
Remove NOPAT labels from Excel model deliverables
Rename Scenarios/DCF row labels and UFCF note to 'EBIT after tax';
wire scrub into the pitch update pipeline.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/LULU_DCF_Valuation_Model.xlsx
+++ b/LULU/LULU_DCF_Valuation_Model.xlsx
@@ -3334,7 +3334,7 @@
     <row r="50">
       <c r="A50" s="153" t="inlineStr">
         <is>
-          <t>NOPAT: year 1</t>
+          <t>EBIT after tax: year 1</t>
         </is>
       </c>
       <c r="B50" s="154">
@@ -3361,7 +3361,7 @@
     <row r="51">
       <c r="A51" s="153" t="inlineStr">
         <is>
-          <t>NOPAT: year 2</t>
+          <t>EBIT after tax: year 2</t>
         </is>
       </c>
       <c r="B51" s="154">
@@ -3384,7 +3384,7 @@
     <row r="52">
       <c r="A52" s="153" t="inlineStr">
         <is>
-          <t>NOPAT: year 3</t>
+          <t>EBIT after tax: year 3</t>
         </is>
       </c>
       <c r="B52" s="154">
@@ -3407,7 +3407,7 @@
     <row r="53">
       <c r="A53" s="153" t="inlineStr">
         <is>
-          <t>NOPAT: year 4</t>
+          <t>EBIT after tax: year 4</t>
         </is>
       </c>
       <c r="B53" s="154">
@@ -3430,7 +3430,7 @@
     <row r="54">
       <c r="A54" s="153" t="inlineStr">
         <is>
-          <t>NOPAT: year 5</t>
+          <t>EBIT after tax: year 5</t>
         </is>
       </c>
       <c r="B54" s="154">
@@ -5137,7 +5137,7 @@
       <c r="E125" s="174" t="n"/>
       <c r="F125" s="179" t="inlineStr">
         <is>
-          <t>NOPAT plus depreciation minus capex plus working capital.</t>
+          <t>After-tax EBIT plus depreciation minus capex plus working capital.</t>
         </is>
       </c>
       <c r="G125" s="42" t="n"/>
@@ -9574,7 +9574,7 @@
     <row r="14">
       <c r="A14" s="23" t="inlineStr">
         <is>
-          <t>NOPAT</t>
+          <t>EBIT after tax</t>
         </is>
       </c>
       <c r="B14" s="171" t="n"/>

</xml_diff>